<commit_message>
Add Escalation Follow-Up and Next Session Focus sections to scoring form
- Insert Escalation Follow-Up block (rows 108-114) immediately after the
  Escalation Judgment scoring category: captures what L2/next agent did
  and 3 L1 learning points derived from the escalation outcome
- Insert Next Session Focus block (rows 209-212) in §8 Coaching & Feedback
  after the Coaching Recommendation, before Q3 org insights: 3 numbered
  specific behaviors the agent should practice before the next review
- Update Score Summary cross-block formulas (D31, D32, E33, F33) to
  reference CE and Documentation rows at their new shifted positions
- All DVs, merges, and row heights remapped correctly after insertion

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -250,7 +250,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -435,11 +435,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -791,6 +831,9 @@
     <xf numFmtId="164" fontId="26" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3186,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:F219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3623,7 +3666,7 @@
         <v>0.05</v>
       </c>
       <c r="D31" s="23">
-        <f>IF(C120="",C119,C120)</f>
+        <f>IF(C127="",C126,C127)</f>
         <v/>
       </c>
       <c r="E31" s="24">
@@ -3645,7 +3688,7 @@
         <v>0.05</v>
       </c>
       <c r="D32" s="18">
-        <f>IF(C135="",C134,C135)</f>
+        <f>IF(C142="",C141,C142)</f>
         <v/>
       </c>
       <c r="E32" s="19">
@@ -3669,11 +3712,11 @@
       </c>
       <c r="D33" s="27" t="n"/>
       <c r="E33" s="28">
-        <f>IF(OR(C171="No",C172="No",C173="No",COUNTIF(C175:C185,"Yes")&gt;0,COUNTIF(C150:C165,"Yes")&gt;0),0,SUM(E26:E32))</f>
+        <f>IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),0,SUM(E26:E32))</f>
         <v/>
       </c>
       <c r="F33" s="29">
-        <f>IF(E33="","",IF(OR(C171="No",C172="No",C173="No",COUNTIF(C175:C185,"Yes")&gt;0,COUNTIF(C150:C165,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E33&gt;=0.85,"MEETS / EXCEEDS",IF(E33&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
+        <f>IF(E33="","",IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E33&gt;=0.85,"MEETS / EXCEEDS",IF(E33&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
         <v/>
       </c>
     </row>
@@ -4549,603 +4592,576 @@
       <c r="E107" s="82" t="n"/>
       <c r="F107" s="71" t="n"/>
     </row>
-    <row r="108">
-      <c r="B108" s="11" t="n"/>
-      <c r="C108" s="12" t="n"/>
-      <c r="D108" s="92" t="n"/>
-    </row>
-    <row r="109" ht="18" customHeight="1">
-      <c r="B109" s="80" t="inlineStr">
-        <is>
-          <t>6. CUSTOMER EXPERIENCE</t>
-        </is>
-      </c>
-      <c r="C109" s="90" t="n"/>
-      <c r="D109" s="90" t="n"/>
-      <c r="E109" s="74" t="n"/>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="28" customHeight="1">
-      <c r="B110" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
-        </is>
-      </c>
-      <c r="C110" s="82" t="n"/>
-      <c r="D110" s="82" t="n"/>
-      <c r="E110" s="82" t="n"/>
-      <c r="F110" s="71" t="n"/>
-    </row>
-    <row r="111">
-      <c r="B111" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C111" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D111" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
-      <c r="E111" s="82" t="n"/>
-      <c r="F111" s="71" t="n"/>
+    <row r="108" ht="20" customHeight="1">
+      <c r="B108" s="80" t="inlineStr">
+        <is>
+          <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
+        </is>
+      </c>
+      <c r="C108" s="90" t="n"/>
+      <c r="D108" s="90" t="n"/>
+      <c r="E108" s="90" t="n"/>
+      <c r="F108" s="74" t="n"/>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="B109" s="13" t="inlineStr">
+        <is>
+          <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
+        </is>
+      </c>
+      <c r="C109" s="123" t="n"/>
+      <c r="F109" s="6" t="n"/>
+    </row>
+    <row r="110" ht="45" customHeight="1">
+      <c r="B110" s="124" t="n"/>
+      <c r="C110" s="125" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="B111" s="80" t="inlineStr">
+        <is>
+          <t>L1 learning points from this escalation outcome</t>
+        </is>
+      </c>
+      <c r="C111" s="90" t="n"/>
+      <c r="D111" s="90" t="n"/>
+      <c r="E111" s="90" t="n"/>
+      <c r="F111" s="74" t="n"/>
     </row>
     <row r="112" ht="28" customHeight="1">
-      <c r="B112" s="81" t="inlineStr">
-        <is>
-          <t>Empathy was demonstrated (incl. acknowledging cumulative effort and fatigue on repeat contacts)</t>
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>1.</t>
         </is>
       </c>
       <c r="C112" s="9" t="n"/>
-      <c r="D112" s="81" t="n"/>
+      <c r="D112" s="82" t="n"/>
       <c r="E112" s="82" t="n"/>
       <c r="F112" s="71" t="n"/>
     </row>
     <row r="113" ht="28" customHeight="1">
-      <c r="B113" s="83" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained throughout</t>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>2.</t>
         </is>
       </c>
       <c r="C113" s="9" t="n"/>
-      <c r="D113" s="83" t="n"/>
+      <c r="D113" s="82" t="n"/>
       <c r="E113" s="82" t="n"/>
       <c r="F113" s="71" t="n"/>
     </row>
     <row r="114" ht="28" customHeight="1">
-      <c r="B114" s="81" t="inlineStr">
-        <is>
-          <t>Communication style was adapted to the customer</t>
+      <c r="B114" s="13" t="inlineStr">
+        <is>
+          <t>3.</t>
         </is>
       </c>
       <c r="C114" s="9" t="n"/>
-      <c r="D114" s="81" t="n"/>
+      <c r="D114" s="82" t="n"/>
       <c r="E114" s="82" t="n"/>
       <c r="F114" s="71" t="n"/>
     </row>
     <row r="115" ht="28" customHeight="1">
-      <c r="B115" s="83" t="inlineStr">
-        <is>
-          <t>Patience was maintained, even under pressure</t>
-        </is>
-      </c>
+      <c r="B115" s="83" t="n"/>
       <c r="C115" s="9" t="n"/>
       <c r="D115" s="83" t="n"/>
-      <c r="E115" s="82" t="n"/>
-      <c r="F115" s="71" t="n"/>
-    </row>
-    <row r="116" ht="28" customHeight="1">
-      <c r="B116" s="81" t="inlineStr">
-        <is>
-          <t>Customer effort was reduced where possible</t>
-        </is>
-      </c>
-      <c r="C116" s="9" t="n"/>
-      <c r="D116" s="81" t="n"/>
-      <c r="E116" s="82" t="n"/>
-      <c r="F116" s="71" t="n"/>
+    </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="B116" s="80" t="inlineStr">
+        <is>
+          <t>6. CUSTOMER EXPERIENCE</t>
+        </is>
+      </c>
+      <c r="C116" s="90" t="n"/>
+      <c r="D116" s="90" t="n"/>
+      <c r="E116" s="74" t="n"/>
+      <c r="F116" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 5%</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="28" customHeight="1">
-      <c r="B117" s="83" t="inlineStr">
-        <is>
-          <t>Customer felt heard, understood next steps, and remained engaged</t>
-        </is>
-      </c>
-      <c r="C117" s="9" t="n"/>
-      <c r="D117" s="83" t="n"/>
+      <c r="B117" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
+        </is>
+      </c>
+      <c r="C117" s="82" t="n"/>
+      <c r="D117" s="82" t="n"/>
       <c r="E117" s="82" t="n"/>
       <c r="F117" s="71" t="n"/>
     </row>
     <row r="118" ht="28" customHeight="1">
-      <c r="B118" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="C118" s="82" t="n"/>
-      <c r="D118" s="82" t="n"/>
+      <c r="B118" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D118" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E118" s="82" t="n"/>
       <c r="F118" s="71" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1">
-      <c r="B119" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C119" s="122">
-        <f>IF((COUNTIF(C112:C117,"Met")+COUNTIF(C112:C117,"Partial")+COUNTIF(C112:C117,"Missed"))=0,"",ROUND((COUNTIF(C112:C117,"Met")*5+COUNTIF(C112:C117,"Partial")*2.5)/(COUNTIF(C112:C117,"Met")+COUNTIF(C112:C117,"Partial")+COUNTIF(C112:C117,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D119" s="92" t="n"/>
+      <c r="B119" s="81" t="inlineStr">
+        <is>
+          <t>Empathy was demonstrated (incl. acknowledging cumulative effort and fatigue on repeat contacts)</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="n"/>
+      <c r="D119" s="81" t="n"/>
       <c r="E119" s="82" t="n"/>
       <c r="F119" s="71" t="n"/>
     </row>
-    <row r="120" ht="24" customHeight="1">
-      <c r="B120" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C120" s="14" t="n"/>
-      <c r="D120" s="84">
-        <f>IF(IF(C120="",C119,C120)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C120="",C119,C120)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="120" ht="28" customHeight="1">
+      <c r="B120" s="83" t="inlineStr">
+        <is>
+          <t>Professionalism was maintained throughout</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="n"/>
+      <c r="D120" s="83" t="n"/>
       <c r="E120" s="82" t="n"/>
       <c r="F120" s="71" t="n"/>
     </row>
-    <row r="121" ht="36" customHeight="1">
-      <c r="B121" s="13" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
-      <c r="C121" s="86" t="n"/>
-      <c r="D121" s="82" t="n"/>
+    <row r="121" ht="28" customHeight="1">
+      <c r="B121" s="81" t="inlineStr">
+        <is>
+          <t>Communication style was adapted to the customer</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="n"/>
+      <c r="D121" s="81" t="n"/>
       <c r="E121" s="82" t="n"/>
       <c r="F121" s="71" t="n"/>
     </row>
     <row r="122" ht="28" customHeight="1">
-      <c r="B122" s="85" t="n"/>
-    </row>
-    <row r="123" ht="18" customHeight="1">
-      <c r="B123" s="80" t="inlineStr">
-        <is>
-          <t>7. DOCUMENTATION &amp; NOTES</t>
-        </is>
-      </c>
-      <c r="C123" s="90" t="n"/>
-      <c r="D123" s="90" t="n"/>
-      <c r="E123" s="74" t="n"/>
-      <c r="F123" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 5%</t>
-        </is>
-      </c>
+      <c r="B122" s="83" t="inlineStr">
+        <is>
+          <t>Patience was maintained, even under pressure</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="n"/>
+      <c r="D122" s="83" t="n"/>
+      <c r="E122" s="82" t="n"/>
+      <c r="F122" s="71" t="n"/>
+    </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="B123" s="81" t="inlineStr">
+        <is>
+          <t>Customer effort was reduced where possible</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="n"/>
+      <c r="D123" s="81" t="n"/>
+      <c r="E123" s="82" t="n"/>
+      <c r="F123" s="71" t="n"/>
     </row>
     <row r="124" ht="28" customHeight="1">
-      <c r="B124" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
-        </is>
-      </c>
-      <c r="C124" s="82" t="n"/>
-      <c r="D124" s="82" t="n"/>
+      <c r="B124" s="83" t="inlineStr">
+        <is>
+          <t>Customer felt heard, understood next steps, and remained engaged</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="n"/>
+      <c r="D124" s="83" t="n"/>
       <c r="E124" s="82" t="n"/>
       <c r="F124" s="71" t="n"/>
     </row>
-    <row r="125" ht="36" customHeight="1">
-      <c r="B125" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C125" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D125" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+    <row r="125" ht="28" customHeight="1">
+      <c r="B125" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
+        </is>
+      </c>
+      <c r="C125" s="82" t="n"/>
+      <c r="D125" s="82" t="n"/>
       <c r="E125" s="82" t="n"/>
       <c r="F125" s="71" t="n"/>
     </row>
     <row r="126" ht="28" customHeight="1">
-      <c r="B126" s="81" t="inlineStr">
-        <is>
-          <t>Customer issue summary recorded</t>
-        </is>
-      </c>
-      <c r="C126" s="9" t="n"/>
-      <c r="D126" s="81" t="n"/>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C126" s="122">
+        <f>IF((COUNTIF(C119:C124,"Met")+COUNTIF(C119:C124,"Partial")+COUNTIF(C119:C124,"Missed"))=0,"",ROUND((COUNTIF(C119:C124,"Met")*5+COUNTIF(C119:C124,"Partial")*2.5)/(COUNTIF(C119:C124,"Met")+COUNTIF(C119:C124,"Partial")+COUNTIF(C119:C124,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D126" s="92" t="n"/>
       <c r="E126" s="82" t="n"/>
       <c r="F126" s="71" t="n"/>
     </row>
-    <row r="127" ht="28" customHeight="1">
-      <c r="B127" s="83" t="inlineStr">
-        <is>
-          <t>Troubleshooting performed is documented</t>
-        </is>
-      </c>
-      <c r="C127" s="9" t="n"/>
-      <c r="D127" s="83" t="n"/>
+    <row r="127" ht="24" customHeight="1">
+      <c r="B127" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C127" s="14" t="n"/>
+      <c r="D127" s="84">
+        <f>IF(IF(C127="",C126,C127)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C127="",C126,C127)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E127" s="82" t="n"/>
       <c r="F127" s="71" t="n"/>
     </row>
-    <row r="128" ht="28" customHeight="1">
-      <c r="B128" s="81" t="inlineStr">
-        <is>
-          <t>Key findings / discoveries noted</t>
-        </is>
-      </c>
-      <c r="C128" s="9" t="n"/>
-      <c r="D128" s="81" t="n"/>
+    <row r="128" ht="36" customHeight="1">
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
+        </is>
+      </c>
+      <c r="C128" s="86" t="n"/>
+      <c r="D128" s="82" t="n"/>
       <c r="E128" s="82" t="n"/>
       <c r="F128" s="71" t="n"/>
     </row>
     <row r="129" ht="28" customHeight="1">
-      <c r="B129" s="83" t="inlineStr">
-        <is>
-          <t>Agent reasoning is captured</t>
-        </is>
-      </c>
+      <c r="B129" s="85" t="n"/>
       <c r="C129" s="9" t="n"/>
       <c r="D129" s="83" t="n"/>
-      <c r="E129" s="82" t="n"/>
-      <c r="F129" s="71" t="n"/>
-    </row>
-    <row r="130" ht="28" customHeight="1">
-      <c r="B130" s="81" t="inlineStr">
-        <is>
-          <t>Escalation justification included — mark N.A. if no escalation</t>
-        </is>
-      </c>
-      <c r="C130" s="9" t="n"/>
-      <c r="D130" s="81" t="n"/>
-      <c r="E130" s="82" t="n"/>
-      <c r="F130" s="71" t="n"/>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="B130" s="80" t="inlineStr">
+        <is>
+          <t>7. DOCUMENTATION &amp; NOTES</t>
+        </is>
+      </c>
+      <c r="C130" s="90" t="n"/>
+      <c r="D130" s="90" t="n"/>
+      <c r="E130" s="74" t="n"/>
+      <c r="F130" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 5%</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="28" customHeight="1">
-      <c r="B131" s="83" t="inlineStr">
-        <is>
-          <t>Next steps and follow-up actions listed (incl. callback records)</t>
-        </is>
-      </c>
-      <c r="C131" s="9" t="n"/>
-      <c r="D131" s="83" t="n"/>
+      <c r="B131" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
+        </is>
+      </c>
+      <c r="C131" s="82" t="n"/>
+      <c r="D131" s="82" t="n"/>
       <c r="E131" s="82" t="n"/>
       <c r="F131" s="71" t="n"/>
     </row>
-    <row r="132" ht="28" customHeight="1">
-      <c r="B132" s="81" t="inlineStr">
-        <is>
-          <t>Ticket status accurately reflects case state (no premature RESOLVED; closure reason documented)</t>
-        </is>
-      </c>
-      <c r="C132" s="9" t="n"/>
-      <c r="D132" s="81" t="n"/>
+    <row r="132" ht="36" customHeight="1">
+      <c r="B132" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D132" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E132" s="82" t="n"/>
       <c r="F132" s="71" t="n"/>
     </row>
     <row r="133" ht="28" customHeight="1">
-      <c r="B133" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="C133" s="82" t="n"/>
-      <c r="D133" s="82" t="n"/>
+      <c r="B133" s="81" t="inlineStr">
+        <is>
+          <t>Customer issue summary recorded</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="n"/>
+      <c r="D133" s="81" t="n"/>
       <c r="E133" s="82" t="n"/>
       <c r="F133" s="71" t="n"/>
     </row>
-    <row r="134">
-      <c r="B134" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C134" s="122">
-        <f>IF((COUNTIF(C126:C132,"Met")+COUNTIF(C126:C132,"Partial")+COUNTIF(C126:C132,"Missed"))=0,"",ROUND((COUNTIF(C126:C132,"Met")*5+COUNTIF(C126:C132,"Partial")*2.5)/(COUNTIF(C126:C132,"Met")+COUNTIF(C126:C132,"Partial")+COUNTIF(C126:C132,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D134" s="92" t="n"/>
+    <row r="134" ht="28" customHeight="1">
+      <c r="B134" s="83" t="inlineStr">
+        <is>
+          <t>Troubleshooting performed is documented</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="n"/>
+      <c r="D134" s="83" t="n"/>
       <c r="E134" s="82" t="n"/>
       <c r="F134" s="71" t="n"/>
     </row>
-    <row r="135" ht="24" customHeight="1">
-      <c r="B135" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C135" s="14" t="n"/>
-      <c r="D135" s="84">
-        <f>IF(IF(C135="",C134,C135)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C135="",C134,C135)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="135" ht="28" customHeight="1">
+      <c r="B135" s="81" t="inlineStr">
+        <is>
+          <t>Key findings / discoveries noted</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="n"/>
+      <c r="D135" s="81" t="n"/>
       <c r="E135" s="82" t="n"/>
       <c r="F135" s="71" t="n"/>
     </row>
-    <row r="136" ht="36" customHeight="1">
-      <c r="B136" s="13" t="inlineStr">
-        <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
-      <c r="C136" s="86" t="n"/>
-      <c r="D136" s="82" t="n"/>
+    <row r="136" ht="28" customHeight="1">
+      <c r="B136" s="83" t="inlineStr">
+        <is>
+          <t>Agent reasoning is captured</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="n"/>
+      <c r="D136" s="83" t="n"/>
       <c r="E136" s="82" t="n"/>
       <c r="F136" s="71" t="n"/>
     </row>
-    <row r="137"/>
-    <row r="138">
-      <c r="B138" s="80" t="n"/>
-    </row>
-    <row r="139">
-      <c r="B139" s="80" t="inlineStr">
-        <is>
-          <t>4 · RESOLUTION OUTCOME</t>
-        </is>
-      </c>
-      <c r="C139" s="90" t="n"/>
-      <c r="D139" s="90" t="n"/>
-      <c r="E139" s="90" t="n"/>
-      <c r="F139" s="74" t="n"/>
-    </row>
-    <row r="140">
-      <c r="B140" s="94" t="inlineStr">
-        <is>
-          <t>Outcome classification</t>
-        </is>
-      </c>
-      <c r="C140" s="97" t="n"/>
+    <row r="137" ht="28" customHeight="1">
+      <c r="B137" s="81" t="inlineStr">
+        <is>
+          <t>Escalation justification included — mark N.A. if no escalation</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="n"/>
+      <c r="D137" s="81" t="n"/>
+      <c r="E137" s="82" t="n"/>
+      <c r="F137" s="71" t="n"/>
+    </row>
+    <row r="138" ht="28" customHeight="1">
+      <c r="B138" s="83" t="inlineStr">
+        <is>
+          <t>Next steps and follow-up actions listed (incl. callback records)</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="n"/>
+      <c r="D138" s="83" t="n"/>
+      <c r="E138" s="82" t="n"/>
+      <c r="F138" s="71" t="n"/>
+    </row>
+    <row r="139" ht="28" customHeight="1">
+      <c r="B139" s="81" t="inlineStr">
+        <is>
+          <t>Ticket status accurately reflects case state (no premature RESOLVED; closure reason documented)</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="n"/>
+      <c r="D139" s="81" t="n"/>
+      <c r="E139" s="82" t="n"/>
+      <c r="F139" s="71" t="n"/>
+    </row>
+    <row r="140" ht="28" customHeight="1">
+      <c r="B140" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
+        </is>
+      </c>
+      <c r="C140" s="82" t="n"/>
       <c r="D140" s="82" t="n"/>
       <c r="E140" s="82" t="n"/>
       <c r="F140" s="71" t="n"/>
     </row>
     <row r="141" ht="52" customHeight="1">
-      <c r="B141" s="87" t="inlineStr">
-        <is>
-          <t>Primary positive outcome achieved</t>
-        </is>
-      </c>
-      <c r="C141" s="88" t="n"/>
-      <c r="D141" s="82" t="n"/>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C141" s="122">
+        <f>IF((COUNTIF(C133:C139,"Met")+COUNTIF(C133:C139,"Partial")+COUNTIF(C133:C139,"Missed"))=0,"",ROUND((COUNTIF(C133:C139,"Met")*5+COUNTIF(C133:C139,"Partial")*2.5)/(COUNTIF(C133:C139,"Met")+COUNTIF(C133:C139,"Partial")+COUNTIF(C133:C139,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D141" s="92" t="n"/>
       <c r="E141" s="82" t="n"/>
       <c r="F141" s="71" t="n"/>
     </row>
-    <row r="142" ht="52" customHeight="1">
-      <c r="B142" s="94" t="inlineStr">
-        <is>
-          <t>Justification</t>
-        </is>
-      </c>
-      <c r="C142" s="86" t="n"/>
-      <c r="D142" s="82" t="n"/>
+    <row r="142" ht="24" customHeight="1">
+      <c r="B142" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C142" s="14" t="n"/>
+      <c r="D142" s="84">
+        <f>IF(IF(C142="",C141,C142)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C142="",C141,C142)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E142" s="82" t="n"/>
       <c r="F142" s="71" t="n"/>
     </row>
-    <row r="143">
-      <c r="B143" s="80" t="n"/>
+    <row r="143" ht="36" customHeight="1">
+      <c r="B143" s="13" t="inlineStr">
+        <is>
+          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
+        </is>
+      </c>
+      <c r="C143" s="86" t="n"/>
+      <c r="D143" s="82" t="n"/>
+      <c r="E143" s="82" t="n"/>
+      <c r="F143" s="71" t="n"/>
     </row>
     <row r="144">
-      <c r="B144" s="80" t="inlineStr">
+      <c r="B144" s="80" t="n"/>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="B145" s="80" t="n"/>
+      <c r="C145" s="9" t="n"/>
+      <c r="D145" s="85" t="n"/>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="B146" s="80" t="inlineStr">
+        <is>
+          <t>4 · RESOLUTION OUTCOME</t>
+        </is>
+      </c>
+      <c r="C146" s="90" t="n"/>
+      <c r="D146" s="90" t="n"/>
+      <c r="E146" s="90" t="n"/>
+      <c r="F146" s="74" t="n"/>
+    </row>
+    <row r="147">
+      <c r="B147" s="94" t="inlineStr">
+        <is>
+          <t>Outcome classification</t>
+        </is>
+      </c>
+      <c r="C147" s="97" t="n"/>
+      <c r="D147" s="82" t="n"/>
+      <c r="E147" s="82" t="n"/>
+      <c r="F147" s="71" t="n"/>
+    </row>
+    <row r="148" ht="52" customHeight="1">
+      <c r="B148" s="87" t="inlineStr">
+        <is>
+          <t>Primary positive outcome achieved</t>
+        </is>
+      </c>
+      <c r="C148" s="88" t="n"/>
+      <c r="D148" s="82" t="n"/>
+      <c r="E148" s="82" t="n"/>
+      <c r="F148" s="71" t="n"/>
+    </row>
+    <row r="149" ht="52" customHeight="1">
+      <c r="B149" s="94" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
+      <c r="C149" s="86" t="n"/>
+      <c r="D149" s="82" t="n"/>
+      <c r="E149" s="82" t="n"/>
+      <c r="F149" s="71" t="n"/>
+    </row>
+    <row r="150" ht="26" customHeight="1">
+      <c r="B150" s="80" t="n"/>
+      <c r="C150" s="9" t="n"/>
+      <c r="D150" s="81" t="n"/>
+    </row>
+    <row r="151" ht="26" customHeight="1">
+      <c r="B151" s="80" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
       </c>
-      <c r="C144" s="90" t="n"/>
-      <c r="D144" s="90" t="n"/>
-      <c r="E144" s="90" t="n"/>
-      <c r="F144" s="74" t="n"/>
-    </row>
-    <row r="145" ht="30" customHeight="1">
-      <c r="B145" s="87" t="inlineStr">
+      <c r="C151" s="90" t="n"/>
+      <c r="D151" s="90" t="n"/>
+      <c r="E151" s="90" t="n"/>
+      <c r="F151" s="74" t="n"/>
+    </row>
+    <row r="152" ht="30" customHeight="1">
+      <c r="B152" s="87" t="inlineStr">
         <is>
           <t>Did the interaction disconnect before completion?</t>
         </is>
       </c>
-      <c r="C145" s="9" t="inlineStr">
+      <c r="C152" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D145" s="85" t="inlineStr">
+      <c r="D152" s="85" t="inlineStr">
         <is>
           <t>If Yes, at least one documented follow-up action is required.</t>
         </is>
       </c>
-      <c r="E145" s="82" t="n"/>
-      <c r="F145" s="71" t="n"/>
-    </row>
-    <row r="146" ht="30" customHeight="1">
-      <c r="B146" s="94" t="inlineStr">
-        <is>
-          <t>Follow-up action taken</t>
-        </is>
-      </c>
-      <c r="C146" s="88" t="inlineStr">
-        <is>
-          <t>N.A. — no disconnect</t>
-        </is>
-      </c>
-      <c r="D146" s="71" t="n"/>
-      <c r="E146" s="79">
-        <f>IF(AND(C145="Yes",OR(C146="None",C146="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
-        <v/>
-      </c>
-      <c r="F146" s="71" t="n"/>
-    </row>
-    <row r="147">
-      <c r="B147" s="98" t="n"/>
-    </row>
-    <row r="148">
-      <c r="B148" s="98" t="inlineStr">
-        <is>
-          <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
-        </is>
-      </c>
-      <c r="C148" s="90" t="n"/>
-      <c r="D148" s="90" t="n"/>
-      <c r="E148" s="90" t="n"/>
-      <c r="F148" s="74" t="n"/>
-    </row>
-    <row r="149" ht="26" customHeight="1">
-      <c r="B149" s="80" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="C149" s="119" t="inlineStr">
-        <is>
-          <t>Present?</t>
-        </is>
-      </c>
-      <c r="D149" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E149" s="90" t="n"/>
-      <c r="F149" s="74" t="n"/>
-    </row>
-    <row r="150" ht="26" customHeight="1">
-      <c r="B150" s="81" t="inlineStr">
-        <is>
-          <t>Harmful or incorrect troubleshooting provided</t>
-        </is>
-      </c>
-      <c r="C150" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D150" s="81" t="n"/>
-      <c r="E150" s="82" t="n"/>
-      <c r="F150" s="71" t="n"/>
-    </row>
-    <row r="151" ht="26" customHeight="1">
-      <c r="B151" s="83" t="inlineStr">
-        <is>
-          <t>Misrepresented product capabilities</t>
-        </is>
-      </c>
-      <c r="C151" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D151" s="83" t="n"/>
-      <c r="E151" s="82" t="n"/>
-      <c r="F151" s="71" t="n"/>
-    </row>
-    <row r="152" ht="26" customHeight="1">
-      <c r="B152" s="81" t="inlineStr">
-        <is>
-          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
-        </is>
-      </c>
-      <c r="C152" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D152" s="81" t="n"/>
       <c r="E152" s="82" t="n"/>
       <c r="F152" s="71" t="n"/>
     </row>
-    <row r="153" ht="26" customHeight="1">
-      <c r="B153" s="83" t="inlineStr">
-        <is>
-          <t>No follow-up after disconnected call</t>
-        </is>
-      </c>
-      <c r="C153" s="9" t="inlineStr">
+    <row r="153" ht="30" customHeight="1">
+      <c r="B153" s="94" t="inlineStr">
+        <is>
+          <t>Follow-up action taken</t>
+        </is>
+      </c>
+      <c r="C153" s="88" t="inlineStr">
+        <is>
+          <t>N.A. — no disconnect</t>
+        </is>
+      </c>
+      <c r="D153" s="71" t="n"/>
+      <c r="E153" s="79">
+        <f>IF(AND(C152="Yes",OR(C153="None",C153="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
+        <v/>
+      </c>
+      <c r="F153" s="71" t="n"/>
+    </row>
+    <row r="154" ht="26" customHeight="1">
+      <c r="B154" s="98" t="n"/>
+      <c r="C154" s="9" t="n"/>
+      <c r="D154" s="81" t="n"/>
+    </row>
+    <row r="155" ht="26" customHeight="1">
+      <c r="B155" s="98" t="inlineStr">
+        <is>
+          <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
+        </is>
+      </c>
+      <c r="C155" s="90" t="n"/>
+      <c r="D155" s="90" t="n"/>
+      <c r="E155" s="90" t="n"/>
+      <c r="F155" s="74" t="n"/>
+    </row>
+    <row r="156" ht="26" customHeight="1">
+      <c r="B156" s="80" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="C156" s="119" t="inlineStr">
+        <is>
+          <t>Present?</t>
+        </is>
+      </c>
+      <c r="D156" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E156" s="90" t="n"/>
+      <c r="F156" s="74" t="n"/>
+    </row>
+    <row r="157" ht="26" customHeight="1">
+      <c r="B157" s="81" t="inlineStr">
+        <is>
+          <t>Harmful or incorrect troubleshooting provided</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D153" s="83" t="n"/>
-      <c r="E153" s="82" t="n"/>
-      <c r="F153" s="71" t="n"/>
-    </row>
-    <row r="154" ht="26" customHeight="1">
-      <c r="B154" s="81" t="inlineStr">
-        <is>
-          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
-        </is>
-      </c>
-      <c r="C154" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D154" s="81" t="n"/>
-      <c r="E154" s="82" t="n"/>
-      <c r="F154" s="71" t="n"/>
-    </row>
-    <row r="155" ht="26" customHeight="1">
-      <c r="B155" s="83" t="inlineStr">
-        <is>
-          <t>Abandoned customer without a path forward</t>
-        </is>
-      </c>
-      <c r="C155" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D155" s="83" t="n"/>
-      <c r="E155" s="82" t="n"/>
-      <c r="F155" s="71" t="n"/>
-    </row>
-    <row r="156" ht="26" customHeight="1">
-      <c r="B156" s="81" t="inlineStr">
-        <is>
-          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
-        </is>
-      </c>
-      <c r="C156" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D156" s="81" t="n"/>
-      <c r="E156" s="82" t="n"/>
-      <c r="F156" s="71" t="n"/>
-    </row>
-    <row r="157" ht="26" customHeight="1">
-      <c r="B157" s="83" t="inlineStr">
-        <is>
-          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
-        </is>
-      </c>
-      <c r="C157" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D157" s="83" t="n"/>
+      <c r="D157" s="81" t="n"/>
       <c r="E157" s="82" t="n"/>
       <c r="F157" s="71" t="n"/>
     </row>
     <row r="158" ht="26" customHeight="1">
-      <c r="B158" s="81" t="inlineStr">
-        <is>
-          <t>Compliance / security violation (e.g., payment card data spoken or stored in plaintext — PCI DSS)</t>
+      <c r="B158" s="83" t="inlineStr">
+        <is>
+          <t>Misrepresented product capabilities</t>
         </is>
       </c>
       <c r="C158" s="9" t="inlineStr">
@@ -5153,14 +5169,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D158" s="81" t="n"/>
+      <c r="D158" s="83" t="n"/>
       <c r="E158" s="82" t="n"/>
       <c r="F158" s="71" t="n"/>
     </row>
     <row r="159" ht="26" customHeight="1">
-      <c r="B159" s="83" t="inlineStr">
-        <is>
-          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
+      <c r="B159" s="81" t="inlineStr">
+        <is>
+          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
         </is>
       </c>
       <c r="C159" s="9" t="inlineStr">
@@ -5168,14 +5184,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D159" s="83" t="n"/>
+      <c r="D159" s="81" t="n"/>
       <c r="E159" s="82" t="n"/>
       <c r="F159" s="71" t="n"/>
     </row>
     <row r="160" ht="26" customHeight="1">
-      <c r="B160" s="81" t="inlineStr">
-        <is>
-          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
+      <c r="B160" s="83" t="inlineStr">
+        <is>
+          <t>No follow-up after disconnected call</t>
         </is>
       </c>
       <c r="C160" s="9" t="inlineStr">
@@ -5183,14 +5199,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D160" s="81" t="n"/>
+      <c r="D160" s="83" t="n"/>
       <c r="E160" s="82" t="n"/>
       <c r="F160" s="71" t="n"/>
     </row>
     <row r="161" ht="26" customHeight="1">
       <c r="B161" s="81" t="inlineStr">
         <is>
-          <t>Line release — agent ended a live, unresolved contact</t>
+          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
         </is>
       </c>
       <c r="C161" s="9" t="inlineStr">
@@ -5203,9 +5219,9 @@
       <c r="F161" s="71" t="n"/>
     </row>
     <row r="162" ht="26" customHeight="1">
-      <c r="B162" s="81" t="inlineStr">
-        <is>
-          <t>Call / session avoidance or evasion</t>
+      <c r="B162" s="83" t="inlineStr">
+        <is>
+          <t>Abandoned customer without a path forward</t>
         </is>
       </c>
       <c r="C162" s="9" t="inlineStr">
@@ -5213,14 +5229,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D162" s="81" t="n"/>
+      <c r="D162" s="83" t="n"/>
       <c r="E162" s="82" t="n"/>
       <c r="F162" s="71" t="n"/>
     </row>
     <row r="163" ht="26" customHeight="1">
       <c r="B163" s="81" t="inlineStr">
         <is>
-          <t>Survey / CSAT manipulation</t>
+          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
         </is>
       </c>
       <c r="C163" s="9" t="inlineStr">
@@ -5233,9 +5249,9 @@
       <c r="F163" s="71" t="n"/>
     </row>
     <row r="164" ht="26" customHeight="1">
-      <c r="B164" s="81" t="inlineStr">
-        <is>
-          <t>Hard-selling or other sales-related irregularity</t>
+      <c r="B164" s="83" t="inlineStr">
+        <is>
+          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
         </is>
       </c>
       <c r="C164" s="9" t="inlineStr">
@@ -5243,14 +5259,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D164" s="81" t="n"/>
+      <c r="D164" s="83" t="n"/>
       <c r="E164" s="82" t="n"/>
       <c r="F164" s="71" t="n"/>
     </row>
     <row r="165" ht="26" customHeight="1">
       <c r="B165" s="81" t="inlineStr">
         <is>
-          <t>Unofficial email used, or failed to capture customer email</t>
+          <t>Compliance / security violation (e.g., payment card data spoken or stored in plaintext — PCI DSS)</t>
         </is>
       </c>
       <c r="C165" s="9" t="inlineStr">
@@ -5262,73 +5278,90 @@
       <c r="E165" s="82" t="n"/>
       <c r="F165" s="71" t="n"/>
     </row>
-    <row r="166">
-      <c r="B166" s="98" t="inlineStr">
-        <is>
-          <t>CRITICAL FAILURE FLAGGED?</t>
-        </is>
-      </c>
-      <c r="C166" s="93">
-        <f>IF(COUNTIF(C150:C165,"Yes")&gt;0,"YES — "&amp;COUNTIF(C150:C165,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
-        <v/>
-      </c>
-      <c r="D166" s="90" t="n"/>
-      <c r="E166" s="90" t="n"/>
-      <c r="F166" s="74" t="n"/>
-    </row>
-    <row r="167" ht="20" customHeight="1">
-      <c r="B167" s="96" t="n"/>
-    </row>
-    <row r="168" ht="22" customHeight="1">
-      <c r="B168" s="98" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
-      <c r="C168" s="90" t="n"/>
-      <c r="D168" s="90" t="n"/>
-      <c r="E168" s="90" t="n"/>
-      <c r="F168" s="74" t="n"/>
-    </row>
-    <row r="169" ht="30" customHeight="1">
-      <c r="B169" s="85" t="inlineStr">
-        <is>
-          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
-        </is>
-      </c>
-      <c r="C169" s="82" t="n"/>
-      <c r="D169" s="82" t="n"/>
+    <row r="166" ht="26" customHeight="1">
+      <c r="B166" s="83" t="inlineStr">
+        <is>
+          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
+        </is>
+      </c>
+      <c r="C166" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D166" s="83" t="n"/>
+      <c r="E166" s="82" t="n"/>
+      <c r="F166" s="71" t="n"/>
+    </row>
+    <row r="167" ht="26" customHeight="1">
+      <c r="B167" s="81" t="inlineStr">
+        <is>
+          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D167" s="81" t="n"/>
+      <c r="E167" s="82" t="n"/>
+      <c r="F167" s="71" t="n"/>
+    </row>
+    <row r="168" ht="26" customHeight="1">
+      <c r="B168" s="81" t="inlineStr">
+        <is>
+          <t>Line release — agent ended a live, unresolved contact</t>
+        </is>
+      </c>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D168" s="81" t="n"/>
+      <c r="E168" s="82" t="n"/>
+      <c r="F168" s="71" t="n"/>
+    </row>
+    <row r="169" ht="26" customHeight="1">
+      <c r="B169" s="81" t="inlineStr">
+        <is>
+          <t>Call / session avoidance or evasion</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D169" s="81" t="n"/>
       <c r="E169" s="82" t="n"/>
       <c r="F169" s="71" t="n"/>
     </row>
-    <row r="170" ht="30" customHeight="1">
-      <c r="B170" s="80" t="inlineStr">
-        <is>
-          <t>Compliance gate  (mark Yes if adhered)</t>
-        </is>
-      </c>
-      <c r="C170" s="119" t="inlineStr">
-        <is>
-          <t>Adherent?</t>
-        </is>
-      </c>
-      <c r="D170" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E170" s="90" t="n"/>
-      <c r="F170" s="74" t="n"/>
+    <row r="170" ht="26" customHeight="1">
+      <c r="B170" s="81" t="inlineStr">
+        <is>
+          <t>Survey / CSAT manipulation</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D170" s="81" t="n"/>
+      <c r="E170" s="82" t="n"/>
+      <c r="F170" s="71" t="n"/>
     </row>
     <row r="171" ht="26" customHeight="1">
       <c r="B171" s="81" t="inlineStr">
         <is>
-          <t>Adherence to Callback Hours</t>
+          <t>Hard-selling or other sales-related irregularity</t>
         </is>
       </c>
       <c r="C171" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D171" s="81" t="n"/>
@@ -5338,12 +5371,12 @@
     <row r="172" ht="26" customHeight="1">
       <c r="B172" s="81" t="inlineStr">
         <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
+          <t>Unofficial email used, or failed to capture customer email</t>
         </is>
       </c>
       <c r="C172" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D172" s="81" t="n"/>
@@ -5351,93 +5384,74 @@
       <c r="F172" s="71" t="n"/>
     </row>
     <row r="173" ht="26" customHeight="1">
-      <c r="B173" s="81" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C173" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D173" s="81" t="n"/>
-      <c r="E173" s="82" t="n"/>
-      <c r="F173" s="71" t="n"/>
-    </row>
-    <row r="174" ht="32" customHeight="1">
-      <c r="B174" s="80" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
-        </is>
-      </c>
-      <c r="C174" s="119" t="inlineStr">
-        <is>
-          <t>Occurred?</t>
-        </is>
-      </c>
-      <c r="D174" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E174" s="90" t="n"/>
-      <c r="F174" s="74" t="n"/>
-    </row>
-    <row r="175" ht="26" customHeight="1">
-      <c r="B175" s="81" t="inlineStr">
-        <is>
-          <t>A.  Call / Session Abandonment</t>
-        </is>
-      </c>
-      <c r="C175" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D175" s="81" t="n"/>
-      <c r="E175" s="82" t="n"/>
-      <c r="F175" s="71" t="n"/>
-    </row>
-    <row r="176" ht="26" customHeight="1">
-      <c r="B176" s="81" t="inlineStr">
-        <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
-        </is>
-      </c>
-      <c r="C176" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D176" s="81" t="n"/>
+      <c r="B173" s="98" t="inlineStr">
+        <is>
+          <t>CRITICAL FAILURE FLAGGED?</t>
+        </is>
+      </c>
+      <c r="C173" s="93">
+        <f>IF(COUNTIF(C157:C172,"Yes")&gt;0,"YES — "&amp;COUNTIF(C157:C172,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
+        <v/>
+      </c>
+      <c r="D173" s="90" t="n"/>
+      <c r="E173" s="90" t="n"/>
+      <c r="F173" s="74" t="n"/>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="B174" s="96" t="n"/>
+      <c r="C174" s="119" t="n"/>
+      <c r="D174" s="80" t="n"/>
+    </row>
+    <row r="175" ht="22" customHeight="1">
+      <c r="B175" s="98" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
+      <c r="C175" s="90" t="n"/>
+      <c r="D175" s="90" t="n"/>
+      <c r="E175" s="90" t="n"/>
+      <c r="F175" s="74" t="n"/>
+    </row>
+    <row r="176" ht="30" customHeight="1">
+      <c r="B176" s="85" t="inlineStr">
+        <is>
+          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
+        </is>
+      </c>
+      <c r="C176" s="82" t="n"/>
+      <c r="D176" s="82" t="n"/>
       <c r="E176" s="82" t="n"/>
       <c r="F176" s="71" t="n"/>
     </row>
-    <row r="177" ht="26" customHeight="1">
-      <c r="B177" s="81" t="inlineStr">
-        <is>
-          <t>C.  Discourtesy</t>
-        </is>
-      </c>
-      <c r="C177" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D177" s="81" t="n"/>
-      <c r="E177" s="82" t="n"/>
-      <c r="F177" s="71" t="n"/>
+    <row r="177" ht="30" customHeight="1">
+      <c r="B177" s="80" t="inlineStr">
+        <is>
+          <t>Compliance gate  (mark Yes if adhered)</t>
+        </is>
+      </c>
+      <c r="C177" s="119" t="inlineStr">
+        <is>
+          <t>Adherent?</t>
+        </is>
+      </c>
+      <c r="D177" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E177" s="90" t="n"/>
+      <c r="F177" s="74" t="n"/>
     </row>
     <row r="178" ht="26" customHeight="1">
       <c r="B178" s="81" t="inlineStr">
         <is>
-          <t>D.  Escalation</t>
+          <t>Adherence to Callback Hours</t>
         </is>
       </c>
       <c r="C178" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D178" s="81" t="n"/>
@@ -5447,12 +5461,12 @@
     <row r="179" ht="26" customHeight="1">
       <c r="B179" s="81" t="inlineStr">
         <is>
-          <t>E.  Failure to ask for the email address</t>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
         </is>
       </c>
       <c r="C179" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D179" s="81" t="n"/>
@@ -5462,37 +5476,41 @@
     <row r="180" ht="26" customHeight="1">
       <c r="B180" s="81" t="inlineStr">
         <is>
-          <t>F.  Fraud</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C180" s="9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D180" s="81" t="n"/>
       <c r="E180" s="82" t="n"/>
       <c r="F180" s="71" t="n"/>
     </row>
-    <row r="181" ht="26" customHeight="1">
-      <c r="B181" s="81" t="inlineStr">
-        <is>
-          <t>G.  Hard-selling</t>
-        </is>
-      </c>
-      <c r="C181" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D181" s="81" t="n"/>
-      <c r="E181" s="82" t="n"/>
-      <c r="F181" s="71" t="n"/>
+    <row r="181" ht="32" customHeight="1">
+      <c r="B181" s="80" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
+        </is>
+      </c>
+      <c r="C181" s="119" t="inlineStr">
+        <is>
+          <t>Occurred?</t>
+        </is>
+      </c>
+      <c r="D181" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E181" s="90" t="n"/>
+      <c r="F181" s="74" t="n"/>
     </row>
     <row r="182" ht="26" customHeight="1">
       <c r="B182" s="81" t="inlineStr">
         <is>
-          <t>H.  Line Release</t>
+          <t>A.  Call / Session Abandonment</t>
         </is>
       </c>
       <c r="C182" s="9" t="inlineStr">
@@ -5507,7 +5525,7 @@
     <row r="183" ht="26" customHeight="1">
       <c r="B183" s="81" t="inlineStr">
         <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
+          <t>B.  Call / Session Avoidance / Evasion</t>
         </is>
       </c>
       <c r="C183" s="9" t="inlineStr">
@@ -5522,7 +5540,7 @@
     <row r="184" ht="26" customHeight="1">
       <c r="B184" s="81" t="inlineStr">
         <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+          <t>C.  Discourtesy</t>
         </is>
       </c>
       <c r="C184" s="9" t="inlineStr">
@@ -5537,7 +5555,7 @@
     <row r="185" ht="26" customHeight="1">
       <c r="B185" s="81" t="inlineStr">
         <is>
-          <t>K.  Non-First Call Resolution</t>
+          <t>D.  Escalation</t>
         </is>
       </c>
       <c r="C185" s="9" t="inlineStr">
@@ -5549,184 +5567,217 @@
       <c r="E185" s="82" t="n"/>
       <c r="F185" s="71" t="n"/>
     </row>
-    <row r="186" ht="24" customHeight="1">
-      <c r="B186" s="98" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO TRIGGERED?</t>
-        </is>
-      </c>
-      <c r="C186" s="93">
-        <f>IF(OR(C171="No",C172="No",C173="No",COUNTIF(C175:C185,"Yes")&gt;0,COUNTIF(C150:C165,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
-      <c r="D186" s="90" t="n"/>
-      <c r="E186" s="90" t="n"/>
-      <c r="F186" s="74" t="n"/>
-    </row>
-    <row r="187" ht="58" customHeight="1">
-      <c r="B187" s="86" t="n"/>
-    </row>
-    <row r="188" ht="20" customHeight="1">
-      <c r="B188" s="96" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
-        </is>
-      </c>
-      <c r="C188" s="90" t="n"/>
-      <c r="D188" s="90" t="n"/>
-      <c r="E188" s="90" t="n"/>
-      <c r="F188" s="74" t="n"/>
-    </row>
-    <row r="189" ht="30" customHeight="1">
-      <c r="B189" s="91" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
-        </is>
-      </c>
-      <c r="C189" s="90" t="n"/>
-      <c r="D189" s="90" t="n"/>
-      <c r="E189" s="90" t="n"/>
-      <c r="F189" s="74" t="n"/>
-    </row>
-    <row r="190" ht="58" customHeight="1">
-      <c r="B190" s="86" t="n"/>
-      <c r="C190" s="82" t="n"/>
-      <c r="D190" s="82" t="n"/>
+    <row r="186" ht="26" customHeight="1">
+      <c r="B186" s="81" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="C186" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D186" s="81" t="n"/>
+      <c r="E186" s="82" t="n"/>
+      <c r="F186" s="71" t="n"/>
+    </row>
+    <row r="187" ht="26" customHeight="1">
+      <c r="B187" s="81" t="inlineStr">
+        <is>
+          <t>F.  Fraud</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D187" s="81" t="n"/>
+      <c r="E187" s="82" t="n"/>
+      <c r="F187" s="71" t="n"/>
+    </row>
+    <row r="188" ht="26" customHeight="1">
+      <c r="B188" s="81" t="inlineStr">
+        <is>
+          <t>G.  Hard-selling</t>
+        </is>
+      </c>
+      <c r="C188" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D188" s="81" t="n"/>
+      <c r="E188" s="82" t="n"/>
+      <c r="F188" s="71" t="n"/>
+    </row>
+    <row r="189" ht="26" customHeight="1">
+      <c r="B189" s="81" t="inlineStr">
+        <is>
+          <t>H.  Line Release</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D189" s="81" t="n"/>
+      <c r="E189" s="82" t="n"/>
+      <c r="F189" s="71" t="n"/>
+    </row>
+    <row r="190" ht="26" customHeight="1">
+      <c r="B190" s="81" t="inlineStr">
+        <is>
+          <t>I.  Non-Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C190" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D190" s="81" t="n"/>
       <c r="E190" s="82" t="n"/>
       <c r="F190" s="71" t="n"/>
     </row>
-    <row r="191" ht="30" customHeight="1">
-      <c r="B191" s="91" t="inlineStr">
-        <is>
-          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
-        </is>
-      </c>
-      <c r="C191" s="90" t="n"/>
-      <c r="D191" s="90" t="n"/>
-      <c r="E191" s="90" t="n"/>
-      <c r="F191" s="74" t="n"/>
-    </row>
-    <row r="192" ht="24" customHeight="1">
-      <c r="B192" s="87" t="inlineStr">
-        <is>
-          <t>What went well — behaviors to repeat</t>
-        </is>
-      </c>
-      <c r="C192" s="82" t="n"/>
-      <c r="D192" s="82" t="n"/>
+    <row r="191" ht="26" customHeight="1">
+      <c r="B191" s="81" t="inlineStr">
+        <is>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C191" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D191" s="81" t="n"/>
+      <c r="E191" s="82" t="n"/>
+      <c r="F191" s="71" t="n"/>
+    </row>
+    <row r="192" ht="26" customHeight="1">
+      <c r="B192" s="81" t="inlineStr">
+        <is>
+          <t>K.  Non-First Call Resolution</t>
+        </is>
+      </c>
+      <c r="C192" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D192" s="81" t="n"/>
       <c r="E192" s="82" t="n"/>
       <c r="F192" s="71" t="n"/>
     </row>
-    <row r="193" ht="32" customHeight="1">
-      <c r="B193" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C193" s="86" t="n"/>
-      <c r="D193" s="82" t="n"/>
-      <c r="E193" s="82" t="n"/>
-      <c r="F193" s="71" t="n"/>
-    </row>
-    <row r="194" ht="32" customHeight="1">
-      <c r="B194" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
+    <row r="193" ht="24" customHeight="1">
+      <c r="B193" s="98" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO TRIGGERED?</t>
+        </is>
+      </c>
+      <c r="C193" s="93">
+        <f>IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
+      <c r="D193" s="90" t="n"/>
+      <c r="E193" s="90" t="n"/>
+      <c r="F193" s="74" t="n"/>
+    </row>
+    <row r="194" ht="58" customHeight="1">
+      <c r="B194" s="86" t="n"/>
       <c r="C194" s="86" t="n"/>
-      <c r="D194" s="82" t="n"/>
-      <c r="E194" s="82" t="n"/>
-      <c r="F194" s="71" t="n"/>
-    </row>
-    <row r="195" ht="32" customHeight="1">
-      <c r="B195" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C195" s="86" t="n"/>
-      <c r="D195" s="82" t="n"/>
-      <c r="E195" s="82" t="n"/>
-      <c r="F195" s="71" t="n"/>
-    </row>
-    <row r="196" ht="24" customHeight="1">
-      <c r="B196" s="87" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
-      <c r="C196" s="82" t="n"/>
-      <c r="D196" s="82" t="n"/>
-      <c r="E196" s="82" t="n"/>
-      <c r="F196" s="71" t="n"/>
-    </row>
-    <row r="197" ht="32" customHeight="1">
-      <c r="B197" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C197" s="86" t="n"/>
+    </row>
+    <row r="195" ht="20" customHeight="1">
+      <c r="B195" s="96" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
+        </is>
+      </c>
+      <c r="C195" s="90" t="n"/>
+      <c r="D195" s="90" t="n"/>
+      <c r="E195" s="90" t="n"/>
+      <c r="F195" s="74" t="n"/>
+    </row>
+    <row r="196" ht="30" customHeight="1">
+      <c r="B196" s="91" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+        </is>
+      </c>
+      <c r="C196" s="90" t="n"/>
+      <c r="D196" s="90" t="n"/>
+      <c r="E196" s="90" t="n"/>
+      <c r="F196" s="74" t="n"/>
+    </row>
+    <row r="197" ht="58" customHeight="1">
+      <c r="B197" s="86" t="n"/>
+      <c r="C197" s="82" t="n"/>
       <c r="D197" s="82" t="n"/>
       <c r="E197" s="82" t="n"/>
       <c r="F197" s="71" t="n"/>
     </row>
-    <row r="198" ht="32" customHeight="1">
-      <c r="B198" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C198" s="86" t="n"/>
-      <c r="D198" s="82" t="n"/>
-      <c r="E198" s="82" t="n"/>
-      <c r="F198" s="71" t="n"/>
-    </row>
-    <row r="199" ht="32" customHeight="1">
-      <c r="B199" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C199" s="86" t="n"/>
+    <row r="198" ht="30" customHeight="1">
+      <c r="B198" s="91" t="inlineStr">
+        <is>
+          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
+        </is>
+      </c>
+      <c r="C198" s="90" t="n"/>
+      <c r="D198" s="90" t="n"/>
+      <c r="E198" s="90" t="n"/>
+      <c r="F198" s="74" t="n"/>
+    </row>
+    <row r="199" ht="24" customHeight="1">
+      <c r="B199" s="87" t="inlineStr">
+        <is>
+          <t>What went well — behaviors to repeat</t>
+        </is>
+      </c>
+      <c r="C199" s="82" t="n"/>
       <c r="D199" s="82" t="n"/>
       <c r="E199" s="82" t="n"/>
       <c r="F199" s="71" t="n"/>
     </row>
-    <row r="200" ht="24" customHeight="1">
-      <c r="B200" s="87" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
-      <c r="C200" s="82" t="n"/>
+    <row r="200" ht="32" customHeight="1">
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C200" s="86" t="n"/>
       <c r="D200" s="82" t="n"/>
       <c r="E200" s="82" t="n"/>
       <c r="F200" s="71" t="n"/>
     </row>
-    <row r="201" ht="58" customHeight="1">
-      <c r="B201" s="86" t="n"/>
-      <c r="C201" s="82" t="n"/>
+    <row r="201" ht="32" customHeight="1">
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C201" s="86" t="n"/>
       <c r="D201" s="82" t="n"/>
       <c r="E201" s="82" t="n"/>
       <c r="F201" s="71" t="n"/>
     </row>
     <row r="202" ht="32" customHeight="1">
-      <c r="B202" s="91" t="inlineStr">
-        <is>
-          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
-        </is>
-      </c>
-      <c r="C202" s="90" t="n"/>
-      <c r="D202" s="90" t="n"/>
-      <c r="E202" s="90" t="n"/>
-      <c r="F202" s="74" t="n"/>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C202" s="86" t="n"/>
+      <c r="D202" s="82" t="n"/>
+      <c r="E202" s="82" t="n"/>
+      <c r="F202" s="71" t="n"/>
     </row>
     <row r="203" ht="24" customHeight="1">
       <c r="B203" s="87" t="inlineStr">
         <is>
-          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
+          <t>Improvement opportunities — behaviors to improve</t>
         </is>
       </c>
       <c r="C203" s="82" t="n"/>
@@ -5734,27 +5785,35 @@
       <c r="E203" s="82" t="n"/>
       <c r="F203" s="71" t="n"/>
     </row>
-    <row r="204" ht="58" customHeight="1">
-      <c r="B204" s="86" t="n"/>
-      <c r="C204" s="82" t="n"/>
+    <row r="204" ht="32" customHeight="1">
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C204" s="86" t="n"/>
       <c r="D204" s="82" t="n"/>
       <c r="E204" s="82" t="n"/>
       <c r="F204" s="71" t="n"/>
     </row>
-    <row r="205" ht="24" customHeight="1">
-      <c r="B205" s="87" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
-      <c r="C205" s="82" t="n"/>
+    <row r="205" ht="32" customHeight="1">
+      <c r="B205" s="7" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C205" s="86" t="n"/>
       <c r="D205" s="82" t="n"/>
       <c r="E205" s="82" t="n"/>
       <c r="F205" s="71" t="n"/>
     </row>
-    <row r="206" ht="58" customHeight="1">
-      <c r="B206" s="86" t="n"/>
-      <c r="C206" s="82" t="n"/>
+    <row r="206" ht="32" customHeight="1">
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C206" s="86" t="n"/>
       <c r="D206" s="82" t="n"/>
       <c r="E206" s="82" t="n"/>
       <c r="F206" s="71" t="n"/>
@@ -5762,7 +5821,7 @@
     <row r="207" ht="24" customHeight="1">
       <c r="B207" s="87" t="inlineStr">
         <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
         </is>
       </c>
       <c r="C207" s="82" t="n"/>
@@ -5777,195 +5836,300 @@
       <c r="E208" s="82" t="n"/>
       <c r="F208" s="71" t="n"/>
     </row>
-    <row r="209"/>
-    <row r="210"/>
+    <row r="209" ht="20" customHeight="1">
+      <c r="B209" s="87" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
+      <c r="C209" s="82" t="n"/>
+      <c r="D209" s="82" t="n"/>
+      <c r="E209" s="82" t="n"/>
+      <c r="F209" s="71" t="n"/>
+    </row>
+    <row r="210" ht="28" customHeight="1">
+      <c r="B210" s="86" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="28" customHeight="1">
+      <c r="B211" s="86" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="28" customHeight="1">
+      <c r="B212" s="86" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="32" customHeight="1">
+      <c r="B213" s="91" t="inlineStr">
+        <is>
+          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
+        </is>
+      </c>
+      <c r="C213" s="90" t="n"/>
+      <c r="D213" s="90" t="n"/>
+      <c r="E213" s="90" t="n"/>
+      <c r="F213" s="74" t="n"/>
+    </row>
+    <row r="214" ht="24" customHeight="1">
+      <c r="B214" s="87" t="inlineStr">
+        <is>
+          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
+        </is>
+      </c>
+      <c r="C214" s="82" t="n"/>
+      <c r="D214" s="82" t="n"/>
+      <c r="E214" s="82" t="n"/>
+      <c r="F214" s="71" t="n"/>
+    </row>
+    <row r="215" ht="58" customHeight="1">
+      <c r="B215" s="86" t="n"/>
+      <c r="C215" s="82" t="n"/>
+      <c r="D215" s="82" t="n"/>
+      <c r="E215" s="82" t="n"/>
+      <c r="F215" s="71" t="n"/>
+    </row>
+    <row r="216" ht="24" customHeight="1">
+      <c r="B216" s="87" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
+      <c r="C216" s="82" t="n"/>
+      <c r="D216" s="82" t="n"/>
+      <c r="E216" s="82" t="n"/>
+      <c r="F216" s="71" t="n"/>
+    </row>
+    <row r="217" ht="58" customHeight="1">
+      <c r="B217" s="86" t="n"/>
+      <c r="C217" s="82" t="n"/>
+      <c r="D217" s="82" t="n"/>
+      <c r="E217" s="82" t="n"/>
+      <c r="F217" s="71" t="n"/>
+    </row>
+    <row r="218" ht="24" customHeight="1">
+      <c r="B218" s="87" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
+      <c r="C218" s="82" t="n"/>
+      <c r="D218" s="82" t="n"/>
+      <c r="E218" s="82" t="n"/>
+      <c r="F218" s="71" t="n"/>
+    </row>
+    <row r="219" ht="58" customHeight="1">
+      <c r="B219" s="86" t="n"/>
+      <c r="C219" s="82" t="n"/>
+      <c r="D219" s="82" t="n"/>
+      <c r="E219" s="82" t="n"/>
+      <c r="F219" s="71" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="185">
+  <mergeCells count="195">
+    <mergeCell ref="D189:F189"/>
     <mergeCell ref="D76:F76"/>
-    <mergeCell ref="B200:F200"/>
-    <mergeCell ref="D116:F116"/>
     <mergeCell ref="B81:F81"/>
+    <mergeCell ref="B209:F209"/>
+    <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
-    <mergeCell ref="D179:F179"/>
     <mergeCell ref="D53:F53"/>
+    <mergeCell ref="D166:F166"/>
+    <mergeCell ref="B131:F131"/>
+    <mergeCell ref="B214:F214"/>
+    <mergeCell ref="B36:E36"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="C186:F186"/>
-    <mergeCell ref="B36:E36"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="D181:F181"/>
-    <mergeCell ref="C136:F136"/>
     <mergeCell ref="C78:F78"/>
+    <mergeCell ref="E153:F153"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
-    <mergeCell ref="C146:D146"/>
+    <mergeCell ref="B195:F195"/>
+    <mergeCell ref="D168:F168"/>
+    <mergeCell ref="C210:F210"/>
+    <mergeCell ref="D165:F165"/>
     <mergeCell ref="C62:F62"/>
-    <mergeCell ref="D165:F165"/>
-    <mergeCell ref="B109:E109"/>
     <mergeCell ref="D92:F92"/>
     <mergeCell ref="D152:F152"/>
     <mergeCell ref="D39:F39"/>
     <mergeCell ref="C107:F107"/>
     <mergeCell ref="B44:F44"/>
-    <mergeCell ref="D129:F129"/>
+    <mergeCell ref="D133:F133"/>
+    <mergeCell ref="D142:F142"/>
     <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B168:F168"/>
-    <mergeCell ref="C121:F121"/>
-    <mergeCell ref="B118:F118"/>
+    <mergeCell ref="B108:F108"/>
+    <mergeCell ref="D191:F191"/>
+    <mergeCell ref="C212:F212"/>
+    <mergeCell ref="C173:F173"/>
     <mergeCell ref="D119:F119"/>
-    <mergeCell ref="D128:F128"/>
+    <mergeCell ref="D190:F190"/>
     <mergeCell ref="D159:F159"/>
-    <mergeCell ref="B133:F133"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="D186:F186"/>
+    <mergeCell ref="B213:F213"/>
     <mergeCell ref="D183:F183"/>
-    <mergeCell ref="E146:F146"/>
     <mergeCell ref="D105:F105"/>
+    <mergeCell ref="D170:F170"/>
     <mergeCell ref="D57:F57"/>
-    <mergeCell ref="D170:F170"/>
-    <mergeCell ref="B144:F144"/>
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="D154:F154"/>
     <mergeCell ref="D185:F185"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B125:F125"/>
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="D163:F163"/>
+    <mergeCell ref="C149:F149"/>
+    <mergeCell ref="B199:F199"/>
     <mergeCell ref="B64:E64"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="B208:F208"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="D162:F162"/>
-    <mergeCell ref="C199:F199"/>
     <mergeCell ref="D156:F156"/>
     <mergeCell ref="D171:F171"/>
     <mergeCell ref="D43:F43"/>
+    <mergeCell ref="B219:F219"/>
+    <mergeCell ref="B176:F176"/>
     <mergeCell ref="D106:F106"/>
+    <mergeCell ref="D137:F137"/>
+    <mergeCell ref="B111:F111"/>
     <mergeCell ref="D93:F93"/>
     <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D130:F130"/>
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
     <mergeCell ref="C14:F14"/>
-    <mergeCell ref="D117:F117"/>
+    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="D188:F188"/>
+    <mergeCell ref="D55:F55"/>
     <mergeCell ref="D157:F157"/>
-    <mergeCell ref="B148:F148"/>
-    <mergeCell ref="D55:F55"/>
     <mergeCell ref="D67:F67"/>
+    <mergeCell ref="C200:F200"/>
     <mergeCell ref="D132:F132"/>
     <mergeCell ref="D85:F85"/>
     <mergeCell ref="D54:F54"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="C147:F147"/>
+    <mergeCell ref="B146:F146"/>
+    <mergeCell ref="B217:F217"/>
     <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D182:F182"/>
+    <mergeCell ref="D100:F100"/>
     <mergeCell ref="D69:F69"/>
-    <mergeCell ref="D100:F100"/>
-    <mergeCell ref="D182:F182"/>
-    <mergeCell ref="D174:F174"/>
+    <mergeCell ref="B109:C110"/>
+    <mergeCell ref="C202:F202"/>
+    <mergeCell ref="C211:F211"/>
     <mergeCell ref="E16:F16"/>
+    <mergeCell ref="D158:F158"/>
+    <mergeCell ref="C201:F201"/>
+    <mergeCell ref="D40:F40"/>
     <mergeCell ref="D46:F46"/>
-    <mergeCell ref="B124:F124"/>
-    <mergeCell ref="D158:F158"/>
+    <mergeCell ref="B116:E116"/>
     <mergeCell ref="B207:F207"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="B189:F189"/>
-    <mergeCell ref="D111:F111"/>
-    <mergeCell ref="B204:F204"/>
+    <mergeCell ref="C148:F148"/>
+    <mergeCell ref="B198:F198"/>
+    <mergeCell ref="B216:F216"/>
     <mergeCell ref="D86:F86"/>
-    <mergeCell ref="C194:F194"/>
-    <mergeCell ref="B188:F188"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="D160:F160"/>
     <mergeCell ref="B75:F75"/>
-    <mergeCell ref="D150:F150"/>
-    <mergeCell ref="D145:F145"/>
+    <mergeCell ref="B218:F218"/>
+    <mergeCell ref="D136:F136"/>
     <mergeCell ref="B59:F59"/>
-    <mergeCell ref="B202:F202"/>
-    <mergeCell ref="B190:F190"/>
+    <mergeCell ref="B215:F215"/>
     <mergeCell ref="B80:E80"/>
     <mergeCell ref="D87:F87"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
+    <mergeCell ref="D122:F122"/>
     <mergeCell ref="D184:F184"/>
     <mergeCell ref="D71:F71"/>
     <mergeCell ref="D58:F58"/>
-    <mergeCell ref="C166:F166"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="D121:F121"/>
     <mergeCell ref="D177:F177"/>
-    <mergeCell ref="C141:F141"/>
+    <mergeCell ref="D192:F192"/>
     <mergeCell ref="D73:F73"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="D51:F51"/>
     <mergeCell ref="D42:F42"/>
     <mergeCell ref="D164:F164"/>
-    <mergeCell ref="D113:F113"/>
-    <mergeCell ref="B191:F191"/>
-    <mergeCell ref="D173:F173"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="C128:F128"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C113:F113"/>
+    <mergeCell ref="D123:F123"/>
     <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C143:F143"/>
+    <mergeCell ref="C112:F112"/>
+    <mergeCell ref="C205:F205"/>
     <mergeCell ref="C94:F94"/>
-    <mergeCell ref="D115:F115"/>
     <mergeCell ref="C47:F47"/>
+    <mergeCell ref="D138:F138"/>
     <mergeCell ref="D178:F178"/>
     <mergeCell ref="D172:F172"/>
+    <mergeCell ref="D187:F187"/>
+    <mergeCell ref="D99:F99"/>
+    <mergeCell ref="B65:F65"/>
     <mergeCell ref="C193:F193"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="C142:F142"/>
-    <mergeCell ref="B192:F192"/>
-    <mergeCell ref="D99:F99"/>
-    <mergeCell ref="B201:F201"/>
+    <mergeCell ref="C114:F114"/>
     <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B139:F139"/>
     <mergeCell ref="D84:F84"/>
-    <mergeCell ref="D155:F155"/>
-    <mergeCell ref="D149:F149"/>
+    <mergeCell ref="D45:F45"/>
     <mergeCell ref="D101:F101"/>
-    <mergeCell ref="B206:F206"/>
-    <mergeCell ref="D45:F45"/>
+    <mergeCell ref="D124:F124"/>
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B110:F110"/>
+    <mergeCell ref="B203:F203"/>
     <mergeCell ref="D77:F77"/>
-    <mergeCell ref="B203:F203"/>
     <mergeCell ref="B91:F91"/>
-    <mergeCell ref="D151:F151"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="D126:F126"/>
+    <mergeCell ref="D141:F141"/>
     <mergeCell ref="D70:F70"/>
     <mergeCell ref="D135:F135"/>
-    <mergeCell ref="D175:F175"/>
+    <mergeCell ref="B140:F140"/>
+    <mergeCell ref="B155:F155"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="E17:F17"/>
-    <mergeCell ref="D125:F125"/>
-    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="B97:F97"/>
     <mergeCell ref="D134:F134"/>
     <mergeCell ref="D72:F72"/>
-    <mergeCell ref="C140:F140"/>
-    <mergeCell ref="D112:F112"/>
+    <mergeCell ref="D103:F103"/>
+    <mergeCell ref="B117:F117"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D180:F180"/>
+    <mergeCell ref="B151:F151"/>
+    <mergeCell ref="D118:F118"/>
     <mergeCell ref="D56:F56"/>
-    <mergeCell ref="C195:F195"/>
     <mergeCell ref="D127:F127"/>
+    <mergeCell ref="D167:F167"/>
+    <mergeCell ref="C204:F204"/>
     <mergeCell ref="D161:F161"/>
-    <mergeCell ref="D176:F176"/>
-    <mergeCell ref="D114:F114"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D89:F89"/>
     <mergeCell ref="D98:F98"/>
-    <mergeCell ref="D89:F89"/>
-    <mergeCell ref="C197:F197"/>
+    <mergeCell ref="D169:F169"/>
+    <mergeCell ref="C206:F206"/>
     <mergeCell ref="B196:F196"/>
     <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B205:F205"/>
+    <mergeCell ref="B35:F35"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="D88:F88"/>
-    <mergeCell ref="D153:F153"/>
+    <mergeCell ref="C153:D153"/>
     <mergeCell ref="D90:F90"/>
     <mergeCell ref="B24:F24"/>
-    <mergeCell ref="C198:F198"/>
     <mergeCell ref="B104:F104"/>
-    <mergeCell ref="B169:F169"/>
-    <mergeCell ref="D131:F131"/>
+    <mergeCell ref="D139:F139"/>
     <mergeCell ref="D52:F52"/>
-    <mergeCell ref="B97:F97"/>
-    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B197:F197"/>
   </mergeCells>
   <conditionalFormatting sqref="C20:C24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
@@ -6166,13 +6330,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C39 C40 C41 C42 C43 C52 C53 C54 C55 C56 C57 C58 C67 C68 C69 C70 C71 C72 C73 C74 C83 C84 C85 C86 C87 C88 C89 C90 C99 C100 C101 C102 C103 C112 C113 C114 C115 C116 C117 C126 C127 C128 C129 C130 C131 C132" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C39 C40 C41 C42 C43 C52 C53 C54 C55 C56 C57 C58 C67 C68 C69 C70 C71 C72 C73 C74 C83 C84 C85 C86 C87 C88 C89 C90 C99 C100 C101 C102 C103 C119 C120 C121 C122 C123 C124 C133 C134 C135 C136 C137 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C46 C61 C77 C93 C106 C120 C135" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
+    <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C145 C150:C165 C175:C185 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C152 C157:C172 C182:C192 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6187,16 +6351,16 @@
     <dataValidation sqref="E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Within SLA,Breached,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Successful Resolution,Partial Resolution,Appropriate Escalation,Ownership Gap,Unresolved"</formula1>
     </dataValidation>
-    <dataValidation sqref="C141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_xlfn._LONGTEXT("Issue resolved,Proper RMA initiated (in-warranty / approved exception),Valid escalation submitted,Known limitation explained accurately,Customer educated with actionable next steps,Valid self-help guidance provided (out-of-warranty),Upgrade path recommend","ed appropriately (out-of-warranty),Customer declined further troubleshooting after reasonable effort,None achieved")</formula1>
     </dataValidation>
-    <dataValidation sqref="C146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C171:C173" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C178:C180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
     </dataValidation>
   </dataValidations>
@@ -12528,13 +12692,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Clarify overlapping communication indicators in scoring form
- Row 74 (Communication & Call Control): sharpen to 'Communication
  delivery adjusted for the customer's accessibility needs (hearing,
  vision, language barrier, age, cognitive)' — focuses on overcoming
  barriers to participation
- Row 121 (Customer Experience): sharpen to 'Communication style matched
  the customer's tone, pace, and language level' — focuses on style
  calibration to the customer's knowledge and personality

The two indicators now measure distinct things: one is accommodation
of a limitation, the other is stylistic matching.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -3229,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F219"/>
+  <dimension ref="B1:F219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4191,7 +4191,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="B74" s="83" t="inlineStr">
         <is>
-          <t>Communication adapted to the customer's accessibility needs (hearing, vision, age)</t>
+          <t>Communication delivery adjusted for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
         </is>
       </c>
       <c r="C74" s="9" t="n"/>
@@ -4735,7 +4735,7 @@
     <row r="121" ht="28" customHeight="1">
       <c r="B121" s="81" t="inlineStr">
         <is>
-          <t>Communication style was adapted to the customer</t>
+          <t>Communication style matched the customer's tone, pace, and language level</t>
         </is>
       </c>
       <c r="C121" s="9" t="n"/>
@@ -5941,12 +5941,12 @@
     <mergeCell ref="B209:F209"/>
     <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
+    <mergeCell ref="B131:F131"/>
+    <mergeCell ref="D166:F166"/>
     <mergeCell ref="D53:F53"/>
-    <mergeCell ref="D166:F166"/>
-    <mergeCell ref="B131:F131"/>
     <mergeCell ref="B214:F214"/>
+    <mergeCell ref="E8:F8"/>
     <mergeCell ref="B36:E36"/>
-    <mergeCell ref="E8:F8"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="D181:F181"/>
     <mergeCell ref="C78:F78"/>
@@ -5956,8 +5956,8 @@
     <mergeCell ref="B195:F195"/>
     <mergeCell ref="D168:F168"/>
     <mergeCell ref="C210:F210"/>
+    <mergeCell ref="C62:F62"/>
     <mergeCell ref="D165:F165"/>
-    <mergeCell ref="C62:F62"/>
     <mergeCell ref="D92:F92"/>
     <mergeCell ref="D152:F152"/>
     <mergeCell ref="D39:F39"/>
@@ -5981,11 +5981,11 @@
     <mergeCell ref="D170:F170"/>
     <mergeCell ref="D57:F57"/>
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="D120:F120"/>
     <mergeCell ref="D185:F185"/>
-    <mergeCell ref="D120:F120"/>
     <mergeCell ref="B49:E49"/>
+    <mergeCell ref="D41:F41"/>
     <mergeCell ref="B125:F125"/>
-    <mergeCell ref="D41:F41"/>
     <mergeCell ref="D163:F163"/>
     <mergeCell ref="C149:F149"/>
     <mergeCell ref="B199:F199"/>
@@ -6006,8 +6006,8 @@
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
+    <mergeCell ref="B175:F175"/>
     <mergeCell ref="C14:F14"/>
-    <mergeCell ref="B175:F175"/>
     <mergeCell ref="D188:F188"/>
     <mergeCell ref="D55:F55"/>
     <mergeCell ref="D157:F157"/>
@@ -6028,15 +6028,15 @@
     <mergeCell ref="C202:F202"/>
     <mergeCell ref="C211:F211"/>
     <mergeCell ref="E16:F16"/>
+    <mergeCell ref="D46:F46"/>
     <mergeCell ref="D158:F158"/>
     <mergeCell ref="C201:F201"/>
     <mergeCell ref="D40:F40"/>
-    <mergeCell ref="D46:F46"/>
     <mergeCell ref="B116:E116"/>
     <mergeCell ref="B207:F207"/>
     <mergeCell ref="C148:F148"/>
+    <mergeCell ref="B216:F216"/>
     <mergeCell ref="B198:F198"/>
-    <mergeCell ref="B216:F216"/>
     <mergeCell ref="D86:F86"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="D160:F160"/>
@@ -6058,12 +6058,12 @@
     <mergeCell ref="D177:F177"/>
     <mergeCell ref="D192:F192"/>
     <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D82:F82"/>
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D82:F82"/>
     <mergeCell ref="D164:F164"/>
+    <mergeCell ref="E6:F6"/>
     <mergeCell ref="C128:F128"/>
-    <mergeCell ref="E6:F6"/>
     <mergeCell ref="C113:F113"/>
     <mergeCell ref="D123:F123"/>
     <mergeCell ref="C20:F20"/>
@@ -6076,9 +6076,9 @@
     <mergeCell ref="D178:F178"/>
     <mergeCell ref="D172:F172"/>
     <mergeCell ref="D187:F187"/>
-    <mergeCell ref="D99:F99"/>
     <mergeCell ref="B65:F65"/>
     <mergeCell ref="C193:F193"/>
+    <mergeCell ref="D99:F99"/>
     <mergeCell ref="C114:F114"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D84:F84"/>
@@ -6098,10 +6098,9 @@
     <mergeCell ref="B155:F155"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="E17:F17"/>
-    <mergeCell ref="B97:F97"/>
-    <mergeCell ref="D134:F134"/>
     <mergeCell ref="D72:F72"/>
     <mergeCell ref="D103:F103"/>
+    <mergeCell ref="D134:F134"/>
     <mergeCell ref="B117:F117"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D180:F180"/>
@@ -6117,10 +6116,9 @@
     <mergeCell ref="D89:F89"/>
     <mergeCell ref="D98:F98"/>
     <mergeCell ref="D169:F169"/>
+    <mergeCell ref="B196:F196"/>
     <mergeCell ref="C206:F206"/>
-    <mergeCell ref="B196:F196"/>
     <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B35:F35"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="D88:F88"/>
     <mergeCell ref="C153:D153"/>
@@ -6130,6 +6128,8 @@
     <mergeCell ref="D139:F139"/>
     <mergeCell ref="D52:F52"/>
     <mergeCell ref="B197:F197"/>
+    <mergeCell ref="B97:F97"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
   <conditionalFormatting sqref="C20:C24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
@@ -12692,13 +12692,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Remove 5 duplicate Critical Failure Conditions already covered by Auto-Zero
§6 had 16 conditions; 5 were exact duplicates of §8 Auto-Zero items:
- Compliance/security violation (PCI)  ← §8 gate + item J
- Line release                          ← §8 item H
- Call/session avoidance or evasion    ← §8 item B
- Hard-selling / sales irregularity    ← §8 gate + item G
- Unofficial email / failed to capture ← §8 item E

§6 now has 11 unique coaching/conduct conditions not covered elsewhere.
All cross-section formulas (E33, F33, C168, C188) and DVs updated to
reflect the new row positions and reduced §6 range (C157:C167).

Also add Agent-A/B/C-Coaching-Report.md source files.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -3229,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F219"/>
+  <dimension ref="A1:F219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3712,11 +3712,11 @@
       </c>
       <c r="D33" s="27" t="n"/>
       <c r="E33" s="28">
-        <f>IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),0,SUM(E26:E32))</f>
+        <f>IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),0,SUM(E26:E32))</f>
         <v/>
       </c>
       <c r="F33" s="29">
-        <f>IF(E33="","",IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E33&gt;=0.85,"MEETS / EXCEEDS",IF(E33&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
+        <f>IF(E33="","",IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E33&gt;=0.85,"MEETS / EXCEEDS",IF(E33&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
         <v/>
       </c>
     </row>
@@ -5264,9 +5264,9 @@
       <c r="F164" s="71" t="n"/>
     </row>
     <row r="165" ht="26" customHeight="1">
-      <c r="B165" s="81" t="inlineStr">
-        <is>
-          <t>Compliance / security violation (e.g., payment card data spoken or stored in plaintext — PCI DSS)</t>
+      <c r="B165" s="83" t="inlineStr">
+        <is>
+          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
         </is>
       </c>
       <c r="C165" s="9" t="inlineStr">
@@ -5274,14 +5274,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D165" s="81" t="n"/>
+      <c r="D165" s="83" t="n"/>
       <c r="E165" s="82" t="n"/>
       <c r="F165" s="71" t="n"/>
     </row>
     <row r="166" ht="26" customHeight="1">
-      <c r="B166" s="83" t="inlineStr">
-        <is>
-          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
+      <c r="B166" s="81" t="inlineStr">
+        <is>
+          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
         </is>
       </c>
       <c r="C166" s="9" t="inlineStr">
@@ -5289,14 +5289,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D166" s="83" t="n"/>
+      <c r="D166" s="81" t="n"/>
       <c r="E166" s="82" t="n"/>
       <c r="F166" s="71" t="n"/>
     </row>
     <row r="167" ht="26" customHeight="1">
       <c r="B167" s="81" t="inlineStr">
         <is>
-          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
+          <t>Survey / CSAT manipulation</t>
         </is>
       </c>
       <c r="C167" s="9" t="inlineStr">
@@ -5309,149 +5309,153 @@
       <c r="F167" s="71" t="n"/>
     </row>
     <row r="168" ht="26" customHeight="1">
-      <c r="B168" s="81" t="inlineStr">
-        <is>
-          <t>Line release — agent ended a live, unresolved contact</t>
-        </is>
-      </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D168" s="81" t="n"/>
-      <c r="E168" s="82" t="n"/>
-      <c r="F168" s="71" t="n"/>
-    </row>
-    <row r="169" ht="26" customHeight="1">
-      <c r="B169" s="81" t="inlineStr">
-        <is>
-          <t>Call / session avoidance or evasion</t>
-        </is>
-      </c>
-      <c r="C169" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D169" s="81" t="n"/>
-      <c r="E169" s="82" t="n"/>
-      <c r="F169" s="71" t="n"/>
-    </row>
-    <row r="170" ht="26" customHeight="1">
-      <c r="B170" s="81" t="inlineStr">
-        <is>
-          <t>Survey / CSAT manipulation</t>
-        </is>
-      </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D170" s="81" t="n"/>
-      <c r="E170" s="82" t="n"/>
-      <c r="F170" s="71" t="n"/>
-    </row>
-    <row r="171" ht="26" customHeight="1">
-      <c r="B171" s="81" t="inlineStr">
-        <is>
-          <t>Hard-selling or other sales-related irregularity</t>
-        </is>
-      </c>
-      <c r="C171" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D171" s="81" t="n"/>
+      <c r="B168" s="98" t="inlineStr">
+        <is>
+          <t>CRITICAL FAILURE FLAGGED?</t>
+        </is>
+      </c>
+      <c r="C168" s="93">
+        <f>IF(COUNTIF(C157:C167,"Yes")&gt;0,"YES — "&amp;COUNTIF(C157:C167,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
+        <v/>
+      </c>
+      <c r="D168" s="90" t="n"/>
+      <c r="E168" s="90" t="n"/>
+      <c r="F168" s="74" t="n"/>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="B169" s="96" t="n"/>
+      <c r="C169" s="119" t="n"/>
+      <c r="D169" s="80" t="n"/>
+    </row>
+    <row r="170" ht="22" customHeight="1">
+      <c r="B170" s="98" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
+      <c r="C170" s="90" t="n"/>
+      <c r="D170" s="90" t="n"/>
+      <c r="E170" s="90" t="n"/>
+      <c r="F170" s="74" t="n"/>
+    </row>
+    <row r="171" ht="30" customHeight="1">
+      <c r="B171" s="85" t="inlineStr">
+        <is>
+          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
+        </is>
+      </c>
+      <c r="C171" s="82" t="n"/>
+      <c r="D171" s="82" t="n"/>
       <c r="E171" s="82" t="n"/>
       <c r="F171" s="71" t="n"/>
     </row>
-    <row r="172" ht="26" customHeight="1">
-      <c r="B172" s="81" t="inlineStr">
-        <is>
-          <t>Unofficial email used, or failed to capture customer email</t>
-        </is>
-      </c>
-      <c r="C172" s="9" t="inlineStr">
+    <row r="172" ht="30" customHeight="1">
+      <c r="B172" s="80" t="inlineStr">
+        <is>
+          <t>Compliance gate  (mark Yes if adhered)</t>
+        </is>
+      </c>
+      <c r="C172" s="119" t="inlineStr">
+        <is>
+          <t>Adherent?</t>
+        </is>
+      </c>
+      <c r="D172" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E172" s="90" t="n"/>
+      <c r="F172" s="74" t="n"/>
+    </row>
+    <row r="173" ht="26" customHeight="1">
+      <c r="B173" s="81" t="inlineStr">
+        <is>
+          <t>Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C173" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D173" s="81" t="n"/>
+      <c r="E173" s="82" t="n"/>
+      <c r="F173" s="71" t="n"/>
+    </row>
+    <row r="174" ht="26" customHeight="1">
+      <c r="B174" s="81" t="inlineStr">
+        <is>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C174" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D174" s="81" t="n"/>
+      <c r="E174" s="82" t="n"/>
+      <c r="F174" s="71" t="n"/>
+    </row>
+    <row r="175" ht="26" customHeight="1">
+      <c r="B175" s="81" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C175" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D175" s="81" t="n"/>
+      <c r="E175" s="82" t="n"/>
+      <c r="F175" s="71" t="n"/>
+    </row>
+    <row r="176" ht="32" customHeight="1">
+      <c r="B176" s="80" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
+        </is>
+      </c>
+      <c r="C176" s="119" t="inlineStr">
+        <is>
+          <t>Occurred?</t>
+        </is>
+      </c>
+      <c r="D176" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E176" s="90" t="n"/>
+      <c r="F176" s="74" t="n"/>
+    </row>
+    <row r="177" ht="26" customHeight="1">
+      <c r="B177" s="81" t="inlineStr">
+        <is>
+          <t>A.  Call / Session Abandonment</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D172" s="81" t="n"/>
-      <c r="E172" s="82" t="n"/>
-      <c r="F172" s="71" t="n"/>
-    </row>
-    <row r="173" ht="26" customHeight="1">
-      <c r="B173" s="98" t="inlineStr">
-        <is>
-          <t>CRITICAL FAILURE FLAGGED?</t>
-        </is>
-      </c>
-      <c r="C173" s="93">
-        <f>IF(COUNTIF(C157:C172,"Yes")&gt;0,"YES — "&amp;COUNTIF(C157:C172,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
-        <v/>
-      </c>
-      <c r="D173" s="90" t="n"/>
-      <c r="E173" s="90" t="n"/>
-      <c r="F173" s="74" t="n"/>
-    </row>
-    <row r="174" ht="20" customHeight="1">
-      <c r="B174" s="96" t="n"/>
-      <c r="C174" s="119" t="n"/>
-      <c r="D174" s="80" t="n"/>
-    </row>
-    <row r="175" ht="22" customHeight="1">
-      <c r="B175" s="98" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
-      <c r="C175" s="90" t="n"/>
-      <c r="D175" s="90" t="n"/>
-      <c r="E175" s="90" t="n"/>
-      <c r="F175" s="74" t="n"/>
-    </row>
-    <row r="176" ht="30" customHeight="1">
-      <c r="B176" s="85" t="inlineStr">
-        <is>
-          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
-        </is>
-      </c>
-      <c r="C176" s="82" t="n"/>
-      <c r="D176" s="82" t="n"/>
-      <c r="E176" s="82" t="n"/>
-      <c r="F176" s="71" t="n"/>
-    </row>
-    <row r="177" ht="30" customHeight="1">
-      <c r="B177" s="80" t="inlineStr">
-        <is>
-          <t>Compliance gate  (mark Yes if adhered)</t>
-        </is>
-      </c>
-      <c r="C177" s="119" t="inlineStr">
-        <is>
-          <t>Adherent?</t>
-        </is>
-      </c>
-      <c r="D177" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E177" s="90" t="n"/>
-      <c r="F177" s="74" t="n"/>
+      <c r="D177" s="81" t="n"/>
+      <c r="E177" s="82" t="n"/>
+      <c r="F177" s="71" t="n"/>
     </row>
     <row r="178" ht="26" customHeight="1">
       <c r="B178" s="81" t="inlineStr">
         <is>
-          <t>Adherence to Callback Hours</t>
+          <t>B.  Call / Session Avoidance / Evasion</t>
         </is>
       </c>
       <c r="C178" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D178" s="81" t="n"/>
@@ -5461,12 +5465,12 @@
     <row r="179" ht="26" customHeight="1">
       <c r="B179" s="81" t="inlineStr">
         <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
+          <t>C.  Discourtesy</t>
         </is>
       </c>
       <c r="C179" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D179" s="81" t="n"/>
@@ -5476,41 +5480,37 @@
     <row r="180" ht="26" customHeight="1">
       <c r="B180" s="81" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>D.  Escalation</t>
         </is>
       </c>
       <c r="C180" s="9" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D180" s="81" t="n"/>
       <c r="E180" s="82" t="n"/>
       <c r="F180" s="71" t="n"/>
     </row>
-    <row r="181" ht="32" customHeight="1">
-      <c r="B181" s="80" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
-        </is>
-      </c>
-      <c r="C181" s="119" t="inlineStr">
-        <is>
-          <t>Occurred?</t>
-        </is>
-      </c>
-      <c r="D181" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E181" s="90" t="n"/>
-      <c r="F181" s="74" t="n"/>
+    <row r="181" ht="26" customHeight="1">
+      <c r="B181" s="81" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D181" s="81" t="n"/>
+      <c r="E181" s="82" t="n"/>
+      <c r="F181" s="71" t="n"/>
     </row>
     <row r="182" ht="26" customHeight="1">
       <c r="B182" s="81" t="inlineStr">
         <is>
-          <t>A.  Call / Session Abandonment</t>
+          <t>F.  Fraud</t>
         </is>
       </c>
       <c r="C182" s="9" t="inlineStr">
@@ -5525,7 +5525,7 @@
     <row r="183" ht="26" customHeight="1">
       <c r="B183" s="81" t="inlineStr">
         <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
+          <t>G.  Hard-selling</t>
         </is>
       </c>
       <c r="C183" s="9" t="inlineStr">
@@ -5540,7 +5540,7 @@
     <row r="184" ht="26" customHeight="1">
       <c r="B184" s="81" t="inlineStr">
         <is>
-          <t>C.  Discourtesy</t>
+          <t>H.  Line Release</t>
         </is>
       </c>
       <c r="C184" s="9" t="inlineStr">
@@ -5555,7 +5555,7 @@
     <row r="185" ht="26" customHeight="1">
       <c r="B185" s="81" t="inlineStr">
         <is>
-          <t>D.  Escalation</t>
+          <t>I.  Non-Adherence to Callback Hours</t>
         </is>
       </c>
       <c r="C185" s="9" t="inlineStr">
@@ -5570,7 +5570,7 @@
     <row r="186" ht="26" customHeight="1">
       <c r="B186" s="81" t="inlineStr">
         <is>
-          <t>E.  Failure to ask for the email address</t>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
         </is>
       </c>
       <c r="C186" s="9" t="inlineStr">
@@ -5585,7 +5585,7 @@
     <row r="187" ht="26" customHeight="1">
       <c r="B187" s="81" t="inlineStr">
         <is>
-          <t>F.  Fraud</t>
+          <t>K.  Non-First Call Resolution</t>
         </is>
       </c>
       <c r="C187" s="9" t="inlineStr">
@@ -5597,146 +5597,127 @@
       <c r="E187" s="82" t="n"/>
       <c r="F187" s="71" t="n"/>
     </row>
-    <row r="188" ht="26" customHeight="1">
-      <c r="B188" s="81" t="inlineStr">
-        <is>
-          <t>G.  Hard-selling</t>
-        </is>
-      </c>
-      <c r="C188" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D188" s="81" t="n"/>
-      <c r="E188" s="82" t="n"/>
-      <c r="F188" s="71" t="n"/>
-    </row>
-    <row r="189" ht="26" customHeight="1">
-      <c r="B189" s="81" t="inlineStr">
-        <is>
-          <t>H.  Line Release</t>
-        </is>
-      </c>
-      <c r="C189" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+    <row r="188" ht="24" customHeight="1">
+      <c r="B188" s="98" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO TRIGGERED?</t>
+        </is>
+      </c>
+      <c r="C188" s="93">
+        <f>IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
+      <c r="D188" s="90" t="n"/>
+      <c r="E188" s="90" t="n"/>
+      <c r="F188" s="74" t="n"/>
+    </row>
+    <row r="189" ht="58" customHeight="1">
+      <c r="B189" s="86" t="n"/>
+      <c r="C189" s="86" t="n"/>
       <c r="D189" s="81" t="n"/>
-      <c r="E189" s="82" t="n"/>
-      <c r="F189" s="71" t="n"/>
-    </row>
-    <row r="190" ht="26" customHeight="1">
-      <c r="B190" s="81" t="inlineStr">
-        <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C190" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D190" s="81" t="n"/>
-      <c r="E190" s="82" t="n"/>
-      <c r="F190" s="71" t="n"/>
-    </row>
-    <row r="191" ht="26" customHeight="1">
-      <c r="B191" s="81" t="inlineStr">
-        <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C191" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D191" s="81" t="n"/>
-      <c r="E191" s="82" t="n"/>
-      <c r="F191" s="71" t="n"/>
-    </row>
-    <row r="192" ht="26" customHeight="1">
-      <c r="B192" s="81" t="inlineStr">
-        <is>
-          <t>K.  Non-First Call Resolution</t>
-        </is>
-      </c>
-      <c r="C192" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D192" s="81" t="n"/>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="B190" s="96" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
+        </is>
+      </c>
+      <c r="C190" s="90" t="n"/>
+      <c r="D190" s="90" t="n"/>
+      <c r="E190" s="90" t="n"/>
+      <c r="F190" s="74" t="n"/>
+    </row>
+    <row r="191" ht="30" customHeight="1">
+      <c r="B191" s="91" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+        </is>
+      </c>
+      <c r="C191" s="90" t="n"/>
+      <c r="D191" s="90" t="n"/>
+      <c r="E191" s="90" t="n"/>
+      <c r="F191" s="74" t="n"/>
+    </row>
+    <row r="192" ht="58" customHeight="1">
+      <c r="B192" s="86" t="n"/>
+      <c r="C192" s="82" t="n"/>
+      <c r="D192" s="82" t="n"/>
       <c r="E192" s="82" t="n"/>
       <c r="F192" s="71" t="n"/>
     </row>
-    <row r="193" ht="24" customHeight="1">
-      <c r="B193" s="98" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO TRIGGERED?</t>
-        </is>
-      </c>
-      <c r="C193" s="93">
-        <f>IF(OR(C178="No",C179="No",C180="No",COUNTIF(C182:C192,"Yes")&gt;0,COUNTIF(C157:C172,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
+    <row r="193" ht="30" customHeight="1">
+      <c r="B193" s="91" t="inlineStr">
+        <is>
+          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
+        </is>
+      </c>
+      <c r="C193" s="90" t="n"/>
       <c r="D193" s="90" t="n"/>
       <c r="E193" s="90" t="n"/>
       <c r="F193" s="74" t="n"/>
     </row>
-    <row r="194" ht="58" customHeight="1">
-      <c r="B194" s="86" t="n"/>
-      <c r="C194" s="86" t="n"/>
-    </row>
-    <row r="195" ht="20" customHeight="1">
-      <c r="B195" s="96" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
-        </is>
-      </c>
-      <c r="C195" s="90" t="n"/>
-      <c r="D195" s="90" t="n"/>
-      <c r="E195" s="90" t="n"/>
-      <c r="F195" s="74" t="n"/>
-    </row>
-    <row r="196" ht="30" customHeight="1">
-      <c r="B196" s="91" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
-        </is>
-      </c>
-      <c r="C196" s="90" t="n"/>
-      <c r="D196" s="90" t="n"/>
-      <c r="E196" s="90" t="n"/>
-      <c r="F196" s="74" t="n"/>
-    </row>
-    <row r="197" ht="58" customHeight="1">
-      <c r="B197" s="86" t="n"/>
-      <c r="C197" s="82" t="n"/>
+    <row r="194" ht="24" customHeight="1">
+      <c r="B194" s="87" t="inlineStr">
+        <is>
+          <t>What went well — behaviors to repeat</t>
+        </is>
+      </c>
+      <c r="C194" s="82" t="n"/>
+      <c r="D194" s="82" t="n"/>
+      <c r="E194" s="82" t="n"/>
+      <c r="F194" s="71" t="n"/>
+    </row>
+    <row r="195" ht="32" customHeight="1">
+      <c r="B195" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C195" s="86" t="n"/>
+      <c r="D195" s="82" t="n"/>
+      <c r="E195" s="82" t="n"/>
+      <c r="F195" s="71" t="n"/>
+    </row>
+    <row r="196" ht="32" customHeight="1">
+      <c r="B196" s="7" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C196" s="86" t="n"/>
+      <c r="D196" s="82" t="n"/>
+      <c r="E196" s="82" t="n"/>
+      <c r="F196" s="71" t="n"/>
+    </row>
+    <row r="197" ht="32" customHeight="1">
+      <c r="B197" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C197" s="86" t="n"/>
       <c r="D197" s="82" t="n"/>
       <c r="E197" s="82" t="n"/>
       <c r="F197" s="71" t="n"/>
     </row>
-    <row r="198" ht="30" customHeight="1">
-      <c r="B198" s="91" t="inlineStr">
-        <is>
-          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
-        </is>
-      </c>
-      <c r="C198" s="90" t="n"/>
-      <c r="D198" s="90" t="n"/>
-      <c r="E198" s="90" t="n"/>
-      <c r="F198" s="74" t="n"/>
-    </row>
-    <row r="199" ht="24" customHeight="1">
-      <c r="B199" s="87" t="inlineStr">
-        <is>
-          <t>What went well — behaviors to repeat</t>
-        </is>
-      </c>
-      <c r="C199" s="82" t="n"/>
+    <row r="198" ht="24" customHeight="1">
+      <c r="B198" s="87" t="inlineStr">
+        <is>
+          <t>Improvement opportunities — behaviors to improve</t>
+        </is>
+      </c>
+      <c r="C198" s="82" t="n"/>
+      <c r="D198" s="82" t="n"/>
+      <c r="E198" s="82" t="n"/>
+      <c r="F198" s="71" t="n"/>
+    </row>
+    <row r="199" ht="32" customHeight="1">
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C199" s="86" t="n"/>
       <c r="D199" s="82" t="n"/>
       <c r="E199" s="82" t="n"/>
       <c r="F199" s="71" t="n"/>
@@ -5744,7 +5725,7 @@
     <row r="200" ht="32" customHeight="1">
       <c r="B200" s="7" t="inlineStr">
         <is>
-          <t>1.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="C200" s="86" t="n"/>
@@ -5755,7 +5736,7 @@
     <row r="201" ht="32" customHeight="1">
       <c r="B201" s="7" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>3.</t>
         </is>
       </c>
       <c r="C201" s="86" t="n"/>
@@ -5763,43 +5744,39 @@
       <c r="E201" s="82" t="n"/>
       <c r="F201" s="71" t="n"/>
     </row>
-    <row r="202" ht="32" customHeight="1">
-      <c r="B202" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C202" s="86" t="n"/>
+    <row r="202" ht="24" customHeight="1">
+      <c r="B202" s="87" t="inlineStr">
+        <is>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
+        </is>
+      </c>
+      <c r="C202" s="82" t="n"/>
       <c r="D202" s="82" t="n"/>
       <c r="E202" s="82" t="n"/>
       <c r="F202" s="71" t="n"/>
     </row>
-    <row r="203" ht="24" customHeight="1">
-      <c r="B203" s="87" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
+    <row r="203" ht="58" customHeight="1">
+      <c r="B203" s="86" t="n"/>
       <c r="C203" s="82" t="n"/>
       <c r="D203" s="82" t="n"/>
       <c r="E203" s="82" t="n"/>
       <c r="F203" s="71" t="n"/>
     </row>
-    <row r="204" ht="32" customHeight="1">
-      <c r="B204" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C204" s="86" t="n"/>
+    <row r="204" ht="20" customHeight="1">
+      <c r="B204" s="87" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
+      <c r="C204" s="82" t="n"/>
       <c r="D204" s="82" t="n"/>
       <c r="E204" s="82" t="n"/>
       <c r="F204" s="71" t="n"/>
     </row>
-    <row r="205" ht="32" customHeight="1">
-      <c r="B205" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
+    <row r="205" ht="28" customHeight="1">
+      <c r="B205" s="86" t="inlineStr">
+        <is>
+          <t>1.</t>
         </is>
       </c>
       <c r="C205" s="86" t="n"/>
@@ -5807,10 +5784,10 @@
       <c r="E205" s="82" t="n"/>
       <c r="F205" s="71" t="n"/>
     </row>
-    <row r="206" ht="32" customHeight="1">
-      <c r="B206" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
+    <row r="206" ht="28" customHeight="1">
+      <c r="B206" s="86" t="inlineStr">
+        <is>
+          <t>2.</t>
         </is>
       </c>
       <c r="C206" s="86" t="n"/>
@@ -5818,28 +5795,28 @@
       <c r="E206" s="82" t="n"/>
       <c r="F206" s="71" t="n"/>
     </row>
-    <row r="207" ht="24" customHeight="1">
-      <c r="B207" s="87" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
-      <c r="C207" s="82" t="n"/>
-      <c r="D207" s="82" t="n"/>
-      <c r="E207" s="82" t="n"/>
-      <c r="F207" s="71" t="n"/>
-    </row>
-    <row r="208" ht="58" customHeight="1">
-      <c r="B208" s="86" t="n"/>
-      <c r="C208" s="82" t="n"/>
-      <c r="D208" s="82" t="n"/>
-      <c r="E208" s="82" t="n"/>
-      <c r="F208" s="71" t="n"/>
-    </row>
-    <row r="209" ht="20" customHeight="1">
+    <row r="207" ht="28" customHeight="1">
+      <c r="B207" s="86" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="32" customHeight="1">
+      <c r="B208" s="91" t="inlineStr">
+        <is>
+          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
+        </is>
+      </c>
+      <c r="C208" s="90" t="n"/>
+      <c r="D208" s="90" t="n"/>
+      <c r="E208" s="90" t="n"/>
+      <c r="F208" s="74" t="n"/>
+    </row>
+    <row r="209" ht="24" customHeight="1">
       <c r="B209" s="87" t="inlineStr">
         <is>
-          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
         </is>
       </c>
       <c r="C209" s="82" t="n"/>
@@ -5847,44 +5824,44 @@
       <c r="E209" s="82" t="n"/>
       <c r="F209" s="71" t="n"/>
     </row>
-    <row r="210" ht="28" customHeight="1">
-      <c r="B210" s="86" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="211" ht="28" customHeight="1">
-      <c r="B211" s="86" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="212" ht="28" customHeight="1">
-      <c r="B212" s="86" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="213" ht="32" customHeight="1">
-      <c r="B213" s="91" t="inlineStr">
-        <is>
-          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
-        </is>
-      </c>
-      <c r="C213" s="90" t="n"/>
-      <c r="D213" s="90" t="n"/>
-      <c r="E213" s="90" t="n"/>
-      <c r="F213" s="74" t="n"/>
-    </row>
-    <row r="214" ht="24" customHeight="1">
-      <c r="B214" s="87" t="inlineStr">
-        <is>
-          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
-        </is>
-      </c>
+    <row r="210" ht="58" customHeight="1">
+      <c r="B210" s="86" t="n"/>
+      <c r="C210" s="82" t="n"/>
+      <c r="D210" s="82" t="n"/>
+      <c r="E210" s="82" t="n"/>
+      <c r="F210" s="71" t="n"/>
+    </row>
+    <row r="211" ht="24" customHeight="1">
+      <c r="B211" s="87" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
+      <c r="C211" s="82" t="n"/>
+      <c r="D211" s="82" t="n"/>
+      <c r="E211" s="82" t="n"/>
+      <c r="F211" s="71" t="n"/>
+    </row>
+    <row r="212" ht="58" customHeight="1">
+      <c r="B212" s="86" t="n"/>
+      <c r="C212" s="82" t="n"/>
+      <c r="D212" s="82" t="n"/>
+      <c r="E212" s="82" t="n"/>
+      <c r="F212" s="71" t="n"/>
+    </row>
+    <row r="213" ht="24" customHeight="1">
+      <c r="B213" s="87" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
+      <c r="C213" s="82" t="n"/>
+      <c r="D213" s="82" t="n"/>
+      <c r="E213" s="82" t="n"/>
+      <c r="F213" s="71" t="n"/>
+    </row>
+    <row r="214" ht="58" customHeight="1">
+      <c r="B214" s="86" t="n"/>
       <c r="C214" s="82" t="n"/>
       <c r="D214" s="82" t="n"/>
       <c r="E214" s="82" t="n"/>
@@ -5892,10 +5869,6 @@
     </row>
     <row r="215" ht="58" customHeight="1">
       <c r="B215" s="86" t="n"/>
-      <c r="C215" s="82" t="n"/>
-      <c r="D215" s="82" t="n"/>
-      <c r="E215" s="82" t="n"/>
-      <c r="F215" s="71" t="n"/>
     </row>
     <row r="216" ht="24" customHeight="1">
       <c r="B216" s="87" t="inlineStr">
@@ -5903,17 +5876,9 @@
           <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
         </is>
       </c>
-      <c r="C216" s="82" t="n"/>
-      <c r="D216" s="82" t="n"/>
-      <c r="E216" s="82" t="n"/>
-      <c r="F216" s="71" t="n"/>
     </row>
     <row r="217" ht="58" customHeight="1">
       <c r="B217" s="86" t="n"/>
-      <c r="C217" s="82" t="n"/>
-      <c r="D217" s="82" t="n"/>
-      <c r="E217" s="82" t="n"/>
-      <c r="F217" s="71" t="n"/>
     </row>
     <row r="218" ht="24" customHeight="1">
       <c r="B218" s="87" t="inlineStr">
@@ -5921,152 +5886,136 @@
           <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
         </is>
       </c>
-      <c r="C218" s="82" t="n"/>
-      <c r="D218" s="82" t="n"/>
-      <c r="E218" s="82" t="n"/>
-      <c r="F218" s="71" t="n"/>
     </row>
     <row r="219" ht="58" customHeight="1">
       <c r="B219" s="86" t="n"/>
-      <c r="C219" s="82" t="n"/>
-      <c r="D219" s="82" t="n"/>
-      <c r="E219" s="82" t="n"/>
-      <c r="F219" s="71" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="195">
-    <mergeCell ref="D189:F189"/>
+  <mergeCells count="190">
     <mergeCell ref="D76:F76"/>
+    <mergeCell ref="B194:F194"/>
     <mergeCell ref="B81:F81"/>
     <mergeCell ref="B209:F209"/>
     <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="D166:F166"/>
+    <mergeCell ref="B214:F214"/>
     <mergeCell ref="B131:F131"/>
-    <mergeCell ref="D166:F166"/>
     <mergeCell ref="D53:F53"/>
-    <mergeCell ref="B214:F214"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="B36:E36"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="D181:F181"/>
     <mergeCell ref="C78:F78"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="E153:F153"/>
-    <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
-    <mergeCell ref="B195:F195"/>
-    <mergeCell ref="D168:F168"/>
-    <mergeCell ref="C210:F210"/>
     <mergeCell ref="C62:F62"/>
     <mergeCell ref="D165:F165"/>
     <mergeCell ref="D92:F92"/>
+    <mergeCell ref="B170:F170"/>
+    <mergeCell ref="D39:F39"/>
     <mergeCell ref="D152:F152"/>
-    <mergeCell ref="D39:F39"/>
     <mergeCell ref="C107:F107"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="D133:F133"/>
     <mergeCell ref="D142:F142"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B108:F108"/>
-    <mergeCell ref="D191:F191"/>
-    <mergeCell ref="C212:F212"/>
-    <mergeCell ref="C173:F173"/>
     <mergeCell ref="D119:F119"/>
-    <mergeCell ref="D190:F190"/>
     <mergeCell ref="D159:F159"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="D186:F186"/>
     <mergeCell ref="B213:F213"/>
     <mergeCell ref="D183:F183"/>
     <mergeCell ref="D105:F105"/>
-    <mergeCell ref="D170:F170"/>
+    <mergeCell ref="C207:F207"/>
     <mergeCell ref="D57:F57"/>
     <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B49:E49"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="D185:F185"/>
-    <mergeCell ref="B49:E49"/>
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="B125:F125"/>
+    <mergeCell ref="C149:F149"/>
     <mergeCell ref="D163:F163"/>
-    <mergeCell ref="C149:F149"/>
-    <mergeCell ref="B199:F199"/>
     <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B208:F208"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="B208:F208"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="D162:F162"/>
+    <mergeCell ref="C199:F199"/>
+    <mergeCell ref="D43:F43"/>
     <mergeCell ref="D156:F156"/>
-    <mergeCell ref="D171:F171"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="B219:F219"/>
-    <mergeCell ref="B176:F176"/>
+    <mergeCell ref="D137:F137"/>
     <mergeCell ref="D106:F106"/>
-    <mergeCell ref="D137:F137"/>
+    <mergeCell ref="B210:F210"/>
     <mergeCell ref="B111:F111"/>
     <mergeCell ref="D93:F93"/>
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
-    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="D157:F157"/>
+    <mergeCell ref="D55:F55"/>
     <mergeCell ref="C14:F14"/>
-    <mergeCell ref="D188:F188"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D157:F157"/>
     <mergeCell ref="D67:F67"/>
+    <mergeCell ref="B171:F171"/>
     <mergeCell ref="C200:F200"/>
     <mergeCell ref="D132:F132"/>
     <mergeCell ref="D85:F85"/>
+    <mergeCell ref="C147:F147"/>
+    <mergeCell ref="B130:E130"/>
     <mergeCell ref="D54:F54"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="C147:F147"/>
     <mergeCell ref="B146:F146"/>
-    <mergeCell ref="B217:F217"/>
     <mergeCell ref="D60:F60"/>
     <mergeCell ref="D182:F182"/>
+    <mergeCell ref="D69:F69"/>
     <mergeCell ref="D100:F100"/>
-    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="D174:F174"/>
     <mergeCell ref="B109:C110"/>
-    <mergeCell ref="C202:F202"/>
-    <mergeCell ref="C211:F211"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D46:F46"/>
+    <mergeCell ref="C201:F201"/>
+    <mergeCell ref="C148:F148"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="D40:F40"/>
     <mergeCell ref="D158:F158"/>
-    <mergeCell ref="C201:F201"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B207:F207"/>
-    <mergeCell ref="C148:F148"/>
-    <mergeCell ref="B216:F216"/>
+    <mergeCell ref="B204:F204"/>
+    <mergeCell ref="C188:F188"/>
     <mergeCell ref="B198:F198"/>
     <mergeCell ref="D86:F86"/>
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B75:F75"/>
     <mergeCell ref="D160:F160"/>
-    <mergeCell ref="B75:F75"/>
-    <mergeCell ref="B218:F218"/>
     <mergeCell ref="D136:F136"/>
     <mergeCell ref="B59:F59"/>
-    <mergeCell ref="B215:F215"/>
+    <mergeCell ref="B193:F193"/>
+    <mergeCell ref="B190:F190"/>
+    <mergeCell ref="B202:F202"/>
     <mergeCell ref="B80:E80"/>
     <mergeCell ref="D87:F87"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="D122:F122"/>
+    <mergeCell ref="D71:F71"/>
     <mergeCell ref="D184:F184"/>
-    <mergeCell ref="D71:F71"/>
     <mergeCell ref="D58:F58"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="D121:F121"/>
     <mergeCell ref="D177:F177"/>
-    <mergeCell ref="D192:F192"/>
     <mergeCell ref="D73:F73"/>
+    <mergeCell ref="D164:F164"/>
+    <mergeCell ref="D82:F82"/>
+    <mergeCell ref="D42:F42"/>
     <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D164:F164"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="D173:F173"/>
     <mergeCell ref="C128:F128"/>
+    <mergeCell ref="B191:F191"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="D123:F123"/>
     <mergeCell ref="C113:F113"/>
-    <mergeCell ref="D123:F123"/>
-    <mergeCell ref="C20:F20"/>
     <mergeCell ref="C143:F143"/>
     <mergeCell ref="C112:F112"/>
     <mergeCell ref="C205:F205"/>
@@ -6074,60 +6023,63 @@
     <mergeCell ref="C47:F47"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="D178:F178"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="D187:F187"/>
     <mergeCell ref="D172:F172"/>
-    <mergeCell ref="D187:F187"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="C193:F193"/>
     <mergeCell ref="D99:F99"/>
+    <mergeCell ref="B192:F192"/>
     <mergeCell ref="C114:F114"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D84:F84"/>
     <mergeCell ref="D45:F45"/>
+    <mergeCell ref="B212:F212"/>
     <mergeCell ref="D101:F101"/>
+    <mergeCell ref="B50:F50"/>
     <mergeCell ref="D124:F124"/>
-    <mergeCell ref="B50:F50"/>
     <mergeCell ref="B203:F203"/>
     <mergeCell ref="D77:F77"/>
     <mergeCell ref="B91:F91"/>
+    <mergeCell ref="D126:F126"/>
     <mergeCell ref="D61:F61"/>
-    <mergeCell ref="D126:F126"/>
     <mergeCell ref="D141:F141"/>
     <mergeCell ref="D70:F70"/>
     <mergeCell ref="D135:F135"/>
+    <mergeCell ref="D175:F175"/>
+    <mergeCell ref="B155:F155"/>
     <mergeCell ref="B140:F140"/>
-    <mergeCell ref="B155:F155"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="E17:F17"/>
+    <mergeCell ref="D103:F103"/>
     <mergeCell ref="D72:F72"/>
-    <mergeCell ref="D103:F103"/>
     <mergeCell ref="D134:F134"/>
     <mergeCell ref="B117:F117"/>
     <mergeCell ref="E10:F10"/>
+    <mergeCell ref="B151:F151"/>
     <mergeCell ref="D180:F180"/>
-    <mergeCell ref="B151:F151"/>
     <mergeCell ref="D118:F118"/>
+    <mergeCell ref="C195:F195"/>
     <mergeCell ref="D56:F56"/>
+    <mergeCell ref="D167:F167"/>
     <mergeCell ref="D127:F127"/>
-    <mergeCell ref="D167:F167"/>
-    <mergeCell ref="C204:F204"/>
     <mergeCell ref="D161:F161"/>
+    <mergeCell ref="D176:F176"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D98:F98"/>
     <mergeCell ref="D89:F89"/>
-    <mergeCell ref="D98:F98"/>
-    <mergeCell ref="D169:F169"/>
-    <mergeCell ref="B196:F196"/>
+    <mergeCell ref="C197:F197"/>
     <mergeCell ref="C206:F206"/>
     <mergeCell ref="B96:E96"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="D88:F88"/>
+    <mergeCell ref="C196:F196"/>
+    <mergeCell ref="C168:F168"/>
+    <mergeCell ref="B211:F211"/>
     <mergeCell ref="C153:D153"/>
     <mergeCell ref="D90:F90"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B104:F104"/>
     <mergeCell ref="D139:F139"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="B197:F197"/>
     <mergeCell ref="B97:F97"/>
     <mergeCell ref="B35:F35"/>
   </mergeCells>
@@ -6336,7 +6288,7 @@
     <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C152 C157:C172 C182:C192 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C152 C157:C167 C177:C187 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6360,7 +6312,7 @@
     <dataValidation sqref="C153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C178:C180" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C173:C175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
     </dataValidation>
   </dataValidations>
@@ -12692,13 +12644,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Implement team behavioral indicator proposals from comparison file
Applied changes from Behavior_Indicators_Comparison_Consolidated.xlsx:

§1 Resolution: 5 → 3 indicators (merged rows 6+7+8; refreshed wording)
§2 Technical: 7 → 4 indicators (merged 11+12, 14+15, 16+17; root cause
  moved to 2nd position per team request)
§3 Communication: minor rewrites on rows 68, 70, 72, 73, 74; rows 69
  and 71 kept unchanged (item 2 not implemented)
§4 Ownership: 8 → 5 active indicators (merged 30+31, 32+33, 36+37;
  rows 87+88 kept unchanged per item 3 not implemented)
§5 Escalation: 5 → 4 indicators (merged 42+43; removed redundant
  "for a valid reason" from row 99 per item 1 clarification)
§6 Customer Experience: 6 → 5 indicators (merged patience into professionalism)
§7 Documentation: 7 → 6 indicators (merged escalation justification
  into agent reasoning with expanded wording)

Behavioral indicator DV updated: 46 → 35 active cells

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -3229,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F219"/>
+  <dimension ref="B1:F219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3784,7 +3784,7 @@
     <row r="39" ht="28" customHeight="1">
       <c r="B39" s="81" t="inlineStr">
         <is>
-          <t>Issue resolved, or the strongest available outcome was achieved (RMA, valid escalation, limitation explained, education)</t>
+          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
         </is>
       </c>
       <c r="C39" s="9" t="n"/>
@@ -3795,7 +3795,7 @@
     <row r="40" ht="28" customHeight="1">
       <c r="B40" s="83" t="inlineStr">
         <is>
-          <t>Reasonable troubleshooting was completed before any conclusion was reached</t>
+          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
         </is>
       </c>
       <c r="C40" s="9" t="n"/>
@@ -3806,7 +3806,7 @@
     <row r="41" ht="28" customHeight="1">
       <c r="B41" s="81" t="inlineStr">
         <is>
-          <t>Clear, actionable next steps were provided to the customer</t>
+          <t>Used the appropriate resolution path for the situation and warranty status, moving the customer closer to a solution with clear next steps.</t>
         </is>
       </c>
       <c r="C41" s="9" t="n"/>
@@ -3815,22 +3815,14 @@
       <c r="F41" s="71" t="n"/>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="B42" s="83" t="inlineStr">
-        <is>
-          <t>Resolution path was appropriate for the situation and warranty status</t>
-        </is>
-      </c>
+      <c r="B42" s="83" t="n"/>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="83" t="n"/>
       <c r="E42" s="82" t="n"/>
       <c r="F42" s="71" t="n"/>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="B43" s="81" t="inlineStr">
-        <is>
-          <t>Customer was moved meaningfully closer to a solution</t>
-        </is>
-      </c>
+      <c r="B43" s="81" t="n"/>
       <c r="C43" s="9" t="n"/>
       <c r="D43" s="81" t="n"/>
       <c r="E43" s="82" t="n"/>
@@ -3937,7 +3929,7 @@
     <row r="52" ht="28" customHeight="1">
       <c r="B52" s="81" t="inlineStr">
         <is>
-          <t>Symptoms were identified correctly</t>
+          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
         </is>
       </c>
       <c r="C52" s="9" t="n"/>
@@ -3948,7 +3940,7 @@
     <row r="53" ht="28" customHeight="1">
       <c r="B53" s="83" t="inlineStr">
         <is>
-          <t>Relevant diagnostic questions were asked</t>
+          <t>Identified the root cause (or likely cause) when possible</t>
         </is>
       </c>
       <c r="C53" s="9" t="n"/>
@@ -3959,7 +3951,7 @@
     <row r="54" ht="28" customHeight="1">
       <c r="B54" s="81" t="inlineStr">
         <is>
-          <t>Logical troubleshooting methodology was followed</t>
+          <t>Followed a logical troubleshooting process, and available tools were used, efficiently and appropriately.</t>
         </is>
       </c>
       <c r="C54" s="9" t="n"/>
@@ -3968,11 +3960,7 @@
       <c r="F54" s="71" t="n"/>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="B55" s="83" t="inlineStr">
-        <is>
-          <t>Available tools were used appropriately</t>
-        </is>
-      </c>
+      <c r="B55" s="83" t="n"/>
       <c r="C55" s="9" t="n"/>
       <c r="D55" s="83" t="n"/>
       <c r="E55" s="82" t="n"/>
@@ -3981,7 +3969,7 @@
     <row r="56" ht="28" customHeight="1">
       <c r="B56" s="81" t="inlineStr">
         <is>
-          <t>Information provided was technically accurate</t>
+          <t>Gave technically accurate information; no unsupported conclusions</t>
         </is>
       </c>
       <c r="C56" s="9" t="n"/>
@@ -3990,22 +3978,14 @@
       <c r="F56" s="71" t="n"/>
     </row>
     <row r="57" ht="28" customHeight="1">
-      <c r="B57" s="83" t="inlineStr">
-        <is>
-          <t>Assumptions were validated; no unsupported conclusions</t>
-        </is>
-      </c>
+      <c r="B57" s="83" t="n"/>
       <c r="C57" s="9" t="n"/>
       <c r="D57" s="83" t="n"/>
       <c r="E57" s="82" t="n"/>
       <c r="F57" s="71" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="B58" s="81" t="inlineStr">
-        <is>
-          <t>Root cause (or likely cause) was identified when possible</t>
-        </is>
-      </c>
+      <c r="B58" s="81" t="n"/>
       <c r="C58" s="9" t="n"/>
       <c r="D58" s="81" t="n"/>
       <c r="E58" s="82" t="n"/>
@@ -4125,7 +4105,7 @@
     <row r="68" ht="28" customHeight="1">
       <c r="B68" s="83" t="inlineStr">
         <is>
-          <t>Agent maintained control of the troubleshooting flow</t>
+          <t>Agent maintained call control and troubleshooting flow</t>
         </is>
       </c>
       <c r="C68" s="9" t="n"/>
@@ -4147,7 +4127,7 @@
     <row r="70" ht="28" customHeight="1">
       <c r="B70" s="83" t="inlineStr">
         <is>
-          <t>Questions were purposeful (no repetitive questioning)</t>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
         </is>
       </c>
       <c r="C70" s="9" t="n"/>
@@ -4169,7 +4149,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="B72" s="83" t="inlineStr">
         <is>
-          <t>Clear transitions between troubleshooting steps; effective time management</t>
+          <t>Managed time well, with clear transitions between steps</t>
         </is>
       </c>
       <c r="C72" s="9" t="n"/>
@@ -4180,7 +4160,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="B73" s="81" t="inlineStr">
         <is>
-          <t>Difficult moments were managed professionally</t>
+          <t>Handled difficult moments when needed to maintain call control</t>
         </is>
       </c>
       <c r="C73" s="9" t="n"/>
@@ -4191,7 +4171,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="B74" s="83" t="inlineStr">
         <is>
-          <t>Communication delivery adjusted for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
         </is>
       </c>
       <c r="C74" s="9" t="n"/>
@@ -4302,7 +4282,7 @@
     <row r="83" ht="28" customHeight="1">
       <c r="B83" s="81" t="inlineStr">
         <is>
-          <t>Agent demonstrated accountability for the customer's outcome</t>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
         </is>
       </c>
       <c r="C83" s="9" t="n"/>
@@ -4311,11 +4291,7 @@
       <c r="F83" s="71" t="n"/>
     </row>
     <row r="84" ht="28" customHeight="1">
-      <c r="B84" s="83" t="inlineStr">
-        <is>
-          <t>Unnecessary transfers were avoided</t>
-        </is>
-      </c>
+      <c r="B84" s="83" t="n"/>
       <c r="C84" s="9" t="n"/>
       <c r="D84" s="83" t="n"/>
       <c r="E84" s="82" t="n"/>
@@ -4324,7 +4300,7 @@
     <row r="85" ht="28" customHeight="1">
       <c r="B85" s="81" t="inlineStr">
         <is>
-          <t>Commitments made during the interaction were followed through</t>
+          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
         </is>
       </c>
       <c r="C85" s="9" t="n"/>
@@ -4333,11 +4309,7 @@
       <c r="F85" s="71" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1">
-      <c r="B86" s="83" t="inlineStr">
-        <is>
-          <t>A clear path forward was created for the customer</t>
-        </is>
-      </c>
+      <c r="B86" s="83" t="n"/>
       <c r="C86" s="9" t="n"/>
       <c r="D86" s="83" t="n"/>
       <c r="E86" s="82" t="n"/>
@@ -4368,7 +4340,7 @@
     <row r="89" ht="28" customHeight="1">
       <c r="B89" s="81" t="inlineStr">
         <is>
-          <t>Disconnect follow-up completed (callback / email / note) — mark N.A. if no disconnect</t>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
         </is>
       </c>
       <c r="C89" s="9" t="n"/>
@@ -4377,11 +4349,7 @@
       <c r="F89" s="71" t="n"/>
     </row>
     <row r="90" ht="28" customHeight="1">
-      <c r="B90" s="83" t="inlineStr">
-        <is>
-          <t>Callback commitments were met within the agreed window (or proactively renegotiated before it lapsed)</t>
-        </is>
-      </c>
+      <c r="B90" s="83" t="n"/>
       <c r="C90" s="9" t="n"/>
       <c r="D90" s="83" t="n"/>
       <c r="E90" s="82" t="n"/>
@@ -4490,7 +4458,7 @@
     <row r="99" ht="28" customHeight="1">
       <c r="B99" s="81" t="inlineStr">
         <is>
-          <t>Reasonable troubleshooting was completed before escalating</t>
+          <t>Completed reasonable troubleshooting before escalating</t>
         </is>
       </c>
       <c r="C99" s="9" t="n"/>
@@ -4501,7 +4469,7 @@
     <row r="100" ht="28" customHeight="1">
       <c r="B100" s="83" t="inlineStr">
         <is>
-          <t>Legitimate escalation criteria were identified (incl. complaint / management / legal-risk triggers)</t>
+          <t>Identified a valid reason to escalate</t>
         </is>
       </c>
       <c r="C100" s="9" t="n"/>
@@ -4512,7 +4480,7 @@
     <row r="101" ht="28" customHeight="1">
       <c r="B101" s="81" t="inlineStr">
         <is>
-          <t>Escalation contained complete, useful details (logs, findings, steps tried)</t>
+          <t>Provided complete escalation details using the correct escalation path</t>
         </is>
       </c>
       <c r="C101" s="9" t="n"/>
@@ -4521,11 +4489,7 @@
       <c r="F101" s="71" t="n"/>
     </row>
     <row r="102" ht="28" customHeight="1">
-      <c r="B102" s="83" t="inlineStr">
-        <is>
-          <t>Correct escalation path was chosen</t>
-        </is>
-      </c>
+      <c r="B102" s="83" t="n"/>
       <c r="C102" s="9" t="n"/>
       <c r="D102" s="83" t="n"/>
       <c r="E102" s="82" t="n"/>
@@ -4534,7 +4498,7 @@
     <row r="103" ht="28" customHeight="1">
       <c r="B103" s="81" t="inlineStr">
         <is>
-          <t>Customer expectations about the escalation were set appropriately</t>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
         </is>
       </c>
       <c r="C103" s="9" t="n"/>
@@ -4713,7 +4677,7 @@
     <row r="119" ht="28" customHeight="1">
       <c r="B119" s="81" t="inlineStr">
         <is>
-          <t>Empathy was demonstrated (incl. acknowledging cumulative effort and fatigue on repeat contacts)</t>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
         </is>
       </c>
       <c r="C119" s="9" t="n"/>
@@ -4724,7 +4688,7 @@
     <row r="120" ht="28" customHeight="1">
       <c r="B120" s="83" t="inlineStr">
         <is>
-          <t>Professionalism was maintained throughout</t>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
         </is>
       </c>
       <c r="C120" s="9" t="n"/>
@@ -4735,7 +4699,7 @@
     <row r="121" ht="28" customHeight="1">
       <c r="B121" s="81" t="inlineStr">
         <is>
-          <t>Communication style matched the customer's tone, pace, and language level</t>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
         </is>
       </c>
       <c r="C121" s="9" t="n"/>
@@ -4744,11 +4708,7 @@
       <c r="F121" s="71" t="n"/>
     </row>
     <row r="122" ht="28" customHeight="1">
-      <c r="B122" s="83" t="inlineStr">
-        <is>
-          <t>Patience was maintained, even under pressure</t>
-        </is>
-      </c>
+      <c r="B122" s="83" t="n"/>
       <c r="C122" s="9" t="n"/>
       <c r="D122" s="83" t="n"/>
       <c r="E122" s="82" t="n"/>
@@ -4757,7 +4717,7 @@
     <row r="123" ht="28" customHeight="1">
       <c r="B123" s="81" t="inlineStr">
         <is>
-          <t>Customer effort was reduced where possible</t>
+          <t>Minimized customer effort</t>
         </is>
       </c>
       <c r="C123" s="9" t="n"/>
@@ -4768,7 +4728,7 @@
     <row r="124" ht="28" customHeight="1">
       <c r="B124" s="83" t="inlineStr">
         <is>
-          <t>Customer felt heard, understood next steps, and remained engaged</t>
+          <t>Maintained customer understanding and engagement</t>
         </is>
       </c>
       <c r="C124" s="9" t="n"/>
@@ -4879,7 +4839,7 @@
     <row r="133" ht="28" customHeight="1">
       <c r="B133" s="81" t="inlineStr">
         <is>
-          <t>Customer issue summary recorded</t>
+          <t>Recorded customer issue summary</t>
         </is>
       </c>
       <c r="C133" s="9" t="n"/>
@@ -4890,7 +4850,7 @@
     <row r="134" ht="28" customHeight="1">
       <c r="B134" s="83" t="inlineStr">
         <is>
-          <t>Troubleshooting performed is documented</t>
+          <t>Documented troubleshooting steps</t>
         </is>
       </c>
       <c r="C134" s="9" t="n"/>
@@ -4901,7 +4861,7 @@
     <row r="135" ht="28" customHeight="1">
       <c r="B135" s="81" t="inlineStr">
         <is>
-          <t>Key findings / discoveries noted</t>
+          <t>Noted key findings</t>
         </is>
       </c>
       <c r="C135" s="9" t="n"/>
@@ -4912,7 +4872,7 @@
     <row r="136" ht="28" customHeight="1">
       <c r="B136" s="83" t="inlineStr">
         <is>
-          <t>Agent reasoning is captured</t>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
         </is>
       </c>
       <c r="C136" s="9" t="n"/>
@@ -4921,11 +4881,7 @@
       <c r="F136" s="71" t="n"/>
     </row>
     <row r="137" ht="28" customHeight="1">
-      <c r="B137" s="81" t="inlineStr">
-        <is>
-          <t>Escalation justification included — mark N.A. if no escalation</t>
-        </is>
-      </c>
+      <c r="B137" s="81" t="n"/>
       <c r="C137" s="9" t="n"/>
       <c r="D137" s="81" t="n"/>
       <c r="E137" s="82" t="n"/>
@@ -4934,7 +4890,7 @@
     <row r="138" ht="28" customHeight="1">
       <c r="B138" s="83" t="inlineStr">
         <is>
-          <t>Next steps and follow-up actions listed (incl. callback records)</t>
+          <t>Documented next steps and follow-ups</t>
         </is>
       </c>
       <c r="C138" s="9" t="n"/>
@@ -4945,7 +4901,7 @@
     <row r="139" ht="28" customHeight="1">
       <c r="B139" s="81" t="inlineStr">
         <is>
-          <t>Ticket status accurately reflects case state (no premature RESOLVED; closure reason documented)</t>
+          <t>Updated ticket status accurately</t>
         </is>
       </c>
       <c r="C139" s="9" t="n"/>
@@ -5894,22 +5850,21 @@
   <mergeCells count="190">
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="B194:F194"/>
+    <mergeCell ref="B209:F209"/>
     <mergeCell ref="B81:F81"/>
-    <mergeCell ref="B209:F209"/>
     <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
-    <mergeCell ref="D52:F52"/>
     <mergeCell ref="D166:F166"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="B131:F131"/>
     <mergeCell ref="B214:F214"/>
-    <mergeCell ref="B131:F131"/>
-    <mergeCell ref="D53:F53"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="B36:E36"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="D181:F181"/>
     <mergeCell ref="C78:F78"/>
+    <mergeCell ref="E153:F153"/>
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="E153:F153"/>
     <mergeCell ref="D102:F102"/>
     <mergeCell ref="C62:F62"/>
     <mergeCell ref="D165:F165"/>
@@ -5938,11 +5893,11 @@
     <mergeCell ref="D185:F185"/>
     <mergeCell ref="D41:F41"/>
     <mergeCell ref="B125:F125"/>
+    <mergeCell ref="D163:F163"/>
     <mergeCell ref="C149:F149"/>
-    <mergeCell ref="D163:F163"/>
     <mergeCell ref="B64:E64"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="B208:F208"/>
-    <mergeCell ref="E5:F5"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="D162:F162"/>
     <mergeCell ref="C199:F199"/>
@@ -5956,9 +5911,9 @@
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
+    <mergeCell ref="C14:F14"/>
     <mergeCell ref="D157:F157"/>
     <mergeCell ref="D55:F55"/>
-    <mergeCell ref="C14:F14"/>
     <mergeCell ref="D67:F67"/>
     <mergeCell ref="B171:F171"/>
     <mergeCell ref="C200:F200"/>
@@ -5972,14 +5927,14 @@
     <mergeCell ref="D182:F182"/>
     <mergeCell ref="D69:F69"/>
     <mergeCell ref="D100:F100"/>
+    <mergeCell ref="B109:C110"/>
     <mergeCell ref="D174:F174"/>
-    <mergeCell ref="B109:C110"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D46:F46"/>
     <mergeCell ref="C201:F201"/>
+    <mergeCell ref="D40:F40"/>
     <mergeCell ref="C148:F148"/>
     <mergeCell ref="B116:E116"/>
-    <mergeCell ref="D40:F40"/>
     <mergeCell ref="D158:F158"/>
     <mergeCell ref="B204:F204"/>
     <mergeCell ref="C188:F188"/>
@@ -6006,13 +5961,13 @@
     <mergeCell ref="D177:F177"/>
     <mergeCell ref="D73:F73"/>
     <mergeCell ref="D164:F164"/>
+    <mergeCell ref="D42:F42"/>
     <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D42:F42"/>
     <mergeCell ref="D51:F51"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="D173:F173"/>
+    <mergeCell ref="B191:F191"/>
     <mergeCell ref="C128:F128"/>
-    <mergeCell ref="B191:F191"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="D123:F123"/>
     <mergeCell ref="C113:F113"/>
@@ -6023,9 +5978,9 @@
     <mergeCell ref="C47:F47"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="D178:F178"/>
+    <mergeCell ref="D172:F172"/>
+    <mergeCell ref="D187:F187"/>
     <mergeCell ref="B65:F65"/>
-    <mergeCell ref="D187:F187"/>
-    <mergeCell ref="D172:F172"/>
     <mergeCell ref="D99:F99"/>
     <mergeCell ref="B192:F192"/>
     <mergeCell ref="C114:F114"/>
@@ -6039,8 +5994,8 @@
     <mergeCell ref="B203:F203"/>
     <mergeCell ref="D77:F77"/>
     <mergeCell ref="B91:F91"/>
+    <mergeCell ref="D61:F61"/>
     <mergeCell ref="D126:F126"/>
-    <mergeCell ref="D61:F61"/>
     <mergeCell ref="D141:F141"/>
     <mergeCell ref="D70:F70"/>
     <mergeCell ref="D135:F135"/>
@@ -6054,11 +6009,11 @@
     <mergeCell ref="D134:F134"/>
     <mergeCell ref="B117:F117"/>
     <mergeCell ref="E10:F10"/>
+    <mergeCell ref="D180:F180"/>
     <mergeCell ref="B151:F151"/>
-    <mergeCell ref="D180:F180"/>
     <mergeCell ref="D118:F118"/>
+    <mergeCell ref="D56:F56"/>
     <mergeCell ref="C195:F195"/>
-    <mergeCell ref="D56:F56"/>
     <mergeCell ref="D167:F167"/>
     <mergeCell ref="D127:F127"/>
     <mergeCell ref="D161:F161"/>
@@ -6080,6 +6035,7 @@
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B104:F104"/>
     <mergeCell ref="D139:F139"/>
+    <mergeCell ref="D52:F52"/>
     <mergeCell ref="B97:F97"/>
     <mergeCell ref="B35:F35"/>
   </mergeCells>
@@ -6282,7 +6238,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C39 C40 C41 C42 C43 C52 C53 C54 C55 C56 C57 C58 C67 C68 C69 C70 C71 C72 C73 C74 C83 C84 C85 C86 C87 C88 C89 C90 C99 C100 C101 C102 C103 C119 C120 C121 C122 C123 C124 C133 C134 C135 C136 C137 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C39 C40 C41 C52 C53 C54 C56 C67 C68 C69 C70 C71 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
@@ -12644,13 +12600,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Implement item 2: merge Communication rows 69+71
Row 69: 'Use appropriate language, as needed, and confirmed customer
understanding' (merged from jargon-free language + confirming understanding)
Row 71: cleared — absorbed into row 69
Behavioral indicator DV: 35 → 34 active cells (C71 removed)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4116,7 +4116,7 @@
     <row r="69" ht="28" customHeight="1">
       <c r="B69" s="81" t="inlineStr">
         <is>
-          <t>Actions were explained in understandable, jargon-free language</t>
+          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
         </is>
       </c>
       <c r="C69" s="9" t="n"/>
@@ -4136,11 +4136,7 @@
       <c r="F70" s="71" t="n"/>
     </row>
     <row r="71" ht="28" customHeight="1">
-      <c r="B71" s="81" t="inlineStr">
-        <is>
-          <t>Customer understanding was confirmed at key points</t>
-        </is>
-      </c>
+      <c r="B71" s="81" t="n"/>
       <c r="C71" s="9" t="n"/>
       <c r="D71" s="81" t="n"/>
       <c r="E71" s="82" t="n"/>
@@ -5855,8 +5851,8 @@
     <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
     <mergeCell ref="D166:F166"/>
+    <mergeCell ref="B131:F131"/>
     <mergeCell ref="D53:F53"/>
-    <mergeCell ref="B131:F131"/>
     <mergeCell ref="B214:F214"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="B36:E36"/>
@@ -6238,7 +6234,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C39 C40 C41 C52 C53 C54 C56 C67 C68 C69 C70 C71 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C39 C40 C41 C52 C53 C54 C56 C67 C68 C69 C70 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
@@ -12600,13 +12596,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Split Resolution §1 merged indicator back into two distinct indicators
Row 41: 'Resolution path was appropriate for the situation and warranty status'
Row 42: 'Customer was moved meaningfully closer to a solution'

These measure different dimensions: row 41 evaluates the agent's
decision-making (was the chosen approach correct?), row 42 evaluates
the actual outcome (did the customer advance toward resolution?). A
correct path can still yield no progress; progress can still happen
via a suboptimal path. Keeping them separate makes both visible.

DV updated: 34 → 35 active cells (C42 restored)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -3806,7 +3806,7 @@
     <row r="41" ht="28" customHeight="1">
       <c r="B41" s="81" t="inlineStr">
         <is>
-          <t>Used the appropriate resolution path for the situation and warranty status, moving the customer closer to a solution with clear next steps.</t>
+          <t>Resolution path was appropriate for the situation and warranty status</t>
         </is>
       </c>
       <c r="C41" s="9" t="n"/>
@@ -3815,7 +3815,11 @@
       <c r="F41" s="71" t="n"/>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="B42" s="83" t="n"/>
+      <c r="B42" s="83" t="inlineStr">
+        <is>
+          <t>Customer was moved meaningfully closer to a solution</t>
+        </is>
+      </c>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="83" t="n"/>
       <c r="E42" s="82" t="n"/>
@@ -5851,8 +5855,8 @@
     <mergeCell ref="D179:F179"/>
     <mergeCell ref="D66:F66"/>
     <mergeCell ref="D166:F166"/>
+    <mergeCell ref="D53:F53"/>
     <mergeCell ref="B131:F131"/>
-    <mergeCell ref="D53:F53"/>
     <mergeCell ref="B214:F214"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="B36:E36"/>
@@ -6234,7 +6238,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C39 C40 C41 C52 C53 C54 C56 C67 C68 C69 C70 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C39 C40 C41 C42 C52 C53 C54 C56 C67 C68 C69 C70 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
@@ -12596,13 +12600,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Remove all blank rows from Scoring Form; compact to 187 rows
Removed 32 blank rows:
- Section separators between major sections (rows 3, 22, 23, 34, 48,
  63, 79, 95, 115, 129, 144, 145, 150, 154, 169, 189)
- Gaps left by previously merged behavioral indicators (rows 43, 55,
  57, 58, 71, 84, 86, 90, 102, 122, 137)
- Orphaned/duplicate rows at end of sheet (rows 215-219, incl. stale
  Multi-touch and Final Assessment duplicates at 216/218)

Kept 6 functional blank input rows:
- Row 93  – Escalation Follow-Up extended input (L2 action)
- Row 165 – §8 Q1 answer area
- Row 176 – Coaching recommendation input
- Row 183 – Org insights input
- Row 185 – Multi-touch notes input
- Row 187 – Final QA assessment input

All formulas, merges, DVs, and row heights remapped automatically via
row_map. Weighted total, auto-zero gate, critical failure flag, and
all auto-score COUNTIF ranges verified correct at new positions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -186,6 +186,7 @@
       <color rgb="FF1F3864"/>
       <sz val="11"/>
     </font>
+    <font/>
   </fonts>
   <fills count="13">
     <fill>
@@ -250,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -475,11 +476,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -834,6 +836,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3229,7 +3232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F219"/>
+  <dimension ref="B1:F187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3263,27 +3266,42 @@
       <c r="E2" s="90" t="n"/>
       <c r="F2" s="74" t="n"/>
     </row>
-    <row r="4">
-      <c r="B4" s="80" t="inlineStr">
+    <row r="3">
+      <c r="B3" s="80" t="inlineStr">
         <is>
           <t>1 · CASE INFORMATION</t>
         </is>
       </c>
-      <c r="C4" s="90" t="n"/>
-      <c r="D4" s="90" t="n"/>
-      <c r="E4" s="90" t="n"/>
-      <c r="F4" s="74" t="n"/>
+      <c r="C3" s="90" t="n"/>
+      <c r="D3" s="90" t="n"/>
+      <c r="E3" s="90" t="n"/>
+      <c r="F3" s="74" t="n"/>
+    </row>
+    <row r="4" ht="29" customHeight="1">
+      <c r="B4" s="94" t="inlineStr">
+        <is>
+          <t>Agent Name</t>
+        </is>
+      </c>
+      <c r="C4" s="88" t="n"/>
+      <c r="D4" s="87" t="inlineStr">
+        <is>
+          <t>Case / Ticket ID</t>
+        </is>
+      </c>
+      <c r="E4" s="88" t="n"/>
+      <c r="F4" s="71" t="n"/>
     </row>
     <row r="5" ht="29" customHeight="1">
       <c r="B5" s="94" t="inlineStr">
         <is>
-          <t>Agent Name</t>
+          <t>Evaluator (QA)</t>
         </is>
       </c>
       <c r="C5" s="88" t="n"/>
       <c r="D5" s="87" t="inlineStr">
         <is>
-          <t>Case / Ticket ID</t>
+          <t>Interaction Date</t>
         </is>
       </c>
       <c r="E5" s="88" t="n"/>
@@ -3292,13 +3310,13 @@
     <row r="6" ht="29" customHeight="1">
       <c r="B6" s="94" t="inlineStr">
         <is>
-          <t>Evaluator (QA)</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="C6" s="88" t="n"/>
       <c r="D6" s="87" t="inlineStr">
         <is>
-          <t>Interaction Date</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="E6" s="88" t="n"/>
@@ -3307,28 +3325,28 @@
     <row r="7">
       <c r="B7" s="94" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Warranty Status</t>
         </is>
       </c>
       <c r="C7" s="88" t="n"/>
       <c r="D7" s="87" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Review Date</t>
         </is>
       </c>
       <c r="E7" s="88" t="n"/>
       <c r="F7" s="71" t="n"/>
     </row>
-    <row r="8">
+    <row r="8" ht="29" customHeight="1">
       <c r="B8" s="94" t="inlineStr">
         <is>
-          <t>Warranty Status</t>
+          <t>Case Type</t>
         </is>
       </c>
       <c r="C8" s="88" t="n"/>
       <c r="D8" s="87" t="inlineStr">
         <is>
-          <t>Review Date</t>
+          <t>Interaction Duration</t>
         </is>
       </c>
       <c r="E8" s="88" t="n"/>
@@ -3337,13 +3355,13 @@
     <row r="9" ht="29" customHeight="1">
       <c r="B9" s="94" t="inlineStr">
         <is>
-          <t>Case Type</t>
+          <t>Touch # (multi-touch case)</t>
         </is>
       </c>
       <c r="C9" s="88" t="n"/>
       <c r="D9" s="87" t="inlineStr">
         <is>
-          <t>Interaction Duration</t>
+          <t>Prior touches reviewed?</t>
         </is>
       </c>
       <c r="E9" s="88" t="n"/>
@@ -3352,13 +3370,13 @@
     <row r="10" ht="29" customHeight="1">
       <c r="B10" s="94" t="inlineStr">
         <is>
-          <t>Touch # (multi-touch case)</t>
+          <t>CSAT / Survey result</t>
         </is>
       </c>
       <c r="C10" s="88" t="n"/>
       <c r="D10" s="87" t="inlineStr">
         <is>
-          <t>Prior touches reviewed?</t>
+          <t>FCR / total contacts</t>
         </is>
       </c>
       <c r="E10" s="88" t="n"/>
@@ -3367,37 +3385,33 @@
     <row r="11" ht="29" customHeight="1">
       <c r="B11" s="94" t="inlineStr">
         <is>
-          <t>CSAT / Survey result</t>
+          <t>Total case time</t>
         </is>
       </c>
       <c r="C11" s="88" t="n"/>
       <c r="D11" s="87" t="inlineStr">
         <is>
-          <t>FCR / total contacts</t>
+          <t>SLA status</t>
         </is>
       </c>
       <c r="E11" s="88" t="n"/>
       <c r="F11" s="71" t="n"/>
     </row>
-    <row r="12">
-      <c r="B12" s="94" t="inlineStr">
-        <is>
-          <t>Total case time</t>
-        </is>
-      </c>
-      <c r="C12" s="88" t="n"/>
-      <c r="D12" s="87" t="inlineStr">
-        <is>
-          <t>SLA status</t>
-        </is>
-      </c>
-      <c r="E12" s="88" t="n"/>
+    <row r="12" ht="58" customHeight="1">
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>Case Summary (customer issue &amp; goal)</t>
+        </is>
+      </c>
+      <c r="C12" s="86" t="n"/>
+      <c r="D12" s="82" t="n"/>
+      <c r="E12" s="82" t="n"/>
       <c r="F12" s="71" t="n"/>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="46" customHeight="1">
       <c r="B13" s="87" t="inlineStr">
         <is>
-          <t>Case Summary (customer issue &amp; goal)</t>
+          <t>Inherited context (what this agent received from prior touches)</t>
         </is>
       </c>
       <c r="C13" s="86" t="n"/>
@@ -3406,37 +3420,41 @@
       <c r="F13" s="71" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
-      <c r="B14" s="87" t="inlineStr">
-        <is>
-          <t>Inherited context (what this agent received from prior touches)</t>
-        </is>
-      </c>
-      <c r="C14" s="86" t="n"/>
-      <c r="D14" s="82" t="n"/>
-      <c r="E14" s="82" t="n"/>
-      <c r="F14" s="71" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="80" t="inlineStr">
+      <c r="B14" s="80" t="inlineStr">
         <is>
           <t>CLASSIFICATION &amp; ROOT-CAUSE   (added from the 360 Form model)</t>
         </is>
       </c>
-      <c r="C15" s="90" t="n"/>
-      <c r="D15" s="90" t="n"/>
-      <c r="E15" s="90" t="n"/>
-      <c r="F15" s="74" t="n"/>
-    </row>
-    <row r="16" ht="58" customHeight="1">
+      <c r="C14" s="90" t="n"/>
+      <c r="D14" s="90" t="n"/>
+      <c r="E14" s="90" t="n"/>
+      <c r="F14" s="74" t="n"/>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="B15" s="94" t="inlineStr">
+        <is>
+          <t>Audit / Review Type</t>
+        </is>
+      </c>
+      <c r="C15" s="88" t="n"/>
+      <c r="D15" s="87" t="inlineStr">
+        <is>
+          <t>Contact iteration (repeat contact)</t>
+        </is>
+      </c>
+      <c r="E15" s="88" t="n"/>
+      <c r="F15" s="71" t="n"/>
+    </row>
+    <row r="16" ht="29" customHeight="1">
       <c r="B16" s="94" t="inlineStr">
         <is>
-          <t>Audit / Review Type</t>
+          <t>Resolution status — detailed</t>
         </is>
       </c>
       <c r="C16" s="88" t="n"/>
       <c r="D16" s="87" t="inlineStr">
         <is>
-          <t>Contact iteration (repeat contact)</t>
+          <t>Primary root-cause domain</t>
         </is>
       </c>
       <c r="E16" s="88" t="n"/>
@@ -3445,22 +3463,18 @@
     <row r="17" ht="29" customHeight="1">
       <c r="B17" s="94" t="inlineStr">
         <is>
-          <t>Resolution status — detailed</t>
+          <t>Process driver (if any)</t>
         </is>
       </c>
       <c r="C17" s="88" t="n"/>
-      <c r="D17" s="87" t="inlineStr">
-        <is>
-          <t>Primary root-cause domain</t>
-        </is>
-      </c>
-      <c r="E17" s="88" t="n"/>
+      <c r="D17" s="82" t="n"/>
+      <c r="E17" s="82" t="n"/>
       <c r="F17" s="71" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="94" t="inlineStr">
         <is>
-          <t>Process driver (if any)</t>
+          <t>Product driver (if any)</t>
         </is>
       </c>
       <c r="C18" s="88" t="n"/>
@@ -3471,7 +3485,7 @@
     <row r="19">
       <c r="B19" s="94" t="inlineStr">
         <is>
-          <t>Product driver (if any)</t>
+          <t>System / tooling driver (if any)</t>
         </is>
       </c>
       <c r="C19" s="88" t="n"/>
@@ -3482,360 +3496,395 @@
     <row r="20">
       <c r="B20" s="94" t="inlineStr">
         <is>
-          <t>System / tooling driver (if any)</t>
-        </is>
-      </c>
-      <c r="C20" s="88" t="n"/>
+          <t>Root-cause / contact-driver notes   (feeds Team Scoring → Team Opportunities Identified)</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="n"/>
       <c r="D20" s="82" t="n"/>
       <c r="E20" s="82" t="n"/>
       <c r="F20" s="71" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="94" t="inlineStr">
-        <is>
-          <t>Root-cause / contact-driver notes   (feeds Team Scoring → Team Opportunities Identified)</t>
-        </is>
-      </c>
-      <c r="C21" s="82" t="n"/>
-      <c r="D21" s="82" t="n"/>
-      <c r="E21" s="82" t="n"/>
-      <c r="F21" s="71" t="n"/>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="B22" s="88" t="n"/>
-      <c r="C22" s="82" t="n"/>
-      <c r="D22" s="82" t="n"/>
-      <c r="E22" s="82" t="n"/>
-      <c r="F22" s="71" t="n"/>
+      <c r="B21" s="96" t="inlineStr">
+        <is>
+          <t>2 · SCORE SUMMARY</t>
+        </is>
+      </c>
+      <c r="C21" s="90" t="n"/>
+      <c r="D21" s="90" t="n"/>
+      <c r="E21" s="90" t="n"/>
+      <c r="F21" s="74" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="119" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C22" s="119" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="D22" s="119" t="inlineStr">
+        <is>
+          <t>Score (0-5)</t>
+        </is>
+      </c>
+      <c r="E22" s="119" t="inlineStr">
+        <is>
+          <t>Weighted</t>
+        </is>
+      </c>
+      <c r="F22" s="119" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Resolution / Progress Toward Resolution</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D23" s="18">
+        <f>IF(C41="",C40,C41)</f>
+        <v/>
+      </c>
+      <c r="E23" s="19">
+        <f>IF(D23="","",(D23/5)*C23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="20">
+        <f>IF(D23="","",IF(D23&gt;=4,"Strong",IF(D23=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
-      <c r="B24" s="96" t="inlineStr">
-        <is>
-          <t>2 · SCORE SUMMARY</t>
-        </is>
-      </c>
-      <c r="C24" s="90" t="n"/>
-      <c r="D24" s="90" t="n"/>
-      <c r="E24" s="90" t="n"/>
-      <c r="F24" s="74" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="119" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C25" s="119" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="D25" s="119" t="inlineStr">
-        <is>
-          <t>Score (0-5)</t>
-        </is>
-      </c>
-      <c r="E25" s="119" t="inlineStr">
-        <is>
-          <t>Weighted</t>
-        </is>
-      </c>
-      <c r="F25" s="119" t="inlineStr">
-        <is>
-          <t>Band</t>
-        </is>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Technical Accuracy</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D24" s="23">
+        <f>IF(C52="",C51,C52)</f>
+        <v/>
+      </c>
+      <c r="E24" s="24">
+        <f>IF(D24="","",(D24/5)*C24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="25">
+        <f>IF(D24="","",IF(D24&gt;=4,"Strong",IF(D24=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Communication &amp; Call Control</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D25" s="18">
+        <f>IF(C66="",C65,C66)</f>
+        <v/>
+      </c>
+      <c r="E25" s="19">
+        <f>IF(D25="","",(D25/5)*C25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="20">
+        <f>IF(D25="","",IF(D25&gt;=4,"Strong",IF(D25=3,"Developing","Needs Focus")))</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="B26" s="16" t="inlineStr">
-        <is>
-          <t>Resolution / Progress Toward Resolution</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D26" s="18">
-        <f>IF(C46="",C45,C46)</f>
-        <v/>
-      </c>
-      <c r="E26" s="19">
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Customer Ownership</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D26" s="23">
+        <f>IF(C78="",C77,C78)</f>
+        <v/>
+      </c>
+      <c r="E26" s="24">
         <f>IF(D26="","",(D26/5)*C26)</f>
         <v/>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="25">
         <f>IF(D26="","",IF(D26&gt;=4,"Strong",IF(D26=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="21" t="inlineStr">
-        <is>
-          <t>Technical Accuracy</t>
-        </is>
-      </c>
-      <c r="C27" s="22" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D27" s="23">
-        <f>IF(C61="",C60,C61)</f>
-        <v/>
-      </c>
-      <c r="E27" s="24">
+    <row r="27" ht="28" customHeight="1">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Escalation Judgment</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D27" s="18">
+        <f>IF(C89="",C88,C89)</f>
+        <v/>
+      </c>
+      <c r="E27" s="19">
         <f>IF(D27="","",(D27/5)*C27)</f>
         <v/>
       </c>
-      <c r="F27" s="25">
+      <c r="F27" s="20">
         <f>IF(D27="","",IF(D27&gt;=4,"Strong",IF(D27=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="B28" s="16" t="inlineStr">
-        <is>
-          <t>Communication &amp; Call Control</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D28" s="18">
-        <f>IF(C77="",C76,C77)</f>
-        <v/>
-      </c>
-      <c r="E28" s="19">
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>Customer Experience</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D28" s="23">
+        <f>IF(C108="",C107,C108)</f>
+        <v/>
+      </c>
+      <c r="E28" s="24">
         <f>IF(D28="","",(D28/5)*C28)</f>
         <v/>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="25">
         <f>IF(D28="","",IF(D28&gt;=4,"Strong",IF(D28=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>Customer Ownership</t>
-        </is>
-      </c>
-      <c r="C29" s="22" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D29" s="23">
-        <f>IF(C93="",C92,C93)</f>
-        <v/>
-      </c>
-      <c r="E29" s="24">
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>Documentation &amp; Notes</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D29" s="18">
+        <f>IF(C121="",C120,C121)</f>
+        <v/>
+      </c>
+      <c r="E29" s="19">
         <f>IF(D29="","",(D29/5)*C29)</f>
         <v/>
       </c>
-      <c r="F29" s="25">
+      <c r="F29" s="20">
         <f>IF(D29="","",IF(D29&gt;=4,"Strong",IF(D29=3,"Developing","Needs Focus")))</f>
         <v/>
       </c>
     </row>
-    <row r="30" ht="28" customHeight="1">
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>Escalation Judgment</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D30" s="18">
-        <f>IF(C106="",C105,C106)</f>
-        <v/>
-      </c>
-      <c r="E30" s="19">
-        <f>IF(D30="","",(D30/5)*C30)</f>
-        <v/>
-      </c>
-      <c r="F30" s="20">
-        <f>IF(D30="","",IF(D30&gt;=4,"Strong",IF(D30=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="21" t="inlineStr">
-        <is>
-          <t>Customer Experience</t>
-        </is>
-      </c>
-      <c r="C31" s="22" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D31" s="23">
-        <f>IF(C127="",C126,C127)</f>
-        <v/>
-      </c>
-      <c r="E31" s="24">
-        <f>IF(D31="","",(D31/5)*C31)</f>
-        <v/>
-      </c>
-      <c r="F31" s="25">
-        <f>IF(D31="","",IF(D31&gt;=4,"Strong",IF(D31=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>Documentation &amp; Notes</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D32" s="18">
-        <f>IF(C142="",C141,C142)</f>
-        <v/>
-      </c>
-      <c r="E32" s="19">
-        <f>IF(D32="","",(D32/5)*C32)</f>
-        <v/>
-      </c>
-      <c r="F32" s="20">
-        <f>IF(D32="","",IF(D32&gt;=4,"Strong",IF(D32=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="B33" s="96" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="B30" s="96" t="inlineStr">
         <is>
           <t>WEIGHTED TOTAL SCORE</t>
         </is>
       </c>
-      <c r="C33" s="26">
-        <f>SUM(C26:C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="27" t="n"/>
-      <c r="E33" s="28">
-        <f>IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),0,SUM(E26:E32))</f>
-        <v/>
-      </c>
-      <c r="F33" s="29">
-        <f>IF(E33="","",IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E33&gt;=0.85,"MEETS / EXCEEDS",IF(E33&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="12" t="n"/>
-      <c r="D34" s="92" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="B35" s="96" t="inlineStr">
+      <c r="C30" s="26">
+        <f>SUM(C23:C29)</f>
+        <v/>
+      </c>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="28">
+        <f>IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),0,SUM(E23:E29))</f>
+        <v/>
+      </c>
+      <c r="F30" s="29">
+        <f>IF(E30="","",IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E30&gt;=0.85,"MEETS / EXCEEDS",IF(E30&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="B31" s="96" t="inlineStr">
         <is>
           <t>3 · CATEGORY ASSESSMENTS</t>
         </is>
       </c>
-      <c r="C35" s="90" t="n"/>
-      <c r="D35" s="90" t="n"/>
-      <c r="E35" s="90" t="n"/>
-      <c r="F35" s="74" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="B36" s="80" t="inlineStr">
+      <c r="C31" s="90" t="n"/>
+      <c r="D31" s="90" t="n"/>
+      <c r="E31" s="90" t="n"/>
+      <c r="F31" s="74" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="B32" s="80" t="inlineStr">
         <is>
           <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
       </c>
-      <c r="C36" s="90" t="n"/>
-      <c r="D36" s="90" t="n"/>
-      <c r="E36" s="74" t="n"/>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="C32" s="90" t="n"/>
+      <c r="D32" s="90" t="n"/>
+      <c r="E32" s="74" t="n"/>
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Weight: 30%</t>
         </is>
       </c>
     </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="B33" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Determine whether the interaction moved the customer meaningfully closer to resolution.</t>
+        </is>
+      </c>
+      <c r="C33" s="82" t="n"/>
+      <c r="D33" s="82" t="n"/>
+      <c r="E33" s="82" t="n"/>
+      <c r="F33" s="71" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D34" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
+      <c r="E34" s="82" t="n"/>
+      <c r="F34" s="71" t="n"/>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="B35" s="81" t="inlineStr">
+        <is>
+          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="81" t="n"/>
+      <c r="E35" s="82" t="n"/>
+      <c r="F35" s="71" t="n"/>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="B36" s="83" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="83" t="n"/>
+      <c r="E36" s="82" t="n"/>
+      <c r="F36" s="71" t="n"/>
+    </row>
     <row r="37" ht="28" customHeight="1">
-      <c r="B37" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Determine whether the interaction moved the customer meaningfully closer to resolution.</t>
-        </is>
-      </c>
-      <c r="C37" s="82" t="n"/>
-      <c r="D37" s="82" t="n"/>
+      <c r="B37" s="81" t="inlineStr">
+        <is>
+          <t>Resolution path was appropriate for the situation and warranty status</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="81" t="n"/>
       <c r="E37" s="82" t="n"/>
       <c r="F37" s="71" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="B38" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D38" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+    <row r="38" ht="28" customHeight="1">
+      <c r="B38" s="83" t="inlineStr">
+        <is>
+          <t>Customer was moved meaningfully closer to a solution</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="83" t="n"/>
       <c r="E38" s="82" t="n"/>
       <c r="F38" s="71" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1">
-      <c r="B39" s="81" t="inlineStr">
-        <is>
-          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="81" t="n"/>
+      <c r="B39" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Does NOT count: customer simply ends call; generic KB sent without troubleshooting; warranty used as reason to stop helping; escalation as shortcut; unsupported ISP blame; 'monitor &amp; call back' with no plan; ownership transferred without expectations or documentation.</t>
+        </is>
+      </c>
+      <c r="C39" s="82" t="n"/>
+      <c r="D39" s="82" t="n"/>
       <c r="E39" s="82" t="n"/>
       <c r="F39" s="71" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
-      <c r="B40" s="83" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="n"/>
-      <c r="D40" s="83" t="n"/>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C40" s="122">
+        <f>IF((COUNTIF(C35:C38,"Met")+COUNTIF(C35:C38,"Partial")+COUNTIF(C35:C38,"Missed"))=0,"",ROUND((COUNTIF(C35:C38,"Met")*5+COUNTIF(C35:C38,"Partial")*2.5)/(COUNTIF(C35:C38,"Met")+COUNTIF(C35:C38,"Partial")+COUNTIF(C35:C38,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D40" s="92" t="n"/>
       <c r="E40" s="82" t="n"/>
       <c r="F40" s="71" t="n"/>
     </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="B41" s="81" t="inlineStr">
-        <is>
-          <t>Resolution path was appropriate for the situation and warranty status</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="n"/>
-      <c r="D41" s="81" t="n"/>
+    <row r="41" ht="24" customHeight="1">
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="84">
+        <f>IF(IF(C41="",C40,C41)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C41="",C40,C41)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E41" s="82" t="n"/>
       <c r="F41" s="71" t="n"/>
     </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="B42" s="83" t="inlineStr">
-        <is>
-          <t>Customer was moved meaningfully closer to a solution</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="83" t="n"/>
+    <row r="42" ht="36" customHeight="1">
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Score reflects the cumulative effect of this touch within the 8-month journey: the Nov 24, 2025 hardware/RMA determination remains undelivered, and the case culminates here in executive-level escalation with no path forward offered.</t>
+        </is>
+      </c>
+      <c r="C42" s="86" t="n"/>
+      <c r="D42" s="82" t="n"/>
       <c r="E42" s="82" t="n"/>
       <c r="F42" s="71" t="n"/>
     </row>
-    <row r="43" ht="28" customHeight="1">
-      <c r="B43" s="81" t="n"/>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="81" t="n"/>
-      <c r="E43" s="82" t="n"/>
-      <c r="F43" s="71" t="n"/>
+    <row r="43" ht="18" customHeight="1">
+      <c r="B43" s="80" t="inlineStr">
+        <is>
+          <t>2. TECHNICAL ACCURACY</t>
+        </is>
+      </c>
+      <c r="C43" s="90" t="n"/>
+      <c r="D43" s="90" t="n"/>
+      <c r="E43" s="74" t="n"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 20%</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="B44" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Does NOT count: customer simply ends call; generic KB sent without troubleshooting; warranty used as reason to stop helping; escalation as shortcut; unsupported ISP blame; 'monitor &amp; call back' with no plan; ownership transferred without expectations or documentation.</t>
+      <c r="B44" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Evaluate the quality of troubleshooting and technical guidance.</t>
         </is>
       </c>
       <c r="C44" s="82" t="n"/>
@@ -3843,67 +3892,73 @@
       <c r="E44" s="82" t="n"/>
       <c r="F44" s="71" t="n"/>
     </row>
-    <row r="45" ht="28" customHeight="1">
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C45" s="122">
-        <f>IF((COUNTIF(C39:C43,"Met")+COUNTIF(C39:C43,"Partial")+COUNTIF(C39:C43,"Missed"))=0,"",ROUND((COUNTIF(C39:C43,"Met")*5+COUNTIF(C39:C43,"Partial")*2.5)/(COUNTIF(C39:C43,"Met")+COUNTIF(C39:C43,"Partial")+COUNTIF(C39:C43,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D45" s="92" t="n"/>
+    <row r="45" ht="36" customHeight="1">
+      <c r="B45" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D45" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E45" s="82" t="n"/>
       <c r="F45" s="71" t="n"/>
     </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="84">
-        <f>IF(IF(C46="",C45,C46)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C46="",C45,C46)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="46" ht="28" customHeight="1">
+      <c r="B46" s="81" t="inlineStr">
+        <is>
+          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="81" t="n"/>
       <c r="E46" s="82" t="n"/>
       <c r="F46" s="71" t="n"/>
     </row>
-    <row r="47" ht="36" customHeight="1">
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>Score reflects the cumulative effect of this touch within the 8-month journey: the Nov 24, 2025 hardware/RMA determination remains undelivered, and the case culminates here in executive-level escalation with no path forward offered.</t>
-        </is>
-      </c>
-      <c r="C47" s="86" t="n"/>
-      <c r="D47" s="82" t="n"/>
+    <row r="47" ht="28" customHeight="1">
+      <c r="B47" s="83" t="inlineStr">
+        <is>
+          <t>Identified the root cause (or likely cause) when possible</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="83" t="n"/>
       <c r="E47" s="82" t="n"/>
       <c r="F47" s="71" t="n"/>
     </row>
     <row r="48" ht="28" customHeight="1">
-      <c r="B48" s="85" t="n"/>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="B49" s="80" t="inlineStr">
-        <is>
-          <t>2. TECHNICAL ACCURACY</t>
-        </is>
-      </c>
-      <c r="C49" s="90" t="n"/>
-      <c r="D49" s="90" t="n"/>
-      <c r="E49" s="74" t="n"/>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 20%</t>
-        </is>
-      </c>
+      <c r="B48" s="81" t="inlineStr">
+        <is>
+          <t>Followed a logical troubleshooting process, and available tools were used, efficiently and appropriately.</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="81" t="n"/>
+      <c r="E48" s="82" t="n"/>
+      <c r="F48" s="71" t="n"/>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="B49" s="81" t="inlineStr">
+        <is>
+          <t>Gave technically accurate information; no unsupported conclusions</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n"/>
+      <c r="D49" s="81" t="n"/>
+      <c r="E49" s="82" t="n"/>
+      <c r="F49" s="71" t="n"/>
     </row>
     <row r="50" ht="28" customHeight="1">
-      <c r="B50" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Evaluate the quality of troubleshooting and technical guidance.</t>
+      <c r="B50" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
         </is>
       </c>
       <c r="C50" s="82" t="n"/>
@@ -3911,256 +3966,288 @@
       <c r="E50" s="82" t="n"/>
       <c r="F50" s="71" t="n"/>
     </row>
-    <row r="51" ht="36" customHeight="1">
-      <c r="B51" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D51" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+    <row r="51" ht="28" customHeight="1">
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C51" s="122">
+        <f>IF((COUNTIF(C46:C49,"Met")+COUNTIF(C46:C49,"Partial")+COUNTIF(C46:C49,"Missed"))=0,"",ROUND((COUNTIF(C46:C49,"Met")*5+COUNTIF(C46:C49,"Partial")*2.5)/(COUNTIF(C46:C49,"Met")+COUNTIF(C46:C49,"Partial")+COUNTIF(C46:C49,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D51" s="92" t="n"/>
       <c r="E51" s="82" t="n"/>
       <c r="F51" s="71" t="n"/>
     </row>
-    <row r="52" ht="28" customHeight="1">
-      <c r="B52" s="81" t="inlineStr">
-        <is>
-          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="n"/>
-      <c r="D52" s="81" t="n"/>
+    <row r="52" ht="24" customHeight="1">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="84">
+        <f>IF(IF(C52="",C51,C52)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C52="",C51,C52)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E52" s="82" t="n"/>
       <c r="F52" s="71" t="n"/>
     </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="B53" s="83" t="inlineStr">
-        <is>
-          <t>Identified the root cause (or likely cause) when possible</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="83" t="n"/>
+    <row r="53" ht="36" customHeight="1">
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
+        </is>
+      </c>
+      <c r="C53" s="86" t="n"/>
+      <c r="D53" s="82" t="n"/>
       <c r="E53" s="82" t="n"/>
       <c r="F53" s="71" t="n"/>
     </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="B54" s="81" t="inlineStr">
-        <is>
-          <t>Followed a logical troubleshooting process, and available tools were used, efficiently and appropriately.</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="n"/>
-      <c r="D54" s="81" t="n"/>
-      <c r="E54" s="82" t="n"/>
-      <c r="F54" s="71" t="n"/>
+    <row r="54" ht="18" customHeight="1">
+      <c r="B54" s="80" t="inlineStr">
+        <is>
+          <t>3. COMMUNICATION &amp; CALL CONTROL</t>
+        </is>
+      </c>
+      <c r="C54" s="90" t="n"/>
+      <c r="D54" s="90" t="n"/>
+      <c r="E54" s="74" t="n"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 15%</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="B55" s="83" t="n"/>
-      <c r="C55" s="9" t="n"/>
-      <c r="D55" s="83" t="n"/>
+      <c r="B55" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Evaluate how effectively the agent managed the interaction.</t>
+        </is>
+      </c>
+      <c r="C55" s="82" t="n"/>
+      <c r="D55" s="82" t="n"/>
       <c r="E55" s="82" t="n"/>
       <c r="F55" s="71" t="n"/>
     </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="B56" s="81" t="inlineStr">
-        <is>
-          <t>Gave technically accurate information; no unsupported conclusions</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="n"/>
-      <c r="D56" s="81" t="n"/>
+    <row r="56" ht="24" customHeight="1">
+      <c r="B56" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D56" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E56" s="82" t="n"/>
       <c r="F56" s="71" t="n"/>
     </row>
     <row r="57" ht="28" customHeight="1">
-      <c r="B57" s="83" t="n"/>
+      <c r="B57" s="81" t="inlineStr">
+        <is>
+          <t>Expectations were set clearly from the start</t>
+        </is>
+      </c>
       <c r="C57" s="9" t="n"/>
-      <c r="D57" s="83" t="n"/>
+      <c r="D57" s="81" t="n"/>
       <c r="E57" s="82" t="n"/>
       <c r="F57" s="71" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="B58" s="81" t="n"/>
+      <c r="B58" s="83" t="inlineStr">
+        <is>
+          <t>Agent maintained call control and troubleshooting flow</t>
+        </is>
+      </c>
       <c r="C58" s="9" t="n"/>
-      <c r="D58" s="81" t="n"/>
+      <c r="D58" s="83" t="n"/>
       <c r="E58" s="82" t="n"/>
       <c r="F58" s="71" t="n"/>
     </row>
     <row r="59" ht="28" customHeight="1">
-      <c r="B59" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
-        </is>
-      </c>
-      <c r="C59" s="82" t="n"/>
-      <c r="D59" s="82" t="n"/>
+      <c r="B59" s="81" t="inlineStr">
+        <is>
+          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="n"/>
+      <c r="D59" s="81" t="n"/>
       <c r="E59" s="82" t="n"/>
       <c r="F59" s="71" t="n"/>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C60" s="122">
-        <f>IF((COUNTIF(C52:C58,"Met")+COUNTIF(C52:C58,"Partial")+COUNTIF(C52:C58,"Missed"))=0,"",ROUND((COUNTIF(C52:C58,"Met")*5+COUNTIF(C52:C58,"Partial")*2.5)/(COUNTIF(C52:C58,"Met")+COUNTIF(C52:C58,"Partial")+COUNTIF(C52:C58,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D60" s="92" t="n"/>
+      <c r="B60" s="83" t="inlineStr">
+        <is>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="n"/>
+      <c r="D60" s="83" t="n"/>
       <c r="E60" s="82" t="n"/>
       <c r="F60" s="71" t="n"/>
     </row>
-    <row r="61" ht="24" customHeight="1">
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C61" s="14" t="n"/>
-      <c r="D61" s="84">
-        <f>IF(IF(C61="",C60,C61)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C61="",C60,C61)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="61" ht="28" customHeight="1">
+      <c r="B61" s="83" t="inlineStr">
+        <is>
+          <t>Managed time well, with clear transitions between steps</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="n"/>
+      <c r="D61" s="83" t="n"/>
       <c r="E61" s="82" t="n"/>
       <c r="F61" s="71" t="n"/>
     </row>
-    <row r="62" ht="36" customHeight="1">
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
-        </is>
-      </c>
-      <c r="C62" s="86" t="n"/>
-      <c r="D62" s="82" t="n"/>
+    <row r="62" ht="28" customHeight="1">
+      <c r="B62" s="81" t="inlineStr">
+        <is>
+          <t>Handled difficult moments when needed to maintain call control</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="n"/>
+      <c r="D62" s="81" t="n"/>
       <c r="E62" s="82" t="n"/>
       <c r="F62" s="71" t="n"/>
     </row>
     <row r="63" ht="28" customHeight="1">
-      <c r="B63" s="83" t="n"/>
+      <c r="B63" s="83" t="inlineStr">
+        <is>
+          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+        </is>
+      </c>
       <c r="C63" s="9" t="n"/>
       <c r="D63" s="83" t="n"/>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="B64" s="80" t="inlineStr">
-        <is>
-          <t>3. COMMUNICATION &amp; CALL CONTROL</t>
-        </is>
-      </c>
-      <c r="C64" s="90" t="n"/>
-      <c r="D64" s="90" t="n"/>
-      <c r="E64" s="74" t="n"/>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 15%</t>
-        </is>
-      </c>
+      <c r="E63" s="82" t="n"/>
+      <c r="F63" s="71" t="n"/>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="B64" s="85" t="inlineStr">
+        <is>
+          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
+        </is>
+      </c>
+      <c r="C64" s="82" t="n"/>
+      <c r="D64" s="82" t="n"/>
+      <c r="E64" s="82" t="n"/>
+      <c r="F64" s="71" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="B65" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Evaluate how effectively the agent managed the interaction.</t>
-        </is>
-      </c>
-      <c r="C65" s="82" t="n"/>
-      <c r="D65" s="82" t="n"/>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C65" s="122">
+        <f>IF((COUNTIF(C57:C63,"Met")+COUNTIF(C57:C63,"Partial")+COUNTIF(C57:C63,"Missed"))=0,"",ROUND((COUNTIF(C57:C63,"Met")*5+COUNTIF(C57:C63,"Partial")*2.5)/(COUNTIF(C57:C63,"Met")+COUNTIF(C57:C63,"Partial")+COUNTIF(C57:C63,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D65" s="92" t="n"/>
       <c r="E65" s="82" t="n"/>
       <c r="F65" s="71" t="n"/>
     </row>
     <row r="66" ht="24" customHeight="1">
-      <c r="B66" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D66" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C66" s="14" t="n"/>
+      <c r="D66" s="84">
+        <f>IF(IF(C66="",C65,C66)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C66="",C65,C66)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
       </c>
       <c r="E66" s="82" t="n"/>
       <c r="F66" s="71" t="n"/>
     </row>
-    <row r="67" ht="28" customHeight="1">
-      <c r="B67" s="81" t="inlineStr">
-        <is>
-          <t>Expectations were set clearly from the start</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="n"/>
-      <c r="D67" s="81" t="n"/>
+    <row r="67" ht="36" customHeight="1">
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
+        </is>
+      </c>
+      <c r="C67" s="86" t="n"/>
+      <c r="D67" s="82" t="n"/>
       <c r="E67" s="82" t="n"/>
       <c r="F67" s="71" t="n"/>
     </row>
-    <row r="68" ht="28" customHeight="1">
-      <c r="B68" s="83" t="inlineStr">
-        <is>
-          <t>Agent maintained call control and troubleshooting flow</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="n"/>
-      <c r="D68" s="83" t="n"/>
-      <c r="E68" s="82" t="n"/>
-      <c r="F68" s="71" t="n"/>
+    <row r="68" ht="18" customHeight="1">
+      <c r="B68" s="80" t="inlineStr">
+        <is>
+          <t>4. CUSTOMER OWNERSHIP</t>
+        </is>
+      </c>
+      <c r="C68" s="90" t="n"/>
+      <c r="D68" s="90" t="n"/>
+      <c r="E68" s="74" t="n"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 15%</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="28" customHeight="1">
-      <c r="B69" s="81" t="inlineStr">
-        <is>
-          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="n"/>
-      <c r="D69" s="81" t="n"/>
+      <c r="B69" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Measure the degree to which the agent accepted responsibility for moving the customer forward.</t>
+        </is>
+      </c>
+      <c r="C69" s="82" t="n"/>
+      <c r="D69" s="82" t="n"/>
       <c r="E69" s="82" t="n"/>
       <c r="F69" s="71" t="n"/>
     </row>
-    <row r="70" ht="28" customHeight="1">
-      <c r="B70" s="83" t="inlineStr">
-        <is>
-          <t>Actively listened and showed comprehension throughout the interaction/s</t>
-        </is>
-      </c>
-      <c r="C70" s="9" t="n"/>
-      <c r="D70" s="83" t="n"/>
+    <row r="70" ht="24" customHeight="1">
+      <c r="B70" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D70" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E70" s="82" t="n"/>
       <c r="F70" s="71" t="n"/>
     </row>
     <row r="71" ht="28" customHeight="1">
-      <c r="B71" s="81" t="n"/>
+      <c r="B71" s="81" t="inlineStr">
+        <is>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
+        </is>
+      </c>
       <c r="C71" s="9" t="n"/>
       <c r="D71" s="81" t="n"/>
       <c r="E71" s="82" t="n"/>
       <c r="F71" s="71" t="n"/>
     </row>
     <row r="72" ht="28" customHeight="1">
-      <c r="B72" s="83" t="inlineStr">
-        <is>
-          <t>Managed time well, with clear transitions between steps</t>
+      <c r="B72" s="81" t="inlineStr">
+        <is>
+          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
         </is>
       </c>
       <c r="C72" s="9" t="n"/>
-      <c r="D72" s="83" t="n"/>
+      <c r="D72" s="81" t="n"/>
       <c r="E72" s="82" t="n"/>
       <c r="F72" s="71" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1">
       <c r="B73" s="81" t="inlineStr">
         <is>
-          <t>Handled difficult moments when needed to maintain call control</t>
+          <t>Next actions were documented</t>
         </is>
       </c>
       <c r="C73" s="9" t="n"/>
@@ -4171,7 +4258,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="B74" s="83" t="inlineStr">
         <is>
-          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+          <t>Realistic expectations were set</t>
         </is>
       </c>
       <c r="C74" s="9" t="n"/>
@@ -4180,64 +4267,70 @@
       <c r="F74" s="71" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1">
-      <c r="B75" s="85" t="inlineStr">
-        <is>
-          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
-        </is>
-      </c>
-      <c r="C75" s="82" t="n"/>
-      <c r="D75" s="82" t="n"/>
+      <c r="B75" s="81" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="n"/>
+      <c r="D75" s="81" t="n"/>
       <c r="E75" s="82" t="n"/>
       <c r="F75" s="71" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1">
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C76" s="122">
-        <f>IF((COUNTIF(C67:C74,"Met")+COUNTIF(C67:C74,"Partial")+COUNTIF(C67:C74,"Missed"))=0,"",ROUND((COUNTIF(C67:C74,"Met")*5+COUNTIF(C67:C74,"Partial")*2.5)/(COUNTIF(C67:C74,"Met")+COUNTIF(C67:C74,"Partial")+COUNTIF(C67:C74,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D76" s="92" t="n"/>
+      <c r="B76" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
+        </is>
+      </c>
+      <c r="C76" s="82" t="n"/>
+      <c r="D76" s="82" t="n"/>
       <c r="E76" s="82" t="n"/>
       <c r="F76" s="71" t="n"/>
     </row>
-    <row r="77" ht="24" customHeight="1">
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C77" s="14" t="n"/>
-      <c r="D77" s="84">
-        <f>IF(IF(C77="",C76,C77)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C77="",C76,C77)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="77" ht="28" customHeight="1">
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C77" s="122">
+        <f>IF((COUNTIF(C71:C75,"Met")+COUNTIF(C71:C75,"Partial")+COUNTIF(C71:C75,"Missed"))=0,"",ROUND((COUNTIF(C71:C75,"Met")*5+COUNTIF(C71:C75,"Partial")*2.5)/(COUNTIF(C71:C75,"Met")+COUNTIF(C71:C75,"Partial")+COUNTIF(C71:C75,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D77" s="92" t="n"/>
       <c r="E77" s="82" t="n"/>
       <c r="F77" s="71" t="n"/>
     </row>
-    <row r="78" ht="36" customHeight="1">
+    <row r="78" ht="24" customHeight="1">
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
-        </is>
-      </c>
-      <c r="C78" s="86" t="n"/>
-      <c r="D78" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C78" s="14" t="n"/>
+      <c r="D78" s="84">
+        <f>IF(IF(C78="",C77,C78)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C78="",C77,C78)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E78" s="82" t="n"/>
       <c r="F78" s="71" t="n"/>
     </row>
-    <row r="79" ht="28" customHeight="1">
-      <c r="B79" s="83" t="n"/>
-      <c r="C79" s="9" t="n"/>
-      <c r="D79" s="83" t="n"/>
+    <row r="79" ht="36" customHeight="1">
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
+        </is>
+      </c>
+      <c r="C79" s="86" t="n"/>
+      <c r="D79" s="82" t="n"/>
+      <c r="E79" s="82" t="n"/>
+      <c r="F79" s="71" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="B80" s="80" t="inlineStr">
         <is>
-          <t>4. CUSTOMER OWNERSHIP</t>
+          <t>5. ESCALATION JUDGMENT</t>
         </is>
       </c>
       <c r="C80" s="90" t="n"/>
@@ -4245,14 +4338,14 @@
       <c r="E80" s="74" t="n"/>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>Weight: 15%</t>
+          <t>Weight: 10%</t>
         </is>
       </c>
     </row>
     <row r="81" ht="28" customHeight="1">
       <c r="B81" s="121" t="inlineStr">
         <is>
-          <t>Objective: Measure the degree to which the agent accepted responsibility for moving the customer forward.</t>
+          <t>Objective: Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted.</t>
         </is>
       </c>
       <c r="C81" s="82" t="n"/>
@@ -4260,7 +4353,7 @@
       <c r="E81" s="82" t="n"/>
       <c r="F81" s="71" t="n"/>
     </row>
-    <row r="82" ht="24" customHeight="1">
+    <row r="82" ht="18" customHeight="1">
       <c r="B82" s="94" t="inlineStr">
         <is>
           <t>Behavioral Indicator</t>
@@ -4282,7 +4375,7 @@
     <row r="83" ht="28" customHeight="1">
       <c r="B83" s="81" t="inlineStr">
         <is>
-          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
+          <t>Completed reasonable troubleshooting before escalating</t>
         </is>
       </c>
       <c r="C83" s="9" t="n"/>
@@ -4291,7 +4384,11 @@
       <c r="F83" s="71" t="n"/>
     </row>
     <row r="84" ht="28" customHeight="1">
-      <c r="B84" s="83" t="n"/>
+      <c r="B84" s="83" t="inlineStr">
+        <is>
+          <t>Identified a valid reason to escalate</t>
+        </is>
+      </c>
       <c r="C84" s="9" t="n"/>
       <c r="D84" s="83" t="n"/>
       <c r="E84" s="82" t="n"/>
@@ -4300,7 +4397,7 @@
     <row r="85" ht="28" customHeight="1">
       <c r="B85" s="81" t="inlineStr">
         <is>
-          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+          <t>Provided complete escalation details using the correct escalation path</t>
         </is>
       </c>
       <c r="C85" s="9" t="n"/>
@@ -4309,178 +4406,185 @@
       <c r="F85" s="71" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1">
-      <c r="B86" s="83" t="n"/>
+      <c r="B86" s="81" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+        </is>
+      </c>
       <c r="C86" s="9" t="n"/>
-      <c r="D86" s="83" t="n"/>
+      <c r="D86" s="81" t="n"/>
       <c r="E86" s="82" t="n"/>
       <c r="F86" s="71" t="n"/>
     </row>
     <row r="87" ht="28" customHeight="1">
-      <c r="B87" s="81" t="inlineStr">
-        <is>
-          <t>Next actions were documented</t>
-        </is>
-      </c>
-      <c r="C87" s="9" t="n"/>
-      <c r="D87" s="81" t="n"/>
+      <c r="B87" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
+        </is>
+      </c>
+      <c r="C87" s="82" t="n"/>
+      <c r="D87" s="82" t="n"/>
       <c r="E87" s="82" t="n"/>
       <c r="F87" s="71" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1">
-      <c r="B88" s="83" t="inlineStr">
-        <is>
-          <t>Realistic expectations were set</t>
-        </is>
-      </c>
-      <c r="C88" s="9" t="n"/>
-      <c r="D88" s="83" t="n"/>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C88" s="122">
+        <f>IF((COUNTIF(C83:C86,"Met")+COUNTIF(C83:C86,"Partial")+COUNTIF(C83:C86,"Missed"))=0,"",ROUND((COUNTIF(C83:C86,"Met")*5+COUNTIF(C83:C86,"Partial")*2.5)/(COUNTIF(C83:C86,"Met")+COUNTIF(C83:C86,"Partial")+COUNTIF(C83:C86,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D88" s="92" t="n"/>
       <c r="E88" s="82" t="n"/>
       <c r="F88" s="71" t="n"/>
     </row>
-    <row r="89" ht="28" customHeight="1">
-      <c r="B89" s="81" t="inlineStr">
-        <is>
-          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
-        </is>
-      </c>
-      <c r="C89" s="9" t="n"/>
-      <c r="D89" s="81" t="n"/>
+    <row r="89" ht="24" customHeight="1">
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C89" s="14" t="n"/>
+      <c r="D89" s="84">
+        <f>IF(IF(C89="",C88,C89)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C89="",C88,C89)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E89" s="82" t="n"/>
       <c r="F89" s="71" t="n"/>
     </row>
-    <row r="90" ht="28" customHeight="1">
-      <c r="B90" s="83" t="n"/>
-      <c r="C90" s="9" t="n"/>
-      <c r="D90" s="83" t="n"/>
+    <row r="90" ht="36" customHeight="1">
+      <c r="B90" s="13" t="inlineStr">
+        <is>
+          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
+        </is>
+      </c>
+      <c r="C90" s="86" t="n"/>
+      <c r="D90" s="82" t="n"/>
       <c r="E90" s="82" t="n"/>
       <c r="F90" s="71" t="n"/>
     </row>
-    <row r="91" ht="28" customHeight="1">
-      <c r="B91" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
-        </is>
-      </c>
-      <c r="C91" s="82" t="n"/>
-      <c r="D91" s="82" t="n"/>
-      <c r="E91" s="82" t="n"/>
-      <c r="F91" s="71" t="n"/>
-    </row>
-    <row r="92" ht="28" customHeight="1">
-      <c r="B92" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C92" s="122">
-        <f>IF((COUNTIF(C83:C90,"Met")+COUNTIF(C83:C90,"Partial")+COUNTIF(C83:C90,"Missed"))=0,"",ROUND((COUNTIF(C83:C90,"Met")*5+COUNTIF(C83:C90,"Partial")*2.5)/(COUNTIF(C83:C90,"Met")+COUNTIF(C83:C90,"Partial")+COUNTIF(C83:C90,"Missed")),0))</f>
-        <v/>
-      </c>
+    <row r="91" ht="20" customHeight="1">
+      <c r="B91" s="80" t="inlineStr">
+        <is>
+          <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
+        </is>
+      </c>
+      <c r="C91" s="90" t="n"/>
+      <c r="D91" s="90" t="n"/>
+      <c r="E91" s="90" t="n"/>
+      <c r="F91" s="74" t="n"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="B92" s="13" t="inlineStr">
+        <is>
+          <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
+        </is>
+      </c>
+      <c r="C92" s="123" t="n"/>
       <c r="D92" s="92" t="n"/>
-      <c r="E92" s="82" t="n"/>
-      <c r="F92" s="71" t="n"/>
-    </row>
-    <row r="93" ht="24" customHeight="1">
-      <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C93" s="14" t="n"/>
-      <c r="D93" s="84">
-        <f>IF(IF(C93="",C92,C93)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C93="",C92,C93)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
-      <c r="E93" s="82" t="n"/>
-      <c r="F93" s="71" t="n"/>
-    </row>
-    <row r="94" ht="36" customHeight="1">
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
-        </is>
-      </c>
-      <c r="C94" s="86" t="n"/>
-      <c r="D94" s="82" t="n"/>
-      <c r="E94" s="82" t="n"/>
-      <c r="F94" s="71" t="n"/>
-    </row>
-    <row r="95" ht="24" customHeight="1">
-      <c r="B95" s="13" t="n"/>
-      <c r="C95" s="14" t="n"/>
-      <c r="D95" s="84" t="n"/>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="B96" s="80" t="inlineStr">
-        <is>
-          <t>5. ESCALATION JUDGMENT</t>
-        </is>
-      </c>
-      <c r="C96" s="90" t="n"/>
-      <c r="D96" s="90" t="n"/>
-      <c r="E96" s="74" t="n"/>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 10%</t>
-        </is>
-      </c>
+      <c r="F92" s="6" t="n"/>
+    </row>
+    <row r="93" ht="45" customHeight="1">
+      <c r="B93" s="124" t="n"/>
+      <c r="C93" s="125" t="n"/>
+      <c r="D93" s="84" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="B94" s="80" t="inlineStr">
+        <is>
+          <t>L1 learning points from this escalation outcome</t>
+        </is>
+      </c>
+      <c r="C94" s="90" t="n"/>
+      <c r="D94" s="90" t="n"/>
+      <c r="E94" s="90" t="n"/>
+      <c r="F94" s="74" t="n"/>
+    </row>
+    <row r="95" ht="28" customHeight="1">
+      <c r="B95" s="13" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C95" s="9" t="n"/>
+      <c r="D95" s="82" t="n"/>
+      <c r="E95" s="82" t="n"/>
+      <c r="F95" s="71" t="n"/>
+    </row>
+    <row r="96" ht="28" customHeight="1">
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="n"/>
+      <c r="D96" s="82" t="n"/>
+      <c r="E96" s="82" t="n"/>
+      <c r="F96" s="71" t="n"/>
     </row>
     <row r="97" ht="28" customHeight="1">
-      <c r="B97" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted.</t>
-        </is>
-      </c>
-      <c r="C97" s="82" t="n"/>
+      <c r="B97" s="13" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C97" s="9" t="n"/>
       <c r="D97" s="82" t="n"/>
       <c r="E97" s="82" t="n"/>
       <c r="F97" s="71" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1">
-      <c r="B98" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D98" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
-      <c r="E98" s="82" t="n"/>
-      <c r="F98" s="71" t="n"/>
+      <c r="B98" s="80" t="inlineStr">
+        <is>
+          <t>6. CUSTOMER EXPERIENCE</t>
+        </is>
+      </c>
+      <c r="C98" s="90" t="n"/>
+      <c r="D98" s="90" t="n"/>
+      <c r="E98" s="74" t="n"/>
+      <c r="F98" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 5%</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="28" customHeight="1">
-      <c r="B99" s="81" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before escalating</t>
-        </is>
-      </c>
-      <c r="C99" s="9" t="n"/>
-      <c r="D99" s="81" t="n"/>
+      <c r="B99" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
+        </is>
+      </c>
+      <c r="C99" s="82" t="n"/>
+      <c r="D99" s="82" t="n"/>
       <c r="E99" s="82" t="n"/>
       <c r="F99" s="71" t="n"/>
     </row>
     <row r="100" ht="28" customHeight="1">
-      <c r="B100" s="83" t="inlineStr">
-        <is>
-          <t>Identified a valid reason to escalate</t>
-        </is>
-      </c>
-      <c r="C100" s="9" t="n"/>
-      <c r="D100" s="83" t="n"/>
+      <c r="B100" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C100" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D100" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E100" s="82" t="n"/>
       <c r="F100" s="71" t="n"/>
     </row>
     <row r="101" ht="28" customHeight="1">
       <c r="B101" s="81" t="inlineStr">
         <is>
-          <t>Provided complete escalation details using the correct escalation path</t>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
         </is>
       </c>
       <c r="C101" s="9" t="n"/>
@@ -4489,7 +4593,11 @@
       <c r="F101" s="71" t="n"/>
     </row>
     <row r="102" ht="28" customHeight="1">
-      <c r="B102" s="83" t="n"/>
+      <c r="B102" s="83" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+        </is>
+      </c>
       <c r="C102" s="9" t="n"/>
       <c r="D102" s="83" t="n"/>
       <c r="E102" s="82" t="n"/>
@@ -4498,7 +4606,7 @@
     <row r="103" ht="28" customHeight="1">
       <c r="B103" s="81" t="inlineStr">
         <is>
-          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
         </is>
       </c>
       <c r="C103" s="9" t="n"/>
@@ -4507,530 +4615,663 @@
       <c r="F103" s="71" t="n"/>
     </row>
     <row r="104" ht="28" customHeight="1">
-      <c r="B104" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
-        </is>
-      </c>
-      <c r="C104" s="82" t="n"/>
-      <c r="D104" s="82" t="n"/>
+      <c r="B104" s="81" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="n"/>
+      <c r="D104" s="81" t="n"/>
       <c r="E104" s="82" t="n"/>
       <c r="F104" s="71" t="n"/>
     </row>
     <row r="105" ht="28" customHeight="1">
-      <c r="B105" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C105" s="122">
-        <f>IF((COUNTIF(C99:C103,"Met")+COUNTIF(C99:C103,"Partial")+COUNTIF(C99:C103,"Missed"))=0,"",ROUND((COUNTIF(C99:C103,"Met")*5+COUNTIF(C99:C103,"Partial")*2.5)/(COUNTIF(C99:C103,"Met")+COUNTIF(C99:C103,"Partial")+COUNTIF(C99:C103,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D105" s="92" t="n"/>
+      <c r="B105" s="83" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="n"/>
+      <c r="D105" s="83" t="n"/>
       <c r="E105" s="82" t="n"/>
       <c r="F105" s="71" t="n"/>
     </row>
-    <row r="106" ht="24" customHeight="1">
-      <c r="B106" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C106" s="14" t="n"/>
-      <c r="D106" s="84">
-        <f>IF(IF(C106="",C105,C106)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C106="",C105,C106)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="106" ht="28" customHeight="1">
+      <c r="B106" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
+        </is>
+      </c>
+      <c r="C106" s="82" t="n"/>
+      <c r="D106" s="82" t="n"/>
       <c r="E106" s="82" t="n"/>
       <c r="F106" s="71" t="n"/>
     </row>
-    <row r="107" ht="36" customHeight="1">
-      <c r="B107" s="13" t="inlineStr">
-        <is>
-          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
-        </is>
-      </c>
-      <c r="C107" s="86" t="n"/>
-      <c r="D107" s="82" t="n"/>
+    <row r="107" ht="28" customHeight="1">
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C107" s="122">
+        <f>IF((COUNTIF(C101:C105,"Met")+COUNTIF(C101:C105,"Partial")+COUNTIF(C101:C105,"Missed"))=0,"",ROUND((COUNTIF(C101:C105,"Met")*5+COUNTIF(C101:C105,"Partial")*2.5)/(COUNTIF(C101:C105,"Met")+COUNTIF(C101:C105,"Partial")+COUNTIF(C101:C105,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D107" s="92" t="n"/>
       <c r="E107" s="82" t="n"/>
       <c r="F107" s="71" t="n"/>
     </row>
-    <row r="108" ht="20" customHeight="1">
-      <c r="B108" s="80" t="inlineStr">
-        <is>
-          <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
-        </is>
-      </c>
-      <c r="C108" s="90" t="n"/>
-      <c r="D108" s="90" t="n"/>
-      <c r="E108" s="90" t="n"/>
-      <c r="F108" s="74" t="n"/>
-    </row>
-    <row r="109" ht="20" customHeight="1">
+    <row r="108" ht="24" customHeight="1">
+      <c r="B108" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C108" s="14" t="n"/>
+      <c r="D108" s="84">
+        <f>IF(IF(C108="",C107,C108)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C108="",C107,C108)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
+      <c r="E108" s="82" t="n"/>
+      <c r="F108" s="71" t="n"/>
+    </row>
+    <row r="109" ht="36" customHeight="1">
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
-        </is>
-      </c>
-      <c r="C109" s="123" t="n"/>
-      <c r="F109" s="6" t="n"/>
-    </row>
-    <row r="110" ht="45" customHeight="1">
-      <c r="B110" s="124" t="n"/>
-      <c r="C110" s="125" t="n"/>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="B111" s="80" t="inlineStr">
-        <is>
-          <t>L1 learning points from this escalation outcome</t>
-        </is>
-      </c>
-      <c r="C111" s="90" t="n"/>
-      <c r="D111" s="90" t="n"/>
-      <c r="E111" s="90" t="n"/>
-      <c r="F111" s="74" t="n"/>
-    </row>
-    <row r="112" ht="28" customHeight="1">
-      <c r="B112" s="13" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C112" s="9" t="n"/>
-      <c r="D112" s="82" t="n"/>
+          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
+        </is>
+      </c>
+      <c r="C109" s="86" t="n"/>
+      <c r="D109" s="82" t="n"/>
+      <c r="E109" s="82" t="n"/>
+      <c r="F109" s="71" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="B110" s="80" t="inlineStr">
+        <is>
+          <t>7. DOCUMENTATION &amp; NOTES</t>
+        </is>
+      </c>
+      <c r="C110" s="90" t="n"/>
+      <c r="D110" s="90" t="n"/>
+      <c r="E110" s="74" t="n"/>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>Weight: 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="28" customHeight="1">
+      <c r="B111" s="121" t="inlineStr">
+        <is>
+          <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
+        </is>
+      </c>
+      <c r="C111" s="82" t="n"/>
+      <c r="D111" s="82" t="n"/>
+      <c r="E111" s="82" t="n"/>
+      <c r="F111" s="71" t="n"/>
+    </row>
+    <row r="112" ht="36" customHeight="1">
+      <c r="B112" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D112" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E112" s="82" t="n"/>
       <c r="F112" s="71" t="n"/>
     </row>
     <row r="113" ht="28" customHeight="1">
-      <c r="B113" s="13" t="inlineStr">
-        <is>
-          <t>2.</t>
+      <c r="B113" s="81" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
         </is>
       </c>
       <c r="C113" s="9" t="n"/>
-      <c r="D113" s="82" t="n"/>
+      <c r="D113" s="81" t="n"/>
       <c r="E113" s="82" t="n"/>
       <c r="F113" s="71" t="n"/>
     </row>
     <row r="114" ht="28" customHeight="1">
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>3.</t>
+      <c r="B114" s="83" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
         </is>
       </c>
       <c r="C114" s="9" t="n"/>
-      <c r="D114" s="82" t="n"/>
+      <c r="D114" s="83" t="n"/>
       <c r="E114" s="82" t="n"/>
       <c r="F114" s="71" t="n"/>
     </row>
     <row r="115" ht="28" customHeight="1">
-      <c r="B115" s="83" t="n"/>
+      <c r="B115" s="81" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
+        </is>
+      </c>
       <c r="C115" s="9" t="n"/>
-      <c r="D115" s="83" t="n"/>
-    </row>
-    <row r="116" ht="18" customHeight="1">
-      <c r="B116" s="80" t="inlineStr">
-        <is>
-          <t>6. CUSTOMER EXPERIENCE</t>
-        </is>
-      </c>
-      <c r="C116" s="90" t="n"/>
-      <c r="D116" s="90" t="n"/>
-      <c r="E116" s="74" t="n"/>
-      <c r="F116" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 5%</t>
-        </is>
-      </c>
+      <c r="D115" s="81" t="n"/>
+      <c r="E115" s="82" t="n"/>
+      <c r="F115" s="71" t="n"/>
+    </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="B116" s="83" t="inlineStr">
+        <is>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="n"/>
+      <c r="D116" s="83" t="n"/>
+      <c r="E116" s="82" t="n"/>
+      <c r="F116" s="71" t="n"/>
     </row>
     <row r="117" ht="28" customHeight="1">
-      <c r="B117" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
-        </is>
-      </c>
-      <c r="C117" s="82" t="n"/>
-      <c r="D117" s="82" t="n"/>
+      <c r="B117" s="83" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="n"/>
+      <c r="D117" s="83" t="n"/>
       <c r="E117" s="82" t="n"/>
       <c r="F117" s="71" t="n"/>
     </row>
     <row r="118" ht="28" customHeight="1">
-      <c r="B118" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C118" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D118" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="B118" s="81" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="n"/>
+      <c r="D118" s="81" t="n"/>
       <c r="E118" s="82" t="n"/>
       <c r="F118" s="71" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1">
-      <c r="B119" s="81" t="inlineStr">
-        <is>
-          <t>Demonstrated empathy including for repeat-contact fatigue</t>
-        </is>
-      </c>
-      <c r="C119" s="9" t="n"/>
-      <c r="D119" s="81" t="n"/>
+      <c r="B119" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
+        </is>
+      </c>
+      <c r="C119" s="82" t="n"/>
+      <c r="D119" s="82" t="n"/>
       <c r="E119" s="82" t="n"/>
       <c r="F119" s="71" t="n"/>
     </row>
-    <row r="120" ht="28" customHeight="1">
-      <c r="B120" s="83" t="inlineStr">
-        <is>
-          <t>Stayed professional throughout and maintained patience, even under pressure</t>
-        </is>
-      </c>
-      <c r="C120" s="9" t="n"/>
-      <c r="D120" s="83" t="n"/>
+    <row r="120" ht="52" customHeight="1">
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C120" s="122">
+        <f>IF((COUNTIF(C113:C118,"Met")+COUNTIF(C113:C118,"Partial")+COUNTIF(C113:C118,"Missed"))=0,"",ROUND((COUNTIF(C113:C118,"Met")*5+COUNTIF(C113:C118,"Partial")*2.5)/(COUNTIF(C113:C118,"Met")+COUNTIF(C113:C118,"Partial")+COUNTIF(C113:C118,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D120" s="92" t="n"/>
       <c r="E120" s="82" t="n"/>
       <c r="F120" s="71" t="n"/>
     </row>
-    <row r="121" ht="28" customHeight="1">
-      <c r="B121" s="81" t="inlineStr">
-        <is>
-          <t>Agent matched the customer's tone, pace, level, and energy</t>
-        </is>
-      </c>
-      <c r="C121" s="9" t="n"/>
-      <c r="D121" s="81" t="n"/>
+    <row r="121" ht="24" customHeight="1">
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="n"/>
+      <c r="D121" s="84">
+        <f>IF(IF(C121="",C120,C121)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C121="",C120,C121)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E121" s="82" t="n"/>
       <c r="F121" s="71" t="n"/>
     </row>
-    <row r="122" ht="28" customHeight="1">
-      <c r="B122" s="83" t="n"/>
-      <c r="C122" s="9" t="n"/>
-      <c r="D122" s="83" t="n"/>
+    <row r="122" ht="36" customHeight="1">
+      <c r="B122" s="13" t="inlineStr">
+        <is>
+          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
+        </is>
+      </c>
+      <c r="C122" s="86" t="n"/>
+      <c r="D122" s="82" t="n"/>
       <c r="E122" s="82" t="n"/>
       <c r="F122" s="71" t="n"/>
     </row>
-    <row r="123" ht="28" customHeight="1">
-      <c r="B123" s="81" t="inlineStr">
-        <is>
-          <t>Minimized customer effort</t>
-        </is>
-      </c>
-      <c r="C123" s="9" t="n"/>
-      <c r="D123" s="81" t="n"/>
-      <c r="E123" s="82" t="n"/>
-      <c r="F123" s="71" t="n"/>
+    <row r="123" ht="30" customHeight="1">
+      <c r="B123" s="80" t="inlineStr">
+        <is>
+          <t>4 · RESOLUTION OUTCOME</t>
+        </is>
+      </c>
+      <c r="C123" s="90" t="n"/>
+      <c r="D123" s="90" t="n"/>
+      <c r="E123" s="90" t="n"/>
+      <c r="F123" s="74" t="n"/>
     </row>
     <row r="124" ht="28" customHeight="1">
-      <c r="B124" s="83" t="inlineStr">
-        <is>
-          <t>Maintained customer understanding and engagement</t>
-        </is>
-      </c>
-      <c r="C124" s="9" t="n"/>
-      <c r="D124" s="83" t="n"/>
+      <c r="B124" s="94" t="inlineStr">
+        <is>
+          <t>Outcome classification</t>
+        </is>
+      </c>
+      <c r="C124" s="97" t="n"/>
+      <c r="D124" s="82" t="n"/>
       <c r="E124" s="82" t="n"/>
       <c r="F124" s="71" t="n"/>
     </row>
-    <row r="125" ht="28" customHeight="1">
-      <c r="B125" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="C125" s="82" t="n"/>
+    <row r="125" ht="52" customHeight="1">
+      <c r="B125" s="87" t="inlineStr">
+        <is>
+          <t>Primary positive outcome achieved</t>
+        </is>
+      </c>
+      <c r="C125" s="88" t="n"/>
       <c r="D125" s="82" t="n"/>
       <c r="E125" s="82" t="n"/>
       <c r="F125" s="71" t="n"/>
     </row>
-    <row r="126" ht="28" customHeight="1">
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C126" s="122">
-        <f>IF((COUNTIF(C119:C124,"Met")+COUNTIF(C119:C124,"Partial")+COUNTIF(C119:C124,"Missed"))=0,"",ROUND((COUNTIF(C119:C124,"Met")*5+COUNTIF(C119:C124,"Partial")*2.5)/(COUNTIF(C119:C124,"Met")+COUNTIF(C119:C124,"Partial")+COUNTIF(C119:C124,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D126" s="92" t="n"/>
+    <row r="126" ht="52" customHeight="1">
+      <c r="B126" s="94" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
+      <c r="C126" s="86" t="n"/>
+      <c r="D126" s="82" t="n"/>
       <c r="E126" s="82" t="n"/>
       <c r="F126" s="71" t="n"/>
     </row>
-    <row r="127" ht="24" customHeight="1">
-      <c r="B127" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C127" s="14" t="n"/>
-      <c r="D127" s="84">
-        <f>IF(IF(C127="",C126,C127)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C127="",C126,C127)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
-      <c r="E127" s="82" t="n"/>
-      <c r="F127" s="71" t="n"/>
-    </row>
-    <row r="128" ht="36" customHeight="1">
-      <c r="B128" s="13" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
-      <c r="C128" s="86" t="n"/>
-      <c r="D128" s="82" t="n"/>
+    <row r="127" ht="26" customHeight="1">
+      <c r="B127" s="80" t="inlineStr">
+        <is>
+          <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
+        </is>
+      </c>
+      <c r="C127" s="90" t="n"/>
+      <c r="D127" s="90" t="n"/>
+      <c r="E127" s="90" t="n"/>
+      <c r="F127" s="74" t="n"/>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="B128" s="87" t="inlineStr">
+        <is>
+          <t>Did the interaction disconnect before completion?</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D128" s="85" t="inlineStr">
+        <is>
+          <t>If Yes, at least one documented follow-up action is required.</t>
+        </is>
+      </c>
       <c r="E128" s="82" t="n"/>
       <c r="F128" s="71" t="n"/>
     </row>
-    <row r="129" ht="28" customHeight="1">
-      <c r="B129" s="85" t="n"/>
-      <c r="C129" s="9" t="n"/>
-      <c r="D129" s="83" t="n"/>
-    </row>
-    <row r="130" ht="18" customHeight="1">
-      <c r="B130" s="80" t="inlineStr">
-        <is>
-          <t>7. DOCUMENTATION &amp; NOTES</t>
+    <row r="129" ht="30" customHeight="1">
+      <c r="B129" s="94" t="inlineStr">
+        <is>
+          <t>Follow-up action taken</t>
+        </is>
+      </c>
+      <c r="C129" s="88" t="inlineStr">
+        <is>
+          <t>N.A. — no disconnect</t>
+        </is>
+      </c>
+      <c r="D129" s="71" t="n"/>
+      <c r="E129" s="79">
+        <f>IF(AND(C128="Yes",OR(C129="None",C129="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
+        <v/>
+      </c>
+      <c r="F129" s="71" t="n"/>
+    </row>
+    <row r="130" ht="26" customHeight="1">
+      <c r="B130" s="98" t="inlineStr">
+        <is>
+          <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
         </is>
       </c>
       <c r="C130" s="90" t="n"/>
       <c r="D130" s="90" t="n"/>
-      <c r="E130" s="74" t="n"/>
-      <c r="F130" s="6" t="inlineStr">
-        <is>
-          <t>Weight: 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="28" customHeight="1">
-      <c r="B131" s="121" t="inlineStr">
-        <is>
-          <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
-        </is>
-      </c>
-      <c r="C131" s="82" t="n"/>
-      <c r="D131" s="82" t="n"/>
-      <c r="E131" s="82" t="n"/>
-      <c r="F131" s="71" t="n"/>
-    </row>
-    <row r="132" ht="36" customHeight="1">
-      <c r="B132" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C132" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D132" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="E130" s="90" t="n"/>
+      <c r="F130" s="74" t="n"/>
+    </row>
+    <row r="131" ht="26" customHeight="1">
+      <c r="B131" s="80" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="C131" s="119" t="inlineStr">
+        <is>
+          <t>Present?</t>
+        </is>
+      </c>
+      <c r="D131" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E131" s="90" t="n"/>
+      <c r="F131" s="74" t="n"/>
+    </row>
+    <row r="132" ht="26" customHeight="1">
+      <c r="B132" s="81" t="inlineStr">
+        <is>
+          <t>Harmful or incorrect troubleshooting provided</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D132" s="81" t="n"/>
       <c r="E132" s="82" t="n"/>
       <c r="F132" s="71" t="n"/>
     </row>
-    <row r="133" ht="28" customHeight="1">
-      <c r="B133" s="81" t="inlineStr">
-        <is>
-          <t>Recorded customer issue summary</t>
-        </is>
-      </c>
-      <c r="C133" s="9" t="n"/>
-      <c r="D133" s="81" t="n"/>
+    <row r="133" ht="26" customHeight="1">
+      <c r="B133" s="83" t="inlineStr">
+        <is>
+          <t>Misrepresented product capabilities</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D133" s="83" t="n"/>
       <c r="E133" s="82" t="n"/>
       <c r="F133" s="71" t="n"/>
     </row>
-    <row r="134" ht="28" customHeight="1">
-      <c r="B134" s="83" t="inlineStr">
-        <is>
-          <t>Documented troubleshooting steps</t>
-        </is>
-      </c>
-      <c r="C134" s="9" t="n"/>
-      <c r="D134" s="83" t="n"/>
+    <row r="134" ht="26" customHeight="1">
+      <c r="B134" s="81" t="inlineStr">
+        <is>
+          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D134" s="81" t="n"/>
       <c r="E134" s="82" t="n"/>
       <c r="F134" s="71" t="n"/>
     </row>
-    <row r="135" ht="28" customHeight="1">
-      <c r="B135" s="81" t="inlineStr">
-        <is>
-          <t>Noted key findings</t>
-        </is>
-      </c>
-      <c r="C135" s="9" t="n"/>
-      <c r="D135" s="81" t="n"/>
+    <row r="135" ht="26" customHeight="1">
+      <c r="B135" s="83" t="inlineStr">
+        <is>
+          <t>No follow-up after disconnected call</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D135" s="83" t="n"/>
       <c r="E135" s="82" t="n"/>
       <c r="F135" s="71" t="n"/>
     </row>
-    <row r="136" ht="28" customHeight="1">
-      <c r="B136" s="83" t="inlineStr">
-        <is>
-          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
-        </is>
-      </c>
-      <c r="C136" s="9" t="n"/>
-      <c r="D136" s="83" t="n"/>
+    <row r="136" ht="26" customHeight="1">
+      <c r="B136" s="81" t="inlineStr">
+        <is>
+          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D136" s="81" t="n"/>
       <c r="E136" s="82" t="n"/>
       <c r="F136" s="71" t="n"/>
     </row>
-    <row r="137" ht="28" customHeight="1">
-      <c r="B137" s="81" t="n"/>
-      <c r="C137" s="9" t="n"/>
-      <c r="D137" s="81" t="n"/>
+    <row r="137" ht="26" customHeight="1">
+      <c r="B137" s="83" t="inlineStr">
+        <is>
+          <t>Abandoned customer without a path forward</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D137" s="83" t="n"/>
       <c r="E137" s="82" t="n"/>
       <c r="F137" s="71" t="n"/>
     </row>
-    <row r="138" ht="28" customHeight="1">
-      <c r="B138" s="83" t="inlineStr">
-        <is>
-          <t>Documented next steps and follow-ups</t>
-        </is>
-      </c>
-      <c r="C138" s="9" t="n"/>
-      <c r="D138" s="83" t="n"/>
+    <row r="138" ht="26" customHeight="1">
+      <c r="B138" s="81" t="inlineStr">
+        <is>
+          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D138" s="81" t="n"/>
       <c r="E138" s="82" t="n"/>
       <c r="F138" s="71" t="n"/>
     </row>
-    <row r="139" ht="28" customHeight="1">
-      <c r="B139" s="81" t="inlineStr">
-        <is>
-          <t>Updated ticket status accurately</t>
-        </is>
-      </c>
-      <c r="C139" s="9" t="n"/>
-      <c r="D139" s="81" t="n"/>
+    <row r="139" ht="26" customHeight="1">
+      <c r="B139" s="83" t="inlineStr">
+        <is>
+          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D139" s="83" t="n"/>
       <c r="E139" s="82" t="n"/>
       <c r="F139" s="71" t="n"/>
     </row>
-    <row r="140" ht="28" customHeight="1">
-      <c r="B140" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="C140" s="82" t="n"/>
-      <c r="D140" s="82" t="n"/>
+    <row r="140" ht="26" customHeight="1">
+      <c r="B140" s="83" t="inlineStr">
+        <is>
+          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D140" s="83" t="n"/>
       <c r="E140" s="82" t="n"/>
       <c r="F140" s="71" t="n"/>
     </row>
-    <row r="141" ht="52" customHeight="1">
-      <c r="B141" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C141" s="122">
-        <f>IF((COUNTIF(C133:C139,"Met")+COUNTIF(C133:C139,"Partial")+COUNTIF(C133:C139,"Missed"))=0,"",ROUND((COUNTIF(C133:C139,"Met")*5+COUNTIF(C133:C139,"Partial")*2.5)/(COUNTIF(C133:C139,"Met")+COUNTIF(C133:C139,"Partial")+COUNTIF(C133:C139,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D141" s="92" t="n"/>
+    <row r="141" ht="26" customHeight="1">
+      <c r="B141" s="81" t="inlineStr">
+        <is>
+          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D141" s="81" t="n"/>
       <c r="E141" s="82" t="n"/>
       <c r="F141" s="71" t="n"/>
     </row>
-    <row r="142" ht="24" customHeight="1">
-      <c r="B142" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C142" s="14" t="n"/>
-      <c r="D142" s="84">
-        <f>IF(IF(C142="",C141,C142)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C142="",C141,C142)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="142" ht="26" customHeight="1">
+      <c r="B142" s="81" t="inlineStr">
+        <is>
+          <t>Survey / CSAT manipulation</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D142" s="81" t="n"/>
       <c r="E142" s="82" t="n"/>
       <c r="F142" s="71" t="n"/>
     </row>
-    <row r="143" ht="36" customHeight="1">
-      <c r="B143" s="13" t="inlineStr">
-        <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
-      <c r="C143" s="86" t="n"/>
-      <c r="D143" s="82" t="n"/>
-      <c r="E143" s="82" t="n"/>
-      <c r="F143" s="71" t="n"/>
-    </row>
-    <row r="144">
-      <c r="B144" s="80" t="n"/>
+    <row r="143" ht="26" customHeight="1">
+      <c r="B143" s="98" t="inlineStr">
+        <is>
+          <t>CRITICAL FAILURE FLAGGED?</t>
+        </is>
+      </c>
+      <c r="C143" s="93">
+        <f>IF(COUNTIF(C132:C142,"Yes")&gt;0,"YES — "&amp;COUNTIF(C132:C142,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
+        <v/>
+      </c>
+      <c r="D143" s="90" t="n"/>
+      <c r="E143" s="90" t="n"/>
+      <c r="F143" s="74" t="n"/>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="B144" s="98" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
+      <c r="C144" s="90" t="n"/>
+      <c r="D144" s="90" t="n"/>
+      <c r="E144" s="90" t="n"/>
+      <c r="F144" s="74" t="n"/>
     </row>
     <row r="145" ht="30" customHeight="1">
-      <c r="B145" s="80" t="n"/>
-      <c r="C145" s="9" t="n"/>
-      <c r="D145" s="85" t="n"/>
+      <c r="B145" s="85" t="inlineStr">
+        <is>
+          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
+        </is>
+      </c>
+      <c r="C145" s="82" t="n"/>
+      <c r="D145" s="82" t="n"/>
+      <c r="E145" s="82" t="n"/>
+      <c r="F145" s="71" t="n"/>
     </row>
     <row r="146" ht="30" customHeight="1">
       <c r="B146" s="80" t="inlineStr">
         <is>
-          <t>4 · RESOLUTION OUTCOME</t>
-        </is>
-      </c>
-      <c r="C146" s="90" t="n"/>
-      <c r="D146" s="90" t="n"/>
+          <t>Compliance gate  (mark Yes if adhered)</t>
+        </is>
+      </c>
+      <c r="C146" s="119" t="inlineStr">
+        <is>
+          <t>Adherent?</t>
+        </is>
+      </c>
+      <c r="D146" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
       <c r="E146" s="90" t="n"/>
       <c r="F146" s="74" t="n"/>
     </row>
-    <row r="147">
-      <c r="B147" s="94" t="inlineStr">
-        <is>
-          <t>Outcome classification</t>
-        </is>
-      </c>
-      <c r="C147" s="97" t="n"/>
-      <c r="D147" s="82" t="n"/>
+    <row r="147" ht="26" customHeight="1">
+      <c r="B147" s="81" t="inlineStr">
+        <is>
+          <t>Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D147" s="81" t="n"/>
       <c r="E147" s="82" t="n"/>
       <c r="F147" s="71" t="n"/>
     </row>
-    <row r="148" ht="52" customHeight="1">
-      <c r="B148" s="87" t="inlineStr">
-        <is>
-          <t>Primary positive outcome achieved</t>
-        </is>
-      </c>
-      <c r="C148" s="88" t="n"/>
-      <c r="D148" s="82" t="n"/>
+    <row r="148" ht="26" customHeight="1">
+      <c r="B148" s="81" t="inlineStr">
+        <is>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D148" s="81" t="n"/>
       <c r="E148" s="82" t="n"/>
       <c r="F148" s="71" t="n"/>
     </row>
-    <row r="149" ht="52" customHeight="1">
-      <c r="B149" s="94" t="inlineStr">
-        <is>
-          <t>Justification</t>
-        </is>
-      </c>
-      <c r="C149" s="86" t="n"/>
-      <c r="D149" s="82" t="n"/>
+    <row r="149" ht="26" customHeight="1">
+      <c r="B149" s="81" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D149" s="81" t="n"/>
       <c r="E149" s="82" t="n"/>
       <c r="F149" s="71" t="n"/>
     </row>
-    <row r="150" ht="26" customHeight="1">
-      <c r="B150" s="80" t="n"/>
-      <c r="C150" s="9" t="n"/>
-      <c r="D150" s="81" t="n"/>
+    <row r="150" ht="32" customHeight="1">
+      <c r="B150" s="80" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
+        </is>
+      </c>
+      <c r="C150" s="119" t="inlineStr">
+        <is>
+          <t>Occurred?</t>
+        </is>
+      </c>
+      <c r="D150" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E150" s="90" t="n"/>
+      <c r="F150" s="74" t="n"/>
     </row>
     <row r="151" ht="26" customHeight="1">
-      <c r="B151" s="80" t="inlineStr">
-        <is>
-          <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
-        </is>
-      </c>
-      <c r="C151" s="90" t="n"/>
-      <c r="D151" s="90" t="n"/>
-      <c r="E151" s="90" t="n"/>
-      <c r="F151" s="74" t="n"/>
-    </row>
-    <row r="152" ht="30" customHeight="1">
-      <c r="B152" s="87" t="inlineStr">
-        <is>
-          <t>Did the interaction disconnect before completion?</t>
+      <c r="B151" s="81" t="inlineStr">
+        <is>
+          <t>A.  Call / Session Abandonment</t>
+        </is>
+      </c>
+      <c r="C151" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D151" s="81" t="n"/>
+      <c r="E151" s="82" t="n"/>
+      <c r="F151" s="71" t="n"/>
+    </row>
+    <row r="152" ht="26" customHeight="1">
+      <c r="B152" s="81" t="inlineStr">
+        <is>
+          <t>B.  Call / Session Avoidance / Evasion</t>
         </is>
       </c>
       <c r="C152" s="9" t="inlineStr">
@@ -5038,71 +5279,74 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D152" s="85" t="inlineStr">
-        <is>
-          <t>If Yes, at least one documented follow-up action is required.</t>
-        </is>
-      </c>
+      <c r="D152" s="81" t="n"/>
       <c r="E152" s="82" t="n"/>
       <c r="F152" s="71" t="n"/>
     </row>
-    <row r="153" ht="30" customHeight="1">
-      <c r="B153" s="94" t="inlineStr">
-        <is>
-          <t>Follow-up action taken</t>
-        </is>
-      </c>
-      <c r="C153" s="88" t="inlineStr">
-        <is>
-          <t>N.A. — no disconnect</t>
-        </is>
-      </c>
-      <c r="D153" s="71" t="n"/>
-      <c r="E153" s="79">
-        <f>IF(AND(C152="Yes",OR(C153="None",C153="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
-        <v/>
-      </c>
+    <row r="153" ht="26" customHeight="1">
+      <c r="B153" s="81" t="inlineStr">
+        <is>
+          <t>C.  Discourtesy</t>
+        </is>
+      </c>
+      <c r="C153" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D153" s="81" t="n"/>
+      <c r="E153" s="82" t="n"/>
       <c r="F153" s="71" t="n"/>
     </row>
     <row r="154" ht="26" customHeight="1">
-      <c r="B154" s="98" t="n"/>
-      <c r="C154" s="9" t="n"/>
+      <c r="B154" s="81" t="inlineStr">
+        <is>
+          <t>D.  Escalation</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="D154" s="81" t="n"/>
+      <c r="E154" s="82" t="n"/>
+      <c r="F154" s="71" t="n"/>
     </row>
     <row r="155" ht="26" customHeight="1">
-      <c r="B155" s="98" t="inlineStr">
-        <is>
-          <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
-        </is>
-      </c>
-      <c r="C155" s="90" t="n"/>
-      <c r="D155" s="90" t="n"/>
-      <c r="E155" s="90" t="n"/>
-      <c r="F155" s="74" t="n"/>
+      <c r="B155" s="81" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D155" s="81" t="n"/>
+      <c r="E155" s="82" t="n"/>
+      <c r="F155" s="71" t="n"/>
     </row>
     <row r="156" ht="26" customHeight="1">
-      <c r="B156" s="80" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="C156" s="119" t="inlineStr">
-        <is>
-          <t>Present?</t>
-        </is>
-      </c>
-      <c r="D156" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E156" s="90" t="n"/>
-      <c r="F156" s="74" t="n"/>
+      <c r="B156" s="81" t="inlineStr">
+        <is>
+          <t>F.  Fraud</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D156" s="81" t="n"/>
+      <c r="E156" s="82" t="n"/>
+      <c r="F156" s="71" t="n"/>
     </row>
     <row r="157" ht="26" customHeight="1">
       <c r="B157" s="81" t="inlineStr">
         <is>
-          <t>Harmful or incorrect troubleshooting provided</t>
+          <t>G.  Hard-selling</t>
         </is>
       </c>
       <c r="C157" s="9" t="inlineStr">
@@ -5115,9 +5359,9 @@
       <c r="F157" s="71" t="n"/>
     </row>
     <row r="158" ht="26" customHeight="1">
-      <c r="B158" s="83" t="inlineStr">
-        <is>
-          <t>Misrepresented product capabilities</t>
+      <c r="B158" s="81" t="inlineStr">
+        <is>
+          <t>H.  Line Release</t>
         </is>
       </c>
       <c r="C158" s="9" t="inlineStr">
@@ -5125,14 +5369,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D158" s="83" t="n"/>
+      <c r="D158" s="81" t="n"/>
       <c r="E158" s="82" t="n"/>
       <c r="F158" s="71" t="n"/>
     </row>
     <row r="159" ht="26" customHeight="1">
       <c r="B159" s="81" t="inlineStr">
         <is>
-          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
+          <t>I.  Non-Adherence to Callback Hours</t>
         </is>
       </c>
       <c r="C159" s="9" t="inlineStr">
@@ -5145,9 +5389,9 @@
       <c r="F159" s="71" t="n"/>
     </row>
     <row r="160" ht="26" customHeight="1">
-      <c r="B160" s="83" t="inlineStr">
-        <is>
-          <t>No follow-up after disconnected call</t>
+      <c r="B160" s="81" t="inlineStr">
+        <is>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
         </is>
       </c>
       <c r="C160" s="9" t="inlineStr">
@@ -5155,14 +5399,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D160" s="83" t="n"/>
+      <c r="D160" s="81" t="n"/>
       <c r="E160" s="82" t="n"/>
       <c r="F160" s="71" t="n"/>
     </row>
     <row r="161" ht="26" customHeight="1">
       <c r="B161" s="81" t="inlineStr">
         <is>
-          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
+          <t>K.  Non-First Call Resolution</t>
         </is>
       </c>
       <c r="C161" s="9" t="inlineStr">
@@ -5174,130 +5418,108 @@
       <c r="E161" s="82" t="n"/>
       <c r="F161" s="71" t="n"/>
     </row>
-    <row r="162" ht="26" customHeight="1">
-      <c r="B162" s="83" t="inlineStr">
-        <is>
-          <t>Abandoned customer without a path forward</t>
-        </is>
-      </c>
-      <c r="C162" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D162" s="83" t="n"/>
-      <c r="E162" s="82" t="n"/>
-      <c r="F162" s="71" t="n"/>
-    </row>
-    <row r="163" ht="26" customHeight="1">
-      <c r="B163" s="81" t="inlineStr">
-        <is>
-          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
-        </is>
-      </c>
-      <c r="C163" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D163" s="81" t="n"/>
-      <c r="E163" s="82" t="n"/>
-      <c r="F163" s="71" t="n"/>
-    </row>
-    <row r="164" ht="26" customHeight="1">
-      <c r="B164" s="83" t="inlineStr">
-        <is>
-          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
-        </is>
-      </c>
-      <c r="C164" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D164" s="83" t="n"/>
-      <c r="E164" s="82" t="n"/>
-      <c r="F164" s="71" t="n"/>
-    </row>
-    <row r="165" ht="26" customHeight="1">
-      <c r="B165" s="83" t="inlineStr">
-        <is>
-          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
-        </is>
-      </c>
-      <c r="C165" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D165" s="83" t="n"/>
+    <row r="162" ht="24" customHeight="1">
+      <c r="B162" s="98" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO TRIGGERED?</t>
+        </is>
+      </c>
+      <c r="C162" s="93">
+        <f>IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
+      <c r="D162" s="90" t="n"/>
+      <c r="E162" s="90" t="n"/>
+      <c r="F162" s="74" t="n"/>
+    </row>
+    <row r="163" ht="20" customHeight="1">
+      <c r="B163" s="96" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
+        </is>
+      </c>
+      <c r="C163" s="90" t="n"/>
+      <c r="D163" s="90" t="n"/>
+      <c r="E163" s="90" t="n"/>
+      <c r="F163" s="74" t="n"/>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="B164" s="91" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+        </is>
+      </c>
+      <c r="C164" s="90" t="n"/>
+      <c r="D164" s="90" t="n"/>
+      <c r="E164" s="90" t="n"/>
+      <c r="F164" s="74" t="n"/>
+    </row>
+    <row r="165" ht="58" customHeight="1">
+      <c r="B165" s="86" t="n"/>
+      <c r="C165" s="82" t="n"/>
+      <c r="D165" s="82" t="n"/>
       <c r="E165" s="82" t="n"/>
       <c r="F165" s="71" t="n"/>
     </row>
-    <row r="166" ht="26" customHeight="1">
-      <c r="B166" s="81" t="inlineStr">
-        <is>
-          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
-        </is>
-      </c>
-      <c r="C166" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D166" s="81" t="n"/>
-      <c r="E166" s="82" t="n"/>
-      <c r="F166" s="71" t="n"/>
-    </row>
-    <row r="167" ht="26" customHeight="1">
-      <c r="B167" s="81" t="inlineStr">
-        <is>
-          <t>Survey / CSAT manipulation</t>
-        </is>
-      </c>
-      <c r="C167" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D167" s="81" t="n"/>
+    <row r="166" ht="30" customHeight="1">
+      <c r="B166" s="91" t="inlineStr">
+        <is>
+          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
+        </is>
+      </c>
+      <c r="C166" s="90" t="n"/>
+      <c r="D166" s="90" t="n"/>
+      <c r="E166" s="90" t="n"/>
+      <c r="F166" s="74" t="n"/>
+    </row>
+    <row r="167" ht="24" customHeight="1">
+      <c r="B167" s="87" t="inlineStr">
+        <is>
+          <t>What went well — behaviors to repeat</t>
+        </is>
+      </c>
+      <c r="C167" s="82" t="n"/>
+      <c r="D167" s="82" t="n"/>
       <c r="E167" s="82" t="n"/>
       <c r="F167" s="71" t="n"/>
     </row>
-    <row r="168" ht="26" customHeight="1">
-      <c r="B168" s="98" t="inlineStr">
-        <is>
-          <t>CRITICAL FAILURE FLAGGED?</t>
-        </is>
-      </c>
-      <c r="C168" s="93">
-        <f>IF(COUNTIF(C157:C167,"Yes")&gt;0,"YES — "&amp;COUNTIF(C157:C167,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
-        <v/>
-      </c>
-      <c r="D168" s="90" t="n"/>
-      <c r="E168" s="90" t="n"/>
-      <c r="F168" s="74" t="n"/>
-    </row>
-    <row r="169" ht="20" customHeight="1">
-      <c r="B169" s="96" t="n"/>
-      <c r="C169" s="119" t="n"/>
-      <c r="D169" s="80" t="n"/>
-    </row>
-    <row r="170" ht="22" customHeight="1">
-      <c r="B170" s="98" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
-      <c r="C170" s="90" t="n"/>
-      <c r="D170" s="90" t="n"/>
-      <c r="E170" s="90" t="n"/>
-      <c r="F170" s="74" t="n"/>
-    </row>
-    <row r="171" ht="30" customHeight="1">
-      <c r="B171" s="85" t="inlineStr">
-        <is>
-          <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
+    <row r="168" ht="32" customHeight="1">
+      <c r="B168" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C168" s="86" t="n"/>
+      <c r="D168" s="82" t="n"/>
+      <c r="E168" s="82" t="n"/>
+      <c r="F168" s="71" t="n"/>
+    </row>
+    <row r="169" ht="32" customHeight="1">
+      <c r="B169" s="7" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C169" s="86" t="n"/>
+      <c r="D169" s="82" t="n"/>
+      <c r="E169" s="82" t="n"/>
+      <c r="F169" s="71" t="n"/>
+    </row>
+    <row r="170" ht="32" customHeight="1">
+      <c r="B170" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C170" s="86" t="n"/>
+      <c r="D170" s="82" t="n"/>
+      <c r="E170" s="82" t="n"/>
+      <c r="F170" s="71" t="n"/>
+    </row>
+    <row r="171" ht="24" customHeight="1">
+      <c r="B171" s="87" t="inlineStr">
+        <is>
+          <t>Improvement opportunities — behaviors to improve</t>
         </is>
       </c>
       <c r="C171" s="82" t="n"/>
@@ -5305,739 +5527,378 @@
       <c r="E171" s="82" t="n"/>
       <c r="F171" s="71" t="n"/>
     </row>
-    <row r="172" ht="30" customHeight="1">
-      <c r="B172" s="80" t="inlineStr">
-        <is>
-          <t>Compliance gate  (mark Yes if adhered)</t>
-        </is>
-      </c>
-      <c r="C172" s="119" t="inlineStr">
-        <is>
-          <t>Adherent?</t>
-        </is>
-      </c>
-      <c r="D172" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E172" s="90" t="n"/>
-      <c r="F172" s="74" t="n"/>
-    </row>
-    <row r="173" ht="26" customHeight="1">
-      <c r="B173" s="81" t="inlineStr">
-        <is>
-          <t>Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C173" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D173" s="81" t="n"/>
+    <row r="172" ht="32" customHeight="1">
+      <c r="B172" s="7" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C172" s="86" t="n"/>
+      <c r="D172" s="82" t="n"/>
+      <c r="E172" s="82" t="n"/>
+      <c r="F172" s="71" t="n"/>
+    </row>
+    <row r="173" ht="32" customHeight="1">
+      <c r="B173" s="7" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C173" s="86" t="n"/>
+      <c r="D173" s="82" t="n"/>
       <c r="E173" s="82" t="n"/>
       <c r="F173" s="71" t="n"/>
     </row>
-    <row r="174" ht="26" customHeight="1">
-      <c r="B174" s="81" t="inlineStr">
-        <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C174" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D174" s="81" t="n"/>
+    <row r="174" ht="32" customHeight="1">
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C174" s="86" t="n"/>
+      <c r="D174" s="82" t="n"/>
       <c r="E174" s="82" t="n"/>
       <c r="F174" s="71" t="n"/>
     </row>
-    <row r="175" ht="26" customHeight="1">
-      <c r="B175" s="81" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C175" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D175" s="81" t="n"/>
+    <row r="175" ht="24" customHeight="1">
+      <c r="B175" s="87" t="inlineStr">
+        <is>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
+        </is>
+      </c>
+      <c r="C175" s="82" t="n"/>
+      <c r="D175" s="82" t="n"/>
       <c r="E175" s="82" t="n"/>
       <c r="F175" s="71" t="n"/>
     </row>
-    <row r="176" ht="32" customHeight="1">
-      <c r="B176" s="80" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
-        </is>
-      </c>
-      <c r="C176" s="119" t="inlineStr">
-        <is>
-          <t>Occurred?</t>
-        </is>
-      </c>
-      <c r="D176" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
-      <c r="E176" s="90" t="n"/>
-      <c r="F176" s="74" t="n"/>
-    </row>
-    <row r="177" ht="26" customHeight="1">
-      <c r="B177" s="81" t="inlineStr">
-        <is>
-          <t>A.  Call / Session Abandonment</t>
-        </is>
-      </c>
-      <c r="C177" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D177" s="81" t="n"/>
+    <row r="176" ht="58" customHeight="1">
+      <c r="B176" s="86" t="n"/>
+      <c r="C176" s="82" t="n"/>
+      <c r="D176" s="82" t="n"/>
+      <c r="E176" s="82" t="n"/>
+      <c r="F176" s="71" t="n"/>
+    </row>
+    <row r="177" ht="20" customHeight="1">
+      <c r="B177" s="87" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
+      <c r="C177" s="82" t="n"/>
+      <c r="D177" s="82" t="n"/>
       <c r="E177" s="82" t="n"/>
       <c r="F177" s="71" t="n"/>
     </row>
-    <row r="178" ht="26" customHeight="1">
-      <c r="B178" s="81" t="inlineStr">
-        <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
-        </is>
-      </c>
-      <c r="C178" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D178" s="81" t="n"/>
+    <row r="178" ht="28" customHeight="1">
+      <c r="B178" s="86" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C178" s="86" t="n"/>
+      <c r="D178" s="82" t="n"/>
       <c r="E178" s="82" t="n"/>
       <c r="F178" s="71" t="n"/>
     </row>
-    <row r="179" ht="26" customHeight="1">
-      <c r="B179" s="81" t="inlineStr">
-        <is>
-          <t>C.  Discourtesy</t>
-        </is>
-      </c>
-      <c r="C179" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D179" s="81" t="n"/>
+    <row r="179" ht="28" customHeight="1">
+      <c r="B179" s="86" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C179" s="86" t="n"/>
+      <c r="D179" s="82" t="n"/>
       <c r="E179" s="82" t="n"/>
       <c r="F179" s="71" t="n"/>
     </row>
-    <row r="180" ht="26" customHeight="1">
-      <c r="B180" s="81" t="inlineStr">
-        <is>
-          <t>D.  Escalation</t>
-        </is>
-      </c>
-      <c r="C180" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D180" s="81" t="n"/>
+    <row r="180" ht="28" customHeight="1">
+      <c r="B180" s="86" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C180" s="9" t="n"/>
+      <c r="D180" s="82" t="n"/>
       <c r="E180" s="82" t="n"/>
       <c r="F180" s="71" t="n"/>
     </row>
-    <row r="181" ht="26" customHeight="1">
-      <c r="B181" s="81" t="inlineStr">
-        <is>
-          <t>E.  Failure to ask for the email address</t>
-        </is>
-      </c>
-      <c r="C181" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D181" s="81" t="n"/>
-      <c r="E181" s="82" t="n"/>
-      <c r="F181" s="71" t="n"/>
-    </row>
-    <row r="182" ht="26" customHeight="1">
-      <c r="B182" s="81" t="inlineStr">
-        <is>
-          <t>F.  Fraud</t>
-        </is>
-      </c>
-      <c r="C182" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D182" s="81" t="n"/>
+    <row r="181" ht="32" customHeight="1">
+      <c r="B181" s="91" t="inlineStr">
+        <is>
+          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
+        </is>
+      </c>
+      <c r="C181" s="90" t="n"/>
+      <c r="D181" s="90" t="n"/>
+      <c r="E181" s="90" t="n"/>
+      <c r="F181" s="74" t="n"/>
+    </row>
+    <row r="182" ht="24" customHeight="1">
+      <c r="B182" s="87" t="inlineStr">
+        <is>
+          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
+        </is>
+      </c>
+      <c r="C182" s="82" t="n"/>
+      <c r="D182" s="82" t="n"/>
       <c r="E182" s="82" t="n"/>
       <c r="F182" s="71" t="n"/>
     </row>
-    <row r="183" ht="26" customHeight="1">
-      <c r="B183" s="81" t="inlineStr">
-        <is>
-          <t>G.  Hard-selling</t>
-        </is>
-      </c>
-      <c r="C183" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D183" s="81" t="n"/>
+    <row r="183" ht="58" customHeight="1">
+      <c r="B183" s="86" t="n"/>
+      <c r="C183" s="82" t="n"/>
+      <c r="D183" s="82" t="n"/>
       <c r="E183" s="82" t="n"/>
       <c r="F183" s="71" t="n"/>
     </row>
-    <row r="184" ht="26" customHeight="1">
-      <c r="B184" s="81" t="inlineStr">
-        <is>
-          <t>H.  Line Release</t>
-        </is>
-      </c>
-      <c r="C184" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D184" s="81" t="n"/>
+    <row r="184" ht="24" customHeight="1">
+      <c r="B184" s="87" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
+      <c r="C184" s="82" t="n"/>
+      <c r="D184" s="82" t="n"/>
       <c r="E184" s="82" t="n"/>
       <c r="F184" s="71" t="n"/>
     </row>
-    <row r="185" ht="26" customHeight="1">
-      <c r="B185" s="81" t="inlineStr">
-        <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C185" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D185" s="81" t="n"/>
+    <row r="185" ht="58" customHeight="1">
+      <c r="B185" s="86" t="n"/>
+      <c r="C185" s="82" t="n"/>
+      <c r="D185" s="82" t="n"/>
       <c r="E185" s="82" t="n"/>
       <c r="F185" s="71" t="n"/>
     </row>
-    <row r="186" ht="26" customHeight="1">
-      <c r="B186" s="81" t="inlineStr">
-        <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C186" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D186" s="81" t="n"/>
+    <row r="186" ht="24" customHeight="1">
+      <c r="B186" s="87" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
+      <c r="C186" s="82" t="n"/>
+      <c r="D186" s="82" t="n"/>
       <c r="E186" s="82" t="n"/>
       <c r="F186" s="71" t="n"/>
     </row>
-    <row r="187" ht="26" customHeight="1">
-      <c r="B187" s="81" t="inlineStr">
-        <is>
-          <t>K.  Non-First Call Resolution</t>
-        </is>
-      </c>
-      <c r="C187" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D187" s="81" t="n"/>
+    <row r="187" ht="58" customHeight="1">
+      <c r="B187" s="86" t="n"/>
+      <c r="C187" s="82" t="n"/>
+      <c r="D187" s="82" t="n"/>
       <c r="E187" s="82" t="n"/>
       <c r="F187" s="71" t="n"/>
     </row>
-    <row r="188" ht="24" customHeight="1">
-      <c r="B188" s="98" t="inlineStr">
-        <is>
-          <t>AUTO-ZERO TRIGGERED?</t>
-        </is>
-      </c>
-      <c r="C188" s="93">
-        <f>IF(OR(C173="No",C174="No",C175="No",COUNTIF(C177:C187,"Yes")&gt;0,COUNTIF(C157:C167,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
-      <c r="D188" s="90" t="n"/>
-      <c r="E188" s="90" t="n"/>
-      <c r="F188" s="74" t="n"/>
-    </row>
-    <row r="189" ht="58" customHeight="1">
-      <c r="B189" s="86" t="n"/>
-      <c r="C189" s="86" t="n"/>
-      <c r="D189" s="81" t="n"/>
-    </row>
-    <row r="190" ht="20" customHeight="1">
-      <c r="B190" s="96" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
-        </is>
-      </c>
-      <c r="C190" s="90" t="n"/>
-      <c r="D190" s="90" t="n"/>
-      <c r="E190" s="90" t="n"/>
-      <c r="F190" s="74" t="n"/>
-    </row>
-    <row r="191" ht="30" customHeight="1">
-      <c r="B191" s="91" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
-        </is>
-      </c>
-      <c r="C191" s="90" t="n"/>
-      <c r="D191" s="90" t="n"/>
-      <c r="E191" s="90" t="n"/>
-      <c r="F191" s="74" t="n"/>
-    </row>
-    <row r="192" ht="58" customHeight="1">
-      <c r="B192" s="86" t="n"/>
-      <c r="C192" s="82" t="n"/>
-      <c r="D192" s="82" t="n"/>
-      <c r="E192" s="82" t="n"/>
-      <c r="F192" s="71" t="n"/>
-    </row>
-    <row r="193" ht="30" customHeight="1">
-      <c r="B193" s="91" t="inlineStr">
-        <is>
-          <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
-        </is>
-      </c>
-      <c r="C193" s="90" t="n"/>
-      <c r="D193" s="90" t="n"/>
-      <c r="E193" s="90" t="n"/>
-      <c r="F193" s="74" t="n"/>
-    </row>
-    <row r="194" ht="24" customHeight="1">
-      <c r="B194" s="87" t="inlineStr">
-        <is>
-          <t>What went well — behaviors to repeat</t>
-        </is>
-      </c>
-      <c r="C194" s="82" t="n"/>
-      <c r="D194" s="82" t="n"/>
-      <c r="E194" s="82" t="n"/>
-      <c r="F194" s="71" t="n"/>
-    </row>
-    <row r="195" ht="32" customHeight="1">
-      <c r="B195" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C195" s="86" t="n"/>
-      <c r="D195" s="82" t="n"/>
-      <c r="E195" s="82" t="n"/>
-      <c r="F195" s="71" t="n"/>
-    </row>
-    <row r="196" ht="32" customHeight="1">
-      <c r="B196" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C196" s="86" t="n"/>
-      <c r="D196" s="82" t="n"/>
-      <c r="E196" s="82" t="n"/>
-      <c r="F196" s="71" t="n"/>
-    </row>
-    <row r="197" ht="32" customHeight="1">
-      <c r="B197" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C197" s="86" t="n"/>
-      <c r="D197" s="82" t="n"/>
-      <c r="E197" s="82" t="n"/>
-      <c r="F197" s="71" t="n"/>
-    </row>
-    <row r="198" ht="24" customHeight="1">
-      <c r="B198" s="87" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
-      <c r="C198" s="82" t="n"/>
-      <c r="D198" s="82" t="n"/>
-      <c r="E198" s="82" t="n"/>
-      <c r="F198" s="71" t="n"/>
-    </row>
-    <row r="199" ht="32" customHeight="1">
-      <c r="B199" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C199" s="86" t="n"/>
-      <c r="D199" s="82" t="n"/>
-      <c r="E199" s="82" t="n"/>
-      <c r="F199" s="71" t="n"/>
-    </row>
-    <row r="200" ht="32" customHeight="1">
-      <c r="B200" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C200" s="86" t="n"/>
-      <c r="D200" s="82" t="n"/>
-      <c r="E200" s="82" t="n"/>
-      <c r="F200" s="71" t="n"/>
-    </row>
-    <row r="201" ht="32" customHeight="1">
-      <c r="B201" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C201" s="86" t="n"/>
-      <c r="D201" s="82" t="n"/>
-      <c r="E201" s="82" t="n"/>
-      <c r="F201" s="71" t="n"/>
-    </row>
-    <row r="202" ht="24" customHeight="1">
-      <c r="B202" s="87" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
-      <c r="C202" s="82" t="n"/>
-      <c r="D202" s="82" t="n"/>
-      <c r="E202" s="82" t="n"/>
-      <c r="F202" s="71" t="n"/>
-    </row>
-    <row r="203" ht="58" customHeight="1">
-      <c r="B203" s="86" t="n"/>
-      <c r="C203" s="82" t="n"/>
-      <c r="D203" s="82" t="n"/>
-      <c r="E203" s="82" t="n"/>
-      <c r="F203" s="71" t="n"/>
-    </row>
-    <row r="204" ht="20" customHeight="1">
-      <c r="B204" s="87" t="inlineStr">
-        <is>
-          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
-        </is>
-      </c>
-      <c r="C204" s="82" t="n"/>
-      <c r="D204" s="82" t="n"/>
-      <c r="E204" s="82" t="n"/>
-      <c r="F204" s="71" t="n"/>
-    </row>
-    <row r="205" ht="28" customHeight="1">
-      <c r="B205" s="86" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C205" s="86" t="n"/>
-      <c r="D205" s="82" t="n"/>
-      <c r="E205" s="82" t="n"/>
-      <c r="F205" s="71" t="n"/>
-    </row>
-    <row r="206" ht="28" customHeight="1">
-      <c r="B206" s="86" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C206" s="86" t="n"/>
-      <c r="D206" s="82" t="n"/>
-      <c r="E206" s="82" t="n"/>
-      <c r="F206" s="71" t="n"/>
-    </row>
-    <row r="207" ht="28" customHeight="1">
-      <c r="B207" s="86" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" ht="32" customHeight="1">
-      <c r="B208" s="91" t="inlineStr">
-        <is>
-          <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
-        </is>
-      </c>
-      <c r="C208" s="90" t="n"/>
-      <c r="D208" s="90" t="n"/>
-      <c r="E208" s="90" t="n"/>
-      <c r="F208" s="74" t="n"/>
-    </row>
-    <row r="209" ht="24" customHeight="1">
-      <c r="B209" s="87" t="inlineStr">
-        <is>
-          <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
-        </is>
-      </c>
-      <c r="C209" s="82" t="n"/>
-      <c r="D209" s="82" t="n"/>
-      <c r="E209" s="82" t="n"/>
-      <c r="F209" s="71" t="n"/>
-    </row>
-    <row r="210" ht="58" customHeight="1">
-      <c r="B210" s="86" t="n"/>
-      <c r="C210" s="82" t="n"/>
-      <c r="D210" s="82" t="n"/>
-      <c r="E210" s="82" t="n"/>
-      <c r="F210" s="71" t="n"/>
-    </row>
-    <row r="211" ht="24" customHeight="1">
-      <c r="B211" s="87" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
-      <c r="C211" s="82" t="n"/>
-      <c r="D211" s="82" t="n"/>
-      <c r="E211" s="82" t="n"/>
-      <c r="F211" s="71" t="n"/>
-    </row>
-    <row r="212" ht="58" customHeight="1">
-      <c r="B212" s="86" t="n"/>
-      <c r="C212" s="82" t="n"/>
-      <c r="D212" s="82" t="n"/>
-      <c r="E212" s="82" t="n"/>
-      <c r="F212" s="71" t="n"/>
-    </row>
-    <row r="213" ht="24" customHeight="1">
-      <c r="B213" s="87" t="inlineStr">
-        <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
-        </is>
-      </c>
-      <c r="C213" s="82" t="n"/>
-      <c r="D213" s="82" t="n"/>
-      <c r="E213" s="82" t="n"/>
-      <c r="F213" s="71" t="n"/>
-    </row>
-    <row r="214" ht="58" customHeight="1">
-      <c r="B214" s="86" t="n"/>
-      <c r="C214" s="82" t="n"/>
-      <c r="D214" s="82" t="n"/>
-      <c r="E214" s="82" t="n"/>
-      <c r="F214" s="71" t="n"/>
-    </row>
-    <row r="215" ht="58" customHeight="1">
-      <c r="B215" s="86" t="n"/>
-    </row>
-    <row r="216" ht="24" customHeight="1">
-      <c r="B216" s="87" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
-    </row>
-    <row r="217" ht="58" customHeight="1">
-      <c r="B217" s="86" t="n"/>
-    </row>
-    <row r="218" ht="24" customHeight="1">
-      <c r="B218" s="87" t="inlineStr">
-        <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
-        </is>
-      </c>
-    </row>
-    <row r="219" ht="58" customHeight="1">
-      <c r="B219" s="86" t="n"/>
-    </row>
+    <row r="188" ht="24" customHeight="1"/>
+    <row r="189" ht="58" customHeight="1"/>
+    <row r="190" ht="20" customHeight="1"/>
+    <row r="191" ht="30" customHeight="1"/>
+    <row r="192" ht="58" customHeight="1"/>
+    <row r="193" ht="30" customHeight="1"/>
+    <row r="194" ht="24" customHeight="1"/>
+    <row r="195" ht="32" customHeight="1"/>
+    <row r="196" ht="32" customHeight="1"/>
+    <row r="197" ht="32" customHeight="1"/>
+    <row r="198" ht="24" customHeight="1"/>
+    <row r="199" ht="32" customHeight="1"/>
+    <row r="200" ht="32" customHeight="1"/>
+    <row r="201" ht="32" customHeight="1"/>
+    <row r="202" ht="24" customHeight="1"/>
+    <row r="203" ht="58" customHeight="1"/>
+    <row r="204" ht="20" customHeight="1"/>
+    <row r="205" ht="28" customHeight="1"/>
+    <row r="206" ht="28" customHeight="1"/>
+    <row r="207" ht="28" customHeight="1"/>
+    <row r="208" ht="32" customHeight="1"/>
+    <row r="209" ht="24" customHeight="1"/>
+    <row r="210" ht="58" customHeight="1"/>
+    <row r="211" ht="24" customHeight="1"/>
+    <row r="212" ht="58" customHeight="1"/>
+    <row r="213" ht="24" customHeight="1"/>
+    <row r="214" ht="58" customHeight="1"/>
+    <row r="215" ht="58" customHeight="1"/>
+    <row r="216" ht="24" customHeight="1"/>
+    <row r="217" ht="58" customHeight="1"/>
+    <row r="218" ht="24" customHeight="1"/>
+    <row r="219" ht="58" customHeight="1"/>
   </sheetData>
-  <mergeCells count="190">
-    <mergeCell ref="D76:F76"/>
-    <mergeCell ref="B194:F194"/>
-    <mergeCell ref="B209:F209"/>
+  <mergeCells count="178">
+    <mergeCell ref="B106:F106"/>
+    <mergeCell ref="D116:F116"/>
+    <mergeCell ref="C122:F122"/>
     <mergeCell ref="B81:F81"/>
-    <mergeCell ref="D179:F179"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B68:E68"/>
     <mergeCell ref="D66:F66"/>
-    <mergeCell ref="D166:F166"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="B131:F131"/>
-    <mergeCell ref="B214:F214"/>
+    <mergeCell ref="D75:F75"/>
+    <mergeCell ref="C125:F125"/>
+    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B36:E36"/>
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="D181:F181"/>
-    <mergeCell ref="C78:F78"/>
-    <mergeCell ref="E153:F153"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="D37:F37"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
-    <mergeCell ref="C62:F62"/>
-    <mergeCell ref="D165:F165"/>
-    <mergeCell ref="D92:F92"/>
-    <mergeCell ref="B170:F170"/>
-    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="B92:C93"/>
     <mergeCell ref="D152:F152"/>
-    <mergeCell ref="C107:F107"/>
+    <mergeCell ref="B166:F166"/>
+    <mergeCell ref="C172:F172"/>
+    <mergeCell ref="D133:F133"/>
     <mergeCell ref="B44:F44"/>
-    <mergeCell ref="D133:F133"/>
     <mergeCell ref="D142:F142"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B108:F108"/>
-    <mergeCell ref="D119:F119"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="B186:F186"/>
+    <mergeCell ref="C173:F173"/>
+    <mergeCell ref="D128:F128"/>
     <mergeCell ref="D159:F159"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="D186:F186"/>
-    <mergeCell ref="B213:F213"/>
-    <mergeCell ref="D183:F183"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B94:F94"/>
     <mergeCell ref="D105:F105"/>
-    <mergeCell ref="C207:F207"/>
     <mergeCell ref="D57:F57"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B144:F144"/>
+    <mergeCell ref="C17:F17"/>
     <mergeCell ref="D120:F120"/>
-    <mergeCell ref="D185:F185"/>
     <mergeCell ref="D41:F41"/>
-    <mergeCell ref="B125:F125"/>
-    <mergeCell ref="D163:F163"/>
-    <mergeCell ref="C149:F149"/>
-    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="D154:F154"/>
+    <mergeCell ref="B185:F185"/>
+    <mergeCell ref="D107:F107"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="B208:F208"/>
+    <mergeCell ref="C67:F67"/>
     <mergeCell ref="C19:F19"/>
-    <mergeCell ref="D162:F162"/>
-    <mergeCell ref="C199:F199"/>
-    <mergeCell ref="D43:F43"/>
+    <mergeCell ref="D147:F147"/>
     <mergeCell ref="D156:F156"/>
+    <mergeCell ref="B167:F167"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B176:F176"/>
     <mergeCell ref="D137:F137"/>
-    <mergeCell ref="D106:F106"/>
-    <mergeCell ref="B210:F210"/>
     <mergeCell ref="B111:F111"/>
-    <mergeCell ref="D93:F93"/>
+    <mergeCell ref="C96:F96"/>
+    <mergeCell ref="D146:F146"/>
     <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
-    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="D117:F117"/>
     <mergeCell ref="D157:F157"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D67:F67"/>
     <mergeCell ref="B171:F171"/>
-    <mergeCell ref="C200:F200"/>
     <mergeCell ref="D132:F132"/>
     <mergeCell ref="D85:F85"/>
-    <mergeCell ref="C147:F147"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="B146:F146"/>
+    <mergeCell ref="C162:F162"/>
     <mergeCell ref="D60:F60"/>
-    <mergeCell ref="D182:F182"/>
-    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="B99:F99"/>
     <mergeCell ref="D100:F100"/>
-    <mergeCell ref="B109:C110"/>
-    <mergeCell ref="D174:F174"/>
+    <mergeCell ref="B187:F187"/>
+    <mergeCell ref="C124:F124"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D46:F46"/>
-    <mergeCell ref="C201:F201"/>
+    <mergeCell ref="D158:F158"/>
     <mergeCell ref="D40:F40"/>
-    <mergeCell ref="C148:F148"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="D158:F158"/>
-    <mergeCell ref="B204:F204"/>
-    <mergeCell ref="C188:F188"/>
-    <mergeCell ref="B198:F198"/>
+    <mergeCell ref="C90:F90"/>
+    <mergeCell ref="B76:F76"/>
+    <mergeCell ref="D108:F108"/>
     <mergeCell ref="D86:F86"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B75:F75"/>
+    <mergeCell ref="D104:F104"/>
     <mergeCell ref="D160:F160"/>
     <mergeCell ref="D136:F136"/>
-    <mergeCell ref="B59:F59"/>
-    <mergeCell ref="B193:F193"/>
-    <mergeCell ref="B190:F190"/>
-    <mergeCell ref="B202:F202"/>
+    <mergeCell ref="D150:F150"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="C174:F174"/>
     <mergeCell ref="B80:E80"/>
-    <mergeCell ref="D87:F87"/>
+    <mergeCell ref="D78:F78"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="D122:F122"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="B39:F39"/>
     <mergeCell ref="D71:F71"/>
-    <mergeCell ref="D184:F184"/>
+    <mergeCell ref="B54:E54"/>
     <mergeCell ref="D58:F58"/>
+    <mergeCell ref="C179:F179"/>
+    <mergeCell ref="B145:F145"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="D121:F121"/>
-    <mergeCell ref="D177:F177"/>
+    <mergeCell ref="B181:F181"/>
+    <mergeCell ref="C129:D129"/>
     <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D164:F164"/>
-    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D51:F51"/>
     <mergeCell ref="D82:F82"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D113:F113"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="D173:F173"/>
-    <mergeCell ref="B191:F191"/>
-    <mergeCell ref="C128:F128"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="D123:F123"/>
-    <mergeCell ref="C113:F113"/>
+    <mergeCell ref="B87:F87"/>
+    <mergeCell ref="C97:F97"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="D148:F148"/>
+    <mergeCell ref="D35:F35"/>
     <mergeCell ref="C143:F143"/>
-    <mergeCell ref="C112:F112"/>
-    <mergeCell ref="C205:F205"/>
-    <mergeCell ref="C94:F94"/>
-    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="C109:F109"/>
+    <mergeCell ref="D115:F115"/>
     <mergeCell ref="D138:F138"/>
-    <mergeCell ref="D178:F178"/>
-    <mergeCell ref="D172:F172"/>
-    <mergeCell ref="D187:F187"/>
-    <mergeCell ref="B65:F65"/>
-    <mergeCell ref="D99:F99"/>
-    <mergeCell ref="B192:F192"/>
-    <mergeCell ref="C114:F114"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="B183:F183"/>
+    <mergeCell ref="B164:F164"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D84:F84"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="D155:F155"/>
+    <mergeCell ref="D140:F140"/>
+    <mergeCell ref="D36:F36"/>
+    <mergeCell ref="D149:F149"/>
     <mergeCell ref="D45:F45"/>
-    <mergeCell ref="B212:F212"/>
+    <mergeCell ref="B123:F123"/>
     <mergeCell ref="D101:F101"/>
+    <mergeCell ref="C95:F95"/>
+    <mergeCell ref="C178:F178"/>
+    <mergeCell ref="B163:F163"/>
     <mergeCell ref="B50:F50"/>
-    <mergeCell ref="D124:F124"/>
-    <mergeCell ref="B203:F203"/>
     <mergeCell ref="D77:F77"/>
     <mergeCell ref="B91:F91"/>
+    <mergeCell ref="D151:F151"/>
     <mergeCell ref="D61:F61"/>
-    <mergeCell ref="D126:F126"/>
+    <mergeCell ref="B165:F165"/>
     <mergeCell ref="D141:F141"/>
     <mergeCell ref="D70:F70"/>
     <mergeCell ref="D135:F135"/>
-    <mergeCell ref="D175:F175"/>
-    <mergeCell ref="B155:F155"/>
-    <mergeCell ref="B140:F140"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="C170:F170"/>
     <mergeCell ref="D103:F103"/>
     <mergeCell ref="D72:F72"/>
     <mergeCell ref="D134:F134"/>
-    <mergeCell ref="B117:F117"/>
+    <mergeCell ref="B130:F130"/>
+    <mergeCell ref="D112:F112"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="D180:F180"/>
-    <mergeCell ref="B151:F151"/>
+    <mergeCell ref="D62:F62"/>
     <mergeCell ref="D118:F118"/>
     <mergeCell ref="D56:F56"/>
-    <mergeCell ref="C195:F195"/>
-    <mergeCell ref="D167:F167"/>
-    <mergeCell ref="D127:F127"/>
     <mergeCell ref="D161:F161"/>
-    <mergeCell ref="D176:F176"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="D114:F114"/>
+    <mergeCell ref="C42:F42"/>
     <mergeCell ref="E9:F9"/>
+    <mergeCell ref="B119:F119"/>
     <mergeCell ref="D38:F38"/>
-    <mergeCell ref="D98:F98"/>
+    <mergeCell ref="C126:F126"/>
     <mergeCell ref="D89:F89"/>
-    <mergeCell ref="C197:F197"/>
-    <mergeCell ref="C206:F206"/>
-    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B69:F69"/>
+    <mergeCell ref="B182:F182"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="D88:F88"/>
-    <mergeCell ref="C196:F196"/>
+    <mergeCell ref="D153:F153"/>
+    <mergeCell ref="B127:F127"/>
     <mergeCell ref="C168:F168"/>
-    <mergeCell ref="B211:F211"/>
-    <mergeCell ref="C153:D153"/>
-    <mergeCell ref="D90:F90"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B104:F104"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="C180:F180"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="B177:F177"/>
+    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D131:F131"/>
     <mergeCell ref="D139:F139"/>
     <mergeCell ref="D52:F52"/>
-    <mergeCell ref="B97:F97"/>
-    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="C169:F169"/>
+    <mergeCell ref="D49:F49"/>
   </mergeCells>
   <conditionalFormatting sqref="C20:C24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
@@ -6238,37 +6099,37 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C39 C40 C41 C42 C52 C53 C54 C56 C67 C68 C69 C70 C72 C73 C74 C83 C85 C87 C88 C89 C99 C100 C101 C103 C119 C120 C121 C123 C124 C133 C134 C135 C136 C138 C139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C57 C58 C59 C60 C61 C62 C63 C71 C72 C73 C74 C75 C83 C84 C85 C86 C101 C102 C103 C104 C105 C113 C114 C115 C116 C117 C118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C46 C61 C77 C93 C106 C127 C142" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
+    <dataValidation sqref="C41 C52 C66 C78 C89 C108 C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C152 C157:C167 C177:C187 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C128 C132:C142 C151:C161 E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
-    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-Warranty,Out-of-Warranty,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="E7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Phone,Chat,Email,Social,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Technical Issue,Setup/How-To,RMA/Replacement,Billing/Account,Connectivity,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Within SLA,Breached,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Successful Resolution,Partial Resolution,Appropriate Escalation,Ownership Gap,Unresolved"</formula1>
     </dataValidation>
-    <dataValidation sqref="C148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_xlfn._LONGTEXT("Issue resolved,Proper RMA initiated (in-warranty / approved exception),Valid escalation submitted,Known limitation explained accurately,Customer educated with actionable next steps,Valid self-help guidance provided (out-of-warranty),Upgrade path recommend","ed appropriately (out-of-warranty),Customer declined further troubleshooting after reasonable effort,None achieved")</formula1>
     </dataValidation>
-    <dataValidation sqref="C153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C173:C175" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C147:C149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
     </dataValidation>
   </dataValidations>
@@ -12600,13 +12461,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Implement item 3: update Ownership §4 rows 73-74
Row 73 (was 'Next actions were documented'):
  → 'All required actions as part of the solution and next steps
     were clearly articulated and documented'

Row 74 (was 'Realistic expectations were set'):
  → 'Clearly explained realistic next steps to the customer'

Distinction: row 73 covers internal articulation and documentation of
actions; row 74 covers the customer-facing explanation of what to expect.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4247,7 +4247,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="B73" s="81" t="inlineStr">
         <is>
-          <t>Next actions were documented</t>
+          <t>All required actions as part of the solution and next steps were clearly articulated and documented</t>
         </is>
       </c>
       <c r="C73" s="9" t="n"/>
@@ -4258,7 +4258,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="B74" s="83" t="inlineStr">
         <is>
-          <t>Realistic expectations were set</t>
+          <t>Clearly explained realistic next steps to the customer</t>
         </is>
       </c>
       <c r="C74" s="9" t="n"/>
@@ -12461,13 +12461,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Option B: remove redundant Ownership row 73, reword row 74
Row 73 ('All required actions... articulated and documented') removed —
the documentation of next steps is already covered by §7 Documentation
row 117 ('Documented next steps and follow-ups'), making it redundant
across sections.

Row 74 reworded to 'Clearly set customer expectations for next steps
and realistic timelines' — keeps Customer Ownership focused on
accountability and what the customer was told, not on case notes.

DV updated: 34 → 33 active cells (C73 removed).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4245,11 +4245,7 @@
       <c r="F72" s="71" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1">
-      <c r="B73" s="81" t="inlineStr">
-        <is>
-          <t>All required actions as part of the solution and next steps were clearly articulated and documented</t>
-        </is>
-      </c>
+      <c r="B73" s="81" t="n"/>
       <c r="C73" s="9" t="n"/>
       <c r="D73" s="81" t="n"/>
       <c r="E73" s="82" t="n"/>
@@ -4258,7 +4254,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="B74" s="83" t="inlineStr">
         <is>
-          <t>Clearly explained realistic next steps to the customer</t>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
         </is>
       </c>
       <c r="C74" s="9" t="n"/>
@@ -6099,7 +6095,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C57 C58 C59 C60 C61 C62 C63 C71 C72 C73 C74 C75 C83 C84 C85 C86 C101 C102 C103 C104 C105 C113 C114 C115 C116 C117 C118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C57 C58 C59 C60 C61 C62 C63 C71 C72 C74 C75 C83 C84 C85 C86 C101 C102 C103 C104 C105 C113 C114 C115 C116 C117 C118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C41 C52 C66 C78 C89 C108 C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
@@ -12461,13 +12457,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Split Technical Accuracy merged indicator back into two; fix Score Summary
Split row 48 back into:
- Row 48: 'Followed a logical troubleshooting process'
- Row 49: 'Available tools were used efficiently and appropriately'
These measure different behaviors: methodology quality vs. tool usage.

Fixed 8 Score Summary formulas that were off by 1 after the row insert:
- D24–D29 (effective score refs for Technical through Documentation)
- E30 (weighted total: gates C148:C150, A-K C152:C162, CFC C133:C143)
- F30 (performance band: same condition refs as E30)
- C52 auto-score COUNTIF range corrected to C46:C50 (all 5 indicators)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -3232,7 +3232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F187"/>
+  <dimension ref="B1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3574,7 +3574,7 @@
         <v>0.2</v>
       </c>
       <c r="D24" s="23">
-        <f>IF(C52="",C51,C52)</f>
+        <f>IF(C53="",C52,C53)</f>
         <v/>
       </c>
       <c r="E24" s="24">
@@ -3596,7 +3596,7 @@
         <v>0.15</v>
       </c>
       <c r="D25" s="18">
-        <f>IF(C66="",C65,C66)</f>
+        <f>IF(C67="",C66,C67)</f>
         <v/>
       </c>
       <c r="E25" s="19">
@@ -3618,7 +3618,7 @@
         <v>0.15</v>
       </c>
       <c r="D26" s="23">
-        <f>IF(C78="",C77,C78)</f>
+        <f>IF(C79="",C78,C79)</f>
         <v/>
       </c>
       <c r="E26" s="24">
@@ -3640,7 +3640,7 @@
         <v>0.1</v>
       </c>
       <c r="D27" s="18">
-        <f>IF(C89="",C88,C89)</f>
+        <f>IF(C90="",C89,C90)</f>
         <v/>
       </c>
       <c r="E27" s="19">
@@ -3662,7 +3662,7 @@
         <v>0.05</v>
       </c>
       <c r="D28" s="23">
-        <f>IF(C108="",C107,C108)</f>
+        <f>IF(C109="",C108,C109)</f>
         <v/>
       </c>
       <c r="E28" s="24">
@@ -3684,7 +3684,7 @@
         <v>0.05</v>
       </c>
       <c r="D29" s="18">
-        <f>IF(C121="",C120,C121)</f>
+        <f>IF(C122="",C121,C122)</f>
         <v/>
       </c>
       <c r="E29" s="19">
@@ -3708,11 +3708,11 @@
       </c>
       <c r="D30" s="27" t="n"/>
       <c r="E30" s="28">
-        <f>IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),0,SUM(E23:E29))</f>
+        <f>IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0,COUNTIF(C133:C143,"Yes")&gt;0),0,SUM(E23:E29))</f>
         <v/>
       </c>
       <c r="F30" s="29">
-        <f>IF(E30="","",IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E30&gt;=0.85,"MEETS / EXCEEDS",IF(E30&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
+        <f>IF(E30="","",IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0,COUNTIF(C133:C143,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E30&gt;=0.85,"MEETS / EXCEEDS",IF(E30&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
         <v/>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
     <row r="48" ht="28" customHeight="1">
       <c r="B48" s="81" t="inlineStr">
         <is>
-          <t>Followed a logical troubleshooting process, and available tools were used, efficiently and appropriately.</t>
+          <t>Followed a logical troubleshooting process</t>
         </is>
       </c>
       <c r="C48" s="9" t="n"/>
@@ -3947,157 +3947,155 @@
     <row r="49" ht="28" customHeight="1">
       <c r="B49" s="81" t="inlineStr">
         <is>
-          <t>Gave technically accurate information; no unsupported conclusions</t>
+          <t>Available tools were used efficiently and appropriately</t>
         </is>
       </c>
       <c r="C49" s="9" t="n"/>
       <c r="D49" s="81" t="n"/>
-      <c r="E49" s="82" t="n"/>
-      <c r="F49" s="71" t="n"/>
     </row>
     <row r="50" ht="28" customHeight="1">
-      <c r="B50" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
-        </is>
-      </c>
-      <c r="C50" s="82" t="n"/>
-      <c r="D50" s="82" t="n"/>
+      <c r="B50" s="81" t="inlineStr">
+        <is>
+          <t>Gave technically accurate information; no unsupported conclusions</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="81" t="n"/>
       <c r="E50" s="82" t="n"/>
       <c r="F50" s="71" t="n"/>
     </row>
     <row r="51" ht="28" customHeight="1">
-      <c r="B51" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C51" s="122">
-        <f>IF((COUNTIF(C46:C49,"Met")+COUNTIF(C46:C49,"Partial")+COUNTIF(C46:C49,"Missed"))=0,"",ROUND((COUNTIF(C46:C49,"Met")*5+COUNTIF(C46:C49,"Partial")*2.5)/(COUNTIF(C46:C49,"Met")+COUNTIF(C46:C49,"Partial")+COUNTIF(C46:C49,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D51" s="92" t="n"/>
+      <c r="B51" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
+        </is>
+      </c>
+      <c r="C51" s="82" t="n"/>
+      <c r="D51" s="82" t="n"/>
       <c r="E51" s="82" t="n"/>
       <c r="F51" s="71" t="n"/>
     </row>
-    <row r="52" ht="24" customHeight="1">
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C52" s="14" t="n"/>
-      <c r="D52" s="84">
-        <f>IF(IF(C52="",C51,C52)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C52="",C51,C52)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="52" ht="28" customHeight="1">
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C52" s="122">
+        <f>IF((COUNTIF(C46:C50,"Met")+COUNTIF(C46:C50,"Partial")+COUNTIF(C46:C50,"Missed"))=0,"",ROUND((COUNTIF(C46:C50,"Met")*5+COUNTIF(C46:C50,"Partial")*2.5)/(COUNTIF(C46:C50,"Met")+COUNTIF(C46:C50,"Partial")+COUNTIF(C46:C50,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D52" s="92" t="n"/>
       <c r="E52" s="82" t="n"/>
       <c r="F52" s="71" t="n"/>
     </row>
-    <row r="53" ht="36" customHeight="1">
+    <row r="53" ht="24" customHeight="1">
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
-        </is>
-      </c>
-      <c r="C53" s="86" t="n"/>
-      <c r="D53" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="84">
+        <f>IF(IF(C53="",C52,C53)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C53="",C52,C53)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E53" s="82" t="n"/>
       <c r="F53" s="71" t="n"/>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="B54" s="80" t="inlineStr">
+    <row r="54" ht="36" customHeight="1">
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
+        </is>
+      </c>
+      <c r="C54" s="86" t="n"/>
+      <c r="D54" s="82" t="n"/>
+      <c r="E54" s="82" t="n"/>
+      <c r="F54" s="71" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="B55" s="80" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
       </c>
-      <c r="C54" s="90" t="n"/>
-      <c r="D54" s="90" t="n"/>
-      <c r="E54" s="74" t="n"/>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="C55" s="90" t="n"/>
+      <c r="D55" s="90" t="n"/>
+      <c r="E55" s="74" t="n"/>
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Weight: 15%</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="B55" s="121" t="inlineStr">
+    <row r="56" ht="28" customHeight="1">
+      <c r="B56" s="121" t="inlineStr">
         <is>
           <t>Objective: Evaluate how effectively the agent managed the interaction.</t>
         </is>
       </c>
-      <c r="C55" s="82" t="n"/>
-      <c r="D55" s="82" t="n"/>
-      <c r="E55" s="82" t="n"/>
-      <c r="F55" s="71" t="n"/>
-    </row>
-    <row r="56" ht="24" customHeight="1">
-      <c r="B56" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D56" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C56" s="82" t="n"/>
+      <c r="D56" s="82" t="n"/>
       <c r="E56" s="82" t="n"/>
       <c r="F56" s="71" t="n"/>
     </row>
-    <row r="57" ht="28" customHeight="1">
-      <c r="B57" s="81" t="inlineStr">
-        <is>
-          <t>Expectations were set clearly from the start</t>
-        </is>
-      </c>
-      <c r="C57" s="9" t="n"/>
-      <c r="D57" s="81" t="n"/>
+    <row r="57" ht="24" customHeight="1">
+      <c r="B57" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D57" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E57" s="82" t="n"/>
       <c r="F57" s="71" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="B58" s="83" t="inlineStr">
-        <is>
-          <t>Agent maintained call control and troubleshooting flow</t>
+      <c r="B58" s="81" t="inlineStr">
+        <is>
+          <t>Expectations were set clearly from the start</t>
         </is>
       </c>
       <c r="C58" s="9" t="n"/>
-      <c r="D58" s="83" t="n"/>
+      <c r="D58" s="81" t="n"/>
       <c r="E58" s="82" t="n"/>
       <c r="F58" s="71" t="n"/>
     </row>
     <row r="59" ht="28" customHeight="1">
-      <c r="B59" s="81" t="inlineStr">
-        <is>
-          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+      <c r="B59" s="83" t="inlineStr">
+        <is>
+          <t>Agent maintained call control and troubleshooting flow</t>
         </is>
       </c>
       <c r="C59" s="9" t="n"/>
-      <c r="D59" s="81" t="n"/>
+      <c r="D59" s="83" t="n"/>
       <c r="E59" s="82" t="n"/>
       <c r="F59" s="71" t="n"/>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="B60" s="83" t="inlineStr">
-        <is>
-          <t>Actively listened and showed comprehension throughout the interaction/s</t>
+      <c r="B60" s="81" t="inlineStr">
+        <is>
+          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
         </is>
       </c>
       <c r="C60" s="9" t="n"/>
-      <c r="D60" s="83" t="n"/>
+      <c r="D60" s="81" t="n"/>
       <c r="E60" s="82" t="n"/>
       <c r="F60" s="71" t="n"/>
     </row>
     <row r="61" ht="28" customHeight="1">
       <c r="B61" s="83" t="inlineStr">
         <is>
-          <t>Managed time well, with clear transitions between steps</t>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
         </is>
       </c>
       <c r="C61" s="9" t="n"/>
@@ -4106,137 +4104,137 @@
       <c r="F61" s="71" t="n"/>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="B62" s="81" t="inlineStr">
-        <is>
-          <t>Handled difficult moments when needed to maintain call control</t>
+      <c r="B62" s="83" t="inlineStr">
+        <is>
+          <t>Managed time well, with clear transitions between steps</t>
         </is>
       </c>
       <c r="C62" s="9" t="n"/>
-      <c r="D62" s="81" t="n"/>
+      <c r="D62" s="83" t="n"/>
       <c r="E62" s="82" t="n"/>
       <c r="F62" s="71" t="n"/>
     </row>
     <row r="63" ht="28" customHeight="1">
-      <c r="B63" s="83" t="inlineStr">
-        <is>
-          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+      <c r="B63" s="81" t="inlineStr">
+        <is>
+          <t>Handled difficult moments when needed to maintain call control</t>
         </is>
       </c>
       <c r="C63" s="9" t="n"/>
-      <c r="D63" s="83" t="n"/>
+      <c r="D63" s="81" t="n"/>
       <c r="E63" s="82" t="n"/>
       <c r="F63" s="71" t="n"/>
     </row>
     <row r="64" ht="28" customHeight="1">
-      <c r="B64" s="85" t="inlineStr">
-        <is>
-          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
-        </is>
-      </c>
-      <c r="C64" s="82" t="n"/>
-      <c r="D64" s="82" t="n"/>
+      <c r="B64" s="83" t="inlineStr">
+        <is>
+          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="n"/>
+      <c r="D64" s="83" t="n"/>
       <c r="E64" s="82" t="n"/>
       <c r="F64" s="71" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C65" s="122">
-        <f>IF((COUNTIF(C57:C63,"Met")+COUNTIF(C57:C63,"Partial")+COUNTIF(C57:C63,"Missed"))=0,"",ROUND((COUNTIF(C57:C63,"Met")*5+COUNTIF(C57:C63,"Partial")*2.5)/(COUNTIF(C57:C63,"Met")+COUNTIF(C57:C63,"Partial")+COUNTIF(C57:C63,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D65" s="92" t="n"/>
+      <c r="B65" s="85" t="inlineStr">
+        <is>
+          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
+        </is>
+      </c>
+      <c r="C65" s="82" t="n"/>
+      <c r="D65" s="82" t="n"/>
       <c r="E65" s="82" t="n"/>
       <c r="F65" s="71" t="n"/>
     </row>
-    <row r="66" ht="24" customHeight="1">
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C66" s="14" t="n"/>
-      <c r="D66" s="84">
-        <f>IF(IF(C66="",C65,C66)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C66="",C65,C66)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="66" ht="28" customHeight="1">
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C66" s="122">
+        <f>IF((COUNTIF(C58:C64,"Met")+COUNTIF(C58:C64,"Partial")+COUNTIF(C58:C64,"Missed"))=0,"",ROUND((COUNTIF(C58:C64,"Met")*5+COUNTIF(C58:C64,"Partial")*2.5)/(COUNTIF(C58:C64,"Met")+COUNTIF(C58:C64,"Partial")+COUNTIF(C58:C64,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D66" s="92" t="n"/>
       <c r="E66" s="82" t="n"/>
       <c r="F66" s="71" t="n"/>
     </row>
-    <row r="67" ht="36" customHeight="1">
+    <row r="67" ht="24" customHeight="1">
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
-        </is>
-      </c>
-      <c r="C67" s="86" t="n"/>
-      <c r="D67" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="n"/>
+      <c r="D67" s="84">
+        <f>IF(IF(C67="",C66,C67)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C67="",C66,C67)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E67" s="82" t="n"/>
       <c r="F67" s="71" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="B68" s="80" t="inlineStr">
+    <row r="68" ht="36" customHeight="1">
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
+        </is>
+      </c>
+      <c r="C68" s="86" t="n"/>
+      <c r="D68" s="82" t="n"/>
+      <c r="E68" s="82" t="n"/>
+      <c r="F68" s="71" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="B69" s="80" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
       </c>
-      <c r="C68" s="90" t="n"/>
-      <c r="D68" s="90" t="n"/>
-      <c r="E68" s="74" t="n"/>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="C69" s="90" t="n"/>
+      <c r="D69" s="90" t="n"/>
+      <c r="E69" s="74" t="n"/>
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>Weight: 15%</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="28" customHeight="1">
-      <c r="B69" s="121" t="inlineStr">
+    <row r="70" ht="28" customHeight="1">
+      <c r="B70" s="121" t="inlineStr">
         <is>
           <t>Objective: Measure the degree to which the agent accepted responsibility for moving the customer forward.</t>
         </is>
       </c>
-      <c r="C69" s="82" t="n"/>
-      <c r="D69" s="82" t="n"/>
-      <c r="E69" s="82" t="n"/>
-      <c r="F69" s="71" t="n"/>
-    </row>
-    <row r="70" ht="24" customHeight="1">
-      <c r="B70" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D70" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C70" s="82" t="n"/>
+      <c r="D70" s="82" t="n"/>
       <c r="E70" s="82" t="n"/>
       <c r="F70" s="71" t="n"/>
     </row>
-    <row r="71" ht="28" customHeight="1">
-      <c r="B71" s="81" t="inlineStr">
-        <is>
-          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="n"/>
-      <c r="D71" s="81" t="n"/>
+    <row r="71" ht="24" customHeight="1">
+      <c r="B71" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D71" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E71" s="82" t="n"/>
       <c r="F71" s="71" t="n"/>
     </row>
     <row r="72" ht="28" customHeight="1">
       <c r="B72" s="81" t="inlineStr">
         <is>
-          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
         </is>
       </c>
       <c r="C72" s="9" t="n"/>
@@ -4245,166 +4243,166 @@
       <c r="F72" s="71" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1">
-      <c r="B73" s="81" t="n"/>
+      <c r="B73" s="81" t="inlineStr">
+        <is>
+          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+        </is>
+      </c>
       <c r="C73" s="9" t="n"/>
       <c r="D73" s="81" t="n"/>
       <c r="E73" s="82" t="n"/>
       <c r="F73" s="71" t="n"/>
     </row>
     <row r="74" ht="28" customHeight="1">
-      <c r="B74" s="83" t="inlineStr">
-        <is>
-          <t>Clearly set customer expectations for next steps and realistic timelines</t>
-        </is>
-      </c>
+      <c r="B74" s="81" t="n"/>
       <c r="C74" s="9" t="n"/>
-      <c r="D74" s="83" t="n"/>
+      <c r="D74" s="81" t="n"/>
       <c r="E74" s="82" t="n"/>
       <c r="F74" s="71" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1">
-      <c r="B75" s="81" t="inlineStr">
-        <is>
-          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+      <c r="B75" s="83" t="inlineStr">
+        <is>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
         </is>
       </c>
       <c r="C75" s="9" t="n"/>
-      <c r="D75" s="81" t="n"/>
+      <c r="D75" s="83" t="n"/>
       <c r="E75" s="82" t="n"/>
       <c r="F75" s="71" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1">
-      <c r="B76" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
-        </is>
-      </c>
-      <c r="C76" s="82" t="n"/>
-      <c r="D76" s="82" t="n"/>
+      <c r="B76" s="81" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="n"/>
+      <c r="D76" s="81" t="n"/>
       <c r="E76" s="82" t="n"/>
       <c r="F76" s="71" t="n"/>
     </row>
     <row r="77" ht="28" customHeight="1">
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C77" s="122">
-        <f>IF((COUNTIF(C71:C75,"Met")+COUNTIF(C71:C75,"Partial")+COUNTIF(C71:C75,"Missed"))=0,"",ROUND((COUNTIF(C71:C75,"Met")*5+COUNTIF(C71:C75,"Partial")*2.5)/(COUNTIF(C71:C75,"Met")+COUNTIF(C71:C75,"Partial")+COUNTIF(C71:C75,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D77" s="92" t="n"/>
+      <c r="B77" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
+        </is>
+      </c>
+      <c r="C77" s="82" t="n"/>
+      <c r="D77" s="82" t="n"/>
       <c r="E77" s="82" t="n"/>
       <c r="F77" s="71" t="n"/>
     </row>
-    <row r="78" ht="24" customHeight="1">
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C78" s="14" t="n"/>
-      <c r="D78" s="84">
-        <f>IF(IF(C78="",C77,C78)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C78="",C77,C78)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="78" ht="28" customHeight="1">
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C78" s="122">
+        <f>IF((COUNTIF(C72:C76,"Met")+COUNTIF(C72:C76,"Partial")+COUNTIF(C72:C76,"Missed"))=0,"",ROUND((COUNTIF(C72:C76,"Met")*5+COUNTIF(C72:C76,"Partial")*2.5)/(COUNTIF(C72:C76,"Met")+COUNTIF(C72:C76,"Partial")+COUNTIF(C72:C76,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D78" s="92" t="n"/>
       <c r="E78" s="82" t="n"/>
       <c r="F78" s="71" t="n"/>
     </row>
-    <row r="79" ht="36" customHeight="1">
+    <row r="79" ht="24" customHeight="1">
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
-        </is>
-      </c>
-      <c r="C79" s="86" t="n"/>
-      <c r="D79" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C79" s="14" t="n"/>
+      <c r="D79" s="84">
+        <f>IF(IF(C79="",C78,C79)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C79="",C78,C79)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E79" s="82" t="n"/>
       <c r="F79" s="71" t="n"/>
     </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="B80" s="80" t="inlineStr">
+    <row r="80" ht="36" customHeight="1">
+      <c r="B80" s="13" t="inlineStr">
+        <is>
+          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
+        </is>
+      </c>
+      <c r="C80" s="86" t="n"/>
+      <c r="D80" s="82" t="n"/>
+      <c r="E80" s="82" t="n"/>
+      <c r="F80" s="71" t="n"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="B81" s="80" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
       </c>
-      <c r="C80" s="90" t="n"/>
-      <c r="D80" s="90" t="n"/>
-      <c r="E80" s="74" t="n"/>
-      <c r="F80" s="6" t="inlineStr">
+      <c r="C81" s="90" t="n"/>
+      <c r="D81" s="90" t="n"/>
+      <c r="E81" s="74" t="n"/>
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <t>Weight: 10%</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="28" customHeight="1">
-      <c r="B81" s="121" t="inlineStr">
+    <row r="82" ht="28" customHeight="1">
+      <c r="B82" s="121" t="inlineStr">
         <is>
           <t>Objective: Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted.</t>
         </is>
       </c>
-      <c r="C81" s="82" t="n"/>
-      <c r="D81" s="82" t="n"/>
-      <c r="E81" s="82" t="n"/>
-      <c r="F81" s="71" t="n"/>
-    </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="B82" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D82" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C82" s="82" t="n"/>
+      <c r="D82" s="82" t="n"/>
       <c r="E82" s="82" t="n"/>
       <c r="F82" s="71" t="n"/>
     </row>
-    <row r="83" ht="28" customHeight="1">
-      <c r="B83" s="81" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before escalating</t>
-        </is>
-      </c>
-      <c r="C83" s="9" t="n"/>
-      <c r="D83" s="81" t="n"/>
+    <row r="83" ht="18" customHeight="1">
+      <c r="B83" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D83" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E83" s="82" t="n"/>
       <c r="F83" s="71" t="n"/>
     </row>
     <row r="84" ht="28" customHeight="1">
-      <c r="B84" s="83" t="inlineStr">
-        <is>
-          <t>Identified a valid reason to escalate</t>
+      <c r="B84" s="81" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before escalating</t>
         </is>
       </c>
       <c r="C84" s="9" t="n"/>
-      <c r="D84" s="83" t="n"/>
+      <c r="D84" s="81" t="n"/>
       <c r="E84" s="82" t="n"/>
       <c r="F84" s="71" t="n"/>
     </row>
     <row r="85" ht="28" customHeight="1">
-      <c r="B85" s="81" t="inlineStr">
-        <is>
-          <t>Provided complete escalation details using the correct escalation path</t>
+      <c r="B85" s="83" t="inlineStr">
+        <is>
+          <t>Identified a valid reason to escalate</t>
         </is>
       </c>
       <c r="C85" s="9" t="n"/>
-      <c r="D85" s="81" t="n"/>
+      <c r="D85" s="83" t="n"/>
       <c r="E85" s="82" t="n"/>
       <c r="F85" s="71" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1">
       <c r="B86" s="81" t="inlineStr">
         <is>
-          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+          <t>Provided complete escalation details using the correct escalation path</t>
         </is>
       </c>
       <c r="C86" s="9" t="n"/>
@@ -4413,107 +4411,107 @@
       <c r="F86" s="71" t="n"/>
     </row>
     <row r="87" ht="28" customHeight="1">
-      <c r="B87" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
-        </is>
-      </c>
-      <c r="C87" s="82" t="n"/>
-      <c r="D87" s="82" t="n"/>
+      <c r="B87" s="81" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="n"/>
+      <c r="D87" s="81" t="n"/>
       <c r="E87" s="82" t="n"/>
       <c r="F87" s="71" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1">
-      <c r="B88" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C88" s="122">
-        <f>IF((COUNTIF(C83:C86,"Met")+COUNTIF(C83:C86,"Partial")+COUNTIF(C83:C86,"Missed"))=0,"",ROUND((COUNTIF(C83:C86,"Met")*5+COUNTIF(C83:C86,"Partial")*2.5)/(COUNTIF(C83:C86,"Met")+COUNTIF(C83:C86,"Partial")+COUNTIF(C83:C86,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D88" s="92" t="n"/>
+      <c r="B88" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
+        </is>
+      </c>
+      <c r="C88" s="82" t="n"/>
+      <c r="D88" s="82" t="n"/>
       <c r="E88" s="82" t="n"/>
       <c r="F88" s="71" t="n"/>
     </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C89" s="14" t="n"/>
-      <c r="D89" s="84">
-        <f>IF(IF(C89="",C88,C89)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C89="",C88,C89)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="89" ht="28" customHeight="1">
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C89" s="122">
+        <f>IF((COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed"))=0,"",ROUND((COUNTIF(C84:C87,"Met")*5+COUNTIF(C84:C87,"Partial")*2.5)/(COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D89" s="92" t="n"/>
       <c r="E89" s="82" t="n"/>
       <c r="F89" s="71" t="n"/>
     </row>
-    <row r="90" ht="36" customHeight="1">
+    <row r="90" ht="24" customHeight="1">
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
-        </is>
-      </c>
-      <c r="C90" s="86" t="n"/>
-      <c r="D90" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C90" s="14" t="n"/>
+      <c r="D90" s="84">
+        <f>IF(IF(C90="",C89,C90)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C90="",C89,C90)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E90" s="82" t="n"/>
       <c r="F90" s="71" t="n"/>
     </row>
-    <row r="91" ht="20" customHeight="1">
-      <c r="B91" s="80" t="inlineStr">
+    <row r="91" ht="36" customHeight="1">
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
+        </is>
+      </c>
+      <c r="C91" s="86" t="n"/>
+      <c r="D91" s="82" t="n"/>
+      <c r="E91" s="82" t="n"/>
+      <c r="F91" s="71" t="n"/>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="B92" s="80" t="inlineStr">
         <is>
           <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
         </is>
       </c>
-      <c r="C91" s="90" t="n"/>
-      <c r="D91" s="90" t="n"/>
-      <c r="E91" s="90" t="n"/>
-      <c r="F91" s="74" t="n"/>
-    </row>
-    <row r="92" ht="20" customHeight="1">
-      <c r="B92" s="13" t="inlineStr">
+      <c r="C92" s="90" t="n"/>
+      <c r="D92" s="90" t="n"/>
+      <c r="E92" s="90" t="n"/>
+      <c r="F92" s="74" t="n"/>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="B93" s="13" t="inlineStr">
         <is>
           <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
         </is>
       </c>
-      <c r="C92" s="123" t="n"/>
-      <c r="D92" s="92" t="n"/>
-      <c r="F92" s="6" t="n"/>
-    </row>
-    <row r="93" ht="45" customHeight="1">
-      <c r="B93" s="124" t="n"/>
-      <c r="C93" s="125" t="n"/>
-      <c r="D93" s="84" t="n"/>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="B94" s="80" t="inlineStr">
+      <c r="C93" s="123" t="n"/>
+      <c r="D93" s="92" t="n"/>
+      <c r="F93" s="6" t="n"/>
+    </row>
+    <row r="94" ht="45" customHeight="1">
+      <c r="B94" s="124" t="n"/>
+      <c r="C94" s="125" t="n"/>
+      <c r="D94" s="84" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="B95" s="80" t="inlineStr">
         <is>
           <t>L1 learning points from this escalation outcome</t>
         </is>
       </c>
-      <c r="C94" s="90" t="n"/>
-      <c r="D94" s="90" t="n"/>
-      <c r="E94" s="90" t="n"/>
-      <c r="F94" s="74" t="n"/>
-    </row>
-    <row r="95" ht="28" customHeight="1">
-      <c r="B95" s="13" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C95" s="9" t="n"/>
-      <c r="D95" s="82" t="n"/>
-      <c r="E95" s="82" t="n"/>
-      <c r="F95" s="71" t="n"/>
+      <c r="C95" s="90" t="n"/>
+      <c r="D95" s="90" t="n"/>
+      <c r="E95" s="90" t="n"/>
+      <c r="F95" s="74" t="n"/>
     </row>
     <row r="96" ht="28" customHeight="1">
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="C96" s="9" t="n"/>
@@ -4524,7 +4522,7 @@
     <row r="97" ht="28" customHeight="1">
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="C97" s="9" t="n"/>
@@ -4532,88 +4530,88 @@
       <c r="E97" s="82" t="n"/>
       <c r="F97" s="71" t="n"/>
     </row>
-    <row r="98" ht="18" customHeight="1">
-      <c r="B98" s="80" t="inlineStr">
+    <row r="98" ht="28" customHeight="1">
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="n"/>
+      <c r="D98" s="82" t="n"/>
+      <c r="E98" s="82" t="n"/>
+      <c r="F98" s="71" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="B99" s="80" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
       </c>
-      <c r="C98" s="90" t="n"/>
-      <c r="D98" s="90" t="n"/>
-      <c r="E98" s="74" t="n"/>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="C99" s="90" t="n"/>
+      <c r="D99" s="90" t="n"/>
+      <c r="E99" s="74" t="n"/>
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="28" customHeight="1">
-      <c r="B99" s="121" t="inlineStr">
+    <row r="100" ht="28" customHeight="1">
+      <c r="B100" s="121" t="inlineStr">
         <is>
           <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
         </is>
       </c>
-      <c r="C99" s="82" t="n"/>
-      <c r="D99" s="82" t="n"/>
-      <c r="E99" s="82" t="n"/>
-      <c r="F99" s="71" t="n"/>
-    </row>
-    <row r="100" ht="28" customHeight="1">
-      <c r="B100" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C100" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D100" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C100" s="82" t="n"/>
+      <c r="D100" s="82" t="n"/>
       <c r="E100" s="82" t="n"/>
       <c r="F100" s="71" t="n"/>
     </row>
     <row r="101" ht="28" customHeight="1">
-      <c r="B101" s="81" t="inlineStr">
-        <is>
-          <t>Demonstrated empathy including for repeat-contact fatigue</t>
-        </is>
-      </c>
-      <c r="C101" s="9" t="n"/>
-      <c r="D101" s="81" t="n"/>
+      <c r="B101" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D101" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E101" s="82" t="n"/>
       <c r="F101" s="71" t="n"/>
     </row>
     <row r="102" ht="28" customHeight="1">
-      <c r="B102" s="83" t="inlineStr">
-        <is>
-          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+      <c r="B102" s="81" t="inlineStr">
+        <is>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
         </is>
       </c>
       <c r="C102" s="9" t="n"/>
-      <c r="D102" s="83" t="n"/>
+      <c r="D102" s="81" t="n"/>
       <c r="E102" s="82" t="n"/>
       <c r="F102" s="71" t="n"/>
     </row>
     <row r="103" ht="28" customHeight="1">
-      <c r="B103" s="81" t="inlineStr">
-        <is>
-          <t>Agent matched the customer's tone, pace, level, and energy</t>
+      <c r="B103" s="83" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
         </is>
       </c>
       <c r="C103" s="9" t="n"/>
-      <c r="D103" s="81" t="n"/>
+      <c r="D103" s="83" t="n"/>
       <c r="E103" s="82" t="n"/>
       <c r="F103" s="71" t="n"/>
     </row>
     <row r="104" ht="28" customHeight="1">
       <c r="B104" s="81" t="inlineStr">
         <is>
-          <t>Minimized customer effort</t>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
         </is>
       </c>
       <c r="C104" s="9" t="n"/>
@@ -4622,159 +4620,159 @@
       <c r="F104" s="71" t="n"/>
     </row>
     <row r="105" ht="28" customHeight="1">
-      <c r="B105" s="83" t="inlineStr">
-        <is>
-          <t>Maintained customer understanding and engagement</t>
+      <c r="B105" s="81" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
         </is>
       </c>
       <c r="C105" s="9" t="n"/>
-      <c r="D105" s="83" t="n"/>
+      <c r="D105" s="81" t="n"/>
       <c r="E105" s="82" t="n"/>
       <c r="F105" s="71" t="n"/>
     </row>
     <row r="106" ht="28" customHeight="1">
-      <c r="B106" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="C106" s="82" t="n"/>
-      <c r="D106" s="82" t="n"/>
+      <c r="B106" s="83" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="n"/>
+      <c r="D106" s="83" t="n"/>
       <c r="E106" s="82" t="n"/>
       <c r="F106" s="71" t="n"/>
     </row>
     <row r="107" ht="28" customHeight="1">
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C107" s="122">
-        <f>IF((COUNTIF(C101:C105,"Met")+COUNTIF(C101:C105,"Partial")+COUNTIF(C101:C105,"Missed"))=0,"",ROUND((COUNTIF(C101:C105,"Met")*5+COUNTIF(C101:C105,"Partial")*2.5)/(COUNTIF(C101:C105,"Met")+COUNTIF(C101:C105,"Partial")+COUNTIF(C101:C105,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D107" s="92" t="n"/>
+      <c r="B107" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
+        </is>
+      </c>
+      <c r="C107" s="82" t="n"/>
+      <c r="D107" s="82" t="n"/>
       <c r="E107" s="82" t="n"/>
       <c r="F107" s="71" t="n"/>
     </row>
-    <row r="108" ht="24" customHeight="1">
-      <c r="B108" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C108" s="14" t="n"/>
-      <c r="D108" s="84">
-        <f>IF(IF(C108="",C107,C108)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C108="",C107,C108)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="108" ht="28" customHeight="1">
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C108" s="122">
+        <f>IF((COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed"))=0,"",ROUND((COUNTIF(C102:C106,"Met")*5+COUNTIF(C102:C106,"Partial")*2.5)/(COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D108" s="92" t="n"/>
       <c r="E108" s="82" t="n"/>
       <c r="F108" s="71" t="n"/>
     </row>
-    <row r="109" ht="36" customHeight="1">
+    <row r="109" ht="24" customHeight="1">
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
-      <c r="C109" s="86" t="n"/>
-      <c r="D109" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C109" s="14" t="n"/>
+      <c r="D109" s="84">
+        <f>IF(IF(C109="",C108,C109)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C109="",C108,C109)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E109" s="82" t="n"/>
       <c r="F109" s="71" t="n"/>
     </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="B110" s="80" t="inlineStr">
+    <row r="110" ht="36" customHeight="1">
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
+        </is>
+      </c>
+      <c r="C110" s="86" t="n"/>
+      <c r="D110" s="82" t="n"/>
+      <c r="E110" s="82" t="n"/>
+      <c r="F110" s="71" t="n"/>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="B111" s="80" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
       </c>
-      <c r="C110" s="90" t="n"/>
-      <c r="D110" s="90" t="n"/>
-      <c r="E110" s="74" t="n"/>
-      <c r="F110" s="6" t="inlineStr">
+      <c r="C111" s="90" t="n"/>
+      <c r="D111" s="90" t="n"/>
+      <c r="E111" s="74" t="n"/>
+      <c r="F111" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="28" customHeight="1">
-      <c r="B111" s="121" t="inlineStr">
+    <row r="112" ht="28" customHeight="1">
+      <c r="B112" s="121" t="inlineStr">
         <is>
           <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
         </is>
       </c>
-      <c r="C111" s="82" t="n"/>
-      <c r="D111" s="82" t="n"/>
-      <c r="E111" s="82" t="n"/>
-      <c r="F111" s="71" t="n"/>
-    </row>
-    <row r="112" ht="36" customHeight="1">
-      <c r="B112" s="94" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C112" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D112" s="94" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C112" s="82" t="n"/>
+      <c r="D112" s="82" t="n"/>
       <c r="E112" s="82" t="n"/>
       <c r="F112" s="71" t="n"/>
     </row>
-    <row r="113" ht="28" customHeight="1">
-      <c r="B113" s="81" t="inlineStr">
-        <is>
-          <t>Recorded customer issue summary</t>
-        </is>
-      </c>
-      <c r="C113" s="9" t="n"/>
-      <c r="D113" s="81" t="n"/>
+    <row r="113" ht="36" customHeight="1">
+      <c r="B113" s="94" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D113" s="94" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E113" s="82" t="n"/>
       <c r="F113" s="71" t="n"/>
     </row>
     <row r="114" ht="28" customHeight="1">
-      <c r="B114" s="83" t="inlineStr">
-        <is>
-          <t>Documented troubleshooting steps</t>
+      <c r="B114" s="81" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
         </is>
       </c>
       <c r="C114" s="9" t="n"/>
-      <c r="D114" s="83" t="n"/>
+      <c r="D114" s="81" t="n"/>
       <c r="E114" s="82" t="n"/>
       <c r="F114" s="71" t="n"/>
     </row>
     <row r="115" ht="28" customHeight="1">
-      <c r="B115" s="81" t="inlineStr">
-        <is>
-          <t>Noted key findings</t>
+      <c r="B115" s="83" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
         </is>
       </c>
       <c r="C115" s="9" t="n"/>
-      <c r="D115" s="81" t="n"/>
+      <c r="D115" s="83" t="n"/>
       <c r="E115" s="82" t="n"/>
       <c r="F115" s="71" t="n"/>
     </row>
     <row r="116" ht="28" customHeight="1">
-      <c r="B116" s="83" t="inlineStr">
-        <is>
-          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
+      <c r="B116" s="81" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
         </is>
       </c>
       <c r="C116" s="9" t="n"/>
-      <c r="D116" s="83" t="n"/>
+      <c r="D116" s="81" t="n"/>
       <c r="E116" s="82" t="n"/>
       <c r="F116" s="71" t="n"/>
     </row>
     <row r="117" ht="28" customHeight="1">
       <c r="B117" s="83" t="inlineStr">
         <is>
-          <t>Documented next steps and follow-ups</t>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
         </is>
       </c>
       <c r="C117" s="9" t="n"/>
@@ -4783,222 +4781,218 @@
       <c r="F117" s="71" t="n"/>
     </row>
     <row r="118" ht="28" customHeight="1">
-      <c r="B118" s="81" t="inlineStr">
-        <is>
-          <t>Updated ticket status accurately</t>
+      <c r="B118" s="83" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
         </is>
       </c>
       <c r="C118" s="9" t="n"/>
-      <c r="D118" s="81" t="n"/>
+      <c r="D118" s="83" t="n"/>
       <c r="E118" s="82" t="n"/>
       <c r="F118" s="71" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1">
-      <c r="B119" s="85" t="inlineStr">
-        <is>
-          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="C119" s="82" t="n"/>
-      <c r="D119" s="82" t="n"/>
+      <c r="B119" s="81" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="n"/>
+      <c r="D119" s="81" t="n"/>
       <c r="E119" s="82" t="n"/>
       <c r="F119" s="71" t="n"/>
     </row>
-    <row r="120" ht="52" customHeight="1">
-      <c r="B120" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C120" s="122">
-        <f>IF((COUNTIF(C113:C118,"Met")+COUNTIF(C113:C118,"Partial")+COUNTIF(C113:C118,"Missed"))=0,"",ROUND((COUNTIF(C113:C118,"Met")*5+COUNTIF(C113:C118,"Partial")*2.5)/(COUNTIF(C113:C118,"Met")+COUNTIF(C113:C118,"Partial")+COUNTIF(C113:C118,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D120" s="92" t="n"/>
+    <row r="120" ht="28" customHeight="1">
+      <c r="B120" s="85" t="inlineStr">
+        <is>
+          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
+        </is>
+      </c>
+      <c r="C120" s="82" t="n"/>
+      <c r="D120" s="82" t="n"/>
       <c r="E120" s="82" t="n"/>
       <c r="F120" s="71" t="n"/>
     </row>
-    <row r="121" ht="24" customHeight="1">
-      <c r="B121" s="13" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C121" s="14" t="n"/>
-      <c r="D121" s="84">
-        <f>IF(IF(C121="",C120,C121)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C121="",C120,C121)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="121" ht="52" customHeight="1">
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C121" s="122">
+        <f>IF((COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed"))=0,"",ROUND((COUNTIF(C114:C119,"Met")*5+COUNTIF(C114:C119,"Partial")*2.5)/(COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D121" s="92" t="n"/>
       <c r="E121" s="82" t="n"/>
       <c r="F121" s="71" t="n"/>
     </row>
-    <row r="122" ht="36" customHeight="1">
+    <row r="122" ht="24" customHeight="1">
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
-      <c r="C122" s="86" t="n"/>
-      <c r="D122" s="82" t="n"/>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C122" s="14" t="n"/>
+      <c r="D122" s="84">
+        <f>IF(IF(C122="",C121,C122)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C122="",C121,C122)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E122" s="82" t="n"/>
       <c r="F122" s="71" t="n"/>
     </row>
-    <row r="123" ht="30" customHeight="1">
-      <c r="B123" s="80" t="inlineStr">
+    <row r="123" ht="36" customHeight="1">
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
+        </is>
+      </c>
+      <c r="C123" s="86" t="n"/>
+      <c r="D123" s="82" t="n"/>
+      <c r="E123" s="82" t="n"/>
+      <c r="F123" s="71" t="n"/>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="B124" s="80" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
       </c>
-      <c r="C123" s="90" t="n"/>
-      <c r="D123" s="90" t="n"/>
-      <c r="E123" s="90" t="n"/>
-      <c r="F123" s="74" t="n"/>
-    </row>
-    <row r="124" ht="28" customHeight="1">
-      <c r="B124" s="94" t="inlineStr">
+      <c r="C124" s="90" t="n"/>
+      <c r="D124" s="90" t="n"/>
+      <c r="E124" s="90" t="n"/>
+      <c r="F124" s="74" t="n"/>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="B125" s="94" t="inlineStr">
         <is>
           <t>Outcome classification</t>
         </is>
       </c>
-      <c r="C124" s="97" t="n"/>
-      <c r="D124" s="82" t="n"/>
-      <c r="E124" s="82" t="n"/>
-      <c r="F124" s="71" t="n"/>
-    </row>
-    <row r="125" ht="52" customHeight="1">
-      <c r="B125" s="87" t="inlineStr">
-        <is>
-          <t>Primary positive outcome achieved</t>
-        </is>
-      </c>
-      <c r="C125" s="88" t="n"/>
+      <c r="C125" s="97" t="n"/>
       <c r="D125" s="82" t="n"/>
       <c r="E125" s="82" t="n"/>
       <c r="F125" s="71" t="n"/>
     </row>
     <row r="126" ht="52" customHeight="1">
-      <c r="B126" s="94" t="inlineStr">
-        <is>
-          <t>Justification</t>
-        </is>
-      </c>
-      <c r="C126" s="86" t="n"/>
+      <c r="B126" s="87" t="inlineStr">
+        <is>
+          <t>Primary positive outcome achieved</t>
+        </is>
+      </c>
+      <c r="C126" s="88" t="n"/>
       <c r="D126" s="82" t="n"/>
       <c r="E126" s="82" t="n"/>
       <c r="F126" s="71" t="n"/>
     </row>
-    <row r="127" ht="26" customHeight="1">
-      <c r="B127" s="80" t="inlineStr">
+    <row r="127" ht="52" customHeight="1">
+      <c r="B127" s="94" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
+      <c r="C127" s="86" t="n"/>
+      <c r="D127" s="82" t="n"/>
+      <c r="E127" s="82" t="n"/>
+      <c r="F127" s="71" t="n"/>
+    </row>
+    <row r="128" ht="26" customHeight="1">
+      <c r="B128" s="80" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
       </c>
-      <c r="C127" s="90" t="n"/>
-      <c r="D127" s="90" t="n"/>
-      <c r="E127" s="90" t="n"/>
-      <c r="F127" s="74" t="n"/>
-    </row>
-    <row r="128" ht="30" customHeight="1">
-      <c r="B128" s="87" t="inlineStr">
+      <c r="C128" s="90" t="n"/>
+      <c r="D128" s="90" t="n"/>
+      <c r="E128" s="90" t="n"/>
+      <c r="F128" s="74" t="n"/>
+    </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="B129" s="87" t="inlineStr">
         <is>
           <t>Did the interaction disconnect before completion?</t>
         </is>
       </c>
-      <c r="C128" s="9" t="inlineStr">
+      <c r="C129" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D128" s="85" t="inlineStr">
+      <c r="D129" s="85" t="inlineStr">
         <is>
           <t>If Yes, at least one documented follow-up action is required.</t>
         </is>
       </c>
-      <c r="E128" s="82" t="n"/>
-      <c r="F128" s="71" t="n"/>
-    </row>
-    <row r="129" ht="30" customHeight="1">
-      <c r="B129" s="94" t="inlineStr">
+      <c r="E129" s="82" t="n"/>
+      <c r="F129" s="71" t="n"/>
+    </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="B130" s="94" t="inlineStr">
         <is>
           <t>Follow-up action taken</t>
         </is>
       </c>
-      <c r="C129" s="88" t="inlineStr">
+      <c r="C130" s="88" t="inlineStr">
         <is>
           <t>N.A. — no disconnect</t>
         </is>
       </c>
-      <c r="D129" s="71" t="n"/>
-      <c r="E129" s="79">
-        <f>IF(AND(C128="Yes",OR(C129="None",C129="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
-        <v/>
-      </c>
-      <c r="F129" s="71" t="n"/>
-    </row>
-    <row r="130" ht="26" customHeight="1">
-      <c r="B130" s="98" t="inlineStr">
+      <c r="D130" s="71" t="n"/>
+      <c r="E130" s="79">
+        <f>IF(AND(C129="Yes",OR(C130="None",C130="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
+        <v/>
+      </c>
+      <c r="F130" s="71" t="n"/>
+    </row>
+    <row r="131" ht="26" customHeight="1">
+      <c r="B131" s="98" t="inlineStr">
         <is>
           <t>6 · CRITICAL FAILURE CONDITIONS  (any 'Yes' triggers automatic review / coaching / QA failure regardless of score)</t>
         </is>
       </c>
-      <c r="C130" s="90" t="n"/>
-      <c r="D130" s="90" t="n"/>
-      <c r="E130" s="90" t="n"/>
-      <c r="F130" s="74" t="n"/>
-    </row>
-    <row r="131" ht="26" customHeight="1">
-      <c r="B131" s="80" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="C131" s="119" t="inlineStr">
-        <is>
-          <t>Present?</t>
-        </is>
-      </c>
-      <c r="D131" s="80" t="inlineStr">
-        <is>
-          <t>Notes / Evidence</t>
-        </is>
-      </c>
+      <c r="C131" s="90" t="n"/>
+      <c r="D131" s="90" t="n"/>
       <c r="E131" s="90" t="n"/>
       <c r="F131" s="74" t="n"/>
     </row>
     <row r="132" ht="26" customHeight="1">
-      <c r="B132" s="81" t="inlineStr">
+      <c r="B132" s="80" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="C132" s="119" t="inlineStr">
+        <is>
+          <t>Present?</t>
+        </is>
+      </c>
+      <c r="D132" s="80" t="inlineStr">
+        <is>
+          <t>Notes / Evidence</t>
+        </is>
+      </c>
+      <c r="E132" s="90" t="n"/>
+      <c r="F132" s="74" t="n"/>
+    </row>
+    <row r="133" ht="26" customHeight="1">
+      <c r="B133" s="81" t="inlineStr">
         <is>
           <t>Harmful or incorrect troubleshooting provided</t>
         </is>
       </c>
-      <c r="C132" s="9" t="inlineStr">
+      <c r="C133" s="9" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D132" s="81" t="n"/>
-      <c r="E132" s="82" t="n"/>
-      <c r="F132" s="71" t="n"/>
-    </row>
-    <row r="133" ht="26" customHeight="1">
-      <c r="B133" s="83" t="inlineStr">
-        <is>
-          <t>Misrepresented product capabilities</t>
-        </is>
-      </c>
-      <c r="C133" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D133" s="83" t="n"/>
+      <c r="D133" s="81" t="n"/>
       <c r="E133" s="82" t="n"/>
       <c r="F133" s="71" t="n"/>
     </row>
     <row r="134" ht="26" customHeight="1">
-      <c r="B134" s="81" t="inlineStr">
-        <is>
-          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
+      <c r="B134" s="83" t="inlineStr">
+        <is>
+          <t>Misrepresented product capabilities</t>
         </is>
       </c>
       <c r="C134" s="9" t="inlineStr">
@@ -5006,14 +5000,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D134" s="81" t="n"/>
+      <c r="D134" s="83" t="n"/>
       <c r="E134" s="82" t="n"/>
       <c r="F134" s="71" t="n"/>
     </row>
     <row r="135" ht="26" customHeight="1">
-      <c r="B135" s="83" t="inlineStr">
-        <is>
-          <t>No follow-up after disconnected call</t>
+      <c r="B135" s="81" t="inlineStr">
+        <is>
+          <t>Unsupported root-cause claims (e.g., ISP/customer blame w/o evidence)</t>
         </is>
       </c>
       <c r="C135" s="9" t="inlineStr">
@@ -5021,14 +5015,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D135" s="83" t="n"/>
+      <c r="D135" s="81" t="n"/>
       <c r="E135" s="82" t="n"/>
       <c r="F135" s="71" t="n"/>
     </row>
     <row r="136" ht="26" customHeight="1">
-      <c r="B136" s="81" t="inlineStr">
-        <is>
-          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
+      <c r="B136" s="83" t="inlineStr">
+        <is>
+          <t>No follow-up after disconnected call</t>
         </is>
       </c>
       <c r="C136" s="9" t="inlineStr">
@@ -5036,14 +5030,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D136" s="81" t="n"/>
+      <c r="D136" s="83" t="n"/>
       <c r="E136" s="82" t="n"/>
       <c r="F136" s="71" t="n"/>
     </row>
     <row r="137" ht="26" customHeight="1">
-      <c r="B137" s="83" t="inlineStr">
-        <is>
-          <t>Abandoned customer without a path forward</t>
+      <c r="B137" s="81" t="inlineStr">
+        <is>
+          <t>Failed to complete a promised action (incl. missed agreed callback window)</t>
         </is>
       </c>
       <c r="C137" s="9" t="inlineStr">
@@ -5051,14 +5045,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D137" s="83" t="n"/>
+      <c r="D137" s="81" t="n"/>
       <c r="E137" s="82" t="n"/>
       <c r="F137" s="71" t="n"/>
     </row>
     <row r="138" ht="26" customHeight="1">
-      <c r="B138" s="81" t="inlineStr">
-        <is>
-          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
+      <c r="B138" s="83" t="inlineStr">
+        <is>
+          <t>Abandoned customer without a path forward</t>
         </is>
       </c>
       <c r="C138" s="9" t="inlineStr">
@@ -5066,14 +5060,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D138" s="81" t="n"/>
+      <c r="D138" s="83" t="n"/>
       <c r="E138" s="82" t="n"/>
       <c r="F138" s="71" t="n"/>
     </row>
     <row r="139" ht="26" customHeight="1">
-      <c r="B139" s="83" t="inlineStr">
-        <is>
-          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
+      <c r="B139" s="81" t="inlineStr">
+        <is>
+          <t>Escalated without reasonable troubleshooting / to avoid ownership</t>
         </is>
       </c>
       <c r="C139" s="9" t="inlineStr">
@@ -5081,14 +5075,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D139" s="83" t="n"/>
+      <c r="D139" s="81" t="n"/>
       <c r="E139" s="82" t="n"/>
       <c r="F139" s="71" t="n"/>
     </row>
     <row r="140" ht="26" customHeight="1">
       <c r="B140" s="83" t="inlineStr">
         <is>
-          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
+          <t>Unprofessional, rude, or dismissive conduct / policy violation</t>
         </is>
       </c>
       <c r="C140" s="9" t="inlineStr">
@@ -5101,9 +5095,9 @@
       <c r="F140" s="71" t="n"/>
     </row>
     <row r="141" ht="26" customHeight="1">
-      <c r="B141" s="81" t="inlineStr">
-        <is>
-          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
+      <c r="B141" s="83" t="inlineStr">
+        <is>
+          <t>Case marked Resolved while issue known to be unresolved (premature closure / no closure reason)</t>
         </is>
       </c>
       <c r="C141" s="9" t="inlineStr">
@@ -5111,14 +5105,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="D141" s="81" t="n"/>
+      <c r="D141" s="83" t="n"/>
       <c r="E141" s="82" t="n"/>
       <c r="F141" s="71" t="n"/>
     </row>
     <row r="142" ht="26" customHeight="1">
       <c r="B142" s="81" t="inlineStr">
         <is>
-          <t>Survey / CSAT manipulation</t>
+          <t>Customer complaint, management-contact, or legal-risk request not escalated</t>
         </is>
       </c>
       <c r="C142" s="9" t="inlineStr">
@@ -5131,79 +5125,79 @@
       <c r="F142" s="71" t="n"/>
     </row>
     <row r="143" ht="26" customHeight="1">
-      <c r="B143" s="98" t="inlineStr">
+      <c r="B143" s="81" t="inlineStr">
+        <is>
+          <t>Survey / CSAT manipulation</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D143" s="81" t="n"/>
+      <c r="E143" s="82" t="n"/>
+      <c r="F143" s="71" t="n"/>
+    </row>
+    <row r="144" ht="26" customHeight="1">
+      <c r="B144" s="98" t="inlineStr">
         <is>
           <t>CRITICAL FAILURE FLAGGED?</t>
         </is>
       </c>
-      <c r="C143" s="93">
-        <f>IF(COUNTIF(C132:C142,"Yes")&gt;0,"YES — "&amp;COUNTIF(C132:C142,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
-        <v/>
-      </c>
-      <c r="D143" s="90" t="n"/>
-      <c r="E143" s="90" t="n"/>
-      <c r="F143" s="74" t="n"/>
-    </row>
-    <row r="144" ht="22" customHeight="1">
-      <c r="B144" s="98" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
-      <c r="C144" s="90" t="n"/>
+      <c r="C144" s="93">
+        <f>IF(COUNTIF(C133:C143,"Yes")&gt;0,"YES — "&amp;COUNTIF(C133:C143,"Yes")&amp;" condition(s) flagged — automatic review required regardless of weighted score","No critical failures")</f>
+        <v/>
+      </c>
       <c r="D144" s="90" t="n"/>
       <c r="E144" s="90" t="n"/>
       <c r="F144" s="74" t="n"/>
     </row>
-    <row r="145" ht="30" customHeight="1">
-      <c r="B145" s="85" t="inlineStr">
+    <row r="145" ht="22" customHeight="1">
+      <c r="B145" s="98" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
+      <c r="C145" s="90" t="n"/>
+      <c r="D145" s="90" t="n"/>
+      <c r="E145" s="90" t="n"/>
+      <c r="F145" s="74" t="n"/>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="B146" s="85" t="inlineStr">
         <is>
           <t>A gate marked 'No', any A–K item marked 'Yes', or any §6 critical-failure condition forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
         </is>
       </c>
-      <c r="C145" s="82" t="n"/>
-      <c r="D145" s="82" t="n"/>
-      <c r="E145" s="82" t="n"/>
-      <c r="F145" s="71" t="n"/>
-    </row>
-    <row r="146" ht="30" customHeight="1">
-      <c r="B146" s="80" t="inlineStr">
+      <c r="C146" s="82" t="n"/>
+      <c r="D146" s="82" t="n"/>
+      <c r="E146" s="82" t="n"/>
+      <c r="F146" s="71" t="n"/>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="B147" s="80" t="inlineStr">
         <is>
           <t>Compliance gate  (mark Yes if adhered)</t>
         </is>
       </c>
-      <c r="C146" s="119" t="inlineStr">
+      <c r="C147" s="119" t="inlineStr">
         <is>
           <t>Adherent?</t>
         </is>
       </c>
-      <c r="D146" s="80" t="inlineStr">
+      <c r="D147" s="80" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E146" s="90" t="n"/>
-      <c r="F146" s="74" t="n"/>
-    </row>
-    <row r="147" ht="26" customHeight="1">
-      <c r="B147" s="81" t="inlineStr">
-        <is>
-          <t>Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C147" s="9" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D147" s="81" t="n"/>
-      <c r="E147" s="82" t="n"/>
-      <c r="F147" s="71" t="n"/>
+      <c r="E147" s="90" t="n"/>
+      <c r="F147" s="74" t="n"/>
     </row>
     <row r="148" ht="26" customHeight="1">
       <c r="B148" s="81" t="inlineStr">
         <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
+          <t>Adherence to Callback Hours</t>
         </is>
       </c>
       <c r="C148" s="9" t="inlineStr">
@@ -5218,7 +5212,7 @@
     <row r="149" ht="26" customHeight="1">
       <c r="B149" s="81" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
         </is>
       </c>
       <c r="C149" s="9" t="inlineStr">
@@ -5230,44 +5224,44 @@
       <c r="E149" s="82" t="n"/>
       <c r="F149" s="71" t="n"/>
     </row>
-    <row r="150" ht="32" customHeight="1">
-      <c r="B150" s="80" t="inlineStr">
+    <row r="150" ht="26" customHeight="1">
+      <c r="B150" s="81" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D150" s="81" t="n"/>
+      <c r="E150" s="82" t="n"/>
+      <c r="F150" s="71" t="n"/>
+    </row>
+    <row r="151" ht="32" customHeight="1">
+      <c r="B151" s="80" t="inlineStr">
         <is>
           <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
         </is>
       </c>
-      <c r="C150" s="119" t="inlineStr">
+      <c r="C151" s="119" t="inlineStr">
         <is>
           <t>Occurred?</t>
         </is>
       </c>
-      <c r="D150" s="80" t="inlineStr">
+      <c r="D151" s="80" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E150" s="90" t="n"/>
-      <c r="F150" s="74" t="n"/>
-    </row>
-    <row r="151" ht="26" customHeight="1">
-      <c r="B151" s="81" t="inlineStr">
-        <is>
-          <t>A.  Call / Session Abandonment</t>
-        </is>
-      </c>
-      <c r="C151" s="9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D151" s="81" t="n"/>
-      <c r="E151" s="82" t="n"/>
-      <c r="F151" s="71" t="n"/>
+      <c r="E151" s="90" t="n"/>
+      <c r="F151" s="74" t="n"/>
     </row>
     <row r="152" ht="26" customHeight="1">
       <c r="B152" s="81" t="inlineStr">
         <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
+          <t>A.  Call / Session Abandonment</t>
         </is>
       </c>
       <c r="C152" s="9" t="inlineStr">
@@ -5282,7 +5276,7 @@
     <row r="153" ht="26" customHeight="1">
       <c r="B153" s="81" t="inlineStr">
         <is>
-          <t>C.  Discourtesy</t>
+          <t>B.  Call / Session Avoidance / Evasion</t>
         </is>
       </c>
       <c r="C153" s="9" t="inlineStr">
@@ -5297,7 +5291,7 @@
     <row r="154" ht="26" customHeight="1">
       <c r="B154" s="81" t="inlineStr">
         <is>
-          <t>D.  Escalation</t>
+          <t>C.  Discourtesy</t>
         </is>
       </c>
       <c r="C154" s="9" t="inlineStr">
@@ -5312,7 +5306,7 @@
     <row r="155" ht="26" customHeight="1">
       <c r="B155" s="81" t="inlineStr">
         <is>
-          <t>E.  Failure to ask for the email address</t>
+          <t>D.  Escalation</t>
         </is>
       </c>
       <c r="C155" s="9" t="inlineStr">
@@ -5327,7 +5321,7 @@
     <row r="156" ht="26" customHeight="1">
       <c r="B156" s="81" t="inlineStr">
         <is>
-          <t>F.  Fraud</t>
+          <t>E.  Failure to ask for the email address</t>
         </is>
       </c>
       <c r="C156" s="9" t="inlineStr">
@@ -5342,7 +5336,7 @@
     <row r="157" ht="26" customHeight="1">
       <c r="B157" s="81" t="inlineStr">
         <is>
-          <t>G.  Hard-selling</t>
+          <t>F.  Fraud</t>
         </is>
       </c>
       <c r="C157" s="9" t="inlineStr">
@@ -5357,7 +5351,7 @@
     <row r="158" ht="26" customHeight="1">
       <c r="B158" s="81" t="inlineStr">
         <is>
-          <t>H.  Line Release</t>
+          <t>G.  Hard-selling</t>
         </is>
       </c>
       <c r="C158" s="9" t="inlineStr">
@@ -5372,7 +5366,7 @@
     <row r="159" ht="26" customHeight="1">
       <c r="B159" s="81" t="inlineStr">
         <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
+          <t>H.  Line Release</t>
         </is>
       </c>
       <c r="C159" s="9" t="inlineStr">
@@ -5387,7 +5381,7 @@
     <row r="160" ht="26" customHeight="1">
       <c r="B160" s="81" t="inlineStr">
         <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+          <t>I.  Non-Adherence to Callback Hours</t>
         </is>
       </c>
       <c r="C160" s="9" t="inlineStr">
@@ -5402,7 +5396,7 @@
     <row r="161" ht="26" customHeight="1">
       <c r="B161" s="81" t="inlineStr">
         <is>
-          <t>K.  Non-First Call Resolution</t>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
         </is>
       </c>
       <c r="C161" s="9" t="inlineStr">
@@ -5414,35 +5408,39 @@
       <c r="E161" s="82" t="n"/>
       <c r="F161" s="71" t="n"/>
     </row>
-    <row r="162" ht="24" customHeight="1">
-      <c r="B162" s="98" t="inlineStr">
+    <row r="162" ht="26" customHeight="1">
+      <c r="B162" s="81" t="inlineStr">
+        <is>
+          <t>K.  Non-First Call Resolution</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D162" s="81" t="n"/>
+      <c r="E162" s="82" t="n"/>
+      <c r="F162" s="71" t="n"/>
+    </row>
+    <row r="163" ht="24" customHeight="1">
+      <c r="B163" s="98" t="inlineStr">
         <is>
           <t>AUTO-ZERO TRIGGERED?</t>
         </is>
       </c>
-      <c r="C162" s="93">
-        <f>IF(OR(C147="No",C148="No",C149="No",COUNTIF(C151:C161,"Yes")&gt;0,COUNTIF(C132:C142,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
-      <c r="D162" s="90" t="n"/>
-      <c r="E162" s="90" t="n"/>
-      <c r="F162" s="74" t="n"/>
-    </row>
-    <row r="163" ht="20" customHeight="1">
-      <c r="B163" s="96" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
-        </is>
-      </c>
-      <c r="C163" s="90" t="n"/>
+      <c r="C163" s="93">
+        <f>IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0,COUNTIF(C133:C143,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
       <c r="D163" s="90" t="n"/>
       <c r="E163" s="90" t="n"/>
       <c r="F163" s="74" t="n"/>
     </row>
-    <row r="164" ht="30" customHeight="1">
-      <c r="B164" s="91" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+    <row r="164" ht="20" customHeight="1">
+      <c r="B164" s="96" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
         </is>
       </c>
       <c r="C164" s="90" t="n"/>
@@ -5450,42 +5448,42 @@
       <c r="E164" s="90" t="n"/>
       <c r="F164" s="74" t="n"/>
     </row>
-    <row r="165" ht="58" customHeight="1">
-      <c r="B165" s="86" t="n"/>
-      <c r="C165" s="82" t="n"/>
-      <c r="D165" s="82" t="n"/>
-      <c r="E165" s="82" t="n"/>
-      <c r="F165" s="71" t="n"/>
-    </row>
-    <row r="166" ht="30" customHeight="1">
-      <c r="B166" s="91" t="inlineStr">
+    <row r="165" ht="30" customHeight="1">
+      <c r="B165" s="91" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+        </is>
+      </c>
+      <c r="C165" s="90" t="n"/>
+      <c r="D165" s="90" t="n"/>
+      <c r="E165" s="90" t="n"/>
+      <c r="F165" s="74" t="n"/>
+    </row>
+    <row r="166" ht="58" customHeight="1">
+      <c r="B166" s="86" t="n"/>
+      <c r="C166" s="82" t="n"/>
+      <c r="D166" s="82" t="n"/>
+      <c r="E166" s="82" t="n"/>
+      <c r="F166" s="71" t="n"/>
+    </row>
+    <row r="167" ht="30" customHeight="1">
+      <c r="B167" s="91" t="inlineStr">
         <is>
           <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
         </is>
       </c>
-      <c r="C166" s="90" t="n"/>
-      <c r="D166" s="90" t="n"/>
-      <c r="E166" s="90" t="n"/>
-      <c r="F166" s="74" t="n"/>
-    </row>
-    <row r="167" ht="24" customHeight="1">
-      <c r="B167" s="87" t="inlineStr">
+      <c r="C167" s="90" t="n"/>
+      <c r="D167" s="90" t="n"/>
+      <c r="E167" s="90" t="n"/>
+      <c r="F167" s="74" t="n"/>
+    </row>
+    <row r="168" ht="24" customHeight="1">
+      <c r="B168" s="87" t="inlineStr">
         <is>
           <t>What went well — behaviors to repeat</t>
         </is>
       </c>
-      <c r="C167" s="82" t="n"/>
-      <c r="D167" s="82" t="n"/>
-      <c r="E167" s="82" t="n"/>
-      <c r="F167" s="71" t="n"/>
-    </row>
-    <row r="168" ht="32" customHeight="1">
-      <c r="B168" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C168" s="86" t="n"/>
+      <c r="C168" s="82" t="n"/>
       <c r="D168" s="82" t="n"/>
       <c r="E168" s="82" t="n"/>
       <c r="F168" s="71" t="n"/>
@@ -5493,7 +5491,7 @@
     <row r="169" ht="32" customHeight="1">
       <c r="B169" s="7" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="C169" s="86" t="n"/>
@@ -5504,7 +5502,7 @@
     <row r="170" ht="32" customHeight="1">
       <c r="B170" s="7" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="C170" s="86" t="n"/>
@@ -5512,24 +5510,24 @@
       <c r="E170" s="82" t="n"/>
       <c r="F170" s="71" t="n"/>
     </row>
-    <row r="171" ht="24" customHeight="1">
-      <c r="B171" s="87" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
-      <c r="C171" s="82" t="n"/>
+    <row r="171" ht="32" customHeight="1">
+      <c r="B171" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C171" s="86" t="n"/>
       <c r="D171" s="82" t="n"/>
       <c r="E171" s="82" t="n"/>
       <c r="F171" s="71" t="n"/>
     </row>
-    <row r="172" ht="32" customHeight="1">
-      <c r="B172" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C172" s="86" t="n"/>
+    <row r="172" ht="24" customHeight="1">
+      <c r="B172" s="87" t="inlineStr">
+        <is>
+          <t>Improvement opportunities — behaviors to improve</t>
+        </is>
+      </c>
+      <c r="C172" s="82" t="n"/>
       <c r="D172" s="82" t="n"/>
       <c r="E172" s="82" t="n"/>
       <c r="F172" s="71" t="n"/>
@@ -5537,7 +5535,7 @@
     <row r="173" ht="32" customHeight="1">
       <c r="B173" s="7" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="C173" s="86" t="n"/>
@@ -5548,7 +5546,7 @@
     <row r="174" ht="32" customHeight="1">
       <c r="B174" s="7" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>2.</t>
         </is>
       </c>
       <c r="C174" s="86" t="n"/>
@@ -5556,42 +5554,42 @@
       <c r="E174" s="82" t="n"/>
       <c r="F174" s="71" t="n"/>
     </row>
-    <row r="175" ht="24" customHeight="1">
-      <c r="B175" s="87" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
-      <c r="C175" s="82" t="n"/>
+    <row r="175" ht="32" customHeight="1">
+      <c r="B175" s="7" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C175" s="86" t="n"/>
       <c r="D175" s="82" t="n"/>
       <c r="E175" s="82" t="n"/>
       <c r="F175" s="71" t="n"/>
     </row>
-    <row r="176" ht="58" customHeight="1">
-      <c r="B176" s="86" t="n"/>
+    <row r="176" ht="24" customHeight="1">
+      <c r="B176" s="87" t="inlineStr">
+        <is>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
+        </is>
+      </c>
       <c r="C176" s="82" t="n"/>
       <c r="D176" s="82" t="n"/>
       <c r="E176" s="82" t="n"/>
       <c r="F176" s="71" t="n"/>
     </row>
-    <row r="177" ht="20" customHeight="1">
-      <c r="B177" s="87" t="inlineStr">
-        <is>
-          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
-        </is>
-      </c>
+    <row r="177" ht="58" customHeight="1">
+      <c r="B177" s="86" t="n"/>
       <c r="C177" s="82" t="n"/>
       <c r="D177" s="82" t="n"/>
       <c r="E177" s="82" t="n"/>
       <c r="F177" s="71" t="n"/>
     </row>
-    <row r="178" ht="28" customHeight="1">
-      <c r="B178" s="86" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C178" s="86" t="n"/>
+    <row r="178" ht="20" customHeight="1">
+      <c r="B178" s="87" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
+      <c r="C178" s="82" t="n"/>
       <c r="D178" s="82" t="n"/>
       <c r="E178" s="82" t="n"/>
       <c r="F178" s="71" t="n"/>
@@ -5599,7 +5597,7 @@
     <row r="179" ht="28" customHeight="1">
       <c r="B179" s="86" t="inlineStr">
         <is>
-          <t>2.</t>
+          <t>1.</t>
         </is>
       </c>
       <c r="C179" s="86" t="n"/>
@@ -5610,228 +5608,250 @@
     <row r="180" ht="28" customHeight="1">
       <c r="B180" s="86" t="inlineStr">
         <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C180" s="9" t="n"/>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C180" s="86" t="n"/>
       <c r="D180" s="82" t="n"/>
       <c r="E180" s="82" t="n"/>
       <c r="F180" s="71" t="n"/>
     </row>
-    <row r="181" ht="32" customHeight="1">
-      <c r="B181" s="91" t="inlineStr">
+    <row r="181" ht="28" customHeight="1">
+      <c r="B181" s="86" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="n"/>
+      <c r="D181" s="82" t="n"/>
+      <c r="E181" s="82" t="n"/>
+      <c r="F181" s="71" t="n"/>
+    </row>
+    <row r="182" ht="32" customHeight="1">
+      <c r="B182" s="91" t="inlineStr">
         <is>
           <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
         </is>
       </c>
-      <c r="C181" s="90" t="n"/>
-      <c r="D181" s="90" t="n"/>
-      <c r="E181" s="90" t="n"/>
-      <c r="F181" s="74" t="n"/>
-    </row>
-    <row r="182" ht="24" customHeight="1">
-      <c r="B182" s="87" t="inlineStr">
+      <c r="C182" s="90" t="n"/>
+      <c r="D182" s="90" t="n"/>
+      <c r="E182" s="90" t="n"/>
+      <c r="F182" s="74" t="n"/>
+    </row>
+    <row r="183" ht="24" customHeight="1">
+      <c r="B183" s="87" t="inlineStr">
         <is>
           <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
         </is>
       </c>
-      <c r="C182" s="82" t="n"/>
-      <c r="D182" s="82" t="n"/>
-      <c r="E182" s="82" t="n"/>
-      <c r="F182" s="71" t="n"/>
-    </row>
-    <row r="183" ht="58" customHeight="1">
-      <c r="B183" s="86" t="n"/>
       <c r="C183" s="82" t="n"/>
       <c r="D183" s="82" t="n"/>
       <c r="E183" s="82" t="n"/>
       <c r="F183" s="71" t="n"/>
     </row>
-    <row r="184" ht="24" customHeight="1">
-      <c r="B184" s="87" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
+    <row r="184" ht="58" customHeight="1">
+      <c r="B184" s="86" t="n"/>
       <c r="C184" s="82" t="n"/>
       <c r="D184" s="82" t="n"/>
       <c r="E184" s="82" t="n"/>
       <c r="F184" s="71" t="n"/>
     </row>
-    <row r="185" ht="58" customHeight="1">
-      <c r="B185" s="86" t="n"/>
+    <row r="185" ht="24" customHeight="1">
+      <c r="B185" s="87" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
       <c r="C185" s="82" t="n"/>
       <c r="D185" s="82" t="n"/>
       <c r="E185" s="82" t="n"/>
       <c r="F185" s="71" t="n"/>
     </row>
-    <row r="186" ht="24" customHeight="1">
-      <c r="B186" s="87" t="inlineStr">
-        <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
-        </is>
-      </c>
+    <row r="186" ht="58" customHeight="1">
+      <c r="B186" s="86" t="n"/>
       <c r="C186" s="82" t="n"/>
       <c r="D186" s="82" t="n"/>
       <c r="E186" s="82" t="n"/>
       <c r="F186" s="71" t="n"/>
     </row>
-    <row r="187" ht="58" customHeight="1">
-      <c r="B187" s="86" t="n"/>
+    <row r="187" ht="24" customHeight="1">
+      <c r="B187" s="87" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
       <c r="C187" s="82" t="n"/>
       <c r="D187" s="82" t="n"/>
       <c r="E187" s="82" t="n"/>
       <c r="F187" s="71" t="n"/>
     </row>
-    <row r="188" ht="24" customHeight="1"/>
-    <row r="189" ht="58" customHeight="1"/>
-    <row r="190" ht="20" customHeight="1"/>
-    <row r="191" ht="30" customHeight="1"/>
-    <row r="192" ht="58" customHeight="1"/>
-    <row r="193" ht="30" customHeight="1"/>
-    <row r="194" ht="24" customHeight="1"/>
-    <row r="195" ht="32" customHeight="1"/>
+    <row r="188" ht="58" customHeight="1">
+      <c r="B188" s="86" t="n"/>
+      <c r="C188" s="82" t="n"/>
+      <c r="D188" s="82" t="n"/>
+      <c r="E188" s="82" t="n"/>
+      <c r="F188" s="71" t="n"/>
+    </row>
+    <row r="189" ht="24" customHeight="1"/>
+    <row r="190" ht="58" customHeight="1"/>
+    <row r="191" ht="20" customHeight="1"/>
+    <row r="192" ht="30" customHeight="1"/>
+    <row r="193" ht="58" customHeight="1"/>
+    <row r="194" ht="30" customHeight="1"/>
+    <row r="195" ht="24" customHeight="1"/>
     <row r="196" ht="32" customHeight="1"/>
     <row r="197" ht="32" customHeight="1"/>
-    <row r="198" ht="24" customHeight="1"/>
-    <row r="199" ht="32" customHeight="1"/>
+    <row r="198" ht="32" customHeight="1"/>
+    <row r="199" ht="24" customHeight="1"/>
     <row r="200" ht="32" customHeight="1"/>
     <row r="201" ht="32" customHeight="1"/>
-    <row r="202" ht="24" customHeight="1"/>
-    <row r="203" ht="58" customHeight="1"/>
-    <row r="204" ht="20" customHeight="1"/>
-    <row r="205" ht="28" customHeight="1"/>
+    <row r="202" ht="32" customHeight="1"/>
+    <row r="203" ht="24" customHeight="1"/>
+    <row r="204" ht="58" customHeight="1"/>
+    <row r="205" ht="20" customHeight="1"/>
     <row r="206" ht="28" customHeight="1"/>
     <row r="207" ht="28" customHeight="1"/>
-    <row r="208" ht="32" customHeight="1"/>
-    <row r="209" ht="24" customHeight="1"/>
-    <row r="210" ht="58" customHeight="1"/>
-    <row r="211" ht="24" customHeight="1"/>
-    <row r="212" ht="58" customHeight="1"/>
-    <row r="213" ht="24" customHeight="1"/>
-    <row r="214" ht="58" customHeight="1"/>
+    <row r="208" ht="28" customHeight="1"/>
+    <row r="209" ht="32" customHeight="1"/>
+    <row r="210" ht="24" customHeight="1"/>
+    <row r="211" ht="58" customHeight="1"/>
+    <row r="212" ht="24" customHeight="1"/>
+    <row r="213" ht="58" customHeight="1"/>
+    <row r="214" ht="24" customHeight="1"/>
     <row r="215" ht="58" customHeight="1"/>
-    <row r="216" ht="24" customHeight="1"/>
-    <row r="217" ht="58" customHeight="1"/>
-    <row r="218" ht="24" customHeight="1"/>
-    <row r="219" ht="58" customHeight="1"/>
+    <row r="216" ht="58" customHeight="1"/>
+    <row r="217" ht="24" customHeight="1"/>
+    <row r="218" ht="58" customHeight="1"/>
+    <row r="219" ht="24" customHeight="1"/>
+    <row r="220" ht="58" customHeight="1"/>
   </sheetData>
   <mergeCells count="178">
-    <mergeCell ref="B106:F106"/>
+    <mergeCell ref="D76:F76"/>
+    <mergeCell ref="C144:F144"/>
     <mergeCell ref="D116:F116"/>
-    <mergeCell ref="C122:F122"/>
-    <mergeCell ref="B81:F81"/>
-    <mergeCell ref="E129:F129"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B68:E68"/>
     <mergeCell ref="D66:F66"/>
+    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="C125:F125"/>
+    <mergeCell ref="B131:F131"/>
+    <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
-    <mergeCell ref="C125:F125"/>
-    <mergeCell ref="B184:F184"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="B2:F2"/>
     <mergeCell ref="D37:F37"/>
-    <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
-    <mergeCell ref="B92:C93"/>
+    <mergeCell ref="D143:F143"/>
     <mergeCell ref="D152:F152"/>
     <mergeCell ref="B166:F166"/>
-    <mergeCell ref="C172:F172"/>
     <mergeCell ref="D133:F133"/>
     <mergeCell ref="B44:F44"/>
     <mergeCell ref="D142:F142"/>
-    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="B172:F172"/>
+    <mergeCell ref="D129:F129"/>
+    <mergeCell ref="C171:F171"/>
     <mergeCell ref="B186:F186"/>
+    <mergeCell ref="C54:F54"/>
+    <mergeCell ref="B168:F168"/>
+    <mergeCell ref="B92:F92"/>
     <mergeCell ref="C173:F173"/>
-    <mergeCell ref="D128:F128"/>
+    <mergeCell ref="D119:F119"/>
     <mergeCell ref="D159:F159"/>
     <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B94:F94"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="C163:F163"/>
     <mergeCell ref="D105:F105"/>
     <mergeCell ref="D57:F57"/>
-    <mergeCell ref="B144:F144"/>
     <mergeCell ref="C17:F17"/>
-    <mergeCell ref="D120:F120"/>
+    <mergeCell ref="D154:F154"/>
     <mergeCell ref="D41:F41"/>
-    <mergeCell ref="D154:F154"/>
     <mergeCell ref="B185:F185"/>
-    <mergeCell ref="D107:F107"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="C67:F67"/>
+    <mergeCell ref="D147:F147"/>
     <mergeCell ref="C19:F19"/>
-    <mergeCell ref="D147:F147"/>
+    <mergeCell ref="D162:F162"/>
+    <mergeCell ref="B56:F56"/>
     <mergeCell ref="D156:F156"/>
     <mergeCell ref="B167:F167"/>
     <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="B176:F176"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="B176:F176"/>
+    <mergeCell ref="D106:F106"/>
     <mergeCell ref="D137:F137"/>
-    <mergeCell ref="B111:F111"/>
     <mergeCell ref="C96:F96"/>
-    <mergeCell ref="D146:F146"/>
+    <mergeCell ref="B120:F120"/>
+    <mergeCell ref="C175:F175"/>
+    <mergeCell ref="B107:F107"/>
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D83:F83"/>
-    <mergeCell ref="B175:F175"/>
     <mergeCell ref="D117:F117"/>
+    <mergeCell ref="B88:F88"/>
     <mergeCell ref="D157:F157"/>
-    <mergeCell ref="B171:F171"/>
+    <mergeCell ref="C98:F98"/>
+    <mergeCell ref="B82:F82"/>
+    <mergeCell ref="D67:F67"/>
     <mergeCell ref="D132:F132"/>
     <mergeCell ref="D85:F85"/>
-    <mergeCell ref="C162:F162"/>
+    <mergeCell ref="B146:F146"/>
     <mergeCell ref="D60:F60"/>
-    <mergeCell ref="B99:F99"/>
-    <mergeCell ref="D100:F100"/>
     <mergeCell ref="B187:F187"/>
-    <mergeCell ref="C124:F124"/>
+    <mergeCell ref="D109:F109"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D46:F46"/>
+    <mergeCell ref="B124:F124"/>
     <mergeCell ref="D158:F158"/>
     <mergeCell ref="D40:F40"/>
-    <mergeCell ref="C90:F90"/>
-    <mergeCell ref="B76:F76"/>
     <mergeCell ref="D108:F108"/>
     <mergeCell ref="D86:F86"/>
+    <mergeCell ref="C123:F123"/>
+    <mergeCell ref="B188:F188"/>
     <mergeCell ref="D104:F104"/>
     <mergeCell ref="D160:F160"/>
+    <mergeCell ref="C110:F110"/>
+    <mergeCell ref="C181:F181"/>
+    <mergeCell ref="E130:F130"/>
     <mergeCell ref="D136:F136"/>
+    <mergeCell ref="C91:F91"/>
     <mergeCell ref="D150:F150"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="C174:F174"/>
-    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="B55:E55"/>
     <mergeCell ref="D78:F78"/>
+    <mergeCell ref="D87:F87"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C53:F53"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="D122:F122"/>
     <mergeCell ref="D71:F71"/>
-    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="C179:F179"/>
     <mergeCell ref="D58:F58"/>
-    <mergeCell ref="C179:F179"/>
+    <mergeCell ref="C68:F68"/>
     <mergeCell ref="B145:F145"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B81:E81"/>
     <mergeCell ref="D121:F121"/>
-    <mergeCell ref="B181:F181"/>
-    <mergeCell ref="C129:D129"/>
     <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="D82:F82"/>
     <mergeCell ref="D113:F113"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="B87:F87"/>
     <mergeCell ref="C97:F97"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B178:F178"/>
     <mergeCell ref="D148:F148"/>
     <mergeCell ref="D35:F35"/>
-    <mergeCell ref="C143:F143"/>
+    <mergeCell ref="B128:F128"/>
+    <mergeCell ref="D50:F50"/>
     <mergeCell ref="D59:F59"/>
-    <mergeCell ref="C109:F109"/>
     <mergeCell ref="D115:F115"/>
+    <mergeCell ref="B93:C94"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="D34:F34"/>
     <mergeCell ref="B183:F183"/>
+    <mergeCell ref="B65:F65"/>
+    <mergeCell ref="C127:F127"/>
+    <mergeCell ref="C80:F80"/>
     <mergeCell ref="B164:F164"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D84:F84"/>
@@ -5841,60 +5861,49 @@
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="D149:F149"/>
     <mergeCell ref="D45:F45"/>
-    <mergeCell ref="B123:F123"/>
     <mergeCell ref="D101:F101"/>
-    <mergeCell ref="C95:F95"/>
-    <mergeCell ref="C178:F178"/>
-    <mergeCell ref="B163:F163"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="D77:F77"/>
-    <mergeCell ref="B91:F91"/>
+    <mergeCell ref="B99:E99"/>
     <mergeCell ref="D151:F151"/>
+    <mergeCell ref="B100:F100"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="B165:F165"/>
     <mergeCell ref="D141:F141"/>
-    <mergeCell ref="D70:F70"/>
     <mergeCell ref="D135:F135"/>
     <mergeCell ref="D48:F48"/>
     <mergeCell ref="C170:F170"/>
+    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D103:F103"/>
-    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D134:F134"/>
-    <mergeCell ref="B130:F130"/>
-    <mergeCell ref="D112:F112"/>
+    <mergeCell ref="B77:F77"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="D118:F118"/>
-    <mergeCell ref="D56:F56"/>
     <mergeCell ref="D161:F161"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="D114:F114"/>
     <mergeCell ref="C42:F42"/>
     <mergeCell ref="E9:F9"/>
-    <mergeCell ref="B119:F119"/>
+    <mergeCell ref="D64:F64"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="C126:F126"/>
     <mergeCell ref="D89:F89"/>
-    <mergeCell ref="B69:F69"/>
     <mergeCell ref="B182:F182"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="B112:F112"/>
+    <mergeCell ref="D79:F79"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="D88:F88"/>
     <mergeCell ref="D153:F153"/>
-    <mergeCell ref="B127:F127"/>
-    <mergeCell ref="C168:F168"/>
+    <mergeCell ref="B111:E111"/>
     <mergeCell ref="D63:F63"/>
-    <mergeCell ref="B98:E98"/>
     <mergeCell ref="C180:F180"/>
-    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="D90:F90"/>
     <mergeCell ref="B177:F177"/>
-    <mergeCell ref="B64:F64"/>
+    <mergeCell ref="B95:F95"/>
     <mergeCell ref="B33:F33"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="D131:F131"/>
+    <mergeCell ref="B51:F51"/>
     <mergeCell ref="D139:F139"/>
     <mergeCell ref="D52:F52"/>
     <mergeCell ref="C169:F169"/>
-    <mergeCell ref="D49:F49"/>
   </mergeCells>
   <conditionalFormatting sqref="C20:C24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
@@ -6095,13 +6104,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C57 C58 C59 C60 C61 C62 C63 C71 C72 C74 C75 C83 C84 C85 C86 C101 C102 C103 C104 C105 C113 C114 C115 C116 C117 C118" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C50 C58 C59 C60 C61 C62 C63 C64 C72 C73 C75 C76 C84 C85 C86 C87 C102 C103 C104 C105 C106 C114 C115 C116 C117 C118 C119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C41 C52 C66 C78 C89 C108 C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
+    <dataValidation sqref="C41 C53 C67 C79 C90 C109 C122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C128 C132:C142 C151:C161 E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C129 C133:C143 C152:C162 E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6116,16 +6125,16 @@
     <dataValidation sqref="E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Within SLA,Breached,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C124" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Successful Resolution,Partial Resolution,Appropriate Escalation,Ownership Gap,Unresolved"</formula1>
     </dataValidation>
-    <dataValidation sqref="C125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_xlfn._LONGTEXT("Issue resolved,Proper RMA initiated (in-warranty / approved exception),Valid escalation submitted,Known limitation explained accurately,Customer educated with actionable next steps,Valid self-help guidance provided (out-of-warranty),Upgrade path recommend","ed appropriately (out-of-warranty),Customer declined further troubleshooting after reasonable effort,None achieved")</formula1>
     </dataValidation>
-    <dataValidation sqref="C129" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C147:C149" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C148:C150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
     </dataValidation>
   </dataValidations>
@@ -12457,13 +12466,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>

</xml_diff>

<commit_message>
Add comprehensive Scoring Guide sheet with Met/Partial/Missed/N.A. definitions
New 'Scoring Guide' tab covers all 30 active behavioral indicators across
7 scoring categories. Each indicator includes:
- Met: what full achievement looks like (criteria + confirmation)
- Partial: what partial achievement looks like (what is missing)
- Missed: what failure looks like (specific gap)
- N/A: when the indicator does not apply to the interaction

Each rating includes a concrete example scenario drawn from the
Linksys support context (Velop mesh, MX/WHW series, etc.).

Sheet design: color-coded by rating (green/yellow/salmon/grey),
section labels merged across their indicator blocks, frozen header
at row 4, all cells text-wrapped for readability.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -8,12 +8,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Form" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multi-Touch Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multi-Touch Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="39">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -187,8 +187,62 @@
       <sz val="11"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A5E20"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001A1A5E"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B4F00"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B1919"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003D3D3D"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -250,8 +304,53 @@
         <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003F3F3F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -477,11 +576,25 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -837,6 +950,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="18" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="19" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="20" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="20" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6148,472 +6312,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="B1" s="99" t="inlineStr">
-        <is>
-          <t>SCORING GUIDE &amp; CATEGORY CRITERIA</t>
-        </is>
-      </c>
-      <c r="C1" s="90" t="n"/>
-      <c r="D1" s="74" t="n"/>
-    </row>
-    <row r="3">
-      <c r="B3" s="80" t="inlineStr">
-        <is>
-          <t>How to use this form</t>
-        </is>
-      </c>
-      <c r="C3" s="90" t="n"/>
-      <c r="D3" s="74" t="n"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="81" t="inlineStr">
-        <is>
-          <t>1. Fill in Case Information, the Case Summary, and (for multi-touch cases) the Inherited Context field.</t>
-        </is>
-      </c>
-      <c r="C4" s="82" t="n"/>
-      <c r="D4" s="71" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="83" t="inlineStr">
-        <is>
-          <t>2. For each category, rate every behavioral indicator: Met / Partial / Missed / N.A. (N.A. excludes it from the suggested score).</t>
-        </is>
-      </c>
-      <c r="C5" s="82" t="n"/>
-      <c r="D5" s="71" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="81" t="inlineStr">
-        <is>
-          <t>3. Record evidence — quotes, timestamps, or note excerpts — beside each indicator.</t>
-        </is>
-      </c>
-      <c r="C6" s="82" t="n"/>
-      <c r="D6" s="71" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="83" t="inlineStr">
-        <is>
-          <t>4. Review the auto-suggested score, then assign the FINAL 0-5 score using evaluator judgment and the anchors below.</t>
-        </is>
-      </c>
-      <c r="C7" s="82" t="n"/>
-      <c r="D7" s="71" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="81" t="inlineStr">
-        <is>
-          <t>5. Classify the Resolution Outcome and the primary positive outcome achieved.</t>
-        </is>
-      </c>
-      <c r="C8" s="82" t="n"/>
-      <c r="D8" s="71" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="83" t="inlineStr">
-        <is>
-          <t>6. Complete the Disconnect Follow-Up check and the Critical Failure checklist.</t>
-        </is>
-      </c>
-      <c r="C9" s="82" t="n"/>
-      <c r="D9" s="71" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="81" t="inlineStr">
-        <is>
-          <t>7. Write coaching feedback: at least one actionable coaching opportunity is required; add an operational improvement recommendation where applicable.</t>
-        </is>
-      </c>
-      <c r="C10" s="82" t="n"/>
-      <c r="D10" s="71" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="83" t="inlineStr">
-        <is>
-          <t>8. For multi-touch cases, also read the Multi-Touch Guide sheet and log every touch in the Case Tracker under the same Case ID.</t>
-        </is>
-      </c>
-      <c r="C11" s="82" t="n"/>
-      <c r="D11" s="71" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="80" t="inlineStr">
-        <is>
-          <t>Score Anchors (0–5 scale)</t>
-        </is>
-      </c>
-      <c r="C13" s="90" t="n"/>
-      <c r="D13" s="74" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="119" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="C14" s="80" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D14" s="74" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="31" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C15" s="81" t="inlineStr">
-        <is>
-          <t>Issue resolved or strongest available outcome achieved</t>
-        </is>
-      </c>
-      <c r="D15" s="71" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="32" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C16" s="83" t="inlineStr">
-        <is>
-          <t>Significant progress made with clear next steps</t>
-        </is>
-      </c>
-      <c r="D16" s="71" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="31" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C17" s="81" t="inlineStr">
-        <is>
-          <t>Partial progress made but opportunities missed</t>
-        </is>
-      </c>
-      <c r="D17" s="71" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="32" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C18" s="83" t="inlineStr">
-        <is>
-          <t>Limited progress despite available troubleshooting paths</t>
-        </is>
-      </c>
-      <c r="D18" s="71" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C19" s="81" t="inlineStr">
-        <is>
-          <t>Little or no meaningful progress</t>
-        </is>
-      </c>
-      <c r="D19" s="71" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C20" s="83" t="inlineStr">
-        <is>
-          <t>Agent actions delayed, prevented, or negatively impacted resolution</t>
-        </is>
-      </c>
-      <c r="D20" s="71" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="80" t="inlineStr">
-        <is>
-          <t>Indicator ratings</t>
-        </is>
-      </c>
-      <c r="C22" s="90" t="n"/>
-      <c r="D22" s="74" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="31" t="inlineStr">
-        <is>
-          <t>Met</t>
-        </is>
-      </c>
-      <c r="C23" s="81" t="inlineStr">
-        <is>
-          <t>Behavior fully demonstrated (counts as 5 toward the suggested score)</t>
-        </is>
-      </c>
-      <c r="D23" s="71" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="C24" s="83" t="inlineStr">
-        <is>
-          <t>Behavior attempted but incomplete or inconsistent (counts as 2.5)</t>
-        </is>
-      </c>
-      <c r="D24" s="71" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="31" t="inlineStr">
-        <is>
-          <t>Missed</t>
-        </is>
-      </c>
-      <c r="C25" s="81" t="inlineStr">
-        <is>
-          <t>Behavior expected but not demonstrated (counts as 0)</t>
-        </is>
-      </c>
-      <c r="D25" s="71" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="32" t="inlineStr">
-        <is>
-          <t>N.A.</t>
-        </is>
-      </c>
-      <c r="C26" s="83" t="inlineStr">
-        <is>
-          <t>Not applicable to this interaction (excluded from the suggested score)</t>
-        </is>
-      </c>
-      <c r="D26" s="71" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="80" t="inlineStr">
-        <is>
-          <t>Category Objectives &amp; Watch-Fors</t>
-        </is>
-      </c>
-      <c r="C28" s="90" t="n"/>
-      <c r="D28" s="74" t="n"/>
-    </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>Resolution / Progress Toward Resolution (30%)</t>
-        </is>
-      </c>
-      <c r="C29" s="81" t="inlineStr">
-        <is>
-          <t>Determine whether the interaction moved the customer meaningfully closer to resolution. Does NOT count: customer simply ends call; generic KB sent without troubleshooting; warranty used as reason to stop helping; escalation as shortcut; unsupported ISP blame; 'monitor &amp; call back' with no plan; ownership transferred without expectations or documentation.</t>
-        </is>
-      </c>
-      <c r="D29" s="71" t="n"/>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="B30" s="34" t="inlineStr">
-        <is>
-          <t>Technical Accuracy (20%)</t>
-        </is>
-      </c>
-      <c r="C30" s="100" t="inlineStr">
-        <is>
-          <t>Evaluate the quality of troubleshooting and technical guidance. Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
-        </is>
-      </c>
-      <c r="D30" s="71" t="n"/>
-    </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t>Communication &amp; Call Control (15%)</t>
-        </is>
-      </c>
-      <c r="C31" s="81" t="inlineStr">
-        <is>
-          <t>Evaluate how effectively the agent managed the interaction. High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
-        </is>
-      </c>
-      <c r="D31" s="71" t="n"/>
-    </row>
-    <row r="32" ht="60" customHeight="1">
-      <c r="B32" s="34" t="inlineStr">
-        <is>
-          <t>Customer Ownership (15%)</t>
-        </is>
-      </c>
-      <c r="C32" s="100" t="inlineStr">
-        <is>
-          <t>Measure the degree to which the agent accepted responsibility for moving the customer forward. Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
-        </is>
-      </c>
-      <c r="D32" s="71" t="n"/>
-    </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>Escalation Judgment (10%)</t>
-        </is>
-      </c>
-      <c r="C33" s="81" t="inlineStr">
-        <is>
-          <t>Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted. Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
-        </is>
-      </c>
-      <c r="D33" s="71" t="n"/>
-    </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="B34" s="34" t="inlineStr">
-        <is>
-          <t>Customer Experience (5%)</t>
-        </is>
-      </c>
-      <c r="C34" s="100" t="inlineStr">
-        <is>
-          <t>Measure the overall customer experience delivered during the interaction. Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="D34" s="71" t="n"/>
-    </row>
-    <row r="35" ht="60" customHeight="1">
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>Documentation &amp; Notes (5%)</t>
-        </is>
-      </c>
-      <c r="C35" s="81" t="inlineStr">
-        <is>
-          <t>Ensure future agents can quickly understand the case. Purpose is continuity, not compliance. Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="D35" s="71" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="80" t="inlineStr">
-        <is>
-          <t>Overall Result Bands</t>
-        </is>
-      </c>
-      <c r="C37" s="90" t="n"/>
-      <c r="D37" s="74" t="n"/>
-    </row>
-    <row r="38">
-      <c r="B38" s="36" t="inlineStr">
-        <is>
-          <t>≥ 85%</t>
-        </is>
-      </c>
-      <c r="C38" s="104" t="inlineStr">
-        <is>
-          <t>Meets / Exceeds — strong support behavior</t>
-        </is>
-      </c>
-      <c r="D38" s="71" t="n"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="37" t="inlineStr">
-        <is>
-          <t>70–84%</t>
-        </is>
-      </c>
-      <c r="C39" s="103" t="inlineStr">
-        <is>
-          <t>Developing — coaching opportunities present</t>
-        </is>
-      </c>
-      <c r="D39" s="71" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="38" t="inlineStr">
-        <is>
-          <t>&lt; 70%</t>
-        </is>
-      </c>
-      <c r="C40" s="102" t="inlineStr">
-        <is>
-          <t>Needs improvement — prioritized coaching required</t>
-        </is>
-      </c>
-      <c r="D40" s="71" t="n"/>
-    </row>
-    <row r="42" ht="40" customHeight="1">
-      <c r="B42" s="101" t="inlineStr">
-        <is>
-          <t>A critical failure overrides the band: any flagged condition requires automatic review regardless of the weighted total. Every review must produce at least one actionable coaching opportunity and, where applicable, one operational improvement recommendation.</t>
-        </is>
-      </c>
-      <c r="C42" s="90" t="n"/>
-      <c r="D42" s="74" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C18:D18"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="B1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
@@ -7073,7 +6771,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7947,7 +7645,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10939,7 +10637,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12466,13 +12164,13 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
     <mergeCell ref="A3:P3"/>
     <mergeCell ref="A51:D51"/>
-    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A55:B55"/>
@@ -12585,7 +12283,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12989,4 +12687,2564 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E143"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="127" t="inlineStr">
+        <is>
+          <t>QA SCORING GUIDE — Behavioral Indicator Rating Definitions &amp; Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="128" t="inlineStr">
+        <is>
+          <t>Met = fully achieved  ·  Partial = achieved in part  ·  Missed = not achieved  ·  N/A = not applicable to this interaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="129" t="inlineStr">
+        <is>
+          <t>Category / Section</t>
+        </is>
+      </c>
+      <c r="B3" s="129" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C3" s="129" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="D3" s="129" t="inlineStr">
+        <is>
+          <t>What This Looks Like</t>
+        </is>
+      </c>
+      <c r="E3" s="129" t="inlineStr">
+        <is>
+          <t>Example Scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
+      <c r="A4" s="130" t="inlineStr">
+        <is>
+          <t>1 · RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
+        </is>
+      </c>
+      <c r="B4" s="131" t="inlineStr">
+        <is>
+          <t>Resolved the issue or achieved the best possible outcome
+(RMA, valid escalation, limitation explained, education)</t>
+        </is>
+      </c>
+      <c r="C4" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D4" s="133" t="inlineStr">
+        <is>
+          <t>Issue fully resolved and confirmed with the customer. Alternatively, the strongest available outcome was properly executed: RMA correctly initiated, valid escalation submitted with complete documentation, product limitation accurately explained, or appropriate customer education provided.</t>
+        </is>
+      </c>
+      <c r="E4" s="134" t="inlineStr">
+        <is>
+          <t>Customer reported no internet on Velop node. Agent guided 5-press reset and re-pairing. Node showed solid white. Customer confirmed internet restored and agent verified before closing. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="C5" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D5" s="136" t="inlineStr">
+        <is>
+          <t>An outcome was pursued but not fully executed or confirmed — RMA initiated but missing a required field, escalation submitted with sparse notes, or issue appeared resolved but the customer did not confirm.</t>
+        </is>
+      </c>
+      <c r="E5" s="137" t="inlineStr">
+        <is>
+          <t>Agent guided a factory reset. Node appeared to re-pair. Agent closed the ticket without asking the customer to test internet. Customer did not confirm. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="C6" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D6" s="139" t="inlineStr">
+        <is>
+          <t>Case closed without any meaningful outcome. Generic KB link sent without investigation. Escalation used with no prior troubleshooting. Out-of-warranty product dismissed with no attempt to help.</t>
+        </is>
+      </c>
+      <c r="E6" s="140" t="inlineStr">
+        <is>
+          <t>Customer called about no internet. Agent immediately sent a KB article without asking any questions, then marked the ticket Resolved. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="C7" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D7" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Every interaction must produce some form of documented outcome or attempt.</t>
+        </is>
+      </c>
+      <c r="E7" s="143" t="inlineStr"/>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="B8" s="131" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
+        </is>
+      </c>
+      <c r="C8" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D8" s="133" t="inlineStr">
+        <is>
+          <t>Agent worked through relevant diagnostic steps — appropriate to the product and symptom — before arriving at any conclusion. Steps were logical, sequenced, and evidence-based.</t>
+        </is>
+      </c>
+      <c r="E8" s="134" t="inlineStr">
+        <is>
+          <t>Customer reported intermittent drops. Agent checked for IP conflicts, verified firmware version, tested wired vs. wireless, confirmed drops were wireless-only, identified channel congestion and changed channels. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="C9" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D9" s="136" t="inlineStr">
+        <is>
+          <t>Some troubleshooting was done but key steps were skipped. Conclusion reached without fully validating all likely causes.</t>
+        </is>
+      </c>
+      <c r="E9" s="137" t="inlineStr">
+        <is>
+          <t>Customer reported no internet. Agent rebooted the router without first verifying the modem had a working WAN connection. The modem was offline. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="C10" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D10" s="139" t="inlineStr">
+        <is>
+          <t>No meaningful troubleshooting performed. Agent jumped to a conclusion, blamed ISP without evidence, or escalated after a single failed step.</t>
+        </is>
+      </c>
+      <c r="E10" s="140" t="inlineStr">
+        <is>
+          <t>Customer reported slow speeds. Agent immediately told the customer to contact their ISP without running any diagnostics. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="C11" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D11" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Troubleshooting is always possible or its absence must be documented.</t>
+        </is>
+      </c>
+      <c r="E11" s="143" t="inlineStr"/>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="B12" s="131" t="inlineStr">
+        <is>
+          <t>Resolution path was appropriate for the situation and warranty status</t>
+        </is>
+      </c>
+      <c r="C12" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D12" s="133" t="inlineStr">
+        <is>
+          <t>Agent correctly determined warranty status and recommended the right resolution path for the situation: in-warranty hardware failure → RMA; out-of-warranty → self-help or paid support; software or config issue → troubleshooting; known limitation → education.</t>
+        </is>
+      </c>
+      <c r="E12" s="134" t="inlineStr">
+        <is>
+          <t>Customer reported a hardware failure 8 months after purchase. Agent verified in-warranty status, confirmed the fault through troubleshooting, and correctly initiated an RMA. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="C13" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D13" s="136" t="inlineStr">
+        <is>
+          <t>Resolution path was mostly right but one element was misaligned — offered paid support when product was in warranty, or denied help to an in-warranty customer citing an incorrect out-of-warranty determination.</t>
+        </is>
+      </c>
+      <c r="E13" s="137" t="inlineStr">
+        <is>
+          <t>Customer had an in-warranty device with a confirmed hardware fault. Agent correctly identified the issue but initially offered paid remote support before being corrected. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="C14" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D14" s="139" t="inlineStr">
+        <is>
+          <t>Completely wrong path taken — free replacement for a clearly out-of-warranty product; denied assistance to in-warranty customer; escalated a simple config issue without troubleshooting.</t>
+        </is>
+      </c>
+      <c r="E14" s="140" t="inlineStr">
+        <is>
+          <t>Agent told the customer their 3-year-old router was still under warranty and initiated an RMA that would later be rejected. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="C15" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D15" s="142" t="inlineStr">
+        <is>
+          <t>N/A only when warranty status was genuinely impossible to determine despite a reasonable lookup, and agent documented that limitation.</t>
+        </is>
+      </c>
+      <c r="E15" s="143" t="inlineStr"/>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="B16" s="131" t="inlineStr">
+        <is>
+          <t>Customer was moved meaningfully closer to a solution</t>
+        </is>
+      </c>
+      <c r="C16" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D16" s="133" t="inlineStr">
+        <is>
+          <t>The interaction produced real, documented progress — the issue was resolved, a specific actionable next step was executed, or the customer's situation clearly advanced (RMA in process, escalation queued with full context, specific fix confirmed).</t>
+        </is>
+      </c>
+      <c r="E16" s="134" t="inlineStr">
+        <is>
+          <t>Issue was not fully resolved but agent identified the root cause, submitted a complete escalation to the right team, and customer understood the next step. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
+      <c r="C17" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D17" s="136" t="inlineStr">
+        <is>
+          <t>Some progress was made but the outcome was unclear or the next step was vague. Customer was helped but left without a clear picture of where things stand.</t>
+        </is>
+      </c>
+      <c r="E17" s="137" t="inlineStr">
+        <is>
+          <t>Agent troubleshot and suggested the customer 'monitor and see if it happens again' with no timeframe, no trigger condition, and no follow-up plan. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1">
+      <c r="C18" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D18" s="139" t="inlineStr">
+        <is>
+          <t>Customer ends the interaction in the same state as when they called — no resolution, no clear next step, no advancement toward a fix.</t>
+        </is>
+      </c>
+      <c r="E18" s="140" t="inlineStr">
+        <is>
+          <t>After a 30-minute call, agent concluded 'it might be your ISP' with no evidence and no follow-up plan, then closed the ticket. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="C19" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D19" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E19" s="143" t="inlineStr"/>
+    </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="130" t="inlineStr">
+        <is>
+          <t>2 · TECHNICAL ACCURACY</t>
+        </is>
+      </c>
+      <c r="B20" s="131" t="inlineStr">
+        <is>
+          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
+        </is>
+      </c>
+      <c r="C20" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D20" s="133" t="inlineStr">
+        <is>
+          <t>Agent identified the specific symptom — not just 'internet issue' — and asked targeted follow-up questions to narrow scope: which devices affected, wired vs. wireless, when it started, any recent changes.</t>
+        </is>
+      </c>
+      <c r="E20" s="134" t="inlineStr">
+        <is>
+          <t>Customer said 'internet is down.' Agent asked: all devices or one? Wired or wireless? When did it start? Anything change recently? Identified the issue was wireless-only on one device, not a full outage. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="C21" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D21" s="136" t="inlineStr">
+        <is>
+          <t>Symptoms partially identified but agent asked generic questions without building on the answers; or missed a key clarifying question that would have changed the diagnostic path.</t>
+        </is>
+      </c>
+      <c r="E21" s="137" t="inlineStr">
+        <is>
+          <t>Customer reported 'internet issues.' Agent asked for the router model and ran a standard reset without determining whether the problem was connectivity, speed, or intermittent. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="C22" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D22" s="139" t="inlineStr">
+        <is>
+          <t>Agent proceeded with generic troubleshooting without understanding the actual symptom; or misidentified the symptom and pursued the wrong path entirely.</t>
+        </is>
+      </c>
+      <c r="E22" s="140" t="inlineStr">
+        <is>
+          <t>Customer reported slow speeds. Agent assumed it was a full outage and guided a factory reset. The actual issue was a speed tier mismatch with the ISP. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="C23" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D23" s="142" t="inlineStr">
+        <is>
+          <t>Customer immediately requested escalation and declined any diagnostic interaction.</t>
+        </is>
+      </c>
+      <c r="E23" s="143" t="inlineStr"/>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="B24" s="131" t="inlineStr">
+        <is>
+          <t>Identified the root cause (or likely cause) when possible</t>
+        </is>
+      </c>
+      <c r="C24" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D24" s="133" t="inlineStr">
+        <is>
+          <t>Based on evidence gathered, agent correctly identified the root cause or articulated the most likely cause with supporting observations — not a guess, but a conclusion drawn from test results and symptoms.</t>
+        </is>
+      </c>
+      <c r="E24" s="134" t="inlineStr">
+        <is>
+          <t>After finding wired connection fine but wireless dropping, and noting drops coincided with device movement, agent concluded: likely signal interference or channel congestion on the 2.4 GHz band — supported by evidence. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="C25" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D25" s="136" t="inlineStr">
+        <is>
+          <t>Agent identified a possible cause but could not narrow it down further, or stated a cause without supporting evidence. Cause was speculative.</t>
+        </is>
+      </c>
+      <c r="E25" s="137" t="inlineStr">
+        <is>
+          <t>Agent said 'it's probably the firmware' without checking the firmware version or running any test to support that conclusion. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
+      <c r="C26" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D26" s="139" t="inlineStr">
+        <is>
+          <t>Agent failed to identify a cause or stated an unsupported cause — ISP blame, customer-side blame — without running any diagnostic to justify it.</t>
+        </is>
+      </c>
+      <c r="E26" s="140" t="inlineStr">
+        <is>
+          <t>After a single failed ping test, agent concluded 'it must be your ISP' without checking modem status, WAN connection, or any device-side diagnostics. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="C27" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" s="142" t="inlineStr">
+        <is>
+          <t>Issue resolved without a definitive cause identifiable (e.g., self-clearing intermittent fault); or customer declined further investigation after an initial fix attempt.</t>
+        </is>
+      </c>
+      <c r="E27" s="143" t="inlineStr"/>
+    </row>
+    <row r="28" ht="72" customHeight="1">
+      <c r="B28" s="131" t="inlineStr">
+        <is>
+          <t>Followed a logical troubleshooting process</t>
+        </is>
+      </c>
+      <c r="C28" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D28" s="133" t="inlineStr">
+        <is>
+          <t>Steps built on each other in a structured sequence — simple checks before complex changes, verification before action, each step building on the previous result. No skipping foundational checks.</t>
+        </is>
+      </c>
+      <c r="E28" s="134" t="inlineStr">
+        <is>
+          <t>Agent verified modem online → confirmed WAN port connection → opened router admin page → identified duplicate IP assignment → fixed with static IP. Clear progression from ISP side inward. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
+      <c r="C29" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D29" s="136" t="inlineStr">
+        <is>
+          <t>Generally logical but steps were slightly out of order or a key verification step was skipped.</t>
+        </is>
+      </c>
+      <c r="E29" s="137" t="inlineStr">
+        <is>
+          <t>Agent guided a full factory reset without first verifying the modem had a working internet connection. The actual problem was the modem, which L2 identified immediately. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="C30" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D30" s="139" t="inlineStr">
+        <is>
+          <t>Troubleshooting was random, reversed (complex before simple), or repeated unnecessarily with no response to the outcomes.</t>
+        </is>
+      </c>
+      <c r="E30" s="140" t="inlineStr">
+        <is>
+          <t>Agent had the customer reset the router three times, then recommended a firmware update, then another factory reset — no logic, no response to results at each step. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="C31" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D31" s="142" t="inlineStr">
+        <is>
+          <t>No troubleshooting was applicable — product end-of-life with no available fix, or customer declined.</t>
+        </is>
+      </c>
+      <c r="E31" s="143" t="inlineStr"/>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="B32" s="131" t="inlineStr">
+        <is>
+          <t>Available tools were used efficiently and appropriately</t>
+        </is>
+      </c>
+      <c r="C32" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D32" s="133" t="inlineStr">
+        <is>
+          <t>Agent used relevant tools at the right point in the process — remote session when hands-on was needed, admin dashboard for logs, modem test for WAN verification, KB for procedure confirmation — and interpreted results correctly.</t>
+        </is>
+      </c>
+      <c r="E32" s="134" t="inlineStr">
+        <is>
+          <t>Agent remotely accessed the router admin panel, reviewed the DHCP lease table and event logs, identified a firmware error code, cross-referenced the KB, and pinpointed the fix without requiring the customer to navigate menus. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="C33" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D33" s="136" t="inlineStr">
+        <is>
+          <t>Agent used some tools but missed relevant ones; or used a tool at the wrong moment; or initiated a tool but could not correctly interpret the results.</t>
+        </is>
+      </c>
+      <c r="E33" s="137" t="inlineStr">
+        <is>
+          <t>Agent ran a speed test (appropriate) but did not check event logs or the admin panel, which would have shown the firmware error causing the speed issue. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="C34" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D34" s="139" t="inlineStr">
+        <is>
+          <t>Agent did not use any available tools despite the situation requiring them; or used a tool that was irrelevant to the reported symptom.</t>
+        </is>
+      </c>
+      <c r="E34" s="140" t="inlineStr">
+        <is>
+          <t>Customer reported frequent node drops. Agent only asked the customer to visually describe the LEDs rather than using the remote session or admin panel already available. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="C35" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D35" s="142" t="inlineStr">
+        <is>
+          <t>No tools were available or applicable — offline issue prevented tool access; or customer declined remote assistance.</t>
+        </is>
+      </c>
+      <c r="E35" s="143" t="inlineStr"/>
+    </row>
+    <row r="36" ht="72" customHeight="1">
+      <c r="B36" s="131" t="inlineStr">
+        <is>
+          <t>Gave technically accurate information; no unsupported conclusions</t>
+        </is>
+      </c>
+      <c r="C36" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D36" s="133" t="inlineStr">
+        <is>
+          <t>All technical guidance, product specifications, and procedural instructions were factually correct and aligned with KB documentation. Agent validated assumptions before presenting conclusions.</t>
+        </is>
+      </c>
+      <c r="E36" s="134" t="inlineStr">
+        <is>
+          <t>Agent correctly described the Velop factory reset as 10 seconds, confirmed the LED sequence per KB, and matched the admin password to the product label. All verified before advising. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="C37" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D37" s="136" t="inlineStr">
+        <is>
+          <t>Most information was accurate but one or two minor inaccuracies were present — slightly wrong reset duration, incorrect LED color description — unlikely to cause serious harm but reflecting a knowledge gap.</t>
+        </is>
+      </c>
+      <c r="E37" s="137" t="inlineStr">
+        <is>
+          <t>Agent said the reset required 'about 10 to 15 seconds' (KB specifies 10). Customer held the button too long and triggered a factory reset when a soft reset was intended. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="C38" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D38" s="139" t="inlineStr">
+        <is>
+          <t>Agent provided materially incorrect information — wrong default password, non-existent LED state, unsupported pairing method, or made claims without evidence (ISP blame, customer-side blame).</t>
+        </is>
+      </c>
+      <c r="E38" s="140" t="inlineStr">
+        <is>
+          <t>Agent told the customer the default admin password was 'admin admin.' Customer could not access the admin panel. The correct credential was printed on the device label. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="C39" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D39" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Technical accuracy is always required.</t>
+        </is>
+      </c>
+      <c r="E39" s="143" t="inlineStr"/>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" s="130" t="inlineStr">
+        <is>
+          <t>3 · COMMUNICATION &amp; CALL CONTROL</t>
+        </is>
+      </c>
+      <c r="B40" s="131" t="inlineStr">
+        <is>
+          <t>Expectations were set clearly from the start</t>
+        </is>
+      </c>
+      <c r="C40" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D40" s="133" t="inlineStr">
+        <is>
+          <t>Agent acknowledged the issue, outlined what the interaction would involve, and gave a realistic estimate of time and likely outcome at the opening of the call. Customer knew what to expect before troubleshooting began.</t>
+        </is>
+      </c>
+      <c r="E40" s="134" t="inlineStr">
+        <is>
+          <t>'I can see you're having connectivity issues. I'm going to walk you through a few diagnostic steps — should take about 10–15 minutes. Our goal is to get you back online today or confirm the next step.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="C41" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D41" s="136" t="inlineStr">
+        <is>
+          <t>Agent acknowledged the issue but gave no indication of what to expect in terms of process, time, or possible outcome.</t>
+        </is>
+      </c>
+      <c r="E41" s="137" t="inlineStr">
+        <is>
+          <t>Agent said 'I'll help you with that' and immediately started troubleshooting without framing the interaction. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="72" customHeight="1">
+      <c r="C42" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D42" s="139" t="inlineStr">
+        <is>
+          <t>Agent went directly into troubleshooting with no introduction, no framing, and no expectation-setting of any kind.</t>
+        </is>
+      </c>
+      <c r="E42" s="140" t="inlineStr">
+        <is>
+          <t>Agent's first statement was 'Have you tried restarting your router?' with no acknowledgment of the issue or explanation of what was about to happen. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="72" customHeight="1">
+      <c r="C43" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D43" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Expectations can always be set, even briefly.</t>
+        </is>
+      </c>
+      <c r="E43" s="143" t="inlineStr"/>
+    </row>
+    <row r="44" ht="72" customHeight="1">
+      <c r="B44" s="131" t="inlineStr">
+        <is>
+          <t>Agent maintained call control and troubleshooting flow</t>
+        </is>
+      </c>
+      <c r="C44" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D44" s="133" t="inlineStr">
+        <is>
+          <t>Agent kept the conversation on track, redirected tangents professionally, paced the troubleshooting steps deliberately, and ensured the diagnostic path remained purposeful throughout.</t>
+        </is>
+      </c>
+      <c r="E44" s="134" t="inlineStr">
+        <is>
+          <t>When the customer started discussing a separate device issue, agent said: 'That's worth looking at — let's note that and address it right after we sort the connectivity issue. Can you try the reset now?' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="72" customHeight="1">
+      <c r="C45" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D45" s="136" t="inlineStr">
+        <is>
+          <t>Agent generally maintained control but lost direction at one or two points — allowed a long tangent, let the customer perform steps out of order, or lost momentum mid-call.</t>
+        </is>
+      </c>
+      <c r="E45" s="137" t="inlineStr">
+        <is>
+          <t>Agent allowed the customer to spend 10 minutes describing their internet history before redirecting. The call ran significantly long as a result. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="72" customHeight="1">
+      <c r="C46" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D46" s="139" t="inlineStr">
+        <is>
+          <t>Customer dominated the interaction. Agent was reactive throughout, allowed the customer to dictate the troubleshooting path, or the interaction lacked any meaningful structure.</t>
+        </is>
+      </c>
+      <c r="E46" s="140" t="inlineStr">
+        <is>
+          <t>Customer insisted 'just replace it.' Agent agreed to submit an RMA without completing any troubleshooting, despite the issue being a misconfigured setting fixable in minutes. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="72" customHeight="1">
+      <c r="C47" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D47" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E47" s="143" t="inlineStr"/>
+    </row>
+    <row r="48" ht="72" customHeight="1">
+      <c r="B48" s="131" t="inlineStr">
+        <is>
+          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+        </is>
+      </c>
+      <c r="C48" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D48" s="133" t="inlineStr">
+        <is>
+          <t>Agent adapted terminology to the customer's demonstrated level — explained jargon when used, avoided unnecessary technical terms with non-technical customers, and verified comprehension at key transition points.</t>
+        </is>
+      </c>
+      <c r="E48" s="134" t="inlineStr">
+        <is>
+          <t>For an elderly customer, agent said 'Find the small button on the back of the router — it may say Reset next to it. Let me know when you find it.' Rather than 'Locate the factory reset pinhole adjacent to the WAN port.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="72" customHeight="1">
+      <c r="C49" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D49" s="136" t="inlineStr">
+        <is>
+          <t>Language was mostly appropriate but agent used unexplained jargon on one or two occasions, or confirmed understanding only at the end rather than throughout.</t>
+        </is>
+      </c>
+      <c r="E49" s="137" t="inlineStr">
+        <is>
+          <t>Agent used the term 'DHCP lease' without explanation. Customer nodded along but was clearly confused. Agent did not notice and moved on. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="72" customHeight="1">
+      <c r="C50" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D50" s="139" t="inlineStr">
+        <is>
+          <t>Agent used technical language throughout with no adaptation. Customer was visibly confused at multiple points and agent never addressed the comprehension gaps.</t>
+        </is>
+      </c>
+      <c r="E50" s="140" t="inlineStr">
+        <is>
+          <t>Agent walked a non-technical customer through MAC filtering and DNS settings without checking whether the customer understood what these terms meant. Customer followed instructions incorrectly. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="72" customHeight="1">
+      <c r="C51" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D51" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E51" s="143" t="inlineStr"/>
+    </row>
+    <row r="52" ht="72" customHeight="1">
+      <c r="B52" s="131" t="inlineStr">
+        <is>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
+        </is>
+      </c>
+      <c r="C52" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D52" s="133" t="inlineStr">
+        <is>
+          <t>Agent demonstrated active listening — accurately reflected back what the customer said, built each question on the previous answer, and never asked for information the customer had already provided.</t>
+        </is>
+      </c>
+      <c r="E52" s="134" t="inlineStr">
+        <is>
+          <t>Customer mentioned the issue started after a power outage. Later, agent said: 'Since you mentioned the power outage, let's check whether the router's settings were affected — that can happen when power is cut abruptly.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="72" customHeight="1">
+      <c r="C53" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D53" s="136" t="inlineStr">
+        <is>
+          <t>Agent generally listened but repeated a question already answered, or moved forward without fully incorporating a key detail the customer had shared.</t>
+        </is>
+      </c>
+      <c r="E53" s="137" t="inlineStr">
+        <is>
+          <t>Customer mentioned they had already rebooted the router three times. Agent's next instruction was to reboot the router — without acknowledging this. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1">
+      <c r="C54" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D54" s="139" t="inlineStr">
+        <is>
+          <t>Agent repeatedly asked for information already provided, talked over the customer, or failed to incorporate what the customer said into the troubleshooting approach.</t>
+        </is>
+      </c>
+      <c r="E54" s="140" t="inlineStr">
+        <is>
+          <t>Customer provided the router model, purchase date, and symptom upfront. Agent then asked for the router model, purchase date, and symptom again as if the customer had said nothing. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1">
+      <c r="C55" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D55" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E55" s="143" t="inlineStr"/>
+    </row>
+    <row r="56" ht="72" customHeight="1">
+      <c r="B56" s="131" t="inlineStr">
+        <is>
+          <t>Managed time well, with clear transitions between steps</t>
+        </is>
+      </c>
+      <c r="C56" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D56" s="133" t="inlineStr">
+        <is>
+          <t>Interaction was efficient. Holds were managed with advance notice and updates. Agent transitioned clearly between troubleshooting phases using narration to keep the customer oriented.</t>
+        </is>
+      </c>
+      <c r="E56" s="134" t="inlineStr">
+        <is>
+          <t>'We've confirmed the modem is working — good. Now let's look at the router. I'm going to put you on a brief hold to pull your device history — back in about 2 minutes.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="72" customHeight="1">
+      <c r="C57" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D57" s="136" t="inlineStr">
+        <is>
+          <t>Time management was generally adequate but there were noticeable silences, abrupt transitions between steps, or holds placed without warning.</t>
+        </is>
+      </c>
+      <c r="E57" s="137" t="inlineStr">
+        <is>
+          <t>Agent placed the customer on hold without warning three times, returning each time to ask a new question rather than coming back with an answer. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="72" customHeight="1">
+      <c r="C58" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D58" s="139" t="inlineStr">
+        <is>
+          <t>Interaction ran well beyond what was necessary. Long unexplained silences. Customer left waiting with no update. Steps repeated unnecessarily.</t>
+        </is>
+      </c>
+      <c r="E58" s="140" t="inlineStr">
+        <is>
+          <t>Agent left the customer on silent hold for 8 minutes with no update, returned to ask questions already answered, and the call ended unresolved after 45 minutes. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="72" customHeight="1">
+      <c r="C59" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D59" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E59" s="143" t="inlineStr"/>
+    </row>
+    <row r="60" ht="72" customHeight="1">
+      <c r="B60" s="131" t="inlineStr">
+        <is>
+          <t>Handled difficult moments when needed to maintain call control</t>
+        </is>
+      </c>
+      <c r="C60" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D60" s="133" t="inlineStr">
+        <is>
+          <t>When the customer became frustrated, escalatory, or emotional, agent acknowledged the feeling empathetically, maintained composure, de-escalated professionally, and returned the interaction to productive troubleshooting.</t>
+        </is>
+      </c>
+      <c r="E60" s="134" t="inlineStr">
+        <is>
+          <t>When customer said 'I've called three times and no one can fix this!' agent responded: 'I completely understand — that's incredibly frustrating, and I'm sorry. I'm going to review everything from your prior contacts and give this my full attention right now.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="72" customHeight="1">
+      <c r="C61" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D61" s="136" t="inlineStr">
+        <is>
+          <t>Agent attempted to handle the moment but de-escalation was mechanical or brief. Customer remained frustrated but interaction continued. Professionalism maintained.</t>
+        </is>
+      </c>
+      <c r="E61" s="137" t="inlineStr">
+        <is>
+          <t>Customer was angry. Agent said 'I understand your frustration' and immediately moved to the next step without genuine acknowledgment. Customer stayed agitated. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="72" customHeight="1">
+      <c r="C62" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D62" s="139" t="inlineStr">
+        <is>
+          <t>Agent ignored frustration, matched negative energy, became defensive, or allowed the difficult moment to derail the interaction entirely.</t>
+        </is>
+      </c>
+      <c r="E62" s="140" t="inlineStr">
+        <is>
+          <t>Customer raised their voice. Agent responded: 'I'm just trying to help you, there's no need to be rude.' Customer escalated further and requested a supervisor. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="72" customHeight="1">
+      <c r="C63" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D63" s="142" t="inlineStr">
+        <is>
+          <t>No difficult moments occurred — customer was cooperative throughout the interaction.</t>
+        </is>
+      </c>
+      <c r="E63" s="143" t="inlineStr"/>
+    </row>
+    <row r="64" ht="72" customHeight="1">
+      <c r="B64" s="131" t="inlineStr">
+        <is>
+          <t>Adjusted communication for the customer's accessibility needs
+(hearing, vision, language barrier, age, cognitive)</t>
+        </is>
+      </c>
+      <c r="C64" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D64" s="133" t="inlineStr">
+        <is>
+          <t>Agent identified or proactively accommodated an accessibility need and measurably adjusted delivery — slower speech, simpler vocabulary, avoiding visual-reference instructions, using plain step-by-step guidance suited to the customer's specific limitation.</t>
+        </is>
+      </c>
+      <c r="E64" s="134" t="inlineStr">
+        <is>
+          <t>Customer mentioned they were hard of hearing. Agent slowed their pace, spoke clearly, emailed all instructions as numbered steps, and confirmed each step was understood before moving on. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="72" customHeight="1">
+      <c r="C65" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D65" s="136" t="inlineStr">
+        <is>
+          <t>Agent partially accommodated — slowed down initially but reverted to standard pace; or addressed one aspect of the need but overlooked another.</t>
+        </is>
+      </c>
+      <c r="E65" s="137" t="inlineStr">
+        <is>
+          <t>Agent noticed a language barrier and simplified vocabulary but still used terms like 'firmware' and 'SSID' without explanation. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="72" customHeight="1">
+      <c r="C66" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D66" s="139" t="inlineStr">
+        <is>
+          <t>Agent was aware of or should have been aware of an accessibility need and made no accommodation. Instructions were inaccessible or impractical for the customer.</t>
+        </is>
+      </c>
+      <c r="E66" s="140" t="inlineStr">
+        <is>
+          <t>Customer mentioned they could not see the back of the router clearly. Agent continued giving visual-reference instructions ('the button is next to the yellow port') without offering an alternative. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="72" customHeight="1">
+      <c r="C67" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D67" s="142" t="inlineStr">
+        <is>
+          <t>No accessibility accommodation was required — customer had no communication barrier.</t>
+        </is>
+      </c>
+      <c r="E67" s="143" t="inlineStr"/>
+    </row>
+    <row r="68" ht="72" customHeight="1">
+      <c r="A68" s="130" t="inlineStr">
+        <is>
+          <t>4 · CUSTOMER OWNERSHIP</t>
+        </is>
+      </c>
+      <c r="B68" s="131" t="inlineStr">
+        <is>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
+        </is>
+      </c>
+      <c r="C68" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D68" s="133" t="inlineStr">
+        <is>
+          <t>Agent owned the case from contact to close, made reasonable efforts to resolve or advance it personally, and only transferred when there was a clear, documented legitimate reason — wrong queue, specialized team required after L1 work was completed.</t>
+        </is>
+      </c>
+      <c r="E68" s="134" t="inlineStr">
+        <is>
+          <t>Agent inherited a complex multi-touch case, reviewed all prior notes, re-diagnosed without making the customer repeat everything, and escalated only after completing thorough L1 troubleshooting with full documentation. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="72" customHeight="1">
+      <c r="C69" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D69" s="136" t="inlineStr">
+        <is>
+          <t>Agent generally owned the case but transferred at a point where further effort was reasonable and expected; or the transfer was made with some context but the handoff documentation was incomplete.</t>
+        </is>
+      </c>
+      <c r="E69" s="137" t="inlineStr">
+        <is>
+          <t>Agent attempted troubleshooting for 5 minutes and transferred to L2 citing complexity — the issue was a basic configuration problem clearly within L1 scope. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="72" customHeight="1">
+      <c r="C70" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D70" s="139" t="inlineStr">
+        <is>
+          <t>Agent transferred immediately or after minimal effort to avoid a difficult issue. Transfer happened without documentation or context for the receiving agent.</t>
+        </is>
+      </c>
+      <c r="E70" s="140" t="inlineStr">
+        <is>
+          <t>Agent saw the case involved a mesh system and immediately routed to L2 without troubleshooting, noting only 'customer has Velop issue' in the ticket. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="72" customHeight="1">
+      <c r="C71" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D71" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Ownership is always expected.</t>
+        </is>
+      </c>
+      <c r="E71" s="143" t="inlineStr"/>
+    </row>
+    <row r="72" ht="72" customHeight="1">
+      <c r="B72" s="131" t="inlineStr">
+        <is>
+          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+        </is>
+      </c>
+      <c r="C72" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D72" s="133" t="inlineStr">
+        <is>
+          <t>Every commitment made during the interaction was executed within the call or documented with a specific owner and timeline. Customer left with a defined, actionable next step.</t>
+        </is>
+      </c>
+      <c r="E72" s="134" t="inlineStr">
+        <is>
+          <t>Agent committed to submitting the escalation before end of day, told the customer what L2 would do and when to expect contact, and updated the ticket accordingly before closing. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="72" customHeight="1">
+      <c r="C73" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D73" s="136" t="inlineStr">
+        <is>
+          <t>Path forward was defined but vague — no specifics on who, when, or what. Or a commitment was made verbally but not documented in the case.</t>
+        </is>
+      </c>
+      <c r="E73" s="137" t="inlineStr">
+        <is>
+          <t>Agent told the customer 'someone will follow up with you' but did not specify the team, timeline, or the nature of the follow-up. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="72" customHeight="1">
+      <c r="C74" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D74" s="139" t="inlineStr">
+        <is>
+          <t>Agent made a commitment that was not kept and not documented. Customer ends the interaction with no defined next step.</t>
+        </is>
+      </c>
+      <c r="E74" s="140" t="inlineStr">
+        <is>
+          <t>Agent promised to call back within 24 hours. No callback was made and no note was left in the ticket. Customer called back the next day. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="72" customHeight="1">
+      <c r="C75" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D75" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. A path forward is always relevant.</t>
+        </is>
+      </c>
+      <c r="E75" s="143" t="inlineStr"/>
+    </row>
+    <row r="76" ht="72" customHeight="1">
+      <c r="B76" s="131" t="inlineStr">
+        <is>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
+        </is>
+      </c>
+      <c r="C76" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D76" s="133" t="inlineStr">
+        <is>
+          <t>Agent told the customer specifically what would happen after the interaction — who would contact them, when, what to do while waiting, and any conditions or contingencies. Timelines given were realistic and achievable.</t>
+        </is>
+      </c>
+      <c r="E76" s="134" t="inlineStr">
+        <is>
+          <t>'Your case is with our Level 2 team. They will reach out within 24–48 business hours at the number on file. Please don't reset the device again in the meantime — that will help them diagnose it when they call.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="72" customHeight="1">
+      <c r="C77" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D77" s="136" t="inlineStr">
+        <is>
+          <t>Some expectation-setting occurred but it was incomplete — timeline provided without a team name, or team named without a timeframe, or the customer's own role in the next step was unclear.</t>
+        </is>
+      </c>
+      <c r="E77" s="137" t="inlineStr">
+        <is>
+          <t>Agent said 'L2 will reach out to you' with no indication of when, how, or what the customer should prepare. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="72" customHeight="1">
+      <c r="C78" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D78" s="139" t="inlineStr">
+        <is>
+          <t>Customer received no information about what happens next. Or was given a timeline that was clearly unrealistic and would not be met.</t>
+        </is>
+      </c>
+      <c r="E78" s="140" t="inlineStr">
+        <is>
+          <t>Agent told the customer they would hear back 'very soon' for an escalation that typically takes 3–5 business days. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="72" customHeight="1">
+      <c r="C79" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D79" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Expectations should always be set.</t>
+        </is>
+      </c>
+      <c r="E79" s="143" t="inlineStr"/>
+    </row>
+    <row r="80" ht="72" customHeight="1">
+      <c r="B80" s="131" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C80" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D80" s="133" t="inlineStr">
+        <is>
+          <t>If the call disconnected, agent made a documented callback attempt within the expected window. If a callback was promised at a specific time, it was made on time — or proactively renegotiated before the window lapsed.</t>
+        </is>
+      </c>
+      <c r="E80" s="134" t="inlineStr">
+        <is>
+          <t>Call dropped mid-troubleshooting. Agent immediately called back, reached the customer, resumed from where they left off, and noted the disconnect and callback in the ticket. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="72" customHeight="1">
+      <c r="C81" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D81" s="136" t="inlineStr">
+        <is>
+          <t>Follow-up was attempted but documentation was incomplete; or callback was made but slightly outside the agreed window without proactive communication to the customer.</t>
+        </is>
+      </c>
+      <c r="E81" s="137" t="inlineStr">
+        <is>
+          <t>Agent called back after a disconnect but did not update the ticket, leaving no record of the follow-up for the next agent. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="72" customHeight="1">
+      <c r="C82" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D82" s="139" t="inlineStr">
+        <is>
+          <t>Call disconnected and no follow-up was made or documented. Callback was promised and not delivered.</t>
+        </is>
+      </c>
+      <c r="E82" s="140" t="inlineStr">
+        <is>
+          <t>Call dropped at a critical point. Agent did not call back. Customer called in the following day and had to start over with a new agent who had no record of the prior session. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="72" customHeight="1">
+      <c r="C83" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D83" s="142" t="inlineStr">
+        <is>
+          <t>No disconnect occurred during the interaction and no callback was committed.</t>
+        </is>
+      </c>
+      <c r="E83" s="143" t="inlineStr"/>
+    </row>
+    <row r="84" ht="72" customHeight="1">
+      <c r="A84" s="130" t="inlineStr">
+        <is>
+          <t>5 · ESCALATION JUDGMENT</t>
+        </is>
+      </c>
+      <c r="B84" s="131" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before escalating</t>
+        </is>
+      </c>
+      <c r="C84" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D84" s="133" t="inlineStr">
+        <is>
+          <t>Agent completed all relevant L1 troubleshooting steps applicable to the issue — sufficient to establish that L2 intervention was genuinely needed. Steps documented before escalating.</t>
+        </is>
+      </c>
+      <c r="E84" s="134" t="inlineStr">
+        <is>
+          <t>Customer's mesh node was stuck on red after multiple reset attempts across two contacts. Agent completed all standard recovery steps, documented results, and escalated with full history. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="72" customHeight="1">
+      <c r="C85" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D85" s="136" t="inlineStr">
+        <is>
+          <t>Some troubleshooting was completed but one or two standard L1 steps were skipped that could have resolved the issue or provided clearer diagnostic data for L2.</t>
+        </is>
+      </c>
+      <c r="E85" s="137" t="inlineStr">
+        <is>
+          <t>Agent ran a factory reset but did not check modem connectivity first. Escalated citing 'hardware failure' — L2 immediately identified the modem as the actual culprit. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="72" customHeight="1">
+      <c r="C86" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D86" s="139" t="inlineStr">
+        <is>
+          <t>Agent escalated immediately or after minimal effort. L2 received a case where basic troubleshooting had not been attempted.</t>
+        </is>
+      </c>
+      <c r="E86" s="140" t="inlineStr">
+        <is>
+          <t>Customer reported no internet. Agent ran one restart, found the issue unresolved, and immediately escalated to L2 with no modem check and no other diagnostic steps. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="72" customHeight="1">
+      <c r="C87" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D87" s="142" t="inlineStr">
+        <is>
+          <t>No escalation occurred during this interaction.</t>
+        </is>
+      </c>
+      <c r="E87" s="143" t="inlineStr"/>
+    </row>
+    <row r="88" ht="72" customHeight="1">
+      <c r="B88" s="131" t="inlineStr">
+        <is>
+          <t>Identified a valid reason to escalate</t>
+        </is>
+      </c>
+      <c r="C88" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D88" s="133" t="inlineStr">
+        <is>
+          <t>Escalation criterion was clearly met — technical complexity beyond L1 scope, confirmed hardware failure, repeat unresolved issue with documented history, customer complaint or legal-risk trigger, or issue requiring L2 tools or authority.</t>
+        </is>
+      </c>
+      <c r="E88" s="134" t="inlineStr">
+        <is>
+          <t>After two contacts and complete L1 troubleshooting, the node consistently failed to re-pair. Agent identified likely hardware defect, documented the repeated failure, and escalated with evidence. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="72" customHeight="1">
+      <c r="C89" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D89" s="136" t="inlineStr">
+        <is>
+          <t>Reason for escalation was present but borderline — issue may have been resolvable at L1 with more effort; or the escalation trigger was identified but not clearly documented.</t>
+        </is>
+      </c>
+      <c r="E89" s="137" t="inlineStr">
+        <is>
+          <t>Agent escalated citing 'customer is frustrated' — a secondary factor, but no technical criterion was articulated and the issue was within L1 scope. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="72" customHeight="1">
+      <c r="C90" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D90" s="139" t="inlineStr">
+        <is>
+          <t>No valid escalation criterion was met. Agent escalated to avoid a difficult call, or escalated a routine issue clearly within L1 scope without any supporting rationale.</t>
+        </is>
+      </c>
+      <c r="E90" s="140" t="inlineStr">
+        <is>
+          <t>Customer asked for an escalation. Agent complied immediately without completing any troubleshooting or documenting a technical reason. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="72" customHeight="1">
+      <c r="C91" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D91" s="142" t="inlineStr">
+        <is>
+          <t>No escalation occurred during this interaction.</t>
+        </is>
+      </c>
+      <c r="E91" s="143" t="inlineStr"/>
+    </row>
+    <row r="92" ht="72" customHeight="1">
+      <c r="B92" s="131" t="inlineStr">
+        <is>
+          <t>Provided complete escalation details using the correct escalation path</t>
+        </is>
+      </c>
+      <c r="C92" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D92" s="133" t="inlineStr">
+        <is>
+          <t>Escalation contained: specific symptom description, all troubleshooting steps and their results, root cause hypothesis, reason for escalation, customer contact details, case history reference, and was submitted to the correct team or queue.</t>
+        </is>
+      </c>
+      <c r="E92" s="134" t="inlineStr">
+        <is>
+          <t>Escalation note: 'Customer reports node stuck on red LED after 3 reset attempts across 2 contacts. Modem confirmed online. Factory reset performed — node pairs briefly then drops. Likely hardware defect. All steps in prior case #12345. Submitted to Tier 2 Hardware.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="72" customHeight="1">
+      <c r="C93" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D93" s="136" t="inlineStr">
+        <is>
+          <t>Escalation submitted to the right team but missing some useful detail — no test results, no case history, no contact info. L2 can action it but may need to re-contact the customer for context.</t>
+        </is>
+      </c>
+      <c r="E93" s="137" t="inlineStr">
+        <is>
+          <t>Escalation note: 'Customer has connectivity issue. Troubleshooting performed. Escalating.' Missing results, steps, and contact. L2 had to call the customer to understand the issue. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="72" customHeight="1">
+      <c r="C94" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D94" s="139" t="inlineStr">
+        <is>
+          <t>Critical information missing — no troubleshooting details, no customer contact, no symptom description. Or escalated to the wrong team or queue entirely.</t>
+        </is>
+      </c>
+      <c r="E94" s="140" t="inlineStr">
+        <is>
+          <t>Escalation note: 'Escalating per customer request.' No technical reason, no troubleshooting summary, no case history. L2 had to start from scratch. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="72" customHeight="1">
+      <c r="C95" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D95" s="142" t="inlineStr">
+        <is>
+          <t>No escalation occurred during this interaction.</t>
+        </is>
+      </c>
+      <c r="E95" s="143" t="inlineStr"/>
+    </row>
+    <row r="96" ht="72" customHeight="1">
+      <c r="B96" s="131" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+        </is>
+      </c>
+      <c r="C96" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D96" s="133" t="inlineStr">
+        <is>
+          <t>Agent explained in plain language why the case needed to go to L2 — what the issue required that L1 couldn't provide — what the escalation process looked like, and what the customer should realistically expect.</t>
+        </is>
+      </c>
+      <c r="E96" s="134" t="inlineStr">
+        <is>
+          <t>'The tests suggest a hardware issue with the node that our Level 2 specialists are better equipped to assess. They'll reach out within 24–48 hours. If confirmed defective, they'll start the replacement process.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="72" customHeight="1">
+      <c r="C97" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D97" s="136" t="inlineStr">
+        <is>
+          <t>Agent told the customer about the escalation but didn't explain why, or gave a vague timeline without specifics about what L2 would actually do.</t>
+        </is>
+      </c>
+      <c r="E97" s="137" t="inlineStr">
+        <is>
+          <t>Agent said 'I'm escalating this to our next level of support — they'll be in touch.' No explanation of why, no L2 action described, no timeline given. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="72" customHeight="1">
+      <c r="C98" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D98" s="139" t="inlineStr">
+        <is>
+          <t>Agent submitted the escalation without telling the customer, or told the customer the case was resolved when it was actually being escalated.</t>
+        </is>
+      </c>
+      <c r="E98" s="140" t="inlineStr">
+        <is>
+          <t>Agent escalated the case, marked the ticket Resolved, and ended the call. Customer was confused when L2 called two days later. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="72" customHeight="1">
+      <c r="C99" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D99" s="142" t="inlineStr">
+        <is>
+          <t>No escalation occurred during this interaction.</t>
+        </is>
+      </c>
+      <c r="E99" s="143" t="inlineStr"/>
+    </row>
+    <row r="100" ht="72" customHeight="1">
+      <c r="A100" s="130" t="inlineStr">
+        <is>
+          <t>6 · CUSTOMER EXPERIENCE</t>
+        </is>
+      </c>
+      <c r="B100" s="131" t="inlineStr">
+        <is>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
+        </is>
+      </c>
+      <c r="C100" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D100" s="133" t="inlineStr">
+        <is>
+          <t>Agent acknowledged the customer's frustration or history in a sincere, specific way. For repeat contacts, explicitly recognized the customer's repeated effort and validated their experience — not a scripted phrase.</t>
+        </is>
+      </c>
+      <c r="E100" s="134" t="inlineStr">
+        <is>
+          <t>'I can see this is your third call about this issue — that must be incredibly frustrating. I want to make sure we get to the bottom of this today. I've reviewed your prior contacts so you won't need to start over.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="72" customHeight="1">
+      <c r="C101" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D101" s="136" t="inlineStr">
+        <is>
+          <t>Empathy was expressed but generic and scripted-sounding, without acknowledging the specific situation or the customer's contact history.</t>
+        </is>
+      </c>
+      <c r="E101" s="137" t="inlineStr">
+        <is>
+          <t>Agent said 'I understand your frustration' and immediately moved to troubleshooting with no further acknowledgment of the customer's experience. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="72" customHeight="1">
+      <c r="C102" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D102" s="139" t="inlineStr">
+        <is>
+          <t>Agent was entirely transactional. No acknowledgment of frustration, no recognition of repeat contact history. Customer felt processed, not heard.</t>
+        </is>
+      </c>
+      <c r="E102" s="140" t="inlineStr">
+        <is>
+          <t>Customer's fourth call about the same unresolved issue. Agent's first statement was 'Can I have your model number?' with no acknowledgment of the history. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="72" customHeight="1">
+      <c r="C103" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D103" s="142" t="inlineStr">
+        <is>
+          <t>Customer expressed no frustration and had no prior contact history requiring acknowledgment.</t>
+        </is>
+      </c>
+      <c r="E103" s="143" t="inlineStr"/>
+    </row>
+    <row r="104" ht="72" customHeight="1">
+      <c r="B104" s="131" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+        </is>
+      </c>
+      <c r="C104" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D104" s="133" t="inlineStr">
+        <is>
+          <t>Agent remained composed, courteous, and helpful throughout — even when the customer was frustrated, demanding, or uncooperative. Did not take provocations personally or let them alter tone.</t>
+        </is>
+      </c>
+      <c r="E104" s="134" t="inlineStr">
+        <is>
+          <t>Customer was rude and demanding across a 45-minute call. Agent remained calm, professional, and solution-focused at every point without becoming defensive. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="72" customHeight="1">
+      <c r="C105" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D105" s="136" t="inlineStr">
+        <is>
+          <t>Agent was mostly professional but had a brief moment of visible impatience or a slightly defensive response — noticeable but not significantly damaging to the interaction.</t>
+        </is>
+      </c>
+      <c r="E105" s="137" t="inlineStr">
+        <is>
+          <t>After a long, difficult call, agent said 'I've been very patient with you today' in a tone that implied criticism. Customer filed a complaint. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="72" customHeight="1">
+      <c r="C106" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D106" s="139" t="inlineStr">
+        <is>
+          <t>Agent became visibly impatient, sarcastic, dismissive, or defensive in a way that materially damaged the interaction or made the customer feel disrespected.</t>
+        </is>
+      </c>
+      <c r="E106" s="140" t="inlineStr">
+        <is>
+          <t>Customer raised their voice. Agent responded: 'I'm just trying to help you, there's no need to be rude.' Customer escalated further. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="72" customHeight="1">
+      <c r="C107" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D107" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Professionalism is always required.</t>
+        </is>
+      </c>
+      <c r="E107" s="143" t="inlineStr"/>
+    </row>
+    <row r="108" ht="72" customHeight="1">
+      <c r="B108" s="131" t="inlineStr">
+        <is>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
+        </is>
+      </c>
+      <c r="C108" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D108" s="133" t="inlineStr">
+        <is>
+          <t>Agent adapted naturally to the customer's communication style — technical and precise with a knowledgeable customer, warm and patient with an anxious first-time user, efficient and direct with an experienced caller who wanted a quick resolution.</t>
+        </is>
+      </c>
+      <c r="E108" s="134" t="inlineStr">
+        <is>
+          <t>Customer identified themselves as a network engineer. Agent shifted to technical terminology, skipped basic explanations, and engaged as a peer. Customer appreciated the efficient, direct exchange. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="72" customHeight="1">
+      <c r="C109" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D109" s="136" t="inlineStr">
+        <is>
+          <t>Agent mostly matched the customer but one dimension was off — too formal with a casual customer, too technical with someone clearly out of their depth, or too slow with an experienced user who wanted speed.</t>
+        </is>
+      </c>
+      <c r="E109" s="137" t="inlineStr">
+        <is>
+          <t>Customer was casual and relaxed. Agent maintained a stiff, formal tone throughout, creating a slight but noticeable disconnect even though the technical help was sound. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="72" customHeight="1">
+      <c r="C110" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D110" s="139" t="inlineStr">
+        <is>
+          <t>Agent maintained a one-size-fits-all tone throughout regardless of the customer's cues. Interaction felt scripted and impersonal.</t>
+        </is>
+      </c>
+      <c r="E110" s="140" t="inlineStr">
+        <is>
+          <t>Elderly customer was nervous and uncertain. Agent delivered fast, jargon-heavy instructions as if speaking to a technical audience. Customer became more confused. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="72" customHeight="1">
+      <c r="C111" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D111" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Tone matching is always relevant.</t>
+        </is>
+      </c>
+      <c r="E111" s="143" t="inlineStr"/>
+    </row>
+    <row r="112" ht="72" customHeight="1">
+      <c r="B112" s="131" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
+        </is>
+      </c>
+      <c r="C112" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D112" s="133" t="inlineStr">
+        <is>
+          <t>Agent proactively reduced what the customer needed to do — did not ask for information already known, handled actions agent-side where possible, confirmed information before asking the customer to perform steps.</t>
+        </is>
+      </c>
+      <c r="E112" s="134" t="inlineStr">
+        <is>
+          <t>Agent had the device model and serial from the account before the call and only asked the customer to confirm the current symptom — saving several minutes and avoiding repetitive questions. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="72" customHeight="1">
+      <c r="C113" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D113" s="136" t="inlineStr">
+        <is>
+          <t>Agent made some effort to reduce customer effort but had areas where the customer was asked to repeat known information or perform steps that could have been handled more efficiently.</t>
+        </is>
+      </c>
+      <c r="E113" s="137" t="inlineStr">
+        <is>
+          <t>Agent asked the customer for the device model that was already visible in the ticket from the prior interaction. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="72" customHeight="1">
+      <c r="C114" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D114" s="139" t="inlineStr">
+        <is>
+          <t>Customer had to repeat information multiple times, was sent through unnecessary steps, or experienced avoidable friction because the agent did not use available information.</t>
+        </is>
+      </c>
+      <c r="E114" s="140" t="inlineStr">
+        <is>
+          <t>Customer on their third contact was asked by the agent to re-explain the issue and repeat all troubleshooting already performed in the prior two contacts. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="72" customHeight="1">
+      <c r="C115" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D115" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E115" s="143" t="inlineStr"/>
+    </row>
+    <row r="116" ht="72" customHeight="1">
+      <c r="B116" s="131" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C116" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D116" s="133" t="inlineStr">
+        <is>
+          <t>Throughout the interaction, the customer remained engaged, understood what was happening and why, and knew what they were supposed to do at each step. Agent verified comprehension and addressed confusion immediately.</t>
+        </is>
+      </c>
+      <c r="E116" s="134" t="inlineStr">
+        <is>
+          <t>Before each step, agent explained what they were looking for and why. After each step, confirmed the result. Customer was an active, informed participant. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="72" customHeight="1">
+      <c r="C117" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D117" s="136" t="inlineStr">
+        <is>
+          <t>Customer was generally engaged but had moments of confusion that were only partially addressed; or the customer's engagement dropped and the agent did not notice or respond.</t>
+        </is>
+      </c>
+      <c r="E117" s="137" t="inlineStr">
+        <is>
+          <t>Customer said 'sorry, I'm a bit lost.' Agent repeated the last instruction without simplifying or reframing. Customer continued but remained uncertain. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="72" customHeight="1">
+      <c r="C118" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D118" s="139" t="inlineStr">
+        <is>
+          <t>Customer was disengaged or lost at multiple points. Agent continued troubleshooting without addressing the comprehension gaps. Customer was sidelined in their own support call.</t>
+        </is>
+      </c>
+      <c r="E118" s="140" t="inlineStr">
+        <is>
+          <t>Agent performed all steps remotely without explaining what was being done. Customer had no idea what was happening and did not feel involved. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="72" customHeight="1">
+      <c r="C119" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D119" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E119" s="143" t="inlineStr"/>
+    </row>
+    <row r="120" ht="72" customHeight="1">
+      <c r="A120" s="130" t="inlineStr">
+        <is>
+          <t>7 · DOCUMENTATION &amp; NOTES</t>
+        </is>
+      </c>
+      <c r="B120" s="131" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
+        </is>
+      </c>
+      <c r="C120" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D120" s="133" t="inlineStr">
+        <is>
+          <t>Case notes clearly describe what the customer reported — specific symptom, affected device(s), scope of impact, when it started, and what the customer had already tried before calling.</t>
+        </is>
+      </c>
+      <c r="E120" s="134" t="inlineStr">
+        <is>
+          <t>'Customer reports wireless drops on all 3 Velop nodes. Issue started 3 days ago after an overnight firmware update. Customer has rebooted all nodes. Wired connection to main node is unaffected.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="72" customHeight="1">
+      <c r="C121" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D121" s="136" t="inlineStr">
+        <is>
+          <t>Issue summary present but vague — 'customer called about connectivity issue' without specific symptom, scope, or prior steps. Next agent cannot tell what was actually wrong.</t>
+        </is>
+      </c>
+      <c r="E121" s="137" t="inlineStr">
+        <is>
+          <t>Case note: 'Customer experiencing internet issues with their router. Troubleshooting performed.' → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="72" customHeight="1">
+      <c r="C122" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D122" s="139" t="inlineStr">
+        <is>
+          <t>No issue summary recorded at all. Next agent has no starting context.</t>
+        </is>
+      </c>
+      <c r="E122" s="140" t="inlineStr">
+        <is>
+          <t>Case closed with only 'Resolved' in the notes — no description of what the customer reported or what was wrong. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="72" customHeight="1">
+      <c r="C123" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D123" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable.</t>
+        </is>
+      </c>
+      <c r="E123" s="143" t="inlineStr"/>
+    </row>
+    <row r="124" ht="72" customHeight="1">
+      <c r="B124" s="131" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
+        </is>
+      </c>
+      <c r="C124" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D124" s="133" t="inlineStr">
+        <is>
+          <t>Notes clearly list troubleshooting steps performed during the interaction in a logical sequence — what was done, in what order, with what result at each step.</t>
+        </is>
+      </c>
+      <c r="E124" s="134" t="inlineStr">
+        <is>
+          <t>'1. Verified modem online — WAN light confirmed on. 2. Checked DHCP lease — IP assigned correctly. 3. Ran wireless diagnostic — signal weak on 2.4 GHz. 4. Changed Wi-Fi channel to channel 6. 5. Customer tested — connectivity restored.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="72" customHeight="1">
+      <c r="C125" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D125" s="136" t="inlineStr">
+        <is>
+          <t>Some steps noted but the list is incomplete — key steps missing, or outcomes of individual steps not recorded.</t>
+        </is>
+      </c>
+      <c r="E125" s="137" t="inlineStr">
+        <is>
+          <t>'Reset router and reconfigured Wi-Fi settings.' No detail on which settings, what the reset revealed, or the outcome of each action. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="72" customHeight="1">
+      <c r="C126" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D126" s="139" t="inlineStr">
+        <is>
+          <t>No troubleshooting steps documented despite a full troubleshooting session. Next agent cannot tell what was tried.</t>
+        </is>
+      </c>
+      <c r="E126" s="140" t="inlineStr">
+        <is>
+          <t>After a 45-minute call: case note reads 'Troubleshooting performed. Escalated.' Nothing else. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="72" customHeight="1">
+      <c r="C127" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D127" s="142" t="inlineStr">
+        <is>
+          <t>No troubleshooting was performed — call was informational only, or customer declined.</t>
+        </is>
+      </c>
+      <c r="E127" s="143" t="inlineStr"/>
+    </row>
+    <row r="128" ht="72" customHeight="1">
+      <c r="B128" s="131" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
+        </is>
+      </c>
+      <c r="C128" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D128" s="133" t="inlineStr">
+        <is>
+          <t>Notes capture what was discovered — test results, error messages observed, device behavior, what worked and what did not. Findings are specific and actionable for the next agent.</t>
+        </is>
+      </c>
+      <c r="E128" s="134" t="inlineStr">
+        <is>
+          <t>'Admin panel shows firmware version 3.8.1 — latest is 4.1.2. Firmware update failed twice. Event log shows error code E404: firmware download timeout. Likely firmware corruption or server-side download issue.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="72" customHeight="1">
+      <c r="C129" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D129" s="136" t="inlineStr">
+        <is>
+          <t>Some findings noted but key observations are missing — outcome of a test not recorded, error message observed but not documented, inconsistency noticed but not noted.</t>
+        </is>
+      </c>
+      <c r="E129" s="137" t="inlineStr">
+        <is>
+          <t>Notes mention a factory reset was performed but don't record what happened afterward or whether the issue persisted. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="72" customHeight="1">
+      <c r="C130" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D130" s="139" t="inlineStr">
+        <is>
+          <t>No findings documented at all. Next agent cannot tell what was learned from the interaction.</t>
+        </is>
+      </c>
+      <c r="E130" s="140" t="inlineStr">
+        <is>
+          <t>Notes record only actions. No results, no observations, no test outcomes. Next agent has to start from scratch. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="72" customHeight="1">
+      <c r="C131" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D131" s="142" t="inlineStr">
+        <is>
+          <t>No diagnostic findings to record — quick informational inquiry with no testing involved.</t>
+        </is>
+      </c>
+      <c r="E131" s="143" t="inlineStr"/>
+    </row>
+    <row r="132" ht="72" customHeight="1">
+      <c r="B132" s="131" t="inlineStr">
+        <is>
+          <t>Captured agent reasoning — escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action</t>
+        </is>
+      </c>
+      <c r="C132" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D132" s="133" t="inlineStr">
+        <is>
+          <t>Notes explain key decisions — why a specific troubleshooting path was chosen, why the case was escalated (what criterion was met), and any colleague or SME consultations that shaped the approach. If no private notes are available, colleague input is captured in the case notes.</t>
+        </is>
+      </c>
+      <c r="E132" s="134" t="inlineStr">
+        <is>
+          <t>'Consulted with Team Lead before escalating. TL confirmed this meets the hardware defect threshold after three failed factory resets. Escalated to Tier 2 Hardware with full history. TL input documented here as no private note was available.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="72" customHeight="1">
+      <c r="C133" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D133" s="136" t="inlineStr">
+        <is>
+          <t>Some reasoning captured but key decisions lack explanation — escalation submitted with no documented rationale, or colleague input followed but not attributed in any note.</t>
+        </is>
+      </c>
+      <c r="E133" s="137" t="inlineStr">
+        <is>
+          <t>Agent escalated and noted 'escalated per policy' but did not document which criterion was met, what troubleshooting led to that conclusion, or who they consulted. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="72" customHeight="1">
+      <c r="C134" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D134" s="139" t="inlineStr">
+        <is>
+          <t>Notes contain only actions — what was done — with no explanation of why. Next agent or QA reviewer cannot understand the decision-making.</t>
+        </is>
+      </c>
+      <c r="E134" s="140" t="inlineStr">
+        <is>
+          <t>Agent escalated the case. Escalation note: 'Escalating to L2.' No reason, no troubleshooting summary, no colleague reference. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="72" customHeight="1">
+      <c r="C135" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D135" s="142" t="inlineStr">
+        <is>
+          <t>Straightforward interaction with no escalation, no colleague consultation, and no ambiguous decisions requiring explanation.</t>
+        </is>
+      </c>
+      <c r="E135" s="143" t="inlineStr"/>
+    </row>
+    <row r="136" ht="72" customHeight="1">
+      <c r="B136" s="131" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
+        </is>
+      </c>
+      <c r="C136" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D136" s="133" t="inlineStr">
+        <is>
+          <t>Notes specify what happens after the interaction — who is responsible for the next action, what that action is, and any relevant timeline or conditions. Callback details fully recorded where applicable.</t>
+        </is>
+      </c>
+      <c r="E136" s="134" t="inlineStr">
+        <is>
+          <t>'Escalated to L2 Hardware (ticket #67890). Customer to be contacted within 24–48 hours at 555-0100. Customer advised not to factory reset again until L2 makes contact.' → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="72" customHeight="1">
+      <c r="C137" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D137" s="136" t="inlineStr">
+        <is>
+          <t>Next steps mentioned in general terms but lacking specifics — no owner, no timeline, no conditions.</t>
+        </is>
+      </c>
+      <c r="E137" s="137" t="inlineStr">
+        <is>
+          <t>'Escalated. Customer to wait for follow-up.' No team named, no timeframe, no detail on what the follow-up entails. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="72" customHeight="1">
+      <c r="C138" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D138" s="139" t="inlineStr">
+        <is>
+          <t>No next steps documented. Case cannot be picked up by another agent without re-contacting the customer.</t>
+        </is>
+      </c>
+      <c r="E138" s="140" t="inlineStr">
+        <is>
+          <t>Case closed after escalation with no note on what was submitted, which team received it, or when the customer should expect contact. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="72" customHeight="1">
+      <c r="C139" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D139" s="142" t="inlineStr">
+        <is>
+          <t>Issue fully resolved with no pending actions required.</t>
+        </is>
+      </c>
+      <c r="E139" s="143" t="inlineStr"/>
+    </row>
+    <row r="140" ht="72" customHeight="1">
+      <c r="B140" s="131" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C140" s="132" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="D140" s="133" t="inlineStr">
+        <is>
+          <t>Ticket status accurately reflects the true state of the case at close — Resolved only when the issue was confirmed resolved, Escalated when escalated, Callback when a return call is pending. Closure reason documented.</t>
+        </is>
+      </c>
+      <c r="E140" s="134" t="inlineStr">
+        <is>
+          <t>Issue was unresolved at close. Agent marked the ticket 'Escalated,' noted the receiving team and escalation ticket number, and documented the current issue state before closing. → Met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="72" customHeight="1">
+      <c r="C141" s="135" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D141" s="136" t="inlineStr">
+        <is>
+          <t>Status is mostly accurate but the closure reason is missing or too brief; or the correct status was used but applied late.</t>
+        </is>
+      </c>
+      <c r="E141" s="137" t="inlineStr">
+        <is>
+          <t>Ticket was marked 'Resolved' with a closure note that said only 'fixed' — no description of what was done, confirmed, or by whom. → Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="72" customHeight="1">
+      <c r="C142" s="138" t="inlineStr">
+        <is>
+          <t>Missed</t>
+        </is>
+      </c>
+      <c r="D142" s="139" t="inlineStr">
+        <is>
+          <t>Ticket marked Resolved when the issue was not resolved. Or marked Closed without a closure reason. Or left in a status that would mislead the next agent.</t>
+        </is>
+      </c>
+      <c r="E142" s="140" t="inlineStr">
+        <is>
+          <t>Agent submitted an escalation but marked the ticket 'Resolved' because the call ended. L2 received the case with a Resolved status and deprioritized it. → Missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="72" customHeight="1">
+      <c r="C143" s="141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D143" s="142" t="inlineStr">
+        <is>
+          <t>Not applicable. Ticket status must always reflect reality.</t>
+        </is>
+      </c>
+      <c r="E143" s="143" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="44">
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B140:B143"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="B96:B99"/>
+    <mergeCell ref="B72:B75"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A40:A67"/>
+    <mergeCell ref="B120:B123"/>
+    <mergeCell ref="B52:B55"/>
+    <mergeCell ref="B136:B139"/>
+    <mergeCell ref="A4:A19"/>
+    <mergeCell ref="A120:A143"/>
+    <mergeCell ref="B132:B135"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="B88:B91"/>
+    <mergeCell ref="A20:A39"/>
+    <mergeCell ref="A100:A119"/>
+    <mergeCell ref="B116:B119"/>
+    <mergeCell ref="A68:A83"/>
+    <mergeCell ref="B48:B51"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="B44:B47"/>
+    <mergeCell ref="B84:B87"/>
+    <mergeCell ref="B60:B63"/>
+    <mergeCell ref="B40:B43"/>
+    <mergeCell ref="B128:B131"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B112:B115"/>
+    <mergeCell ref="B92:B95"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="B124:B127"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B80:B83"/>
+    <mergeCell ref="B36:B39"/>
+    <mergeCell ref="A84:A99"/>
+    <mergeCell ref="B108:B111"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B64:B67"/>
+    <mergeCell ref="B104:B107"/>
+    <mergeCell ref="B100:B103"/>
+    <mergeCell ref="B76:B79"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="B32:B35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Agent Level field to Case Information with Team Score Weight indicator
New row 5 in Case Information: dropdown for Level 1 / Level 2, plus a
Team Score Weight formula (1.0x for L1, 1.5x for L2) that surfaces the
weight a team aggregation system should apply to this evaluation.
All formulas, DVs, merges, and conditional formatting shifted +1 to
accommodate the new row.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="42">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -263,6 +263,11 @@
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="27">
@@ -724,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="205">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1209,6 +1214,94 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="23" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3605,7 +3698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" style="136" min="1" max="1"/>
@@ -3666,202 +3759,209 @@
       <c r="F4" s="84" t="n"/>
     </row>
     <row r="5" ht="29" customHeight="1" s="136">
-      <c r="B5" s="100" t="inlineStr">
+      <c r="B5" s="175" t="inlineStr">
+        <is>
+          <t>Agent Level</t>
+        </is>
+      </c>
+      <c r="C5" s="176" t="n"/>
+      <c r="D5" s="177" t="inlineStr">
+        <is>
+          <t>Team Score Weight</t>
+        </is>
+      </c>
+      <c r="E5" s="178">
+        <f>IF(C5="Level 2","1.5×  —  senior support (L2 weight applies to team aggregations)",IF(C5="Level 1","1.0×  —  standard support (L1 weight applies to team aggregations)",""))</f>
+        <v/>
+      </c>
+      <c r="F5" s="84" t="n"/>
+    </row>
+    <row r="6" ht="29" customHeight="1" s="136">
+      <c r="B6" s="144" t="inlineStr">
         <is>
           <t>Evaluator (QA)</t>
         </is>
       </c>
-      <c r="C5" s="95" t="n"/>
-      <c r="D5" s="98" t="inlineStr">
+      <c r="C6" s="179" t="n"/>
+      <c r="D6" s="167" t="inlineStr">
         <is>
           <t>Interaction Date</t>
         </is>
       </c>
-      <c r="E5" s="142" t="n"/>
-      <c r="F5" s="84" t="n"/>
-    </row>
-    <row r="6" ht="29" customHeight="1" s="136">
-      <c r="B6" s="100" t="inlineStr">
+      <c r="E6" s="179" t="n"/>
+      <c r="F6" s="84" t="n"/>
+    </row>
+    <row r="7" ht="29" customHeight="1" s="136">
+      <c r="B7" s="144" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C6" s="95" t="n"/>
-      <c r="D6" s="98" t="inlineStr">
+      <c r="C7" s="179" t="n"/>
+      <c r="D7" s="167" t="inlineStr">
         <is>
           <t>Channel</t>
         </is>
       </c>
-      <c r="E6" s="142" t="n"/>
-      <c r="F6" s="84" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="100" t="inlineStr">
+      <c r="E7" s="179" t="n"/>
+      <c r="F7" s="84" t="n"/>
+    </row>
+    <row r="8" ht="29" customHeight="1" s="136">
+      <c r="B8" s="144" t="inlineStr">
         <is>
           <t>Warranty Status</t>
         </is>
       </c>
-      <c r="C7" s="95" t="n"/>
-      <c r="D7" s="98" t="inlineStr">
+      <c r="C8" s="179" t="n"/>
+      <c r="D8" s="167" t="inlineStr">
         <is>
           <t>Review Date</t>
         </is>
       </c>
-      <c r="E7" s="142" t="n"/>
-      <c r="F7" s="84" t="n"/>
-    </row>
-    <row r="8" ht="29" customHeight="1" s="136">
-      <c r="B8" s="100" t="inlineStr">
+      <c r="E8" s="179" t="n"/>
+      <c r="F8" s="84" t="n"/>
+    </row>
+    <row r="9" ht="29" customHeight="1" s="136">
+      <c r="B9" s="144" t="inlineStr">
         <is>
           <t>Case Type</t>
         </is>
       </c>
-      <c r="C8" s="95" t="n"/>
-      <c r="D8" s="98" t="inlineStr">
+      <c r="C9" s="179" t="n"/>
+      <c r="D9" s="167" t="inlineStr">
         <is>
           <t>Interaction Duration</t>
         </is>
       </c>
-      <c r="E8" s="142" t="n"/>
-      <c r="F8" s="84" t="n"/>
-    </row>
-    <row r="9" ht="29" customHeight="1" s="136">
-      <c r="B9" s="100" t="inlineStr">
+      <c r="E9" s="179" t="n"/>
+      <c r="F9" s="84" t="n"/>
+    </row>
+    <row r="10" ht="29" customHeight="1" s="136">
+      <c r="B10" s="144" t="inlineStr">
         <is>
           <t>Touch # (multi-touch case)</t>
         </is>
       </c>
-      <c r="C9" s="95" t="n"/>
-      <c r="D9" s="98" t="inlineStr">
+      <c r="C10" s="179" t="n"/>
+      <c r="D10" s="167" t="inlineStr">
         <is>
           <t>Prior touches reviewed?</t>
         </is>
       </c>
-      <c r="E9" s="142" t="n"/>
-      <c r="F9" s="84" t="n"/>
-    </row>
-    <row r="10" ht="29" customHeight="1" s="136">
-      <c r="B10" s="100" t="inlineStr">
+      <c r="E10" s="179" t="n"/>
+      <c r="F10" s="84" t="n"/>
+    </row>
+    <row r="11" ht="29" customHeight="1" s="136">
+      <c r="B11" s="144" t="inlineStr">
         <is>
           <t>CSAT / Survey result</t>
         </is>
       </c>
-      <c r="C10" s="95" t="n"/>
-      <c r="D10" s="98" t="inlineStr">
+      <c r="C11" s="179" t="n"/>
+      <c r="D11" s="167" t="inlineStr">
         <is>
           <t>FCR / total contacts</t>
         </is>
       </c>
-      <c r="E10" s="142" t="n"/>
-      <c r="F10" s="84" t="n"/>
-    </row>
-    <row r="11" ht="29" customHeight="1" s="136">
-      <c r="B11" s="100" t="inlineStr">
+      <c r="E11" s="179" t="n"/>
+      <c r="F11" s="84" t="n"/>
+    </row>
+    <row r="12" ht="29" customHeight="1" s="136">
+      <c r="B12" s="144" t="inlineStr">
         <is>
           <t>Total case time</t>
         </is>
       </c>
-      <c r="C11" s="95" t="n"/>
-      <c r="D11" s="98" t="inlineStr">
+      <c r="C12" s="179" t="n"/>
+      <c r="D12" s="167" t="inlineStr">
         <is>
           <t>SLA status</t>
         </is>
       </c>
-      <c r="E11" s="142" t="n"/>
-      <c r="F11" s="84" t="n"/>
-    </row>
-    <row r="12" ht="58" customHeight="1" s="136">
-      <c r="B12" s="98" t="inlineStr">
+      <c r="E12" s="179" t="n"/>
+      <c r="F12" s="84" t="n"/>
+    </row>
+    <row r="13" ht="58" customHeight="1" s="136">
+      <c r="B13" s="167" t="inlineStr">
         <is>
           <t>Case Summary (customer issue &amp; goal)</t>
         </is>
       </c>
-      <c r="C12" s="143" t="n"/>
-      <c r="D12" s="83" t="n"/>
-      <c r="E12" s="83" t="n"/>
-      <c r="F12" s="84" t="n"/>
-    </row>
-    <row r="13" ht="46" customHeight="1" s="136">
-      <c r="B13" s="98" t="inlineStr">
-        <is>
-          <t>Inherited context (what this agent received from prior touches)</t>
-        </is>
-      </c>
-      <c r="C13" s="143" t="n"/>
+      <c r="C13" s="180" t="n"/>
       <c r="D13" s="83" t="n"/>
       <c r="E13" s="83" t="n"/>
       <c r="F13" s="84" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1" s="136">
-      <c r="B14" s="88" t="inlineStr">
+      <c r="B14" s="167" t="inlineStr">
+        <is>
+          <t>Inherited context (what this agent received from prior touches)</t>
+        </is>
+      </c>
+      <c r="C14" s="180" t="n"/>
+      <c r="D14" s="83" t="n"/>
+      <c r="E14" s="83" t="n"/>
+      <c r="F14" s="84" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1" s="136">
+      <c r="B15" s="88" t="inlineStr">
         <is>
           <t>CLASSIFICATION &amp; ROOT-CAUSE   (added from the 360 Form model)</t>
         </is>
       </c>
-      <c r="C14" s="86" t="n"/>
-      <c r="D14" s="86" t="n"/>
-      <c r="E14" s="86" t="n"/>
-      <c r="F14" s="87" t="n"/>
-    </row>
-    <row r="15" ht="58" customHeight="1" s="136">
-      <c r="B15" s="100" t="inlineStr">
+      <c r="C15" s="86" t="n"/>
+      <c r="D15" s="86" t="n"/>
+      <c r="E15" s="86" t="n"/>
+      <c r="F15" s="87" t="n"/>
+    </row>
+    <row r="16" ht="58" customHeight="1" s="136">
+      <c r="B16" s="144" t="inlineStr">
         <is>
           <t>Audit / Review Type</t>
         </is>
       </c>
-      <c r="C15" s="95" t="n"/>
-      <c r="D15" s="98" t="inlineStr">
+      <c r="C16" s="179" t="n"/>
+      <c r="D16" s="167" t="inlineStr">
         <is>
           <t>Contact iteration (repeat contact)</t>
         </is>
       </c>
-      <c r="E15" s="142" t="n"/>
-      <c r="F15" s="84" t="n"/>
-    </row>
-    <row r="16" ht="29" customHeight="1" s="136">
-      <c r="B16" s="100" t="inlineStr">
+      <c r="E16" s="179" t="n"/>
+      <c r="F16" s="84" t="n"/>
+    </row>
+    <row r="17" ht="29" customHeight="1" s="136">
+      <c r="B17" s="144" t="inlineStr">
         <is>
           <t>Resolution status — detailed</t>
         </is>
       </c>
-      <c r="C16" s="95" t="n"/>
-      <c r="D16" s="98" t="inlineStr">
+      <c r="C17" s="179" t="n"/>
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Primary root-cause domain</t>
         </is>
       </c>
-      <c r="E16" s="142" t="n"/>
-      <c r="F16" s="84" t="n"/>
-    </row>
-    <row r="17" ht="29" customHeight="1" s="136">
-      <c r="B17" s="100" t="inlineStr">
+      <c r="E17" s="179" t="n"/>
+      <c r="F17" s="84" t="n"/>
+    </row>
+    <row r="18" ht="29" customHeight="1" s="136">
+      <c r="B18" s="144" t="inlineStr">
         <is>
           <t>Process driver (if any)</t>
         </is>
       </c>
-      <c r="C17" s="142" t="n"/>
-      <c r="D17" s="83" t="n"/>
-      <c r="E17" s="83" t="n"/>
-      <c r="F17" s="84" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="100" t="inlineStr">
-        <is>
-          <t>Product driver (if any)</t>
-        </is>
-      </c>
-      <c r="C18" s="142" t="n"/>
+      <c r="C18" s="179" t="n"/>
       <c r="D18" s="83" t="n"/>
       <c r="E18" s="83" t="n"/>
       <c r="F18" s="84" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="100" t="inlineStr">
-        <is>
-          <t>System / tooling driver (if any)</t>
-        </is>
-      </c>
-      <c r="C19" s="142" t="n"/>
+      <c r="B19" s="144" t="inlineStr">
+        <is>
+          <t>Product driver (if any)</t>
+        </is>
+      </c>
+      <c r="C19" s="179" t="n"/>
       <c r="D19" s="83" t="n"/>
       <c r="E19" s="83" t="n"/>
       <c r="F19" s="84" t="n"/>
@@ -3869,1593 +3969,1586 @@
     <row r="20">
       <c r="B20" s="144" t="inlineStr">
         <is>
-          <t>Root-cause / contact-driver notes   (feeds Team Scoring → Team Opportunities Identified)</t>
-        </is>
-      </c>
-      <c r="C20" s="83" t="n"/>
+          <t>System / tooling driver (if any)</t>
+        </is>
+      </c>
+      <c r="C20" s="179" t="n"/>
       <c r="D20" s="83" t="n"/>
       <c r="E20" s="83" t="n"/>
       <c r="F20" s="84" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="104" t="inlineStr">
+      <c r="B21" s="144" t="inlineStr">
+        <is>
+          <t>Root-cause / contact-driver notes   (feeds Team Scoring → Team Opportunities Identified)</t>
+        </is>
+      </c>
+      <c r="C21" s="83" t="n"/>
+      <c r="D21" s="83" t="n"/>
+      <c r="E21" s="83" t="n"/>
+      <c r="F21" s="84" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="136">
+      <c r="B22" s="181" t="inlineStr">
         <is>
           <t>2 · SCORE SUMMARY</t>
         </is>
       </c>
-      <c r="C21" s="86" t="n"/>
-      <c r="D21" s="86" t="n"/>
-      <c r="E21" s="86" t="n"/>
-      <c r="F21" s="87" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" s="136">
-      <c r="B22" s="133" t="inlineStr">
+      <c r="C22" s="86" t="n"/>
+      <c r="D22" s="86" t="n"/>
+      <c r="E22" s="86" t="n"/>
+      <c r="F22" s="87" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="136">
+      <c r="B23" s="133" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C22" s="133" t="inlineStr">
+      <c r="C23" s="133" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="D22" s="133" t="inlineStr">
+      <c r="D23" s="133" t="inlineStr">
         <is>
           <t>Score (0-5)</t>
         </is>
       </c>
-      <c r="E22" s="133" t="inlineStr">
+      <c r="E23" s="133" t="inlineStr">
         <is>
           <t>Weighted</t>
         </is>
       </c>
-      <c r="F22" s="133" t="inlineStr">
+      <c r="F23" s="133" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="28" customHeight="1" s="136">
-      <c r="B23" s="16" t="inlineStr">
+    <row r="24" ht="28" customHeight="1" s="136">
+      <c r="B24" s="182" t="inlineStr">
         <is>
           <t>Resolution / Progress Toward Resolution</t>
         </is>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C24" s="183" t="n">
         <v>0.3</v>
       </c>
-      <c r="D23" s="18">
-        <f>IF(C41="",C40,C41)</f>
-        <v/>
-      </c>
-      <c r="E23" s="19">
-        <f>IF(D23="","",(D23/5)*C23)</f>
-        <v/>
-      </c>
-      <c r="F23" s="20">
-        <f>IF(D23="","",IF(D23&gt;=4,"Strong",IF(D23=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="21" t="inlineStr">
+      <c r="D24" s="184">
+        <f>IF(C42="",C41,C42)</f>
+        <v/>
+      </c>
+      <c r="E24" s="185">
+        <f>IF(D24="","",(D24/5)*C24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="186">
+        <f>IF(D24="","",IF(D24&gt;=4,"Strong",IF(D24=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1" s="136">
+      <c r="B25" s="187" t="inlineStr">
         <is>
           <t>Technical Accuracy</t>
         </is>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C25" s="188" t="n">
         <v>0.2</v>
       </c>
-      <c r="D24" s="23">
-        <f>IF(C53="",C52,C53)</f>
-        <v/>
-      </c>
-      <c r="E24" s="24">
-        <f>IF(D24="","",(D24/5)*C24)</f>
-        <v/>
-      </c>
-      <c r="F24" s="25">
-        <f>IF(D24="","",IF(D24&gt;=4,"Strong",IF(D24=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="28" customHeight="1" s="136">
-      <c r="B25" s="16" t="inlineStr">
+      <c r="D25" s="189">
+        <f>IF(C54="",C53,C54)</f>
+        <v/>
+      </c>
+      <c r="E25" s="190">
+        <f>IF(D25="","",(D25/5)*C25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="191">
+        <f>IF(D25="","",IF(D25&gt;=4,"Strong",IF(D25=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1" s="136">
+      <c r="B26" s="182" t="inlineStr">
         <is>
           <t>Communication &amp; Call Control</t>
         </is>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C26" s="183" t="n">
         <v>0.15</v>
       </c>
-      <c r="D25" s="18">
-        <f>IF(C67="",C66,C67)</f>
-        <v/>
-      </c>
-      <c r="E25" s="19">
-        <f>IF(D25="","",(D25/5)*C25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="20">
-        <f>IF(D25="","",IF(D25&gt;=4,"Strong",IF(D25=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1" s="136">
-      <c r="B26" s="21" t="inlineStr">
+      <c r="D26" s="184">
+        <f>IF(C68="",C67,C68)</f>
+        <v/>
+      </c>
+      <c r="E26" s="185">
+        <f>IF(D26="","",(D26/5)*C26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="186">
+        <f>IF(D26="","",IF(D26&gt;=4,"Strong",IF(D26=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1" s="136">
+      <c r="B27" s="187" t="inlineStr">
         <is>
           <t>Customer Ownership</t>
         </is>
       </c>
-      <c r="C26" s="22" t="n">
+      <c r="C27" s="188" t="n">
         <v>0.15</v>
       </c>
-      <c r="D26" s="23">
-        <f>IF(C79="",C78,C79)</f>
-        <v/>
-      </c>
-      <c r="E26" s="24">
-        <f>IF(D26="","",(D26/5)*C26)</f>
-        <v/>
-      </c>
-      <c r="F26" s="25">
-        <f>IF(D26="","",IF(D26&gt;=4,"Strong",IF(D26=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="28" customHeight="1" s="136">
-      <c r="B27" s="16" t="inlineStr">
+      <c r="D27" s="189">
+        <f>IF(C80="",C79,C80)</f>
+        <v/>
+      </c>
+      <c r="E27" s="190">
+        <f>IF(D27="","",(D27/5)*C27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="191">
+        <f>IF(D27="","",IF(D27&gt;=4,"Strong",IF(D27=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1" s="136">
+      <c r="B28" s="182" t="inlineStr">
         <is>
           <t>Escalation Judgment</t>
         </is>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C28" s="183" t="n">
         <v>0.1</v>
       </c>
-      <c r="D27" s="18">
-        <f>IF(C90="",C89,C90)</f>
-        <v/>
-      </c>
-      <c r="E27" s="19">
-        <f>IF(D27="","",(D27/5)*C27)</f>
-        <v/>
-      </c>
-      <c r="F27" s="20">
-        <f>IF(D27="","",IF(D27&gt;=4,"Strong",IF(D27=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="28" customHeight="1" s="136">
-      <c r="B28" s="21" t="inlineStr">
+      <c r="D28" s="184">
+        <f>IF(C91="",C90,C91)</f>
+        <v/>
+      </c>
+      <c r="E28" s="185">
+        <f>IF(D28="","",(D28/5)*C28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="186">
+        <f>IF(D28="","",IF(D28&gt;=4,"Strong",IF(D28=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1" s="136">
+      <c r="B29" s="187" t="inlineStr">
         <is>
           <t>Customer Experience</t>
         </is>
       </c>
-      <c r="C28" s="22" t="n">
+      <c r="C29" s="188" t="n">
         <v>0.05</v>
       </c>
-      <c r="D28" s="23">
-        <f>IF(C109="",C108,C109)</f>
-        <v/>
-      </c>
-      <c r="E28" s="24">
-        <f>IF(D28="","",(D28/5)*C28)</f>
-        <v/>
-      </c>
-      <c r="F28" s="25">
-        <f>IF(D28="","",IF(D28&gt;=4,"Strong",IF(D28=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="28" customHeight="1" s="136">
-      <c r="B29" s="16" t="inlineStr">
+      <c r="D29" s="189">
+        <f>IF(C110="",C109,C110)</f>
+        <v/>
+      </c>
+      <c r="E29" s="190">
+        <f>IF(D29="","",(D29/5)*C29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="191">
+        <f>IF(D29="","",IF(D29&gt;=4,"Strong",IF(D29=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1" s="136">
+      <c r="B30" s="182" t="inlineStr">
         <is>
           <t>Documentation &amp; Notes</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C30" s="183" t="n">
         <v>0.05</v>
       </c>
-      <c r="D29" s="18">
-        <f>IF(C122="",C121,C122)</f>
-        <v/>
-      </c>
-      <c r="E29" s="19">
-        <f>IF(D29="","",(D29/5)*C29)</f>
-        <v/>
-      </c>
-      <c r="F29" s="20">
-        <f>IF(D29="","",IF(D29&gt;=4,"Strong",IF(D29=3,"Developing","Needs Focus")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1" s="136">
-      <c r="B30" s="104" t="inlineStr">
+      <c r="D30" s="184">
+        <f>IF(C123="",C122,C123)</f>
+        <v/>
+      </c>
+      <c r="E30" s="185">
+        <f>IF(D30="","",(D30/5)*C30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="186">
+        <f>IF(D30="","",IF(D30&gt;=4,"Strong",IF(D30=3,"Developing","Needs Focus")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1" s="136">
+      <c r="B31" s="181" t="inlineStr">
         <is>
           <t>WEIGHTED TOTAL SCORE</t>
         </is>
       </c>
-      <c r="C30" s="26">
-        <f>SUM(C23:C29)</f>
-        <v/>
-      </c>
-      <c r="D30" s="27" t="n"/>
-      <c r="E30" s="28">
-        <f>IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0),0,SUM(E23:E29))</f>
-        <v/>
-      </c>
-      <c r="F30" s="29">
-        <f>IF(E30="","",IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E30&gt;=0.85,"MEETS / EXCEEDS",IF(E30&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="24" customHeight="1" s="136">
-      <c r="B31" s="104" t="inlineStr">
+      <c r="C31" s="192">
+        <f>SUM(C24:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="193" t="n"/>
+      <c r="E31" s="194">
+        <f>IF(OR(C149="No",C150="No",C151="No",COUNTIF(C153:C163,"Yes")&gt;0),0,SUM(E24:E30))</f>
+        <v/>
+      </c>
+      <c r="F31" s="195">
+        <f>IF(E31="","",IF(OR(C149="No",C150="No",C151="No",COUNTIF(C153:C163,"Yes")&gt;0),"AUTO-ZERO (0%)",IF(E31&gt;=0.85,"MEETS / EXCEEDS",IF(E31&gt;=0.7,"DEVELOPING","NEEDS IMPROVEMENT"))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" s="136">
+      <c r="B32" s="181" t="inlineStr">
         <is>
           <t>3 · CATEGORY ASSESSMENTS</t>
-        </is>
-      </c>
-      <c r="C31" s="86" t="n"/>
-      <c r="D31" s="86" t="n"/>
-      <c r="E31" s="86" t="n"/>
-      <c r="F31" s="87" t="n"/>
-    </row>
-    <row r="32" ht="18" customHeight="1" s="136">
-      <c r="B32" s="88" t="inlineStr">
-        <is>
-          <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
         </is>
       </c>
       <c r="C32" s="86" t="n"/>
       <c r="D32" s="86" t="n"/>
-      <c r="E32" s="87" t="n"/>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="E32" s="86" t="n"/>
+      <c r="F32" s="87" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="136">
+      <c r="B33" s="88" t="inlineStr">
+        <is>
+          <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
+        </is>
+      </c>
+      <c r="C33" s="86" t="n"/>
+      <c r="D33" s="86" t="n"/>
+      <c r="E33" s="87" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Weight: 30%</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1" s="136">
-      <c r="B33" s="145" t="inlineStr">
+    <row r="34" ht="28" customHeight="1" s="136">
+      <c r="B34" s="145" t="inlineStr">
         <is>
           <t>Objective: Determine whether the interaction moved the customer meaningfully closer to resolution.</t>
         </is>
       </c>
-      <c r="C33" s="83" t="n"/>
-      <c r="D33" s="83" t="n"/>
-      <c r="E33" s="83" t="n"/>
-      <c r="F33" s="84" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1" s="136">
-      <c r="B34" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D34" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C34" s="83" t="n"/>
+      <c r="D34" s="83" t="n"/>
       <c r="E34" s="83" t="n"/>
       <c r="F34" s="84" t="n"/>
     </row>
-    <row r="35" ht="28" customHeight="1" s="136">
-      <c r="B35" s="82" t="inlineStr">
-        <is>
-          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
-        </is>
-      </c>
-      <c r="C35" s="102" t="n"/>
-      <c r="D35" s="146" t="n"/>
+    <row r="35" ht="18" customHeight="1" s="136">
+      <c r="B35" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C35" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D35" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E35" s="83" t="n"/>
       <c r="F35" s="84" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1" s="136">
-      <c r="B36" s="94" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
-        </is>
-      </c>
-      <c r="C36" s="102" t="n"/>
-      <c r="D36" s="147" t="n"/>
+      <c r="B36" s="146" t="inlineStr">
+        <is>
+          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
+        </is>
+      </c>
+      <c r="C36" s="197" t="n"/>
+      <c r="D36" s="146" t="n"/>
       <c r="E36" s="83" t="n"/>
       <c r="F36" s="84" t="n"/>
     </row>
     <row r="37" ht="28" customHeight="1" s="136">
-      <c r="B37" s="82" t="inlineStr">
-        <is>
-          <t>Resolution path was appropriate for the situation and warranty status</t>
-        </is>
-      </c>
-      <c r="C37" s="102" t="n"/>
-      <c r="D37" s="146" t="n"/>
+      <c r="B37" s="198" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
+        </is>
+      </c>
+      <c r="C37" s="197" t="n"/>
+      <c r="D37" s="198" t="n"/>
       <c r="E37" s="83" t="n"/>
       <c r="F37" s="84" t="n"/>
     </row>
     <row r="38" ht="28" customHeight="1" s="136">
-      <c r="B38" s="94" t="inlineStr">
-        <is>
-          <t>Customer was moved meaningfully closer to a solution</t>
-        </is>
-      </c>
-      <c r="C38" s="102" t="n"/>
-      <c r="D38" s="147" t="n"/>
+      <c r="B38" s="146" t="inlineStr">
+        <is>
+          <t>Resolution path was appropriate for the situation and warranty status</t>
+        </is>
+      </c>
+      <c r="C38" s="197" t="n"/>
+      <c r="D38" s="146" t="n"/>
       <c r="E38" s="83" t="n"/>
       <c r="F38" s="84" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1" s="136">
-      <c r="B39" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Does NOT count: customer simply ends call; generic KB sent without troubleshooting; warranty used as reason to stop helping; escalation as shortcut; unsupported ISP blame; 'monitor &amp; call back' with no plan; ownership transferred without expectations or documentation.</t>
-        </is>
-      </c>
-      <c r="C39" s="83" t="n"/>
-      <c r="D39" s="83" t="n"/>
+      <c r="B39" s="198" t="inlineStr">
+        <is>
+          <t>Customer was moved meaningfully closer to a solution</t>
+        </is>
+      </c>
+      <c r="C39" s="197" t="n"/>
+      <c r="D39" s="198" t="n"/>
       <c r="E39" s="83" t="n"/>
       <c r="F39" s="84" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1" s="136">
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C40" s="68">
-        <f>IF((COUNTIF(C35:C38,"Met")+COUNTIF(C35:C38,"Partial")+COUNTIF(C35:C38,"Missed"))=0,"",ROUND((COUNTIF(C35:C38,"Met")*5+COUNTIF(C35:C38,"Partial")*2.5)/(COUNTIF(C35:C38,"Met")+COUNTIF(C35:C38,"Partial")+COUNTIF(C35:C38,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D40" s="149" t="n"/>
+      <c r="B40" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Does NOT count: customer simply ends call; generic KB sent without troubleshooting; warranty used as reason to stop helping; escalation as shortcut; unsupported ISP blame; 'monitor &amp; call back' with no plan; ownership transferred without expectations or documentation.</t>
+        </is>
+      </c>
+      <c r="C40" s="83" t="n"/>
+      <c r="D40" s="83" t="n"/>
       <c r="E40" s="83" t="n"/>
       <c r="F40" s="84" t="n"/>
     </row>
-    <row r="41" ht="24" customHeight="1" s="136">
-      <c r="B41" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C41" s="14" t="n"/>
-      <c r="D41" s="150">
-        <f>IF(IF(C41="",C40,C41)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C41="",C40,C41)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="41" ht="28" customHeight="1" s="136">
+      <c r="B41" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C41" s="200">
+        <f>IF((COUNTIF(C36:C39,"Met")+COUNTIF(C36:C39,"Partial")+COUNTIF(C36:C39,"Missed"))=0,"",ROUND((COUNTIF(C36:C39,"Met")*5+COUNTIF(C36:C39,"Partial")*2.5)/(COUNTIF(C36:C39,"Met")+COUNTIF(C36:C39,"Partial")+COUNTIF(C36:C39,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D41" s="149" t="n"/>
       <c r="E41" s="83" t="n"/>
       <c r="F41" s="84" t="n"/>
     </row>
-    <row r="42" ht="36" customHeight="1" s="136">
-      <c r="B42" s="106" t="inlineStr">
-        <is>
-          <t>Score reflects the cumulative effect of this touch within the 8-month journey: the Nov 24, 2025 hardware/RMA determination remains undelivered, and the case culminates here in executive-level escalation with no path forward offered.</t>
-        </is>
-      </c>
-      <c r="C42" s="143" t="n"/>
-      <c r="D42" s="83" t="n"/>
+    <row r="42" ht="24" customHeight="1" s="136">
+      <c r="B42" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C42" s="201" t="n"/>
+      <c r="D42" s="150">
+        <f>IF(IF(C42="",C41,C42)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C42="",C41,C42)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E42" s="83" t="n"/>
       <c r="F42" s="84" t="n"/>
     </row>
-    <row r="43" ht="18" customHeight="1" s="136">
-      <c r="B43" s="88" t="inlineStr">
+    <row r="43" ht="36" customHeight="1" s="136">
+      <c r="B43" s="151" t="inlineStr">
+        <is>
+          <t>Score reflects the cumulative effect of this touch within the 8-month journey: the Nov 24, 2025 hardware/RMA determination remains undelivered, and the case culminates here in executive-level escalation with no path forward offered.</t>
+        </is>
+      </c>
+      <c r="C43" s="180" t="n"/>
+      <c r="D43" s="83" t="n"/>
+      <c r="E43" s="83" t="n"/>
+      <c r="F43" s="84" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="136">
+      <c r="B44" s="88" t="inlineStr">
         <is>
           <t>2. TECHNICAL ACCURACY</t>
         </is>
       </c>
-      <c r="C43" s="86" t="n"/>
-      <c r="D43" s="86" t="n"/>
-      <c r="E43" s="87" t="n"/>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="C44" s="86" t="n"/>
+      <c r="D44" s="86" t="n"/>
+      <c r="E44" s="87" t="n"/>
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Weight: 20%</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1" s="136">
-      <c r="B44" s="145" t="inlineStr">
+    <row r="45" ht="28" customHeight="1" s="136">
+      <c r="B45" s="145" t="inlineStr">
         <is>
           <t>Objective: Evaluate the quality of troubleshooting and technical guidance.</t>
         </is>
       </c>
-      <c r="C44" s="83" t="n"/>
-      <c r="D44" s="83" t="n"/>
-      <c r="E44" s="83" t="n"/>
-      <c r="F44" s="84" t="n"/>
-    </row>
-    <row r="45" ht="36" customHeight="1" s="136">
-      <c r="B45" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D45" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C45" s="83" t="n"/>
+      <c r="D45" s="83" t="n"/>
       <c r="E45" s="83" t="n"/>
       <c r="F45" s="84" t="n"/>
     </row>
-    <row r="46" ht="28" customHeight="1" s="136">
-      <c r="B46" s="82" t="inlineStr">
-        <is>
-          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
-        </is>
-      </c>
-      <c r="C46" s="102" t="n"/>
-      <c r="D46" s="146" t="n"/>
+    <row r="46" ht="36" customHeight="1" s="136">
+      <c r="B46" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C46" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D46" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E46" s="83" t="n"/>
       <c r="F46" s="84" t="n"/>
     </row>
     <row r="47" ht="28" customHeight="1" s="136">
-      <c r="B47" s="94" t="inlineStr">
-        <is>
-          <t>Identified the root cause (or likely cause) when possible</t>
-        </is>
-      </c>
-      <c r="C47" s="102" t="n"/>
-      <c r="D47" s="147" t="n"/>
+      <c r="B47" s="146" t="inlineStr">
+        <is>
+          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
+        </is>
+      </c>
+      <c r="C47" s="197" t="n"/>
+      <c r="D47" s="146" t="n"/>
       <c r="E47" s="83" t="n"/>
       <c r="F47" s="84" t="n"/>
     </row>
     <row r="48" ht="28" customHeight="1" s="136">
-      <c r="B48" s="82" t="inlineStr">
-        <is>
-          <t>Followed a logical troubleshooting process</t>
-        </is>
-      </c>
-      <c r="C48" s="102" t="n"/>
-      <c r="D48" s="146" t="n"/>
+      <c r="B48" s="198" t="inlineStr">
+        <is>
+          <t>Identified the root cause (or likely cause) when possible</t>
+        </is>
+      </c>
+      <c r="C48" s="197" t="n"/>
+      <c r="D48" s="198" t="n"/>
       <c r="E48" s="83" t="n"/>
       <c r="F48" s="84" t="n"/>
     </row>
     <row r="49" ht="28" customHeight="1" s="136">
-      <c r="B49" s="82" t="inlineStr">
+      <c r="B49" s="146" t="inlineStr">
+        <is>
+          <t>Followed a logical troubleshooting process</t>
+        </is>
+      </c>
+      <c r="C49" s="197" t="n"/>
+      <c r="D49" s="146" t="n"/>
+      <c r="E49" s="83" t="n"/>
+      <c r="F49" s="84" t="n"/>
+    </row>
+    <row r="50" ht="28" customHeight="1" s="136">
+      <c r="B50" s="146" t="inlineStr">
         <is>
           <t>Available tools were used efficiently and appropriately</t>
         </is>
       </c>
-      <c r="C49" s="102" t="n"/>
-      <c r="D49" s="82" t="n"/>
-    </row>
-    <row r="50" ht="28" customHeight="1" s="136">
-      <c r="B50" s="82" t="inlineStr">
+      <c r="C50" s="197" t="n"/>
+      <c r="D50" s="146" t="n"/>
+    </row>
+    <row r="51" ht="28" customHeight="1" s="136">
+      <c r="B51" s="146" t="inlineStr">
         <is>
           <t>Gave technically accurate information; no unsupported conclusions</t>
         </is>
       </c>
-      <c r="C50" s="102" t="n"/>
-      <c r="D50" s="146" t="n"/>
-      <c r="E50" s="83" t="n"/>
-      <c r="F50" s="84" t="n"/>
-    </row>
-    <row r="51" ht="28" customHeight="1" s="136">
-      <c r="B51" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
-        </is>
-      </c>
-      <c r="C51" s="83" t="n"/>
-      <c r="D51" s="83" t="n"/>
+      <c r="C51" s="197" t="n"/>
+      <c r="D51" s="146" t="n"/>
       <c r="E51" s="83" t="n"/>
       <c r="F51" s="84" t="n"/>
     </row>
     <row r="52" ht="28" customHeight="1" s="136">
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C52" s="68">
-        <f>IF((COUNTIF(C46:C50,"Met")+COUNTIF(C46:C50,"Partial")+COUNTIF(C46:C50,"Missed"))=0,"",ROUND((COUNTIF(C46:C50,"Met")*5+COUNTIF(C46:C50,"Partial")*2.5)/(COUNTIF(C46:C50,"Met")+COUNTIF(C46:C50,"Partial")+COUNTIF(C46:C50,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D52" s="149" t="n"/>
+      <c r="B52" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Deduct for: incorrect technical information; skipped critical troubleshooting; misdiagnosis; unnecessary actions recommended; ISP or customer blamed without evidence; repeating basic steps the customer already completed.</t>
+        </is>
+      </c>
+      <c r="C52" s="83" t="n"/>
+      <c r="D52" s="83" t="n"/>
       <c r="E52" s="83" t="n"/>
       <c r="F52" s="84" t="n"/>
     </row>
-    <row r="53" ht="24" customHeight="1" s="136">
-      <c r="B53" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C53" s="14" t="n"/>
-      <c r="D53" s="150">
-        <f>IF(IF(C53="",C52,C53)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C53="",C52,C53)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="53" ht="28" customHeight="1" s="136">
+      <c r="B53" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C53" s="200">
+        <f>IF((COUNTIF(C47:C51,"Met")+COUNTIF(C47:C51,"Partial")+COUNTIF(C47:C51,"Missed"))=0,"",ROUND((COUNTIF(C47:C51,"Met")*5+COUNTIF(C47:C51,"Partial")*2.5)/(COUNTIF(C47:C51,"Met")+COUNTIF(C47:C51,"Partial")+COUNTIF(C47:C51,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D53" s="149" t="n"/>
       <c r="E53" s="83" t="n"/>
       <c r="F53" s="84" t="n"/>
     </row>
-    <row r="54" ht="36" customHeight="1" s="136">
-      <c r="B54" s="106" t="inlineStr">
-        <is>
-          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
-        </is>
-      </c>
-      <c r="C54" s="143" t="n"/>
-      <c r="D54" s="83" t="n"/>
+    <row r="54" ht="24" customHeight="1" s="136">
+      <c r="B54" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C54" s="201" t="n"/>
+      <c r="D54" s="150">
+        <f>IF(IF(C54="",C53,C54)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C54="",C53,C54)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E54" s="83" t="n"/>
       <c r="F54" s="84" t="n"/>
     </row>
-    <row r="55" ht="18" customHeight="1" s="136">
-      <c r="B55" s="88" t="inlineStr">
+    <row r="55" ht="36" customHeight="1" s="136">
+      <c r="B55" s="151" t="inlineStr">
+        <is>
+          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
+        </is>
+      </c>
+      <c r="C55" s="180" t="n"/>
+      <c r="D55" s="83" t="n"/>
+      <c r="E55" s="83" t="n"/>
+      <c r="F55" s="84" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1" s="136">
+      <c r="B56" s="88" t="inlineStr">
         <is>
           <t>3. COMMUNICATION &amp; CALL CONTROL</t>
         </is>
       </c>
-      <c r="C55" s="86" t="n"/>
-      <c r="D55" s="86" t="n"/>
-      <c r="E55" s="87" t="n"/>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="C56" s="86" t="n"/>
+      <c r="D56" s="86" t="n"/>
+      <c r="E56" s="87" t="n"/>
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Weight: 15%</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="28" customHeight="1" s="136">
-      <c r="B56" s="145" t="inlineStr">
+    <row r="57" ht="28" customHeight="1" s="136">
+      <c r="B57" s="145" t="inlineStr">
         <is>
           <t>Objective: Evaluate how effectively the agent managed the interaction.</t>
         </is>
       </c>
-      <c r="C56" s="83" t="n"/>
-      <c r="D56" s="83" t="n"/>
-      <c r="E56" s="83" t="n"/>
-      <c r="F56" s="84" t="n"/>
-    </row>
-    <row r="57" ht="24" customHeight="1" s="136">
-      <c r="B57" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D57" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C57" s="83" t="n"/>
+      <c r="D57" s="83" t="n"/>
       <c r="E57" s="83" t="n"/>
       <c r="F57" s="84" t="n"/>
     </row>
-    <row r="58" ht="28" customHeight="1" s="136">
-      <c r="B58" s="82" t="inlineStr">
-        <is>
-          <t>Expectations were set clearly from the start</t>
-        </is>
-      </c>
-      <c r="C58" s="102" t="n"/>
-      <c r="D58" s="146" t="n"/>
+    <row r="58" ht="24" customHeight="1" s="136">
+      <c r="B58" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C58" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D58" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E58" s="83" t="n"/>
       <c r="F58" s="84" t="n"/>
     </row>
     <row r="59" ht="28" customHeight="1" s="136">
-      <c r="B59" s="94" t="inlineStr">
-        <is>
-          <t>Agent maintained call control and troubleshooting flow</t>
-        </is>
-      </c>
-      <c r="C59" s="102" t="n"/>
-      <c r="D59" s="147" t="n"/>
+      <c r="B59" s="146" t="inlineStr">
+        <is>
+          <t>Expectations were set clearly from the start</t>
+        </is>
+      </c>
+      <c r="C59" s="197" t="n"/>
+      <c r="D59" s="146" t="n"/>
       <c r="E59" s="83" t="n"/>
       <c r="F59" s="84" t="n"/>
     </row>
     <row r="60" ht="28" customHeight="1" s="136">
-      <c r="B60" s="82" t="inlineStr">
-        <is>
-          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
-        </is>
-      </c>
-      <c r="C60" s="102" t="n"/>
-      <c r="D60" s="146" t="n"/>
+      <c r="B60" s="198" t="inlineStr">
+        <is>
+          <t>Agent maintained call control and troubleshooting flow</t>
+        </is>
+      </c>
+      <c r="C60" s="197" t="n"/>
+      <c r="D60" s="198" t="n"/>
       <c r="E60" s="83" t="n"/>
       <c r="F60" s="84" t="n"/>
     </row>
     <row r="61" ht="28" customHeight="1" s="136">
-      <c r="B61" s="94" t="inlineStr">
-        <is>
-          <t>Actively listened and showed comprehension throughout the interaction/s</t>
-        </is>
-      </c>
-      <c r="C61" s="102" t="n"/>
-      <c r="D61" s="147" t="n"/>
+      <c r="B61" s="146" t="inlineStr">
+        <is>
+          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+        </is>
+      </c>
+      <c r="C61" s="197" t="n"/>
+      <c r="D61" s="146" t="n"/>
       <c r="E61" s="83" t="n"/>
       <c r="F61" s="84" t="n"/>
     </row>
     <row r="62" ht="28" customHeight="1" s="136">
-      <c r="B62" s="94" t="inlineStr">
-        <is>
-          <t>Managed time well, with clear transitions between steps</t>
-        </is>
-      </c>
-      <c r="C62" s="102" t="n"/>
-      <c r="D62" s="147" t="n"/>
+      <c r="B62" s="198" t="inlineStr">
+        <is>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
+        </is>
+      </c>
+      <c r="C62" s="197" t="n"/>
+      <c r="D62" s="198" t="n"/>
       <c r="E62" s="83" t="n"/>
       <c r="F62" s="84" t="n"/>
     </row>
     <row r="63" ht="28" customHeight="1" s="136">
-      <c r="B63" s="82" t="inlineStr">
-        <is>
-          <t>Handled difficult moments when needed to maintain call control</t>
-        </is>
-      </c>
-      <c r="C63" s="102" t="n"/>
-      <c r="D63" s="146" t="n"/>
+      <c r="B63" s="198" t="inlineStr">
+        <is>
+          <t>Managed time well, with clear transitions between steps</t>
+        </is>
+      </c>
+      <c r="C63" s="197" t="n"/>
+      <c r="D63" s="198" t="n"/>
       <c r="E63" s="83" t="n"/>
       <c r="F63" s="84" t="n"/>
     </row>
     <row r="64" ht="28" customHeight="1" s="136">
-      <c r="B64" s="94" t="inlineStr">
-        <is>
-          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
-        </is>
-      </c>
-      <c r="C64" s="102" t="n"/>
-      <c r="D64" s="147" t="n"/>
+      <c r="B64" s="146" t="inlineStr">
+        <is>
+          <t>Handled difficult moments when needed to maintain call control</t>
+        </is>
+      </c>
+      <c r="C64" s="197" t="n"/>
+      <c r="D64" s="146" t="n"/>
       <c r="E64" s="83" t="n"/>
       <c r="F64" s="84" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1" s="136">
-      <c r="B65" s="148" t="inlineStr">
-        <is>
-          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
-        </is>
-      </c>
-      <c r="C65" s="83" t="n"/>
-      <c r="D65" s="83" t="n"/>
+      <c r="B65" s="198" t="inlineStr">
+        <is>
+          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+        </is>
+      </c>
+      <c r="C65" s="197" t="n"/>
+      <c r="D65" s="198" t="n"/>
       <c r="E65" s="83" t="n"/>
       <c r="F65" s="84" t="n"/>
     </row>
     <row r="66" ht="28" customHeight="1" s="136">
-      <c r="B66" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C66" s="68">
-        <f>IF((COUNTIF(C58:C64,"Met")+COUNTIF(C58:C64,"Partial")+COUNTIF(C58:C64,"Missed"))=0,"",ROUND((COUNTIF(C58:C64,"Met")*5+COUNTIF(C58:C64,"Partial")*2.5)/(COUNTIF(C58:C64,"Met")+COUNTIF(C58:C64,"Partial")+COUNTIF(C58:C64,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D66" s="149" t="n"/>
+      <c r="B66" s="148" t="inlineStr">
+        <is>
+          <t>⚠ High performance: customer always knows what is happening and the agent drives the call confidently. One instruction at a time for customers who need it.</t>
+        </is>
+      </c>
+      <c r="C66" s="83" t="n"/>
+      <c r="D66" s="83" t="n"/>
       <c r="E66" s="83" t="n"/>
       <c r="F66" s="84" t="n"/>
     </row>
-    <row r="67" ht="24" customHeight="1" s="136">
-      <c r="B67" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C67" s="14" t="n"/>
-      <c r="D67" s="150">
-        <f>IF(IF(C67="",C66,C67)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C67="",C66,C67)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="67" ht="28" customHeight="1" s="136">
+      <c r="B67" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C67" s="200">
+        <f>IF((COUNTIF(C59:C65,"Met")+COUNTIF(C59:C65,"Partial")+COUNTIF(C59:C65,"Missed"))=0,"",ROUND((COUNTIF(C59:C65,"Met")*5+COUNTIF(C59:C65,"Partial")*2.5)/(COUNTIF(C59:C65,"Met")+COUNTIF(C59:C65,"Partial")+COUNTIF(C59:C65,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D67" s="149" t="n"/>
       <c r="E67" s="83" t="n"/>
       <c r="F67" s="84" t="n"/>
     </row>
-    <row r="68" ht="36" customHeight="1" s="136">
-      <c r="B68" s="106" t="inlineStr">
-        <is>
-          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
-        </is>
-      </c>
-      <c r="C68" s="143" t="n"/>
-      <c r="D68" s="83" t="n"/>
+    <row r="68" ht="24" customHeight="1" s="136">
+      <c r="B68" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C68" s="201" t="n"/>
+      <c r="D68" s="150">
+        <f>IF(IF(C68="",C67,C68)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C68="",C67,C68)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E68" s="83" t="n"/>
       <c r="F68" s="84" t="n"/>
     </row>
-    <row r="69" ht="18" customHeight="1" s="136">
-      <c r="B69" s="88" t="inlineStr">
+    <row r="69" ht="36" customHeight="1" s="136">
+      <c r="B69" s="151" t="inlineStr">
+        <is>
+          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
+        </is>
+      </c>
+      <c r="C69" s="180" t="n"/>
+      <c r="D69" s="83" t="n"/>
+      <c r="E69" s="83" t="n"/>
+      <c r="F69" s="84" t="n"/>
+    </row>
+    <row r="70" ht="18" customHeight="1" s="136">
+      <c r="B70" s="88" t="inlineStr">
         <is>
           <t>4. CUSTOMER OWNERSHIP</t>
         </is>
       </c>
-      <c r="C69" s="86" t="n"/>
-      <c r="D69" s="86" t="n"/>
-      <c r="E69" s="87" t="n"/>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="C70" s="86" t="n"/>
+      <c r="D70" s="86" t="n"/>
+      <c r="E70" s="87" t="n"/>
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>Weight: 15%</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="28" customHeight="1" s="136">
-      <c r="B70" s="145" t="inlineStr">
+    <row r="71" ht="28" customHeight="1" s="136">
+      <c r="B71" s="145" t="inlineStr">
         <is>
           <t>Objective: Measure the degree to which the agent accepted responsibility for moving the customer forward.</t>
         </is>
       </c>
-      <c r="C70" s="83" t="n"/>
-      <c r="D70" s="83" t="n"/>
-      <c r="E70" s="83" t="n"/>
-      <c r="F70" s="84" t="n"/>
-    </row>
-    <row r="71" ht="24" customHeight="1" s="136">
-      <c r="B71" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D71" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C71" s="83" t="n"/>
+      <c r="D71" s="83" t="n"/>
       <c r="E71" s="83" t="n"/>
       <c r="F71" s="84" t="n"/>
     </row>
-    <row r="72" ht="28" customHeight="1" s="136">
-      <c r="B72" s="82" t="inlineStr">
-        <is>
-          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
-        </is>
-      </c>
-      <c r="C72" s="102" t="n"/>
-      <c r="D72" s="146" t="n"/>
+    <row r="72" ht="24" customHeight="1" s="136">
+      <c r="B72" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C72" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D72" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E72" s="83" t="n"/>
       <c r="F72" s="84" t="n"/>
     </row>
     <row r="73" ht="28" customHeight="1" s="136">
-      <c r="B73" s="82" t="inlineStr">
-        <is>
-          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
-        </is>
-      </c>
-      <c r="C73" s="102" t="n"/>
+      <c r="B73" s="146" t="inlineStr">
+        <is>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
+        </is>
+      </c>
+      <c r="C73" s="197" t="n"/>
       <c r="D73" s="146" t="n"/>
       <c r="E73" s="83" t="n"/>
       <c r="F73" s="84" t="n"/>
     </row>
     <row r="74" ht="28" customHeight="1" s="136">
-      <c r="B74" s="82" t="n"/>
-      <c r="C74" s="102" t="n"/>
+      <c r="B74" s="146" t="inlineStr">
+        <is>
+          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+        </is>
+      </c>
+      <c r="C74" s="197" t="n"/>
       <c r="D74" s="146" t="n"/>
       <c r="E74" s="83" t="n"/>
       <c r="F74" s="84" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1" s="136">
-      <c r="B75" s="94" t="inlineStr">
-        <is>
-          <t>Clearly set customer expectations for next steps and realistic timelines</t>
-        </is>
-      </c>
-      <c r="C75" s="102" t="n"/>
-      <c r="D75" s="147" t="n"/>
+      <c r="B75" s="146" t="n"/>
+      <c r="C75" s="197" t="n"/>
+      <c r="D75" s="146" t="n"/>
       <c r="E75" s="83" t="n"/>
       <c r="F75" s="84" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1" s="136">
-      <c r="B76" s="82" t="inlineStr">
-        <is>
-          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
-        </is>
-      </c>
-      <c r="C76" s="102" t="n"/>
-      <c r="D76" s="146" t="n"/>
+      <c r="B76" s="198" t="inlineStr">
+        <is>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
+        </is>
+      </c>
+      <c r="C76" s="197" t="n"/>
+      <c r="D76" s="198" t="n"/>
       <c r="E76" s="83" t="n"/>
       <c r="F76" s="84" t="n"/>
     </row>
     <row r="77" ht="28" customHeight="1" s="136">
-      <c r="B77" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
-        </is>
-      </c>
-      <c r="C77" s="83" t="n"/>
-      <c r="D77" s="83" t="n"/>
+      <c r="B77" s="146" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C77" s="197" t="n"/>
+      <c r="D77" s="146" t="n"/>
       <c r="E77" s="83" t="n"/>
       <c r="F77" s="84" t="n"/>
     </row>
     <row r="78" ht="28" customHeight="1" s="136">
-      <c r="B78" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C78" s="68">
-        <f>IF((COUNTIF(C72:C76,"Met")+COUNTIF(C72:C76,"Partial")+COUNTIF(C72:C76,"Missed"))=0,"",ROUND((COUNTIF(C72:C76,"Met")*5+COUNTIF(C72:C76,"Partial")*2.5)/(COUNTIF(C72:C76,"Met")+COUNTIF(C72:C76,"Partial")+COUNTIF(C72:C76,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D78" s="149" t="n"/>
+      <c r="B78" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
+        </is>
+      </c>
+      <c r="C78" s="83" t="n"/>
+      <c r="D78" s="83" t="n"/>
       <c r="E78" s="83" t="n"/>
       <c r="F78" s="84" t="n"/>
     </row>
-    <row r="79" ht="24" customHeight="1" s="136">
-      <c r="B79" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C79" s="14" t="n"/>
-      <c r="D79" s="150">
-        <f>IF(IF(C79="",C78,C79)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C79="",C78,C79)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="79" ht="28" customHeight="1" s="136">
+      <c r="B79" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C79" s="200">
+        <f>IF((COUNTIF(C73:C77,"Met")+COUNTIF(C73:C77,"Partial")+COUNTIF(C73:C77,"Missed"))=0,"",ROUND((COUNTIF(C73:C77,"Met")*5+COUNTIF(C73:C77,"Partial")*2.5)/(COUNTIF(C73:C77,"Met")+COUNTIF(C73:C77,"Partial")+COUNTIF(C73:C77,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D79" s="149" t="n"/>
       <c r="E79" s="83" t="n"/>
       <c r="F79" s="84" t="n"/>
     </row>
-    <row r="80" ht="36" customHeight="1" s="136">
-      <c r="B80" s="106" t="inlineStr">
-        <is>
-          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
-        </is>
-      </c>
-      <c r="C80" s="143" t="n"/>
-      <c r="D80" s="83" t="n"/>
+    <row r="80" ht="24" customHeight="1" s="136">
+      <c r="B80" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C80" s="201" t="n"/>
+      <c r="D80" s="150">
+        <f>IF(IF(C80="",C79,C80)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C80="",C79,C80)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E80" s="83" t="n"/>
       <c r="F80" s="84" t="n"/>
     </row>
-    <row r="81" ht="18" customHeight="1" s="136">
-      <c r="B81" s="88" t="inlineStr">
+    <row r="81" ht="36" customHeight="1" s="136">
+      <c r="B81" s="151" t="inlineStr">
+        <is>
+          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
+        </is>
+      </c>
+      <c r="C81" s="180" t="n"/>
+      <c r="D81" s="83" t="n"/>
+      <c r="E81" s="83" t="n"/>
+      <c r="F81" s="84" t="n"/>
+    </row>
+    <row r="82" ht="18" customHeight="1" s="136">
+      <c r="B82" s="88" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
       </c>
-      <c r="C81" s="86" t="n"/>
-      <c r="D81" s="86" t="n"/>
-      <c r="E81" s="87" t="n"/>
-      <c r="F81" s="6" t="inlineStr">
+      <c r="C82" s="86" t="n"/>
+      <c r="D82" s="86" t="n"/>
+      <c r="E82" s="87" t="n"/>
+      <c r="F82" s="6" t="inlineStr">
         <is>
           <t>Weight: 10%</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="28" customHeight="1" s="136">
-      <c r="B82" s="145" t="inlineStr">
+    <row r="83" ht="28" customHeight="1" s="136">
+      <c r="B83" s="145" t="inlineStr">
         <is>
           <t>Objective: Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted.</t>
         </is>
       </c>
-      <c r="C82" s="83" t="n"/>
-      <c r="D82" s="83" t="n"/>
-      <c r="E82" s="83" t="n"/>
-      <c r="F82" s="84" t="n"/>
-    </row>
-    <row r="83" ht="18" customHeight="1" s="136">
-      <c r="B83" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C83" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D83" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C83" s="83" t="n"/>
+      <c r="D83" s="83" t="n"/>
       <c r="E83" s="83" t="n"/>
       <c r="F83" s="84" t="n"/>
     </row>
-    <row r="84" ht="28" customHeight="1" s="136">
-      <c r="B84" s="82" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before escalating</t>
-        </is>
-      </c>
-      <c r="C84" s="102" t="n"/>
-      <c r="D84" s="146" t="n"/>
+    <row r="84" ht="18" customHeight="1" s="136">
+      <c r="B84" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C84" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D84" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E84" s="83" t="n"/>
       <c r="F84" s="84" t="n"/>
     </row>
     <row r="85" ht="28" customHeight="1" s="136">
-      <c r="B85" s="94" t="inlineStr">
-        <is>
-          <t>Identified a valid reason to escalate</t>
-        </is>
-      </c>
-      <c r="C85" s="102" t="n"/>
-      <c r="D85" s="147" t="n"/>
+      <c r="B85" s="146" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before escalating</t>
+        </is>
+      </c>
+      <c r="C85" s="197" t="n"/>
+      <c r="D85" s="146" t="n"/>
       <c r="E85" s="83" t="n"/>
       <c r="F85" s="84" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1" s="136">
-      <c r="B86" s="82" t="inlineStr">
-        <is>
-          <t>Provided complete escalation details using the correct escalation path</t>
-        </is>
-      </c>
-      <c r="C86" s="102" t="n"/>
-      <c r="D86" s="146" t="n"/>
+      <c r="B86" s="198" t="inlineStr">
+        <is>
+          <t>Identified a valid reason to escalate</t>
+        </is>
+      </c>
+      <c r="C86" s="197" t="n"/>
+      <c r="D86" s="198" t="n"/>
       <c r="E86" s="83" t="n"/>
       <c r="F86" s="84" t="n"/>
     </row>
     <row r="87" ht="28" customHeight="1" s="136">
-      <c r="B87" s="82" t="inlineStr">
-        <is>
-          <t>Clearly explained why escalation was necessary and what would happen next.</t>
-        </is>
-      </c>
-      <c r="C87" s="102" t="n"/>
+      <c r="B87" s="146" t="inlineStr">
+        <is>
+          <t>Provided complete escalation details using the correct escalation path</t>
+        </is>
+      </c>
+      <c r="C87" s="197" t="n"/>
       <c r="D87" s="146" t="n"/>
       <c r="E87" s="83" t="n"/>
       <c r="F87" s="84" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1" s="136">
-      <c r="B88" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
-        </is>
-      </c>
-      <c r="C88" s="83" t="n"/>
-      <c r="D88" s="83" t="n"/>
+      <c r="B88" s="146" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+        </is>
+      </c>
+      <c r="C88" s="197" t="n"/>
+      <c r="D88" s="146" t="n"/>
       <c r="E88" s="83" t="n"/>
       <c r="F88" s="84" t="n"/>
     </row>
     <row r="89" ht="28" customHeight="1" s="136">
-      <c r="B89" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C89" s="68">
-        <f>IF((COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed"))=0,"",ROUND((COUNTIF(C84:C87,"Met")*5+COUNTIF(C84:C87,"Partial")*2.5)/(COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D89" s="149" t="n"/>
+      <c r="B89" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
+        </is>
+      </c>
+      <c r="C89" s="83" t="n"/>
+      <c r="D89" s="83" t="n"/>
       <c r="E89" s="83" t="n"/>
       <c r="F89" s="84" t="n"/>
     </row>
-    <row r="90" ht="24" customHeight="1" s="136">
-      <c r="B90" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C90" s="14" t="n"/>
-      <c r="D90" s="150">
-        <f>IF(IF(C90="",C89,C90)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C90="",C89,C90)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="90" ht="28" customHeight="1" s="136">
+      <c r="B90" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C90" s="200">
+        <f>IF((COUNTIF(C85:C88,"Met")+COUNTIF(C85:C88,"Partial")+COUNTIF(C85:C88,"Missed"))=0,"",ROUND((COUNTIF(C85:C88,"Met")*5+COUNTIF(C85:C88,"Partial")*2.5)/(COUNTIF(C85:C88,"Met")+COUNTIF(C85:C88,"Partial")+COUNTIF(C85:C88,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D90" s="149" t="n"/>
       <c r="E90" s="83" t="n"/>
       <c r="F90" s="84" t="n"/>
     </row>
-    <row r="91" ht="36" customHeight="1" s="136">
-      <c r="B91" s="106" t="inlineStr">
-        <is>
-          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
-        </is>
-      </c>
-      <c r="C91" s="143" t="n"/>
-      <c r="D91" s="83" t="n"/>
+    <row r="91" ht="24" customHeight="1" s="136">
+      <c r="B91" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C91" s="201" t="n"/>
+      <c r="D91" s="150">
+        <f>IF(IF(C91="",C90,C91)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C91="",C90,C91)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E91" s="83" t="n"/>
       <c r="F91" s="84" t="n"/>
     </row>
-    <row r="92" ht="20" customHeight="1" s="136">
-      <c r="B92" s="88" t="inlineStr">
+    <row r="92" ht="36" customHeight="1" s="136">
+      <c r="B92" s="151" t="inlineStr">
+        <is>
+          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
+        </is>
+      </c>
+      <c r="C92" s="180" t="n"/>
+      <c r="D92" s="83" t="n"/>
+      <c r="E92" s="83" t="n"/>
+      <c r="F92" s="84" t="n"/>
+    </row>
+    <row r="93" ht="20" customHeight="1" s="136">
+      <c r="B93" s="88" t="inlineStr">
         <is>
           <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
         </is>
       </c>
-      <c r="C92" s="86" t="n"/>
-      <c r="D92" s="86" t="n"/>
-      <c r="E92" s="86" t="n"/>
-      <c r="F92" s="87" t="n"/>
-    </row>
-    <row r="93" ht="20" customHeight="1" s="136">
-      <c r="B93" s="151" t="inlineStr">
+      <c r="C93" s="86" t="n"/>
+      <c r="D93" s="86" t="n"/>
+      <c r="E93" s="86" t="n"/>
+      <c r="F93" s="87" t="n"/>
+    </row>
+    <row r="94" ht="20" customHeight="1" s="136">
+      <c r="B94" s="151" t="inlineStr">
         <is>
           <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
         </is>
       </c>
-      <c r="C93" s="107" t="n"/>
-      <c r="D93" s="89" t="n"/>
-      <c r="F93" s="6" t="n"/>
-    </row>
-    <row r="94" ht="45" customHeight="1" s="136">
-      <c r="B94" s="108" t="n"/>
-      <c r="C94" s="109" t="n"/>
-      <c r="D94" s="93" t="n"/>
-    </row>
-    <row r="95" ht="18" customHeight="1" s="136">
-      <c r="B95" s="88" t="inlineStr">
+      <c r="C94" s="107" t="n"/>
+      <c r="D94" s="149" t="n"/>
+      <c r="F94" s="6" t="n"/>
+    </row>
+    <row r="95" ht="45" customHeight="1" s="136">
+      <c r="B95" s="108" t="n"/>
+      <c r="C95" s="109" t="n"/>
+      <c r="D95" s="150" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1" s="136">
+      <c r="B96" s="88" t="inlineStr">
         <is>
           <t>L1 learning points from this escalation outcome</t>
         </is>
       </c>
-      <c r="C95" s="86" t="n"/>
-      <c r="D95" s="86" t="n"/>
-      <c r="E95" s="86" t="n"/>
-      <c r="F95" s="87" t="n"/>
-    </row>
-    <row r="96" ht="28" customHeight="1" s="136">
-      <c r="B96" s="106" t="inlineStr">
+      <c r="C96" s="86" t="n"/>
+      <c r="D96" s="86" t="n"/>
+      <c r="E96" s="86" t="n"/>
+      <c r="F96" s="87" t="n"/>
+    </row>
+    <row r="97" ht="28" customHeight="1" s="136">
+      <c r="B97" s="151" t="inlineStr">
         <is>
           <t>1.</t>
         </is>
       </c>
-      <c r="C96" s="152" t="n"/>
-      <c r="D96" s="83" t="n"/>
-      <c r="E96" s="83" t="n"/>
-      <c r="F96" s="84" t="n"/>
-    </row>
-    <row r="97" ht="28" customHeight="1" s="136">
-      <c r="B97" s="106" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C97" s="152" t="n"/>
+      <c r="C97" s="197" t="n"/>
       <c r="D97" s="83" t="n"/>
       <c r="E97" s="83" t="n"/>
       <c r="F97" s="84" t="n"/>
     </row>
     <row r="98" ht="28" customHeight="1" s="136">
-      <c r="B98" s="106" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C98" s="152" t="n"/>
+      <c r="B98" s="151" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C98" s="197" t="n"/>
       <c r="D98" s="83" t="n"/>
       <c r="E98" s="83" t="n"/>
       <c r="F98" s="84" t="n"/>
     </row>
-    <row r="99" ht="18" customHeight="1" s="136">
-      <c r="B99" s="88" t="inlineStr">
+    <row r="99" ht="28" customHeight="1" s="136">
+      <c r="B99" s="151" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C99" s="197" t="n"/>
+      <c r="D99" s="83" t="n"/>
+      <c r="E99" s="83" t="n"/>
+      <c r="F99" s="84" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1" s="136">
+      <c r="B100" s="88" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
       </c>
-      <c r="C99" s="86" t="n"/>
-      <c r="D99" s="86" t="n"/>
-      <c r="E99" s="87" t="n"/>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="C100" s="86" t="n"/>
+      <c r="D100" s="86" t="n"/>
+      <c r="E100" s="87" t="n"/>
+      <c r="F100" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="28" customHeight="1" s="136">
-      <c r="B100" s="145" t="inlineStr">
+    <row r="101" ht="28" customHeight="1" s="136">
+      <c r="B101" s="145" t="inlineStr">
         <is>
           <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
         </is>
       </c>
-      <c r="C100" s="83" t="n"/>
-      <c r="D100" s="83" t="n"/>
-      <c r="E100" s="83" t="n"/>
-      <c r="F100" s="84" t="n"/>
-    </row>
-    <row r="101" ht="28" customHeight="1" s="136">
-      <c r="B101" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C101" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D101" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C101" s="83" t="n"/>
+      <c r="D101" s="83" t="n"/>
       <c r="E101" s="83" t="n"/>
       <c r="F101" s="84" t="n"/>
     </row>
     <row r="102" ht="28" customHeight="1" s="136">
-      <c r="B102" s="82" t="inlineStr">
-        <is>
-          <t>Demonstrated empathy including for repeat-contact fatigue</t>
-        </is>
-      </c>
-      <c r="C102" s="102" t="n"/>
-      <c r="D102" s="146" t="n"/>
+      <c r="B102" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C102" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D102" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E102" s="83" t="n"/>
       <c r="F102" s="84" t="n"/>
     </row>
     <row r="103" ht="28" customHeight="1" s="136">
-      <c r="B103" s="94" t="inlineStr">
-        <is>
-          <t>Stayed professional throughout and maintained patience, even under pressure</t>
-        </is>
-      </c>
-      <c r="C103" s="102" t="n"/>
-      <c r="D103" s="147" t="n"/>
+      <c r="B103" s="146" t="inlineStr">
+        <is>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
+        </is>
+      </c>
+      <c r="C103" s="197" t="n"/>
+      <c r="D103" s="146" t="n"/>
       <c r="E103" s="83" t="n"/>
       <c r="F103" s="84" t="n"/>
     </row>
     <row r="104" ht="28" customHeight="1" s="136">
-      <c r="B104" s="82" t="inlineStr">
-        <is>
-          <t>Agent matched the customer's tone, pace, level, and energy</t>
-        </is>
-      </c>
-      <c r="C104" s="102" t="n"/>
-      <c r="D104" s="146" t="n"/>
+      <c r="B104" s="198" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+        </is>
+      </c>
+      <c r="C104" s="197" t="n"/>
+      <c r="D104" s="198" t="n"/>
       <c r="E104" s="83" t="n"/>
       <c r="F104" s="84" t="n"/>
     </row>
     <row r="105" ht="28" customHeight="1" s="136">
-      <c r="B105" s="82" t="inlineStr">
-        <is>
-          <t>Minimized customer effort</t>
-        </is>
-      </c>
-      <c r="C105" s="102" t="n"/>
+      <c r="B105" s="146" t="inlineStr">
+        <is>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
+        </is>
+      </c>
+      <c r="C105" s="197" t="n"/>
       <c r="D105" s="146" t="n"/>
       <c r="E105" s="83" t="n"/>
       <c r="F105" s="84" t="n"/>
     </row>
     <row r="106" ht="28" customHeight="1" s="136">
-      <c r="B106" s="94" t="inlineStr">
-        <is>
-          <t>Maintained customer understanding and engagement</t>
-        </is>
-      </c>
-      <c r="C106" s="102" t="n"/>
-      <c r="D106" s="147" t="n"/>
+      <c r="B106" s="146" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
+        </is>
+      </c>
+      <c r="C106" s="197" t="n"/>
+      <c r="D106" s="146" t="n"/>
       <c r="E106" s="83" t="n"/>
       <c r="F106" s="84" t="n"/>
     </row>
     <row r="107" ht="28" customHeight="1" s="136">
-      <c r="B107" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="C107" s="83" t="n"/>
-      <c r="D107" s="83" t="n"/>
+      <c r="B107" s="198" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C107" s="197" t="n"/>
+      <c r="D107" s="198" t="n"/>
       <c r="E107" s="83" t="n"/>
       <c r="F107" s="84" t="n"/>
     </row>
     <row r="108" ht="28" customHeight="1" s="136">
-      <c r="B108" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C108" s="68">
-        <f>IF((COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed"))=0,"",ROUND((COUNTIF(C102:C106,"Met")*5+COUNTIF(C102:C106,"Partial")*2.5)/(COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D108" s="149" t="n"/>
+      <c r="B108" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
+        </is>
+      </c>
+      <c r="C108" s="83" t="n"/>
+      <c r="D108" s="83" t="n"/>
       <c r="E108" s="83" t="n"/>
       <c r="F108" s="84" t="n"/>
     </row>
-    <row r="109" ht="24" customHeight="1" s="136">
-      <c r="B109" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C109" s="14" t="n"/>
-      <c r="D109" s="150">
-        <f>IF(IF(C109="",C108,C109)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C109="",C108,C109)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="109" ht="28" customHeight="1" s="136">
+      <c r="B109" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C109" s="200">
+        <f>IF((COUNTIF(C103:C107,"Met")+COUNTIF(C103:C107,"Partial")+COUNTIF(C103:C107,"Missed"))=0,"",ROUND((COUNTIF(C103:C107,"Met")*5+COUNTIF(C103:C107,"Partial")*2.5)/(COUNTIF(C103:C107,"Met")+COUNTIF(C103:C107,"Partial")+COUNTIF(C103:C107,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D109" s="149" t="n"/>
       <c r="E109" s="83" t="n"/>
       <c r="F109" s="84" t="n"/>
     </row>
-    <row r="110" ht="36" customHeight="1" s="136">
-      <c r="B110" s="106" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
-      <c r="C110" s="143" t="n"/>
-      <c r="D110" s="83" t="n"/>
+    <row r="110" ht="24" customHeight="1" s="136">
+      <c r="B110" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C110" s="201" t="n"/>
+      <c r="D110" s="150">
+        <f>IF(IF(C110="",C109,C110)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C110="",C109,C110)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E110" s="83" t="n"/>
       <c r="F110" s="84" t="n"/>
     </row>
-    <row r="111" ht="18" customHeight="1" s="136">
-      <c r="B111" s="88" t="inlineStr">
+    <row r="111" ht="36" customHeight="1" s="136">
+      <c r="B111" s="151" t="inlineStr">
+        <is>
+          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
+        </is>
+      </c>
+      <c r="C111" s="180" t="n"/>
+      <c r="D111" s="83" t="n"/>
+      <c r="E111" s="83" t="n"/>
+      <c r="F111" s="84" t="n"/>
+    </row>
+    <row r="112" ht="18" customHeight="1" s="136">
+      <c r="B112" s="88" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
       </c>
-      <c r="C111" s="86" t="n"/>
-      <c r="D111" s="86" t="n"/>
-      <c r="E111" s="87" t="n"/>
-      <c r="F111" s="6" t="inlineStr">
+      <c r="C112" s="86" t="n"/>
+      <c r="D112" s="86" t="n"/>
+      <c r="E112" s="87" t="n"/>
+      <c r="F112" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="28" customHeight="1" s="136">
-      <c r="B112" s="145" t="inlineStr">
+    <row r="113" ht="28" customHeight="1" s="136">
+      <c r="B113" s="145" t="inlineStr">
         <is>
           <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
         </is>
       </c>
-      <c r="C112" s="83" t="n"/>
-      <c r="D112" s="83" t="n"/>
-      <c r="E112" s="83" t="n"/>
-      <c r="F112" s="84" t="n"/>
-    </row>
-    <row r="113" ht="36" customHeight="1" s="136">
-      <c r="B113" s="100" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C113" s="7" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D113" s="144" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="C113" s="83" t="n"/>
+      <c r="D113" s="83" t="n"/>
       <c r="E113" s="83" t="n"/>
       <c r="F113" s="84" t="n"/>
     </row>
-    <row r="114" ht="28" customHeight="1" s="136">
-      <c r="B114" s="82" t="inlineStr">
-        <is>
-          <t>Recorded customer issue summary</t>
-        </is>
-      </c>
-      <c r="C114" s="102" t="n"/>
-      <c r="D114" s="146" t="n"/>
+    <row r="114" ht="36" customHeight="1" s="136">
+      <c r="B114" s="144" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C114" s="196" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D114" s="144" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E114" s="83" t="n"/>
       <c r="F114" s="84" t="n"/>
     </row>
     <row r="115" ht="28" customHeight="1" s="136">
-      <c r="B115" s="94" t="inlineStr">
-        <is>
-          <t>Documented troubleshooting steps</t>
-        </is>
-      </c>
-      <c r="C115" s="102" t="n"/>
-      <c r="D115" s="147" t="n"/>
+      <c r="B115" s="146" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
+        </is>
+      </c>
+      <c r="C115" s="197" t="n"/>
+      <c r="D115" s="146" t="n"/>
       <c r="E115" s="83" t="n"/>
       <c r="F115" s="84" t="n"/>
     </row>
     <row r="116" ht="28" customHeight="1" s="136">
-      <c r="B116" s="82" t="inlineStr">
-        <is>
-          <t>Noted key findings</t>
-        </is>
-      </c>
-      <c r="C116" s="102" t="n"/>
-      <c r="D116" s="146" t="n"/>
+      <c r="B116" s="198" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
+        </is>
+      </c>
+      <c r="C116" s="197" t="n"/>
+      <c r="D116" s="198" t="n"/>
       <c r="E116" s="83" t="n"/>
       <c r="F116" s="84" t="n"/>
     </row>
     <row r="117" ht="28" customHeight="1" s="136">
-      <c r="B117" s="94" t="inlineStr">
-        <is>
-          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
-        </is>
-      </c>
-      <c r="C117" s="102" t="n"/>
-      <c r="D117" s="147" t="n"/>
+      <c r="B117" s="146" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
+        </is>
+      </c>
+      <c r="C117" s="197" t="n"/>
+      <c r="D117" s="146" t="n"/>
       <c r="E117" s="83" t="n"/>
       <c r="F117" s="84" t="n"/>
     </row>
     <row r="118" ht="28" customHeight="1" s="136">
-      <c r="B118" s="94" t="inlineStr">
-        <is>
-          <t>Documented next steps and follow-ups</t>
-        </is>
-      </c>
-      <c r="C118" s="102" t="n"/>
-      <c r="D118" s="147" t="n"/>
+      <c r="B118" s="198" t="inlineStr">
+        <is>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
+        </is>
+      </c>
+      <c r="C118" s="197" t="n"/>
+      <c r="D118" s="198" t="n"/>
       <c r="E118" s="83" t="n"/>
       <c r="F118" s="84" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1" s="136">
-      <c r="B119" s="82" t="inlineStr">
-        <is>
-          <t>Updated ticket status accurately</t>
-        </is>
-      </c>
-      <c r="C119" s="102" t="n"/>
-      <c r="D119" s="146" t="n"/>
+      <c r="B119" s="198" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
+        </is>
+      </c>
+      <c r="C119" s="197" t="n"/>
+      <c r="D119" s="198" t="n"/>
       <c r="E119" s="83" t="n"/>
       <c r="F119" s="84" t="n"/>
     </row>
     <row r="120" ht="28" customHeight="1" s="136">
-      <c r="B120" s="148" t="inlineStr">
-        <is>
-          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="C120" s="83" t="n"/>
-      <c r="D120" s="83" t="n"/>
+      <c r="B120" s="146" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C120" s="197" t="n"/>
+      <c r="D120" s="146" t="n"/>
       <c r="E120" s="83" t="n"/>
       <c r="F120" s="84" t="n"/>
     </row>
-    <row r="121" ht="52" customHeight="1" s="136">
-      <c r="B121" s="11" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C121" s="68">
-        <f>IF((COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed"))=0,"",ROUND((COUNTIF(C114:C119,"Met")*5+COUNTIF(C114:C119,"Partial")*2.5)/(COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D121" s="149" t="n"/>
+    <row r="121" ht="28" customHeight="1" s="136">
+      <c r="B121" s="148" t="inlineStr">
+        <is>
+          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
+        </is>
+      </c>
+      <c r="C121" s="83" t="n"/>
+      <c r="D121" s="83" t="n"/>
       <c r="E121" s="83" t="n"/>
       <c r="F121" s="84" t="n"/>
     </row>
-    <row r="122" ht="24" customHeight="1" s="136">
-      <c r="B122" s="106" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C122" s="14" t="n"/>
-      <c r="D122" s="150">
-        <f>IF(IF(C122="",C121,C122)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C122="",C121,C122)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="122" ht="52" customHeight="1" s="136">
+      <c r="B122" s="199" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C122" s="200">
+        <f>IF((COUNTIF(C115:C120,"Met")+COUNTIF(C115:C120,"Partial")+COUNTIF(C115:C120,"Missed"))=0,"",ROUND((COUNTIF(C115:C120,"Met")*5+COUNTIF(C115:C120,"Partial")*2.5)/(COUNTIF(C115:C120,"Met")+COUNTIF(C115:C120,"Partial")+COUNTIF(C115:C120,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D122" s="149" t="n"/>
       <c r="E122" s="83" t="n"/>
       <c r="F122" s="84" t="n"/>
     </row>
-    <row r="123" ht="36" customHeight="1" s="136">
-      <c r="B123" s="106" t="inlineStr">
-        <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
-      <c r="C123" s="143" t="n"/>
-      <c r="D123" s="83" t="n"/>
+    <row r="123" ht="24" customHeight="1" s="136">
+      <c r="B123" s="151" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C123" s="201" t="n"/>
+      <c r="D123" s="150">
+        <f>IF(IF(C123="",C122,C123)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C123="",C122,C123)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E123" s="83" t="n"/>
       <c r="F123" s="84" t="n"/>
     </row>
-    <row r="124" ht="30" customHeight="1" s="136">
-      <c r="B124" s="88" t="inlineStr">
+    <row r="124" ht="36" customHeight="1" s="136">
+      <c r="B124" s="151" t="inlineStr">
+        <is>
+          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
+        </is>
+      </c>
+      <c r="C124" s="180" t="n"/>
+      <c r="D124" s="83" t="n"/>
+      <c r="E124" s="83" t="n"/>
+      <c r="F124" s="84" t="n"/>
+    </row>
+    <row r="125" ht="30" customHeight="1" s="136">
+      <c r="B125" s="88" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
       </c>
-      <c r="C124" s="86" t="n"/>
-      <c r="D124" s="86" t="n"/>
-      <c r="E124" s="86" t="n"/>
-      <c r="F124" s="87" t="n"/>
-    </row>
-    <row r="125" ht="28" customHeight="1" s="136">
-      <c r="B125" s="100" t="inlineStr">
+      <c r="C125" s="86" t="n"/>
+      <c r="D125" s="86" t="n"/>
+      <c r="E125" s="86" t="n"/>
+      <c r="F125" s="87" t="n"/>
+    </row>
+    <row r="126" ht="28" customHeight="1" s="136">
+      <c r="B126" s="144" t="inlineStr">
         <is>
           <t>Outcome classification</t>
         </is>
       </c>
-      <c r="C125" s="153" t="n"/>
-      <c r="D125" s="83" t="n"/>
-      <c r="E125" s="83" t="n"/>
-      <c r="F125" s="84" t="n"/>
-    </row>
-    <row r="126" ht="52" customHeight="1" s="136">
-      <c r="B126" s="98" t="inlineStr">
-        <is>
-          <t>Primary positive outcome achieved</t>
-        </is>
-      </c>
-      <c r="C126" s="142" t="n"/>
+      <c r="C126" s="202" t="n"/>
       <c r="D126" s="83" t="n"/>
       <c r="E126" s="83" t="n"/>
       <c r="F126" s="84" t="n"/>
     </row>
     <row r="127" ht="52" customHeight="1" s="136">
-      <c r="B127" s="100" t="inlineStr">
-        <is>
-          <t>Justification</t>
-        </is>
-      </c>
-      <c r="C127" s="143" t="n"/>
+      <c r="B127" s="167" t="inlineStr">
+        <is>
+          <t>Primary positive outcome achieved</t>
+        </is>
+      </c>
+      <c r="C127" s="179" t="n"/>
       <c r="D127" s="83" t="n"/>
       <c r="E127" s="83" t="n"/>
       <c r="F127" s="84" t="n"/>
     </row>
-    <row r="128" ht="26" customHeight="1" s="136">
-      <c r="B128" s="88" t="inlineStr">
+    <row r="128" ht="52" customHeight="1" s="136">
+      <c r="B128" s="144" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
+      <c r="C128" s="180" t="n"/>
+      <c r="D128" s="83" t="n"/>
+      <c r="E128" s="83" t="n"/>
+      <c r="F128" s="84" t="n"/>
+    </row>
+    <row r="129" ht="26" customHeight="1" s="136">
+      <c r="B129" s="88" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
       </c>
-      <c r="C128" s="86" t="n"/>
-      <c r="D128" s="86" t="n"/>
-      <c r="E128" s="86" t="n"/>
-      <c r="F128" s="87" t="n"/>
-    </row>
-    <row r="129" ht="30" customHeight="1" s="136">
-      <c r="B129" s="98" t="inlineStr">
+      <c r="C129" s="86" t="n"/>
+      <c r="D129" s="86" t="n"/>
+      <c r="E129" s="86" t="n"/>
+      <c r="F129" s="87" t="n"/>
+    </row>
+    <row r="130" ht="30" customHeight="1" s="136">
+      <c r="B130" s="167" t="inlineStr">
         <is>
           <t>Did the interaction disconnect before completion?</t>
         </is>
       </c>
-      <c r="C129" s="102" t="inlineStr">
+      <c r="C130" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D129" s="148" t="inlineStr">
+      <c r="D130" s="148" t="inlineStr">
         <is>
           <t>If Yes, at least one documented follow-up action is required.</t>
         </is>
       </c>
-      <c r="E129" s="83" t="n"/>
-      <c r="F129" s="84" t="n"/>
-    </row>
-    <row r="130" ht="30" customHeight="1" s="136">
-      <c r="B130" s="100" t="inlineStr">
+      <c r="E130" s="83" t="n"/>
+      <c r="F130" s="84" t="n"/>
+    </row>
+    <row r="131" ht="30" customHeight="1" s="136">
+      <c r="A131" s="155" t="n"/>
+      <c r="B131" s="144" t="inlineStr">
         <is>
           <t>Follow-up action taken</t>
         </is>
       </c>
-      <c r="C130" s="142" t="inlineStr">
+      <c r="C131" s="179" t="inlineStr">
         <is>
           <t>N.A. — no disconnect</t>
         </is>
       </c>
-      <c r="D130" s="84" t="n"/>
-      <c r="E130" s="154">
-        <f>IF(AND(C129="Yes",OR(C130="None",C130="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
-        <v/>
-      </c>
-      <c r="F130" s="84" t="n"/>
-    </row>
-    <row r="131" ht="22" customHeight="1" s="136">
-      <c r="A131" s="155" t="n"/>
-      <c r="B131" s="156" t="inlineStr">
+      <c r="D131" s="84" t="n"/>
+      <c r="E131" s="203">
+        <f>IF(AND(C130="Yes",OR(C131="None",C131="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
+        <v/>
+      </c>
+      <c r="F131" s="84" t="n"/>
+      <c r="G131" s="155" t="n"/>
+    </row>
+    <row r="132" ht="22" customHeight="1" s="136">
+      <c r="A132" s="155" t="n"/>
+      <c r="B132" s="156" t="inlineStr">
         <is>
           <t>COACHING FLAGS   ·   Auto-populated from Partial and Missed ratings   ·   Each flagged item requires a coaching or review action</t>
         </is>
       </c>
-      <c r="C131" s="86" t="n"/>
-      <c r="D131" s="86" t="n"/>
-      <c r="E131" s="86" t="n"/>
-      <c r="F131" s="87" t="n"/>
-      <c r="G131" s="155" t="n"/>
-    </row>
-    <row r="132" ht="18" customHeight="1" s="136">
-      <c r="A132" s="155" t="n"/>
-      <c r="B132" s="157" t="inlineStr">
-        <is>
-          <t>Flag Condition</t>
-        </is>
-      </c>
-      <c r="C132" s="157" t="inlineStr">
-        <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="D132" s="157" t="inlineStr">
-        <is>
-          <t>Coaching Focus / Required Action</t>
-        </is>
-      </c>
+      <c r="C132" s="158" t="n"/>
+      <c r="D132" s="158" t="n"/>
       <c r="E132" s="158" t="n"/>
       <c r="F132" s="159" t="n"/>
       <c r="G132" s="155" t="n"/>
     </row>
-    <row r="133" ht="28" customHeight="1" s="136">
+    <row r="133" ht="18" customHeight="1" s="136">
       <c r="A133" s="155" t="n"/>
-      <c r="B133" s="160" t="inlineStr">
-        <is>
-          <t>Technical accuracy failure</t>
-        </is>
-      </c>
-      <c r="C133" s="161">
-        <f>IF(OR(C50="Partial",C50="Missed"),C50,"")</f>
-        <v/>
-      </c>
-      <c r="D133" s="162" t="inlineStr">
-        <is>
-          <t>Review for incorrect guidance, product misrepresentation, or unsupported root-cause conclusions</t>
-        </is>
-      </c>
-      <c r="E133" s="83" t="n"/>
-      <c r="F133" s="84" t="n"/>
+      <c r="B133" s="157" t="inlineStr">
+        <is>
+          <t>Flag Condition</t>
+        </is>
+      </c>
+      <c r="C133" s="157" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="D133" s="157" t="inlineStr">
+        <is>
+          <t>Coaching Focus / Required Action</t>
+        </is>
+      </c>
+      <c r="E133" s="158" t="n"/>
+      <c r="F133" s="159" t="n"/>
       <c r="G133" s="155" t="n"/>
     </row>
     <row r="134" ht="28" customHeight="1" s="136">
       <c r="A134" s="155" t="n"/>
       <c r="B134" s="160" t="inlineStr">
         <is>
-          <t>No follow-up after disconnected call</t>
+          <t>Technical accuracy failure</t>
         </is>
       </c>
       <c r="C134" s="161">
-        <f>IF(OR(C76="Partial",C76="Missed"),C76,"")</f>
+        <f>IF(OR(C51="Partial",C51="Missed"),C51,"")</f>
         <v/>
       </c>
       <c r="D134" s="162" t="inlineStr">
         <is>
-          <t>Mandatory callback attempt required; document outcome in case notes</t>
-        </is>
-      </c>
-      <c r="E134" s="83" t="n"/>
-      <c r="F134" s="84" t="n"/>
+          <t>Review for incorrect guidance, product misrepresentation, or unsupported root-cause conclusions</t>
+        </is>
+      </c>
+      <c r="E134" s="158" t="n"/>
+      <c r="F134" s="159" t="n"/>
       <c r="G134" s="155" t="n"/>
     </row>
     <row r="135" ht="28" customHeight="1" s="136">
       <c r="A135" s="155" t="n"/>
       <c r="B135" s="160" t="inlineStr">
         <is>
-          <t>Commitments not fulfilled / clear path forward missing</t>
+          <t>No follow-up after disconnected call</t>
         </is>
       </c>
       <c r="C135" s="161">
-        <f>IF(OR(C73="Partial",C73="Missed"),C73,"")</f>
+        <f>IF(OR(C77="Partial",C77="Missed"),C77,"")</f>
         <v/>
       </c>
       <c r="D135" s="162" t="inlineStr">
         <is>
-          <t>Review what was promised; confirm the customer was left with actionable next steps</t>
-        </is>
-      </c>
-      <c r="E135" s="83" t="n"/>
-      <c r="F135" s="84" t="n"/>
+          <t>Mandatory callback attempt required; document outcome in case notes</t>
+        </is>
+      </c>
+      <c r="E135" s="158" t="n"/>
+      <c r="F135" s="159" t="n"/>
       <c r="G135" s="155" t="n"/>
     </row>
     <row r="136" ht="28" customHeight="1" s="136">
       <c r="A136" s="155" t="n"/>
       <c r="B136" s="160" t="inlineStr">
         <is>
-          <t>Customer abandoned without a path forward</t>
+          <t>Commitments not fulfilled / clear path forward missing</t>
         </is>
       </c>
       <c r="C136" s="161">
-        <f>IF(OR(C38="Partial",C38="Missed"),C38,"")</f>
+        <f>IF(OR(C74="Partial",C74="Missed"),C74,"")</f>
         <v/>
       </c>
       <c r="D136" s="162" t="inlineStr">
         <is>
-          <t>Review whether the customer had any defined next step at close; address in coaching session</t>
-        </is>
-      </c>
-      <c r="E136" s="83" t="n"/>
-      <c r="F136" s="84" t="n"/>
+          <t>Review what was promised; confirm the customer was left with actionable next steps</t>
+        </is>
+      </c>
+      <c r="E136" s="158" t="n"/>
+      <c r="F136" s="159" t="n"/>
       <c r="G136" s="155" t="n"/>
     </row>
     <row r="137" ht="28" customHeight="1" s="136">
       <c r="A137" s="155" t="n"/>
       <c r="B137" s="160" t="inlineStr">
         <is>
-          <t>Escalated without completing reasonable troubleshooting</t>
+          <t>Customer abandoned without a path forward</t>
         </is>
       </c>
       <c r="C137" s="161">
-        <f>IF(OR(C84="Partial",C84="Missed"),C84,"")</f>
+        <f>IF(OR(C39="Partial",C39="Missed"),C39,"")</f>
         <v/>
       </c>
       <c r="D137" s="162" t="inlineStr">
         <is>
-          <t>Review L1 steps completed before escalation; identify gaps and add to troubleshooting playbook</t>
-        </is>
-      </c>
-      <c r="E137" s="83" t="n"/>
-      <c r="F137" s="84" t="n"/>
+          <t>Review whether the customer had any defined next step at close; address in coaching session</t>
+        </is>
+      </c>
+      <c r="E137" s="158" t="n"/>
+      <c r="F137" s="159" t="n"/>
       <c r="G137" s="155" t="n"/>
     </row>
     <row r="138" ht="28" customHeight="1" s="136">
       <c r="A138" s="155" t="n"/>
       <c r="B138" s="160" t="inlineStr">
         <is>
-          <t>Escalation criteria not met / complaint or legal-risk not escalated</t>
+          <t>Escalated without completing reasonable troubleshooting</t>
         </is>
       </c>
       <c r="C138" s="161">
@@ -5464,162 +5557,167 @@
       </c>
       <c r="D138" s="162" t="inlineStr">
         <is>
-          <t>Review whether a valid escalation trigger existed; coach on recognising escalation criteria</t>
-        </is>
-      </c>
-      <c r="E138" s="83" t="n"/>
-      <c r="F138" s="84" t="n"/>
+          <t>Review L1 steps completed before escalation; identify gaps and add to troubleshooting playbook</t>
+        </is>
+      </c>
+      <c r="E138" s="158" t="n"/>
+      <c r="F138" s="159" t="n"/>
       <c r="G138" s="155" t="n"/>
     </row>
     <row r="139" ht="28" customHeight="1" s="136">
       <c r="A139" s="155" t="n"/>
       <c r="B139" s="160" t="inlineStr">
         <is>
-          <t>Professionalism concern</t>
+          <t>Escalation criteria not met / complaint or legal-risk not escalated</t>
         </is>
       </c>
       <c r="C139" s="161">
-        <f>IF(OR(C103="Partial",C103="Missed"),C103,"")</f>
+        <f>IF(OR(C86="Partial",C86="Missed"),C86,"")</f>
         <v/>
       </c>
       <c r="D139" s="162" t="inlineStr">
         <is>
-          <t>Mandatory review; assess tone, conduct, and whether a policy violation occurred</t>
-        </is>
-      </c>
-      <c r="E139" s="83" t="n"/>
-      <c r="F139" s="84" t="n"/>
+          <t>Review whether a valid escalation trigger existed; coach on recognising escalation criteria</t>
+        </is>
+      </c>
+      <c r="E139" s="158" t="n"/>
+      <c r="F139" s="159" t="n"/>
       <c r="G139" s="155" t="n"/>
     </row>
     <row r="140" ht="28" customHeight="1" s="136">
       <c r="A140" s="155" t="n"/>
       <c r="B140" s="160" t="inlineStr">
         <is>
+          <t>Professionalism concern</t>
+        </is>
+      </c>
+      <c r="C140" s="161">
+        <f>IF(OR(C104="Partial",C104="Missed"),C104,"")</f>
+        <v/>
+      </c>
+      <c r="D140" s="162" t="inlineStr">
+        <is>
+          <t>Mandatory review; assess tone, conduct, and whether a policy violation occurred</t>
+        </is>
+      </c>
+      <c r="E140" s="158" t="n"/>
+      <c r="F140" s="159" t="n"/>
+      <c r="G140" s="155" t="n"/>
+    </row>
+    <row r="141" ht="28" customHeight="1" s="136">
+      <c r="A141" s="155" t="n"/>
+      <c r="B141" s="160" t="inlineStr">
+        <is>
           <t>Ticket status inaccurate / premature closure</t>
         </is>
       </c>
-      <c r="C140" s="161">
-        <f>IF(OR(C119="Partial",C119="Missed"),C119,"")</f>
-        <v/>
-      </c>
-      <c r="D140" s="162" t="inlineStr">
+      <c r="C141" s="161">
+        <f>IF(OR(C120="Partial",C120="Missed"),C120,"")</f>
+        <v/>
+      </c>
+      <c r="D141" s="162" t="inlineStr">
         <is>
           <t>Review ticket state at close; verify status accurately reflected the case outcome</t>
         </is>
       </c>
-      <c r="E140" s="83" t="n"/>
-      <c r="F140" s="84" t="n"/>
-      <c r="G140" s="155" t="n"/>
-    </row>
-    <row r="141" ht="22" customHeight="1" s="136">
-      <c r="A141" s="155" t="n"/>
-      <c r="B141" s="163" t="inlineStr">
-        <is>
-          <t>⚠  Survey / CSAT manipulation has no matching behavioral indicator and cannot be auto-detected — flag manually in §8 Coaching &amp; Feedback if suspected.</t>
-        </is>
-      </c>
-      <c r="C141" s="83" t="n"/>
-      <c r="D141" s="83" t="n"/>
-      <c r="E141" s="83" t="n"/>
-      <c r="F141" s="84" t="n"/>
+      <c r="E141" s="158" t="n"/>
+      <c r="F141" s="159" t="n"/>
       <c r="G141" s="155" t="n"/>
     </row>
     <row r="142" ht="22" customHeight="1" s="136">
       <c r="A142" s="155" t="n"/>
-      <c r="B142" s="164">
-        <f>IF(COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")=0,"✓  No coaching flags triggered — all key indicators met",COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")&amp;" coaching flag(s) triggered — review and coaching action required")</f>
-        <v/>
-      </c>
-      <c r="C142" s="83" t="n"/>
-      <c r="D142" s="83" t="n"/>
-      <c r="E142" s="83" t="n"/>
-      <c r="F142" s="84" t="n"/>
+      <c r="B142" s="163" t="inlineStr">
+        <is>
+          <t>⚠  Survey / CSAT manipulation has no matching behavioral indicator and cannot be auto-detected — flag manually in §8 Coaching &amp; Feedback if suspected.</t>
+        </is>
+      </c>
+      <c r="C142" s="158" t="n"/>
+      <c r="D142" s="158" t="n"/>
+      <c r="E142" s="158" t="n"/>
+      <c r="F142" s="159" t="n"/>
       <c r="G142" s="155" t="n"/>
     </row>
-    <row r="143" ht="65" customHeight="1" s="136">
+    <row r="143" ht="22" customHeight="1" s="136">
       <c r="A143" s="155" t="n"/>
-      <c r="B143" s="165">
-        <f>IF(COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")=0,"All key indicators met — no coaching action required",TEXTJOIN(CHAR(10),TRUE,IF(C133&lt;&gt;"","⚑ "&amp;B133&amp;" ["&amp;C133&amp;"]",""),IF(C134&lt;&gt;"","⚑ "&amp;B134&amp;" ["&amp;C134&amp;"]",""),IF(C135&lt;&gt;"","⚑ "&amp;B135&amp;" ["&amp;C135&amp;"]",""),IF(C136&lt;&gt;"","⚑ "&amp;B136&amp;" ["&amp;C136&amp;"]",""),IF(C137&lt;&gt;"","⚑ "&amp;B137&amp;" ["&amp;C137&amp;"]",""),IF(C138&lt;&gt;"","⚑ "&amp;B138&amp;" ["&amp;C138&amp;"]",""),IF(C139&lt;&gt;"","⚑ "&amp;B139&amp;" ["&amp;C139&amp;"]",""),IF(C140&lt;&gt;"","⚑ "&amp;B140&amp;" ["&amp;C140&amp;"]","")))</f>
-        <v/>
-      </c>
-      <c r="C143" s="83" t="n"/>
-      <c r="D143" s="83" t="n"/>
-      <c r="E143" s="83" t="n"/>
-      <c r="F143" s="84" t="n"/>
+      <c r="B143" s="164">
+        <f>IF(COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")=0,"✓  No coaching flags triggered — all key indicators met",COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")&amp;" coaching flag(s) triggered — review and coaching action required")</f>
+        <v/>
+      </c>
+      <c r="C143" s="158" t="n"/>
+      <c r="D143" s="158" t="n"/>
+      <c r="E143" s="158" t="n"/>
+      <c r="F143" s="159" t="n"/>
       <c r="G143" s="155" t="n"/>
     </row>
-    <row r="144" ht="6" customHeight="1" s="136">
+    <row r="144" ht="65" customHeight="1" s="136">
       <c r="A144" s="155" t="n"/>
-      <c r="B144" s="166" t="n"/>
-      <c r="C144" s="86" t="n"/>
-      <c r="D144" s="86" t="n"/>
-      <c r="E144" s="86" t="n"/>
-      <c r="F144" s="87" t="n"/>
+      <c r="B144" s="165">
+        <f>IF(COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")=0,"All key indicators met — no coaching action required",TEXTJOIN(CHAR(10),TRUE,IF(C134&lt;&gt;"","⚑ "&amp;B134&amp;" ["&amp;C134&amp;"]",""),IF(C135&lt;&gt;"","⚑ "&amp;B135&amp;" ["&amp;C135&amp;"]",""),IF(C136&lt;&gt;"","⚑ "&amp;B136&amp;" ["&amp;C136&amp;"]",""),IF(C137&lt;&gt;"","⚑ "&amp;B137&amp;" ["&amp;C137&amp;"]",""),IF(C138&lt;&gt;"","⚑ "&amp;B138&amp;" ["&amp;C138&amp;"]",""),IF(C139&lt;&gt;"","⚑ "&amp;B139&amp;" ["&amp;C139&amp;"]",""),IF(C140&lt;&gt;"","⚑ "&amp;B140&amp;" ["&amp;C140&amp;"]",""),IF(C141&lt;&gt;"","⚑ "&amp;B141&amp;" ["&amp;C141&amp;"]","")))</f>
+        <v/>
+      </c>
+      <c r="C144" s="158" t="n"/>
+      <c r="D144" s="158" t="n"/>
+      <c r="E144" s="158" t="n"/>
+      <c r="F144" s="159" t="n"/>
       <c r="G144" s="155" t="n"/>
     </row>
-    <row r="145" ht="22" customHeight="1" s="136">
-      <c r="B145" s="92" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
+    <row r="145" ht="6" customHeight="1" s="136">
+      <c r="A145" s="155" t="n"/>
+      <c r="B145" s="166" t="n"/>
       <c r="C145" s="86" t="n"/>
       <c r="D145" s="86" t="n"/>
       <c r="E145" s="86" t="n"/>
       <c r="F145" s="87" t="n"/>
-    </row>
-    <row r="146" ht="30" customHeight="1" s="136">
-      <c r="B146" s="148" t="inlineStr">
+      <c r="G145" s="155" t="n"/>
+    </row>
+    <row r="146" ht="22" customHeight="1" s="136">
+      <c r="B146" s="92" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
+      <c r="C146" s="86" t="n"/>
+      <c r="D146" s="86" t="n"/>
+      <c r="E146" s="86" t="n"/>
+      <c r="F146" s="87" t="n"/>
+    </row>
+    <row r="147" ht="30" customHeight="1" s="136">
+      <c r="B147" s="148" t="inlineStr">
         <is>
           <t>A gate marked 'No', any A–K item marked 'Yes' forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
         </is>
       </c>
-      <c r="C146" s="83" t="n"/>
-      <c r="D146" s="83" t="n"/>
-      <c r="E146" s="83" t="n"/>
-      <c r="F146" s="84" t="n"/>
-    </row>
-    <row r="147" ht="30" customHeight="1" s="136">
-      <c r="B147" s="88" t="inlineStr">
+      <c r="C147" s="83" t="n"/>
+      <c r="D147" s="83" t="n"/>
+      <c r="E147" s="83" t="n"/>
+      <c r="F147" s="84" t="n"/>
+    </row>
+    <row r="148" ht="30" customHeight="1" s="136">
+      <c r="B148" s="88" t="inlineStr">
         <is>
           <t>Compliance gate  (mark Yes if adhered)</t>
         </is>
       </c>
-      <c r="C147" s="133" t="inlineStr">
+      <c r="C148" s="133" t="inlineStr">
         <is>
           <t>Adherent?</t>
         </is>
       </c>
-      <c r="D147" s="88" t="inlineStr">
+      <c r="D148" s="88" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E147" s="86" t="n"/>
-      <c r="F147" s="87" t="n"/>
-    </row>
-    <row r="148" ht="26" customHeight="1" s="136">
-      <c r="B148" s="82" t="inlineStr">
+      <c r="E148" s="86" t="n"/>
+      <c r="F148" s="87" t="n"/>
+    </row>
+    <row r="149" ht="26" customHeight="1" s="136">
+      <c r="B149" s="146" t="inlineStr">
         <is>
           <t>Adherence to Callback Hours</t>
         </is>
       </c>
-      <c r="C148" s="102" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D148" s="146" t="n"/>
-      <c r="E148" s="83" t="n"/>
-      <c r="F148" s="84" t="n"/>
-    </row>
-    <row r="149" ht="26" customHeight="1" s="136">
-      <c r="B149" s="82" t="inlineStr">
-        <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C149" s="102" t="inlineStr">
+      <c r="C149" s="197" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5629,12 +5727,12 @@
       <c r="F149" s="84" t="n"/>
     </row>
     <row r="150" ht="26" customHeight="1" s="136">
-      <c r="B150" s="82" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C150" s="102" t="inlineStr">
+      <c r="B150" s="146" t="inlineStr">
+        <is>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C150" s="197" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -5643,47 +5741,47 @@
       <c r="E150" s="83" t="n"/>
       <c r="F150" s="84" t="n"/>
     </row>
-    <row r="151" ht="32" customHeight="1" s="136">
-      <c r="B151" s="88" t="inlineStr">
+    <row r="151" ht="26" customHeight="1" s="136">
+      <c r="B151" s="146" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C151" s="197" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D151" s="146" t="n"/>
+      <c r="E151" s="83" t="n"/>
+      <c r="F151" s="84" t="n"/>
+    </row>
+    <row r="152" ht="32" customHeight="1" s="136">
+      <c r="B152" s="88" t="inlineStr">
         <is>
           <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
         </is>
       </c>
-      <c r="C151" s="133" t="inlineStr">
+      <c r="C152" s="133" t="inlineStr">
         <is>
           <t>Occurred?</t>
         </is>
       </c>
-      <c r="D151" s="88" t="inlineStr">
+      <c r="D152" s="88" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E151" s="86" t="n"/>
-      <c r="F151" s="87" t="n"/>
-    </row>
-    <row r="152" ht="26" customHeight="1" s="136">
-      <c r="B152" s="82" t="inlineStr">
+      <c r="E152" s="86" t="n"/>
+      <c r="F152" s="87" t="n"/>
+    </row>
+    <row r="153" ht="26" customHeight="1" s="136">
+      <c r="B153" s="146" t="inlineStr">
         <is>
           <t>A.  Call / Session Abandonment</t>
         </is>
       </c>
-      <c r="C152" s="102" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D152" s="146" t="n"/>
-      <c r="E152" s="83" t="n"/>
-      <c r="F152" s="84" t="n"/>
-    </row>
-    <row r="153" ht="26" customHeight="1" s="136">
-      <c r="B153" s="82" t="inlineStr">
-        <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
-        </is>
-      </c>
-      <c r="C153" s="102" t="inlineStr">
+      <c r="C153" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5693,12 +5791,12 @@
       <c r="F153" s="84" t="n"/>
     </row>
     <row r="154" ht="26" customHeight="1" s="136">
-      <c r="B154" s="82" t="inlineStr">
-        <is>
-          <t>C.  Discourtesy</t>
-        </is>
-      </c>
-      <c r="C154" s="102" t="inlineStr">
+      <c r="B154" s="146" t="inlineStr">
+        <is>
+          <t>B.  Call / Session Avoidance / Evasion</t>
+        </is>
+      </c>
+      <c r="C154" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5708,12 +5806,12 @@
       <c r="F154" s="84" t="n"/>
     </row>
     <row r="155" ht="26" customHeight="1" s="136">
-      <c r="B155" s="82" t="inlineStr">
-        <is>
-          <t>D.  Escalation</t>
-        </is>
-      </c>
-      <c r="C155" s="102" t="inlineStr">
+      <c r="B155" s="146" t="inlineStr">
+        <is>
+          <t>C.  Discourtesy</t>
+        </is>
+      </c>
+      <c r="C155" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5723,12 +5821,12 @@
       <c r="F155" s="84" t="n"/>
     </row>
     <row r="156" ht="26" customHeight="1" s="136">
-      <c r="B156" s="82" t="inlineStr">
-        <is>
-          <t>E.  Failure to ask for the email address</t>
-        </is>
-      </c>
-      <c r="C156" s="102" t="inlineStr">
+      <c r="B156" s="146" t="inlineStr">
+        <is>
+          <t>D.  Escalation</t>
+        </is>
+      </c>
+      <c r="C156" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5738,12 +5836,12 @@
       <c r="F156" s="84" t="n"/>
     </row>
     <row r="157" ht="26" customHeight="1" s="136">
-      <c r="B157" s="82" t="inlineStr">
-        <is>
-          <t>F.  Fraud</t>
-        </is>
-      </c>
-      <c r="C157" s="102" t="inlineStr">
+      <c r="B157" s="146" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="C157" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5753,12 +5851,12 @@
       <c r="F157" s="84" t="n"/>
     </row>
     <row r="158" ht="26" customHeight="1" s="136">
-      <c r="B158" s="82" t="inlineStr">
-        <is>
-          <t>G.  Hard-selling</t>
-        </is>
-      </c>
-      <c r="C158" s="102" t="inlineStr">
+      <c r="B158" s="146" t="inlineStr">
+        <is>
+          <t>F.  Fraud</t>
+        </is>
+      </c>
+      <c r="C158" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5768,12 +5866,12 @@
       <c r="F158" s="84" t="n"/>
     </row>
     <row r="159" ht="26" customHeight="1" s="136">
-      <c r="B159" s="82" t="inlineStr">
-        <is>
-          <t>H.  Line Release</t>
-        </is>
-      </c>
-      <c r="C159" s="102" t="inlineStr">
+      <c r="B159" s="146" t="inlineStr">
+        <is>
+          <t>G.  Hard-selling</t>
+        </is>
+      </c>
+      <c r="C159" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5783,12 +5881,12 @@
       <c r="F159" s="84" t="n"/>
     </row>
     <row r="160" ht="26" customHeight="1" s="136">
-      <c r="B160" s="82" t="inlineStr">
-        <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C160" s="102" t="inlineStr">
+      <c r="B160" s="146" t="inlineStr">
+        <is>
+          <t>H.  Line Release</t>
+        </is>
+      </c>
+      <c r="C160" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5798,12 +5896,12 @@
       <c r="F160" s="84" t="n"/>
     </row>
     <row r="161" ht="26" customHeight="1" s="136">
-      <c r="B161" s="82" t="inlineStr">
-        <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C161" s="102" t="inlineStr">
+      <c r="B161" s="146" t="inlineStr">
+        <is>
+          <t>I.  Non-Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C161" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5813,12 +5911,12 @@
       <c r="F161" s="84" t="n"/>
     </row>
     <row r="162" ht="26" customHeight="1" s="136">
-      <c r="B162" s="82" t="inlineStr">
-        <is>
-          <t>K.  Non-First Call Resolution</t>
-        </is>
-      </c>
-      <c r="C162" s="102" t="inlineStr">
+      <c r="B162" s="146" t="inlineStr">
+        <is>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C162" s="197" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5827,35 +5925,39 @@
       <c r="E162" s="83" t="n"/>
       <c r="F162" s="84" t="n"/>
     </row>
-    <row r="163" ht="24" customHeight="1" s="136">
-      <c r="B163" s="92" t="inlineStr">
+    <row r="163" ht="26" customHeight="1" s="136">
+      <c r="B163" s="146" t="inlineStr">
+        <is>
+          <t>K.  Non-First Call Resolution</t>
+        </is>
+      </c>
+      <c r="C163" s="197" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D163" s="146" t="n"/>
+      <c r="E163" s="83" t="n"/>
+      <c r="F163" s="84" t="n"/>
+    </row>
+    <row r="164" ht="24" customHeight="1" s="136">
+      <c r="B164" s="92" t="inlineStr">
         <is>
           <t>AUTO-ZERO TRIGGERED?</t>
         </is>
       </c>
-      <c r="C163" s="85">
-        <f>IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
-      <c r="D163" s="86" t="n"/>
-      <c r="E163" s="86" t="n"/>
-      <c r="F163" s="87" t="n"/>
-    </row>
-    <row r="164" ht="20" customHeight="1" s="136">
-      <c r="B164" s="104" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
-        </is>
-      </c>
-      <c r="C164" s="86" t="n"/>
+      <c r="C164" s="204">
+        <f>IF(OR(C149="No",C150="No",C151="No",COUNTIF(C153:C163,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
       <c r="D164" s="86" t="n"/>
       <c r="E164" s="86" t="n"/>
       <c r="F164" s="87" t="n"/>
     </row>
-    <row r="165" ht="30" customHeight="1" s="136">
-      <c r="B165" s="101" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+    <row r="165" ht="20" customHeight="1" s="136">
+      <c r="B165" s="181" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
         </is>
       </c>
       <c r="C165" s="86" t="n"/>
@@ -5863,453 +5965,465 @@
       <c r="E165" s="86" t="n"/>
       <c r="F165" s="87" t="n"/>
     </row>
-    <row r="166" ht="58" customHeight="1" s="136">
-      <c r="B166" s="143" t="n"/>
-      <c r="C166" s="83" t="n"/>
-      <c r="D166" s="83" t="n"/>
-      <c r="E166" s="83" t="n"/>
-      <c r="F166" s="84" t="n"/>
-    </row>
-    <row r="167" ht="30" customHeight="1" s="136">
-      <c r="B167" s="101" t="inlineStr">
+    <row r="166" ht="30" customHeight="1" s="136">
+      <c r="B166" s="101" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
+        </is>
+      </c>
+      <c r="C166" s="86" t="n"/>
+      <c r="D166" s="86" t="n"/>
+      <c r="E166" s="86" t="n"/>
+      <c r="F166" s="87" t="n"/>
+    </row>
+    <row r="167" ht="58" customHeight="1" s="136">
+      <c r="B167" s="180" t="n"/>
+      <c r="C167" s="83" t="n"/>
+      <c r="D167" s="83" t="n"/>
+      <c r="E167" s="83" t="n"/>
+      <c r="F167" s="84" t="n"/>
+    </row>
+    <row r="168" ht="30" customHeight="1" s="136">
+      <c r="B168" s="101" t="inlineStr">
         <is>
           <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
         </is>
       </c>
-      <c r="C167" s="86" t="n"/>
-      <c r="D167" s="86" t="n"/>
-      <c r="E167" s="86" t="n"/>
-      <c r="F167" s="87" t="n"/>
-    </row>
-    <row r="168" ht="24" customHeight="1" s="136">
-      <c r="B168" s="167" t="inlineStr">
+      <c r="C168" s="86" t="n"/>
+      <c r="D168" s="86" t="n"/>
+      <c r="E168" s="86" t="n"/>
+      <c r="F168" s="87" t="n"/>
+    </row>
+    <row r="169" ht="24" customHeight="1" s="136">
+      <c r="B169" s="167" t="inlineStr">
         <is>
           <t>What went well — behaviors to repeat</t>
         </is>
       </c>
-      <c r="C168" s="83" t="n"/>
-      <c r="D168" s="83" t="n"/>
-      <c r="E168" s="83" t="n"/>
-      <c r="F168" s="84" t="n"/>
-    </row>
-    <row r="169" ht="32" customHeight="1" s="136">
-      <c r="B169" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C169" s="143" t="n"/>
+      <c r="C169" s="83" t="n"/>
       <c r="D169" s="83" t="n"/>
       <c r="E169" s="83" t="n"/>
       <c r="F169" s="84" t="n"/>
     </row>
     <row r="170" ht="32" customHeight="1" s="136">
-      <c r="B170" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C170" s="143" t="n"/>
+      <c r="B170" s="196" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C170" s="180" t="n"/>
       <c r="D170" s="83" t="n"/>
       <c r="E170" s="83" t="n"/>
       <c r="F170" s="84" t="n"/>
     </row>
     <row r="171" ht="32" customHeight="1" s="136">
-      <c r="B171" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C171" s="143" t="n"/>
+      <c r="B171" s="196" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C171" s="180" t="n"/>
       <c r="D171" s="83" t="n"/>
       <c r="E171" s="83" t="n"/>
       <c r="F171" s="84" t="n"/>
     </row>
-    <row r="172" ht="24" customHeight="1" s="136">
-      <c r="B172" s="167" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
-      <c r="C172" s="83" t="n"/>
+    <row r="172" ht="32" customHeight="1" s="136">
+      <c r="B172" s="196" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C172" s="180" t="n"/>
       <c r="D172" s="83" t="n"/>
       <c r="E172" s="83" t="n"/>
       <c r="F172" s="84" t="n"/>
     </row>
-    <row r="173" ht="32" customHeight="1" s="136">
-      <c r="B173" s="7" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C173" s="143" t="n"/>
+    <row r="173" ht="24" customHeight="1" s="136">
+      <c r="B173" s="167" t="inlineStr">
+        <is>
+          <t>Improvement opportunities — behaviors to improve</t>
+        </is>
+      </c>
+      <c r="C173" s="83" t="n"/>
       <c r="D173" s="83" t="n"/>
       <c r="E173" s="83" t="n"/>
       <c r="F173" s="84" t="n"/>
     </row>
     <row r="174" ht="32" customHeight="1" s="136">
-      <c r="B174" s="7" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C174" s="143" t="n"/>
+      <c r="B174" s="196" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C174" s="180" t="n"/>
       <c r="D174" s="83" t="n"/>
       <c r="E174" s="83" t="n"/>
       <c r="F174" s="84" t="n"/>
     </row>
     <row r="175" ht="32" customHeight="1" s="136">
-      <c r="B175" s="7" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C175" s="143" t="n"/>
+      <c r="B175" s="196" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C175" s="180" t="n"/>
       <c r="D175" s="83" t="n"/>
       <c r="E175" s="83" t="n"/>
       <c r="F175" s="84" t="n"/>
     </row>
-    <row r="176" ht="24" customHeight="1" s="136">
-      <c r="B176" s="167" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
-      <c r="C176" s="83" t="n"/>
+    <row r="176" ht="32" customHeight="1" s="136">
+      <c r="B176" s="196" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C176" s="180" t="n"/>
       <c r="D176" s="83" t="n"/>
       <c r="E176" s="83" t="n"/>
       <c r="F176" s="84" t="n"/>
     </row>
-    <row r="177" ht="58" customHeight="1" s="136">
-      <c r="B177" s="143" t="n"/>
+    <row r="177" ht="24" customHeight="1" s="136">
+      <c r="B177" s="167" t="inlineStr">
+        <is>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
+        </is>
+      </c>
       <c r="C177" s="83" t="n"/>
       <c r="D177" s="83" t="n"/>
       <c r="E177" s="83" t="n"/>
       <c r="F177" s="84" t="n"/>
     </row>
-    <row r="178" ht="20" customHeight="1" s="136">
-      <c r="B178" s="167" t="inlineStr">
-        <is>
-          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
-        </is>
-      </c>
+    <row r="178" ht="58" customHeight="1" s="136">
+      <c r="B178" s="180" t="n"/>
       <c r="C178" s="83" t="n"/>
       <c r="D178" s="83" t="n"/>
       <c r="E178" s="83" t="n"/>
       <c r="F178" s="84" t="n"/>
     </row>
-    <row r="179" ht="28" customHeight="1" s="136">
-      <c r="B179" s="90" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C179" s="143" t="n"/>
+    <row r="179" ht="20" customHeight="1" s="136">
+      <c r="B179" s="167" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
+      <c r="C179" s="83" t="n"/>
       <c r="D179" s="83" t="n"/>
       <c r="E179" s="83" t="n"/>
       <c r="F179" s="84" t="n"/>
     </row>
     <row r="180" ht="28" customHeight="1" s="136">
-      <c r="B180" s="90" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C180" s="143" t="n"/>
+      <c r="B180" s="180" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C180" s="180" t="n"/>
       <c r="D180" s="83" t="n"/>
       <c r="E180" s="83" t="n"/>
       <c r="F180" s="84" t="n"/>
     </row>
     <row r="181" ht="28" customHeight="1" s="136">
-      <c r="B181" s="90" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C181" s="152" t="n"/>
+      <c r="B181" s="180" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C181" s="180" t="n"/>
       <c r="D181" s="83" t="n"/>
       <c r="E181" s="83" t="n"/>
       <c r="F181" s="84" t="n"/>
     </row>
-    <row r="182" ht="32" customHeight="1" s="136">
-      <c r="B182" s="101" t="inlineStr">
+    <row r="182" ht="28" customHeight="1" s="136">
+      <c r="B182" s="180" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C182" s="197" t="n"/>
+      <c r="D182" s="83" t="n"/>
+      <c r="E182" s="83" t="n"/>
+      <c r="F182" s="84" t="n"/>
+    </row>
+    <row r="183" ht="32" customHeight="1" s="136">
+      <c r="B183" s="101" t="inlineStr">
         <is>
           <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
         </is>
       </c>
-      <c r="C182" s="86" t="n"/>
-      <c r="D182" s="86" t="n"/>
-      <c r="E182" s="86" t="n"/>
-      <c r="F182" s="87" t="n"/>
-    </row>
-    <row r="183" ht="24" customHeight="1" s="136">
-      <c r="B183" s="167" t="inlineStr">
+      <c r="C183" s="86" t="n"/>
+      <c r="D183" s="86" t="n"/>
+      <c r="E183" s="86" t="n"/>
+      <c r="F183" s="87" t="n"/>
+    </row>
+    <row r="184" ht="24" customHeight="1" s="136">
+      <c r="B184" s="167" t="inlineStr">
         <is>
           <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
         </is>
       </c>
-      <c r="C183" s="83" t="n"/>
-      <c r="D183" s="83" t="n"/>
-      <c r="E183" s="83" t="n"/>
-      <c r="F183" s="84" t="n"/>
-    </row>
-    <row r="184" ht="58" customHeight="1" s="136">
-      <c r="B184" s="143" t="n"/>
       <c r="C184" s="83" t="n"/>
       <c r="D184" s="83" t="n"/>
       <c r="E184" s="83" t="n"/>
       <c r="F184" s="84" t="n"/>
     </row>
-    <row r="185" ht="24" customHeight="1" s="136">
-      <c r="B185" s="167" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
+    <row r="185" ht="58" customHeight="1" s="136">
+      <c r="B185" s="180" t="n"/>
       <c r="C185" s="83" t="n"/>
       <c r="D185" s="83" t="n"/>
       <c r="E185" s="83" t="n"/>
       <c r="F185" s="84" t="n"/>
     </row>
-    <row r="186" ht="58" customHeight="1" s="136">
-      <c r="B186" s="143" t="n"/>
+    <row r="186" ht="24" customHeight="1" s="136">
+      <c r="B186" s="167" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
       <c r="C186" s="83" t="n"/>
       <c r="D186" s="83" t="n"/>
       <c r="E186" s="83" t="n"/>
       <c r="F186" s="84" t="n"/>
     </row>
-    <row r="187" ht="24" customHeight="1" s="136">
-      <c r="B187" s="167" t="inlineStr">
-        <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
-        </is>
-      </c>
+    <row r="187" ht="58" customHeight="1" s="136">
+      <c r="B187" s="180" t="n"/>
       <c r="C187" s="83" t="n"/>
       <c r="D187" s="83" t="n"/>
       <c r="E187" s="83" t="n"/>
       <c r="F187" s="84" t="n"/>
     </row>
-    <row r="188" ht="58" customHeight="1" s="136">
-      <c r="B188" s="143" t="n"/>
+    <row r="188" ht="24" customHeight="1" s="136">
+      <c r="B188" s="167" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
       <c r="C188" s="83" t="n"/>
       <c r="D188" s="83" t="n"/>
       <c r="E188" s="83" t="n"/>
       <c r="F188" s="84" t="n"/>
     </row>
-    <row r="189" ht="24" customHeight="1" s="136"/>
-    <row r="190" ht="58" customHeight="1" s="136"/>
-    <row r="191" ht="20" customHeight="1" s="136"/>
-    <row r="192" ht="30" customHeight="1" s="136"/>
-    <row r="193" ht="58" customHeight="1" s="136"/>
-    <row r="194" ht="30" customHeight="1" s="136"/>
-    <row r="195" ht="24" customHeight="1" s="136"/>
-    <row r="196" ht="32" customHeight="1" s="136"/>
+    <row r="189" ht="58" customHeight="1" s="136">
+      <c r="B189" s="180" t="n"/>
+      <c r="C189" s="83" t="n"/>
+      <c r="D189" s="83" t="n"/>
+      <c r="E189" s="83" t="n"/>
+      <c r="F189" s="84" t="n"/>
+    </row>
+    <row r="190" ht="24" customHeight="1" s="136"/>
+    <row r="191" ht="58" customHeight="1" s="136"/>
+    <row r="192" ht="20" customHeight="1" s="136"/>
+    <row r="193" ht="30" customHeight="1" s="136"/>
+    <row r="194" ht="58" customHeight="1" s="136"/>
+    <row r="195" ht="30" customHeight="1" s="136"/>
+    <row r="196" ht="24" customHeight="1" s="136"/>
     <row r="197" ht="32" customHeight="1" s="136"/>
     <row r="198" ht="32" customHeight="1" s="136"/>
-    <row r="199" ht="24" customHeight="1" s="136"/>
-    <row r="200" ht="32" customHeight="1" s="136"/>
+    <row r="199" ht="32" customHeight="1" s="136"/>
+    <row r="200" ht="24" customHeight="1" s="136"/>
     <row r="201" ht="32" customHeight="1" s="136"/>
     <row r="202" ht="32" customHeight="1" s="136"/>
-    <row r="203" ht="24" customHeight="1" s="136"/>
-    <row r="204" ht="58" customHeight="1" s="136"/>
-    <row r="205" ht="20" customHeight="1" s="136"/>
-    <row r="206" ht="28" customHeight="1" s="136"/>
+    <row r="203" ht="32" customHeight="1" s="136"/>
+    <row r="204" ht="24" customHeight="1" s="136"/>
+    <row r="205" ht="58" customHeight="1" s="136"/>
+    <row r="206" ht="20" customHeight="1" s="136"/>
     <row r="207" ht="28" customHeight="1" s="136"/>
     <row r="208" ht="28" customHeight="1" s="136"/>
-    <row r="209" ht="32" customHeight="1" s="136"/>
-    <row r="210" ht="24" customHeight="1" s="136"/>
-    <row r="211" ht="58" customHeight="1" s="136"/>
-    <row r="212" ht="24" customHeight="1" s="136"/>
-    <row r="213" ht="58" customHeight="1" s="136"/>
-    <row r="214" ht="24" customHeight="1" s="136"/>
-    <row r="215" ht="58" customHeight="1" s="136"/>
+    <row r="209" ht="28" customHeight="1" s="136"/>
+    <row r="210" ht="32" customHeight="1" s="136"/>
+    <row r="211" ht="24" customHeight="1" s="136"/>
+    <row r="212" ht="58" customHeight="1" s="136"/>
+    <row r="213" ht="24" customHeight="1" s="136"/>
+    <row r="214" ht="58" customHeight="1" s="136"/>
+    <row r="215" ht="24" customHeight="1" s="136"/>
     <row r="216" ht="58" customHeight="1" s="136"/>
-    <row r="217" ht="24" customHeight="1" s="136"/>
-    <row r="218" ht="58" customHeight="1" s="136"/>
-    <row r="219" ht="24" customHeight="1" s="136"/>
-    <row r="220" ht="58" customHeight="1" s="136"/>
+    <row r="217" ht="58" customHeight="1" s="136"/>
+    <row r="218" ht="24" customHeight="1" s="136"/>
+    <row r="219" ht="58" customHeight="1" s="136"/>
+    <row r="220" ht="24" customHeight="1" s="136"/>
+    <row r="221" ht="58" customHeight="1" s="136"/>
   </sheetData>
-  <mergeCells count="178">
+  <mergeCells count="179">
+    <mergeCell ref="B129:F129"/>
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="D116:F116"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="C81:F81"/>
     <mergeCell ref="B184:F184"/>
-    <mergeCell ref="C125:F125"/>
-    <mergeCell ref="B131:F131"/>
-    <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
+    <mergeCell ref="B71:F71"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B52:F52"/>
     <mergeCell ref="C13:F13"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="D37:F37"/>
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="D37:F37"/>
     <mergeCell ref="D102:F102"/>
+    <mergeCell ref="B100:E100"/>
     <mergeCell ref="D152:F152"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="B179:F179"/>
     <mergeCell ref="B166:F166"/>
     <mergeCell ref="D133:F133"/>
-    <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B172:F172"/>
-    <mergeCell ref="D129:F129"/>
+    <mergeCell ref="C172:F172"/>
+    <mergeCell ref="B94:C95"/>
+    <mergeCell ref="B34:F34"/>
     <mergeCell ref="C171:F171"/>
+    <mergeCell ref="B108:F108"/>
     <mergeCell ref="B186:F186"/>
-    <mergeCell ref="C54:F54"/>
     <mergeCell ref="B168:F168"/>
     <mergeCell ref="B143:F143"/>
-    <mergeCell ref="B92:F92"/>
-    <mergeCell ref="C173:F173"/>
+    <mergeCell ref="C164:F164"/>
     <mergeCell ref="D119:F119"/>
     <mergeCell ref="D159:F159"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="D80:F80"/>
+    <mergeCell ref="C43:F43"/>
     <mergeCell ref="B142:F142"/>
-    <mergeCell ref="C163:F163"/>
+    <mergeCell ref="B112:E112"/>
     <mergeCell ref="D105:F105"/>
-    <mergeCell ref="D57:F57"/>
     <mergeCell ref="B144:F144"/>
-    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="D120:F120"/>
+    <mergeCell ref="D41:F41"/>
+    <mergeCell ref="B125:F125"/>
     <mergeCell ref="D154:F154"/>
-    <mergeCell ref="D41:F41"/>
     <mergeCell ref="B185:F185"/>
+    <mergeCell ref="D163:F163"/>
+    <mergeCell ref="D107:F107"/>
     <mergeCell ref="E5:F5"/>
-    <mergeCell ref="D147:F147"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B121:F121"/>
+    <mergeCell ref="D91:F91"/>
+    <mergeCell ref="B96:F96"/>
     <mergeCell ref="D162:F162"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B167:F167"/>
+    <mergeCell ref="C111:F111"/>
     <mergeCell ref="D156:F156"/>
-    <mergeCell ref="B167:F167"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="B176:F176"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="D137:F137"/>
     <mergeCell ref="D106:F106"/>
-    <mergeCell ref="D137:F137"/>
-    <mergeCell ref="C96:F96"/>
-    <mergeCell ref="B120:F120"/>
+    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="C92:F92"/>
     <mergeCell ref="C175:F175"/>
-    <mergeCell ref="B107:F107"/>
     <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D83:F83"/>
+    <mergeCell ref="D130:F130"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="B57:F57"/>
+    <mergeCell ref="C14:F14"/>
     <mergeCell ref="D117:F117"/>
-    <mergeCell ref="B88:F88"/>
     <mergeCell ref="D157:F157"/>
     <mergeCell ref="C98:F98"/>
-    <mergeCell ref="B82:F82"/>
     <mergeCell ref="D67:F67"/>
-    <mergeCell ref="D132:F132"/>
+    <mergeCell ref="D110:F110"/>
     <mergeCell ref="D85:F85"/>
+    <mergeCell ref="D54:F54"/>
     <mergeCell ref="B146:F146"/>
     <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D109:F109"/>
     <mergeCell ref="B187:F187"/>
-    <mergeCell ref="D109:F109"/>
+    <mergeCell ref="B83:F83"/>
+    <mergeCell ref="C124:F124"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D46:F46"/>
-    <mergeCell ref="B124:F124"/>
     <mergeCell ref="D158:F158"/>
-    <mergeCell ref="D40:F40"/>
-    <mergeCell ref="D108:F108"/>
+    <mergeCell ref="B189:F189"/>
+    <mergeCell ref="B45:F45"/>
     <mergeCell ref="D86:F86"/>
-    <mergeCell ref="C123:F123"/>
+    <mergeCell ref="B173:F173"/>
     <mergeCell ref="B188:F188"/>
     <mergeCell ref="D104:F104"/>
     <mergeCell ref="D160:F160"/>
-    <mergeCell ref="C110:F110"/>
     <mergeCell ref="C181:F181"/>
-    <mergeCell ref="E130:F130"/>
     <mergeCell ref="D136:F136"/>
-    <mergeCell ref="C91:F91"/>
     <mergeCell ref="D150:F150"/>
-    <mergeCell ref="B141:F141"/>
-    <mergeCell ref="B31:F31"/>
     <mergeCell ref="C174:F174"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="D78:F78"/>
     <mergeCell ref="D87:F87"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="B39:F39"/>
     <mergeCell ref="D122:F122"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="C179:F179"/>
     <mergeCell ref="D58:F58"/>
-    <mergeCell ref="C68:F68"/>
     <mergeCell ref="B145:F145"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="D121:F121"/>
     <mergeCell ref="D73:F73"/>
-    <mergeCell ref="D113:F113"/>
+    <mergeCell ref="D42:F42"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="B56:E56"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C128:F128"/>
+    <mergeCell ref="B147:F147"/>
     <mergeCell ref="C97:F97"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B43:E43"/>
     <mergeCell ref="B178:F178"/>
     <mergeCell ref="D148:F148"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="D123:F123"/>
     <mergeCell ref="D35:F35"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="B128:F128"/>
+    <mergeCell ref="D115:F115"/>
     <mergeCell ref="D59:F59"/>
-    <mergeCell ref="D115:F115"/>
-    <mergeCell ref="B93:C94"/>
     <mergeCell ref="D138:F138"/>
-    <mergeCell ref="D34:F34"/>
     <mergeCell ref="B183:F183"/>
-    <mergeCell ref="B65:F65"/>
     <mergeCell ref="C127:F127"/>
-    <mergeCell ref="C80:F80"/>
-    <mergeCell ref="B164:F164"/>
+    <mergeCell ref="C176:F176"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="D140:F140"/>
     <mergeCell ref="D84:F84"/>
-    <mergeCell ref="C12:F12"/>
     <mergeCell ref="D155:F155"/>
-    <mergeCell ref="D140:F140"/>
+    <mergeCell ref="B44:E44"/>
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="D149:F149"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="D101:F101"/>
-    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="C131:D131"/>
+    <mergeCell ref="D77:F77"/>
+    <mergeCell ref="B113:F113"/>
     <mergeCell ref="D151:F151"/>
-    <mergeCell ref="B100:F100"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="B165:F165"/>
+    <mergeCell ref="D141:F141"/>
+    <mergeCell ref="B66:F66"/>
     <mergeCell ref="D135:F135"/>
     <mergeCell ref="D48:F48"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B93:F93"/>
+    <mergeCell ref="E17:F17"/>
     <mergeCell ref="C170:F170"/>
-    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D103:F103"/>
     <mergeCell ref="D134:F134"/>
-    <mergeCell ref="B77:F77"/>
+    <mergeCell ref="D72:F72"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="D118:F118"/>
+    <mergeCell ref="B132:F132"/>
+    <mergeCell ref="B101:F101"/>
+    <mergeCell ref="D114:F114"/>
     <mergeCell ref="D161:F161"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="D114:F114"/>
-    <mergeCell ref="C42:F42"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D64:F64"/>
+    <mergeCell ref="C19:F19"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="C126:F126"/>
-    <mergeCell ref="D89:F89"/>
-    <mergeCell ref="B182:F182"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="B112:F112"/>
+    <mergeCell ref="B78:F78"/>
     <mergeCell ref="D79:F79"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="E11:F11"/>
+    <mergeCell ref="D88:F88"/>
     <mergeCell ref="D153:F153"/>
-    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="C99:F99"/>
+    <mergeCell ref="B40:F40"/>
     <mergeCell ref="D63:F63"/>
     <mergeCell ref="C180:F180"/>
     <mergeCell ref="D90:F90"/>
     <mergeCell ref="B177:F177"/>
-    <mergeCell ref="B95:F95"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="B89:F89"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="B169:F169"/>
+    <mergeCell ref="B82:E82"/>
     <mergeCell ref="D139:F139"/>
-    <mergeCell ref="D52:F52"/>
-    <mergeCell ref="C169:F169"/>
+    <mergeCell ref="C182:F182"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="D49:F49"/>
   </mergeCells>
-  <conditionalFormatting sqref="C20:C24">
+  <conditionalFormatting sqref="C21:C25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6320,7 +6434,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27">
+  <conditionalFormatting sqref="C28">
     <cfRule type="cellIs" priority="4" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6331,7 +6445,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:C39">
+  <conditionalFormatting sqref="C34:C40">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6342,7 +6456,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C42">
+  <conditionalFormatting sqref="C43">
     <cfRule type="cellIs" priority="10" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6353,7 +6467,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C48:C55">
+  <conditionalFormatting sqref="C49:C56">
     <cfRule type="cellIs" priority="13" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6364,7 +6478,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C58">
+  <conditionalFormatting sqref="C59">
     <cfRule type="cellIs" priority="16" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6375,7 +6489,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C64:C71">
+  <conditionalFormatting sqref="C65:C72">
     <cfRule type="cellIs" priority="19" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6386,7 +6500,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C74">
+  <conditionalFormatting sqref="C75">
     <cfRule type="cellIs" priority="22" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6397,7 +6511,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C80:C84">
+  <conditionalFormatting sqref="C81:C85">
     <cfRule type="cellIs" priority="25" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6408,7 +6522,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C87">
+  <conditionalFormatting sqref="C88">
     <cfRule type="cellIs" priority="28" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6419,7 +6533,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C93:C98">
+  <conditionalFormatting sqref="C94:C99">
     <cfRule type="cellIs" priority="31" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6430,7 +6544,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C101">
+  <conditionalFormatting sqref="C102">
     <cfRule type="cellIs" priority="34" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6441,7 +6555,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C107:C113">
+  <conditionalFormatting sqref="C108:C114">
     <cfRule type="cellIs" priority="37" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6452,7 +6566,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C116">
+  <conditionalFormatting sqref="C117">
     <cfRule type="cellIs" priority="40" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6463,12 +6577,12 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C141:C151">
+  <conditionalFormatting sqref="C142:C152">
     <cfRule type="cellIs" priority="51" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C152">
+  <conditionalFormatting sqref="C153">
     <cfRule type="expression" priority="53" dxfId="2">
       <formula>NOT(ISNUMBER(SEARCH("YES",C152)))</formula>
     </cfRule>
@@ -6476,7 +6590,7 @@
       <formula>ISNUMBER(SEARCH("YES",C152))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E128">
+  <conditionalFormatting sqref="E129">
     <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="30">
       <formula>0.85</formula>
     </cfRule>
@@ -6488,7 +6602,7 @@
       <formula>0.7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E137">
+  <conditionalFormatting sqref="E138">
     <cfRule type="expression" priority="49" dxfId="0">
       <formula>E137&lt;&gt;"OK"</formula>
     </cfRule>
@@ -6496,7 +6610,7 @@
       <formula>E137="OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F121:F127">
+  <conditionalFormatting sqref="F122:F128">
     <cfRule type="cellIs" priority="46" operator="equal" dxfId="9">
       <formula>"Strong"</formula>
     </cfRule>
@@ -6507,7 +6621,7 @@
       <formula>"Developing"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C133:C140">
+  <conditionalFormatting sqref="C134:C141">
     <cfRule type="cellIs" priority="54" operator="equal" dxfId="142">
       <formula>"Partial"</formula>
     </cfRule>
@@ -6515,39 +6629,42 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="11">
-    <dataValidation sqref="C35 C36 C37 C38 C46 C47 C48 C49 C50 C58 C59 C60 C61 C62 C63 C64 C72 C73 C75 C76 C84 C85 C86 C87 C102 C103 C104 C105 C106 C114 C115 C116 C117 C118 C119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="12">
+    <dataValidation sqref="C36 C37 C38 C39 C47 C48 C49 C50 C51 C59 C60 C61 C62 C63 C64 C65 C73 C74 C76 C77 C85 C86 C87 C88 C103 C104 C105 C106 C107 C115 C116 C117 C118 C119 C120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C41 C53 C67 C79 C90 C109 C122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
+    <dataValidation sqref="C42 C54 C68 C80 C91 C110 C123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C129 C152:C162 E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C130 C153:C163 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
-    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-Warranty,Out-of-Warranty,Unknown"</formula1>
     </dataValidation>
-    <dataValidation sqref="E6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Phone,Chat,Email,Social,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Technical Issue,Setup/How-To,RMA/Replacement,Billing/Account,Connectivity,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Within SLA,Breached,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Successful Resolution,Partial Resolution,Appropriate Escalation,Ownership Gap,Unresolved"</formula1>
     </dataValidation>
-    <dataValidation sqref="C126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_xlfn._LONGTEXT("Issue resolved,Proper RMA initiated (in-warranty / approved exception),Valid escalation submitted,Known limitation explained accurately,Customer educated with actionable next steps,Valid self-help guidance provided (out-of-warranty),Upgrade path recommend","ed appropriately (out-of-warranty),Customer declined further troubleshooting after reasonable effort,None achieved")</formula1>
     </dataValidation>
-    <dataValidation sqref="C130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C148:C150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C149:C151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid selection" error="Please choose Level 1 or Level 2." promptTitle="Agent Level" prompt="Select Level 1 for front-line support agents or Level 2 for senior/escalation agents." type="list">
+      <formula1>"Level 1,Level 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15208,8 +15325,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Remove Team Score Weight from Agent Level row — not yet implemented
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -729,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="205">
+  <cellXfs count="208">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1301,6 +1301,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3765,16 +3774,9 @@
         </is>
       </c>
       <c r="C5" s="176" t="n"/>
-      <c r="D5" s="177" t="inlineStr">
-        <is>
-          <t>Team Score Weight</t>
-        </is>
-      </c>
-      <c r="E5" s="178">
-        <f>IF(C5="Level 2","1.5×  —  senior support (L2 weight applies to team aggregations)",IF(C5="Level 1","1.0×  —  standard support (L1 weight applies to team aggregations)",""))</f>
-        <v/>
-      </c>
-      <c r="F5" s="84" t="n"/>
+      <c r="D5" s="205" t="n"/>
+      <c r="E5" s="206" t="n"/>
+      <c r="F5" s="207" t="n"/>
     </row>
     <row r="6" ht="29" customHeight="1" s="136">
       <c r="B6" s="144" t="inlineStr">
@@ -6242,13 +6244,14 @@
     <row r="220" ht="24" customHeight="1" s="136"/>
     <row r="221" ht="58" customHeight="1" s="136"/>
   </sheetData>
-  <mergeCells count="179">
+  <mergeCells count="178">
     <mergeCell ref="B129:F129"/>
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="D116:F116"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B184:F184"/>
     <mergeCell ref="C81:F81"/>
-    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
     <mergeCell ref="B71:F71"/>
     <mergeCell ref="D47:F47"/>
@@ -6291,15 +6294,15 @@
     <mergeCell ref="B185:F185"/>
     <mergeCell ref="D163:F163"/>
     <mergeCell ref="D107:F107"/>
-    <mergeCell ref="E5:F5"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B121:F121"/>
     <mergeCell ref="D91:F91"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="D162:F162"/>
     <mergeCell ref="B96:F96"/>
-    <mergeCell ref="D162:F162"/>
+    <mergeCell ref="D156:F156"/>
     <mergeCell ref="B167:F167"/>
     <mergeCell ref="C111:F111"/>
-    <mergeCell ref="D156:F156"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="D137:F137"/>
     <mergeCell ref="D106:F106"/>
@@ -6309,10 +6312,9 @@
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D130:F130"/>
     <mergeCell ref="D68:F68"/>
-    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="D117:F117"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="C14:F14"/>
-    <mergeCell ref="D117:F117"/>
     <mergeCell ref="D157:F157"/>
     <mergeCell ref="C98:F98"/>
     <mergeCell ref="D67:F67"/>
@@ -6359,15 +6361,15 @@
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="D123:F123"/>
     <mergeCell ref="D35:F35"/>
+    <mergeCell ref="D59:F59"/>
     <mergeCell ref="D115:F115"/>
-    <mergeCell ref="D59:F59"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="B183:F183"/>
     <mergeCell ref="C127:F127"/>
     <mergeCell ref="C176:F176"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="D84:F84"/>
     <mergeCell ref="D140:F140"/>
-    <mergeCell ref="D84:F84"/>
     <mergeCell ref="D155:F155"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="D36:F36"/>
@@ -6387,18 +6389,17 @@
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="C170:F170"/>
     <mergeCell ref="D103:F103"/>
+    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D134:F134"/>
-    <mergeCell ref="D72:F72"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="D118:F118"/>
+    <mergeCell ref="D161:F161"/>
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B101:F101"/>
     <mergeCell ref="D114:F114"/>
-    <mergeCell ref="D161:F161"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D64:F64"/>
-    <mergeCell ref="C19:F19"/>
     <mergeCell ref="D38:F38"/>
     <mergeCell ref="C126:F126"/>
     <mergeCell ref="B78:F78"/>
@@ -15325,8 +15326,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Case Tracker: add Level column and L1/L2 weighted Team Score
- New col Q (Level 1/Level 2 dropdown) on touch log rows 5-49
- Team Score formula: replaces flat 50pct avg touch with
  20pct x L1 avg + 30pct x L2 avg (L2 carries higher weight)
- Row 54 description updated to reflect new formula
- D55 renamed to Avg Touch pct (ref)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -729,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="208">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1311,6 +1311,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13806,7 +13812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P60"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="11" customWidth="1" style="136" min="1" max="1"/>
@@ -13818,6 +13824,7 @@
     <col width="60" customWidth="1" style="136" min="14" max="14"/>
     <col width="22" customWidth="1" style="136" min="15" max="15"/>
     <col width="14" customWidth="1" style="136" min="16" max="16"/>
+    <col width="14" customWidth="1" style="136" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="136">
@@ -13966,6 +13973,11 @@
           <t>Handoff Quality (0-5)</t>
         </is>
       </c>
+      <c r="Q4" s="208" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1" s="136">
       <c r="A5" s="39" t="n"/>
@@ -13990,6 +14002,7 @@
       <c r="N5" s="82" t="n"/>
       <c r="O5" s="20" t="n"/>
       <c r="P5" s="20" t="n"/>
+      <c r="Q5" s="209" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1" s="136">
       <c r="A6" s="39" t="n"/>
@@ -14014,6 +14027,7 @@
       <c r="N6" s="94" t="n"/>
       <c r="O6" s="25" t="n"/>
       <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="209" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1" s="136">
       <c r="A7" s="39" t="n"/>
@@ -14038,6 +14052,7 @@
       <c r="N7" s="82" t="n"/>
       <c r="O7" s="20" t="n"/>
       <c r="P7" s="20" t="n"/>
+      <c r="Q7" s="209" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1" s="136">
       <c r="A8" s="39" t="n"/>
@@ -14062,6 +14077,7 @@
       <c r="N8" s="94" t="n"/>
       <c r="O8" s="25" t="n"/>
       <c r="P8" s="25" t="n"/>
+      <c r="Q8" s="209" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1" s="136">
       <c r="A9" s="39" t="n"/>
@@ -14086,6 +14102,7 @@
       <c r="N9" s="82" t="n"/>
       <c r="O9" s="20" t="n"/>
       <c r="P9" s="20" t="n"/>
+      <c r="Q9" s="209" t="n"/>
     </row>
     <row r="10" ht="40" customHeight="1" s="136">
       <c r="A10" s="39" t="n"/>
@@ -14110,6 +14127,7 @@
       <c r="N10" s="94" t="n"/>
       <c r="O10" s="25" t="n"/>
       <c r="P10" s="25" t="n"/>
+      <c r="Q10" s="209" t="n"/>
     </row>
     <row r="11" ht="40" customHeight="1" s="136">
       <c r="A11" s="39" t="n"/>
@@ -14134,6 +14152,7 @@
       <c r="N11" s="82" t="n"/>
       <c r="O11" s="20" t="n"/>
       <c r="P11" s="20" t="n"/>
+      <c r="Q11" s="209" t="n"/>
     </row>
     <row r="12" ht="40" customHeight="1" s="136">
       <c r="A12" s="39" t="n"/>
@@ -14158,6 +14177,7 @@
       <c r="N12" s="94" t="n"/>
       <c r="O12" s="25" t="n"/>
       <c r="P12" s="25" t="n"/>
+      <c r="Q12" s="209" t="n"/>
     </row>
     <row r="13" ht="40" customHeight="1" s="136">
       <c r="A13" s="39" t="n"/>
@@ -14182,6 +14202,7 @@
       <c r="N13" s="82" t="n"/>
       <c r="O13" s="20" t="n"/>
       <c r="P13" s="20" t="n"/>
+      <c r="Q13" s="209" t="n"/>
     </row>
     <row r="14" ht="40" customHeight="1" s="136">
       <c r="A14" s="39" t="n"/>
@@ -14206,6 +14227,7 @@
       <c r="N14" s="94" t="n"/>
       <c r="O14" s="25" t="n"/>
       <c r="P14" s="25" t="n"/>
+      <c r="Q14" s="209" t="n"/>
     </row>
     <row r="15" ht="40" customHeight="1" s="136">
       <c r="A15" s="39" t="n"/>
@@ -14230,6 +14252,7 @@
       <c r="N15" s="82" t="n"/>
       <c r="O15" s="20" t="n"/>
       <c r="P15" s="20" t="n"/>
+      <c r="Q15" s="209" t="n"/>
     </row>
     <row r="16" ht="40" customHeight="1" s="136">
       <c r="A16" s="39" t="n"/>
@@ -14254,6 +14277,7 @@
       <c r="N16" s="94" t="n"/>
       <c r="O16" s="25" t="n"/>
       <c r="P16" s="25" t="n"/>
+      <c r="Q16" s="209" t="n"/>
     </row>
     <row r="17" ht="40" customHeight="1" s="136">
       <c r="A17" s="39" t="n"/>
@@ -14278,8 +14302,9 @@
       <c r="N17" s="82" t="n"/>
       <c r="O17" s="20" t="n"/>
       <c r="P17" s="20" t="n"/>
-    </row>
-    <row r="18">
+      <c r="Q17" s="209" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="136">
       <c r="A18" s="39" t="n"/>
       <c r="B18" s="39" t="n"/>
       <c r="C18" s="39" t="n"/>
@@ -14302,8 +14327,9 @@
       <c r="N18" s="94" t="n"/>
       <c r="O18" s="25" t="n"/>
       <c r="P18" s="25" t="n"/>
-    </row>
-    <row r="19">
+      <c r="Q18" s="209" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="136">
       <c r="A19" s="39" t="n"/>
       <c r="B19" s="39" t="n"/>
       <c r="C19" s="39" t="n"/>
@@ -14326,8 +14352,9 @@
       <c r="N19" s="82" t="n"/>
       <c r="O19" s="20" t="n"/>
       <c r="P19" s="20" t="n"/>
-    </row>
-    <row r="20">
+      <c r="Q19" s="209" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="136">
       <c r="A20" s="39" t="n"/>
       <c r="B20" s="39" t="n"/>
       <c r="C20" s="39" t="n"/>
@@ -14350,8 +14377,9 @@
       <c r="N20" s="94" t="n"/>
       <c r="O20" s="25" t="n"/>
       <c r="P20" s="25" t="n"/>
-    </row>
-    <row r="21">
+      <c r="Q20" s="209" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="136">
       <c r="A21" s="39" t="n"/>
       <c r="B21" s="39" t="n"/>
       <c r="C21" s="39" t="n"/>
@@ -14374,8 +14402,9 @@
       <c r="N21" s="82" t="n"/>
       <c r="O21" s="20" t="n"/>
       <c r="P21" s="20" t="n"/>
-    </row>
-    <row r="22">
+      <c r="Q21" s="209" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="136">
       <c r="A22" s="39" t="n"/>
       <c r="B22" s="39" t="n"/>
       <c r="C22" s="39" t="n"/>
@@ -14398,8 +14427,9 @@
       <c r="N22" s="94" t="n"/>
       <c r="O22" s="25" t="n"/>
       <c r="P22" s="25" t="n"/>
-    </row>
-    <row r="23">
+      <c r="Q22" s="209" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="136">
       <c r="A23" s="39" t="n"/>
       <c r="B23" s="39" t="n"/>
       <c r="C23" s="39" t="n"/>
@@ -14422,8 +14452,9 @@
       <c r="N23" s="82" t="n"/>
       <c r="O23" s="20" t="n"/>
       <c r="P23" s="20" t="n"/>
-    </row>
-    <row r="24">
+      <c r="Q23" s="209" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="136">
       <c r="A24" s="39" t="n"/>
       <c r="B24" s="39" t="n"/>
       <c r="C24" s="39" t="n"/>
@@ -14446,8 +14477,9 @@
       <c r="N24" s="94" t="n"/>
       <c r="O24" s="25" t="n"/>
       <c r="P24" s="25" t="n"/>
-    </row>
-    <row r="25">
+      <c r="Q24" s="209" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="136">
       <c r="A25" s="39" t="n"/>
       <c r="B25" s="39" t="n"/>
       <c r="C25" s="39" t="n"/>
@@ -14470,8 +14502,9 @@
       <c r="N25" s="82" t="n"/>
       <c r="O25" s="20" t="n"/>
       <c r="P25" s="20" t="n"/>
-    </row>
-    <row r="26">
+      <c r="Q25" s="209" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="136">
       <c r="A26" s="39" t="n"/>
       <c r="B26" s="39" t="n"/>
       <c r="C26" s="39" t="n"/>
@@ -14494,8 +14527,9 @@
       <c r="N26" s="94" t="n"/>
       <c r="O26" s="25" t="n"/>
       <c r="P26" s="25" t="n"/>
-    </row>
-    <row r="27">
+      <c r="Q26" s="209" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="136">
       <c r="A27" s="39" t="n"/>
       <c r="B27" s="39" t="n"/>
       <c r="C27" s="39" t="n"/>
@@ -14518,8 +14552,9 @@
       <c r="N27" s="82" t="n"/>
       <c r="O27" s="20" t="n"/>
       <c r="P27" s="20" t="n"/>
-    </row>
-    <row r="28">
+      <c r="Q27" s="209" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="136">
       <c r="A28" s="39" t="n"/>
       <c r="B28" s="39" t="n"/>
       <c r="C28" s="39" t="n"/>
@@ -14542,8 +14577,9 @@
       <c r="N28" s="94" t="n"/>
       <c r="O28" s="25" t="n"/>
       <c r="P28" s="25" t="n"/>
-    </row>
-    <row r="29">
+      <c r="Q28" s="209" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="136">
       <c r="A29" s="39" t="n"/>
       <c r="B29" s="39" t="n"/>
       <c r="C29" s="39" t="n"/>
@@ -14566,8 +14602,9 @@
       <c r="N29" s="82" t="n"/>
       <c r="O29" s="20" t="n"/>
       <c r="P29" s="20" t="n"/>
-    </row>
-    <row r="30">
+      <c r="Q29" s="209" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="136">
       <c r="A30" s="39" t="n"/>
       <c r="B30" s="39" t="n"/>
       <c r="C30" s="39" t="n"/>
@@ -14590,8 +14627,9 @@
       <c r="N30" s="94" t="n"/>
       <c r="O30" s="25" t="n"/>
       <c r="P30" s="25" t="n"/>
-    </row>
-    <row r="31">
+      <c r="Q30" s="209" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="136">
       <c r="A31" s="39" t="n"/>
       <c r="B31" s="39" t="n"/>
       <c r="C31" s="39" t="n"/>
@@ -14614,8 +14652,9 @@
       <c r="N31" s="82" t="n"/>
       <c r="O31" s="20" t="n"/>
       <c r="P31" s="20" t="n"/>
-    </row>
-    <row r="32">
+      <c r="Q31" s="209" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="136">
       <c r="A32" s="39" t="n"/>
       <c r="B32" s="39" t="n"/>
       <c r="C32" s="39" t="n"/>
@@ -14638,8 +14677,9 @@
       <c r="N32" s="94" t="n"/>
       <c r="O32" s="25" t="n"/>
       <c r="P32" s="25" t="n"/>
-    </row>
-    <row r="33">
+      <c r="Q32" s="209" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="136">
       <c r="A33" s="39" t="n"/>
       <c r="B33" s="39" t="n"/>
       <c r="C33" s="39" t="n"/>
@@ -14662,8 +14702,9 @@
       <c r="N33" s="82" t="n"/>
       <c r="O33" s="20" t="n"/>
       <c r="P33" s="20" t="n"/>
-    </row>
-    <row r="34">
+      <c r="Q33" s="209" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="136">
       <c r="A34" s="39" t="n"/>
       <c r="B34" s="39" t="n"/>
       <c r="C34" s="39" t="n"/>
@@ -14686,8 +14727,9 @@
       <c r="N34" s="94" t="n"/>
       <c r="O34" s="25" t="n"/>
       <c r="P34" s="25" t="n"/>
-    </row>
-    <row r="35">
+      <c r="Q34" s="209" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="136">
       <c r="A35" s="39" t="n"/>
       <c r="B35" s="39" t="n"/>
       <c r="C35" s="39" t="n"/>
@@ -14710,8 +14752,9 @@
       <c r="N35" s="82" t="n"/>
       <c r="O35" s="20" t="n"/>
       <c r="P35" s="20" t="n"/>
-    </row>
-    <row r="36">
+      <c r="Q35" s="209" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="136">
       <c r="A36" s="39" t="n"/>
       <c r="B36" s="39" t="n"/>
       <c r="C36" s="39" t="n"/>
@@ -14734,8 +14777,9 @@
       <c r="N36" s="94" t="n"/>
       <c r="O36" s="25" t="n"/>
       <c r="P36" s="25" t="n"/>
-    </row>
-    <row r="37">
+      <c r="Q36" s="209" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="136">
       <c r="A37" s="39" t="n"/>
       <c r="B37" s="39" t="n"/>
       <c r="C37" s="39" t="n"/>
@@ -14758,8 +14802,9 @@
       <c r="N37" s="82" t="n"/>
       <c r="O37" s="20" t="n"/>
       <c r="P37" s="20" t="n"/>
-    </row>
-    <row r="38">
+      <c r="Q37" s="209" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="136">
       <c r="A38" s="39" t="n"/>
       <c r="B38" s="39" t="n"/>
       <c r="C38" s="39" t="n"/>
@@ -14782,8 +14827,9 @@
       <c r="N38" s="94" t="n"/>
       <c r="O38" s="25" t="n"/>
       <c r="P38" s="25" t="n"/>
-    </row>
-    <row r="39">
+      <c r="Q38" s="209" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="136">
       <c r="A39" s="39" t="n"/>
       <c r="B39" s="39" t="n"/>
       <c r="C39" s="39" t="n"/>
@@ -14806,8 +14852,9 @@
       <c r="N39" s="82" t="n"/>
       <c r="O39" s="20" t="n"/>
       <c r="P39" s="20" t="n"/>
-    </row>
-    <row r="40">
+      <c r="Q39" s="209" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="136">
       <c r="A40" s="39" t="n"/>
       <c r="B40" s="39" t="n"/>
       <c r="C40" s="39" t="n"/>
@@ -14830,8 +14877,9 @@
       <c r="N40" s="94" t="n"/>
       <c r="O40" s="25" t="n"/>
       <c r="P40" s="25" t="n"/>
-    </row>
-    <row r="41">
+      <c r="Q40" s="209" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="136">
       <c r="A41" s="39" t="n"/>
       <c r="B41" s="39" t="n"/>
       <c r="C41" s="39" t="n"/>
@@ -14854,8 +14902,9 @@
       <c r="N41" s="82" t="n"/>
       <c r="O41" s="20" t="n"/>
       <c r="P41" s="20" t="n"/>
-    </row>
-    <row r="42">
+      <c r="Q41" s="209" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="136">
       <c r="A42" s="39" t="n"/>
       <c r="B42" s="39" t="n"/>
       <c r="C42" s="39" t="n"/>
@@ -14878,8 +14927,9 @@
       <c r="N42" s="94" t="n"/>
       <c r="O42" s="25" t="n"/>
       <c r="P42" s="25" t="n"/>
-    </row>
-    <row r="43">
+      <c r="Q42" s="209" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="136">
       <c r="A43" s="39" t="n"/>
       <c r="B43" s="39" t="n"/>
       <c r="C43" s="39" t="n"/>
@@ -14902,8 +14952,9 @@
       <c r="N43" s="82" t="n"/>
       <c r="O43" s="20" t="n"/>
       <c r="P43" s="20" t="n"/>
-    </row>
-    <row r="44">
+      <c r="Q43" s="209" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="136">
       <c r="A44" s="39" t="n"/>
       <c r="B44" s="39" t="n"/>
       <c r="C44" s="39" t="n"/>
@@ -14926,8 +14977,9 @@
       <c r="N44" s="94" t="n"/>
       <c r="O44" s="25" t="n"/>
       <c r="P44" s="25" t="n"/>
-    </row>
-    <row r="45">
+      <c r="Q44" s="209" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="136">
       <c r="A45" s="39" t="n"/>
       <c r="B45" s="39" t="n"/>
       <c r="C45" s="39" t="n"/>
@@ -14950,8 +15002,9 @@
       <c r="N45" s="82" t="n"/>
       <c r="O45" s="20" t="n"/>
       <c r="P45" s="20" t="n"/>
-    </row>
-    <row r="46">
+      <c r="Q45" s="209" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="136">
       <c r="A46" s="39" t="n"/>
       <c r="B46" s="39" t="n"/>
       <c r="C46" s="39" t="n"/>
@@ -14974,8 +15027,9 @@
       <c r="N46" s="94" t="n"/>
       <c r="O46" s="25" t="n"/>
       <c r="P46" s="25" t="n"/>
-    </row>
-    <row r="47">
+      <c r="Q46" s="209" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="136">
       <c r="A47" s="39" t="n"/>
       <c r="B47" s="39" t="n"/>
       <c r="C47" s="39" t="n"/>
@@ -14998,8 +15052,9 @@
       <c r="N47" s="82" t="n"/>
       <c r="O47" s="20" t="n"/>
       <c r="P47" s="20" t="n"/>
-    </row>
-    <row r="48">
+      <c r="Q47" s="209" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="136">
       <c r="A48" s="39" t="n"/>
       <c r="B48" s="39" t="n"/>
       <c r="C48" s="39" t="n"/>
@@ -15022,8 +15077,9 @@
       <c r="N48" s="94" t="n"/>
       <c r="O48" s="25" t="n"/>
       <c r="P48" s="25" t="n"/>
-    </row>
-    <row r="49">
+      <c r="Q48" s="209" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="136">
       <c r="A49" s="39" t="n"/>
       <c r="B49" s="39" t="n"/>
       <c r="C49" s="39" t="n"/>
@@ -15046,6 +15102,7 @@
       <c r="N49" s="82" t="n"/>
       <c r="O49" s="20" t="n"/>
       <c r="P49" s="20" t="n"/>
+      <c r="Q49" s="209" t="n"/>
     </row>
     <row r="51" ht="15.5" customHeight="1" s="136">
       <c r="A51" s="104" t="inlineStr">
@@ -15120,7 +15177,7 @@
     <row r="54" ht="32" customHeight="1" s="136">
       <c r="A54" s="132" t="inlineStr">
         <is>
-          <t>Team Score = 50% × average touch weighted score  +  30% × (Journey Outcome ÷ 5)  +  20% × (Continuity &amp; Handoffs ÷ 5).  Outcome and Continuity are evaluator-judged 0-5 — anchors on the Multi-Touch Guide sheet. The Team Score rates the CHAIN; it feeds team coaching and recognition, never individual discipline.</t>
+          <t>Team Score  =  20% × Level 1 avg touch  +  30% × Level 2 avg touch  +  30% × (Journey Outcome ÷ 5)  +  20% × (Continuity of Support ÷ 5)   │   Level 2 touches carry a higher weight in the team aggregate.</t>
         </is>
       </c>
       <c r="B54" s="86" t="n"/>
@@ -15153,7 +15210,7 @@
       </c>
       <c r="D55" s="38" t="inlineStr">
         <is>
-          <t>Avg Touch %</t>
+          <t>Avg Touch % (ref)</t>
         </is>
       </c>
       <c r="E55" s="38" t="inlineStr">
@@ -15201,7 +15258,7 @@
       <c r="E56" s="102" t="n"/>
       <c r="F56" s="102" t="n"/>
       <c r="G56" s="46">
-        <f>IF(OR(A56="",D56="",E56="",F56=""),"",0.5*D56+0.3*(E56/5)+0.2*(F56/5))</f>
+        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0)+0.3*(E56/5)+0.2*(F56/5),""))</f>
         <v/>
       </c>
       <c r="H56" s="25">
@@ -15229,7 +15286,7 @@
       <c r="E57" s="102" t="n"/>
       <c r="F57" s="102" t="n"/>
       <c r="G57" s="46">
-        <f>IF(OR(A57="",D57="",E57="",F57=""),"",0.5*D57+0.3*(E57/5)+0.2*(F57/5))</f>
+        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0)+0.3*(E57/5)+0.2*(F57/5),""))</f>
         <v/>
       </c>
       <c r="H57" s="25">
@@ -15257,7 +15314,7 @@
       <c r="E58" s="102" t="n"/>
       <c r="F58" s="102" t="n"/>
       <c r="G58" s="47">
-        <f>IF(OR(A58="",D58="",E58="",F58=""),"",0.5*D58+0.3*(E58/5)+0.2*(F58/5))</f>
+        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0)+0.3*(E58/5)+0.2*(F58/5),""))</f>
         <v/>
       </c>
       <c r="H58" s="20">
@@ -15285,7 +15342,7 @@
       <c r="E59" s="102" t="n"/>
       <c r="F59" s="102" t="n"/>
       <c r="G59" s="46">
-        <f>IF(OR(A59="",D59="",E59="",F59=""),"",0.5*D59+0.3*(E59/5)+0.2*(F59/5))</f>
+        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0)+0.3*(E59/5)+0.2*(F59/5),""))</f>
         <v/>
       </c>
       <c r="H59" s="25">
@@ -15326,8 +15383,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
@@ -15425,7 +15482,7 @@
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="E5:K5 E6:K6 E7:K7 E8:K8 E9:K9 E10:K10 E11:K11 E12:K12 E13:K13 E14:K14 E15:K15 E16:K16 E17:K17 E18:K18 E19:K19 E20:K20 E21:K21 E22:K22 E23:K23 E24:K24 E25:K25 E26:K26 E27:K27 E28:K28 E29:K29 E30:K30 E31:K31 E32:K32 E33:K33 E34:K34 E35:K35 E36:K36 E37:K37 E38:K38 E39:K39 E40:K40 E41:K41 E42:K42 E43:K43 E44:K44 E45:K45 E46:K46 E47:K47 E48:K48 E49:K49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5." type="whole">
       <formula1>0</formula1>
       <formula2>5</formula2>
@@ -15440,6 +15497,9 @@
     <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole">
       <formula1>0</formula1>
       <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="Q5:Q49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Please select Level 1 or Level 2." promptTitle="Agent Level" prompt="Level 1 = front-line support.  Level 2 = senior / escalation support." type="list">
+      <formula1>"Level 1,Level 2"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Case Tracker: fall back to original formula for single-level cases
Team Score now uses L1/L2 split (20pct L1 + 30pct L2) only when both
levels appear in the same case. All-L1 or all-L2 cases use the original
0.5 x Avg Touch formula unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -15258,7 +15258,7 @@
       <c r="E56" s="102" t="n"/>
       <c r="F56" s="102" t="n"/>
       <c r="G56" s="46">
-        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0)+0.3*(E56/5)+0.2*(F56/5),""))</f>
+        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(E56/5)+0.2*(F56/5),""))</f>
         <v/>
       </c>
       <c r="H56" s="25">
@@ -15286,7 +15286,7 @@
       <c r="E57" s="102" t="n"/>
       <c r="F57" s="102" t="n"/>
       <c r="G57" s="46">
-        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0)+0.3*(E57/5)+0.2*(F57/5),""))</f>
+        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(E57/5)+0.2*(F57/5),""))</f>
         <v/>
       </c>
       <c r="H57" s="25">
@@ -15314,7 +15314,7 @@
       <c r="E58" s="102" t="n"/>
       <c r="F58" s="102" t="n"/>
       <c r="G58" s="47">
-        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0)+0.3*(E58/5)+0.2*(F58/5),""))</f>
+        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(E58/5)+0.2*(F58/5),""))</f>
         <v/>
       </c>
       <c r="H58" s="20">
@@ -15342,7 +15342,7 @@
       <c r="E59" s="102" t="n"/>
       <c r="F59" s="102" t="n"/>
       <c r="G59" s="46">
-        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0)+0.3*(E59/5)+0.2*(F59/5),""))</f>
+        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(E59/5)+0.2*(F59/5),""))</f>
         <v/>
       </c>
       <c r="H59" s="25">
@@ -15383,8 +15383,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Clear Case Tracker entries for clean template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -530,7 +530,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -823,11 +823,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="218">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1446,6 +1490,8 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9558,6 +9604,10 @@
           <t>TEAM SCORE — JOURNEY OUTCOME &amp; CONTINUITY OF SUPPORT   ·   Used in Case Tracker multi-touch scoring</t>
         </is>
       </c>
+      <c r="B145" s="218" t="n"/>
+      <c r="C145" s="218" t="n"/>
+      <c r="D145" s="218" t="n"/>
+      <c r="E145" s="219" t="n"/>
     </row>
     <row r="146" ht="16" customHeight="1" s="175">
       <c r="A146" s="193" t="inlineStr">
@@ -14402,38 +14452,16 @@
     </row>
     <row r="5" ht="40" customHeight="1" s="175">
       <c r="A5" s="39" t="n"/>
-      <c r="B5" s="39" t="n">
-        <v>12345678</v>
-      </c>
-      <c r="C5" s="39" t="inlineStr">
-        <is>
-          <t>Agent 1</t>
-        </is>
-      </c>
-      <c r="D5" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="H5" s="39" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="K5" s="39" t="n">
-        <v>5</v>
-      </c>
+      <c r="B5" s="39" t="n"/>
+      <c r="C5" s="39" t="n"/>
+      <c r="D5" s="39" t="n"/>
+      <c r="E5" s="39" t="n"/>
+      <c r="F5" s="39" t="n"/>
+      <c r="G5" s="39" t="n"/>
+      <c r="H5" s="39" t="n"/>
+      <c r="I5" s="39" t="n"/>
+      <c r="J5" s="39" t="n"/>
+      <c r="K5" s="39" t="n"/>
       <c r="L5" s="40">
         <f>IF((COUNT(E5)+COUNT(F5)+COUNT(G5)+COUNT(H5)+COUNT(I5)+COUNT(J5)+COUNT(K5))=0,"",IFERROR(E5/5*0.3,0)+IFERROR(F5/5*0.2,0)+IFERROR(G5/5*0.15,0)+IFERROR(H5/5*0.15,0)+IFERROR(I5/5*0.1,0)+IFERROR(J5/5*0.05,0)+IFERROR(K5/5*0.05,0))</f>
         <v/>
@@ -14445,46 +14473,20 @@
       <c r="N5" s="8" t="n"/>
       <c r="O5" s="20" t="n"/>
       <c r="P5" s="20" t="n"/>
-      <c r="Q5" s="114" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
+      <c r="Q5" s="114" t="n"/>
     </row>
     <row r="6" ht="40" customHeight="1" s="175">
       <c r="A6" s="39" t="n"/>
-      <c r="B6" s="39" t="n">
-        <v>12345678</v>
-      </c>
-      <c r="C6" s="39" t="inlineStr">
-        <is>
-          <t>Agent 2</t>
-        </is>
-      </c>
-      <c r="D6" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="39" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="39" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="K6" s="39" t="n">
-        <v>4</v>
-      </c>
+      <c r="B6" s="39" t="n"/>
+      <c r="C6" s="39" t="n"/>
+      <c r="D6" s="39" t="n"/>
+      <c r="E6" s="39" t="n"/>
+      <c r="F6" s="39" t="n"/>
+      <c r="G6" s="39" t="n"/>
+      <c r="H6" s="39" t="n"/>
+      <c r="I6" s="39" t="n"/>
+      <c r="J6" s="39" t="n"/>
+      <c r="K6" s="39" t="n"/>
       <c r="L6" s="41">
         <f>IF((COUNT(E6)+COUNT(F6)+COUNT(G6)+COUNT(H6)+COUNT(I6)+COUNT(J6)+COUNT(K6))=0,"",IFERROR(E6/5*0.3,0)+IFERROR(F6/5*0.2,0)+IFERROR(G6/5*0.15,0)+IFERROR(H6/5*0.15,0)+IFERROR(I6/5*0.1,0)+IFERROR(J6/5*0.05,0)+IFERROR(K6/5*0.05,0))</f>
         <v/>
@@ -14496,46 +14498,20 @@
       <c r="N6" s="10" t="n"/>
       <c r="O6" s="25" t="n"/>
       <c r="P6" s="25" t="n"/>
-      <c r="Q6" s="114" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
+      <c r="Q6" s="114" t="n"/>
     </row>
     <row r="7" ht="40" customHeight="1" s="175">
       <c r="A7" s="39" t="n"/>
-      <c r="B7" s="39" t="n">
-        <v>12345678</v>
-      </c>
-      <c r="C7" s="39" t="inlineStr">
-        <is>
-          <t>Agent 3</t>
-        </is>
-      </c>
-      <c r="D7" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="G7" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="H7" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="39" t="n">
-        <v>4</v>
-      </c>
+      <c r="B7" s="39" t="n"/>
+      <c r="C7" s="39" t="n"/>
+      <c r="D7" s="39" t="n"/>
+      <c r="E7" s="39" t="n"/>
+      <c r="F7" s="39" t="n"/>
+      <c r="G7" s="39" t="n"/>
+      <c r="H7" s="39" t="n"/>
+      <c r="I7" s="39" t="n"/>
+      <c r="J7" s="39" t="n"/>
+      <c r="K7" s="39" t="n"/>
       <c r="L7" s="40">
         <f>IF((COUNT(E7)+COUNT(F7)+COUNT(G7)+COUNT(H7)+COUNT(I7)+COUNT(J7)+COUNT(K7))=0,"",IFERROR(E7/5*0.3,0)+IFERROR(F7/5*0.2,0)+IFERROR(G7/5*0.15,0)+IFERROR(H7/5*0.15,0)+IFERROR(I7/5*0.1,0)+IFERROR(J7/5*0.05,0)+IFERROR(K7/5*0.05,0))</f>
         <v/>
@@ -14547,46 +14523,20 @@
       <c r="N7" s="8" t="n"/>
       <c r="O7" s="20" t="n"/>
       <c r="P7" s="20" t="n"/>
-      <c r="Q7" s="114" t="inlineStr">
-        <is>
-          <t>Level 1</t>
-        </is>
-      </c>
+      <c r="Q7" s="114" t="n"/>
     </row>
     <row r="8" ht="40" customHeight="1" s="175">
       <c r="A8" s="39" t="n"/>
-      <c r="B8" s="39" t="n">
-        <v>12345678</v>
-      </c>
-      <c r="C8" s="39" t="inlineStr">
-        <is>
-          <t>Agent 4</t>
-        </is>
-      </c>
-      <c r="D8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="39" t="n">
-        <v>2</v>
-      </c>
-      <c r="I8" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="39" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" s="39" t="n">
-        <v>3</v>
-      </c>
+      <c r="B8" s="39" t="n"/>
+      <c r="C8" s="39" t="n"/>
+      <c r="D8" s="39" t="n"/>
+      <c r="E8" s="39" t="n"/>
+      <c r="F8" s="39" t="n"/>
+      <c r="G8" s="39" t="n"/>
+      <c r="H8" s="39" t="n"/>
+      <c r="I8" s="39" t="n"/>
+      <c r="J8" s="39" t="n"/>
+      <c r="K8" s="39" t="n"/>
       <c r="L8" s="41">
         <f>IF((COUNT(E8)+COUNT(F8)+COUNT(G8)+COUNT(H8)+COUNT(I8)+COUNT(J8)+COUNT(K8))=0,"",IFERROR(E8/5*0.3,0)+IFERROR(F8/5*0.2,0)+IFERROR(G8/5*0.15,0)+IFERROR(H8/5*0.15,0)+IFERROR(I8/5*0.1,0)+IFERROR(J8/5*0.05,0)+IFERROR(K8/5*0.05,0))</f>
         <v/>
@@ -14598,11 +14548,7 @@
       <c r="N8" s="10" t="n"/>
       <c r="O8" s="25" t="n"/>
       <c r="P8" s="25" t="n"/>
-      <c r="Q8" s="114" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
+      <c r="Q8" s="114" t="n"/>
     </row>
     <row r="9" ht="40" customHeight="1" s="175">
       <c r="A9" s="39" t="n"/>
@@ -15770,9 +15716,7 @@
       <c r="N55" s="120" t="n"/>
     </row>
     <row r="56" ht="48" customHeight="1" s="175">
-      <c r="A56" s="189" t="n">
-        <v>12345678</v>
-      </c>
+      <c r="A56" s="189" t="n"/>
       <c r="B56" s="122" t="n"/>
       <c r="C56" s="25">
         <f>IF(A56="","",COUNTIF(B5:B49,A56))</f>
@@ -15782,12 +15726,8 @@
         <f>IF(A56="","",IFERROR(AVERAGEIF(B5:B49,A56,L5:L49),""))</f>
         <v/>
       </c>
-      <c r="E56" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F56" s="9" t="n">
-        <v>5</v>
-      </c>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="9" t="n"/>
       <c r="G56" s="116">
         <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(E56/5)+0.2*(F56/5),""))</f>
         <v/>
@@ -15914,8 +15854,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Implement Option B: dropdown selectors for Journey Outcome and Continuity
- Lists sheet: added Journey Outcome (col H) and Continuity (col I)
  option lists, each with 6 descriptive anchor-based options (0-5)
- Case Tracker: replaced free 0-5 inputs with list DVs referencing
  Lists sheet; options format '5 - description' for auto-scoring
- Team Score formula updated to extract numeric score from selected
  text via VALUE(LEFT(cell,1))
- Column headers updated: Outcome (0-5) and Continuity (0-5) renamed
  to Journey Outcome and Continuity of Support

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="49">
+  <fonts count="50">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -350,6 +350,10 @@
     <font>
       <color rgb="002E4057"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="36">
@@ -871,7 +875,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="221">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1492,6 +1496,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15686,12 +15691,12 @@
       </c>
       <c r="E55" s="38" t="inlineStr">
         <is>
-          <t>Outcome (0-5)</t>
+          <t>Journey Outcome</t>
         </is>
       </c>
       <c r="F55" s="38" t="inlineStr">
         <is>
-          <t>Continuity (0-5)</t>
+          <t>Continuity of Support</t>
         </is>
       </c>
       <c r="G55" s="38" t="inlineStr">
@@ -15729,7 +15734,7 @@
       <c r="E56" s="9" t="n"/>
       <c r="F56" s="9" t="n"/>
       <c r="G56" s="116">
-        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(E56/5)+0.2*(F56/5),""))</f>
+        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(IFERROR(VALUE(LEFT(E56,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F56,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H56" s="25">
@@ -15757,7 +15762,7 @@
       <c r="E57" s="9" t="n"/>
       <c r="F57" s="9" t="n"/>
       <c r="G57" s="116">
-        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(E57/5)+0.2*(F57/5),""))</f>
+        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(IFERROR(VALUE(LEFT(E57,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F57,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H57" s="25">
@@ -15785,7 +15790,7 @@
       <c r="E58" s="9" t="n"/>
       <c r="F58" s="9" t="n"/>
       <c r="G58" s="117">
-        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(E58/5)+0.2*(F58/5),""))</f>
+        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(IFERROR(VALUE(LEFT(E58,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F58,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H58" s="20">
@@ -15813,7 +15818,7 @@
       <c r="E59" s="9" t="n"/>
       <c r="F59" s="9" t="n"/>
       <c r="G59" s="116">
-        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(E59/5)+0.2*(F59/5),""))</f>
+        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(IFERROR(VALUE(LEFT(E59,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F59,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H59" s="25">
@@ -15854,8 +15859,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>
@@ -15968,13 +15973,11 @@
     <dataValidation sqref="Q5:Q49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Please select Level 1 or Level 2." promptTitle="Agent Level" prompt="Level 1 = front-line support.  Level 2 = senior / escalation support." type="list">
       <formula1>"Level 1,Level 2"</formula1>
     </dataValidation>
-    <dataValidation sqref="E56:E59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Out of range" error="Enter a whole number between 0 and 5." promptTitle="Journey Outcome (0–5)" prompt="5 = Resolved &amp; confirmed  4 = Strong path: RMA / escalation / limitation explained  3 = Partial — next step exists but issue open  2 = Minimal progress  1 = No meaningful progress  0 = Worsened or contradictory guidance" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>5</formula2>
+    <dataValidation sqref="E56:E59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid selection" error="Please choose from the dropdown list." promptTitle="Journey Outcome" prompt="Select the option that best describes the overall resolution achieved across all touches." type="list">
+      <formula1>Lists!$H$2:$H$7</formula1>
     </dataValidation>
-    <dataValidation sqref="F56:F59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Out of range" error="Enter a whole number between 0 and 5." promptTitle="Continuity of Support (0–5)" prompt="5 = Full context, no repeated questions, statuses always truthful  4 = Minor gaps, no customer impact  3 = Customer re-explained parts of issue  2 = Significant context loss across touches  1 = Near-zero continuity  0 = Contradictory guidance or breakdown" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>5</formula2>
+    <dataValidation sqref="F56:F59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid selection" error="Please choose from the dropdown list." promptTitle="Continuity of Support" prompt="Select the option that best describes how well context and ownership were maintained across handoffs." type="list">
+      <formula1>Lists!$I$2:$I$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15991,6 +15994,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="34" customWidth="1" style="175" min="1" max="8"/>
+    <col width="52" customWidth="1" style="175" min="8" max="8"/>
+    <col width="52" customWidth="1" style="175" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16029,6 +16034,16 @@
           <t>System / tooling driver</t>
         </is>
       </c>
+      <c r="H1" s="220" t="inlineStr">
+        <is>
+          <t>Journey Outcome</t>
+        </is>
+      </c>
+      <c r="I1" s="220" t="inlineStr">
+        <is>
+          <t>Continuity of Support</t>
+        </is>
+      </c>
       <c r="J1" t="inlineStr">
         <is>
           <t>Dropdown option source for the Scoring Form (Section 8 + Outcome). Unhide to edit options.</t>
@@ -16071,6 +16086,16 @@
           <t>None</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>5 — Fully resolved and confirmed</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5 — Full context preserved, no repeated questions</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -16108,6 +16133,16 @@
           <t>Public – Website</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>4 — Strong path: RMA / escalation / limitation explained</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>4 — Minor gap at one handoff, no customer impact</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16145,6 +16180,16 @@
           <t>Public – App/Cloud</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3 — Partial — next step exists, issue still open</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>3 — Customer re-explained parts of the issue</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -16182,6 +16227,16 @@
           <t>Public – IVR</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2 — Minimal progress despite multiple touches</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2 — Significant context loss across touches</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -16214,6 +16269,16 @@
           <t>Internal – Salesforce/CRM</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1 — No meaningful progress</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1 — Near-zero continuity, agents restarted fresh</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16239,6 +16304,16 @@
       <c r="G7" t="inlineStr">
         <is>
           <t>Internal – CSC</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0 — Worsened or contradictory guidance</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0 — Contradictory guidance, complete breakdown</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove blank row 75 from Customer Ownership section
Leftover empty row from when the 'Next actions were documented'
indicator was removed as redundant with Documentation section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -875,7 +875,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="221">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1497,6 +1497,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3892,7 +3931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G189"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="4" customWidth="1" style="175" min="1" max="1"/>
@@ -4925,726 +4964,740 @@
       <c r="F74" s="122" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1" s="175">
-      <c r="B75" s="76" t="n"/>
-      <c r="C75" s="105" t="n"/>
-      <c r="D75" s="147" t="n"/>
+      <c r="B75" s="143" t="inlineStr">
+        <is>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
+        </is>
+      </c>
+      <c r="C75" s="221" t="n"/>
+      <c r="D75" s="143" t="n"/>
       <c r="E75" s="126" t="n"/>
       <c r="F75" s="122" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1" s="175">
-      <c r="B76" s="106" t="inlineStr">
-        <is>
-          <t>Clearly set customer expectations for next steps and realistic timelines</t>
-        </is>
-      </c>
-      <c r="C76" s="105" t="n"/>
-      <c r="D76" s="143" t="n"/>
+      <c r="B76" s="222" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C76" s="221" t="n"/>
+      <c r="D76" s="222" t="n"/>
       <c r="E76" s="126" t="n"/>
       <c r="F76" s="122" t="n"/>
     </row>
     <row r="77" ht="28" customHeight="1" s="175">
-      <c r="B77" s="76" t="inlineStr">
-        <is>
-          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
-        </is>
-      </c>
-      <c r="C77" s="105" t="n"/>
-      <c r="D77" s="147" t="n"/>
+      <c r="B77" s="223" t="inlineStr">
+        <is>
+          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
+        </is>
+      </c>
+      <c r="C77" s="126" t="n"/>
+      <c r="D77" s="126" t="n"/>
       <c r="E77" s="126" t="n"/>
       <c r="F77" s="122" t="n"/>
     </row>
     <row r="78" ht="28" customHeight="1" s="175">
-      <c r="B78" s="137" t="inlineStr">
-        <is>
-          <t>⚠ Automatic deductions: no documented follow-up after disconnect; unclear next steps; passing responsibility without context; failure to complete promised actions; missed or late callbacks without proactive renegotiation.</t>
-        </is>
-      </c>
-      <c r="C78" s="126" t="n"/>
-      <c r="D78" s="126" t="n"/>
+      <c r="B78" s="224" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C78" s="225">
+        <f>IF((COUNTIF(C73:C76,"Met")+COUNTIF(C73:C76,"Partial")+COUNTIF(C73:C76,"Missed"))=0,"",ROUND((COUNTIF(C73:C76,"Met")*5+COUNTIF(C73:C76,"Partial")*2.5)/(COUNTIF(C73:C76,"Met")+COUNTIF(C73:C76,"Partial")+COUNTIF(C73:C76,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D78" s="146" t="n"/>
       <c r="E78" s="126" t="n"/>
       <c r="F78" s="122" t="n"/>
     </row>
-    <row r="79" ht="28" customHeight="1" s="175">
-      <c r="B79" s="107" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C79" s="108">
-        <f>IF((COUNTIF(C73:C77,"Met")+COUNTIF(C73:C77,"Partial")+COUNTIF(C73:C77,"Missed"))=0,"",ROUND((COUNTIF(C73:C77,"Met")*5+COUNTIF(C73:C77,"Partial")*2.5)/(COUNTIF(C73:C77,"Met")+COUNTIF(C73:C77,"Partial")+COUNTIF(C73:C77,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D79" s="146" t="n"/>
+    <row r="79" ht="24" customHeight="1" s="175">
+      <c r="B79" s="226" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C79" s="227" t="n"/>
+      <c r="D79" s="161">
+        <f>IF(IF(C79="",C78,C79)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C79="",C78,C79)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E79" s="126" t="n"/>
       <c r="F79" s="122" t="n"/>
     </row>
-    <row r="80" ht="24" customHeight="1" s="175">
-      <c r="B80" s="79" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C80" s="109" t="n"/>
-      <c r="D80" s="161">
-        <f>IF(IF(C80="",C79,C80)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C80="",C79,C80)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="80" ht="36" customHeight="1" s="175">
+      <c r="B80" s="226" t="inlineStr">
+        <is>
+          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
+        </is>
+      </c>
+      <c r="C80" s="228" t="n"/>
+      <c r="D80" s="126" t="n"/>
       <c r="E80" s="126" t="n"/>
       <c r="F80" s="122" t="n"/>
     </row>
-    <row r="81" ht="36" customHeight="1" s="175">
-      <c r="B81" s="79" t="inlineStr">
-        <is>
-          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
-        </is>
-      </c>
-      <c r="C81" s="145" t="n"/>
-      <c r="D81" s="126" t="n"/>
-      <c r="E81" s="126" t="n"/>
-      <c r="F81" s="122" t="n"/>
-    </row>
-    <row r="82" ht="18" customHeight="1" s="175">
-      <c r="B82" s="118" t="inlineStr">
+    <row r="81" ht="18" customHeight="1" s="175">
+      <c r="B81" s="118" t="inlineStr">
         <is>
           <t>5. ESCALATION JUDGMENT</t>
         </is>
       </c>
-      <c r="C82" s="119" t="n"/>
-      <c r="D82" s="119" t="n"/>
-      <c r="E82" s="120" t="n"/>
-      <c r="F82" s="6" t="inlineStr">
+      <c r="C81" s="119" t="n"/>
+      <c r="D81" s="119" t="n"/>
+      <c r="E81" s="120" t="n"/>
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <t>Weight: 10%</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="28" customHeight="1" s="175">
-      <c r="B83" s="148" t="inlineStr">
+    <row r="82" ht="28" customHeight="1" s="175">
+      <c r="B82" s="148" t="inlineStr">
         <is>
           <t>Objective: Determine whether escalation decisions were appropriate — including UPWARD escalations the customer requested (management, complaint, legal). Mark all N.A. if no escalation was involved and none was warranted.</t>
         </is>
       </c>
-      <c r="C83" s="126" t="n"/>
-      <c r="D83" s="126" t="n"/>
+      <c r="C82" s="126" t="n"/>
+      <c r="D82" s="126" t="n"/>
+      <c r="E82" s="126" t="n"/>
+      <c r="F82" s="122" t="n"/>
+    </row>
+    <row r="83" ht="18" customHeight="1" s="175">
+      <c r="B83" s="229" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C83" s="230" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D83" s="229" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E83" s="126" t="n"/>
       <c r="F83" s="122" t="n"/>
     </row>
-    <row r="84" ht="18" customHeight="1" s="175">
-      <c r="B84" s="75" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C84" s="104" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D84" s="152" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+    <row r="84" ht="28" customHeight="1" s="175">
+      <c r="B84" s="222" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before escalating</t>
+        </is>
+      </c>
+      <c r="C84" s="221" t="n"/>
+      <c r="D84" s="222" t="n"/>
       <c r="E84" s="126" t="n"/>
       <c r="F84" s="122" t="n"/>
     </row>
     <row r="85" ht="28" customHeight="1" s="175">
-      <c r="B85" s="76" t="inlineStr">
-        <is>
-          <t>Completed reasonable troubleshooting before escalating</t>
-        </is>
-      </c>
-      <c r="C85" s="105" t="n"/>
-      <c r="D85" s="147" t="n"/>
+      <c r="B85" s="143" t="inlineStr">
+        <is>
+          <t>Identified a valid reason to escalate</t>
+        </is>
+      </c>
+      <c r="C85" s="221" t="n"/>
+      <c r="D85" s="143" t="n"/>
       <c r="E85" s="126" t="n"/>
       <c r="F85" s="122" t="n"/>
     </row>
     <row r="86" ht="28" customHeight="1" s="175">
-      <c r="B86" s="106" t="inlineStr">
-        <is>
-          <t>Identified a valid reason to escalate</t>
-        </is>
-      </c>
-      <c r="C86" s="105" t="n"/>
-      <c r="D86" s="143" t="n"/>
+      <c r="B86" s="222" t="inlineStr">
+        <is>
+          <t>Provided complete escalation details using the correct escalation path</t>
+        </is>
+      </c>
+      <c r="C86" s="221" t="n"/>
+      <c r="D86" s="222" t="n"/>
       <c r="E86" s="126" t="n"/>
       <c r="F86" s="122" t="n"/>
     </row>
     <row r="87" ht="28" customHeight="1" s="175">
-      <c r="B87" s="76" t="inlineStr">
-        <is>
-          <t>Provided complete escalation details using the correct escalation path</t>
-        </is>
-      </c>
-      <c r="C87" s="105" t="n"/>
-      <c r="D87" s="147" t="n"/>
+      <c r="B87" s="222" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next.</t>
+        </is>
+      </c>
+      <c r="C87" s="221" t="n"/>
+      <c r="D87" s="222" t="n"/>
       <c r="E87" s="126" t="n"/>
       <c r="F87" s="122" t="n"/>
     </row>
     <row r="88" ht="28" customHeight="1" s="175">
-      <c r="B88" s="76" t="inlineStr">
-        <is>
-          <t>Clearly explained why escalation was necessary and what would happen next.</t>
-        </is>
-      </c>
-      <c r="C88" s="105" t="n"/>
-      <c r="D88" s="147" t="n"/>
+      <c r="B88" s="223" t="inlineStr">
+        <is>
+          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
+        </is>
+      </c>
+      <c r="C88" s="126" t="n"/>
+      <c r="D88" s="126" t="n"/>
       <c r="E88" s="126" t="n"/>
       <c r="F88" s="122" t="n"/>
     </row>
     <row r="89" ht="28" customHeight="1" s="175">
-      <c r="B89" s="137" t="inlineStr">
-        <is>
-          <t>⚠ Low score: premature, avoidable, poorly documented, used as a substitute for troubleshooting — or a warranted escalation (incl. a customer's management request) that was NOT made.</t>
-        </is>
-      </c>
-      <c r="C89" s="126" t="n"/>
-      <c r="D89" s="126" t="n"/>
+      <c r="B89" s="224" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C89" s="225">
+        <f>IF((COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed"))=0,"",ROUND((COUNTIF(C84:C87,"Met")*5+COUNTIF(C84:C87,"Partial")*2.5)/(COUNTIF(C84:C87,"Met")+COUNTIF(C84:C87,"Partial")+COUNTIF(C84:C87,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D89" s="146" t="n"/>
       <c r="E89" s="126" t="n"/>
       <c r="F89" s="122" t="n"/>
     </row>
-    <row r="90" ht="28" customHeight="1" s="175">
-      <c r="B90" s="107" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C90" s="108">
-        <f>IF((COUNTIF(C85:C88,"Met")+COUNTIF(C85:C88,"Partial")+COUNTIF(C85:C88,"Missed"))=0,"",ROUND((COUNTIF(C85:C88,"Met")*5+COUNTIF(C85:C88,"Partial")*2.5)/(COUNTIF(C85:C88,"Met")+COUNTIF(C85:C88,"Partial")+COUNTIF(C85:C88,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D90" s="146" t="n"/>
+    <row r="90" ht="24" customHeight="1" s="175">
+      <c r="B90" s="226" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C90" s="227" t="n"/>
+      <c r="D90" s="161">
+        <f>IF(IF(C90="",C89,C90)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C90="",C89,C90)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E90" s="126" t="n"/>
       <c r="F90" s="122" t="n"/>
     </row>
-    <row r="91" ht="24" customHeight="1" s="175">
-      <c r="B91" s="79" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C91" s="109" t="n"/>
-      <c r="D91" s="161">
-        <f>IF(IF(C91="",C90,C91)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C91="",C90,C91)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="91" ht="36" customHeight="1" s="175">
+      <c r="B91" s="226" t="inlineStr">
+        <is>
+          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
+        </is>
+      </c>
+      <c r="C91" s="228" t="n"/>
+      <c r="D91" s="126" t="n"/>
       <c r="E91" s="126" t="n"/>
       <c r="F91" s="122" t="n"/>
     </row>
-    <row r="92" ht="36" customHeight="1" s="175">
-      <c r="B92" s="79" t="inlineStr">
-        <is>
-          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
-        </is>
-      </c>
-      <c r="C92" s="145" t="n"/>
-      <c r="D92" s="126" t="n"/>
-      <c r="E92" s="126" t="n"/>
-      <c r="F92" s="122" t="n"/>
+    <row r="92" ht="20" customHeight="1" s="175">
+      <c r="B92" s="118" t="inlineStr">
+        <is>
+          <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
+        </is>
+      </c>
+      <c r="C92" s="119" t="n"/>
+      <c r="D92" s="119" t="n"/>
+      <c r="E92" s="119" t="n"/>
+      <c r="F92" s="120" t="n"/>
     </row>
     <row r="93" ht="20" customHeight="1" s="175">
-      <c r="B93" s="118" t="inlineStr">
-        <is>
-          <t>ESCALATION FOLLOW-UP   ·   Complete only if an escalation was submitted</t>
-        </is>
-      </c>
-      <c r="C93" s="119" t="n"/>
-      <c r="D93" s="119" t="n"/>
-      <c r="E93" s="119" t="n"/>
-      <c r="F93" s="120" t="n"/>
-    </row>
-    <row r="94" ht="20" customHeight="1" s="175">
-      <c r="B94" s="155" t="inlineStr">
+      <c r="B93" s="226" t="inlineStr">
         <is>
           <t>What did the receiving agent / Level 2 do to resolve or advance this case?</t>
         </is>
       </c>
-      <c r="C94" s="156" t="n"/>
-      <c r="D94" s="77" t="n"/>
+      <c r="C93" s="156" t="n"/>
+      <c r="D93" s="146" t="n"/>
+      <c r="F93" s="6" t="n"/>
+    </row>
+    <row r="94" ht="45" customHeight="1" s="175">
+      <c r="B94" s="157" t="n"/>
+      <c r="C94" s="158" t="n"/>
+      <c r="D94" s="161" t="n"/>
       <c r="F94" s="6" t="n"/>
     </row>
-    <row r="95" ht="45" customHeight="1" s="175">
-      <c r="B95" s="157" t="n"/>
-      <c r="C95" s="158" t="n"/>
-      <c r="D95" s="78" t="n"/>
-    </row>
-    <row r="96" ht="18" customHeight="1" s="175">
-      <c r="B96" s="118" t="inlineStr">
+    <row r="95" ht="18" customHeight="1" s="175">
+      <c r="B95" s="118" t="inlineStr">
         <is>
           <t>L1 learning points from this escalation outcome</t>
         </is>
       </c>
-      <c r="C96" s="119" t="n"/>
-      <c r="D96" s="119" t="n"/>
-      <c r="E96" s="119" t="n"/>
-      <c r="F96" s="120" t="n"/>
+      <c r="C95" s="119" t="n"/>
+      <c r="D95" s="119" t="n"/>
+      <c r="E95" s="119" t="n"/>
+      <c r="F95" s="120" t="n"/>
+    </row>
+    <row r="96" ht="28" customHeight="1" s="175">
+      <c r="B96" s="226" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C96" s="221" t="n"/>
+      <c r="D96" s="126" t="n"/>
+      <c r="E96" s="126" t="n"/>
+      <c r="F96" s="122" t="n"/>
     </row>
     <row r="97" ht="28" customHeight="1" s="175">
-      <c r="B97" s="79" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C97" s="166" t="n"/>
+      <c r="B97" s="226" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C97" s="221" t="n"/>
       <c r="D97" s="126" t="n"/>
       <c r="E97" s="126" t="n"/>
       <c r="F97" s="122" t="n"/>
     </row>
     <row r="98" ht="28" customHeight="1" s="175">
-      <c r="B98" s="79" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C98" s="166" t="n"/>
+      <c r="B98" s="226" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C98" s="221" t="n"/>
       <c r="D98" s="126" t="n"/>
       <c r="E98" s="126" t="n"/>
       <c r="F98" s="122" t="n"/>
     </row>
-    <row r="99" ht="28" customHeight="1" s="175">
-      <c r="B99" s="79" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C99" s="166" t="n"/>
-      <c r="D99" s="126" t="n"/>
-      <c r="E99" s="126" t="n"/>
-      <c r="F99" s="122" t="n"/>
-    </row>
-    <row r="100" ht="18" customHeight="1" s="175">
-      <c r="B100" s="118" t="inlineStr">
+    <row r="99" ht="18" customHeight="1" s="175">
+      <c r="B99" s="118" t="inlineStr">
         <is>
           <t>6. CUSTOMER EXPERIENCE</t>
         </is>
       </c>
-      <c r="C100" s="119" t="n"/>
-      <c r="D100" s="119" t="n"/>
-      <c r="E100" s="120" t="n"/>
-      <c r="F100" s="6" t="inlineStr">
+      <c r="C99" s="119" t="n"/>
+      <c r="D99" s="119" t="n"/>
+      <c r="E99" s="120" t="n"/>
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
+    <row r="100" ht="28" customHeight="1" s="175">
+      <c r="B100" s="148" t="inlineStr">
+        <is>
+          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
+        </is>
+      </c>
+      <c r="C100" s="126" t="n"/>
+      <c r="D100" s="126" t="n"/>
+      <c r="E100" s="126" t="n"/>
+      <c r="F100" s="122" t="n"/>
+    </row>
     <row r="101" ht="28" customHeight="1" s="175">
-      <c r="B101" s="148" t="inlineStr">
-        <is>
-          <t>Objective: Measure the overall customer experience delivered during the interaction.</t>
-        </is>
-      </c>
-      <c r="C101" s="126" t="n"/>
-      <c r="D101" s="126" t="n"/>
+      <c r="B101" s="229" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C101" s="230" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D101" s="229" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E101" s="126" t="n"/>
       <c r="F101" s="122" t="n"/>
     </row>
     <row r="102" ht="28" customHeight="1" s="175">
-      <c r="B102" s="75" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C102" s="104" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D102" s="152" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+      <c r="B102" s="222" t="inlineStr">
+        <is>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
+        </is>
+      </c>
+      <c r="C102" s="221" t="n"/>
+      <c r="D102" s="222" t="n"/>
       <c r="E102" s="126" t="n"/>
       <c r="F102" s="122" t="n"/>
     </row>
     <row r="103" ht="28" customHeight="1" s="175">
-      <c r="B103" s="76" t="inlineStr">
-        <is>
-          <t>Demonstrated empathy including for repeat-contact fatigue</t>
-        </is>
-      </c>
-      <c r="C103" s="105" t="n"/>
-      <c r="D103" s="147" t="n"/>
+      <c r="B103" s="143" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+        </is>
+      </c>
+      <c r="C103" s="221" t="n"/>
+      <c r="D103" s="143" t="n"/>
       <c r="E103" s="126" t="n"/>
       <c r="F103" s="122" t="n"/>
     </row>
     <row r="104" ht="28" customHeight="1" s="175">
-      <c r="B104" s="106" t="inlineStr">
-        <is>
-          <t>Stayed professional throughout and maintained patience, even under pressure</t>
-        </is>
-      </c>
-      <c r="C104" s="105" t="n"/>
-      <c r="D104" s="143" t="n"/>
+      <c r="B104" s="222" t="inlineStr">
+        <is>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
+        </is>
+      </c>
+      <c r="C104" s="221" t="n"/>
+      <c r="D104" s="222" t="n"/>
       <c r="E104" s="126" t="n"/>
       <c r="F104" s="122" t="n"/>
     </row>
     <row r="105" ht="28" customHeight="1" s="175">
-      <c r="B105" s="76" t="inlineStr">
-        <is>
-          <t>Agent matched the customer's tone, pace, level, and energy</t>
-        </is>
-      </c>
-      <c r="C105" s="105" t="n"/>
-      <c r="D105" s="147" t="n"/>
+      <c r="B105" s="222" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
+        </is>
+      </c>
+      <c r="C105" s="221" t="n"/>
+      <c r="D105" s="222" t="n"/>
       <c r="E105" s="126" t="n"/>
       <c r="F105" s="122" t="n"/>
     </row>
     <row r="106" ht="28" customHeight="1" s="175">
-      <c r="B106" s="76" t="inlineStr">
-        <is>
-          <t>Minimized customer effort</t>
-        </is>
-      </c>
-      <c r="C106" s="105" t="n"/>
-      <c r="D106" s="147" t="n"/>
+      <c r="B106" s="143" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C106" s="221" t="n"/>
+      <c r="D106" s="143" t="n"/>
       <c r="E106" s="126" t="n"/>
       <c r="F106" s="122" t="n"/>
     </row>
     <row r="107" ht="28" customHeight="1" s="175">
-      <c r="B107" s="106" t="inlineStr">
-        <is>
-          <t>Maintained customer understanding and engagement</t>
-        </is>
-      </c>
-      <c r="C107" s="105" t="n"/>
-      <c r="D107" s="143" t="n"/>
+      <c r="B107" s="223" t="inlineStr">
+        <is>
+          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
+        </is>
+      </c>
+      <c r="C107" s="126" t="n"/>
+      <c r="D107" s="126" t="n"/>
       <c r="E107" s="126" t="n"/>
       <c r="F107" s="122" t="n"/>
     </row>
     <row r="108" ht="28" customHeight="1" s="175">
-      <c r="B108" s="137" t="inlineStr">
-        <is>
-          <t>⚠ Negative indicators: dismissive responses; robotic interactions; frustration escalation caused by agent behavior; marathon sessions pushed onto vulnerable customers without offering to pause and resume.</t>
-        </is>
-      </c>
-      <c r="C108" s="126" t="n"/>
-      <c r="D108" s="126" t="n"/>
+      <c r="B108" s="224" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C108" s="225">
+        <f>IF((COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed"))=0,"",ROUND((COUNTIF(C102:C106,"Met")*5+COUNTIF(C102:C106,"Partial")*2.5)/(COUNTIF(C102:C106,"Met")+COUNTIF(C102:C106,"Partial")+COUNTIF(C102:C106,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D108" s="146" t="n"/>
       <c r="E108" s="126" t="n"/>
       <c r="F108" s="122" t="n"/>
     </row>
-    <row r="109" ht="28" customHeight="1" s="175">
-      <c r="B109" s="107" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C109" s="108">
-        <f>IF((COUNTIF(C103:C107,"Met")+COUNTIF(C103:C107,"Partial")+COUNTIF(C103:C107,"Missed"))=0,"",ROUND((COUNTIF(C103:C107,"Met")*5+COUNTIF(C103:C107,"Partial")*2.5)/(COUNTIF(C103:C107,"Met")+COUNTIF(C103:C107,"Partial")+COUNTIF(C103:C107,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D109" s="146" t="n"/>
+    <row r="109" ht="24" customHeight="1" s="175">
+      <c r="B109" s="226" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C109" s="227" t="n"/>
+      <c r="D109" s="161">
+        <f>IF(IF(C109="",C108,C109)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C109="",C108,C109)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E109" s="126" t="n"/>
       <c r="F109" s="122" t="n"/>
     </row>
-    <row r="110" ht="24" customHeight="1" s="175">
-      <c r="B110" s="79" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C110" s="109" t="n"/>
-      <c r="D110" s="161">
-        <f>IF(IF(C110="",C109,C110)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C110="",C109,C110)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="110" ht="36" customHeight="1" s="175">
+      <c r="B110" s="226" t="inlineStr">
+        <is>
+          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
+        </is>
+      </c>
+      <c r="C110" s="228" t="n"/>
+      <c r="D110" s="126" t="n"/>
       <c r="E110" s="126" t="n"/>
       <c r="F110" s="122" t="n"/>
     </row>
-    <row r="111" ht="36" customHeight="1" s="175">
-      <c r="B111" s="79" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
-      <c r="C111" s="145" t="n"/>
-      <c r="D111" s="126" t="n"/>
-      <c r="E111" s="126" t="n"/>
-      <c r="F111" s="122" t="n"/>
-    </row>
-    <row r="112" ht="18" customHeight="1" s="175">
-      <c r="B112" s="118" t="inlineStr">
+    <row r="111" ht="18" customHeight="1" s="175">
+      <c r="B111" s="118" t="inlineStr">
         <is>
           <t>7. DOCUMENTATION &amp; NOTES</t>
         </is>
       </c>
-      <c r="C112" s="119" t="n"/>
-      <c r="D112" s="119" t="n"/>
-      <c r="E112" s="120" t="n"/>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="C111" s="119" t="n"/>
+      <c r="D111" s="119" t="n"/>
+      <c r="E111" s="120" t="n"/>
+      <c r="F111" s="6" t="inlineStr">
         <is>
           <t>Weight: 5%</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="28" customHeight="1" s="175">
-      <c r="B113" s="148" t="inlineStr">
+    <row r="112" ht="28" customHeight="1" s="175">
+      <c r="B112" s="148" t="inlineStr">
         <is>
           <t>Objective: Ensure future agents can quickly understand the case. Purpose is continuity, not compliance.</t>
         </is>
       </c>
-      <c r="C113" s="126" t="n"/>
-      <c r="D113" s="126" t="n"/>
+      <c r="C112" s="126" t="n"/>
+      <c r="D112" s="126" t="n"/>
+      <c r="E112" s="126" t="n"/>
+      <c r="F112" s="122" t="n"/>
+    </row>
+    <row r="113" ht="36" customHeight="1" s="175">
+      <c r="B113" s="229" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C113" s="230" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D113" s="229" t="inlineStr">
+        <is>
+          <t>Evidence / Observation (quote or timestamp where possible)</t>
+        </is>
+      </c>
       <c r="E113" s="126" t="n"/>
       <c r="F113" s="122" t="n"/>
     </row>
-    <row r="114" ht="36" customHeight="1" s="175">
-      <c r="B114" s="75" t="inlineStr">
-        <is>
-          <t>Behavioral Indicator</t>
-        </is>
-      </c>
-      <c r="C114" s="104" t="inlineStr">
-        <is>
-          <t>Assessment</t>
-        </is>
-      </c>
-      <c r="D114" s="152" t="inlineStr">
-        <is>
-          <t>Evidence / Observation (quote or timestamp where possible)</t>
-        </is>
-      </c>
+    <row r="114" ht="28" customHeight="1" s="175">
+      <c r="B114" s="222" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
+        </is>
+      </c>
+      <c r="C114" s="221" t="n"/>
+      <c r="D114" s="222" t="n"/>
       <c r="E114" s="126" t="n"/>
       <c r="F114" s="122" t="n"/>
     </row>
     <row r="115" ht="28" customHeight="1" s="175">
-      <c r="B115" s="76" t="inlineStr">
-        <is>
-          <t>Recorded customer issue summary</t>
-        </is>
-      </c>
-      <c r="C115" s="105" t="n"/>
-      <c r="D115" s="147" t="n"/>
+      <c r="B115" s="143" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
+        </is>
+      </c>
+      <c r="C115" s="221" t="n"/>
+      <c r="D115" s="143" t="n"/>
       <c r="E115" s="126" t="n"/>
       <c r="F115" s="122" t="n"/>
     </row>
     <row r="116" ht="28" customHeight="1" s="175">
-      <c r="B116" s="106" t="inlineStr">
-        <is>
-          <t>Documented troubleshooting steps</t>
-        </is>
-      </c>
-      <c r="C116" s="105" t="n"/>
-      <c r="D116" s="143" t="n"/>
+      <c r="B116" s="222" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
+        </is>
+      </c>
+      <c r="C116" s="221" t="n"/>
+      <c r="D116" s="222" t="n"/>
       <c r="E116" s="126" t="n"/>
       <c r="F116" s="122" t="n"/>
     </row>
     <row r="117" ht="28" customHeight="1" s="175">
-      <c r="B117" s="76" t="inlineStr">
-        <is>
-          <t>Noted key findings</t>
-        </is>
-      </c>
-      <c r="C117" s="105" t="n"/>
-      <c r="D117" s="147" t="n"/>
+      <c r="B117" s="143" t="inlineStr">
+        <is>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
+        </is>
+      </c>
+      <c r="C117" s="221" t="n"/>
+      <c r="D117" s="143" t="n"/>
       <c r="E117" s="126" t="n"/>
       <c r="F117" s="122" t="n"/>
     </row>
     <row r="118" ht="28" customHeight="1" s="175">
-      <c r="B118" s="106" t="inlineStr">
-        <is>
-          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
-        </is>
-      </c>
-      <c r="C118" s="105" t="n"/>
+      <c r="B118" s="143" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
+        </is>
+      </c>
+      <c r="C118" s="221" t="n"/>
       <c r="D118" s="143" t="n"/>
       <c r="E118" s="126" t="n"/>
       <c r="F118" s="122" t="n"/>
     </row>
     <row r="119" ht="28" customHeight="1" s="175">
-      <c r="B119" s="106" t="inlineStr">
-        <is>
-          <t>Documented next steps and follow-ups</t>
-        </is>
-      </c>
-      <c r="C119" s="105" t="n"/>
-      <c r="D119" s="143" t="n"/>
+      <c r="B119" s="222" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C119" s="221" t="n"/>
+      <c r="D119" s="222" t="n"/>
       <c r="E119" s="126" t="n"/>
       <c r="F119" s="122" t="n"/>
     </row>
     <row r="120" ht="28" customHeight="1" s="175">
-      <c r="B120" s="76" t="inlineStr">
-        <is>
-          <t>Updated ticket status accurately</t>
-        </is>
-      </c>
-      <c r="C120" s="105" t="n"/>
-      <c r="D120" s="147" t="n"/>
+      <c r="B120" s="223" t="inlineStr">
+        <is>
+          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
+        </is>
+      </c>
+      <c r="C120" s="126" t="n"/>
+      <c r="D120" s="126" t="n"/>
       <c r="E120" s="126" t="n"/>
       <c r="F120" s="122" t="n"/>
     </row>
-    <row r="121" ht="28" customHeight="1" s="175">
-      <c r="B121" s="137" t="inlineStr">
-        <is>
-          <t>⚠ Documentation supports outcomes but should not outweigh troubleshooting quality, communication, or ownership. Notes must carry the FULL history — including pre-ticket contacts — so no agent treats a long-running case as new.</t>
-        </is>
-      </c>
-      <c r="C121" s="126" t="n"/>
-      <c r="D121" s="126" t="n"/>
+    <row r="121" ht="52" customHeight="1" s="175">
+      <c r="B121" s="224" t="inlineStr">
+        <is>
+          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
+        </is>
+      </c>
+      <c r="C121" s="225">
+        <f>IF((COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed"))=0,"",ROUND((COUNTIF(C114:C119,"Met")*5+COUNTIF(C114:C119,"Partial")*2.5)/(COUNTIF(C114:C119,"Met")+COUNTIF(C114:C119,"Partial")+COUNTIF(C114:C119,"Missed")),0))</f>
+        <v/>
+      </c>
+      <c r="D121" s="146" t="n"/>
       <c r="E121" s="126" t="n"/>
       <c r="F121" s="122" t="n"/>
     </row>
-    <row r="122" ht="52" customHeight="1" s="175">
-      <c r="B122" s="107" t="inlineStr">
-        <is>
-          <t>Auto score (0–5) from indicator ratings — applies unless overridden</t>
-        </is>
-      </c>
-      <c r="C122" s="108">
-        <f>IF((COUNTIF(C115:C120,"Met")+COUNTIF(C115:C120,"Partial")+COUNTIF(C115:C120,"Missed"))=0,"",ROUND((COUNTIF(C115:C120,"Met")*5+COUNTIF(C115:C120,"Partial")*2.5)/(COUNTIF(C115:C120,"Met")+COUNTIF(C115:C120,"Partial")+COUNTIF(C115:C120,"Missed")),0))</f>
-        <v/>
-      </c>
-      <c r="D122" s="146" t="n"/>
+    <row r="122" ht="24" customHeight="1" s="175">
+      <c r="B122" s="226" t="inlineStr">
+        <is>
+          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
+        </is>
+      </c>
+      <c r="C122" s="227" t="n"/>
+      <c r="D122" s="161">
+        <f>IF(IF(C122="",C121,C122)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C122="",C121,C122)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
+        <v/>
+      </c>
       <c r="E122" s="126" t="n"/>
       <c r="F122" s="122" t="n"/>
     </row>
-    <row r="123" ht="24" customHeight="1" s="175">
-      <c r="B123" s="79" t="inlineStr">
-        <is>
-          <t>FINAL SCORE — leave blank to use the auto score; type 0–5 to override</t>
-        </is>
-      </c>
-      <c r="C123" s="109" t="n"/>
-      <c r="D123" s="161">
-        <f>IF(IF(C123="",C122,C123)="","← rate the indicators above (auto-scores), or type an override",CHOOSE(IF(C123="",C122,C123)+1,"Agent actions delayed, prevented, or negatively impacted resolution","Little or no meaningful progress","Limited progress despite available troubleshooting paths","Partial progress made but opportunities missed","Significant progress made with clear next steps","Issue resolved or strongest available outcome achieved"))</f>
-        <v/>
-      </c>
+    <row r="123" ht="36" customHeight="1" s="175">
+      <c r="B123" s="226" t="inlineStr">
+        <is>
+          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
+        </is>
+      </c>
+      <c r="C123" s="228" t="n"/>
+      <c r="D123" s="126" t="n"/>
       <c r="E123" s="126" t="n"/>
       <c r="F123" s="122" t="n"/>
     </row>
-    <row r="124" ht="36" customHeight="1" s="175">
-      <c r="B124" s="79" t="inlineStr">
-        <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
-      <c r="C124" s="145" t="n"/>
-      <c r="D124" s="126" t="n"/>
-      <c r="E124" s="126" t="n"/>
-      <c r="F124" s="122" t="n"/>
-    </row>
-    <row r="125" ht="30" customHeight="1" s="175">
-      <c r="B125" s="118" t="inlineStr">
+    <row r="124" ht="30" customHeight="1" s="175">
+      <c r="B124" s="118" t="inlineStr">
         <is>
           <t>4 · RESOLUTION OUTCOME</t>
         </is>
       </c>
-      <c r="C125" s="119" t="n"/>
-      <c r="D125" s="119" t="n"/>
-      <c r="E125" s="119" t="n"/>
-      <c r="F125" s="120" t="n"/>
-    </row>
-    <row r="126" ht="28" customHeight="1" s="175">
-      <c r="B126" s="75" t="inlineStr">
+      <c r="C124" s="119" t="n"/>
+      <c r="D124" s="119" t="n"/>
+      <c r="E124" s="119" t="n"/>
+      <c r="F124" s="120" t="n"/>
+    </row>
+    <row r="125" ht="28" customHeight="1" s="175">
+      <c r="B125" s="229" t="inlineStr">
         <is>
           <t>Outcome classification</t>
         </is>
       </c>
-      <c r="C126" s="170" t="n"/>
+      <c r="C125" s="231" t="n"/>
+      <c r="D125" s="126" t="n"/>
+      <c r="E125" s="126" t="n"/>
+      <c r="F125" s="122" t="n"/>
+    </row>
+    <row r="126" ht="52" customHeight="1" s="175">
+      <c r="B126" s="232" t="inlineStr">
+        <is>
+          <t>Primary positive outcome achieved</t>
+        </is>
+      </c>
+      <c r="C126" s="233" t="n"/>
       <c r="D126" s="126" t="n"/>
       <c r="E126" s="126" t="n"/>
       <c r="F126" s="122" t="n"/>
     </row>
     <row r="127" ht="52" customHeight="1" s="175">
-      <c r="B127" s="84" t="inlineStr">
-        <is>
-          <t>Primary positive outcome achieved</t>
-        </is>
-      </c>
-      <c r="C127" s="149" t="n"/>
+      <c r="B127" s="229" t="inlineStr">
+        <is>
+          <t>Justification</t>
+        </is>
+      </c>
+      <c r="C127" s="228" t="n"/>
       <c r="D127" s="126" t="n"/>
       <c r="E127" s="126" t="n"/>
       <c r="F127" s="122" t="n"/>
     </row>
-    <row r="128" ht="52" customHeight="1" s="175">
-      <c r="B128" s="75" t="inlineStr">
-        <is>
-          <t>Justification</t>
-        </is>
-      </c>
-      <c r="C128" s="145" t="n"/>
-      <c r="D128" s="126" t="n"/>
-      <c r="E128" s="126" t="n"/>
-      <c r="F128" s="122" t="n"/>
-    </row>
-    <row r="129" ht="26" customHeight="1" s="175">
-      <c r="B129" s="118" t="inlineStr">
+    <row r="128" ht="26" customHeight="1" s="175">
+      <c r="B128" s="118" t="inlineStr">
         <is>
           <t>5 · DISCONNECTED CALL FOLLOW-UP</t>
         </is>
       </c>
-      <c r="C129" s="119" t="n"/>
-      <c r="D129" s="119" t="n"/>
-      <c r="E129" s="119" t="n"/>
-      <c r="F129" s="120" t="n"/>
+      <c r="C128" s="119" t="n"/>
+      <c r="D128" s="119" t="n"/>
+      <c r="E128" s="119" t="n"/>
+      <c r="F128" s="120" t="n"/>
+    </row>
+    <row r="129" ht="30" customHeight="1" s="175">
+      <c r="B129" s="232" t="inlineStr">
+        <is>
+          <t>Did the interaction disconnect before completion?</t>
+        </is>
+      </c>
+      <c r="C129" s="221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D129" s="223" t="inlineStr">
+        <is>
+          <t>If Yes, at least one documented follow-up action is required.</t>
+        </is>
+      </c>
+      <c r="E129" s="126" t="n"/>
+      <c r="F129" s="122" t="n"/>
     </row>
     <row r="130" ht="30" customHeight="1" s="175">
-      <c r="B130" s="84" t="inlineStr">
-        <is>
-          <t>Did the interaction disconnect before completion?</t>
-        </is>
-      </c>
-      <c r="C130" s="105" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D130" s="137" t="inlineStr">
-        <is>
-          <t>If Yes, at least one documented follow-up action is required.</t>
-        </is>
-      </c>
-      <c r="E130" s="126" t="n"/>
+      <c r="A130" s="80" t="n"/>
+      <c r="B130" s="229" t="inlineStr">
+        <is>
+          <t>Follow-up action taken</t>
+        </is>
+      </c>
+      <c r="C130" s="233" t="inlineStr">
+        <is>
+          <t>N.A. — no disconnect</t>
+        </is>
+      </c>
+      <c r="D130" s="122" t="n"/>
+      <c r="E130" s="150">
+        <f>IF(AND(C129="Yes",OR(C130="None",C130="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
+        <v/>
+      </c>
       <c r="F130" s="122" t="n"/>
-    </row>
-    <row r="131" ht="30" customHeight="1" s="175">
+      <c r="G130" s="80" t="n"/>
+    </row>
+    <row r="131" ht="22" customHeight="1" s="175">
       <c r="A131" s="80" t="n"/>
-      <c r="B131" s="75" t="inlineStr">
-        <is>
-          <t>Follow-up action taken</t>
-        </is>
-      </c>
-      <c r="C131" s="149" t="inlineStr">
-        <is>
-          <t>N.A. — no disconnect</t>
-        </is>
-      </c>
-      <c r="D131" s="122" t="n"/>
-      <c r="E131" s="150">
-        <f>IF(AND(C130="Yes",OR(C131="None",C131="N.A. — no disconnect")),"⚠ MISSED OWNERSHIP OPPORTUNITY — flag in Customer Ownership and Critical Failures","OK")</f>
-        <v/>
-      </c>
+      <c r="B131" s="169" t="inlineStr">
+        <is>
+          <t>COACHING FLAGS   ·   Auto-populated from Partial and Missed ratings   ·   Each flagged item requires a coaching or review action</t>
+        </is>
+      </c>
+      <c r="C131" s="126" t="n"/>
+      <c r="D131" s="126" t="n"/>
+      <c r="E131" s="126" t="n"/>
       <c r="F131" s="122" t="n"/>
       <c r="G131" s="80" t="n"/>
     </row>
-    <row r="132" ht="22" customHeight="1" s="175">
+    <row r="132" ht="18" customHeight="1" s="175">
       <c r="A132" s="80" t="n"/>
-      <c r="B132" s="169" t="inlineStr">
-        <is>
-          <t>COACHING FLAGS   ·   Auto-populated from Partial and Missed ratings   ·   Each flagged item requires a coaching or review action</t>
-        </is>
-      </c>
-      <c r="C132" s="126" t="n"/>
-      <c r="D132" s="126" t="n"/>
+      <c r="B132" s="154" t="inlineStr">
+        <is>
+          <t>Flag Condition</t>
+        </is>
+      </c>
+      <c r="C132" s="154" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="D132" s="154" t="inlineStr">
+        <is>
+          <t>Coaching Focus / Required Action</t>
+        </is>
+      </c>
       <c r="E132" s="126" t="n"/>
       <c r="F132" s="122" t="n"/>
       <c r="G132" s="80" t="n"/>
     </row>
-    <row r="133" ht="18" customHeight="1" s="175">
+    <row r="133" ht="28" customHeight="1" s="175">
       <c r="A133" s="80" t="n"/>
-      <c r="B133" s="154" t="inlineStr">
-        <is>
-          <t>Flag Condition</t>
-        </is>
-      </c>
-      <c r="C133" s="154" t="inlineStr">
-        <is>
-          <t>Rating</t>
-        </is>
-      </c>
-      <c r="D133" s="154" t="inlineStr">
-        <is>
-          <t>Coaching Focus / Required Action</t>
+      <c r="B133" s="82" t="inlineStr">
+        <is>
+          <t>Technical accuracy failure</t>
+        </is>
+      </c>
+      <c r="C133" s="83">
+        <f>IF(OR(C51="Partial",C51="Missed"),C51,"")</f>
+        <v/>
+      </c>
+      <c r="D133" s="165" t="inlineStr">
+        <is>
+          <t>Review for incorrect guidance, product misrepresentation, or unsupported root-cause conclusions</t>
         </is>
       </c>
       <c r="E133" s="126" t="n"/>
@@ -5655,16 +5708,16 @@
       <c r="A134" s="80" t="n"/>
       <c r="B134" s="82" t="inlineStr">
         <is>
-          <t>Technical accuracy failure</t>
+          <t>No follow-up after disconnected call</t>
         </is>
       </c>
       <c r="C134" s="83">
-        <f>IF(OR(C51="Partial",C51="Missed"),C51,"")</f>
+        <f>IF(OR(C76="Partial",C76="Missed"),C76,"")</f>
         <v/>
       </c>
       <c r="D134" s="165" t="inlineStr">
         <is>
-          <t>Review for incorrect guidance, product misrepresentation, or unsupported root-cause conclusions</t>
+          <t>Mandatory callback attempt required; document outcome in case notes</t>
         </is>
       </c>
       <c r="E134" s="126" t="n"/>
@@ -5675,16 +5728,16 @@
       <c r="A135" s="80" t="n"/>
       <c r="B135" s="82" t="inlineStr">
         <is>
-          <t>No follow-up after disconnected call</t>
+          <t>Commitments not fulfilled / clear path forward missing</t>
         </is>
       </c>
       <c r="C135" s="83">
-        <f>IF(OR(C77="Partial",C77="Missed"),C77,"")</f>
+        <f>IF(OR(C74="Partial",C74="Missed"),C74,"")</f>
         <v/>
       </c>
       <c r="D135" s="165" t="inlineStr">
         <is>
-          <t>Mandatory callback attempt required; document outcome in case notes</t>
+          <t>Review what was promised; confirm the customer was left with actionable next steps</t>
         </is>
       </c>
       <c r="E135" s="126" t="n"/>
@@ -5695,16 +5748,16 @@
       <c r="A136" s="80" t="n"/>
       <c r="B136" s="82" t="inlineStr">
         <is>
-          <t>Commitments not fulfilled / clear path forward missing</t>
+          <t>Customer abandoned without a path forward</t>
         </is>
       </c>
       <c r="C136" s="83">
-        <f>IF(OR(C74="Partial",C74="Missed"),C74,"")</f>
+        <f>IF(OR(C39="Partial",C39="Missed"),C39,"")</f>
         <v/>
       </c>
       <c r="D136" s="165" t="inlineStr">
         <is>
-          <t>Review what was promised; confirm the customer was left with actionable next steps</t>
+          <t>Review whether the customer had any defined next step at close; address in coaching session</t>
         </is>
       </c>
       <c r="E136" s="126" t="n"/>
@@ -5715,16 +5768,16 @@
       <c r="A137" s="80" t="n"/>
       <c r="B137" s="82" t="inlineStr">
         <is>
-          <t>Customer abandoned without a path forward</t>
+          <t>Escalated without completing reasonable troubleshooting</t>
         </is>
       </c>
       <c r="C137" s="83">
-        <f>IF(OR(C39="Partial",C39="Missed"),C39,"")</f>
+        <f>IF(OR(C84="Partial",C84="Missed"),C84,"")</f>
         <v/>
       </c>
       <c r="D137" s="165" t="inlineStr">
         <is>
-          <t>Review whether the customer had any defined next step at close; address in coaching session</t>
+          <t>Review L1 steps completed before escalation; identify gaps and add to troubleshooting playbook</t>
         </is>
       </c>
       <c r="E137" s="126" t="n"/>
@@ -5735,7 +5788,7 @@
       <c r="A138" s="80" t="n"/>
       <c r="B138" s="82" t="inlineStr">
         <is>
-          <t>Escalated without completing reasonable troubleshooting</t>
+          <t>Escalation criteria not met / complaint or legal-risk not escalated</t>
         </is>
       </c>
       <c r="C138" s="83">
@@ -5744,7 +5797,7 @@
       </c>
       <c r="D138" s="165" t="inlineStr">
         <is>
-          <t>Review L1 steps completed before escalation; identify gaps and add to troubleshooting playbook</t>
+          <t>Review whether a valid escalation trigger existed; coach on recognising escalation criteria</t>
         </is>
       </c>
       <c r="E138" s="126" t="n"/>
@@ -5755,16 +5808,16 @@
       <c r="A139" s="80" t="n"/>
       <c r="B139" s="82" t="inlineStr">
         <is>
-          <t>Escalation criteria not met / complaint or legal-risk not escalated</t>
+          <t>Professionalism concern</t>
         </is>
       </c>
       <c r="C139" s="83">
-        <f>IF(OR(C86="Partial",C86="Missed"),C86,"")</f>
+        <f>IF(OR(C103="Partial",C103="Missed"),C103,"")</f>
         <v/>
       </c>
       <c r="D139" s="165" t="inlineStr">
         <is>
-          <t>Review whether a valid escalation trigger existed; coach on recognising escalation criteria</t>
+          <t>Mandatory review; assess tone, conduct, and whether a policy violation occurred</t>
         </is>
       </c>
       <c r="E139" s="126" t="n"/>
@@ -5775,48 +5828,40 @@
       <c r="A140" s="80" t="n"/>
       <c r="B140" s="82" t="inlineStr">
         <is>
-          <t>Professionalism concern</t>
+          <t>Ticket status inaccurate / premature closure</t>
         </is>
       </c>
       <c r="C140" s="83">
-        <f>IF(OR(C104="Partial",C104="Missed"),C104,"")</f>
+        <f>IF(OR(C119="Partial",C119="Missed"),C119,"")</f>
         <v/>
       </c>
       <c r="D140" s="165" t="inlineStr">
         <is>
-          <t>Mandatory review; assess tone, conduct, and whether a policy violation occurred</t>
+          <t>Review ticket state at close; verify status accurately reflected the case outcome</t>
         </is>
       </c>
       <c r="E140" s="126" t="n"/>
       <c r="F140" s="122" t="n"/>
       <c r="G140" s="80" t="n"/>
     </row>
-    <row r="141" ht="28" customHeight="1" s="175">
+    <row r="141" ht="22" customHeight="1" s="175">
       <c r="A141" s="80" t="n"/>
-      <c r="B141" s="82" t="inlineStr">
-        <is>
-          <t>Ticket status inaccurate / premature closure</t>
-        </is>
-      </c>
-      <c r="C141" s="83">
-        <f>IF(OR(C120="Partial",C120="Missed"),C120,"")</f>
-        <v/>
-      </c>
-      <c r="D141" s="165" t="inlineStr">
-        <is>
-          <t>Review ticket state at close; verify status accurately reflected the case outcome</t>
-        </is>
-      </c>
+      <c r="B141" s="162" t="inlineStr">
+        <is>
+          <t>⚠  Survey / CSAT manipulation has no matching behavioral indicator and cannot be auto-detected — flag manually in §8 Coaching &amp; Feedback if suspected.</t>
+        </is>
+      </c>
+      <c r="C141" s="126" t="n"/>
+      <c r="D141" s="126" t="n"/>
       <c r="E141" s="126" t="n"/>
       <c r="F141" s="122" t="n"/>
       <c r="G141" s="80" t="n"/>
     </row>
     <row r="142" ht="22" customHeight="1" s="175">
       <c r="A142" s="80" t="n"/>
-      <c r="B142" s="162" t="inlineStr">
-        <is>
-          <t>⚠  Survey / CSAT manipulation has no matching behavioral indicator and cannot be auto-detected — flag manually in §8 Coaching &amp; Feedback if suspected.</t>
-        </is>
+      <c r="B142" s="159">
+        <f>IF(COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")=0,"✓  No coaching flags triggered — all key indicators met",COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")&amp;" coaching flag(s) triggered — review and coaching action required")</f>
+        <v/>
       </c>
       <c r="C142" s="126" t="n"/>
       <c r="D142" s="126" t="n"/>
@@ -5824,10 +5869,10 @@
       <c r="F142" s="122" t="n"/>
       <c r="G142" s="80" t="n"/>
     </row>
-    <row r="143" ht="22" customHeight="1" s="175">
+    <row r="143" ht="65" customHeight="1" s="175">
       <c r="A143" s="80" t="n"/>
-      <c r="B143" s="159">
-        <f>IF(COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")=0,"✓  No coaching flags triggered — all key indicators met",COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")&amp;" coaching flag(s) triggered — review and coaching action required")</f>
+      <c r="B143" s="163">
+        <f>IF(COUNTIF(C133:C140,"Partial")+COUNTIF(C133:C140,"Missed")=0,"All key indicators met — no coaching action required",_xludf.TEXTJOIN(CHAR(10),TRUE,IF(C133&lt;&gt;"","⚑ "&amp;B133&amp;" ["&amp;C133&amp;"]",""),IF(C134&lt;&gt;"","⚑ "&amp;B134&amp;" ["&amp;C134&amp;"]",""),IF(C135&lt;&gt;"","⚑ "&amp;B135&amp;" ["&amp;C135&amp;"]",""),IF(C136&lt;&gt;"","⚑ "&amp;B136&amp;" ["&amp;C136&amp;"]",""),IF(C137&lt;&gt;"","⚑ "&amp;B137&amp;" ["&amp;C137&amp;"]",""),IF(C138&lt;&gt;"","⚑ "&amp;B138&amp;" ["&amp;C138&amp;"]",""),IF(C139&lt;&gt;"","⚑ "&amp;B139&amp;" ["&amp;C139&amp;"]",""),IF(C140&lt;&gt;"","⚑ "&amp;B140&amp;" ["&amp;C140&amp;"]","")))</f>
         <v/>
       </c>
       <c r="C143" s="126" t="n"/>
@@ -5836,315 +5881,316 @@
       <c r="F143" s="122" t="n"/>
       <c r="G143" s="80" t="n"/>
     </row>
-    <row r="144" ht="65" customHeight="1" s="175">
+    <row r="144" ht="6" customHeight="1" s="175">
       <c r="A144" s="80" t="n"/>
-      <c r="B144" s="163">
-        <f>IF(COUNTIF(C134:C141,"Partial")+COUNTIF(C134:C141,"Missed")=0,"All key indicators met — no coaching action required",_xludf.TEXTJOIN(CHAR(10),TRUE,IF(C134&lt;&gt;"","⚑ "&amp;B134&amp;" ["&amp;C134&amp;"]",""),IF(C135&lt;&gt;"","⚑ "&amp;B135&amp;" ["&amp;C135&amp;"]",""),IF(C136&lt;&gt;"","⚑ "&amp;B136&amp;" ["&amp;C136&amp;"]",""),IF(C137&lt;&gt;"","⚑ "&amp;B137&amp;" ["&amp;C137&amp;"]",""),IF(C138&lt;&gt;"","⚑ "&amp;B138&amp;" ["&amp;C138&amp;"]",""),IF(C139&lt;&gt;"","⚑ "&amp;B139&amp;" ["&amp;C139&amp;"]",""),IF(C140&lt;&gt;"","⚑ "&amp;B140&amp;" ["&amp;C140&amp;"]",""),IF(C141&lt;&gt;"","⚑ "&amp;B141&amp;" ["&amp;C141&amp;"]","")))</f>
-        <v/>
-      </c>
-      <c r="C144" s="126" t="n"/>
-      <c r="D144" s="126" t="n"/>
-      <c r="E144" s="126" t="n"/>
-      <c r="F144" s="122" t="n"/>
+      <c r="B144" s="167" t="n"/>
+      <c r="C144" s="119" t="n"/>
+      <c r="D144" s="119" t="n"/>
+      <c r="E144" s="119" t="n"/>
+      <c r="F144" s="120" t="n"/>
       <c r="G144" s="80" t="n"/>
     </row>
-    <row r="145" ht="6" customHeight="1" s="175">
+    <row r="145" ht="22" customHeight="1" s="175">
       <c r="A145" s="80" t="n"/>
-      <c r="B145" s="167" t="n"/>
+      <c r="B145" s="127" t="inlineStr">
+        <is>
+          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
+        </is>
+      </c>
       <c r="C145" s="119" t="n"/>
       <c r="D145" s="119" t="n"/>
       <c r="E145" s="119" t="n"/>
       <c r="F145" s="120" t="n"/>
       <c r="G145" s="80" t="n"/>
     </row>
-    <row r="146" ht="22" customHeight="1" s="175">
-      <c r="B146" s="127" t="inlineStr">
-        <is>
-          <t>7 · AUTO-ZERO   (from the 360 Form — any trigger forces the Quality Score to 0%)</t>
-        </is>
-      </c>
-      <c r="C146" s="119" t="n"/>
-      <c r="D146" s="119" t="n"/>
-      <c r="E146" s="119" t="n"/>
-      <c r="F146" s="120" t="n"/>
+    <row r="146" ht="30" customHeight="1" s="175">
+      <c r="B146" s="223" t="inlineStr">
+        <is>
+          <t>A gate marked 'No', any A–K item marked 'Yes' forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
+        </is>
+      </c>
+      <c r="C146" s="126" t="n"/>
+      <c r="D146" s="126" t="n"/>
+      <c r="E146" s="126" t="n"/>
+      <c r="F146" s="122" t="n"/>
     </row>
     <row r="147" ht="30" customHeight="1" s="175">
-      <c r="B147" s="137" t="inlineStr">
-        <is>
-          <t>A gate marked 'No', any A–K item marked 'Yes' forces the weighted Quality Score (§3) to 0%. Category scores still show for coaching.</t>
-        </is>
-      </c>
-      <c r="C147" s="126" t="n"/>
-      <c r="D147" s="126" t="n"/>
-      <c r="E147" s="126" t="n"/>
-      <c r="F147" s="122" t="n"/>
-    </row>
-    <row r="148" ht="30" customHeight="1" s="175">
-      <c r="B148" s="118" t="inlineStr">
+      <c r="B147" s="118" t="inlineStr">
         <is>
           <t>Compliance gate  (mark Yes if adhered)</t>
         </is>
       </c>
-      <c r="C148" s="190" t="inlineStr">
+      <c r="C147" s="190" t="inlineStr">
         <is>
           <t>Adherent?</t>
         </is>
       </c>
-      <c r="D148" s="118" t="inlineStr">
+      <c r="D147" s="118" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E148" s="119" t="n"/>
-      <c r="F148" s="120" t="n"/>
+      <c r="E147" s="119" t="n"/>
+      <c r="F147" s="120" t="n"/>
+    </row>
+    <row r="148" ht="26" customHeight="1" s="175">
+      <c r="B148" s="222" t="inlineStr">
+        <is>
+          <t>Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C148" s="221" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D148" s="222" t="n"/>
+      <c r="E148" s="126" t="n"/>
+      <c r="F148" s="122" t="n"/>
     </row>
     <row r="149" ht="26" customHeight="1" s="175">
-      <c r="B149" s="76" t="inlineStr">
-        <is>
-          <t>Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C149" s="105" t="inlineStr">
+      <c r="B149" s="222" t="inlineStr">
+        <is>
+          <t>Adherence to PCI &amp; Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C149" s="221" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D149" s="147" t="n"/>
+      <c r="D149" s="222" t="n"/>
       <c r="E149" s="126" t="n"/>
       <c r="F149" s="122" t="n"/>
     </row>
     <row r="150" ht="26" customHeight="1" s="175">
-      <c r="B150" s="76" t="inlineStr">
-        <is>
-          <t>Adherence to PCI &amp; Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C150" s="105" t="inlineStr">
+      <c r="B150" s="222" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C150" s="221" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D150" s="147" t="n"/>
+      <c r="D150" s="222" t="n"/>
       <c r="E150" s="126" t="n"/>
       <c r="F150" s="122" t="n"/>
     </row>
-    <row r="151" ht="26" customHeight="1" s="175">
-      <c r="B151" s="76" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C151" s="105" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D151" s="147" t="n"/>
-      <c r="E151" s="126" t="n"/>
-      <c r="F151" s="122" t="n"/>
-    </row>
-    <row r="152" ht="32" customHeight="1" s="175">
-      <c r="B152" s="118" t="inlineStr">
+    <row r="151" ht="32" customHeight="1" s="175">
+      <c r="B151" s="118" t="inlineStr">
         <is>
           <t>AUTO-ZERO list — A to K  (mark Yes if it occurred)</t>
         </is>
       </c>
-      <c r="C152" s="190" t="inlineStr">
+      <c r="C151" s="190" t="inlineStr">
         <is>
           <t>Occurred?</t>
         </is>
       </c>
-      <c r="D152" s="118" t="inlineStr">
+      <c r="D151" s="118" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
-      <c r="E152" s="119" t="n"/>
-      <c r="F152" s="120" t="n"/>
+      <c r="E151" s="119" t="n"/>
+      <c r="F151" s="120" t="n"/>
+    </row>
+    <row r="152" ht="26" customHeight="1" s="175">
+      <c r="B152" s="222" t="inlineStr">
+        <is>
+          <t>A.  Call / Session Abandonment</t>
+        </is>
+      </c>
+      <c r="C152" s="221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D152" s="222" t="n"/>
+      <c r="E152" s="126" t="n"/>
+      <c r="F152" s="122" t="n"/>
     </row>
     <row r="153" ht="26" customHeight="1" s="175">
-      <c r="B153" s="76" t="inlineStr">
-        <is>
-          <t>A.  Call / Session Abandonment</t>
-        </is>
-      </c>
-      <c r="C153" s="105" t="inlineStr">
+      <c r="B153" s="222" t="inlineStr">
+        <is>
+          <t>B.  Call / Session Avoidance / Evasion</t>
+        </is>
+      </c>
+      <c r="C153" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D153" s="147" t="n"/>
+      <c r="D153" s="222" t="n"/>
       <c r="E153" s="126" t="n"/>
       <c r="F153" s="122" t="n"/>
     </row>
     <row r="154" ht="26" customHeight="1" s="175">
-      <c r="B154" s="76" t="inlineStr">
-        <is>
-          <t>B.  Call / Session Avoidance / Evasion</t>
-        </is>
-      </c>
-      <c r="C154" s="105" t="inlineStr">
+      <c r="B154" s="222" t="inlineStr">
+        <is>
+          <t>C.  Discourtesy</t>
+        </is>
+      </c>
+      <c r="C154" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D154" s="147" t="n"/>
+      <c r="D154" s="222" t="n"/>
       <c r="E154" s="126" t="n"/>
       <c r="F154" s="122" t="n"/>
     </row>
     <row r="155" ht="26" customHeight="1" s="175">
-      <c r="B155" s="76" t="inlineStr">
-        <is>
-          <t>C.  Discourtesy</t>
-        </is>
-      </c>
-      <c r="C155" s="105" t="inlineStr">
+      <c r="B155" s="222" t="inlineStr">
+        <is>
+          <t>D.  Escalation</t>
+        </is>
+      </c>
+      <c r="C155" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D155" s="147" t="n"/>
+      <c r="D155" s="222" t="n"/>
       <c r="E155" s="126" t="n"/>
       <c r="F155" s="122" t="n"/>
     </row>
     <row r="156" ht="26" customHeight="1" s="175">
-      <c r="B156" s="76" t="inlineStr">
-        <is>
-          <t>D.  Escalation</t>
-        </is>
-      </c>
-      <c r="C156" s="105" t="inlineStr">
+      <c r="B156" s="222" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="C156" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D156" s="147" t="n"/>
+      <c r="D156" s="222" t="n"/>
       <c r="E156" s="126" t="n"/>
       <c r="F156" s="122" t="n"/>
     </row>
     <row r="157" ht="26" customHeight="1" s="175">
-      <c r="B157" s="76" t="inlineStr">
-        <is>
-          <t>E.  Failure to ask for the email address</t>
-        </is>
-      </c>
-      <c r="C157" s="105" t="inlineStr">
+      <c r="B157" s="222" t="inlineStr">
+        <is>
+          <t>F.  Fraud</t>
+        </is>
+      </c>
+      <c r="C157" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D157" s="147" t="n"/>
+      <c r="D157" s="222" t="n"/>
       <c r="E157" s="126" t="n"/>
       <c r="F157" s="122" t="n"/>
     </row>
     <row r="158" ht="26" customHeight="1" s="175">
-      <c r="B158" s="76" t="inlineStr">
-        <is>
-          <t>F.  Fraud</t>
-        </is>
-      </c>
-      <c r="C158" s="105" t="inlineStr">
+      <c r="B158" s="222" t="inlineStr">
+        <is>
+          <t>G.  Hard-selling</t>
+        </is>
+      </c>
+      <c r="C158" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D158" s="147" t="n"/>
+      <c r="D158" s="222" t="n"/>
       <c r="E158" s="126" t="n"/>
       <c r="F158" s="122" t="n"/>
     </row>
     <row r="159" ht="26" customHeight="1" s="175">
-      <c r="B159" s="76" t="inlineStr">
-        <is>
-          <t>G.  Hard-selling</t>
-        </is>
-      </c>
-      <c r="C159" s="105" t="inlineStr">
+      <c r="B159" s="222" t="inlineStr">
+        <is>
+          <t>H.  Line Release</t>
+        </is>
+      </c>
+      <c r="C159" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D159" s="147" t="n"/>
+      <c r="D159" s="222" t="n"/>
       <c r="E159" s="126" t="n"/>
       <c r="F159" s="122" t="n"/>
     </row>
     <row r="160" ht="26" customHeight="1" s="175">
-      <c r="B160" s="76" t="inlineStr">
-        <is>
-          <t>H.  Line Release</t>
-        </is>
-      </c>
-      <c r="C160" s="105" t="inlineStr">
+      <c r="B160" s="222" t="inlineStr">
+        <is>
+          <t>I.  Non-Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="C160" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D160" s="147" t="n"/>
+      <c r="D160" s="222" t="n"/>
       <c r="E160" s="126" t="n"/>
       <c r="F160" s="122" t="n"/>
     </row>
     <row r="161" ht="26" customHeight="1" s="175">
-      <c r="B161" s="76" t="inlineStr">
-        <is>
-          <t>I.  Non-Adherence to Callback Hours</t>
-        </is>
-      </c>
-      <c r="C161" s="105" t="inlineStr">
+      <c r="B161" s="222" t="inlineStr">
+        <is>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+        </is>
+      </c>
+      <c r="C161" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D161" s="147" t="n"/>
+      <c r="D161" s="222" t="n"/>
       <c r="E161" s="126" t="n"/>
       <c r="F161" s="122" t="n"/>
     </row>
     <row r="162" ht="26" customHeight="1" s="175">
-      <c r="B162" s="76" t="inlineStr">
-        <is>
-          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
-        </is>
-      </c>
-      <c r="C162" s="105" t="inlineStr">
+      <c r="B162" s="222" t="inlineStr">
+        <is>
+          <t>K.  Non-First Call Resolution</t>
+        </is>
+      </c>
+      <c r="C162" s="221" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D162" s="147" t="n"/>
+      <c r="D162" s="222" t="n"/>
       <c r="E162" s="126" t="n"/>
       <c r="F162" s="122" t="n"/>
     </row>
-    <row r="163" ht="26" customHeight="1" s="175">
-      <c r="B163" s="76" t="inlineStr">
-        <is>
-          <t>K.  Non-First Call Resolution</t>
-        </is>
-      </c>
-      <c r="C163" s="105" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D163" s="147" t="n"/>
-      <c r="E163" s="126" t="n"/>
-      <c r="F163" s="122" t="n"/>
-    </row>
-    <row r="164" ht="24" customHeight="1" s="175">
-      <c r="B164" s="127" t="inlineStr">
+    <row r="163" ht="24" customHeight="1" s="175">
+      <c r="B163" s="127" t="inlineStr">
         <is>
           <t>AUTO-ZERO TRIGGERED?</t>
         </is>
       </c>
-      <c r="C164" s="160">
-        <f>IF(OR(C149="No",C150="No",C151="No",COUNTIF(C153:C163,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
-        <v/>
-      </c>
+      <c r="C163" s="160">
+        <f>IF(OR(C148="No",C149="No",C150="No",COUNTIF(C152:C162,"Yes")&gt;0),"YES — Quality Score forced to 0%","No")</f>
+        <v/>
+      </c>
+      <c r="D163" s="119" t="n"/>
+      <c r="E163" s="119" t="n"/>
+      <c r="F163" s="120" t="n"/>
+    </row>
+    <row r="164" ht="20" customHeight="1" s="175">
+      <c r="B164" s="168" t="inlineStr">
+        <is>
+          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
+        </is>
+      </c>
+      <c r="C164" s="119" t="n"/>
       <c r="D164" s="119" t="n"/>
       <c r="E164" s="119" t="n"/>
       <c r="F164" s="120" t="n"/>
     </row>
-    <row r="165" ht="20" customHeight="1" s="175">
-      <c r="B165" s="168" t="inlineStr">
-        <is>
-          <t>8 · COACHING &amp; FEEDBACK   (every review answers the three QA questions below)</t>
+    <row r="165" ht="30" customHeight="1" s="175">
+      <c r="B165" s="153" t="inlineStr">
+        <is>
+          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
         </is>
       </c>
       <c r="C165" s="119" t="n"/>
@@ -6152,461 +6198,450 @@
       <c r="E165" s="119" t="n"/>
       <c r="F165" s="120" t="n"/>
     </row>
-    <row r="166" ht="30" customHeight="1" s="175">
-      <c r="B166" s="153" t="inlineStr">
-        <is>
-          <t>Q1 · Did we help the customer as effectively as we reasonably could?</t>
-        </is>
-      </c>
-      <c r="C166" s="119" t="n"/>
-      <c r="D166" s="119" t="n"/>
-      <c r="E166" s="119" t="n"/>
-      <c r="F166" s="120" t="n"/>
-    </row>
-    <row r="167" ht="58" customHeight="1" s="175">
-      <c r="B167" s="145" t="n"/>
-      <c r="C167" s="126" t="n"/>
-      <c r="D167" s="126" t="n"/>
-      <c r="E167" s="126" t="n"/>
-      <c r="F167" s="122" t="n"/>
-    </row>
-    <row r="168" ht="30" customHeight="1" s="175">
-      <c r="B168" s="153" t="inlineStr">
+    <row r="166" ht="58" customHeight="1" s="175">
+      <c r="B166" s="228" t="n"/>
+      <c r="C166" s="126" t="n"/>
+      <c r="D166" s="126" t="n"/>
+      <c r="E166" s="126" t="n"/>
+      <c r="F166" s="122" t="n"/>
+    </row>
+    <row r="167" ht="30" customHeight="1" s="175">
+      <c r="B167" s="153" t="inlineStr">
         <is>
           <t>Q2 · Did the agent demonstrate strong technical and communication behavior?</t>
         </is>
       </c>
-      <c r="C168" s="119" t="n"/>
-      <c r="D168" s="119" t="n"/>
-      <c r="E168" s="119" t="n"/>
-      <c r="F168" s="120" t="n"/>
-    </row>
-    <row r="169" ht="24" customHeight="1" s="175">
-      <c r="B169" s="144" t="inlineStr">
+      <c r="C167" s="119" t="n"/>
+      <c r="D167" s="119" t="n"/>
+      <c r="E167" s="119" t="n"/>
+      <c r="F167" s="120" t="n"/>
+    </row>
+    <row r="168" ht="24" customHeight="1" s="175">
+      <c r="B168" s="232" t="inlineStr">
         <is>
           <t>What went well — behaviors to repeat</t>
         </is>
       </c>
-      <c r="C169" s="126" t="n"/>
+      <c r="C168" s="126" t="n"/>
+      <c r="D168" s="126" t="n"/>
+      <c r="E168" s="126" t="n"/>
+      <c r="F168" s="122" t="n"/>
+    </row>
+    <row r="169" ht="32" customHeight="1" s="175">
+      <c r="B169" s="230" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C169" s="228" t="n"/>
       <c r="D169" s="126" t="n"/>
       <c r="E169" s="126" t="n"/>
       <c r="F169" s="122" t="n"/>
     </row>
     <row r="170" ht="32" customHeight="1" s="175">
-      <c r="B170" s="104" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C170" s="145" t="n"/>
+      <c r="B170" s="230" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C170" s="228" t="n"/>
       <c r="D170" s="126" t="n"/>
       <c r="E170" s="126" t="n"/>
       <c r="F170" s="122" t="n"/>
     </row>
     <row r="171" ht="32" customHeight="1" s="175">
-      <c r="B171" s="104" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C171" s="145" t="n"/>
+      <c r="B171" s="230" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C171" s="228" t="n"/>
       <c r="D171" s="126" t="n"/>
       <c r="E171" s="126" t="n"/>
       <c r="F171" s="122" t="n"/>
     </row>
-    <row r="172" ht="32" customHeight="1" s="175">
-      <c r="B172" s="104" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C172" s="145" t="n"/>
+    <row r="172" ht="24" customHeight="1" s="175">
+      <c r="B172" s="232" t="inlineStr">
+        <is>
+          <t>Improvement opportunities — behaviors to improve</t>
+        </is>
+      </c>
+      <c r="C172" s="126" t="n"/>
       <c r="D172" s="126" t="n"/>
       <c r="E172" s="126" t="n"/>
       <c r="F172" s="122" t="n"/>
     </row>
-    <row r="173" ht="24" customHeight="1" s="175">
-      <c r="B173" s="144" t="inlineStr">
-        <is>
-          <t>Improvement opportunities — behaviors to improve</t>
-        </is>
-      </c>
-      <c r="C173" s="126" t="n"/>
+    <row r="173" ht="32" customHeight="1" s="175">
+      <c r="B173" s="230" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C173" s="228" t="n"/>
       <c r="D173" s="126" t="n"/>
       <c r="E173" s="126" t="n"/>
       <c r="F173" s="122" t="n"/>
     </row>
     <row r="174" ht="32" customHeight="1" s="175">
-      <c r="B174" s="104" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C174" s="145" t="n"/>
+      <c r="B174" s="230" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C174" s="228" t="n"/>
       <c r="D174" s="126" t="n"/>
       <c r="E174" s="126" t="n"/>
       <c r="F174" s="122" t="n"/>
     </row>
     <row r="175" ht="32" customHeight="1" s="175">
-      <c r="B175" s="104" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C175" s="145" t="n"/>
+      <c r="B175" s="230" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C175" s="228" t="n"/>
       <c r="D175" s="126" t="n"/>
       <c r="E175" s="126" t="n"/>
       <c r="F175" s="122" t="n"/>
     </row>
-    <row r="176" ht="32" customHeight="1" s="175">
-      <c r="B176" s="104" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C176" s="145" t="n"/>
+    <row r="176" ht="24" customHeight="1" s="175">
+      <c r="B176" s="232" t="inlineStr">
+        <is>
+          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
+        </is>
+      </c>
+      <c r="C176" s="126" t="n"/>
       <c r="D176" s="126" t="n"/>
       <c r="E176" s="126" t="n"/>
       <c r="F176" s="122" t="n"/>
     </row>
-    <row r="177" ht="24" customHeight="1" s="175">
-      <c r="B177" s="144" t="inlineStr">
-        <is>
-          <t>Coaching recommendation — specific actions the agent should apply going forward</t>
-        </is>
-      </c>
+    <row r="177" ht="58" customHeight="1" s="175">
+      <c r="B177" s="228" t="n"/>
       <c r="C177" s="126" t="n"/>
       <c r="D177" s="126" t="n"/>
       <c r="E177" s="126" t="n"/>
       <c r="F177" s="122" t="n"/>
     </row>
-    <row r="178" ht="58" customHeight="1" s="175">
-      <c r="B178" s="145" t="n"/>
+    <row r="178" ht="20" customHeight="1" s="175">
+      <c r="B178" s="232" t="inlineStr">
+        <is>
+          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
+        </is>
+      </c>
       <c r="C178" s="126" t="n"/>
       <c r="D178" s="126" t="n"/>
       <c r="E178" s="126" t="n"/>
       <c r="F178" s="122" t="n"/>
     </row>
-    <row r="179" ht="20" customHeight="1" s="175">
-      <c r="B179" s="144" t="inlineStr">
-        <is>
-          <t>NEXT SESSION FOCUS   ·   Specific behaviors to practice before the next review</t>
-        </is>
-      </c>
-      <c r="C179" s="126" t="n"/>
+    <row r="179" ht="28" customHeight="1" s="175">
+      <c r="B179" s="228" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="C179" s="228" t="n"/>
       <c r="D179" s="126" t="n"/>
       <c r="E179" s="126" t="n"/>
       <c r="F179" s="122" t="n"/>
     </row>
     <row r="180" ht="28" customHeight="1" s="175">
-      <c r="B180" s="88" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="C180" s="145" t="n"/>
+      <c r="B180" s="228" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="C180" s="228" t="n"/>
       <c r="D180" s="126" t="n"/>
       <c r="E180" s="126" t="n"/>
       <c r="F180" s="122" t="n"/>
     </row>
     <row r="181" ht="28" customHeight="1" s="175">
-      <c r="B181" s="88" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="C181" s="145" t="n"/>
+      <c r="B181" s="228" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="C181" s="221" t="n"/>
       <c r="D181" s="126" t="n"/>
       <c r="E181" s="126" t="n"/>
       <c r="F181" s="122" t="n"/>
     </row>
-    <row r="182" ht="28" customHeight="1" s="175">
-      <c r="B182" s="88" t="inlineStr">
-        <is>
-          <t>3.</t>
-        </is>
-      </c>
-      <c r="C182" s="166" t="n"/>
-      <c r="D182" s="126" t="n"/>
-      <c r="E182" s="126" t="n"/>
-      <c r="F182" s="122" t="n"/>
-    </row>
-    <row r="183" ht="32" customHeight="1" s="175">
-      <c r="B183" s="153" t="inlineStr">
+    <row r="182" ht="32" customHeight="1" s="175">
+      <c r="B182" s="153" t="inlineStr">
         <is>
           <t>Q3 · What does this interaction tell us about training, process, or knowledge gaps across the team?</t>
         </is>
       </c>
-      <c r="C183" s="119" t="n"/>
-      <c r="D183" s="119" t="n"/>
-      <c r="E183" s="119" t="n"/>
-      <c r="F183" s="120" t="n"/>
-    </row>
-    <row r="184" ht="24" customHeight="1" s="175">
-      <c r="B184" s="144" t="inlineStr">
+      <c r="C182" s="119" t="n"/>
+      <c r="D182" s="119" t="n"/>
+      <c r="E182" s="119" t="n"/>
+      <c r="F182" s="120" t="n"/>
+    </row>
+    <row r="183" ht="24" customHeight="1" s="175">
+      <c r="B183" s="232" t="inlineStr">
         <is>
           <t>Organizational insights — training / process / KB / chatbot / tooling / product / contact-driver gaps</t>
         </is>
       </c>
+      <c r="C183" s="126" t="n"/>
+      <c r="D183" s="126" t="n"/>
+      <c r="E183" s="126" t="n"/>
+      <c r="F183" s="122" t="n"/>
+    </row>
+    <row r="184" ht="58" customHeight="1" s="175">
+      <c r="B184" s="228" t="n"/>
       <c r="C184" s="126" t="n"/>
       <c r="D184" s="126" t="n"/>
       <c r="E184" s="126" t="n"/>
       <c r="F184" s="122" t="n"/>
     </row>
-    <row r="185" ht="58" customHeight="1" s="175">
-      <c r="B185" s="145" t="n"/>
+    <row r="185" ht="24" customHeight="1" s="175">
+      <c r="B185" s="232" t="inlineStr">
+        <is>
+          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
+        </is>
+      </c>
       <c r="C185" s="126" t="n"/>
       <c r="D185" s="126" t="n"/>
       <c r="E185" s="126" t="n"/>
       <c r="F185" s="122" t="n"/>
     </row>
-    <row r="186" ht="24" customHeight="1" s="175">
-      <c r="B186" s="144" t="inlineStr">
-        <is>
-          <t>Multi-touch / journey notes — handoff quality, continuity, where the chain strengthened or broke</t>
-        </is>
-      </c>
+    <row r="186" ht="58" customHeight="1" s="175">
+      <c r="B186" s="228" t="n"/>
       <c r="C186" s="126" t="n"/>
       <c r="D186" s="126" t="n"/>
       <c r="E186" s="126" t="n"/>
       <c r="F186" s="122" t="n"/>
     </row>
-    <row r="187" ht="58" customHeight="1" s="175">
-      <c r="B187" s="145" t="n"/>
+    <row r="187" ht="24" customHeight="1" s="175">
+      <c r="B187" s="232" t="inlineStr">
+        <is>
+          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
+        </is>
+      </c>
       <c r="C187" s="126" t="n"/>
       <c r="D187" s="126" t="n"/>
       <c r="E187" s="126" t="n"/>
       <c r="F187" s="122" t="n"/>
     </row>
-    <row r="188" ht="24" customHeight="1" s="175">
-      <c r="B188" s="144" t="inlineStr">
-        <is>
-          <t>Final QA assessment — overall customer outcome, support quality, and coaching value</t>
-        </is>
-      </c>
+    <row r="188" ht="58" customHeight="1" s="175">
+      <c r="B188" s="228" t="n"/>
       <c r="C188" s="126" t="n"/>
       <c r="D188" s="126" t="n"/>
       <c r="E188" s="126" t="n"/>
       <c r="F188" s="122" t="n"/>
     </row>
-    <row r="189" ht="58" customHeight="1" s="175">
-      <c r="B189" s="145" t="n"/>
-      <c r="C189" s="126" t="n"/>
-      <c r="D189" s="126" t="n"/>
-      <c r="E189" s="126" t="n"/>
-      <c r="F189" s="122" t="n"/>
-    </row>
-    <row r="190" ht="24" customHeight="1" s="175"/>
-    <row r="191" ht="58" customHeight="1" s="175"/>
-    <row r="192" ht="20" customHeight="1" s="175"/>
-    <row r="193" ht="30" customHeight="1" s="175"/>
-    <row r="194" ht="58" customHeight="1" s="175"/>
-    <row r="195" ht="30" customHeight="1" s="175"/>
-    <row r="196" ht="24" customHeight="1" s="175"/>
+    <row r="189" ht="24" customHeight="1" s="175"/>
+    <row r="190" ht="58" customHeight="1" s="175"/>
+    <row r="191" ht="20" customHeight="1" s="175"/>
+    <row r="192" ht="30" customHeight="1" s="175"/>
+    <row r="193" ht="58" customHeight="1" s="175"/>
+    <row r="194" ht="30" customHeight="1" s="175"/>
+    <row r="195" ht="24" customHeight="1" s="175"/>
+    <row r="196" ht="32" customHeight="1" s="175"/>
     <row r="197" ht="32" customHeight="1" s="175"/>
     <row r="198" ht="32" customHeight="1" s="175"/>
-    <row r="199" ht="32" customHeight="1" s="175"/>
-    <row r="200" ht="24" customHeight="1" s="175"/>
+    <row r="199" ht="24" customHeight="1" s="175"/>
+    <row r="200" ht="32" customHeight="1" s="175"/>
     <row r="201" ht="32" customHeight="1" s="175"/>
     <row r="202" ht="32" customHeight="1" s="175"/>
-    <row r="203" ht="32" customHeight="1" s="175"/>
-    <row r="204" ht="24" customHeight="1" s="175"/>
-    <row r="205" ht="58" customHeight="1" s="175"/>
-    <row r="206" ht="20" customHeight="1" s="175"/>
+    <row r="203" ht="24" customHeight="1" s="175"/>
+    <row r="204" ht="58" customHeight="1" s="175"/>
+    <row r="205" ht="20" customHeight="1" s="175"/>
+    <row r="206" ht="28" customHeight="1" s="175"/>
     <row r="207" ht="28" customHeight="1" s="175"/>
     <row r="208" ht="28" customHeight="1" s="175"/>
-    <row r="209" ht="28" customHeight="1" s="175"/>
-    <row r="210" ht="32" customHeight="1" s="175"/>
-    <row r="211" ht="24" customHeight="1" s="175"/>
-    <row r="212" ht="58" customHeight="1" s="175"/>
-    <row r="213" ht="24" customHeight="1" s="175"/>
-    <row r="214" ht="58" customHeight="1" s="175"/>
-    <row r="215" ht="24" customHeight="1" s="175"/>
+    <row r="209" ht="32" customHeight="1" s="175"/>
+    <row r="210" ht="24" customHeight="1" s="175"/>
+    <row r="211" ht="58" customHeight="1" s="175"/>
+    <row r="212" ht="24" customHeight="1" s="175"/>
+    <row r="213" ht="58" customHeight="1" s="175"/>
+    <row r="214" ht="24" customHeight="1" s="175"/>
+    <row r="215" ht="58" customHeight="1" s="175"/>
     <row r="216" ht="58" customHeight="1" s="175"/>
-    <row r="217" ht="58" customHeight="1" s="175"/>
-    <row r="218" ht="24" customHeight="1" s="175"/>
-    <row r="219" ht="58" customHeight="1" s="175"/>
-    <row r="220" ht="24" customHeight="1" s="175"/>
+    <row r="217" ht="24" customHeight="1" s="175"/>
+    <row r="218" ht="58" customHeight="1" s="175"/>
+    <row r="219" ht="24" customHeight="1" s="175"/>
+    <row r="220" ht="58" customHeight="1" s="175"/>
     <row r="221" ht="58" customHeight="1" s="175"/>
   </sheetData>
-  <mergeCells count="178">
-    <mergeCell ref="B129:F129"/>
+  <mergeCells count="177">
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="D116:F116"/>
     <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B184:F184"/>
-    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="C125:F125"/>
+    <mergeCell ref="B71:F71"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
-    <mergeCell ref="B71:F71"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="C13:F13"/>
     <mergeCell ref="B52:F52"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="D37:F37"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
-    <mergeCell ref="D37:F37"/>
-    <mergeCell ref="B100:E100"/>
     <mergeCell ref="D152:F152"/>
     <mergeCell ref="D39:F39"/>
-    <mergeCell ref="B179:F179"/>
+    <mergeCell ref="D133:F133"/>
     <mergeCell ref="B166:F166"/>
-    <mergeCell ref="D133:F133"/>
-    <mergeCell ref="C172:F172"/>
-    <mergeCell ref="B94:C95"/>
+    <mergeCell ref="B32:F32"/>
     <mergeCell ref="B34:F34"/>
+    <mergeCell ref="D129:F129"/>
+    <mergeCell ref="B172:F172"/>
     <mergeCell ref="C171:F171"/>
     <mergeCell ref="B186:F186"/>
-    <mergeCell ref="B108:F108"/>
     <mergeCell ref="B168:F168"/>
     <mergeCell ref="B143:F143"/>
-    <mergeCell ref="C164:F164"/>
+    <mergeCell ref="B92:F92"/>
     <mergeCell ref="D119:F119"/>
+    <mergeCell ref="C173:F173"/>
     <mergeCell ref="D159:F159"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="D80:F80"/>
+    <mergeCell ref="B142:F142"/>
+    <mergeCell ref="C163:F163"/>
     <mergeCell ref="C43:F43"/>
-    <mergeCell ref="B142:F142"/>
-    <mergeCell ref="B112:E112"/>
     <mergeCell ref="D105:F105"/>
     <mergeCell ref="B144:F144"/>
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="D120:F120"/>
+    <mergeCell ref="D154:F154"/>
     <mergeCell ref="D41:F41"/>
-    <mergeCell ref="B125:F125"/>
-    <mergeCell ref="D154:F154"/>
     <mergeCell ref="B185:F185"/>
-    <mergeCell ref="D163:F163"/>
-    <mergeCell ref="D107:F107"/>
     <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B121:F121"/>
-    <mergeCell ref="D91:F91"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="D162:F162"/>
-    <mergeCell ref="B96:F96"/>
+    <mergeCell ref="D147:F147"/>
     <mergeCell ref="D156:F156"/>
     <mergeCell ref="B167:F167"/>
-    <mergeCell ref="C111:F111"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B176:F176"/>
     <mergeCell ref="D137:F137"/>
     <mergeCell ref="D106:F106"/>
     <mergeCell ref="C69:F69"/>
-    <mergeCell ref="C92:F92"/>
+    <mergeCell ref="C96:F96"/>
+    <mergeCell ref="B120:F120"/>
     <mergeCell ref="C175:F175"/>
+    <mergeCell ref="B107:F107"/>
     <mergeCell ref="D74:F74"/>
-    <mergeCell ref="D130:F130"/>
     <mergeCell ref="D68:F68"/>
+    <mergeCell ref="D83:F83"/>
     <mergeCell ref="D117:F117"/>
+    <mergeCell ref="D157:F157"/>
+    <mergeCell ref="C14:F14"/>
     <mergeCell ref="B57:F57"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="D157:F157"/>
+    <mergeCell ref="B82:F82"/>
     <mergeCell ref="C98:F98"/>
+    <mergeCell ref="B88:F88"/>
     <mergeCell ref="D67:F67"/>
-    <mergeCell ref="D110:F110"/>
+    <mergeCell ref="D132:F132"/>
     <mergeCell ref="D85:F85"/>
     <mergeCell ref="D54:F54"/>
     <mergeCell ref="B146:F146"/>
     <mergeCell ref="D60:F60"/>
+    <mergeCell ref="B187:F187"/>
     <mergeCell ref="D109:F109"/>
-    <mergeCell ref="B187:F187"/>
-    <mergeCell ref="B83:F83"/>
-    <mergeCell ref="C124:F124"/>
     <mergeCell ref="E16:F16"/>
+    <mergeCell ref="B124:F124"/>
     <mergeCell ref="D46:F46"/>
     <mergeCell ref="D158:F158"/>
-    <mergeCell ref="B189:F189"/>
     <mergeCell ref="B45:F45"/>
+    <mergeCell ref="D108:F108"/>
     <mergeCell ref="D86:F86"/>
-    <mergeCell ref="B173:F173"/>
+    <mergeCell ref="C123:F123"/>
     <mergeCell ref="B188:F188"/>
     <mergeCell ref="D104:F104"/>
+    <mergeCell ref="C110:F110"/>
     <mergeCell ref="D160:F160"/>
     <mergeCell ref="C181:F181"/>
+    <mergeCell ref="E130:F130"/>
     <mergeCell ref="D136:F136"/>
+    <mergeCell ref="C91:F91"/>
+    <mergeCell ref="B141:F141"/>
     <mergeCell ref="D150:F150"/>
     <mergeCell ref="C174:F174"/>
+    <mergeCell ref="D78:F78"/>
     <mergeCell ref="D87:F87"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="D122:F122"/>
+    <mergeCell ref="C179:F179"/>
     <mergeCell ref="D58:F58"/>
     <mergeCell ref="B145:F145"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="D121:F121"/>
     <mergeCell ref="D73:F73"/>
+    <mergeCell ref="D51:F51"/>
     <mergeCell ref="D42:F42"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="D113:F113"/>
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C128:F128"/>
-    <mergeCell ref="B147:F147"/>
     <mergeCell ref="C97:F97"/>
     <mergeCell ref="B178:F178"/>
+    <mergeCell ref="D148:F148"/>
     <mergeCell ref="C20:F20"/>
-    <mergeCell ref="D123:F123"/>
-    <mergeCell ref="D148:F148"/>
     <mergeCell ref="D35:F35"/>
+    <mergeCell ref="B128:F128"/>
     <mergeCell ref="D59:F59"/>
     <mergeCell ref="D115:F115"/>
+    <mergeCell ref="B93:C94"/>
+    <mergeCell ref="B131:F131"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="B183:F183"/>
     <mergeCell ref="C127:F127"/>
-    <mergeCell ref="C176:F176"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="B164:F164"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="D140:F140"/>
     <mergeCell ref="D84:F84"/>
-    <mergeCell ref="D140:F140"/>
+    <mergeCell ref="D155:F155"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="D155:F155"/>
     <mergeCell ref="D36:F36"/>
     <mergeCell ref="D149:F149"/>
-    <mergeCell ref="C131:D131"/>
-    <mergeCell ref="D77:F77"/>
-    <mergeCell ref="B113:F113"/>
+    <mergeCell ref="D101:F101"/>
+    <mergeCell ref="B99:E99"/>
     <mergeCell ref="D151:F151"/>
+    <mergeCell ref="B100:F100"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="B165:F165"/>
-    <mergeCell ref="D141:F141"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="D135:F135"/>
     <mergeCell ref="D48:F48"/>
     <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B93:F93"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="C170:F170"/>
+    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D103:F103"/>
-    <mergeCell ref="D72:F72"/>
     <mergeCell ref="D134:F134"/>
+    <mergeCell ref="B77:F77"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="D118:F118"/>
     <mergeCell ref="D161:F161"/>
-    <mergeCell ref="B132:F132"/>
-    <mergeCell ref="B101:F101"/>
     <mergeCell ref="D114:F114"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D64:F64"/>
+    <mergeCell ref="C126:F126"/>
     <mergeCell ref="D38:F38"/>
-    <mergeCell ref="C126:F126"/>
-    <mergeCell ref="B78:F78"/>
+    <mergeCell ref="B182:F182"/>
+    <mergeCell ref="D89:F89"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="B112:F112"/>
+    <mergeCell ref="B70:E70"/>
     <mergeCell ref="D79:F79"/>
-    <mergeCell ref="B70:E70"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="D88:F88"/>
     <mergeCell ref="D153:F153"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="C55:F55"/>
     <mergeCell ref="B40:F40"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="C99:F99"/>
     <mergeCell ref="D63:F63"/>
     <mergeCell ref="C180:F180"/>
     <mergeCell ref="D90:F90"/>
+    <mergeCell ref="B95:F95"/>
     <mergeCell ref="B177:F177"/>
-    <mergeCell ref="B89:F89"/>
     <mergeCell ref="D65:F65"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="B169:F169"/>
     <mergeCell ref="D139:F139"/>
-    <mergeCell ref="C182:F182"/>
-    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="C169:F169"/>
     <mergeCell ref="D49:F49"/>
   </mergeCells>
   <conditionalFormatting sqref="C21:C25">
@@ -6686,18 +6721,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C75">
-    <cfRule type="cellIs" priority="22" operator="lessThanOrEqual" dxfId="0">
-      <formula>2</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="23" operator="equal" dxfId="1">
-      <formula>3</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="2">
-      <formula>4</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C81:C85">
+  <conditionalFormatting sqref="C80:C84">
     <cfRule type="cellIs" priority="25" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6708,7 +6732,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C88">
+  <conditionalFormatting sqref="C87">
     <cfRule type="cellIs" priority="28" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6719,7 +6743,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C94:C99">
+  <conditionalFormatting sqref="C93:C98">
     <cfRule type="cellIs" priority="31" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6730,7 +6754,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C102">
+  <conditionalFormatting sqref="C101">
     <cfRule type="cellIs" priority="34" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6741,7 +6765,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C108:C114">
+  <conditionalFormatting sqref="C107:C113">
     <cfRule type="cellIs" priority="37" operator="equal" dxfId="2">
       <formula>"Met"</formula>
     </cfRule>
@@ -6752,7 +6776,7 @@
       <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C117">
+  <conditionalFormatting sqref="C116">
     <cfRule type="cellIs" priority="40" operator="lessThanOrEqual" dxfId="0">
       <formula>2</formula>
     </cfRule>
@@ -6763,7 +6787,7 @@
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C134:C141">
+  <conditionalFormatting sqref="C133:C140">
     <cfRule type="cellIs" priority="55" operator="equal" dxfId="101">
       <formula>"Missed"</formula>
     </cfRule>
@@ -6771,12 +6795,12 @@
       <formula>"Partial"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C142:C152">
+  <conditionalFormatting sqref="C141:C151">
     <cfRule type="cellIs" priority="51" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C153">
+  <conditionalFormatting sqref="C152">
     <cfRule type="expression" priority="52" dxfId="0">
       <formula>ISNUMBER(SEARCH("YES",C152))</formula>
     </cfRule>
@@ -6784,7 +6808,7 @@
       <formula>NOT(ISNUMBER(SEARCH("YES",C152)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E129">
+  <conditionalFormatting sqref="E128">
     <cfRule type="cellIs" priority="44" operator="between" dxfId="29">
       <formula>0.7</formula>
       <formula>0.8499</formula>
@@ -6796,7 +6820,7 @@
       <formula>0.85</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E138">
+  <conditionalFormatting sqref="E137">
     <cfRule type="expression" priority="50" dxfId="2">
       <formula>E137="OK"</formula>
     </cfRule>
@@ -6804,7 +6828,7 @@
       <formula>E137&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F122:F128">
+  <conditionalFormatting sqref="F121:F127">
     <cfRule type="cellIs" priority="46" operator="equal" dxfId="9">
       <formula>"Strong"</formula>
     </cfRule>
@@ -6816,13 +6840,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation sqref="C36 C37 C38 C39 C47 C48 C49 C50 C51 C59 C60 C61 C62 C63 C64 C65 C73 C74 C76 C77 C85 C86 C87 C88 C103 C104 C105 C106 C107 C115 C116 C117 C118 C119 C120" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C36 C37 C38 C39 C47 C48 C49 C50 C51 C59 C60 C61 C62 C63 C64 C65 C73 C74 C75 C76 C84 C85 C86 C87 C102 C103 C104 C105 C106 C114 C115 C116 C117 C118 C119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C42 C54 C68 C80 C91 C110 C123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
+    <dataValidation sqref="C42 C54 C68 C79 C90 C109 C122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C130 C153:C163 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C129 C152:C162 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6837,16 +6861,16 @@
     <dataValidation sqref="E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Within SLA,Breached,N.A."</formula1>
     </dataValidation>
-    <dataValidation sqref="C126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Successful Resolution,Partial Resolution,Appropriate Escalation,Ownership Gap,Unresolved"</formula1>
     </dataValidation>
-    <dataValidation sqref="C127" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C126" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>_xlfn._LONGTEXT("Issue resolved,Proper RMA initiated (in-warranty / approved exception),Valid escalation submitted,Known limitation explained accurately,Customer educated with actionable next steps,Valid self-help guidance provided (out-of-warranty),Upgrade path recommend","ed appropriately (out-of-warranty),Customer declined further troubleshooting after reasonable effort,None achieved")</formula1>
     </dataValidation>
-    <dataValidation sqref="C131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Callback attempt,Follow-up email,Private note documenting actions,Documented why follow-up not possible,None,N.A. — no disconnect"</formula1>
     </dataValidation>
-    <dataValidation sqref="C149:C151" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C148:C150" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid selection" error="Please choose Level 1 or Level 2." promptTitle="Agent Level" prompt="Select Level 1 for front-line support agents or Level 2 for senior/escalation agents." type="list">
@@ -15859,8 +15883,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Clean template: remove case-specific notes, fix Row 61 wording
- Cleared pre-filled evaluation text from 7 observation rows (43, 55,
  69, 80, 91, 110, 123) — Stell journey notes that were saved back
  into the template by accident
- Row 61 Communication: reworded from 'Use appropriate language, as
  needed' to 'Used language appropriate to the customer's level and
  confirmed understanding throughout'

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4566,11 +4566,7 @@
       <c r="F42" s="122" t="n"/>
     </row>
     <row r="43" ht="36" customHeight="1" s="175">
-      <c r="B43" s="79" t="inlineStr">
-        <is>
-          <t>Score reflects the cumulative effect of this touch within the 8-month journey: the Nov 24, 2025 hardware/RMA determination remains undelivered, and the case culminates here in executive-level escalation with no path forward offered.</t>
-        </is>
-      </c>
+      <c r="B43" s="79" t="n"/>
       <c r="C43" s="145" t="n"/>
       <c r="D43" s="126" t="n"/>
       <c r="E43" s="126" t="n"/>
@@ -4714,11 +4710,7 @@
       <c r="F54" s="122" t="n"/>
     </row>
     <row r="55" ht="36" customHeight="1" s="175">
-      <c r="B55" s="79" t="inlineStr">
-        <is>
-          <t>Individual diagnostic steps (signal/backhaul check, swap-test proposal) were sound, but the unvalidated reversal of a prior CAT-level conclusion undermines technical credibility.</t>
-        </is>
-      </c>
+      <c r="B55" s="79" t="n"/>
       <c r="C55" s="145" t="n"/>
       <c r="D55" s="126" t="n"/>
       <c r="E55" s="126" t="n"/>
@@ -4794,7 +4786,7 @@
     <row r="61" ht="28" customHeight="1" s="175">
       <c r="B61" s="76" t="inlineStr">
         <is>
-          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+          <t>Used language appropriate to the customer's level and confirmed understanding throughout</t>
         </is>
       </c>
       <c r="C61" s="105" t="n"/>
@@ -4886,11 +4878,7 @@
       <c r="F68" s="122" t="n"/>
     </row>
     <row r="69" ht="36" customHeight="1" s="175">
-      <c r="B69" s="79" t="inlineStr">
-        <is>
-          <t>The core communication failure is the unacknowledged expectation gap: the customer's RMA expectation from Nov 24 was never reconciled with the renewed troubleshooting requests.</t>
-        </is>
-      </c>
+      <c r="B69" s="79" t="n"/>
       <c r="C69" s="145" t="n"/>
       <c r="D69" s="126" t="n"/>
       <c r="E69" s="126" t="n"/>
@@ -5025,11 +5013,7 @@
       <c r="F79" s="122" t="n"/>
     </row>
     <row r="80" ht="36" customHeight="1" s="175">
-      <c r="B80" s="226" t="inlineStr">
-        <is>
-          <t>The escalation itself was a positive ownership step, but follow-through collapsed: the customer's direct questions and the SLA commitment were both left unmet, requiring PMO intervention.</t>
-        </is>
-      </c>
+      <c r="B80" s="226" t="n"/>
       <c r="C80" s="228" t="n"/>
       <c r="D80" s="126" t="n"/>
       <c r="E80" s="126" t="n"/>
@@ -5164,11 +5148,7 @@
       <c r="F90" s="122" t="n"/>
     </row>
     <row r="91" ht="36" customHeight="1" s="175">
-      <c r="B91" s="226" t="inlineStr">
-        <is>
-          <t>The escalation decision and routing were correct; the SLA management and handoff completeness after escalation were not.</t>
-        </is>
-      </c>
+      <c r="B91" s="226" t="n"/>
       <c r="C91" s="228" t="n"/>
       <c r="D91" s="126" t="n"/>
       <c r="E91" s="126" t="n"/>
@@ -5385,11 +5365,7 @@
       <c r="F109" s="122" t="n"/>
     </row>
     <row r="110" ht="36" customHeight="1" s="175">
-      <c r="B110" s="226" t="inlineStr">
-        <is>
-          <t>Professionalism was maintained, but the customer's confidence and engagement collapsed by the end of this touch.</t>
-        </is>
-      </c>
+      <c r="B110" s="226" t="n"/>
       <c r="C110" s="228" t="n"/>
       <c r="D110" s="126" t="n"/>
       <c r="E110" s="126" t="n"/>
@@ -5546,11 +5522,7 @@
       <c r="F122" s="122" t="n"/>
     </row>
     <row r="123" ht="36" customHeight="1" s="175">
-      <c r="B123" s="226" t="inlineStr">
-        <is>
-          <t>Escalation steps are documented, but the case record does not carry the full history forward, and ticket status does not reflect reality.</t>
-        </is>
-      </c>
+      <c r="B123" s="226" t="n"/>
       <c r="C123" s="228" t="n"/>
       <c r="D123" s="126" t="n"/>
       <c r="E123" s="126" t="n"/>
@@ -6469,26 +6441,26 @@
     <mergeCell ref="D76:F76"/>
     <mergeCell ref="D116:F116"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B71:F71"/>
     <mergeCell ref="C125:F125"/>
-    <mergeCell ref="B71:F71"/>
+    <mergeCell ref="B131:F131"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
+    <mergeCell ref="B184:F184"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B184:F184"/>
+    <mergeCell ref="B52:F52"/>
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="B52:F52"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D102:F102"/>
+    <mergeCell ref="D39:F39"/>
     <mergeCell ref="D152:F152"/>
-    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="B166:F166"/>
     <mergeCell ref="D133:F133"/>
-    <mergeCell ref="B166:F166"/>
-    <mergeCell ref="B32:F32"/>
     <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B172:F172"/>
     <mergeCell ref="D129:F129"/>
-    <mergeCell ref="B172:F172"/>
     <mergeCell ref="C171:F171"/>
     <mergeCell ref="B186:F186"/>
     <mergeCell ref="B168:F168"/>
@@ -6498,9 +6470,9 @@
     <mergeCell ref="C173:F173"/>
     <mergeCell ref="D159:F159"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="C43:F43"/>
     <mergeCell ref="B142:F142"/>
     <mergeCell ref="C163:F163"/>
-    <mergeCell ref="C43:F43"/>
     <mergeCell ref="D105:F105"/>
     <mergeCell ref="B144:F144"/>
     <mergeCell ref="E12:F12"/>
@@ -6526,8 +6498,8 @@
     <mergeCell ref="D68:F68"/>
     <mergeCell ref="D83:F83"/>
     <mergeCell ref="D117:F117"/>
+    <mergeCell ref="C14:F14"/>
     <mergeCell ref="D157:F157"/>
-    <mergeCell ref="C14:F14"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B82:F82"/>
     <mergeCell ref="C98:F98"/>
@@ -6585,15 +6557,14 @@
     <mergeCell ref="D59:F59"/>
     <mergeCell ref="D115:F115"/>
     <mergeCell ref="B93:C94"/>
-    <mergeCell ref="B131:F131"/>
     <mergeCell ref="D138:F138"/>
     <mergeCell ref="B183:F183"/>
     <mergeCell ref="C127:F127"/>
     <mergeCell ref="C80:F80"/>
     <mergeCell ref="B164:F164"/>
     <mergeCell ref="E7:F7"/>
+    <mergeCell ref="D84:F84"/>
     <mergeCell ref="D140:F140"/>
-    <mergeCell ref="D84:F84"/>
     <mergeCell ref="D155:F155"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="D36:F36"/>
@@ -6621,10 +6592,10 @@
     <mergeCell ref="D114:F114"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="D64:F64"/>
+    <mergeCell ref="D38:F38"/>
     <mergeCell ref="C126:F126"/>
-    <mergeCell ref="D38:F38"/>
+    <mergeCell ref="D89:F89"/>
     <mergeCell ref="B182:F182"/>
-    <mergeCell ref="D89:F89"/>
     <mergeCell ref="C130:D130"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B70:E70"/>
@@ -6641,6 +6612,7 @@
     <mergeCell ref="B177:F177"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="D139:F139"/>
+    <mergeCell ref="B32:F32"/>
     <mergeCell ref="C169:F169"/>
     <mergeCell ref="D49:F49"/>
   </mergeCells>
@@ -15883,8 +15855,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Row 74 Ownership: sharpen wording to remove overlap with Row 75
'Followed through on all commitments made during the interaction'
— Row 74 is now purely backward-looking (accountability for what was
promised); Row 75 remains the sole forward-looking indicator (what
the customer knows about next steps and timelines).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4943,7 +4943,7 @@
     <row r="74" ht="28" customHeight="1" s="175">
       <c r="B74" s="76" t="inlineStr">
         <is>
-          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+          <t>Followed through on all commitments made during the interaction</t>
         </is>
       </c>
       <c r="C74" s="105" t="n"/>
@@ -6446,9 +6446,9 @@
     <mergeCell ref="B131:F131"/>
     <mergeCell ref="D53:F53"/>
     <mergeCell ref="D75:F75"/>
-    <mergeCell ref="B184:F184"/>
     <mergeCell ref="D47:F47"/>
     <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B184:F184"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="D37:F37"/>
@@ -15855,8 +15855,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Sync Scoring Guide indicator labels and refocus Ownership commitments block
- Sync 3 indicator labels to the current form wording: Communication
  'Used language appropriate to the customer's level...' (Row 61),
  Ownership 'Followed through on all commitments made during the
  interaction' (Row 74), and Documentation punctuation.
- Refocus the Ownership commitments block (guide R72-75) onto commitment
  follow-through, removing 'path forward / next steps' language that now
  belongs to the separate Row 75 indicator. All 35 labels verified in sync.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -7845,7 +7845,7 @@
       <c r="A48" s="172" t="n"/>
       <c r="B48" s="171" t="inlineStr">
         <is>
-          <t>Use appropriate language, as needed, and confirmed customer understanding</t>
+          <t>Used language appropriate to the customer's level and confirmed understanding throughout</t>
         </is>
       </c>
       <c r="C48" s="63" t="inlineStr">
@@ -8306,7 +8306,7 @@
       <c r="A72" s="172" t="n"/>
       <c r="B72" s="171" t="inlineStr">
         <is>
-          <t>Commitments made were followed through, and a clear path forward was created for the customer.</t>
+          <t>Followed through on all commitments made during the interaction</t>
         </is>
       </c>
       <c r="C72" s="63" t="inlineStr">
@@ -8316,12 +8316,12 @@
       </c>
       <c r="D72" s="64" t="inlineStr">
         <is>
-          <t>Every commitment made during the interaction was executed within the call or documented with a specific owner and timeline. Customer left with a defined, actionable next step.</t>
+          <t>Every commitment made during the interaction was honored — executed within the call, or documented with a specific owner and timeline so it would be carried out afterward.</t>
         </is>
       </c>
       <c r="E72" s="65" t="inlineStr">
         <is>
-          <t>Agent committed to submitting the escalation before end of day, told the customer what L2 would do and when to expect contact, and updated the ticket accordingly before closing. → Met.</t>
+          <t>Agent committed to submitting the escalation before end of day, submitted it as promised, and updated the ticket accordingly before closing. → Met.</t>
         </is>
       </c>
     </row>
@@ -8335,12 +8335,12 @@
       </c>
       <c r="D73" s="67" t="inlineStr">
         <is>
-          <t>Path forward was defined but vague — no specifics on who, when, or what. Or a commitment was made verbally but not documented in the case.</t>
+          <t>A commitment was made but only partially honored — fulfilled late, fulfilled without confirming back to the customer, or made verbally without being documented in the case.</t>
         </is>
       </c>
       <c r="E73" s="68" t="inlineStr">
         <is>
-          <t>Agent told the customer 'someone will follow up with you' but did not specify the team, timeline, or the nature of the follow-up. → Partial.</t>
+          <t>Agent committed to emailing the customer setup instructions but never logged it in the ticket, so there is no record the email was sent. → Partial.</t>
         </is>
       </c>
     </row>
@@ -8354,7 +8354,7 @@
       </c>
       <c r="D74" s="70" t="inlineStr">
         <is>
-          <t>Agent made a commitment that was not kept and not documented. Customer ends the interaction with no defined next step.</t>
+          <t>A commitment the agent made was not kept and not documented — the customer was left waiting on something that never happened.</t>
         </is>
       </c>
       <c r="E74" s="71" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="D75" s="73" t="inlineStr">
         <is>
-          <t>Not applicable. A path forward is always relevant.</t>
+          <t>N/A only when the agent made no commitments during the interaction — there is nothing to follow through on.</t>
         </is>
       </c>
       <c r="E75" s="74" t="n"/>
@@ -9458,7 +9458,7 @@
       <c r="A132" s="172" t="n"/>
       <c r="B132" s="171" t="inlineStr">
         <is>
-          <t>Captured agent reasoning — escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action</t>
+          <t>Captured agent reasoning - escalation justification, offline recommendations provided by colleagues and other support POCs especially if no private notes applicable to step/action.</t>
         </is>
       </c>
       <c r="C132" s="63" t="inlineStr">
@@ -15938,8 +15938,8 @@
     <mergeCell ref="I59:N59"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A56:B56"/>
-    <mergeCell ref="A54:P54"/>
     <mergeCell ref="A53:P53"/>
     <mergeCell ref="A60:N60"/>
     <mergeCell ref="I56:N56"/>

</xml_diff>

<commit_message>
Add Auto-Zero Guide sheet, trigger tooltips, and N.A. weight redistribution
- New 'Auto-Zero Guide' sheet documenting each A-K trigger's Against-Agent
  (forces agent Quality Score to 0%) and Against-Team (informs Journey
  Outcome / Continuity) criteria; Against-Agent definitions added as hover
  tooltips on the Scoring Form auto-zero items (C152:C162).
- Redistribute an N.A. category's weight across the applicable categories:
  each weighted contribution = (score/5) x weight / (sum of applicable
  weights). When all 7 categories apply this is unchanged; when a category
  is N.A. (e.g. Escalation when none was needed), the agent is scored only
  on applicable competencies and a flawless case still reaches 100%.
  Verified in Excel across all-apply / N.A. / auto-zero scenarios.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -10,10 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Form" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multi-Touch Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auto-Zero Guide" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -355,6 +356,29 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="36">
     <fill>
@@ -534,7 +558,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -871,11 +895,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="236">
+  <cellXfs count="242">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1541,6 +1579,24 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="3" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="25" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3253,6 +3309,21 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>QA</author>
+  </authors>
+  <commentList>
+    <comment ref="E31" authorId="0" shapeId="0">
+      <text>
+        <t>Weighted total redistributes any N.A. category's weight across the applicable categories: each contribution = (score/5) x weight / (sum of weights of categories that have a score). When all 7 categories apply this equals the standard weighting; when a category is N.A. (e.g. Escalation when none was needed), the total is scored only on applicable competencies and a flawless case still reaches 100%.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4318,7 +4389,7 @@
         <v/>
       </c>
       <c r="E24" s="93">
-        <f>IF(D24="","",(D24/5)*C24)</f>
+        <f>IF(D24="","",(D24/5)*C24/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F24" s="94">
@@ -4340,7 +4411,7 @@
         <v/>
       </c>
       <c r="E25" s="98">
-        <f>IF(D25="","",(D25/5)*C25)</f>
+        <f>IF(D25="","",(D25/5)*C25/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F25" s="99">
@@ -4362,7 +4433,7 @@
         <v/>
       </c>
       <c r="E26" s="93">
-        <f>IF(D26="","",(D26/5)*C26)</f>
+        <f>IF(D26="","",(D26/5)*C26/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F26" s="94">
@@ -4384,7 +4455,7 @@
         <v/>
       </c>
       <c r="E27" s="98">
-        <f>IF(D27="","",(D27/5)*C27)</f>
+        <f>IF(D27="","",(D27/5)*C27/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F27" s="99">
@@ -4406,7 +4477,7 @@
         <v/>
       </c>
       <c r="E28" s="93">
-        <f>IF(D28="","",(D28/5)*C28)</f>
+        <f>IF(D28="","",(D28/5)*C28/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F28" s="94">
@@ -4428,7 +4499,7 @@
         <v/>
       </c>
       <c r="E29" s="98">
-        <f>IF(D29="","",(D29/5)*C29)</f>
+        <f>IF(D29="","",(D29/5)*C29/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F29" s="99">
@@ -4450,7 +4521,7 @@
         <v/>
       </c>
       <c r="E30" s="93">
-        <f>IF(D30="","",(D30/5)*C30)</f>
+        <f>IF(D30="","",(D30/5)*C30/SUMPRODUCT(($D$24:$D$30&lt;&gt;"")*$C$24:$C$30))</f>
         <v/>
       </c>
       <c r="F30" s="94">
@@ -6873,14 +6944,14 @@
       <formula>AND($E$31&lt;&gt;"",$E$31&lt;0.7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="19">
+  <dataValidations count="30">
     <dataValidation sqref="C36 C37 C38 C39 C47 C48 C49 C50 C51 C59 C60 C61 C62 C63 C64 C65 C73 C74 C75 C76 C84 C85 C86 C87 C102 C103 C104 C105 C106 C114 C115 C116 C117 C118 C119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Met,Partial,Missed,N.A."</formula1>
     </dataValidation>
     <dataValidation sqref="C42 C54 C68 C79 C90 C109 C122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C129 C152:C162 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C129 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6931,8 +7002,42 @@
     <dataValidation sqref="C123:F123" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Override reason" prompt="Required only if you entered an override score above. Explain why the indicator-based auto score does not reflect the true outcome (context, customer behavior, judgment, etc.)." type="textLength" operator="lessThanOrEqual">
       <formula1>1000</formula1>
     </dataValidation>
+    <dataValidation sqref="C152" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent disconnects, leaves the session, or fails to return without valid reason or required closure steps. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C153" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent intentionally avoids handling the interaction, transfers unnecessarily, or uses tactics to end/deflect the contact. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C154" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent uses rude, dismissive, sarcastic, argumentative, or unprofessional language/tone. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C155" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent fails to de-escalate appropriately, refuses a valid escalation, or escalates unnecessarily due to poor handling. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C156" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent misses the required step to request or confirm the customer's email address when the process requires it. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C157" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent knowingly participates in, ignores, or enables fraudulent activity, or fails required fraud controls within their role. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C158" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent applies excessive sales pressure, ignores refusal, or uses manipulative tactics beyond approved selling behavior. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C159" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent releases or disconnects the line without proper closure, customer consent, or valid process reason. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C160" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent makes or promises callbacks outside approved hours, or fails to observe required callback windows. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C161" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent fails to follow PCI/InfoSec rules, including improper collection, disclosure, storage, or verification of sensitive information. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C162" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Choose No or Yes." promptTitle="Against Agent (Auto-Zero)" prompt="Agent fails to resolve an issue they could have resolved on first contact due to error, incomplete handling, or wrong information. — triggers this agent's auto-zero (Quality Score → 0%). See the Auto-Zero Guide sheet for team-level handling." type="list">
+      <formula1>"No,Yes"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -10497,6 +10602,282 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="175" min="1" max="1"/>
+    <col width="62" customWidth="1" style="175" min="2" max="2"/>
+    <col width="80" customWidth="1" style="175" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" s="175">
+      <c r="A1" s="236" t="inlineStr">
+        <is>
+          <t>AUTO-ZERO GUIDE — Trigger Definitions (Agent &amp; Team)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="46" customHeight="1" s="175">
+      <c r="A2" s="237" t="inlineStr">
+        <is>
+          <t>'Against Agent' = what forces the individual agent's Quality Score to 0% (Scoring Form §7 Auto-Zero, items A–K).   'Against Team' = how the same issue is weighed across the journey — used to INFORM the Journey Outcome &amp; Continuity of Support (0–5) scores on the Case Tracker. The team column is graded guidance; it does not auto-zero the team score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="175">
+      <c r="A3" s="238" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B3" s="238" t="inlineStr">
+        <is>
+          <t>Against Agent  (forces agent Quality Score → 0%)</t>
+        </is>
+      </c>
+      <c r="C3" s="238" t="inlineStr">
+        <is>
+          <t>Against Team  (informs Journey Outcome / Continuity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1" s="175">
+      <c r="A4" s="239" t="inlineStr">
+        <is>
+          <t>A.  Call / Session Abandonment</t>
+        </is>
+      </c>
+      <c r="B4" s="240" t="inlineStr">
+        <is>
+          <t>Agent disconnects, leaves the session, or fails to return without valid reason or required closure steps.</t>
+        </is>
+      </c>
+      <c r="C4" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the disconnected call.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1" s="175">
+      <c r="A5" s="239" t="inlineStr">
+        <is>
+          <t>B.  Call / Session Avoidance / Evasion</t>
+        </is>
+      </c>
+      <c r="B5" s="240" t="inlineStr">
+        <is>
+          <t>Agent intentionally avoids handling the interaction, transfers unnecessarily, or uses tactics to end/deflect the contact.</t>
+        </is>
+      </c>
+      <c r="C5" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the disconnected call.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1" s="175">
+      <c r="A6" s="239" t="inlineStr">
+        <is>
+          <t>C.  Discourtesy</t>
+        </is>
+      </c>
+      <c r="B6" s="240" t="inlineStr">
+        <is>
+          <t>Agent uses rude, dismissive, sarcastic, argumentative, or unprofessional language/tone.</t>
+        </is>
+      </c>
+      <c r="C6" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about a discourteous agent.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1" s="175">
+      <c r="A7" s="239" t="inlineStr">
+        <is>
+          <t>D.  Escalation</t>
+        </is>
+      </c>
+      <c r="B7" s="240" t="inlineStr">
+        <is>
+          <t>Agent fails to de-escalate appropriately, refuses a valid escalation, or escalates unnecessarily due to poor handling.</t>
+        </is>
+      </c>
+      <c r="C7" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about a missed escalation.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1" s="175">
+      <c r="A8" s="239" t="inlineStr">
+        <is>
+          <t>E.  Failure to ask for the email address</t>
+        </is>
+      </c>
+      <c r="B8" s="240" t="inlineStr">
+        <is>
+          <t>Agent misses the required step to request or confirm the customer's email address when the process requires it.</t>
+        </is>
+      </c>
+      <c r="C8" s="240" t="inlineStr">
+        <is>
+          <t>Continued the interaction without asking for the email address — just picking up from where the previous agent had left off, without gathering the missing email address on record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1" s="175">
+      <c r="A9" s="239" t="inlineStr">
+        <is>
+          <t>F.  Fraud</t>
+        </is>
+      </c>
+      <c r="B9" s="240" t="inlineStr">
+        <is>
+          <t>Agent knowingly participates in, ignores, or enables fraudulent activity, or fails required fraud controls within their role.</t>
+        </is>
+      </c>
+      <c r="C9" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the fraudulent action from a previous contact.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1" s="175">
+      <c r="A10" s="239" t="inlineStr">
+        <is>
+          <t>G.  Hard-selling</t>
+        </is>
+      </c>
+      <c r="B10" s="240" t="inlineStr">
+        <is>
+          <t>Agent applies excessive sales pressure, ignores refusal, or uses manipulative tactics beyond approved selling behavior.</t>
+        </is>
+      </c>
+      <c r="C10" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the hard-selling from a previous contact.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="84" customHeight="1" s="175">
+      <c r="A11" s="239" t="inlineStr">
+        <is>
+          <t>H.  Line Release</t>
+        </is>
+      </c>
+      <c r="B11" s="240" t="inlineStr">
+        <is>
+          <t>Agent releases or disconnects the line without proper closure, customer consent, or valid process reason.</t>
+        </is>
+      </c>
+      <c r="C11" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the previous agent(s) hanging up the call.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1" s="175">
+      <c r="A12" s="239" t="inlineStr">
+        <is>
+          <t>I.  Non-Adherence to Callback Hours</t>
+        </is>
+      </c>
+      <c r="B12" s="240" t="inlineStr">
+        <is>
+          <t>Agent makes or promises callbacks outside approved hours, or fails to observe required callback windows.</t>
+        </is>
+      </c>
+      <c r="C12" s="240" t="inlineStr">
+        <is>
+          <t>Team members involved failed to document and/or notify the team on agreed callback hours.
+Failed to act on the case offline to ensure timely follow-up or callback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="84" customHeight="1" s="175">
+      <c r="A13" s="239" t="inlineStr">
+        <is>
+          <t>J.  Non-Adherence to PCI and Information Security Standards</t>
+        </is>
+      </c>
+      <c r="B13" s="240" t="inlineStr">
+        <is>
+          <t>Agent fails to follow PCI/InfoSec rules, including improper collection, disclosure, storage, or verification of sensitive information.</t>
+        </is>
+      </c>
+      <c r="C13" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about any PCI/InfoSec violations.
+Missed to reassure the customer that this does not align with our support standards.
+Mentioned negative comments about the previous agent the customer complained about.
+Dismissed the complaint altogether and did not advise that the matter can be investigated and appropriate action taken if confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="104" customHeight="1" s="175">
+      <c r="A14" s="239" t="inlineStr">
+        <is>
+          <t>K.  Non-First Call Resolution</t>
+        </is>
+      </c>
+      <c r="B14" s="240" t="inlineStr">
+        <is>
+          <t>Agent fails to resolve an issue they could have resolved on first contact due to error, incomplete handling, or wrong information.</t>
+        </is>
+      </c>
+      <c r="C14" s="240" t="inlineStr">
+        <is>
+          <t>Failed to acknowledge the customer's concern about the inability to get a resolution from a previous contact.
+Mentioned negative comments about the previous agent the customer complained about.
+This should be counted against the TEAM score if the repeat call was caused beyond the original agent. Multiple interactions in the journey were observed, with a per-agent opportunity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1" s="175">
+      <c r="A15" s="241" t="inlineStr">
+        <is>
+          <t>Note: items I and J mirror the compliance gates on the Scoring Form (Adherence to Callback Hours / PCI). The gate asks 'did the agent adhere?' (No → auto-zero); the A–K item asks 'did the violation occur?' (Yes → auto-zero).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11370,7 +11751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14362,7 +14743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16063,7 +16444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix indicator weights for 5 new gap indicators
Cat 1 (Resolution): assign H-weights 2,2 to Gap 4 (KB misuse) and
  Gap 1 (out-of-warranty); expand auto-score formula from C36:C39
  to C36:C41 with weights {3,2,1,2,2,2}

Cat 4 (Customer Ownership): assign H-weights 2,2 to Gap 3 (repeat
  contact) and Gap 5 (handoff quality); expand auto-score formula
  from C75:C78 to C75:C80 with weights {3,2,2,1,2,2}

Example (Filled): update hardcoded array formulas to match —
  Cat 1 C27:C32 {3,2,1,2,2,2}, Cat 4 C72:C77 {3,2,2,1,2,2}
  N.A. indicators auto-excluded from denominator as designed
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="f:\Claude Projects\Linksys QA Rubric\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD92CE8-2792-4B00-A1B6-4630FF54DA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D189E08-F058-497B-8FEA-D2EC84D09F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4460,14 +4460,14 @@
     <xf numFmtId="0" fontId="60" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="58" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="60" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -4946,14 +4946,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
@@ -4964,30 +4956,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5018,8 +4986,40 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5043,18 +5043,6 @@
       <font>
         <b/>
         <sz val="9.5"/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="9.5"/>
         <color rgb="FF7B4F00"/>
       </font>
       <fill>
@@ -5065,71 +5053,13 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <b/>
+        <sz val="9.5"/>
+        <color rgb="FFFFFFFF"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FFC6EFCE"/>
+          <fgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5192,6 +5122,76 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6433,7 +6433,9 @@
       <c r="D40" s="174"/>
       <c r="E40" s="167"/>
       <c r="F40" s="168"/>
-      <c r="H40" s="144"/>
+      <c r="H40" s="144">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="172" t="s">
@@ -6443,7 +6445,9 @@
       <c r="D41" s="174"/>
       <c r="E41" s="167"/>
       <c r="F41" s="168"/>
-      <c r="H41" s="144"/>
+      <c r="H41" s="144">
+        <v>2</v>
+      </c>
     </row>
     <row r="42" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="191" t="s">
@@ -6459,7 +6463,7 @@
         <v>74</v>
       </c>
       <c r="C43" s="90" t="str">
-        <f>IF(SUMPRODUCT(((C36:C39="Met")+(C36:C39="Partial")+(C36:C39="Missed"))*H36:H39)=0,"",ROUND((5*SUMPRODUCT((C36:C39="Met")*H36:H39)+2.5*SUMPRODUCT((C36:C39="Partial")*H36:H39))/SUMPRODUCT(((C36:C39="Met")+(C36:C39="Partial")+(C36:C39="Missed"))*H36:H39),0))</f>
+        <f>IF(SUMPRODUCT(((C36:C41="Met")+(C36:C41="Partial")+(C36:C41="Missed"))*H36:H41)=0,"",ROUND((5*SUMPRODUCT((C36:C41="Met")*H36:H41)+2.5*SUMPRODUCT((C36:C41="Partial")*H36:H41))/SUMPRODUCT(((C36:C41="Met")+(C36:C41="Partial")+(C36:C41="Missed"))*H36:H41),1))</f>
         <v/>
       </c>
       <c r="D43" s="183"/>
@@ -6877,7 +6881,9 @@
       <c r="D79" s="171"/>
       <c r="E79" s="167"/>
       <c r="F79" s="168"/>
-      <c r="H79" s="144"/>
+      <c r="H79" s="144">
+        <v>2</v>
+      </c>
     </row>
     <row r="80" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="169" t="s">
@@ -6887,7 +6893,9 @@
       <c r="D80" s="171"/>
       <c r="E80" s="167"/>
       <c r="F80" s="168"/>
-      <c r="H80" s="144"/>
+      <c r="H80" s="144">
+        <v>2</v>
+      </c>
     </row>
     <row r="81" spans="2:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="196" t="s">
@@ -6903,7 +6911,7 @@
         <v>74</v>
       </c>
       <c r="C82" s="132" t="str">
-        <f>IF(SUMPRODUCT(((C75:C78="Met")+(C75:C78="Partial")+(C75:C78="Missed"))*H75:H78)=0,"",ROUND((5*SUMPRODUCT((C75:C78="Met")*H75:H78)+2.5*SUMPRODUCT((C75:C78="Partial")*H75:H78))/SUMPRODUCT(((C75:C78="Met")+(C75:C78="Partial")+(C75:C78="Missed"))*H75:H78),0))</f>
+        <f>IF(SUMPRODUCT(((C75:C80="Met")+(C75:C80="Partial")+(C75:C80="Missed"))*H75:H80)=0,"",ROUND((5*SUMPRODUCT((C75:C80="Met")*H75:H80)+2.5*SUMPRODUCT((C75:C80="Partial")*H75:H80))/SUMPRODUCT(((C75:C80="Met")+(C75:C80="Partial")+(C75:C80="Missed"))*H75:H80),1))</f>
         <v/>
       </c>
       <c r="D82" s="183"/>
@@ -8368,11 +8376,11 @@
     <cfRule type="cellIs" dxfId="68" priority="67" operator="equal">
       <formula>"Partial"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="68" operator="equal">
+      <formula>"Missed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="67" operator="equal">
       <formula>"Met"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="68" operator="equal">
-      <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C84">
@@ -8381,14 +8389,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C88:C91">
-    <cfRule type="cellIs" dxfId="64" priority="69" operator="equal">
-      <formula>"Met"</formula>
+    <cfRule type="cellIs" dxfId="64" priority="71" operator="equal">
+      <formula>"Missed"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="63" priority="70" operator="equal">
       <formula>"Partial"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="71" operator="equal">
-      <formula>"Missed"</formula>
+    <cfRule type="cellIs" dxfId="62" priority="69" operator="equal">
+      <formula>"Met"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C95">
@@ -8397,11 +8405,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C106:C110">
-    <cfRule type="cellIs" dxfId="60" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="73" operator="equal">
+      <formula>"Partial"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="59" priority="72" operator="equal">
       <formula>"Met"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="73" operator="equal">
-      <formula>"Partial"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="58" priority="74" operator="equal">
       <formula>"Missed"</formula>
@@ -8429,11 +8437,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C137:C144">
-    <cfRule type="cellIs" dxfId="52" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="55" operator="equal">
+      <formula>"Missed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="51" priority="54" operator="equal">
       <formula>"Partial"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="55" operator="equal">
-      <formula>"Missed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C152:C154">
@@ -8445,41 +8453,41 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C156:C166">
-    <cfRule type="cellIs" dxfId="48" priority="91" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="92" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="91" operator="equal">
       <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="92" operator="equal">
-      <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24:D30">
     <cfRule type="expression" dxfId="46" priority="78">
       <formula>AND(ISNUMBER($D24),$D24&lt;=2)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="79">
+    <cfRule type="expression" dxfId="45" priority="80">
+      <formula>AND(ISNUMBER($D24),$D24&gt;=4)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="79">
       <formula>AND(ISNUMBER($D24),$D24=3)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="44" priority="80">
-      <formula>AND(ISNUMBER($D24),$D24&gt;=4)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31">
     <cfRule type="expression" dxfId="43" priority="46">
       <formula>AND($E$31&lt;&gt;"",$E$31&gt;=0.85)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="47">
+    <cfRule type="expression" dxfId="42" priority="48">
+      <formula>AND($E$31&lt;&gt;"",$E$31&lt;0.7)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="41" priority="47">
       <formula>AND($E$31&lt;&gt;"",$E$31&gt;=0.7,$E$31&lt;0.85)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="41" priority="48">
-      <formula>AND($E$31&lt;&gt;"",$E$31&lt;0.7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E134">
-    <cfRule type="expression" dxfId="40" priority="87">
+    <cfRule type="expression" dxfId="40" priority="88">
+      <formula>$E134&lt;&gt;"OK"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="87">
       <formula>$E134="OK"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="39" priority="88">
-      <formula>$E134&lt;&gt;"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F24:F30">
@@ -11971,7 +11979,7 @@
       <c r="G3" s="63"/>
     </row>
     <row r="4" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="251" t="s">
+      <c r="B4" s="249" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="227"/>
@@ -12122,7 +12130,7 @@
       <c r="F14" s="227"/>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="251" t="s">
+      <c r="B15" s="249" t="s">
         <v>39</v>
       </c>
       <c r="C15" s="227"/>
@@ -12223,7 +12231,7 @@
       <c r="F23" s="227"/>
     </row>
     <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="251" t="s">
+      <c r="B24" s="249" t="s">
         <v>57</v>
       </c>
       <c r="C24" s="227"/>
@@ -12234,7 +12242,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="249" t="s">
+      <c r="B25" s="250" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="227"/>
@@ -12275,7 +12283,7 @@
       <c r="C28" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D28" s="250" t="s">
+      <c r="D28" s="251" t="s">
         <v>68</v>
       </c>
       <c r="E28" s="227"/>
@@ -12301,7 +12309,7 @@
       <c r="C30" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="250" t="s">
+      <c r="D30" s="251" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="227"/>
@@ -12343,7 +12351,7 @@
         <v>74</v>
       </c>
       <c r="C34" s="155">
-        <f>IF(SUMPRODUCT(((C27:C30="Met")+(C27:C30="Partial")+(C27:C30="Missed"))*{3,2,1,2})=0,"",ROUND((5*SUMPRODUCT((C27:C30="Met")*{3,2,1,2})+2.5*SUMPRODUCT((C27:C30="Partial")*{3,2,1,2}))/SUMPRODUCT(((C27:C30="Met")+(C27:C30="Partial")+(C27:C30="Missed"))*{3,2,1,2}),0))</f>
+        <f>IF(SUMPRODUCT(((C27:C32="Met")+(C27:C32="Partial")+(C27:C32="Missed"))*{3,2,1,2,2,2})=0,"",ROUND((5*SUMPRODUCT((C27:C32="Met")*{3,2,1,2,2,2})+2.5*SUMPRODUCT((C27:C32="Partial")*{3,2,1,2,2,2}))/SUMPRODUCT(((C27:C32="Met")+(C27:C32="Partial")+(C27:C32="Missed"))*{3,2,1,2,2,2}),1))</f>
         <v>4</v>
       </c>
       <c r="D34" s="156"/>
@@ -12396,7 +12404,7 @@
       <c r="G38" s="63"/>
     </row>
     <row r="39" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="251" t="s">
+      <c r="B39" s="249" t="s">
         <v>80</v>
       </c>
       <c r="C39" s="227"/>
@@ -12407,7 +12415,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="249" t="s">
+      <c r="B40" s="250" t="s">
         <v>82</v>
       </c>
       <c r="C40" s="227"/>
@@ -12448,7 +12456,7 @@
       <c r="C43" s="153" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="250" t="s">
+      <c r="D43" s="251" t="s">
         <v>86</v>
       </c>
       <c r="E43" s="227"/>
@@ -12474,7 +12482,7 @@
       <c r="C45" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D45" s="250" t="s">
+      <c r="D45" s="251" t="s">
         <v>90</v>
       </c>
       <c r="E45" s="227"/>
@@ -12558,7 +12566,7 @@
       <c r="G52" s="63"/>
     </row>
     <row r="53" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="251" t="s">
+      <c r="B53" s="249" t="s">
         <v>95</v>
       </c>
       <c r="C53" s="227"/>
@@ -12569,7 +12577,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="249" t="s">
+      <c r="B54" s="250" t="s">
         <v>97</v>
       </c>
       <c r="C54" s="227"/>
@@ -12610,7 +12618,7 @@
       <c r="C57" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D57" s="250" t="s">
+      <c r="D57" s="251" t="s">
         <v>101</v>
       </c>
       <c r="E57" s="227"/>
@@ -12636,7 +12644,7 @@
       <c r="C59" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D59" s="250" t="s">
+      <c r="D59" s="251" t="s">
         <v>105</v>
       </c>
       <c r="E59" s="227"/>
@@ -12675,7 +12683,7 @@
       <c r="C62" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D62" s="250" t="s">
+      <c r="D62" s="251" t="s">
         <v>112</v>
       </c>
       <c r="E62" s="227"/>
@@ -12748,7 +12756,7 @@
       <c r="G68" s="63"/>
     </row>
     <row r="69" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="251" t="s">
+      <c r="B69" s="249" t="s">
         <v>116</v>
       </c>
       <c r="C69" s="227"/>
@@ -12759,7 +12767,7 @@
       </c>
     </row>
     <row r="70" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="249" t="s">
+      <c r="B70" s="250" t="s">
         <v>117</v>
       </c>
       <c r="C70" s="227"/>
@@ -12800,7 +12808,7 @@
       <c r="C73" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D73" s="250" t="s">
+      <c r="D73" s="251" t="s">
         <v>121</v>
       </c>
       <c r="E73" s="227"/>
@@ -12826,7 +12834,7 @@
       <c r="C75" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D75" s="250" t="s">
+      <c r="D75" s="251" t="s">
         <v>125</v>
       </c>
       <c r="E75" s="227"/>
@@ -12868,8 +12876,8 @@
         <v>74</v>
       </c>
       <c r="C79" s="155">
-        <f>IF(SUMPRODUCT(((C72:C75="Met")+(C72:C75="Partial")+(C72:C75="Missed"))*{3,2,2,1})=0,"",ROUND((5*SUMPRODUCT((C72:C75="Met")*{3,2,2,1})+2.5*SUMPRODUCT((C72:C75="Partial")*{3,2,2,1}))/SUMPRODUCT(((C72:C75="Met")+(C72:C75="Partial")+(C72:C75="Missed"))*{3,2,2,1}),0))</f>
-        <v>1</v>
+        <f>IF(SUMPRODUCT(((C72:C77="Met")+(C72:C77="Partial")+(C72:C77="Missed"))*{3,2,2,1,2,2})=0,"",ROUND((5*SUMPRODUCT((C72:C77="Met")*{3,2,2,1,2,2})+2.5*SUMPRODUCT((C72:C77="Partial")*{3,2,2,1,2,2}))/SUMPRODUCT(((C72:C77="Met")+(C72:C77="Partial")+(C72:C77="Missed"))*{3,2,2,1,2,2}),1))</f>
+        <v>1.7</v>
       </c>
       <c r="D79" s="156"/>
       <c r="E79" s="156"/>
@@ -12921,7 +12929,7 @@
       <c r="G83" s="63"/>
     </row>
     <row r="84" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="251" t="s">
+      <c r="B84" s="249" t="s">
         <v>129</v>
       </c>
       <c r="C84" s="227"/>
@@ -12932,7 +12940,7 @@
       </c>
     </row>
     <row r="85" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="249" t="s">
+      <c r="B85" s="250" t="s">
         <v>131</v>
       </c>
       <c r="C85" s="227"/>
@@ -12973,7 +12981,7 @@
       <c r="C88" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D88" s="250" t="s">
+      <c r="D88" s="251" t="s">
         <v>135</v>
       </c>
       <c r="E88" s="227"/>
@@ -12999,7 +13007,7 @@
       <c r="C90" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D90" s="250" t="s">
+      <c r="D90" s="251" t="s">
         <v>139</v>
       </c>
       <c r="E90" s="227"/>
@@ -13072,7 +13080,7 @@
       <c r="G96" s="63"/>
     </row>
     <row r="97" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="251" t="s">
+      <c r="B97" s="249" t="s">
         <v>143</v>
       </c>
       <c r="C97" s="227"/>
@@ -13092,7 +13100,7 @@
       <c r="F98" s="227"/>
     </row>
     <row r="99" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="251" t="s">
+      <c r="B99" s="249" t="s">
         <v>146</v>
       </c>
       <c r="C99" s="227"/>
@@ -13139,7 +13147,7 @@
       <c r="G103" s="63"/>
     </row>
     <row r="104" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B104" s="251" t="s">
+      <c r="B104" s="249" t="s">
         <v>151</v>
       </c>
       <c r="C104" s="227"/>
@@ -13150,7 +13158,7 @@
       </c>
     </row>
     <row r="105" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="249" t="s">
+      <c r="B105" s="250" t="s">
         <v>153</v>
       </c>
       <c r="C105" s="227"/>
@@ -13191,7 +13199,7 @@
       <c r="C108" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D108" s="250" t="s">
+      <c r="D108" s="251" t="s">
         <v>157</v>
       </c>
       <c r="E108" s="227"/>
@@ -13217,7 +13225,7 @@
       <c r="C110" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D110" s="250" t="s">
+      <c r="D110" s="251" t="s">
         <v>161</v>
       </c>
       <c r="E110" s="227"/>
@@ -13303,7 +13311,7 @@
       <c r="G117" s="63"/>
     </row>
     <row r="118" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="251" t="s">
+      <c r="B118" s="249" t="s">
         <v>167</v>
       </c>
       <c r="C118" s="227"/>
@@ -13314,7 +13322,7 @@
       </c>
     </row>
     <row r="119" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B119" s="249" t="s">
+      <c r="B119" s="250" t="s">
         <v>168</v>
       </c>
       <c r="C119" s="227"/>
@@ -13355,7 +13363,7 @@
       <c r="C122" s="153" t="s">
         <v>67</v>
       </c>
-      <c r="D122" s="250" t="s">
+      <c r="D122" s="251" t="s">
         <v>172</v>
       </c>
       <c r="E122" s="227"/>
@@ -13381,7 +13389,7 @@
       <c r="C124" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D124" s="250" t="s">
+      <c r="D124" s="251" t="s">
         <v>176</v>
       </c>
       <c r="E124" s="227"/>
@@ -13407,7 +13415,7 @@
       <c r="C126" s="153" t="s">
         <v>111</v>
       </c>
-      <c r="D126" s="250" t="s">
+      <c r="D126" s="251" t="s">
         <v>180</v>
       </c>
       <c r="E126" s="227"/>
@@ -13672,7 +13680,7 @@
       <c r="G143" s="63"/>
     </row>
     <row r="144" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B144" s="251" t="s">
+      <c r="B144" s="249" t="s">
         <v>204</v>
       </c>
       <c r="C144" s="227"/>
@@ -13716,7 +13724,7 @@
       <c r="G147" s="63"/>
     </row>
     <row r="148" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B148" s="251" t="s">
+      <c r="B148" s="249" t="s">
         <v>210</v>
       </c>
       <c r="C148" s="227"/>
@@ -13804,7 +13812,7 @@
         <f>IF(OR(C75="Partial",C75="Missed"),C75,"")</f>
         <v>Missed</v>
       </c>
-      <c r="D155" s="250" t="s">
+      <c r="D155" s="251" t="s">
         <v>223</v>
       </c>
       <c r="E155" s="227"/>
@@ -13832,7 +13840,7 @@
         <f>IF(OR(C30="Partial",C30="Missed"),C30,"")</f>
         <v/>
       </c>
-      <c r="D157" s="250" t="s">
+      <c r="D157" s="251" t="s">
         <v>227</v>
       </c>
       <c r="E157" s="227"/>
@@ -13860,7 +13868,7 @@
         <f>IF(OR(C88="Partial",C88="Missed"),C88,"")</f>
         <v>Missed</v>
       </c>
-      <c r="D159" s="250" t="s">
+      <c r="D159" s="251" t="s">
         <v>231</v>
       </c>
       <c r="E159" s="227"/>
@@ -13888,7 +13896,7 @@
         <f>IF(OR(C126="Partial",C126="Missed"),C126,"")</f>
         <v>Missed</v>
       </c>
-      <c r="D161" s="250" t="s">
+      <c r="D161" s="251" t="s">
         <v>235</v>
       </c>
       <c r="E161" s="227"/>
@@ -13913,7 +13921,7 @@
       <c r="F163" s="227"/>
     </row>
     <row r="164" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B164" s="251" t="s">
+      <c r="B164" s="249" t="s">
         <v>237</v>
       </c>
       <c r="C164" s="227"/>
@@ -13955,7 +13963,7 @@
       <c r="F167" s="227"/>
     </row>
     <row r="168" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B168" s="251" t="s">
+      <c r="B168" s="249" t="s">
         <v>241</v>
       </c>
       <c r="C168" s="227"/>
@@ -13997,7 +14005,7 @@
       <c r="F171" s="227"/>
     </row>
     <row r="172" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B172" s="251" t="s">
+      <c r="B172" s="249" t="s">
         <v>245</v>
       </c>
       <c r="C172" s="227"/>
@@ -14015,7 +14023,7 @@
       <c r="F173" s="227"/>
     </row>
     <row r="174" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B174" s="251" t="s">
+      <c r="B174" s="249" t="s">
         <v>247</v>
       </c>
       <c r="C174" s="227"/>
@@ -14033,7 +14041,7 @@
       <c r="F175" s="227"/>
     </row>
     <row r="176" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B176" s="251" t="s">
+      <c r="B176" s="249" t="s">
         <v>249</v>
       </c>
       <c r="C176" s="227"/>
@@ -14051,7 +14059,7 @@
       <c r="F177" s="227"/>
     </row>
     <row r="178" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B178" s="251" t="s">
+      <c r="B178" s="249" t="s">
         <v>251</v>
       </c>
       <c r="C178" s="227"/>
@@ -14070,16 +14078,9 @@
     </row>
   </sheetData>
   <mergeCells count="145">
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C171:F171"/>
-    <mergeCell ref="B99:F99"/>
-    <mergeCell ref="B173:F173"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="C130:F130"/>
-    <mergeCell ref="D93:F93"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="D122:F122"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="D157:F157"/>
@@ -14091,13 +14092,6 @@
     <mergeCell ref="D129:F129"/>
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D107:F107"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="C51:F51"/>
-    <mergeCell ref="D122:F122"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="C169:F169"/>
-    <mergeCell ref="B105:F105"/>
-    <mergeCell ref="C170:F170"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="D125:F125"/>
     <mergeCell ref="D35:F35"/>
@@ -14113,19 +14107,15 @@
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="C67:F67"/>
     <mergeCell ref="C98:F98"/>
-    <mergeCell ref="C131:F131"/>
-    <mergeCell ref="C146:F146"/>
-    <mergeCell ref="B168:F168"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="D88:F88"/>
-    <mergeCell ref="D159:F159"/>
-    <mergeCell ref="D110:F110"/>
-    <mergeCell ref="D153:F153"/>
-    <mergeCell ref="B179:F179"/>
-    <mergeCell ref="B144:E144"/>
-    <mergeCell ref="B175:F175"/>
-    <mergeCell ref="D114:F114"/>
-    <mergeCell ref="D89:F89"/>
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B99:F99"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="D93:F93"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="C37:F37"/>
     <mergeCell ref="D56:F56"/>
     <mergeCell ref="C166:F166"/>
     <mergeCell ref="D62:F62"/>
@@ -14135,13 +14125,33 @@
     <mergeCell ref="B70:F70"/>
     <mergeCell ref="C94:F94"/>
     <mergeCell ref="D90:F90"/>
-    <mergeCell ref="B177:F177"/>
     <mergeCell ref="D108:F108"/>
     <mergeCell ref="C95:F95"/>
     <mergeCell ref="D149:F149"/>
     <mergeCell ref="D154:F154"/>
     <mergeCell ref="B163:F163"/>
     <mergeCell ref="B84:E84"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="B105:F105"/>
+    <mergeCell ref="C131:F131"/>
+    <mergeCell ref="C146:F146"/>
+    <mergeCell ref="C130:F130"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="D159:F159"/>
+    <mergeCell ref="D110:F110"/>
+    <mergeCell ref="D153:F153"/>
+    <mergeCell ref="B179:F179"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B175:F175"/>
+    <mergeCell ref="D114:F114"/>
+    <mergeCell ref="D89:F89"/>
+    <mergeCell ref="B177:F177"/>
+    <mergeCell ref="C169:F169"/>
+    <mergeCell ref="C170:F170"/>
+    <mergeCell ref="B168:F168"/>
+    <mergeCell ref="C171:F171"/>
+    <mergeCell ref="B173:F173"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="E145:F145"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="D126:F126"/>
@@ -14165,7 +14175,7 @@
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="D45:F45"/>
     <mergeCell ref="D160:F160"/>
-    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="D55:F55"/>
     <mergeCell ref="C115:F115"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="C100:F100"/>
@@ -14189,7 +14199,7 @@
     <mergeCell ref="D161:F161"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="D42:F42"/>
-    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="D49:F49"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="C165:F165"/>
     <mergeCell ref="B54:F54"/>
@@ -14213,8 +14223,6 @@
     <mergeCell ref="B85:F85"/>
     <mergeCell ref="D120:F120"/>
     <mergeCell ref="B25:F25"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D49:F49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Indicator Guide sheet — why and justification for all 37 indicators
New sheet inserted at position 4 (after Scoring Guide).
Covers all 7 categories x 37 behavioral indicators with:
- Weight tier (Primary / Core / Supporting)
- Why this indicator is here (3-4 sentences: purpose, importance,
  consequence of absence, connection to Support Organization Reset)
- What failure looks like (concrete examples for coaching use)

Each category has a purpose statement explaining how the category
contributes to the overall QA model. Weight tier color-coded:
Primary = dark navy, Core = medium blue, Supporting = light gray.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -9,13 +9,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Form" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multi-Touch Guide" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auto-Zero Guide" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicator Guide" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Guide" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Multi-Touch Guide" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auto-Zero Guide" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Scoring" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example (Filled)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Tracker" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="72">
+  <fonts count="80">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -503,6 +504,43 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FF595959"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="44">
     <fill>
@@ -730,7 +768,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -1063,11 +1101,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="333">
+  <cellXfs count="347">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -2010,6 +2053,48 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="75" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="20" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="11" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="20" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="20" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="29" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="3" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="29" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="29" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="25" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4119,6 +4204,1701 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" style="187" min="1" max="1"/>
+    <col width="13" customWidth="1" style="187" min="2" max="2"/>
+    <col width="18" customWidth="1" style="187" min="3" max="3"/>
+    <col width="8" customWidth="1" style="187" min="4" max="11"/>
+    <col width="10" customWidth="1" style="187" min="12" max="12"/>
+    <col width="13" customWidth="1" style="187" min="13" max="13"/>
+    <col width="60" customWidth="1" style="187" min="14" max="14"/>
+    <col width="22" customWidth="1" style="187" min="15" max="15"/>
+    <col width="14" customWidth="1" style="187" min="16" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26.1" customHeight="1" s="187">
+      <c r="A1" s="219" t="inlineStr">
+        <is>
+          <t>CASE TRACKER — Multi-Case &amp; Multi-Touch Log</t>
+        </is>
+      </c>
+      <c r="B1" s="212" t="n"/>
+      <c r="C1" s="212" t="n"/>
+      <c r="D1" s="212" t="n"/>
+      <c r="E1" s="212" t="n"/>
+      <c r="F1" s="212" t="n"/>
+      <c r="G1" s="212" t="n"/>
+      <c r="H1" s="212" t="n"/>
+      <c r="I1" s="212" t="n"/>
+      <c r="J1" s="212" t="n"/>
+      <c r="K1" s="212" t="n"/>
+      <c r="L1" s="212" t="n"/>
+      <c r="M1" s="212" t="n"/>
+      <c r="N1" s="212" t="n"/>
+      <c r="O1" s="212" t="n"/>
+      <c r="P1" s="192" t="n"/>
+    </row>
+    <row r="2" ht="15.95" customHeight="1" s="187">
+      <c r="A2" s="282" t="inlineStr">
+        <is>
+          <t>One row per touch. Reuse a Case ID across rows to track a multi-touch journey. Scores 0-5; Weighted % and Result calculate automatically. Pre-loaded: the TE00124020 / TE00127492 journey (see Multi-Touch Guide).</t>
+        </is>
+      </c>
+      <c r="B2" s="212" t="n"/>
+      <c r="C2" s="212" t="n"/>
+      <c r="D2" s="212" t="n"/>
+      <c r="E2" s="212" t="n"/>
+      <c r="F2" s="212" t="n"/>
+      <c r="G2" s="212" t="n"/>
+      <c r="H2" s="212" t="n"/>
+      <c r="I2" s="212" t="n"/>
+      <c r="J2" s="212" t="n"/>
+      <c r="K2" s="212" t="n"/>
+      <c r="L2" s="212" t="n"/>
+      <c r="M2" s="212" t="n"/>
+      <c r="N2" s="212" t="n"/>
+      <c r="O2" s="212" t="n"/>
+      <c r="P2" s="192" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" s="187">
+      <c r="A3" s="275">
+        <f>IF(A56="","  JOURNEY TEAM SCORE  ▸  log touches below, then enter a Case ID + Outcome/Continuity in row 56","  LOADED JOURNEY TEAM SCORE  ▸  "&amp;A56&amp;":  "&amp;TEXT(G56,"0.0%")&amp;"   "&amp;UPPER(H56))</f>
+        <v/>
+      </c>
+      <c r="B3" s="212" t="n"/>
+      <c r="C3" s="212" t="n"/>
+      <c r="D3" s="212" t="n"/>
+      <c r="E3" s="212" t="n"/>
+      <c r="F3" s="212" t="n"/>
+      <c r="G3" s="212" t="n"/>
+      <c r="H3" s="212" t="n"/>
+      <c r="I3" s="212" t="n"/>
+      <c r="J3" s="212" t="n"/>
+      <c r="K3" s="212" t="n"/>
+      <c r="L3" s="212" t="n"/>
+      <c r="M3" s="212" t="n"/>
+      <c r="N3" s="212" t="n"/>
+      <c r="O3" s="212" t="n"/>
+      <c r="P3" s="192" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="187">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Case ID</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Touch #</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>Res 30%</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>Tech 20%</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>Comm 15%</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>Own 15%</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>Esc 10%</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr">
+        <is>
+          <t>CX 5%</t>
+        </is>
+      </c>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>Doc 5%</t>
+        </is>
+      </c>
+      <c r="L4" s="23" t="inlineStr">
+        <is>
+          <t>Weighted</t>
+        </is>
+      </c>
+      <c r="M4" s="23" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="N4" s="23" t="inlineStr">
+        <is>
+          <t>Outcome / Notes</t>
+        </is>
+      </c>
+      <c r="O4" s="46" t="inlineStr">
+        <is>
+          <t>Contribution Type</t>
+        </is>
+      </c>
+      <c r="P4" s="46" t="inlineStr">
+        <is>
+          <t>Handoff Quality (0-5)</t>
+        </is>
+      </c>
+      <c r="Q4" s="95" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39.95" customHeight="1" s="187">
+      <c r="A5" s="24" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="24" t="n"/>
+      <c r="L5" s="325">
+        <f>IF((COUNT(E5)+COUNT(F5)+COUNT(G5)+COUNT(H5)+COUNT(I5)+COUNT(J5)+COUNT(K5))=0,"",IFERROR(E5/5*0.3,0)+IFERROR(F5/5*0.2,0)+IFERROR(G5/5*0.15,0)+IFERROR(H5/5*0.15,0)+IFERROR(I5/5*0.1,0)+IFERROR(J5/5*0.05,0)+IFERROR(K5/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M5" s="11">
+        <f>IF(L5="","",IF(L5&gt;=0.85,"Meets/Exceeds",IF(L5&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="11" t="n"/>
+      <c r="P5" s="11" t="n"/>
+      <c r="Q5" s="96" t="n"/>
+    </row>
+    <row r="6" ht="39.95" customHeight="1" s="187">
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="24" t="n"/>
+      <c r="D6" s="24" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="24" t="n"/>
+      <c r="K6" s="24" t="n"/>
+      <c r="L6" s="326">
+        <f>IF((COUNT(E6)+COUNT(F6)+COUNT(G6)+COUNT(H6)+COUNT(I6)+COUNT(J6)+COUNT(K6))=0,"",IFERROR(E6/5*0.3,0)+IFERROR(F6/5*0.2,0)+IFERROR(G6/5*0.15,0)+IFERROR(H6/5*0.15,0)+IFERROR(I6/5*0.1,0)+IFERROR(J6/5*0.05,0)+IFERROR(K6/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M6" s="13">
+        <f>IF(L6="","",IF(L6&gt;=0.85,"Meets/Exceeds",IF(L6&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N6" s="8" t="n"/>
+      <c r="O6" s="13" t="n"/>
+      <c r="P6" s="13" t="n"/>
+      <c r="Q6" s="96" t="n"/>
+    </row>
+    <row r="7" ht="39.95" customHeight="1" s="187">
+      <c r="A7" s="24" t="n"/>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="24" t="n"/>
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="n"/>
+      <c r="H7" s="24" t="n"/>
+      <c r="I7" s="24" t="n"/>
+      <c r="J7" s="24" t="n"/>
+      <c r="K7" s="24" t="n"/>
+      <c r="L7" s="325">
+        <f>IF((COUNT(E7)+COUNT(F7)+COUNT(G7)+COUNT(H7)+COUNT(I7)+COUNT(J7)+COUNT(K7))=0,"",IFERROR(E7/5*0.3,0)+IFERROR(F7/5*0.2,0)+IFERROR(G7/5*0.15,0)+IFERROR(H7/5*0.15,0)+IFERROR(I7/5*0.1,0)+IFERROR(J7/5*0.05,0)+IFERROR(K7/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M7" s="11">
+        <f>IF(L7="","",IF(L7&gt;=0.85,"Meets/Exceeds",IF(L7&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="11" t="n"/>
+      <c r="P7" s="11" t="n"/>
+      <c r="Q7" s="96" t="n"/>
+    </row>
+    <row r="8" ht="39.95" customHeight="1" s="187">
+      <c r="A8" s="24" t="n"/>
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
+      <c r="J8" s="24" t="n"/>
+      <c r="K8" s="24" t="n"/>
+      <c r="L8" s="326">
+        <f>IF((COUNT(E8)+COUNT(F8)+COUNT(G8)+COUNT(H8)+COUNT(I8)+COUNT(J8)+COUNT(K8))=0,"",IFERROR(E8/5*0.3,0)+IFERROR(F8/5*0.2,0)+IFERROR(G8/5*0.15,0)+IFERROR(H8/5*0.15,0)+IFERROR(I8/5*0.1,0)+IFERROR(J8/5*0.05,0)+IFERROR(K8/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M8" s="13">
+        <f>IF(L8="","",IF(L8&gt;=0.85,"Meets/Exceeds",IF(L8&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N8" s="8" t="n"/>
+      <c r="O8" s="13" t="n"/>
+      <c r="P8" s="13" t="n"/>
+      <c r="Q8" s="96" t="n"/>
+    </row>
+    <row r="9" ht="39.95" customHeight="1" s="187">
+      <c r="A9" s="24" t="n"/>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="24" t="n"/>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="325">
+        <f>IF((COUNT(E9)+COUNT(F9)+COUNT(G9)+COUNT(H9)+COUNT(I9)+COUNT(J9)+COUNT(K9))=0,"",IFERROR(E9/5*0.3,0)+IFERROR(F9/5*0.2,0)+IFERROR(G9/5*0.15,0)+IFERROR(H9/5*0.15,0)+IFERROR(I9/5*0.1,0)+IFERROR(J9/5*0.05,0)+IFERROR(K9/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M9" s="11">
+        <f>IF(L9="","",IF(L9&gt;=0.85,"Meets/Exceeds",IF(L9&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N9" s="6" t="n"/>
+      <c r="O9" s="11" t="n"/>
+      <c r="P9" s="11" t="n"/>
+      <c r="Q9" s="96" t="n"/>
+    </row>
+    <row r="10" ht="39.95" customHeight="1" s="187">
+      <c r="A10" s="24" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
+      <c r="H10" s="24" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="24" t="n"/>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="326">
+        <f>IF((COUNT(E10)+COUNT(F10)+COUNT(G10)+COUNT(H10)+COUNT(I10)+COUNT(J10)+COUNT(K10))=0,"",IFERROR(E10/5*0.3,0)+IFERROR(F10/5*0.2,0)+IFERROR(G10/5*0.15,0)+IFERROR(H10/5*0.15,0)+IFERROR(I10/5*0.1,0)+IFERROR(J10/5*0.05,0)+IFERROR(K10/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M10" s="13">
+        <f>IF(L10="","",IF(L10&gt;=0.85,"Meets/Exceeds",IF(L10&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N10" s="8" t="n"/>
+      <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n"/>
+      <c r="Q10" s="96" t="n"/>
+    </row>
+    <row r="11" ht="39.95" customHeight="1" s="187">
+      <c r="A11" s="24" t="n"/>
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="24" t="n"/>
+      <c r="J11" s="24" t="n"/>
+      <c r="K11" s="24" t="n"/>
+      <c r="L11" s="325">
+        <f>IF((COUNT(E11)+COUNT(F11)+COUNT(G11)+COUNT(H11)+COUNT(I11)+COUNT(J11)+COUNT(K11))=0,"",IFERROR(E11/5*0.3,0)+IFERROR(F11/5*0.2,0)+IFERROR(G11/5*0.15,0)+IFERROR(H11/5*0.15,0)+IFERROR(I11/5*0.1,0)+IFERROR(J11/5*0.05,0)+IFERROR(K11/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M11" s="11">
+        <f>IF(L11="","",IF(L11&gt;=0.85,"Meets/Exceeds",IF(L11&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
+      <c r="Q11" s="96" t="n"/>
+    </row>
+    <row r="12" ht="39.95" customHeight="1" s="187">
+      <c r="A12" s="24" t="n"/>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="24" t="n"/>
+      <c r="G12" s="24" t="n"/>
+      <c r="H12" s="24" t="n"/>
+      <c r="I12" s="24" t="n"/>
+      <c r="J12" s="24" t="n"/>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="326">
+        <f>IF((COUNT(E12)+COUNT(F12)+COUNT(G12)+COUNT(H12)+COUNT(I12)+COUNT(J12)+COUNT(K12))=0,"",IFERROR(E12/5*0.3,0)+IFERROR(F12/5*0.2,0)+IFERROR(G12/5*0.15,0)+IFERROR(H12/5*0.15,0)+IFERROR(I12/5*0.1,0)+IFERROR(J12/5*0.05,0)+IFERROR(K12/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M12" s="13">
+        <f>IF(L12="","",IF(L12&gt;=0.85,"Meets/Exceeds",IF(L12&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N12" s="8" t="n"/>
+      <c r="O12" s="13" t="n"/>
+      <c r="P12" s="13" t="n"/>
+      <c r="Q12" s="96" t="n"/>
+    </row>
+    <row r="13" ht="39.95" customHeight="1" s="187">
+      <c r="A13" s="24" t="n"/>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
+      <c r="H13" s="24" t="n"/>
+      <c r="I13" s="24" t="n"/>
+      <c r="J13" s="24" t="n"/>
+      <c r="K13" s="24" t="n"/>
+      <c r="L13" s="325">
+        <f>IF((COUNT(E13)+COUNT(F13)+COUNT(G13)+COUNT(H13)+COUNT(I13)+COUNT(J13)+COUNT(K13))=0,"",IFERROR(E13/5*0.3,0)+IFERROR(F13/5*0.2,0)+IFERROR(G13/5*0.15,0)+IFERROR(H13/5*0.15,0)+IFERROR(I13/5*0.1,0)+IFERROR(J13/5*0.05,0)+IFERROR(K13/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M13" s="11">
+        <f>IF(L13="","",IF(L13&gt;=0.85,"Meets/Exceeds",IF(L13&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="11" t="n"/>
+      <c r="P13" s="11" t="n"/>
+      <c r="Q13" s="96" t="n"/>
+    </row>
+    <row r="14" ht="39.95" customHeight="1" s="187">
+      <c r="A14" s="24" t="n"/>
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="24" t="n"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="24" t="n"/>
+      <c r="J14" s="24" t="n"/>
+      <c r="K14" s="24" t="n"/>
+      <c r="L14" s="326">
+        <f>IF((COUNT(E14)+COUNT(F14)+COUNT(G14)+COUNT(H14)+COUNT(I14)+COUNT(J14)+COUNT(K14))=0,"",IFERROR(E14/5*0.3,0)+IFERROR(F14/5*0.2,0)+IFERROR(G14/5*0.15,0)+IFERROR(H14/5*0.15,0)+IFERROR(I14/5*0.1,0)+IFERROR(J14/5*0.05,0)+IFERROR(K14/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M14" s="13">
+        <f>IF(L14="","",IF(L14&gt;=0.85,"Meets/Exceeds",IF(L14&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N14" s="8" t="n"/>
+      <c r="O14" s="13" t="n"/>
+      <c r="P14" s="13" t="n"/>
+      <c r="Q14" s="96" t="n"/>
+    </row>
+    <row r="15" ht="39.95" customHeight="1" s="187">
+      <c r="A15" s="24" t="n"/>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="24" t="n"/>
+      <c r="G15" s="24" t="n"/>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="24" t="n"/>
+      <c r="K15" s="24" t="n"/>
+      <c r="L15" s="325">
+        <f>IF((COUNT(E15)+COUNT(F15)+COUNT(G15)+COUNT(H15)+COUNT(I15)+COUNT(J15)+COUNT(K15))=0,"",IFERROR(E15/5*0.3,0)+IFERROR(F15/5*0.2,0)+IFERROR(G15/5*0.15,0)+IFERROR(H15/5*0.15,0)+IFERROR(I15/5*0.1,0)+IFERROR(J15/5*0.05,0)+IFERROR(K15/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M15" s="11">
+        <f>IF(L15="","",IF(L15&gt;=0.85,"Meets/Exceeds",IF(L15&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="11" t="n"/>
+      <c r="P15" s="11" t="n"/>
+      <c r="Q15" s="96" t="n"/>
+    </row>
+    <row r="16" ht="39.95" customHeight="1" s="187">
+      <c r="A16" s="24" t="n"/>
+      <c r="B16" s="24" t="n"/>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="24" t="n"/>
+      <c r="G16" s="24" t="n"/>
+      <c r="H16" s="24" t="n"/>
+      <c r="I16" s="24" t="n"/>
+      <c r="J16" s="24" t="n"/>
+      <c r="K16" s="24" t="n"/>
+      <c r="L16" s="326">
+        <f>IF((COUNT(E16)+COUNT(F16)+COUNT(G16)+COUNT(H16)+COUNT(I16)+COUNT(J16)+COUNT(K16))=0,"",IFERROR(E16/5*0.3,0)+IFERROR(F16/5*0.2,0)+IFERROR(G16/5*0.15,0)+IFERROR(H16/5*0.15,0)+IFERROR(I16/5*0.1,0)+IFERROR(J16/5*0.05,0)+IFERROR(K16/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M16" s="13">
+        <f>IF(L16="","",IF(L16&gt;=0.85,"Meets/Exceeds",IF(L16&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N16" s="8" t="n"/>
+      <c r="O16" s="13" t="n"/>
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="96" t="n"/>
+    </row>
+    <row r="17" ht="39.95" customHeight="1" s="187">
+      <c r="A17" s="24" t="n"/>
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
+      <c r="H17" s="24" t="n"/>
+      <c r="I17" s="24" t="n"/>
+      <c r="J17" s="24" t="n"/>
+      <c r="K17" s="24" t="n"/>
+      <c r="L17" s="325">
+        <f>IF((COUNT(E17)+COUNT(F17)+COUNT(G17)+COUNT(H17)+COUNT(I17)+COUNT(J17)+COUNT(K17))=0,"",IFERROR(E17/5*0.3,0)+IFERROR(F17/5*0.2,0)+IFERROR(G17/5*0.15,0)+IFERROR(H17/5*0.15,0)+IFERROR(I17/5*0.1,0)+IFERROR(J17/5*0.05,0)+IFERROR(K17/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M17" s="11">
+        <f>IF(L17="","",IF(L17&gt;=0.85,"Meets/Exceeds",IF(L17&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="Q17" s="96" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="187">
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="24" t="n"/>
+      <c r="G18" s="24" t="n"/>
+      <c r="H18" s="24" t="n"/>
+      <c r="I18" s="24" t="n"/>
+      <c r="J18" s="24" t="n"/>
+      <c r="K18" s="24" t="n"/>
+      <c r="L18" s="326">
+        <f>IF((COUNT(E18)+COUNT(F18)+COUNT(G18)+COUNT(H18)+COUNT(I18)+COUNT(J18)+COUNT(K18))=0,"",IFERROR(E18/5*0.3,0)+IFERROR(F18/5*0.2,0)+IFERROR(G18/5*0.15,0)+IFERROR(H18/5*0.15,0)+IFERROR(I18/5*0.1,0)+IFERROR(J18/5*0.05,0)+IFERROR(K18/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M18" s="13">
+        <f>IF(L18="","",IF(L18&gt;=0.85,"Meets/Exceeds",IF(L18&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N18" s="8" t="n"/>
+      <c r="O18" s="13" t="n"/>
+      <c r="P18" s="13" t="n"/>
+      <c r="Q18" s="96" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="187">
+      <c r="A19" s="24" t="n"/>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="24" t="n"/>
+      <c r="G19" s="24" t="n"/>
+      <c r="H19" s="24" t="n"/>
+      <c r="I19" s="24" t="n"/>
+      <c r="J19" s="24" t="n"/>
+      <c r="K19" s="24" t="n"/>
+      <c r="L19" s="325">
+        <f>IF((COUNT(E19)+COUNT(F19)+COUNT(G19)+COUNT(H19)+COUNT(I19)+COUNT(J19)+COUNT(K19))=0,"",IFERROR(E19/5*0.3,0)+IFERROR(F19/5*0.2,0)+IFERROR(G19/5*0.15,0)+IFERROR(H19/5*0.15,0)+IFERROR(I19/5*0.1,0)+IFERROR(J19/5*0.05,0)+IFERROR(K19/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M19" s="11">
+        <f>IF(L19="","",IF(L19&gt;=0.85,"Meets/Exceeds",IF(L19&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
+      <c r="Q19" s="96" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="187">
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="24" t="n"/>
+      <c r="G20" s="24" t="n"/>
+      <c r="H20" s="24" t="n"/>
+      <c r="I20" s="24" t="n"/>
+      <c r="J20" s="24" t="n"/>
+      <c r="K20" s="24" t="n"/>
+      <c r="L20" s="326">
+        <f>IF((COUNT(E20)+COUNT(F20)+COUNT(G20)+COUNT(H20)+COUNT(I20)+COUNT(J20)+COUNT(K20))=0,"",IFERROR(E20/5*0.3,0)+IFERROR(F20/5*0.2,0)+IFERROR(G20/5*0.15,0)+IFERROR(H20/5*0.15,0)+IFERROR(I20/5*0.1,0)+IFERROR(J20/5*0.05,0)+IFERROR(K20/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M20" s="13">
+        <f>IF(L20="","",IF(L20&gt;=0.85,"Meets/Exceeds",IF(L20&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N20" s="8" t="n"/>
+      <c r="O20" s="13" t="n"/>
+      <c r="P20" s="13" t="n"/>
+      <c r="Q20" s="96" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="187">
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="24" t="n"/>
+      <c r="H21" s="24" t="n"/>
+      <c r="I21" s="24" t="n"/>
+      <c r="J21" s="24" t="n"/>
+      <c r="K21" s="24" t="n"/>
+      <c r="L21" s="325">
+        <f>IF((COUNT(E21)+COUNT(F21)+COUNT(G21)+COUNT(H21)+COUNT(I21)+COUNT(J21)+COUNT(K21))=0,"",IFERROR(E21/5*0.3,0)+IFERROR(F21/5*0.2,0)+IFERROR(G21/5*0.15,0)+IFERROR(H21/5*0.15,0)+IFERROR(I21/5*0.1,0)+IFERROR(J21/5*0.05,0)+IFERROR(K21/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M21" s="11">
+        <f>IF(L21="","",IF(L21&gt;=0.85,"Meets/Exceeds",IF(L21&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
+      <c r="Q21" s="96" t="n"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="187">
+      <c r="A22" s="24" t="n"/>
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="24" t="n"/>
+      <c r="G22" s="24" t="n"/>
+      <c r="H22" s="24" t="n"/>
+      <c r="I22" s="24" t="n"/>
+      <c r="J22" s="24" t="n"/>
+      <c r="K22" s="24" t="n"/>
+      <c r="L22" s="326">
+        <f>IF((COUNT(E22)+COUNT(F22)+COUNT(G22)+COUNT(H22)+COUNT(I22)+COUNT(J22)+COUNT(K22))=0,"",IFERROR(E22/5*0.3,0)+IFERROR(F22/5*0.2,0)+IFERROR(G22/5*0.15,0)+IFERROR(H22/5*0.15,0)+IFERROR(I22/5*0.1,0)+IFERROR(J22/5*0.05,0)+IFERROR(K22/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M22" s="13">
+        <f>IF(L22="","",IF(L22&gt;=0.85,"Meets/Exceeds",IF(L22&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N22" s="8" t="n"/>
+      <c r="O22" s="13" t="n"/>
+      <c r="P22" s="13" t="n"/>
+      <c r="Q22" s="96" t="n"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="187">
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
+      <c r="F23" s="24" t="n"/>
+      <c r="G23" s="24" t="n"/>
+      <c r="H23" s="24" t="n"/>
+      <c r="I23" s="24" t="n"/>
+      <c r="J23" s="24" t="n"/>
+      <c r="K23" s="24" t="n"/>
+      <c r="L23" s="325">
+        <f>IF((COUNT(E23)+COUNT(F23)+COUNT(G23)+COUNT(H23)+COUNT(I23)+COUNT(J23)+COUNT(K23))=0,"",IFERROR(E23/5*0.3,0)+IFERROR(F23/5*0.2,0)+IFERROR(G23/5*0.15,0)+IFERROR(H23/5*0.15,0)+IFERROR(I23/5*0.1,0)+IFERROR(J23/5*0.05,0)+IFERROR(K23/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M23" s="11">
+        <f>IF(L23="","",IF(L23&gt;=0.85,"Meets/Exceeds",IF(L23&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N23" s="6" t="n"/>
+      <c r="O23" s="11" t="n"/>
+      <c r="P23" s="11" t="n"/>
+      <c r="Q23" s="96" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="187">
+      <c r="A24" s="24" t="n"/>
+      <c r="B24" s="24" t="n"/>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="24" t="n"/>
+      <c r="G24" s="24" t="n"/>
+      <c r="H24" s="24" t="n"/>
+      <c r="I24" s="24" t="n"/>
+      <c r="J24" s="24" t="n"/>
+      <c r="K24" s="24" t="n"/>
+      <c r="L24" s="326">
+        <f>IF((COUNT(E24)+COUNT(F24)+COUNT(G24)+COUNT(H24)+COUNT(I24)+COUNT(J24)+COUNT(K24))=0,"",IFERROR(E24/5*0.3,0)+IFERROR(F24/5*0.2,0)+IFERROR(G24/5*0.15,0)+IFERROR(H24/5*0.15,0)+IFERROR(I24/5*0.1,0)+IFERROR(J24/5*0.05,0)+IFERROR(K24/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M24" s="13">
+        <f>IF(L24="","",IF(L24&gt;=0.85,"Meets/Exceeds",IF(L24&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N24" s="8" t="n"/>
+      <c r="O24" s="13" t="n"/>
+      <c r="P24" s="13" t="n"/>
+      <c r="Q24" s="96" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="187">
+      <c r="A25" s="24" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="24" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="24" t="n"/>
+      <c r="J25" s="24" t="n"/>
+      <c r="K25" s="24" t="n"/>
+      <c r="L25" s="325">
+        <f>IF((COUNT(E25)+COUNT(F25)+COUNT(G25)+COUNT(H25)+COUNT(I25)+COUNT(J25)+COUNT(K25))=0,"",IFERROR(E25/5*0.3,0)+IFERROR(F25/5*0.2,0)+IFERROR(G25/5*0.15,0)+IFERROR(H25/5*0.15,0)+IFERROR(I25/5*0.1,0)+IFERROR(J25/5*0.05,0)+IFERROR(K25/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M25" s="11">
+        <f>IF(L25="","",IF(L25&gt;=0.85,"Meets/Exceeds",IF(L25&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N25" s="6" t="n"/>
+      <c r="O25" s="11" t="n"/>
+      <c r="P25" s="11" t="n"/>
+      <c r="Q25" s="96" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="187">
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="24" t="n"/>
+      <c r="G26" s="24" t="n"/>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="24" t="n"/>
+      <c r="J26" s="24" t="n"/>
+      <c r="K26" s="24" t="n"/>
+      <c r="L26" s="326">
+        <f>IF((COUNT(E26)+COUNT(F26)+COUNT(G26)+COUNT(H26)+COUNT(I26)+COUNT(J26)+COUNT(K26))=0,"",IFERROR(E26/5*0.3,0)+IFERROR(F26/5*0.2,0)+IFERROR(G26/5*0.15,0)+IFERROR(H26/5*0.15,0)+IFERROR(I26/5*0.1,0)+IFERROR(J26/5*0.05,0)+IFERROR(K26/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M26" s="13">
+        <f>IF(L26="","",IF(L26&gt;=0.85,"Meets/Exceeds",IF(L26&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N26" s="8" t="n"/>
+      <c r="O26" s="13" t="n"/>
+      <c r="P26" s="13" t="n"/>
+      <c r="Q26" s="96" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="187">
+      <c r="A27" s="24" t="n"/>
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="24" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="24" t="n"/>
+      <c r="F27" s="24" t="n"/>
+      <c r="G27" s="24" t="n"/>
+      <c r="H27" s="24" t="n"/>
+      <c r="I27" s="24" t="n"/>
+      <c r="J27" s="24" t="n"/>
+      <c r="K27" s="24" t="n"/>
+      <c r="L27" s="325">
+        <f>IF((COUNT(E27)+COUNT(F27)+COUNT(G27)+COUNT(H27)+COUNT(I27)+COUNT(J27)+COUNT(K27))=0,"",IFERROR(E27/5*0.3,0)+IFERROR(F27/5*0.2,0)+IFERROR(G27/5*0.15,0)+IFERROR(H27/5*0.15,0)+IFERROR(I27/5*0.1,0)+IFERROR(J27/5*0.05,0)+IFERROR(K27/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M27" s="11">
+        <f>IF(L27="","",IF(L27&gt;=0.85,"Meets/Exceeds",IF(L27&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="11" t="n"/>
+      <c r="P27" s="11" t="n"/>
+      <c r="Q27" s="96" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="187">
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="24" t="n"/>
+      <c r="J28" s="24" t="n"/>
+      <c r="K28" s="24" t="n"/>
+      <c r="L28" s="326">
+        <f>IF((COUNT(E28)+COUNT(F28)+COUNT(G28)+COUNT(H28)+COUNT(I28)+COUNT(J28)+COUNT(K28))=0,"",IFERROR(E28/5*0.3,0)+IFERROR(F28/5*0.2,0)+IFERROR(G28/5*0.15,0)+IFERROR(H28/5*0.15,0)+IFERROR(I28/5*0.1,0)+IFERROR(J28/5*0.05,0)+IFERROR(K28/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M28" s="13">
+        <f>IF(L28="","",IF(L28&gt;=0.85,"Meets/Exceeds",IF(L28&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N28" s="8" t="n"/>
+      <c r="O28" s="13" t="n"/>
+      <c r="P28" s="13" t="n"/>
+      <c r="Q28" s="96" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="187">
+      <c r="A29" s="24" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
+      <c r="J29" s="24" t="n"/>
+      <c r="K29" s="24" t="n"/>
+      <c r="L29" s="325">
+        <f>IF((COUNT(E29)+COUNT(F29)+COUNT(G29)+COUNT(H29)+COUNT(I29)+COUNT(J29)+COUNT(K29))=0,"",IFERROR(E29/5*0.3,0)+IFERROR(F29/5*0.2,0)+IFERROR(G29/5*0.15,0)+IFERROR(H29/5*0.15,0)+IFERROR(I29/5*0.1,0)+IFERROR(J29/5*0.05,0)+IFERROR(K29/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M29" s="11">
+        <f>IF(L29="","",IF(L29&gt;=0.85,"Meets/Exceeds",IF(L29&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N29" s="6" t="n"/>
+      <c r="O29" s="11" t="n"/>
+      <c r="P29" s="11" t="n"/>
+      <c r="Q29" s="96" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="187">
+      <c r="A30" s="24" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
+      <c r="J30" s="24" t="n"/>
+      <c r="K30" s="24" t="n"/>
+      <c r="L30" s="326">
+        <f>IF((COUNT(E30)+COUNT(F30)+COUNT(G30)+COUNT(H30)+COUNT(I30)+COUNT(J30)+COUNT(K30))=0,"",IFERROR(E30/5*0.3,0)+IFERROR(F30/5*0.2,0)+IFERROR(G30/5*0.15,0)+IFERROR(H30/5*0.15,0)+IFERROR(I30/5*0.1,0)+IFERROR(J30/5*0.05,0)+IFERROR(K30/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M30" s="13">
+        <f>IF(L30="","",IF(L30&gt;=0.85,"Meets/Exceeds",IF(L30&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N30" s="8" t="n"/>
+      <c r="O30" s="13" t="n"/>
+      <c r="P30" s="13" t="n"/>
+      <c r="Q30" s="96" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="187">
+      <c r="A31" s="24" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
+      <c r="J31" s="24" t="n"/>
+      <c r="K31" s="24" t="n"/>
+      <c r="L31" s="325">
+        <f>IF((COUNT(E31)+COUNT(F31)+COUNT(G31)+COUNT(H31)+COUNT(I31)+COUNT(J31)+COUNT(K31))=0,"",IFERROR(E31/5*0.3,0)+IFERROR(F31/5*0.2,0)+IFERROR(G31/5*0.15,0)+IFERROR(H31/5*0.15,0)+IFERROR(I31/5*0.1,0)+IFERROR(J31/5*0.05,0)+IFERROR(K31/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M31" s="11">
+        <f>IF(L31="","",IF(L31&gt;=0.85,"Meets/Exceeds",IF(L31&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="11" t="n"/>
+      <c r="P31" s="11" t="n"/>
+      <c r="Q31" s="96" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="187">
+      <c r="A32" s="24" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
+      <c r="J32" s="24" t="n"/>
+      <c r="K32" s="24" t="n"/>
+      <c r="L32" s="326">
+        <f>IF((COUNT(E32)+COUNT(F32)+COUNT(G32)+COUNT(H32)+COUNT(I32)+COUNT(J32)+COUNT(K32))=0,"",IFERROR(E32/5*0.3,0)+IFERROR(F32/5*0.2,0)+IFERROR(G32/5*0.15,0)+IFERROR(H32/5*0.15,0)+IFERROR(I32/5*0.1,0)+IFERROR(J32/5*0.05,0)+IFERROR(K32/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M32" s="13">
+        <f>IF(L32="","",IF(L32&gt;=0.85,"Meets/Exceeds",IF(L32&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N32" s="8" t="n"/>
+      <c r="O32" s="13" t="n"/>
+      <c r="P32" s="13" t="n"/>
+      <c r="Q32" s="96" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="187">
+      <c r="A33" s="24" t="n"/>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
+      <c r="J33" s="24" t="n"/>
+      <c r="K33" s="24" t="n"/>
+      <c r="L33" s="325">
+        <f>IF((COUNT(E33)+COUNT(F33)+COUNT(G33)+COUNT(H33)+COUNT(I33)+COUNT(J33)+COUNT(K33))=0,"",IFERROR(E33/5*0.3,0)+IFERROR(F33/5*0.2,0)+IFERROR(G33/5*0.15,0)+IFERROR(H33/5*0.15,0)+IFERROR(I33/5*0.1,0)+IFERROR(J33/5*0.05,0)+IFERROR(K33/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M33" s="11">
+        <f>IF(L33="","",IF(L33&gt;=0.85,"Meets/Exceeds",IF(L33&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N33" s="6" t="n"/>
+      <c r="O33" s="11" t="n"/>
+      <c r="P33" s="11" t="n"/>
+      <c r="Q33" s="96" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="187">
+      <c r="A34" s="24" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
+      <c r="J34" s="24" t="n"/>
+      <c r="K34" s="24" t="n"/>
+      <c r="L34" s="326">
+        <f>IF((COUNT(E34)+COUNT(F34)+COUNT(G34)+COUNT(H34)+COUNT(I34)+COUNT(J34)+COUNT(K34))=0,"",IFERROR(E34/5*0.3,0)+IFERROR(F34/5*0.2,0)+IFERROR(G34/5*0.15,0)+IFERROR(H34/5*0.15,0)+IFERROR(I34/5*0.1,0)+IFERROR(J34/5*0.05,0)+IFERROR(K34/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M34" s="13">
+        <f>IF(L34="","",IF(L34&gt;=0.85,"Meets/Exceeds",IF(L34&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N34" s="8" t="n"/>
+      <c r="O34" s="13" t="n"/>
+      <c r="P34" s="13" t="n"/>
+      <c r="Q34" s="96" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="187">
+      <c r="A35" s="24" t="n"/>
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
+      <c r="J35" s="24" t="n"/>
+      <c r="K35" s="24" t="n"/>
+      <c r="L35" s="325">
+        <f>IF((COUNT(E35)+COUNT(F35)+COUNT(G35)+COUNT(H35)+COUNT(I35)+COUNT(J35)+COUNT(K35))=0,"",IFERROR(E35/5*0.3,0)+IFERROR(F35/5*0.2,0)+IFERROR(G35/5*0.15,0)+IFERROR(H35/5*0.15,0)+IFERROR(I35/5*0.1,0)+IFERROR(J35/5*0.05,0)+IFERROR(K35/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M35" s="11">
+        <f>IF(L35="","",IF(L35&gt;=0.85,"Meets/Exceeds",IF(L35&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N35" s="6" t="n"/>
+      <c r="O35" s="11" t="n"/>
+      <c r="P35" s="11" t="n"/>
+      <c r="Q35" s="96" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="187">
+      <c r="A36" s="24" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="24" t="n"/>
+      <c r="J36" s="24" t="n"/>
+      <c r="K36" s="24" t="n"/>
+      <c r="L36" s="326">
+        <f>IF((COUNT(E36)+COUNT(F36)+COUNT(G36)+COUNT(H36)+COUNT(I36)+COUNT(J36)+COUNT(K36))=0,"",IFERROR(E36/5*0.3,0)+IFERROR(F36/5*0.2,0)+IFERROR(G36/5*0.15,0)+IFERROR(H36/5*0.15,0)+IFERROR(I36/5*0.1,0)+IFERROR(J36/5*0.05,0)+IFERROR(K36/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M36" s="13">
+        <f>IF(L36="","",IF(L36&gt;=0.85,"Meets/Exceeds",IF(L36&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N36" s="8" t="n"/>
+      <c r="O36" s="13" t="n"/>
+      <c r="P36" s="13" t="n"/>
+      <c r="Q36" s="96" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="187">
+      <c r="A37" s="24" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="24" t="n"/>
+      <c r="J37" s="24" t="n"/>
+      <c r="K37" s="24" t="n"/>
+      <c r="L37" s="325">
+        <f>IF((COUNT(E37)+COUNT(F37)+COUNT(G37)+COUNT(H37)+COUNT(I37)+COUNT(J37)+COUNT(K37))=0,"",IFERROR(E37/5*0.3,0)+IFERROR(F37/5*0.2,0)+IFERROR(G37/5*0.15,0)+IFERROR(H37/5*0.15,0)+IFERROR(I37/5*0.1,0)+IFERROR(J37/5*0.05,0)+IFERROR(K37/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M37" s="11">
+        <f>IF(L37="","",IF(L37&gt;=0.85,"Meets/Exceeds",IF(L37&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N37" s="6" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="96" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="187">
+      <c r="A38" s="24" t="n"/>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
+      <c r="J38" s="24" t="n"/>
+      <c r="K38" s="24" t="n"/>
+      <c r="L38" s="326">
+        <f>IF((COUNT(E38)+COUNT(F38)+COUNT(G38)+COUNT(H38)+COUNT(I38)+COUNT(J38)+COUNT(K38))=0,"",IFERROR(E38/5*0.3,0)+IFERROR(F38/5*0.2,0)+IFERROR(G38/5*0.15,0)+IFERROR(H38/5*0.15,0)+IFERROR(I38/5*0.1,0)+IFERROR(J38/5*0.05,0)+IFERROR(K38/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M38" s="13">
+        <f>IF(L38="","",IF(L38&gt;=0.85,"Meets/Exceeds",IF(L38&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N38" s="8" t="n"/>
+      <c r="O38" s="13" t="n"/>
+      <c r="P38" s="13" t="n"/>
+      <c r="Q38" s="96" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="187">
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="24" t="n"/>
+      <c r="J39" s="24" t="n"/>
+      <c r="K39" s="24" t="n"/>
+      <c r="L39" s="325">
+        <f>IF((COUNT(E39)+COUNT(F39)+COUNT(G39)+COUNT(H39)+COUNT(I39)+COUNT(J39)+COUNT(K39))=0,"",IFERROR(E39/5*0.3,0)+IFERROR(F39/5*0.2,0)+IFERROR(G39/5*0.15,0)+IFERROR(H39/5*0.15,0)+IFERROR(I39/5*0.1,0)+IFERROR(J39/5*0.05,0)+IFERROR(K39/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M39" s="11">
+        <f>IF(L39="","",IF(L39&gt;=0.85,"Meets/Exceeds",IF(L39&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N39" s="6" t="n"/>
+      <c r="O39" s="11" t="n"/>
+      <c r="P39" s="11" t="n"/>
+      <c r="Q39" s="96" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="187">
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="24" t="n"/>
+      <c r="J40" s="24" t="n"/>
+      <c r="K40" s="24" t="n"/>
+      <c r="L40" s="326">
+        <f>IF((COUNT(E40)+COUNT(F40)+COUNT(G40)+COUNT(H40)+COUNT(I40)+COUNT(J40)+COUNT(K40))=0,"",IFERROR(E40/5*0.3,0)+IFERROR(F40/5*0.2,0)+IFERROR(G40/5*0.15,0)+IFERROR(H40/5*0.15,0)+IFERROR(I40/5*0.1,0)+IFERROR(J40/5*0.05,0)+IFERROR(K40/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M40" s="13">
+        <f>IF(L40="","",IF(L40&gt;=0.85,"Meets/Exceeds",IF(L40&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N40" s="8" t="n"/>
+      <c r="O40" s="13" t="n"/>
+      <c r="P40" s="13" t="n"/>
+      <c r="Q40" s="96" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="187">
+      <c r="A41" s="24" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="24" t="n"/>
+      <c r="J41" s="24" t="n"/>
+      <c r="K41" s="24" t="n"/>
+      <c r="L41" s="325">
+        <f>IF((COUNT(E41)+COUNT(F41)+COUNT(G41)+COUNT(H41)+COUNT(I41)+COUNT(J41)+COUNT(K41))=0,"",IFERROR(E41/5*0.3,0)+IFERROR(F41/5*0.2,0)+IFERROR(G41/5*0.15,0)+IFERROR(H41/5*0.15,0)+IFERROR(I41/5*0.1,0)+IFERROR(J41/5*0.05,0)+IFERROR(K41/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M41" s="11">
+        <f>IF(L41="","",IF(L41&gt;=0.85,"Meets/Exceeds",IF(L41&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N41" s="6" t="n"/>
+      <c r="O41" s="11" t="n"/>
+      <c r="P41" s="11" t="n"/>
+      <c r="Q41" s="96" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="187">
+      <c r="A42" s="24" t="n"/>
+      <c r="B42" s="24" t="n"/>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="24" t="n"/>
+      <c r="H42" s="24" t="n"/>
+      <c r="I42" s="24" t="n"/>
+      <c r="J42" s="24" t="n"/>
+      <c r="K42" s="24" t="n"/>
+      <c r="L42" s="326">
+        <f>IF((COUNT(E42)+COUNT(F42)+COUNT(G42)+COUNT(H42)+COUNT(I42)+COUNT(J42)+COUNT(K42))=0,"",IFERROR(E42/5*0.3,0)+IFERROR(F42/5*0.2,0)+IFERROR(G42/5*0.15,0)+IFERROR(H42/5*0.15,0)+IFERROR(I42/5*0.1,0)+IFERROR(J42/5*0.05,0)+IFERROR(K42/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M42" s="13">
+        <f>IF(L42="","",IF(L42&gt;=0.85,"Meets/Exceeds",IF(L42&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="13" t="n"/>
+      <c r="P42" s="13" t="n"/>
+      <c r="Q42" s="96" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="187">
+      <c r="A43" s="24" t="n"/>
+      <c r="B43" s="24" t="n"/>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="24" t="n"/>
+      <c r="J43" s="24" t="n"/>
+      <c r="K43" s="24" t="n"/>
+      <c r="L43" s="325">
+        <f>IF((COUNT(E43)+COUNT(F43)+COUNT(G43)+COUNT(H43)+COUNT(I43)+COUNT(J43)+COUNT(K43))=0,"",IFERROR(E43/5*0.3,0)+IFERROR(F43/5*0.2,0)+IFERROR(G43/5*0.15,0)+IFERROR(H43/5*0.15,0)+IFERROR(I43/5*0.1,0)+IFERROR(J43/5*0.05,0)+IFERROR(K43/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M43" s="11">
+        <f>IF(L43="","",IF(L43&gt;=0.85,"Meets/Exceeds",IF(L43&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N43" s="6" t="n"/>
+      <c r="O43" s="11" t="n"/>
+      <c r="P43" s="11" t="n"/>
+      <c r="Q43" s="96" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="187">
+      <c r="A44" s="24" t="n"/>
+      <c r="B44" s="24" t="n"/>
+      <c r="C44" s="24" t="n"/>
+      <c r="D44" s="24" t="n"/>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="24" t="n"/>
+      <c r="G44" s="24" t="n"/>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="24" t="n"/>
+      <c r="J44" s="24" t="n"/>
+      <c r="K44" s="24" t="n"/>
+      <c r="L44" s="326">
+        <f>IF((COUNT(E44)+COUNT(F44)+COUNT(G44)+COUNT(H44)+COUNT(I44)+COUNT(J44)+COUNT(K44))=0,"",IFERROR(E44/5*0.3,0)+IFERROR(F44/5*0.2,0)+IFERROR(G44/5*0.15,0)+IFERROR(H44/5*0.15,0)+IFERROR(I44/5*0.1,0)+IFERROR(J44/5*0.05,0)+IFERROR(K44/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M44" s="13">
+        <f>IF(L44="","",IF(L44&gt;=0.85,"Meets/Exceeds",IF(L44&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N44" s="8" t="n"/>
+      <c r="O44" s="13" t="n"/>
+      <c r="P44" s="13" t="n"/>
+      <c r="Q44" s="96" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="187">
+      <c r="A45" s="24" t="n"/>
+      <c r="B45" s="24" t="n"/>
+      <c r="C45" s="24" t="n"/>
+      <c r="D45" s="24" t="n"/>
+      <c r="E45" s="24" t="n"/>
+      <c r="F45" s="24" t="n"/>
+      <c r="G45" s="24" t="n"/>
+      <c r="H45" s="24" t="n"/>
+      <c r="I45" s="24" t="n"/>
+      <c r="J45" s="24" t="n"/>
+      <c r="K45" s="24" t="n"/>
+      <c r="L45" s="325">
+        <f>IF((COUNT(E45)+COUNT(F45)+COUNT(G45)+COUNT(H45)+COUNT(I45)+COUNT(J45)+COUNT(K45))=0,"",IFERROR(E45/5*0.3,0)+IFERROR(F45/5*0.2,0)+IFERROR(G45/5*0.15,0)+IFERROR(H45/5*0.15,0)+IFERROR(I45/5*0.1,0)+IFERROR(J45/5*0.05,0)+IFERROR(K45/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M45" s="11">
+        <f>IF(L45="","",IF(L45&gt;=0.85,"Meets/Exceeds",IF(L45&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N45" s="6" t="n"/>
+      <c r="O45" s="11" t="n"/>
+      <c r="P45" s="11" t="n"/>
+      <c r="Q45" s="96" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="187">
+      <c r="A46" s="24" t="n"/>
+      <c r="B46" s="24" t="n"/>
+      <c r="C46" s="24" t="n"/>
+      <c r="D46" s="24" t="n"/>
+      <c r="E46" s="24" t="n"/>
+      <c r="F46" s="24" t="n"/>
+      <c r="G46" s="24" t="n"/>
+      <c r="H46" s="24" t="n"/>
+      <c r="I46" s="24" t="n"/>
+      <c r="J46" s="24" t="n"/>
+      <c r="K46" s="24" t="n"/>
+      <c r="L46" s="326">
+        <f>IF((COUNT(E46)+COUNT(F46)+COUNT(G46)+COUNT(H46)+COUNT(I46)+COUNT(J46)+COUNT(K46))=0,"",IFERROR(E46/5*0.3,0)+IFERROR(F46/5*0.2,0)+IFERROR(G46/5*0.15,0)+IFERROR(H46/5*0.15,0)+IFERROR(I46/5*0.1,0)+IFERROR(J46/5*0.05,0)+IFERROR(K46/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M46" s="13">
+        <f>IF(L46="","",IF(L46&gt;=0.85,"Meets/Exceeds",IF(L46&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N46" s="8" t="n"/>
+      <c r="O46" s="13" t="n"/>
+      <c r="P46" s="13" t="n"/>
+      <c r="Q46" s="96" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="187">
+      <c r="A47" s="24" t="n"/>
+      <c r="B47" s="24" t="n"/>
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="24" t="n"/>
+      <c r="G47" s="24" t="n"/>
+      <c r="H47" s="24" t="n"/>
+      <c r="I47" s="24" t="n"/>
+      <c r="J47" s="24" t="n"/>
+      <c r="K47" s="24" t="n"/>
+      <c r="L47" s="325">
+        <f>IF((COUNT(E47)+COUNT(F47)+COUNT(G47)+COUNT(H47)+COUNT(I47)+COUNT(J47)+COUNT(K47))=0,"",IFERROR(E47/5*0.3,0)+IFERROR(F47/5*0.2,0)+IFERROR(G47/5*0.15,0)+IFERROR(H47/5*0.15,0)+IFERROR(I47/5*0.1,0)+IFERROR(J47/5*0.05,0)+IFERROR(K47/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M47" s="11">
+        <f>IF(L47="","",IF(L47&gt;=0.85,"Meets/Exceeds",IF(L47&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N47" s="6" t="n"/>
+      <c r="O47" s="11" t="n"/>
+      <c r="P47" s="11" t="n"/>
+      <c r="Q47" s="96" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="187">
+      <c r="A48" s="24" t="n"/>
+      <c r="B48" s="24" t="n"/>
+      <c r="C48" s="24" t="n"/>
+      <c r="D48" s="24" t="n"/>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="24" t="n"/>
+      <c r="G48" s="24" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="24" t="n"/>
+      <c r="J48" s="24" t="n"/>
+      <c r="K48" s="24" t="n"/>
+      <c r="L48" s="326">
+        <f>IF((COUNT(E48)+COUNT(F48)+COUNT(G48)+COUNT(H48)+COUNT(I48)+COUNT(J48)+COUNT(K48))=0,"",IFERROR(E48/5*0.3,0)+IFERROR(F48/5*0.2,0)+IFERROR(G48/5*0.15,0)+IFERROR(H48/5*0.15,0)+IFERROR(I48/5*0.1,0)+IFERROR(J48/5*0.05,0)+IFERROR(K48/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M48" s="13">
+        <f>IF(L48="","",IF(L48&gt;=0.85,"Meets/Exceeds",IF(L48&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N48" s="8" t="n"/>
+      <c r="O48" s="13" t="n"/>
+      <c r="P48" s="13" t="n"/>
+      <c r="Q48" s="96" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="187">
+      <c r="A49" s="24" t="n"/>
+      <c r="B49" s="24" t="n"/>
+      <c r="C49" s="24" t="n"/>
+      <c r="D49" s="24" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="24" t="n"/>
+      <c r="G49" s="24" t="n"/>
+      <c r="H49" s="24" t="n"/>
+      <c r="I49" s="24" t="n"/>
+      <c r="J49" s="24" t="n"/>
+      <c r="K49" s="24" t="n"/>
+      <c r="L49" s="325">
+        <f>IF((COUNT(E49)+COUNT(F49)+COUNT(G49)+COUNT(H49)+COUNT(I49)+COUNT(J49)+COUNT(K49))=0,"",IFERROR(E49/5*0.3,0)+IFERROR(F49/5*0.2,0)+IFERROR(G49/5*0.15,0)+IFERROR(H49/5*0.15,0)+IFERROR(I49/5*0.1,0)+IFERROR(J49/5*0.05,0)+IFERROR(K49/5*0.05,0))</f>
+        <v/>
+      </c>
+      <c r="M49" s="11">
+        <f>IF(L49="","",IF(L49&gt;=0.85,"Meets/Exceeds",IF(L49&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="N49" s="6" t="n"/>
+      <c r="O49" s="11" t="n"/>
+      <c r="P49" s="11" t="n"/>
+      <c r="Q49" s="96" t="n"/>
+    </row>
+    <row r="51" ht="15.6" customHeight="1" s="187">
+      <c r="A51" s="276" t="inlineStr">
+        <is>
+          <t>TEAM AVERAGE</t>
+        </is>
+      </c>
+      <c r="B51" s="212" t="n"/>
+      <c r="C51" s="212" t="n"/>
+      <c r="D51" s="192" t="n"/>
+      <c r="E51" s="327">
+        <f>IFERROR(AVERAGE(E5:E49),"")</f>
+        <v/>
+      </c>
+      <c r="F51" s="327">
+        <f>IFERROR(AVERAGE(F5:F49),"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="327">
+        <f>IFERROR(AVERAGE(G5:G49),"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="327">
+        <f>IFERROR(AVERAGE(H5:H49),"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="327">
+        <f>IFERROR(AVERAGE(I5:I49),"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="327">
+        <f>IFERROR(AVERAGE(J5:J49),"")</f>
+        <v/>
+      </c>
+      <c r="K51" s="327">
+        <f>IFERROR(AVERAGE(K5:K49),"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="328">
+        <f>IFERROR(AVERAGE(L5:L49),"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="14" t="n"/>
+      <c r="N51" s="29" t="inlineStr">
+        <is>
+          <t>Average of logged touches</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="21.95" customHeight="1" s="187">
+      <c r="A53" s="281" t="inlineStr">
+        <is>
+          <t>TEAM / JOURNEY SCORES — MULTI-TOUCH CASES</t>
+        </is>
+      </c>
+      <c r="B53" s="212" t="n"/>
+      <c r="C53" s="212" t="n"/>
+      <c r="D53" s="212" t="n"/>
+      <c r="E53" s="212" t="n"/>
+      <c r="F53" s="212" t="n"/>
+      <c r="G53" s="212" t="n"/>
+      <c r="H53" s="212" t="n"/>
+      <c r="I53" s="212" t="n"/>
+      <c r="J53" s="212" t="n"/>
+      <c r="K53" s="212" t="n"/>
+      <c r="L53" s="212" t="n"/>
+      <c r="M53" s="212" t="n"/>
+      <c r="N53" s="212" t="n"/>
+      <c r="O53" s="212" t="n"/>
+      <c r="P53" s="192" t="n"/>
+    </row>
+    <row r="54" ht="32.1" customHeight="1" s="187">
+      <c r="A54" s="279" t="inlineStr">
+        <is>
+          <t>Team Score  =  20% × Level 1 avg touch  +  30% × Level 2 avg touch  +  30% × (Journey Outcome ÷ 5)  +  20% × (Continuity of Support ÷ 5)   │   Level 2 touches carry a higher weight in the team aggregate.</t>
+        </is>
+      </c>
+      <c r="B54" s="212" t="n"/>
+      <c r="C54" s="212" t="n"/>
+      <c r="D54" s="212" t="n"/>
+      <c r="E54" s="212" t="n"/>
+      <c r="F54" s="212" t="n"/>
+      <c r="G54" s="212" t="n"/>
+      <c r="H54" s="212" t="n"/>
+      <c r="I54" s="212" t="n"/>
+      <c r="J54" s="212" t="n"/>
+      <c r="K54" s="212" t="n"/>
+      <c r="L54" s="212" t="n"/>
+      <c r="M54" s="212" t="n"/>
+      <c r="N54" s="212" t="n"/>
+      <c r="O54" s="212" t="n"/>
+      <c r="P54" s="192" t="n"/>
+    </row>
+    <row r="55" ht="26.1" customHeight="1" s="187">
+      <c r="A55" s="278" t="inlineStr">
+        <is>
+          <t>Journey / Case ID(s)</t>
+        </is>
+      </c>
+      <c r="B55" s="192" t="n"/>
+      <c r="C55" s="278" t="inlineStr">
+        <is>
+          <t>Touches</t>
+        </is>
+      </c>
+      <c r="D55" s="23" t="inlineStr">
+        <is>
+          <t>Avg Touch % (ref)</t>
+        </is>
+      </c>
+      <c r="E55" s="23" t="inlineStr">
+        <is>
+          <t>Journey Outcome</t>
+        </is>
+      </c>
+      <c r="F55" s="23" t="inlineStr">
+        <is>
+          <t>Continuity of Support</t>
+        </is>
+      </c>
+      <c r="G55" s="23" t="inlineStr">
+        <is>
+          <t>TEAM SCORE</t>
+        </is>
+      </c>
+      <c r="H55" s="278" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+      <c r="I55" s="214" t="inlineStr">
+        <is>
+          <t>Journey notes (where the chain broke / recovered)</t>
+        </is>
+      </c>
+      <c r="J55" s="212" t="n"/>
+      <c r="K55" s="212" t="n"/>
+      <c r="L55" s="212" t="n"/>
+      <c r="M55" s="212" t="n"/>
+      <c r="N55" s="192" t="n"/>
+    </row>
+    <row r="56" ht="48" customHeight="1" s="187">
+      <c r="A56" s="329" t="n"/>
+      <c r="B56" s="244" t="n"/>
+      <c r="C56" s="13">
+        <f>IF(A56="","",COUNTIF(B5:B49,A56))</f>
+        <v/>
+      </c>
+      <c r="D56" s="330">
+        <f>IF(A56="","",IFERROR(AVERAGEIF(B5:B49,A56,L5:L49),""))</f>
+        <v/>
+      </c>
+      <c r="E56" s="7" t="n"/>
+      <c r="F56" s="7" t="n"/>
+      <c r="G56" s="98">
+        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(IFERROR(VALUE(LEFT(E56,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F56,1)),0)/5),""))</f>
+        <v/>
+      </c>
+      <c r="H56" s="13">
+        <f>IF(G56="","",IF(G56&gt;=0.85,"Meets/Exceeds",IF(G56&gt;=0.7,"Developing","Needs Improvement")))</f>
+        <v/>
+      </c>
+      <c r="I56" s="322" t="n"/>
+      <c r="J56" s="243" t="n"/>
+      <c r="K56" s="243" t="n"/>
+      <c r="L56" s="243" t="n"/>
+      <c r="M56" s="243" t="n"/>
+      <c r="N56" s="244" t="n"/>
+    </row>
+    <row r="57" ht="27.95" customHeight="1" s="187">
+      <c r="A57" s="289" t="n"/>
+      <c r="B57" s="244" t="n"/>
+      <c r="C57" s="13">
+        <f>IF(A57="","",COUNTIF(B5:B49,A57))</f>
+        <v/>
+      </c>
+      <c r="D57" s="330">
+        <f>IF(A57="","",IFERROR(AVERAGEIF(B5:B49,A57,L5:L49),""))</f>
+        <v/>
+      </c>
+      <c r="E57" s="7" t="n"/>
+      <c r="F57" s="7" t="n"/>
+      <c r="G57" s="98">
+        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(IFERROR(VALUE(LEFT(E57,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F57,1)),0)/5),""))</f>
+        <v/>
+      </c>
+      <c r="H57" s="13">
+        <f>IF(G57="","",IF(G57&gt;=0.85,"Meets/Exceeds",IF(G57&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="I57" s="331" t="n"/>
+      <c r="J57" s="243" t="n"/>
+      <c r="K57" s="243" t="n"/>
+      <c r="L57" s="243" t="n"/>
+      <c r="M57" s="243" t="n"/>
+      <c r="N57" s="244" t="n"/>
+    </row>
+    <row r="58" ht="27.95" customHeight="1" s="187">
+      <c r="A58" s="289" t="n"/>
+      <c r="B58" s="244" t="n"/>
+      <c r="C58" s="11">
+        <f>IF(A58="","",COUNTIF(B5:B49,A58))</f>
+        <v/>
+      </c>
+      <c r="D58" s="332">
+        <f>IF(A58="","",IFERROR(AVERAGEIF(B5:B49,A58,L5:L49),""))</f>
+        <v/>
+      </c>
+      <c r="E58" s="7" t="n"/>
+      <c r="F58" s="7" t="n"/>
+      <c r="G58" s="99">
+        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(IFERROR(VALUE(LEFT(E58,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F58,1)),0)/5),""))</f>
+        <v/>
+      </c>
+      <c r="H58" s="11">
+        <f>IF(G58="","",IF(G58&gt;=0.85,"Meets/Exceeds",IF(G58&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="I58" s="331" t="n"/>
+      <c r="J58" s="243" t="n"/>
+      <c r="K58" s="243" t="n"/>
+      <c r="L58" s="243" t="n"/>
+      <c r="M58" s="243" t="n"/>
+      <c r="N58" s="244" t="n"/>
+    </row>
+    <row r="59" ht="27.95" customHeight="1" s="187">
+      <c r="A59" s="289" t="n"/>
+      <c r="B59" s="244" t="n"/>
+      <c r="C59" s="13">
+        <f>IF(A59="","",COUNTIF(B5:B49,A59))</f>
+        <v/>
+      </c>
+      <c r="D59" s="330">
+        <f>IF(A59="","",IFERROR(AVERAGEIF(B5:B49,A59,L5:L49),""))</f>
+        <v/>
+      </c>
+      <c r="E59" s="7" t="n"/>
+      <c r="F59" s="7" t="n"/>
+      <c r="G59" s="98">
+        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(IFERROR(VALUE(LEFT(E59,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F59,1)),0)/5),""))</f>
+        <v/>
+      </c>
+      <c r="H59" s="13">
+        <f>IF(G59="","",IF(G59&gt;=0.85,"Meets/Exceeds",IF(G59&gt;=0.7,"Developing","Needs Improv.")))</f>
+        <v/>
+      </c>
+      <c r="I59" s="331" t="n"/>
+      <c r="J59" s="243" t="n"/>
+      <c r="K59" s="243" t="n"/>
+      <c r="L59" s="243" t="n"/>
+      <c r="M59" s="243" t="n"/>
+      <c r="N59" s="244" t="n"/>
+    </row>
+    <row r="60" ht="27.95" customHeight="1" s="187">
+      <c r="A60" s="298" t="inlineStr">
+        <is>
+          <t>Template rows: type a Case ID in the first column — Touches and Avg Touch % auto-fill from the log above, then judge Outcome and Continuity (0-5). For journeys spanning multiple Case IDs (like the pre-loaded one), enter the Avg Touch % formula over the journey's row range manually.</t>
+        </is>
+      </c>
+      <c r="B60" s="243" t="n"/>
+      <c r="C60" s="243" t="n"/>
+      <c r="D60" s="243" t="n"/>
+      <c r="E60" s="243" t="n"/>
+      <c r="F60" s="243" t="n"/>
+      <c r="G60" s="243" t="n"/>
+      <c r="H60" s="243" t="n"/>
+      <c r="I60" s="243" t="n"/>
+      <c r="J60" s="243" t="n"/>
+      <c r="K60" s="243" t="n"/>
+      <c r="L60" s="243" t="n"/>
+      <c r="M60" s="243" t="n"/>
+      <c r="N60" s="244" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="I55:N55"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="I59:N59"/>
+    <mergeCell ref="A54:P54"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A53:P53"/>
+    <mergeCell ref="A60:N60"/>
+    <mergeCell ref="I56:N56"/>
+    <mergeCell ref="A3:P3"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="I57:N57"/>
+    <mergeCell ref="I58:N58"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="22">
+      <formula>$G$56&gt;=0.85</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="21">
+      <formula>$G$56&gt;=0.85</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="20">
+      <formula>AND($G$56&gt;=0.7,$G$56&lt;0.85)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="19">
+      <formula>$G$56&lt;0.7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G56:G59">
+    <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="2">
+      <formula>0.85</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="between" dxfId="1">
+      <formula>0.7</formula>
+      <formula>0.8499</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="0">
+      <formula>0.7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H56:H59">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
+      <formula>"Meets/Exceeds"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
+      <formula>"Developing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
+      <formula>"Needs Improv."</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:L49">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="2">
+      <formula>0.85</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>0.7</formula>
+      <formula>0.8499</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
+      <formula>0.7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M49">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="9">
+      <formula>"Meets/Exceeds"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="8">
+      <formula>"Developing"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="7">
+      <formula>"Needs Improv."</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O49">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="2">
+      <formula>"Resolver"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
+      <formula>"Progress Builder"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="4">
+      <formula>"Maintainer"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
+      <formula>"Regression Contributor"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P49">
+    <cfRule type="cellIs" priority="21" operator="greaterThanOrEqual" dxfId="2">
+      <formula>4</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="between" dxfId="1">
+      <formula>2</formula>
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="23" operator="lessThanOrEqual" dxfId="0">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
+    <dataValidation sqref="E5:K49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5." type="whole">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="O5:O49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Resolver, Progress Builder, Maintainer, Breaker, or N/A." type="list">
+      <formula1>"Resolver,Progress Builder,Maintainer,Regression Contributor,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="Q5:Q49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Please select Level 1 or Level 2." promptTitle="Agent Level" prompt="Level 1 = front-line support.  Level 2 = senior / escalation support." type="list">
+      <formula1>"Level 1,Level 2"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8216,6 +9996,1085 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B1:E64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="187" min="1" max="1"/>
+    <col width="52" customWidth="1" style="187" min="2" max="2"/>
+    <col width="18" customWidth="1" style="187" min="3" max="3"/>
+    <col width="68" customWidth="1" style="187" min="4" max="4"/>
+    <col width="56" customWidth="1" style="187" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="187">
+      <c r="B1" s="333" t="inlineStr">
+        <is>
+          <t>BEHAVIORAL INDICATOR GUIDE — WHY EACH INDICATOR IS HERE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="187">
+      <c r="B2" s="334" t="inlineStr">
+        <is>
+          <t>This sheet explains the purpose and justification for every behavioral indicator in the QA Scoring Form. Use it to understand what each indicator is measuring, why it is included, and what a failure to meet it looks like in practice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1" s="187">
+      <c r="B3" s="63" t="n"/>
+      <c r="C3" s="63" t="n"/>
+      <c r="D3" s="63" t="n"/>
+      <c r="E3" s="63" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" s="187">
+      <c r="B4" s="335" t="inlineStr">
+        <is>
+          <t>Behavioral Indicator</t>
+        </is>
+      </c>
+      <c r="C4" s="335" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="D4" s="335" t="inlineStr">
+        <is>
+          <t>Why This Indicator Is Here</t>
+        </is>
+      </c>
+      <c r="E4" s="335" t="inlineStr">
+        <is>
+          <t>What Failure Looks Like</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" s="187">
+      <c r="B5" s="336" t="inlineStr">
+        <is>
+          <t>1. RESOLUTION / PROGRESS TOWARD RESOLUTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1" s="187">
+      <c r="B6" s="337" t="inlineStr">
+        <is>
+          <t>Measures whether the customer left the interaction in a meaningfully better position than when they called. Every other category exists in service of this one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1" s="187">
+      <c r="B7" s="338" t="inlineStr">
+        <is>
+          <t>Resolved the issue or achieved the best possible outcome (RMA, valid escalation, limitation explained, education)</t>
+        </is>
+      </c>
+      <c r="C7" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D7" s="340" t="inlineStr">
+        <is>
+          <t>This is the entire point of a support interaction. Resolution is defined broadly: a fully fixed issue is the strongest outcome, but a correctly initiated RMA, a valid escalation with complete documentation, a clearly explained product limitation, or meaningful customer education all count. When the agent achieves the best available outcome given the situation, the interaction has succeeded at its core purpose. No other category can compensate for a consistent failure to reach any positive outcome.</t>
+        </is>
+      </c>
+      <c r="E7" s="341" t="inlineStr">
+        <is>
+          <t>Customer ends the call with the same problem and no path forward. Case marked Resolved when the issue is unresolved. Generic KB article sent with no investigation. Customer told to monitor and call back with no defined expectation or plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1" s="187">
+      <c r="B8" s="342" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before reaching a conclusion</t>
+        </is>
+      </c>
+      <c r="C8" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D8" s="344" t="inlineStr">
+        <is>
+          <t>Conclusions without evidence are guesses. An agent who decides the problem is the ISP, the customer's device, or a hardware defect without performing the relevant diagnostic steps is as likely to give wrong direction as right. Reasonable troubleshooting is what separates a supported conclusion from an unsupported assumption. It also protects the escalation team from receiving cases that could have been resolved at Level 1.</t>
+        </is>
+      </c>
+      <c r="E8" s="345" t="inlineStr">
+        <is>
+          <t>Agent attributes the problem to the ISP before checking connection from the router. Agent recommends a factory reset without first ruling out configuration issues. Agent escalates after one basic step without exhausting available Level 1 options. Agent skips diagnostic questions and jumps directly to a resolution action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" s="187">
+      <c r="B9" s="338" t="inlineStr">
+        <is>
+          <t>Resolution path was appropriate for the situation and warranty status</t>
+        </is>
+      </c>
+      <c r="C9" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D9" s="340" t="inlineStr">
+        <is>
+          <t>In-warranty and out-of-warranty products require different resolution paths. Recommending an RMA for an out-of-warranty product, or failing to initiate one for an in-warranty product with a confirmed hardware fault, reflects a failure to navigate the support framework correctly. This indicator checks that the agent matched the resolution path to the actual situation including warranty status, product eligibility, and issue type.</t>
+        </is>
+      </c>
+      <c r="E9" s="341" t="inlineStr">
+        <is>
+          <t>Agent initiates an RMA for an out-of-warranty product without a policy exception. Agent closes a confirmed hardware failure on an in-warranty product without initiating replacement. Agent applies an in-warranty resolution script to an out-of-warranty situation. Agent does not confirm which product families qualify for best-effort OOW troubleshooting before dismissing the customer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1" s="187">
+      <c r="B10" s="342" t="inlineStr">
+        <is>
+          <t>Customer was moved meaningfully closer to a solution</t>
+        </is>
+      </c>
+      <c r="C10" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D10" s="344" t="inlineStr">
+        <is>
+          <t>Not every issue can be fully resolved in one interaction. This indicator captures progress: did the customer leave in a materially better position than when they called? A case that ends without full resolution can still succeed if the customer understands their situation clearly, knows exactly what their next step is, and has a realistic reason to believe the problem can be addressed. Progress must be demonstrable. Vague reassurance does not count.</t>
+        </is>
+      </c>
+      <c r="E10" s="345" t="inlineStr">
+        <is>
+          <t>Customer still does not know what is wrong or what to do next. Agent closes the case after troubleshooting fails with no further guidance. Agent says try that and see without a specific action for the customer. Customer calls back immediately after the previous interaction with the same question.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1" s="187">
+      <c r="B11" s="338" t="inlineStr">
+        <is>
+          <t>Troubleshooting was conducted before any self-help content or KB articles were shared — generic self-help was not used as a substitute for investigation</t>
+        </is>
+      </c>
+      <c r="C11" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D11" s="340" t="inlineStr">
+        <is>
+          <t>Sending a customer a KB article without first investigating their specific issue is not support — it is deflection. The agent has shifted the work back to the customer without adding any diagnostic value. Generic self-help can be a useful complement to a completed investigation, but it cannot replace one. This indicator reflects one of the most visible systemic failures the Support Organization Reset is designed to correct: the use of KB articles as a way to close interactions without doing the work.</t>
+        </is>
+      </c>
+      <c r="E11" s="341" t="inlineStr">
+        <is>
+          <t>Agent sends a KB link as the primary response to a reported issue. Agent provides a reset guide before asking a single diagnostic question. Agent shares a general troubleshooting article without confirming whether it applies to the customer's actual configuration. Self-help is provided to an OOW customer as the full extent of assistance with no investigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1" s="187">
+      <c r="B12" s="342" t="inlineStr">
+        <is>
+          <t>For out-of-warranty products: provided best-effort troubleshooting, explained product limitations clearly, and did not use warranty status as a reason to stop helping — mark N.A. if product is in warranty</t>
+        </is>
+      </c>
+      <c r="C12" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D12" s="344" t="inlineStr">
+        <is>
+          <t>The previous operating model treated out-of-warranty status as permission to dismiss the customer with minimal assistance. The Support Organization Reset replaces that model with a best-effort engagement standard for eligible products: agents are expected to investigate, troubleshoot as far as the product and issue type allow, communicate clearly about what is and is not possible, and leave the customer with something useful. OOW status determines the resolution ceiling, not the quality of effort.</t>
+        </is>
+      </c>
+      <c r="E12" s="345" t="inlineStr">
+        <is>
+          <t>Agent says your product is out of warranty, I cannot help without making any troubleshooting attempt. Agent recommends a paid support option before providing any assistance. Agent fails to explain what best-effort troubleshooting means or what the customer can realistically expect. Agent applies a blanket refusal without confirming which product families qualify for OOW troubleshooting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1" s="187">
+      <c r="B13" s="63" t="n"/>
+      <c r="C13" s="63" t="n"/>
+      <c r="D13" s="63" t="n"/>
+      <c r="E13" s="63" t="n"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" s="187">
+      <c r="B14" s="336" t="inlineStr">
+        <is>
+          <t>2. TECHNICAL ACCURACY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1" s="187">
+      <c r="B15" s="337" t="inlineStr">
+        <is>
+          <t>Measures the quality of the agent's diagnostic reasoning and technical guidance. Resolution is impossible without it — correct troubleshooting is the mechanism through which resolution is achieved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" s="187">
+      <c r="B16" s="338" t="inlineStr">
+        <is>
+          <t>Correctly identified the symptoms and asked relevant diagnostic questions</t>
+        </is>
+      </c>
+      <c r="C16" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D16" s="340" t="inlineStr">
+        <is>
+          <t>You cannot fix a problem you have not understood. Correct symptom identification and targeted diagnostic questioning are the first and most important steps in any troubleshooting process. An agent who misidentifies symptoms or asks irrelevant questions will troubleshoot the wrong thing, consume call time on dead ends, and reach wrong conclusions. This indicator captures whether the agent built an accurate picture of the problem before attempting to act on it.</t>
+        </is>
+      </c>
+      <c r="E16" s="341" t="inlineStr">
+        <is>
+          <t>Agent misidentifies a connectivity issue as a speed issue. Agent asks the same clarifying questions a prior agent already documented. Agent skips symptom confirmation and goes straight to a standard resolution script. Agent attributes intermittent disconnections to the wrong component without asking about frequency, affected devices, or network setup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1" s="187">
+      <c r="B17" s="342" t="inlineStr">
+        <is>
+          <t>Identified the root cause (or likely cause) when possible</t>
+        </is>
+      </c>
+      <c r="C17" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D17" s="344" t="inlineStr">
+        <is>
+          <t>Resolution without root cause understanding is unstable — the same issue often recurs when the underlying cause is not addressed. When agents identify the root cause, they resolve it properly, document it meaningfully, and give customers accurate expectations about recurrence. When root cause cannot be confirmed, an honest likely cause with supporting evidence is more useful than a guess. Root cause identification is also the primary input for escalation documentation, KB improvement, and product quality feedback.</t>
+        </is>
+      </c>
+      <c r="E17" s="345" t="inlineStr">
+        <is>
+          <t>Agent resolves the immediate symptom but does not investigate why it occurred. Agent closes a case with unknown cause without exhausting reasonable diagnostic options. Agent states a root cause without providing evidence that supports it. Agent identifies one possible cause and stops without ruling out alternatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1" s="187">
+      <c r="B18" s="338" t="inlineStr">
+        <is>
+          <t>Followed a logical troubleshooting process</t>
+        </is>
+      </c>
+      <c r="C18" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D18" s="340" t="inlineStr">
+        <is>
+          <t>Logical process discipline means working systematically — ruling things in or out in a sensible sequence, not jumping between unrelated steps, and building a coherent picture before acting. Disorganized troubleshooting wastes time, produces contradictory results, and confuses the customer. With the 20-minute escalation pressure removed under the Support Organization Reset, agents are expected to troubleshoot methodically rather than rushing to any available exit.</t>
+        </is>
+      </c>
+      <c r="E18" s="341" t="inlineStr">
+        <is>
+          <t>Agent performs steps in random order without a clear diagnostic rationale. Agent moves from one solution attempt to the next without documenting or analyzing the result of the previous step. Agent circles back to steps already completed without explanation. Agent's approach cannot be justified if asked why a particular step was chosen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1" s="187">
+      <c r="B19" s="342" t="inlineStr">
+        <is>
+          <t>Available tools were used efficiently and appropriately</t>
+        </is>
+      </c>
+      <c r="C19" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D19" s="344" t="inlineStr">
+        <is>
+          <t>Agents have access to remote session capabilities, ticket history, diagnostic portals, and internal knowledge systems. An agent who troubleshoots without using these is working with less information than they could have, effectively handicapping the diagnostic process. This indicator checks that agents are leveraging the tools available to them rather than relying solely on verbal descriptions from the customer, which are often imprecise.</t>
+        </is>
+      </c>
+      <c r="E19" s="345" t="inlineStr">
+        <is>
+          <t>Agent does not initiate a remote session when one would have confirmed or ruled out the issue in minutes. Agent does not review the ticket history before asking the customer to re-explain the problem. Agent uses a tool incorrectly or misinterprets its output. Agent skips tool-based verification and relies on customer self-reporting for a finding that could have been confirmed directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1" s="187">
+      <c r="B20" s="338" t="inlineStr">
+        <is>
+          <t>Gave technically accurate information; no unsupported conclusions</t>
+        </is>
+      </c>
+      <c r="C20" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D20" s="340" t="inlineStr">
+        <is>
+          <t>Inaccurate technical information extends case life, damages customer trust, and sometimes causes real harm — incorrect firmware steps, wrong RMA eligibility, or misrepresented product capabilities can have direct consequences. Unsupported conclusions, particularly ISP blame without evidence, are one of the most recognizable systemic failure patterns the Support Organization Reset names explicitly. Every diagnosis, instruction, and claim should be supportable by evidence, testing, or established technical knowledge.</t>
+        </is>
+      </c>
+      <c r="E20" s="341" t="inlineStr">
+        <is>
+          <t>Agent tells customer their router is defective based on a symptom that could have multiple causes. Agent blames the ISP before checking whether the connection from the router is stable. Agent provides incorrect information about product or firmware compatibility. Agent states a conclusion that contradicts what the diagnostic steps actually showed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1" s="187">
+      <c r="B21" s="63" t="n"/>
+      <c r="C21" s="63" t="n"/>
+      <c r="D21" s="63" t="n"/>
+      <c r="E21" s="63" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="187">
+      <c r="B22" s="336" t="inlineStr">
+        <is>
+          <t>3. COMMUNICATION &amp; CALL CONTROL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1" s="187">
+      <c r="B23" s="337" t="inlineStr">
+        <is>
+          <t>Measures how effectively the agent managed the interaction. Technically correct guidance fails if the customer cannot understand it, follow it, or trust the agent delivering it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1" s="187">
+      <c r="B24" s="338" t="inlineStr">
+        <is>
+          <t>Expectations were set clearly from the start</t>
+        </is>
+      </c>
+      <c r="C24" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D24" s="340" t="inlineStr">
+        <is>
+          <t>Customers who do not know what to expect during a support call become anxious, impatient, and harder to manage. A brief framing at the start — what the agent is about to do, roughly how long a step might take, what the customer should have accessible — reduces friction and increases cooperation throughout the interaction. Setting expectations is also the first visible act of ownership: it signals that the agent is in control and has a plan.</t>
+        </is>
+      </c>
+      <c r="E24" s="341" t="inlineStr">
+        <is>
+          <t>Agent starts troubleshooting immediately without explaining what is about to happen. Customer interrupts frequently because they do not understand what the agent is doing. Agent does not tell the customer how long a hold or diagnostic step will take. Customer is surprised when the call needs to extend or when escalation is needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1" s="187">
+      <c r="B25" s="342" t="inlineStr">
+        <is>
+          <t>Agent maintained call control and troubleshooting flow</t>
+        </is>
+      </c>
+      <c r="C25" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D25" s="344" t="inlineStr">
+        <is>
+          <t>Call control is what allows troubleshooting to proceed without derailment. An agent who cannot maintain the direction of the conversation cannot complete the diagnostic process, cannot meet customer expectations, and cannot deliver the outcome. Call control does not mean dominating the customer — it means keeping the interaction purposeful and directed. Under the Support Organization Reset, longer calls are acceptable when they are productive. Maintaining control across that duration is the critical skill that makes longer calls useful rather than chaotic.</t>
+        </is>
+      </c>
+      <c r="E25" s="345" t="inlineStr">
+        <is>
+          <t>Customer controls the direction of the call and the agent follows rather than leads. Agent allows the conversation to drift into unrelated topics without redirecting. Agent loses control of a frustrated caller and cannot re-engage them productively. Troubleshooting is abandoned mid-process because the agent was unable to navigate a difficult moment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1" s="187">
+      <c r="B26" s="338" t="inlineStr">
+        <is>
+          <t>Used language appropriate to the customer's level and confirmed understanding throughout</t>
+        </is>
+      </c>
+      <c r="C26" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D26" s="340" t="inlineStr">
+        <is>
+          <t>Technical accuracy means nothing if the customer cannot understand the instructions. Agents who use unexplained acronyms, jargon, or overly complex language create confusion that leads to wrong actions, wasted steps, and failed outcomes. Confirming understanding at key points catches comprehension failures before they turn into execution failures. As Linksys moves toward B2B and ISP-aligned support, agents must adjust their communication register depending on the technical sophistication of the person they are serving.</t>
+        </is>
+      </c>
+      <c r="E26" s="341" t="inlineStr">
+        <is>
+          <t>Customer performs the wrong step because the instruction was unclear. Agent uses terms like RSSI, DHCP, or SSID without explanation to a non-technical customer. Agent confirms that the customer understands without actually verifying it through a question or response. Instructions require the customer to ask for clarification on every other step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1" s="187">
+      <c r="B27" s="342" t="inlineStr">
+        <is>
+          <t>Actively listened and showed comprehension throughout the interaction/s</t>
+        </is>
+      </c>
+      <c r="C27" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D27" s="344" t="inlineStr">
+        <is>
+          <t>Active listening is the difference between an agent who genuinely understands the customer's situation and one who is executing a script regardless of what they are hearing. Agents who listen actively ask relevant follow-up questions, avoid asking for information the customer has already given, and build on what they have learned. In multi-touch cases, active listening extends to reviewing prior case notes and picking up the thread rather than requiring the customer to start over.</t>
+        </is>
+      </c>
+      <c r="E27" s="345" t="inlineStr">
+        <is>
+          <t>Agent asks the customer to repeat information already documented in the ticket. Agent misses a key detail the customer mentioned earlier in the call. Agent's follow-up questions are unrelated to what the customer just said. Customer says I already told the last agent this or didn't you read the notes?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1" s="187">
+      <c r="B28" s="338" t="inlineStr">
+        <is>
+          <t>Managed time well, with clear transitions between steps</t>
+        </is>
+      </c>
+      <c r="C28" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D28" s="340" t="inlineStr">
+        <is>
+          <t>Calls that lack clear transitions feel disorganized and undermine customer confidence. Customers do not know whether they should be doing something, waiting for something, or whether the agent has lost their place in the process. Clear transitions — I've confirmed X, now I'm going to check Y, while I do that could you... — keep the customer oriented and the interaction moving with a sense of purpose. Under the Support Organization Reset, clear transitions are the behavioral signal of purposeful troubleshooting versus unnecessary call stretching.</t>
+        </is>
+      </c>
+      <c r="E28" s="341" t="inlineStr">
+        <is>
+          <t>Long periods of silence with no explanation. Customer asks are you still there or what should I be doing now. Agent moves between steps without acknowledging the result of the previous step. The call feels stalled or disorganized even though time is being spent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1" s="187">
+      <c r="B29" s="342" t="inlineStr">
+        <is>
+          <t>Handled difficult moments when needed to maintain call control</t>
+        </is>
+      </c>
+      <c r="C29" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D29" s="344" t="inlineStr">
+        <is>
+          <t>Some customers arrive frustrated, exhausted from prior contacts, or emotionally escalated before the agent has said a word. The previous operating model created many of those customers through deflection and premature closure. An agent who loses control of the call in response to customer emotion cannot complete the troubleshooting process and often makes the situation worse. Handling difficult moments means acknowledging the frustration appropriately, then redirecting the conversation toward a productive path.</t>
+        </is>
+      </c>
+      <c r="E29" s="345" t="inlineStr">
+        <is>
+          <t>Agent responds to customer frustration with defensiveness or disengagement. Agent abandons the troubleshooting process because the customer is difficult. Agent's tone becomes impatient or dismissive in response to repeated questions. Agent matches the customer's emotional escalation instead of de-escalating it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1" s="187">
+      <c r="B30" s="338" t="inlineStr">
+        <is>
+          <t>Adjusted communication for the customer's accessibility needs (hearing, vision, language barrier, age, cognitive)</t>
+        </is>
+      </c>
+      <c r="C30" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D30" s="340" t="inlineStr">
+        <is>
+          <t>Not all customers receive support communication the same way. Older customers, customers with hearing difficulties, customers whose first language is not English, and customers with cognitive challenges require deliberate adjustments: slower pace, simpler language, one instruction at a time, confirmation of each step before moving to the next, and written follow-up. Ignoring these needs produces failed troubleshooting steps, customer distress, and interactions that are technically complete but humanly inadequate.</t>
+        </is>
+      </c>
+      <c r="E30" s="341" t="inlineStr">
+        <is>
+          <t>Agent maintains standard pace and vocabulary with a customer who has a documented hearing difficulty. Agent delivers multiple instructions at once to a customer who is clearly struggling to keep up. Agent does not offer written follow-up for a customer who cannot fully process verbal instructions. Session runs for an extended period with a vulnerable customer without offering a pause or a wellbeing check-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="8" customHeight="1" s="187">
+      <c r="B31" s="63" t="n"/>
+      <c r="C31" s="63" t="n"/>
+      <c r="D31" s="63" t="n"/>
+      <c r="E31" s="63" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" s="187">
+      <c r="B32" s="336" t="inlineStr">
+        <is>
+          <t>4. CUSTOMER OWNERSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1" s="187">
+      <c r="B33" s="337" t="inlineStr">
+        <is>
+          <t>Measures whether the agent took genuine responsibility for the customer's outcome — not just for their own portion of the interaction, but for the continuity of the case across touches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1" s="187">
+      <c r="B34" s="338" t="inlineStr">
+        <is>
+          <t>Took accountability for the customer's outcome and avoided unnecessary transfers</t>
+        </is>
+      </c>
+      <c r="C34" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D34" s="340" t="inlineStr">
+        <is>
+          <t>Ownership means the agent is responsible for what happens to the customer, not just for their own segment of the call. An agent who deflects to other teams without attempting to help, who transfers unnecessarily to avoid a difficult situation, or who stops effort the moment a complication arises is not owning the interaction. The customer experiences the outcome, not the internal handoffs. Under the Support Organization Reset, ownership is not optional — it is the core behavior the entire quality model is designed to incentivize.</t>
+        </is>
+      </c>
+      <c r="E34" s="341" t="inlineStr">
+        <is>
+          <t>Agent transfers the call after one troubleshooting attempt because the product is out of warranty. Agent passes the case to escalation without completing available Level 1 steps. Agent tells the customer to call back later rather than resolving something within their capability. Agent's response to a difficult case is to find someone else to handle it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1" s="187">
+      <c r="B35" s="342" t="inlineStr">
+        <is>
+          <t>Followed through on all commitments made during the interaction</t>
+        </is>
+      </c>
+      <c r="C35" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D35" s="344" t="inlineStr">
+        <is>
+          <t>Every commitment an agent makes during an interaction — a callback at a specific time, instructions to be sent by email, a follow-up action to be taken — is a promise to the customer. Broken promises compound the original support failure with a trust failure. When a customer has already invested significant time in a support interaction, a missed commitment tells them their time was wasted and the agent's word cannot be relied upon. Following through is not a courtesy, it is a basic accountability expectation.</t>
+        </is>
+      </c>
+      <c r="E35" s="345" t="inlineStr">
+        <is>
+          <t>Agent agrees to call back at 4 PM and calls at 6 PM without prior notice. Agent promises to send troubleshooting steps and does not send them. Agent says I'll follow up if the issue recurs but documents nothing and never follows up. Customer contacts support again because the promised action was not completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="90" customHeight="1" s="187">
+      <c r="B36" s="338" t="inlineStr">
+        <is>
+          <t>Clearly set customer expectations for next steps and realistic timelines</t>
+        </is>
+      </c>
+      <c r="C36" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D36" s="340" t="inlineStr">
+        <is>
+          <t>Customers who do not know what happens next — who is responsible for the next action, when to expect it, and what it will consist of — are left in uncertainty that drives repeat contacts and erodes confidence. Clear next steps and realistic timelines give the customer a framework for the continuation of their case. Unrealistic timelines are as harmful as vague ones: telling a customer their issue will be resolved in one hour when it requires three days sets the agent up for an ownership failure before the call is over.</t>
+        </is>
+      </c>
+      <c r="E36" s="341" t="inlineStr">
+        <is>
+          <t>Call ends with we'll look into it and no specific action or timeline. Agent gives an optimistic timeline the support process cannot realistically meet. Agent lists a next step the customer cannot execute without additional information not yet provided. Customer calls back the same day asking what they are supposed to do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="90" customHeight="1" s="187">
+      <c r="B37" s="342" t="inlineStr">
+        <is>
+          <t>Completed required disconnect follow-up and met callback commitments within the agreed window</t>
+        </is>
+      </c>
+      <c r="C37" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D37" s="344" t="inlineStr">
+        <is>
+          <t>Disconnected calls and missed callbacks are among the highest-frustration experiences in the support journey. The customer has invested time in getting help; a disconnect without follow-up tells them their case has been abandoned. Required follow-up is not optional — it is the minimum expected response when a call ends without the customer's consent or without a completed resolution. Callback commitments carry the same weight: if an agent agrees to a specific window, that window is a commitment to the customer.</t>
+        </is>
+      </c>
+      <c r="E37" s="345" t="inlineStr">
+        <is>
+          <t>Call disconnects and agent takes no documented follow-up action. Agent calls back outside the agreed window without prior notification to the customer. Agent documents a callback attempt without confirming the customer was actually reached. Customer calls in after a disconnect and has to explain the full case again because no notes were left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90" customHeight="1" s="187">
+      <c r="B38" s="338" t="inlineStr">
+        <is>
+          <t>Recognized and acknowledged prior contact history; did not treat a repeat contact as a new case without reviewing previous interactions — mark N.A. if this is a confirmed first contact</t>
+        </is>
+      </c>
+      <c r="C38" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D38" s="340" t="inlineStr">
+        <is>
+          <t>Customers who have to re-explain their entire situation on every contact experience the support organization as incompetent and indifferent. Reviewing and referencing prior contact history is a basic continuity act: it signals to the customer that their case is being managed, not just processed. It also prevents agents from repeating troubleshooting steps the customer has already completed, which wastes time and goodwill. In multi-touch case scoring, this indicator captures each agent's individual contribution to the chain's continuity.</t>
+        </is>
+      </c>
+      <c r="E38" s="341" t="inlineStr">
+        <is>
+          <t>Agent asks the customer to describe their issue from the beginning without referencing the ticket history. Agent performs troubleshooting steps already documented in prior notes. Customer says I just told the last agent this. Agent does not acknowledge how many contacts the customer has already made on this issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="90" customHeight="1" s="187">
+      <c r="B39" s="342" t="inlineStr">
+        <is>
+          <t>If the case was handed off or escalated, the receiving agent was given sufficient context to continue without requiring the customer to repeat themselves — mark N.A. if no handoff occurred on this touch</t>
+        </is>
+      </c>
+      <c r="C39" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D39" s="344" t="inlineStr">
+        <is>
+          <t>A handoff without sufficient context restarts the customer's experience from zero. The receiving agent must re-gather all the information the handing-off agent already had, consuming time and damaging trust. A high-quality handoff — with symptoms, findings, steps taken, current status, and specific next-action guidance — protects the customer from repetition and respects the receiving agent's time. In the team scoring model, handoff quality is one of the two evaluator-judged components that can raise or lower the team score independently of individual agent execution.</t>
+        </is>
+      </c>
+      <c r="E39" s="345" t="inlineStr">
+        <is>
+          <t>Escalation notes say customer still has issue or needs Level 2 help without specifics. Receiving agent asks the customer to re-explain the problem from the beginning. Handoff does not include what was tested, what was found, and what specifically is needed from the next agent. Customer has to repeat their entire history on the escalation call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="8" customHeight="1" s="187">
+      <c r="B40" s="63" t="n"/>
+      <c r="C40" s="63" t="n"/>
+      <c r="D40" s="63" t="n"/>
+      <c r="E40" s="63" t="n"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" s="187">
+      <c r="B41" s="336" t="inlineStr">
+        <is>
+          <t>5. ESCALATION JUDGMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1" s="187">
+      <c r="B42" s="337" t="inlineStr">
+        <is>
+          <t>Measures whether escalation decisions — including the decision not to escalate — were appropriate. Both premature escalation and failure to escalate a warranted case are scored failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90" customHeight="1" s="187">
+      <c r="B43" s="338" t="inlineStr">
+        <is>
+          <t>Completed reasonable troubleshooting before escalating</t>
+        </is>
+      </c>
+      <c r="C43" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D43" s="340" t="inlineStr">
+        <is>
+          <t>Escalation without troubleshooting is queue shuffling, not support. Escalation teams are a limited resource; filling them with cases that Level 1 agents could have resolved reduces their capacity for genuinely complex cases. This indicator holds Level 1 agents accountable for doing the diagnostic work available to them before requesting additional help. Under the Support Organization Reset, escalation is repositioned as support for Level 1, not as a mechanism to move difficult calls out of the queue.</t>
+        </is>
+      </c>
+      <c r="E43" s="341" t="inlineStr">
+        <is>
+          <t>Agent escalates after one troubleshooting step. Agent escalates because the product is out of warranty before attempting any investigation. Agent escalates because the customer is frustrated, not because Level 1 options have been exhausted. Escalation notes show minimal investigation with a large number of unresolved diagnostic questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="90" customHeight="1" s="187">
+      <c r="B44" s="342" t="inlineStr">
+        <is>
+          <t>Escalation was triggered by a recognized condition: unresolved after reasonable L1 troubleshooting, customer complaint or management request, ISP/partner-supported product still unresolved, or agent stuck after documented effort — not used solely to transfer a difficult call or avoid ownership</t>
+        </is>
+      </c>
+      <c r="C44" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D44" s="344" t="inlineStr">
+        <is>
+          <t>Escalation must be driven by a legitimate trigger, not by inconvenience. The Support Organization Reset expanded the recognized escalation triggers to include complaint and management-contact requests and legal-risk signals, not just technical complexity. Failing to recognize those triggers — particularly a customer's explicit request to speak with management or a reference to legal action — is a scored failure. Escalating without a legitimate trigger, to avoid ownership, is equally a failure.</t>
+        </is>
+      </c>
+      <c r="E44" s="345" t="inlineStr">
+        <is>
+          <t>Agent escalates without recognizing that a customer's management-contact request constitutes a valid escalation trigger. Agent escalates because the call is difficult, not because Level 1 options are exhausted. Agent fails to escalate a complaint that includes a legal-risk reference. Escalation notes do not explain what the recognized trigger was.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="90" customHeight="1" s="187">
+      <c r="B45" s="338" t="inlineStr">
+        <is>
+          <t>Provided complete escalation details using the correct escalation path</t>
+        </is>
+      </c>
+      <c r="C45" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D45" s="340" t="inlineStr">
+        <is>
+          <t>An escalation is only as useful as the documentation it carries. An escalation with vague or missing notes forces the receiving agent to start over, fails the customer, and wastes escalation capacity. Complete escalation details — issue and symptoms, product and warranty status, steps taken, findings from each step, reason for escalation, and what specifically is needed — allow the next person to act immediately rather than re-gathering everything from scratch. This indicator scores whether the escalation was a useful handoff or an empty transfer.</t>
+        </is>
+      </c>
+      <c r="E45" s="341" t="inlineStr">
+        <is>
+          <t>Escalation notes contain only: customer has no internet, please assist. No steps taken or findings are documented. No clear statement of what specific help is needed from the escalation team. Wrong escalation path used, causing the case to land with the wrong team or the wrong person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="90" customHeight="1" s="187">
+      <c r="B46" s="342" t="inlineStr">
+        <is>
+          <t>Clearly explained why escalation was necessary and what would happen next</t>
+        </is>
+      </c>
+      <c r="C46" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D46" s="344" t="inlineStr">
+        <is>
+          <t>Customers who are escalated without explanation often feel abandoned or passed off. A clear statement — what is happening, why the case is being escalated, who will handle it, and when the customer can expect contact — maintains confidence and sets accurate expectations for the next interaction. This is also the first link in the escalation team's communication chain: if the initiating agent fails to set expectations, the receiving agent must recover from a trust gap before they can begin helping.</t>
+        </is>
+      </c>
+      <c r="E46" s="345" t="inlineStr">
+        <is>
+          <t>Customer is transferred without being told who they are being transferred to or why. Agent says someone will call you back without specifying a timeframe. Customer does not understand that they are being escalated versus being sent to a different department. Customer calls back immediately after the escalation because they had no expectation of what would happen next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="8" customHeight="1" s="187">
+      <c r="B47" s="63" t="n"/>
+      <c r="C47" s="63" t="n"/>
+      <c r="D47" s="63" t="n"/>
+      <c r="E47" s="63" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1" s="187">
+      <c r="B48" s="336" t="inlineStr">
+        <is>
+          <t>6. CUSTOMER EXPERIENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1" s="187">
+      <c r="B49" s="337" t="inlineStr">
+        <is>
+          <t>Measures the human quality of the interaction. Customer experience is largely a downstream outcome of the four categories above — but professionalism, empathy, and effort-reduction matter independently, especially for vulnerable or long-suffering customers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="90" customHeight="1" s="187">
+      <c r="B50" s="338" t="inlineStr">
+        <is>
+          <t>Demonstrated empathy including for repeat-contact fatigue</t>
+        </is>
+      </c>
+      <c r="C50" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D50" s="340" t="inlineStr">
+        <is>
+          <t>Customers who feel unheard or dismissed disengage faster, escalate emotionally, and are less cooperative with troubleshooting steps. Empathy — particularly explicit acknowledgment of how much time and effort a customer has already invested — signals that the agent sees the customer as a person, not a ticket number. Repeat contacts carry a specific emotional weight: the customer has already tried to get help and failed. Acknowledging that history is the human equivalent of reading the case notes — it demonstrates that the agent understands the full context of the customer's experience.</t>
+        </is>
+      </c>
+      <c r="E50" s="341" t="inlineStr">
+        <is>
+          <t>Agent does not acknowledge that the customer has been dealing with this issue for three weeks. Agent's opening tone is transactional and impersonal after a customer explains a frustrating history. Agent apologizes mechanically without demonstrating recognition of the customer's situation. Customer feels they are starting over again despite extensive prior contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="90" customHeight="1" s="187">
+      <c r="B51" s="342" t="inlineStr">
+        <is>
+          <t>Stayed professional throughout and maintained patience, even under pressure</t>
+        </is>
+      </c>
+      <c r="C51" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D51" s="344" t="inlineStr">
+        <is>
+          <t>Professionalism is the floor of every support interaction, not the ceiling. An agent who responds to customer frustration with impatience, dismissiveness, or disengagement makes the situation measurably worse — the customer has now experienced both the original problem and poor treatment on top of it. Maintaining professionalism under pressure is what separates a support agent from a transactional responder: it requires active effort to remain composed when a customer is venting, when a problem is difficult, or when the interaction is going badly.</t>
+        </is>
+      </c>
+      <c r="E51" s="345" t="inlineStr">
+        <is>
+          <t>Agent's tone becomes curt or cold when the customer expresses frustration. Agent makes dismissive or sarcastic remarks about the customer's situation. Agent rushes through the interaction because they are impatient with the customer's pace. Agent's professionalism declines noticeably as the call extends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="90" customHeight="1" s="187">
+      <c r="B52" s="338" t="inlineStr">
+        <is>
+          <t>Agent matched the customer's tone, pace, level, and energy</t>
+        </is>
+      </c>
+      <c r="C52" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D52" s="340" t="inlineStr">
+        <is>
+          <t>Customers interact at different speeds, with different vocabularies, and at different emotional states. An agent who maintains a fixed communication register regardless of the customer creates a mismatch: too technical for a confused consumer, too slow for an impatient B2B contact, too formal for a casual interaction. Matching the customer's pace and level is a baseline adaptability skill. As Linksys moves toward more technically sophisticated B2B and ISP-facing customers, agents must be able to range across different communication registers credibly.</t>
+        </is>
+      </c>
+      <c r="E52" s="341" t="inlineStr">
+        <is>
+          <t>Agent speaks to a non-technical customer using network engineering vocabulary without adjustment. Agent is noticeably over-explanatory with a customer who clearly has technical sophistication. Agent's energy level does not acknowledge that the customer is distressed or experiencing urgency. Mismatch between agent and customer communication style is visible throughout the interaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="90" customHeight="1" s="187">
+      <c r="B53" s="342" t="inlineStr">
+        <is>
+          <t>Minimized customer effort</t>
+        </is>
+      </c>
+      <c r="C53" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D53" s="344" t="inlineStr">
+        <is>
+          <t>Customer effort is one of the strongest predictors of customer satisfaction and loyalty. Every additional contact, every repeated explanation, every unnecessary hold, every missed callback, and every vague next step increases the customer's effort and decreases their confidence in the support organization. Minimizing effort is the aggregate test of whether the agent avoided the behaviors the Support Organization Reset explicitly names as failures: KB deflection, ISP blame without investigation, premature closure, and missed follow-up.</t>
+        </is>
+      </c>
+      <c r="E53" s="345" t="inlineStr">
+        <is>
+          <t>Customer must contact support multiple times for the same unresolved issue. Customer has to explain the same history repeatedly across different agents. Customer is left to initiate the next step without guidance on what it should be. Customer experience survey describes the interaction as difficult, effortful, or exhausting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="90" customHeight="1" s="187">
+      <c r="B54" s="338" t="inlineStr">
+        <is>
+          <t>Maintained customer understanding and engagement</t>
+        </is>
+      </c>
+      <c r="C54" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D54" s="340" t="inlineStr">
+        <is>
+          <t>A customer who has lost the thread of the troubleshooting process cannot follow instructions correctly, cannot report results accurately, and cannot make informed decisions about next steps. Checking for understanding at key moments — particularly before the customer attempts a step that depends on their comprehension — catches confusion before it compounds. Customer engagement is the live signal that the interaction is working: a disengaged customer is either confused, frustrated, or has mentally disconnected from the process.</t>
+        </is>
+      </c>
+      <c r="E54" s="341" t="inlineStr">
+        <is>
+          <t>Customer performs the wrong step because they did not understand what was asked. Customer gives inconsistent status reports because they are confused about what they are observing. Customer stops responding or becomes passive mid-troubleshooting. CSAT feedback describes the experience as confusing despite the agent completing all technical steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="8" customHeight="1" s="187">
+      <c r="B55" s="63" t="n"/>
+      <c r="C55" s="63" t="n"/>
+      <c r="D55" s="63" t="n"/>
+      <c r="E55" s="63" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1" s="187">
+      <c r="B56" s="336" t="inlineStr">
+        <is>
+          <t>7. DOCUMENTATION &amp; NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1" s="187">
+      <c r="B57" s="337" t="inlineStr">
+        <is>
+          <t>Measures whether the case record is complete enough for any other agent or QA analyst to understand what happened, what was found, and what should happen next. Documentation supports continuity, not compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="90" customHeight="1" s="187">
+      <c r="B58" s="338" t="inlineStr">
+        <is>
+          <t>Recorded customer issue summary</t>
+        </is>
+      </c>
+      <c r="C58" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D58" s="340" t="inlineStr">
+        <is>
+          <t>The customer issue summary is the starting point for every subsequent agent, escalation team member, or reviewer who touches the case. Without it, the next person does not know what the customer called about, what they were trying to accomplish, or what the fundamental problem is. A missing or generic summary forces the customer to repeat themselves and wastes the receiving agent's time on re-gathering basic context that should have been captured the first time.</t>
+        </is>
+      </c>
+      <c r="E58" s="341" t="inlineStr">
+        <is>
+          <t>Ticket notes contain only: customer called about internet issue with no description of the symptom, configuration, or environment. Next agent asks the customer to explain the issue from the beginning because the summary is inadequate. Summary is so generic it applies to any call rather than the specific case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="90" customHeight="1" s="187">
+      <c r="B59" s="342" t="inlineStr">
+        <is>
+          <t>Documented troubleshooting steps</t>
+        </is>
+      </c>
+      <c r="C59" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D59" s="344" t="inlineStr">
+        <is>
+          <t>Troubleshooting documentation tells the next agent what has already been tried so they do not repeat steps the customer has already completed. It is also the evidence trail for conclusions: if an agent determines the problem is a hardware failure, the troubleshooting notes should show what was tested to support that determination. Without documentation, even strong technical work produces no organizational value beyond the single interaction — it cannot be reviewed, credited, built upon, or learned from.</t>
+        </is>
+      </c>
+      <c r="E59" s="345" t="inlineStr">
+        <is>
+          <t>Agent performs a remote session and runs multiple diagnostics, but the ticket notes only say performed troubleshooting, issue unresolved. Agent changes a setting during the call but does not note what was changed or why. Next escalation agent repeats steps already completed because they have no record of what was done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="90" customHeight="1" s="187">
+      <c r="B60" s="338" t="inlineStr">
+        <is>
+          <t>Noted key findings</t>
+        </is>
+      </c>
+      <c r="C60" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D60" s="340" t="inlineStr">
+        <is>
+          <t>Key findings — a specific RSSI value, a firmware version, a confirmed port failure, an identified overlap node, a discovered configuration conflict — are the most operationally useful part of any case note. Findings allow the next agent to take immediate, targeted action rather than starting the diagnostic process over. They are also the raw material for KB content improvement, product quality feedback, and training development. A case without documented findings is a missed opportunity to improve the support organization beyond the individual interaction.</t>
+        </is>
+      </c>
+      <c r="E60" s="341" t="inlineStr">
+        <is>
+          <t>Agent discovers that two nodes have RSSI of -90 dBm but does not note the values. Agent identifies a likely root cause during the call but only documents possible hardware issue without supporting evidence. Escalation team member cannot determine what specifically was found because findings are described in general terms only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="90" customHeight="1" s="187">
+      <c r="B61" s="342" t="inlineStr">
+        <is>
+          <t>Captured agent reasoning — escalation justification, offline recommendations provided by colleagues and other support POCs, especially if no private notes are applicable to the step or action</t>
+        </is>
+      </c>
+      <c r="C61" s="339" t="inlineStr">
+        <is>
+          <t>Wt 3  —  Primary</t>
+        </is>
+      </c>
+      <c r="D61" s="344" t="inlineStr">
+        <is>
+          <t>Agent reasoning is the most frequently missing and most frequently needed element of case documentation. When an agent consults a supervisor, receives advice from a colleague, or makes a judgment call — particularly about closure, escalation, or a non-standard resolution path — that context disappears from the record if it is not noted. The next agent or reviewer sees only the decision, not the reasoning behind it. A case closed RESOLVED with no note explaining why is one of the most common documentation failures in multi-touch journeys.</t>
+        </is>
+      </c>
+      <c r="E61" s="345" t="inlineStr">
+        <is>
+          <t>Case is marked RESOLVED but no note explains what confirmed the resolution or why the agent believed the issue was fixed. Agent consulted a team lead before escalating but did not note what guidance was received. Agent took an unusual action or a non-standard configuration but left no explanation of why. Reviewer cannot reconstruct the agent's decision-making from the notes alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="90" customHeight="1" s="187">
+      <c r="B62" s="338" t="inlineStr">
+        <is>
+          <t>Documented next steps and follow-ups</t>
+        </is>
+      </c>
+      <c r="C62" s="343" t="inlineStr">
+        <is>
+          <t>Wt 2  —  Core</t>
+        </is>
+      </c>
+      <c r="D62" s="340" t="inlineStr">
+        <is>
+          <t>Next step documentation is the bridge between the current interaction and the next one. Agents who document what they promised, what the customer agreed to do, and what remains outstanding are creating an accountability record that protects the customer from continuity failures. An undocumented next step is a promise that no one will remember to keep — and in a multi-touch case, a missed next step from one agent becomes the source of confusion for every subsequent agent.</t>
+        </is>
+      </c>
+      <c r="E62" s="341" t="inlineStr">
+        <is>
+          <t>Call ends with an agreed callback but no note is made of the date, time window, or customer contact preference. Agent promises to send instructions but does not document this or confirm it was sent. Escalation team member has no record of what the previous agent promised the customer, leading to a conflicting expectation on the next contact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="90" customHeight="1" s="187">
+      <c r="B63" s="342" t="inlineStr">
+        <is>
+          <t>Updated ticket status accurately</t>
+        </is>
+      </c>
+      <c r="C63" s="346" t="inlineStr">
+        <is>
+          <t>Wt 1  —  Supporting</t>
+        </is>
+      </c>
+      <c r="D63" s="344" t="inlineStr">
+        <is>
+          <t>Ticket status is the operational signal that tells the support organization what state a case is in. An incorrectly closed case looks resolved when it is not; an incorrectly open case may generate unnecessary follow-up or distort queue reporting. Premature closure — marking a case RESOLVED when the issue is known to be unresolved — is among the most harmful documentation failures because it actively misleads every person who subsequently looks at the case and erases the customer's history of trying to get help.</t>
+        </is>
+      </c>
+      <c r="E63" s="345" t="inlineStr">
+        <is>
+          <t>Agent marks a case RESOLVED after internet is temporarily restored but the primary complaint is still unconfirmed. Agent closes a case RESOLVED because the customer agreed to test the proposed solution before that solution has been confirmed to work. Ticket status does not reflect a pending callback, a known-outstanding action, or a disconnect that occurred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="8" customHeight="1" s="187">
+      <c r="B64" s="63" t="n"/>
+      <c r="C64" s="63" t="n"/>
+      <c r="D64" s="63" t="n"/>
+      <c r="E64" s="63" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B32:E32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -11294,7 +14153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11770,7 +14629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12046,7 +14905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12920,7 +15779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15527,1699 +18386,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" style="187" min="1" max="1"/>
-    <col width="13" customWidth="1" style="187" min="2" max="2"/>
-    <col width="18" customWidth="1" style="187" min="3" max="3"/>
-    <col width="8" customWidth="1" style="187" min="4" max="11"/>
-    <col width="10" customWidth="1" style="187" min="12" max="12"/>
-    <col width="13" customWidth="1" style="187" min="13" max="13"/>
-    <col width="60" customWidth="1" style="187" min="14" max="14"/>
-    <col width="22" customWidth="1" style="187" min="15" max="15"/>
-    <col width="14" customWidth="1" style="187" min="16" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26.1" customHeight="1" s="187">
-      <c r="A1" s="219" t="inlineStr">
-        <is>
-          <t>CASE TRACKER — Multi-Case &amp; Multi-Touch Log</t>
-        </is>
-      </c>
-      <c r="B1" s="212" t="n"/>
-      <c r="C1" s="212" t="n"/>
-      <c r="D1" s="212" t="n"/>
-      <c r="E1" s="212" t="n"/>
-      <c r="F1" s="212" t="n"/>
-      <c r="G1" s="212" t="n"/>
-      <c r="H1" s="212" t="n"/>
-      <c r="I1" s="212" t="n"/>
-      <c r="J1" s="212" t="n"/>
-      <c r="K1" s="212" t="n"/>
-      <c r="L1" s="212" t="n"/>
-      <c r="M1" s="212" t="n"/>
-      <c r="N1" s="212" t="n"/>
-      <c r="O1" s="212" t="n"/>
-      <c r="P1" s="192" t="n"/>
-    </row>
-    <row r="2" ht="15.95" customHeight="1" s="187">
-      <c r="A2" s="282" t="inlineStr">
-        <is>
-          <t>One row per touch. Reuse a Case ID across rows to track a multi-touch journey. Scores 0-5; Weighted % and Result calculate automatically. Pre-loaded: the TE00124020 / TE00127492 journey (see Multi-Touch Guide).</t>
-        </is>
-      </c>
-      <c r="B2" s="212" t="n"/>
-      <c r="C2" s="212" t="n"/>
-      <c r="D2" s="212" t="n"/>
-      <c r="E2" s="212" t="n"/>
-      <c r="F2" s="212" t="n"/>
-      <c r="G2" s="212" t="n"/>
-      <c r="H2" s="212" t="n"/>
-      <c r="I2" s="212" t="n"/>
-      <c r="J2" s="212" t="n"/>
-      <c r="K2" s="212" t="n"/>
-      <c r="L2" s="212" t="n"/>
-      <c r="M2" s="212" t="n"/>
-      <c r="N2" s="212" t="n"/>
-      <c r="O2" s="212" t="n"/>
-      <c r="P2" s="192" t="n"/>
-    </row>
-    <row r="3" ht="24" customHeight="1" s="187">
-      <c r="A3" s="275">
-        <f>IF(A56="","  JOURNEY TEAM SCORE  ▸  log touches below, then enter a Case ID + Outcome/Continuity in row 56","  LOADED JOURNEY TEAM SCORE  ▸  "&amp;A56&amp;":  "&amp;TEXT(G56,"0.0%")&amp;"   "&amp;UPPER(H56))</f>
-        <v/>
-      </c>
-      <c r="B3" s="212" t="n"/>
-      <c r="C3" s="212" t="n"/>
-      <c r="D3" s="212" t="n"/>
-      <c r="E3" s="212" t="n"/>
-      <c r="F3" s="212" t="n"/>
-      <c r="G3" s="212" t="n"/>
-      <c r="H3" s="212" t="n"/>
-      <c r="I3" s="212" t="n"/>
-      <c r="J3" s="212" t="n"/>
-      <c r="K3" s="212" t="n"/>
-      <c r="L3" s="212" t="n"/>
-      <c r="M3" s="212" t="n"/>
-      <c r="N3" s="212" t="n"/>
-      <c r="O3" s="212" t="n"/>
-      <c r="P3" s="192" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="187">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>Case ID</t>
-        </is>
-      </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>Agent</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>Touch #</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>Res 30%</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>Tech 20%</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
-        <is>
-          <t>Comm 15%</t>
-        </is>
-      </c>
-      <c r="H4" s="23" t="inlineStr">
-        <is>
-          <t>Own 15%</t>
-        </is>
-      </c>
-      <c r="I4" s="23" t="inlineStr">
-        <is>
-          <t>Esc 10%</t>
-        </is>
-      </c>
-      <c r="J4" s="23" t="inlineStr">
-        <is>
-          <t>CX 5%</t>
-        </is>
-      </c>
-      <c r="K4" s="23" t="inlineStr">
-        <is>
-          <t>Doc 5%</t>
-        </is>
-      </c>
-      <c r="L4" s="23" t="inlineStr">
-        <is>
-          <t>Weighted</t>
-        </is>
-      </c>
-      <c r="M4" s="23" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="N4" s="23" t="inlineStr">
-        <is>
-          <t>Outcome / Notes</t>
-        </is>
-      </c>
-      <c r="O4" s="46" t="inlineStr">
-        <is>
-          <t>Contribution Type</t>
-        </is>
-      </c>
-      <c r="P4" s="46" t="inlineStr">
-        <is>
-          <t>Handoff Quality (0-5)</t>
-        </is>
-      </c>
-      <c r="Q4" s="95" t="inlineStr">
-        <is>
-          <t>Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="39.95" customHeight="1" s="187">
-      <c r="A5" s="24" t="n"/>
-      <c r="B5" s="24" t="n"/>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="H5" s="24" t="n"/>
-      <c r="I5" s="24" t="n"/>
-      <c r="J5" s="24" t="n"/>
-      <c r="K5" s="24" t="n"/>
-      <c r="L5" s="325">
-        <f>IF((COUNT(E5)+COUNT(F5)+COUNT(G5)+COUNT(H5)+COUNT(I5)+COUNT(J5)+COUNT(K5))=0,"",IFERROR(E5/5*0.3,0)+IFERROR(F5/5*0.2,0)+IFERROR(G5/5*0.15,0)+IFERROR(H5/5*0.15,0)+IFERROR(I5/5*0.1,0)+IFERROR(J5/5*0.05,0)+IFERROR(K5/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M5" s="11">
-        <f>IF(L5="","",IF(L5&gt;=0.85,"Meets/Exceeds",IF(L5&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N5" s="6" t="n"/>
-      <c r="O5" s="11" t="n"/>
-      <c r="P5" s="11" t="n"/>
-      <c r="Q5" s="96" t="n"/>
-    </row>
-    <row r="6" ht="39.95" customHeight="1" s="187">
-      <c r="A6" s="24" t="n"/>
-      <c r="B6" s="24" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
-      <c r="H6" s="24" t="n"/>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="24" t="n"/>
-      <c r="K6" s="24" t="n"/>
-      <c r="L6" s="326">
-        <f>IF((COUNT(E6)+COUNT(F6)+COUNT(G6)+COUNT(H6)+COUNT(I6)+COUNT(J6)+COUNT(K6))=0,"",IFERROR(E6/5*0.3,0)+IFERROR(F6/5*0.2,0)+IFERROR(G6/5*0.15,0)+IFERROR(H6/5*0.15,0)+IFERROR(I6/5*0.1,0)+IFERROR(J6/5*0.05,0)+IFERROR(K6/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M6" s="13">
-        <f>IF(L6="","",IF(L6&gt;=0.85,"Meets/Exceeds",IF(L6&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N6" s="8" t="n"/>
-      <c r="O6" s="13" t="n"/>
-      <c r="P6" s="13" t="n"/>
-      <c r="Q6" s="96" t="n"/>
-    </row>
-    <row r="7" ht="39.95" customHeight="1" s="187">
-      <c r="A7" s="24" t="n"/>
-      <c r="B7" s="24" t="n"/>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
-      <c r="H7" s="24" t="n"/>
-      <c r="I7" s="24" t="n"/>
-      <c r="J7" s="24" t="n"/>
-      <c r="K7" s="24" t="n"/>
-      <c r="L7" s="325">
-        <f>IF((COUNT(E7)+COUNT(F7)+COUNT(G7)+COUNT(H7)+COUNT(I7)+COUNT(J7)+COUNT(K7))=0,"",IFERROR(E7/5*0.3,0)+IFERROR(F7/5*0.2,0)+IFERROR(G7/5*0.15,0)+IFERROR(H7/5*0.15,0)+IFERROR(I7/5*0.1,0)+IFERROR(J7/5*0.05,0)+IFERROR(K7/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M7" s="11">
-        <f>IF(L7="","",IF(L7&gt;=0.85,"Meets/Exceeds",IF(L7&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N7" s="6" t="n"/>
-      <c r="O7" s="11" t="n"/>
-      <c r="P7" s="11" t="n"/>
-      <c r="Q7" s="96" t="n"/>
-    </row>
-    <row r="8" ht="39.95" customHeight="1" s="187">
-      <c r="A8" s="24" t="n"/>
-      <c r="B8" s="24" t="n"/>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n"/>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="24" t="n"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="326">
-        <f>IF((COUNT(E8)+COUNT(F8)+COUNT(G8)+COUNT(H8)+COUNT(I8)+COUNT(J8)+COUNT(K8))=0,"",IFERROR(E8/5*0.3,0)+IFERROR(F8/5*0.2,0)+IFERROR(G8/5*0.15,0)+IFERROR(H8/5*0.15,0)+IFERROR(I8/5*0.1,0)+IFERROR(J8/5*0.05,0)+IFERROR(K8/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M8" s="13">
-        <f>IF(L8="","",IF(L8&gt;=0.85,"Meets/Exceeds",IF(L8&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N8" s="8" t="n"/>
-      <c r="O8" s="13" t="n"/>
-      <c r="P8" s="13" t="n"/>
-      <c r="Q8" s="96" t="n"/>
-    </row>
-    <row r="9" ht="39.95" customHeight="1" s="187">
-      <c r="A9" s="24" t="n"/>
-      <c r="B9" s="24" t="n"/>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="24" t="n"/>
-      <c r="I9" s="24" t="n"/>
-      <c r="J9" s="24" t="n"/>
-      <c r="K9" s="24" t="n"/>
-      <c r="L9" s="325">
-        <f>IF((COUNT(E9)+COUNT(F9)+COUNT(G9)+COUNT(H9)+COUNT(I9)+COUNT(J9)+COUNT(K9))=0,"",IFERROR(E9/5*0.3,0)+IFERROR(F9/5*0.2,0)+IFERROR(G9/5*0.15,0)+IFERROR(H9/5*0.15,0)+IFERROR(I9/5*0.1,0)+IFERROR(J9/5*0.05,0)+IFERROR(K9/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M9" s="11">
-        <f>IF(L9="","",IF(L9&gt;=0.85,"Meets/Exceeds",IF(L9&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="11" t="n"/>
-      <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="96" t="n"/>
-    </row>
-    <row r="10" ht="39.95" customHeight="1" s="187">
-      <c r="A10" s="24" t="n"/>
-      <c r="B10" s="24" t="n"/>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="24" t="n"/>
-      <c r="F10" s="24" t="n"/>
-      <c r="G10" s="24" t="n"/>
-      <c r="H10" s="24" t="n"/>
-      <c r="I10" s="24" t="n"/>
-      <c r="J10" s="24" t="n"/>
-      <c r="K10" s="24" t="n"/>
-      <c r="L10" s="326">
-        <f>IF((COUNT(E10)+COUNT(F10)+COUNT(G10)+COUNT(H10)+COUNT(I10)+COUNT(J10)+COUNT(K10))=0,"",IFERROR(E10/5*0.3,0)+IFERROR(F10/5*0.2,0)+IFERROR(G10/5*0.15,0)+IFERROR(H10/5*0.15,0)+IFERROR(I10/5*0.1,0)+IFERROR(J10/5*0.05,0)+IFERROR(K10/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M10" s="13">
-        <f>IF(L10="","",IF(L10&gt;=0.85,"Meets/Exceeds",IF(L10&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N10" s="8" t="n"/>
-      <c r="O10" s="13" t="n"/>
-      <c r="P10" s="13" t="n"/>
-      <c r="Q10" s="96" t="n"/>
-    </row>
-    <row r="11" ht="39.95" customHeight="1" s="187">
-      <c r="A11" s="24" t="n"/>
-      <c r="B11" s="24" t="n"/>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="24" t="n"/>
-      <c r="F11" s="24" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="24" t="n"/>
-      <c r="I11" s="24" t="n"/>
-      <c r="J11" s="24" t="n"/>
-      <c r="K11" s="24" t="n"/>
-      <c r="L11" s="325">
-        <f>IF((COUNT(E11)+COUNT(F11)+COUNT(G11)+COUNT(H11)+COUNT(I11)+COUNT(J11)+COUNT(K11))=0,"",IFERROR(E11/5*0.3,0)+IFERROR(F11/5*0.2,0)+IFERROR(G11/5*0.15,0)+IFERROR(H11/5*0.15,0)+IFERROR(I11/5*0.1,0)+IFERROR(J11/5*0.05,0)+IFERROR(K11/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M11" s="11">
-        <f>IF(L11="","",IF(L11&gt;=0.85,"Meets/Exceeds",IF(L11&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="11" t="n"/>
-      <c r="P11" s="11" t="n"/>
-      <c r="Q11" s="96" t="n"/>
-    </row>
-    <row r="12" ht="39.95" customHeight="1" s="187">
-      <c r="A12" s="24" t="n"/>
-      <c r="B12" s="24" t="n"/>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="24" t="n"/>
-      <c r="F12" s="24" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="H12" s="24" t="n"/>
-      <c r="I12" s="24" t="n"/>
-      <c r="J12" s="24" t="n"/>
-      <c r="K12" s="24" t="n"/>
-      <c r="L12" s="326">
-        <f>IF((COUNT(E12)+COUNT(F12)+COUNT(G12)+COUNT(H12)+COUNT(I12)+COUNT(J12)+COUNT(K12))=0,"",IFERROR(E12/5*0.3,0)+IFERROR(F12/5*0.2,0)+IFERROR(G12/5*0.15,0)+IFERROR(H12/5*0.15,0)+IFERROR(I12/5*0.1,0)+IFERROR(J12/5*0.05,0)+IFERROR(K12/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M12" s="13">
-        <f>IF(L12="","",IF(L12&gt;=0.85,"Meets/Exceeds",IF(L12&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N12" s="8" t="n"/>
-      <c r="O12" s="13" t="n"/>
-      <c r="P12" s="13" t="n"/>
-      <c r="Q12" s="96" t="n"/>
-    </row>
-    <row r="13" ht="39.95" customHeight="1" s="187">
-      <c r="A13" s="24" t="n"/>
-      <c r="B13" s="24" t="n"/>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="24" t="n"/>
-      <c r="F13" s="24" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
-      <c r="I13" s="24" t="n"/>
-      <c r="J13" s="24" t="n"/>
-      <c r="K13" s="24" t="n"/>
-      <c r="L13" s="325">
-        <f>IF((COUNT(E13)+COUNT(F13)+COUNT(G13)+COUNT(H13)+COUNT(I13)+COUNT(J13)+COUNT(K13))=0,"",IFERROR(E13/5*0.3,0)+IFERROR(F13/5*0.2,0)+IFERROR(G13/5*0.15,0)+IFERROR(H13/5*0.15,0)+IFERROR(I13/5*0.1,0)+IFERROR(J13/5*0.05,0)+IFERROR(K13/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M13" s="11">
-        <f>IF(L13="","",IF(L13&gt;=0.85,"Meets/Exceeds",IF(L13&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="11" t="n"/>
-      <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="96" t="n"/>
-    </row>
-    <row r="14" ht="39.95" customHeight="1" s="187">
-      <c r="A14" s="24" t="n"/>
-      <c r="B14" s="24" t="n"/>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="24" t="n"/>
-      <c r="G14" s="24" t="n"/>
-      <c r="H14" s="24" t="n"/>
-      <c r="I14" s="24" t="n"/>
-      <c r="J14" s="24" t="n"/>
-      <c r="K14" s="24" t="n"/>
-      <c r="L14" s="326">
-        <f>IF((COUNT(E14)+COUNT(F14)+COUNT(G14)+COUNT(H14)+COUNT(I14)+COUNT(J14)+COUNT(K14))=0,"",IFERROR(E14/5*0.3,0)+IFERROR(F14/5*0.2,0)+IFERROR(G14/5*0.15,0)+IFERROR(H14/5*0.15,0)+IFERROR(I14/5*0.1,0)+IFERROR(J14/5*0.05,0)+IFERROR(K14/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M14" s="13">
-        <f>IF(L14="","",IF(L14&gt;=0.85,"Meets/Exceeds",IF(L14&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="13" t="n"/>
-      <c r="P14" s="13" t="n"/>
-      <c r="Q14" s="96" t="n"/>
-    </row>
-    <row r="15" ht="39.95" customHeight="1" s="187">
-      <c r="A15" s="24" t="n"/>
-      <c r="B15" s="24" t="n"/>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="24" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="24" t="n"/>
-      <c r="I15" s="24" t="n"/>
-      <c r="J15" s="24" t="n"/>
-      <c r="K15" s="24" t="n"/>
-      <c r="L15" s="325">
-        <f>IF((COUNT(E15)+COUNT(F15)+COUNT(G15)+COUNT(H15)+COUNT(I15)+COUNT(J15)+COUNT(K15))=0,"",IFERROR(E15/5*0.3,0)+IFERROR(F15/5*0.2,0)+IFERROR(G15/5*0.15,0)+IFERROR(H15/5*0.15,0)+IFERROR(I15/5*0.1,0)+IFERROR(J15/5*0.05,0)+IFERROR(K15/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M15" s="11">
-        <f>IF(L15="","",IF(L15&gt;=0.85,"Meets/Exceeds",IF(L15&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N15" s="6" t="n"/>
-      <c r="O15" s="11" t="n"/>
-      <c r="P15" s="11" t="n"/>
-      <c r="Q15" s="96" t="n"/>
-    </row>
-    <row r="16" ht="39.95" customHeight="1" s="187">
-      <c r="A16" s="24" t="n"/>
-      <c r="B16" s="24" t="n"/>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="H16" s="24" t="n"/>
-      <c r="I16" s="24" t="n"/>
-      <c r="J16" s="24" t="n"/>
-      <c r="K16" s="24" t="n"/>
-      <c r="L16" s="326">
-        <f>IF((COUNT(E16)+COUNT(F16)+COUNT(G16)+COUNT(H16)+COUNT(I16)+COUNT(J16)+COUNT(K16))=0,"",IFERROR(E16/5*0.3,0)+IFERROR(F16/5*0.2,0)+IFERROR(G16/5*0.15,0)+IFERROR(H16/5*0.15,0)+IFERROR(I16/5*0.1,0)+IFERROR(J16/5*0.05,0)+IFERROR(K16/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M16" s="13">
-        <f>IF(L16="","",IF(L16&gt;=0.85,"Meets/Exceeds",IF(L16&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="13" t="n"/>
-      <c r="P16" s="13" t="n"/>
-      <c r="Q16" s="96" t="n"/>
-    </row>
-    <row r="17" ht="39.95" customHeight="1" s="187">
-      <c r="A17" s="24" t="n"/>
-      <c r="B17" s="24" t="n"/>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="24" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="H17" s="24" t="n"/>
-      <c r="I17" s="24" t="n"/>
-      <c r="J17" s="24" t="n"/>
-      <c r="K17" s="24" t="n"/>
-      <c r="L17" s="325">
-        <f>IF((COUNT(E17)+COUNT(F17)+COUNT(G17)+COUNT(H17)+COUNT(I17)+COUNT(J17)+COUNT(K17))=0,"",IFERROR(E17/5*0.3,0)+IFERROR(F17/5*0.2,0)+IFERROR(G17/5*0.15,0)+IFERROR(H17/5*0.15,0)+IFERROR(I17/5*0.1,0)+IFERROR(J17/5*0.05,0)+IFERROR(K17/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M17" s="11">
-        <f>IF(L17="","",IF(L17&gt;=0.85,"Meets/Exceeds",IF(L17&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="96" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="187">
-      <c r="A18" s="24" t="n"/>
-      <c r="B18" s="24" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
-      <c r="I18" s="24" t="n"/>
-      <c r="J18" s="24" t="n"/>
-      <c r="K18" s="24" t="n"/>
-      <c r="L18" s="326">
-        <f>IF((COUNT(E18)+COUNT(F18)+COUNT(G18)+COUNT(H18)+COUNT(I18)+COUNT(J18)+COUNT(K18))=0,"",IFERROR(E18/5*0.3,0)+IFERROR(F18/5*0.2,0)+IFERROR(G18/5*0.15,0)+IFERROR(H18/5*0.15,0)+IFERROR(I18/5*0.1,0)+IFERROR(J18/5*0.05,0)+IFERROR(K18/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M18" s="13">
-        <f>IF(L18="","",IF(L18&gt;=0.85,"Meets/Exceeds",IF(L18&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N18" s="8" t="n"/>
-      <c r="O18" s="13" t="n"/>
-      <c r="P18" s="13" t="n"/>
-      <c r="Q18" s="96" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="187">
-      <c r="A19" s="24" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="24" t="n"/>
-      <c r="K19" s="24" t="n"/>
-      <c r="L19" s="325">
-        <f>IF((COUNT(E19)+COUNT(F19)+COUNT(G19)+COUNT(H19)+COUNT(I19)+COUNT(J19)+COUNT(K19))=0,"",IFERROR(E19/5*0.3,0)+IFERROR(F19/5*0.2,0)+IFERROR(G19/5*0.15,0)+IFERROR(H19/5*0.15,0)+IFERROR(I19/5*0.1,0)+IFERROR(J19/5*0.05,0)+IFERROR(K19/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M19" s="11">
-        <f>IF(L19="","",IF(L19&gt;=0.85,"Meets/Exceeds",IF(L19&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N19" s="6" t="n"/>
-      <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="96" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="187">
-      <c r="A20" s="24" t="n"/>
-      <c r="B20" s="24" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="24" t="n"/>
-      <c r="K20" s="24" t="n"/>
-      <c r="L20" s="326">
-        <f>IF((COUNT(E20)+COUNT(F20)+COUNT(G20)+COUNT(H20)+COUNT(I20)+COUNT(J20)+COUNT(K20))=0,"",IFERROR(E20/5*0.3,0)+IFERROR(F20/5*0.2,0)+IFERROR(G20/5*0.15,0)+IFERROR(H20/5*0.15,0)+IFERROR(I20/5*0.1,0)+IFERROR(J20/5*0.05,0)+IFERROR(K20/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M20" s="13">
-        <f>IF(L20="","",IF(L20&gt;=0.85,"Meets/Exceeds",IF(L20&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N20" s="8" t="n"/>
-      <c r="O20" s="13" t="n"/>
-      <c r="P20" s="13" t="n"/>
-      <c r="Q20" s="96" t="n"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" s="187">
-      <c r="A21" s="24" t="n"/>
-      <c r="B21" s="24" t="n"/>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="H21" s="24" t="n"/>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="24" t="n"/>
-      <c r="K21" s="24" t="n"/>
-      <c r="L21" s="325">
-        <f>IF((COUNT(E21)+COUNT(F21)+COUNT(G21)+COUNT(H21)+COUNT(I21)+COUNT(J21)+COUNT(K21))=0,"",IFERROR(E21/5*0.3,0)+IFERROR(F21/5*0.2,0)+IFERROR(G21/5*0.15,0)+IFERROR(H21/5*0.15,0)+IFERROR(I21/5*0.1,0)+IFERROR(J21/5*0.05,0)+IFERROR(K21/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M21" s="11">
-        <f>IF(L21="","",IF(L21&gt;=0.85,"Meets/Exceeds",IF(L21&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N21" s="6" t="n"/>
-      <c r="O21" s="11" t="n"/>
-      <c r="P21" s="11" t="n"/>
-      <c r="Q21" s="96" t="n"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" s="187">
-      <c r="A22" s="24" t="n"/>
-      <c r="B22" s="24" t="n"/>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="24" t="n"/>
-      <c r="H22" s="24" t="n"/>
-      <c r="I22" s="24" t="n"/>
-      <c r="J22" s="24" t="n"/>
-      <c r="K22" s="24" t="n"/>
-      <c r="L22" s="326">
-        <f>IF((COUNT(E22)+COUNT(F22)+COUNT(G22)+COUNT(H22)+COUNT(I22)+COUNT(J22)+COUNT(K22))=0,"",IFERROR(E22/5*0.3,0)+IFERROR(F22/5*0.2,0)+IFERROR(G22/5*0.15,0)+IFERROR(H22/5*0.15,0)+IFERROR(I22/5*0.1,0)+IFERROR(J22/5*0.05,0)+IFERROR(K22/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M22" s="13">
-        <f>IF(L22="","",IF(L22&gt;=0.85,"Meets/Exceeds",IF(L22&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N22" s="8" t="n"/>
-      <c r="O22" s="13" t="n"/>
-      <c r="P22" s="13" t="n"/>
-      <c r="Q22" s="96" t="n"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" s="187">
-      <c r="A23" s="24" t="n"/>
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="24" t="n"/>
-      <c r="H23" s="24" t="n"/>
-      <c r="I23" s="24" t="n"/>
-      <c r="J23" s="24" t="n"/>
-      <c r="K23" s="24" t="n"/>
-      <c r="L23" s="325">
-        <f>IF((COUNT(E23)+COUNT(F23)+COUNT(G23)+COUNT(H23)+COUNT(I23)+COUNT(J23)+COUNT(K23))=0,"",IFERROR(E23/5*0.3,0)+IFERROR(F23/5*0.2,0)+IFERROR(G23/5*0.15,0)+IFERROR(H23/5*0.15,0)+IFERROR(I23/5*0.1,0)+IFERROR(J23/5*0.05,0)+IFERROR(K23/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M23" s="11">
-        <f>IF(L23="","",IF(L23&gt;=0.85,"Meets/Exceeds",IF(L23&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N23" s="6" t="n"/>
-      <c r="O23" s="11" t="n"/>
-      <c r="P23" s="11" t="n"/>
-      <c r="Q23" s="96" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1" s="187">
-      <c r="A24" s="24" t="n"/>
-      <c r="B24" s="24" t="n"/>
-      <c r="C24" s="24" t="n"/>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="n"/>
-      <c r="F24" s="24" t="n"/>
-      <c r="G24" s="24" t="n"/>
-      <c r="H24" s="24" t="n"/>
-      <c r="I24" s="24" t="n"/>
-      <c r="J24" s="24" t="n"/>
-      <c r="K24" s="24" t="n"/>
-      <c r="L24" s="326">
-        <f>IF((COUNT(E24)+COUNT(F24)+COUNT(G24)+COUNT(H24)+COUNT(I24)+COUNT(J24)+COUNT(K24))=0,"",IFERROR(E24/5*0.3,0)+IFERROR(F24/5*0.2,0)+IFERROR(G24/5*0.15,0)+IFERROR(H24/5*0.15,0)+IFERROR(I24/5*0.1,0)+IFERROR(J24/5*0.05,0)+IFERROR(K24/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M24" s="13">
-        <f>IF(L24="","",IF(L24&gt;=0.85,"Meets/Exceeds",IF(L24&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N24" s="8" t="n"/>
-      <c r="O24" s="13" t="n"/>
-      <c r="P24" s="13" t="n"/>
-      <c r="Q24" s="96" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1" s="187">
-      <c r="A25" s="24" t="n"/>
-      <c r="B25" s="24" t="n"/>
-      <c r="C25" s="24" t="n"/>
-      <c r="D25" s="24" t="n"/>
-      <c r="E25" s="24" t="n"/>
-      <c r="F25" s="24" t="n"/>
-      <c r="G25" s="24" t="n"/>
-      <c r="H25" s="24" t="n"/>
-      <c r="I25" s="24" t="n"/>
-      <c r="J25" s="24" t="n"/>
-      <c r="K25" s="24" t="n"/>
-      <c r="L25" s="325">
-        <f>IF((COUNT(E25)+COUNT(F25)+COUNT(G25)+COUNT(H25)+COUNT(I25)+COUNT(J25)+COUNT(K25))=0,"",IFERROR(E25/5*0.3,0)+IFERROR(F25/5*0.2,0)+IFERROR(G25/5*0.15,0)+IFERROR(H25/5*0.15,0)+IFERROR(I25/5*0.1,0)+IFERROR(J25/5*0.05,0)+IFERROR(K25/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M25" s="11">
-        <f>IF(L25="","",IF(L25&gt;=0.85,"Meets/Exceeds",IF(L25&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="11" t="n"/>
-      <c r="P25" s="11" t="n"/>
-      <c r="Q25" s="96" t="n"/>
-    </row>
-    <row r="26" ht="18" customHeight="1" s="187">
-      <c r="A26" s="24" t="n"/>
-      <c r="B26" s="24" t="n"/>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
-      <c r="H26" s="24" t="n"/>
-      <c r="I26" s="24" t="n"/>
-      <c r="J26" s="24" t="n"/>
-      <c r="K26" s="24" t="n"/>
-      <c r="L26" s="326">
-        <f>IF((COUNT(E26)+COUNT(F26)+COUNT(G26)+COUNT(H26)+COUNT(I26)+COUNT(J26)+COUNT(K26))=0,"",IFERROR(E26/5*0.3,0)+IFERROR(F26/5*0.2,0)+IFERROR(G26/5*0.15,0)+IFERROR(H26/5*0.15,0)+IFERROR(I26/5*0.1,0)+IFERROR(J26/5*0.05,0)+IFERROR(K26/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M26" s="13">
-        <f>IF(L26="","",IF(L26&gt;=0.85,"Meets/Exceeds",IF(L26&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N26" s="8" t="n"/>
-      <c r="O26" s="13" t="n"/>
-      <c r="P26" s="13" t="n"/>
-      <c r="Q26" s="96" t="n"/>
-    </row>
-    <row r="27" ht="18" customHeight="1" s="187">
-      <c r="A27" s="24" t="n"/>
-      <c r="B27" s="24" t="n"/>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="24" t="n"/>
-      <c r="F27" s="24" t="n"/>
-      <c r="G27" s="24" t="n"/>
-      <c r="H27" s="24" t="n"/>
-      <c r="I27" s="24" t="n"/>
-      <c r="J27" s="24" t="n"/>
-      <c r="K27" s="24" t="n"/>
-      <c r="L27" s="325">
-        <f>IF((COUNT(E27)+COUNT(F27)+COUNT(G27)+COUNT(H27)+COUNT(I27)+COUNT(J27)+COUNT(K27))=0,"",IFERROR(E27/5*0.3,0)+IFERROR(F27/5*0.2,0)+IFERROR(G27/5*0.15,0)+IFERROR(H27/5*0.15,0)+IFERROR(I27/5*0.1,0)+IFERROR(J27/5*0.05,0)+IFERROR(K27/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M27" s="11">
-        <f>IF(L27="","",IF(L27&gt;=0.85,"Meets/Exceeds",IF(L27&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="11" t="n"/>
-      <c r="P27" s="11" t="n"/>
-      <c r="Q27" s="96" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1" s="187">
-      <c r="A28" s="24" t="n"/>
-      <c r="B28" s="24" t="n"/>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="H28" s="24" t="n"/>
-      <c r="I28" s="24" t="n"/>
-      <c r="J28" s="24" t="n"/>
-      <c r="K28" s="24" t="n"/>
-      <c r="L28" s="326">
-        <f>IF((COUNT(E28)+COUNT(F28)+COUNT(G28)+COUNT(H28)+COUNT(I28)+COUNT(J28)+COUNT(K28))=0,"",IFERROR(E28/5*0.3,0)+IFERROR(F28/5*0.2,0)+IFERROR(G28/5*0.15,0)+IFERROR(H28/5*0.15,0)+IFERROR(I28/5*0.1,0)+IFERROR(J28/5*0.05,0)+IFERROR(K28/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M28" s="13">
-        <f>IF(L28="","",IF(L28&gt;=0.85,"Meets/Exceeds",IF(L28&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N28" s="8" t="n"/>
-      <c r="O28" s="13" t="n"/>
-      <c r="P28" s="13" t="n"/>
-      <c r="Q28" s="96" t="n"/>
-    </row>
-    <row r="29" ht="18" customHeight="1" s="187">
-      <c r="A29" s="24" t="n"/>
-      <c r="B29" s="24" t="n"/>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="24" t="n"/>
-      <c r="F29" s="24" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="H29" s="24" t="n"/>
-      <c r="I29" s="24" t="n"/>
-      <c r="J29" s="24" t="n"/>
-      <c r="K29" s="24" t="n"/>
-      <c r="L29" s="325">
-        <f>IF((COUNT(E29)+COUNT(F29)+COUNT(G29)+COUNT(H29)+COUNT(I29)+COUNT(J29)+COUNT(K29))=0,"",IFERROR(E29/5*0.3,0)+IFERROR(F29/5*0.2,0)+IFERROR(G29/5*0.15,0)+IFERROR(H29/5*0.15,0)+IFERROR(I29/5*0.1,0)+IFERROR(J29/5*0.05,0)+IFERROR(K29/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M29" s="11">
-        <f>IF(L29="","",IF(L29&gt;=0.85,"Meets/Exceeds",IF(L29&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N29" s="6" t="n"/>
-      <c r="O29" s="11" t="n"/>
-      <c r="P29" s="11" t="n"/>
-      <c r="Q29" s="96" t="n"/>
-    </row>
-    <row r="30" ht="18" customHeight="1" s="187">
-      <c r="A30" s="24" t="n"/>
-      <c r="B30" s="24" t="n"/>
-      <c r="C30" s="24" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="24" t="n"/>
-      <c r="F30" s="24" t="n"/>
-      <c r="G30" s="24" t="n"/>
-      <c r="H30" s="24" t="n"/>
-      <c r="I30" s="24" t="n"/>
-      <c r="J30" s="24" t="n"/>
-      <c r="K30" s="24" t="n"/>
-      <c r="L30" s="326">
-        <f>IF((COUNT(E30)+COUNT(F30)+COUNT(G30)+COUNT(H30)+COUNT(I30)+COUNT(J30)+COUNT(K30))=0,"",IFERROR(E30/5*0.3,0)+IFERROR(F30/5*0.2,0)+IFERROR(G30/5*0.15,0)+IFERROR(H30/5*0.15,0)+IFERROR(I30/5*0.1,0)+IFERROR(J30/5*0.05,0)+IFERROR(K30/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M30" s="13">
-        <f>IF(L30="","",IF(L30&gt;=0.85,"Meets/Exceeds",IF(L30&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N30" s="8" t="n"/>
-      <c r="O30" s="13" t="n"/>
-      <c r="P30" s="13" t="n"/>
-      <c r="Q30" s="96" t="n"/>
-    </row>
-    <row r="31" ht="18" customHeight="1" s="187">
-      <c r="A31" s="24" t="n"/>
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="24" t="n"/>
-      <c r="F31" s="24" t="n"/>
-      <c r="G31" s="24" t="n"/>
-      <c r="H31" s="24" t="n"/>
-      <c r="I31" s="24" t="n"/>
-      <c r="J31" s="24" t="n"/>
-      <c r="K31" s="24" t="n"/>
-      <c r="L31" s="325">
-        <f>IF((COUNT(E31)+COUNT(F31)+COUNT(G31)+COUNT(H31)+COUNT(I31)+COUNT(J31)+COUNT(K31))=0,"",IFERROR(E31/5*0.3,0)+IFERROR(F31/5*0.2,0)+IFERROR(G31/5*0.15,0)+IFERROR(H31/5*0.15,0)+IFERROR(I31/5*0.1,0)+IFERROR(J31/5*0.05,0)+IFERROR(K31/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M31" s="11">
-        <f>IF(L31="","",IF(L31&gt;=0.85,"Meets/Exceeds",IF(L31&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N31" s="6" t="n"/>
-      <c r="O31" s="11" t="n"/>
-      <c r="P31" s="11" t="n"/>
-      <c r="Q31" s="96" t="n"/>
-    </row>
-    <row r="32" ht="18" customHeight="1" s="187">
-      <c r="A32" s="24" t="n"/>
-      <c r="B32" s="24" t="n"/>
-      <c r="C32" s="24" t="n"/>
-      <c r="D32" s="24" t="n"/>
-      <c r="E32" s="24" t="n"/>
-      <c r="F32" s="24" t="n"/>
-      <c r="G32" s="24" t="n"/>
-      <c r="H32" s="24" t="n"/>
-      <c r="I32" s="24" t="n"/>
-      <c r="J32" s="24" t="n"/>
-      <c r="K32" s="24" t="n"/>
-      <c r="L32" s="326">
-        <f>IF((COUNT(E32)+COUNT(F32)+COUNT(G32)+COUNT(H32)+COUNT(I32)+COUNT(J32)+COUNT(K32))=0,"",IFERROR(E32/5*0.3,0)+IFERROR(F32/5*0.2,0)+IFERROR(G32/5*0.15,0)+IFERROR(H32/5*0.15,0)+IFERROR(I32/5*0.1,0)+IFERROR(J32/5*0.05,0)+IFERROR(K32/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M32" s="13">
-        <f>IF(L32="","",IF(L32&gt;=0.85,"Meets/Exceeds",IF(L32&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N32" s="8" t="n"/>
-      <c r="O32" s="13" t="n"/>
-      <c r="P32" s="13" t="n"/>
-      <c r="Q32" s="96" t="n"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" s="187">
-      <c r="A33" s="24" t="n"/>
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="24" t="n"/>
-      <c r="D33" s="24" t="n"/>
-      <c r="E33" s="24" t="n"/>
-      <c r="F33" s="24" t="n"/>
-      <c r="G33" s="24" t="n"/>
-      <c r="H33" s="24" t="n"/>
-      <c r="I33" s="24" t="n"/>
-      <c r="J33" s="24" t="n"/>
-      <c r="K33" s="24" t="n"/>
-      <c r="L33" s="325">
-        <f>IF((COUNT(E33)+COUNT(F33)+COUNT(G33)+COUNT(H33)+COUNT(I33)+COUNT(J33)+COUNT(K33))=0,"",IFERROR(E33/5*0.3,0)+IFERROR(F33/5*0.2,0)+IFERROR(G33/5*0.15,0)+IFERROR(H33/5*0.15,0)+IFERROR(I33/5*0.1,0)+IFERROR(J33/5*0.05,0)+IFERROR(K33/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M33" s="11">
-        <f>IF(L33="","",IF(L33&gt;=0.85,"Meets/Exceeds",IF(L33&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N33" s="6" t="n"/>
-      <c r="O33" s="11" t="n"/>
-      <c r="P33" s="11" t="n"/>
-      <c r="Q33" s="96" t="n"/>
-    </row>
-    <row r="34" ht="18" customHeight="1" s="187">
-      <c r="A34" s="24" t="n"/>
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="24" t="n"/>
-      <c r="D34" s="24" t="n"/>
-      <c r="E34" s="24" t="n"/>
-      <c r="F34" s="24" t="n"/>
-      <c r="G34" s="24" t="n"/>
-      <c r="H34" s="24" t="n"/>
-      <c r="I34" s="24" t="n"/>
-      <c r="J34" s="24" t="n"/>
-      <c r="K34" s="24" t="n"/>
-      <c r="L34" s="326">
-        <f>IF((COUNT(E34)+COUNT(F34)+COUNT(G34)+COUNT(H34)+COUNT(I34)+COUNT(J34)+COUNT(K34))=0,"",IFERROR(E34/5*0.3,0)+IFERROR(F34/5*0.2,0)+IFERROR(G34/5*0.15,0)+IFERROR(H34/5*0.15,0)+IFERROR(I34/5*0.1,0)+IFERROR(J34/5*0.05,0)+IFERROR(K34/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M34" s="13">
-        <f>IF(L34="","",IF(L34&gt;=0.85,"Meets/Exceeds",IF(L34&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N34" s="8" t="n"/>
-      <c r="O34" s="13" t="n"/>
-      <c r="P34" s="13" t="n"/>
-      <c r="Q34" s="96" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1" s="187">
-      <c r="A35" s="24" t="n"/>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="24" t="n"/>
-      <c r="D35" s="24" t="n"/>
-      <c r="E35" s="24" t="n"/>
-      <c r="F35" s="24" t="n"/>
-      <c r="G35" s="24" t="n"/>
-      <c r="H35" s="24" t="n"/>
-      <c r="I35" s="24" t="n"/>
-      <c r="J35" s="24" t="n"/>
-      <c r="K35" s="24" t="n"/>
-      <c r="L35" s="325">
-        <f>IF((COUNT(E35)+COUNT(F35)+COUNT(G35)+COUNT(H35)+COUNT(I35)+COUNT(J35)+COUNT(K35))=0,"",IFERROR(E35/5*0.3,0)+IFERROR(F35/5*0.2,0)+IFERROR(G35/5*0.15,0)+IFERROR(H35/5*0.15,0)+IFERROR(I35/5*0.1,0)+IFERROR(J35/5*0.05,0)+IFERROR(K35/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M35" s="11">
-        <f>IF(L35="","",IF(L35&gt;=0.85,"Meets/Exceeds",IF(L35&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N35" s="6" t="n"/>
-      <c r="O35" s="11" t="n"/>
-      <c r="P35" s="11" t="n"/>
-      <c r="Q35" s="96" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1" s="187">
-      <c r="A36" s="24" t="n"/>
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="24" t="n"/>
-      <c r="D36" s="24" t="n"/>
-      <c r="E36" s="24" t="n"/>
-      <c r="F36" s="24" t="n"/>
-      <c r="G36" s="24" t="n"/>
-      <c r="H36" s="24" t="n"/>
-      <c r="I36" s="24" t="n"/>
-      <c r="J36" s="24" t="n"/>
-      <c r="K36" s="24" t="n"/>
-      <c r="L36" s="326">
-        <f>IF((COUNT(E36)+COUNT(F36)+COUNT(G36)+COUNT(H36)+COUNT(I36)+COUNT(J36)+COUNT(K36))=0,"",IFERROR(E36/5*0.3,0)+IFERROR(F36/5*0.2,0)+IFERROR(G36/5*0.15,0)+IFERROR(H36/5*0.15,0)+IFERROR(I36/5*0.1,0)+IFERROR(J36/5*0.05,0)+IFERROR(K36/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M36" s="13">
-        <f>IF(L36="","",IF(L36&gt;=0.85,"Meets/Exceeds",IF(L36&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N36" s="8" t="n"/>
-      <c r="O36" s="13" t="n"/>
-      <c r="P36" s="13" t="n"/>
-      <c r="Q36" s="96" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1" s="187">
-      <c r="A37" s="24" t="n"/>
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="24" t="n"/>
-      <c r="D37" s="24" t="n"/>
-      <c r="E37" s="24" t="n"/>
-      <c r="F37" s="24" t="n"/>
-      <c r="G37" s="24" t="n"/>
-      <c r="H37" s="24" t="n"/>
-      <c r="I37" s="24" t="n"/>
-      <c r="J37" s="24" t="n"/>
-      <c r="K37" s="24" t="n"/>
-      <c r="L37" s="325">
-        <f>IF((COUNT(E37)+COUNT(F37)+COUNT(G37)+COUNT(H37)+COUNT(I37)+COUNT(J37)+COUNT(K37))=0,"",IFERROR(E37/5*0.3,0)+IFERROR(F37/5*0.2,0)+IFERROR(G37/5*0.15,0)+IFERROR(H37/5*0.15,0)+IFERROR(I37/5*0.1,0)+IFERROR(J37/5*0.05,0)+IFERROR(K37/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M37" s="11">
-        <f>IF(L37="","",IF(L37&gt;=0.85,"Meets/Exceeds",IF(L37&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N37" s="6" t="n"/>
-      <c r="O37" s="11" t="n"/>
-      <c r="P37" s="11" t="n"/>
-      <c r="Q37" s="96" t="n"/>
-    </row>
-    <row r="38" ht="18" customHeight="1" s="187">
-      <c r="A38" s="24" t="n"/>
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="24" t="n"/>
-      <c r="D38" s="24" t="n"/>
-      <c r="E38" s="24" t="n"/>
-      <c r="F38" s="24" t="n"/>
-      <c r="G38" s="24" t="n"/>
-      <c r="H38" s="24" t="n"/>
-      <c r="I38" s="24" t="n"/>
-      <c r="J38" s="24" t="n"/>
-      <c r="K38" s="24" t="n"/>
-      <c r="L38" s="326">
-        <f>IF((COUNT(E38)+COUNT(F38)+COUNT(G38)+COUNT(H38)+COUNT(I38)+COUNT(J38)+COUNT(K38))=0,"",IFERROR(E38/5*0.3,0)+IFERROR(F38/5*0.2,0)+IFERROR(G38/5*0.15,0)+IFERROR(H38/5*0.15,0)+IFERROR(I38/5*0.1,0)+IFERROR(J38/5*0.05,0)+IFERROR(K38/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M38" s="13">
-        <f>IF(L38="","",IF(L38&gt;=0.85,"Meets/Exceeds",IF(L38&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N38" s="8" t="n"/>
-      <c r="O38" s="13" t="n"/>
-      <c r="P38" s="13" t="n"/>
-      <c r="Q38" s="96" t="n"/>
-    </row>
-    <row r="39" ht="18" customHeight="1" s="187">
-      <c r="A39" s="24" t="n"/>
-      <c r="B39" s="24" t="n"/>
-      <c r="C39" s="24" t="n"/>
-      <c r="D39" s="24" t="n"/>
-      <c r="E39" s="24" t="n"/>
-      <c r="F39" s="24" t="n"/>
-      <c r="G39" s="24" t="n"/>
-      <c r="H39" s="24" t="n"/>
-      <c r="I39" s="24" t="n"/>
-      <c r="J39" s="24" t="n"/>
-      <c r="K39" s="24" t="n"/>
-      <c r="L39" s="325">
-        <f>IF((COUNT(E39)+COUNT(F39)+COUNT(G39)+COUNT(H39)+COUNT(I39)+COUNT(J39)+COUNT(K39))=0,"",IFERROR(E39/5*0.3,0)+IFERROR(F39/5*0.2,0)+IFERROR(G39/5*0.15,0)+IFERROR(H39/5*0.15,0)+IFERROR(I39/5*0.1,0)+IFERROR(J39/5*0.05,0)+IFERROR(K39/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M39" s="11">
-        <f>IF(L39="","",IF(L39&gt;=0.85,"Meets/Exceeds",IF(L39&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N39" s="6" t="n"/>
-      <c r="O39" s="11" t="n"/>
-      <c r="P39" s="11" t="n"/>
-      <c r="Q39" s="96" t="n"/>
-    </row>
-    <row r="40" ht="18" customHeight="1" s="187">
-      <c r="A40" s="24" t="n"/>
-      <c r="B40" s="24" t="n"/>
-      <c r="C40" s="24" t="n"/>
-      <c r="D40" s="24" t="n"/>
-      <c r="E40" s="24" t="n"/>
-      <c r="F40" s="24" t="n"/>
-      <c r="G40" s="24" t="n"/>
-      <c r="H40" s="24" t="n"/>
-      <c r="I40" s="24" t="n"/>
-      <c r="J40" s="24" t="n"/>
-      <c r="K40" s="24" t="n"/>
-      <c r="L40" s="326">
-        <f>IF((COUNT(E40)+COUNT(F40)+COUNT(G40)+COUNT(H40)+COUNT(I40)+COUNT(J40)+COUNT(K40))=0,"",IFERROR(E40/5*0.3,0)+IFERROR(F40/5*0.2,0)+IFERROR(G40/5*0.15,0)+IFERROR(H40/5*0.15,0)+IFERROR(I40/5*0.1,0)+IFERROR(J40/5*0.05,0)+IFERROR(K40/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M40" s="13">
-        <f>IF(L40="","",IF(L40&gt;=0.85,"Meets/Exceeds",IF(L40&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N40" s="8" t="n"/>
-      <c r="O40" s="13" t="n"/>
-      <c r="P40" s="13" t="n"/>
-      <c r="Q40" s="96" t="n"/>
-    </row>
-    <row r="41" ht="18" customHeight="1" s="187">
-      <c r="A41" s="24" t="n"/>
-      <c r="B41" s="24" t="n"/>
-      <c r="C41" s="24" t="n"/>
-      <c r="D41" s="24" t="n"/>
-      <c r="E41" s="24" t="n"/>
-      <c r="F41" s="24" t="n"/>
-      <c r="G41" s="24" t="n"/>
-      <c r="H41" s="24" t="n"/>
-      <c r="I41" s="24" t="n"/>
-      <c r="J41" s="24" t="n"/>
-      <c r="K41" s="24" t="n"/>
-      <c r="L41" s="325">
-        <f>IF((COUNT(E41)+COUNT(F41)+COUNT(G41)+COUNT(H41)+COUNT(I41)+COUNT(J41)+COUNT(K41))=0,"",IFERROR(E41/5*0.3,0)+IFERROR(F41/5*0.2,0)+IFERROR(G41/5*0.15,0)+IFERROR(H41/5*0.15,0)+IFERROR(I41/5*0.1,0)+IFERROR(J41/5*0.05,0)+IFERROR(K41/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M41" s="11">
-        <f>IF(L41="","",IF(L41&gt;=0.85,"Meets/Exceeds",IF(L41&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N41" s="6" t="n"/>
-      <c r="O41" s="11" t="n"/>
-      <c r="P41" s="11" t="n"/>
-      <c r="Q41" s="96" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" s="187">
-      <c r="A42" s="24" t="n"/>
-      <c r="B42" s="24" t="n"/>
-      <c r="C42" s="24" t="n"/>
-      <c r="D42" s="24" t="n"/>
-      <c r="E42" s="24" t="n"/>
-      <c r="F42" s="24" t="n"/>
-      <c r="G42" s="24" t="n"/>
-      <c r="H42" s="24" t="n"/>
-      <c r="I42" s="24" t="n"/>
-      <c r="J42" s="24" t="n"/>
-      <c r="K42" s="24" t="n"/>
-      <c r="L42" s="326">
-        <f>IF((COUNT(E42)+COUNT(F42)+COUNT(G42)+COUNT(H42)+COUNT(I42)+COUNT(J42)+COUNT(K42))=0,"",IFERROR(E42/5*0.3,0)+IFERROR(F42/5*0.2,0)+IFERROR(G42/5*0.15,0)+IFERROR(H42/5*0.15,0)+IFERROR(I42/5*0.1,0)+IFERROR(J42/5*0.05,0)+IFERROR(K42/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M42" s="13">
-        <f>IF(L42="","",IF(L42&gt;=0.85,"Meets/Exceeds",IF(L42&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N42" s="8" t="n"/>
-      <c r="O42" s="13" t="n"/>
-      <c r="P42" s="13" t="n"/>
-      <c r="Q42" s="96" t="n"/>
-    </row>
-    <row r="43" ht="18" customHeight="1" s="187">
-      <c r="A43" s="24" t="n"/>
-      <c r="B43" s="24" t="n"/>
-      <c r="C43" s="24" t="n"/>
-      <c r="D43" s="24" t="n"/>
-      <c r="E43" s="24" t="n"/>
-      <c r="F43" s="24" t="n"/>
-      <c r="G43" s="24" t="n"/>
-      <c r="H43" s="24" t="n"/>
-      <c r="I43" s="24" t="n"/>
-      <c r="J43" s="24" t="n"/>
-      <c r="K43" s="24" t="n"/>
-      <c r="L43" s="325">
-        <f>IF((COUNT(E43)+COUNT(F43)+COUNT(G43)+COUNT(H43)+COUNT(I43)+COUNT(J43)+COUNT(K43))=0,"",IFERROR(E43/5*0.3,0)+IFERROR(F43/5*0.2,0)+IFERROR(G43/5*0.15,0)+IFERROR(H43/5*0.15,0)+IFERROR(I43/5*0.1,0)+IFERROR(J43/5*0.05,0)+IFERROR(K43/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M43" s="11">
-        <f>IF(L43="","",IF(L43&gt;=0.85,"Meets/Exceeds",IF(L43&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N43" s="6" t="n"/>
-      <c r="O43" s="11" t="n"/>
-      <c r="P43" s="11" t="n"/>
-      <c r="Q43" s="96" t="n"/>
-    </row>
-    <row r="44" ht="18" customHeight="1" s="187">
-      <c r="A44" s="24" t="n"/>
-      <c r="B44" s="24" t="n"/>
-      <c r="C44" s="24" t="n"/>
-      <c r="D44" s="24" t="n"/>
-      <c r="E44" s="24" t="n"/>
-      <c r="F44" s="24" t="n"/>
-      <c r="G44" s="24" t="n"/>
-      <c r="H44" s="24" t="n"/>
-      <c r="I44" s="24" t="n"/>
-      <c r="J44" s="24" t="n"/>
-      <c r="K44" s="24" t="n"/>
-      <c r="L44" s="326">
-        <f>IF((COUNT(E44)+COUNT(F44)+COUNT(G44)+COUNT(H44)+COUNT(I44)+COUNT(J44)+COUNT(K44))=0,"",IFERROR(E44/5*0.3,0)+IFERROR(F44/5*0.2,0)+IFERROR(G44/5*0.15,0)+IFERROR(H44/5*0.15,0)+IFERROR(I44/5*0.1,0)+IFERROR(J44/5*0.05,0)+IFERROR(K44/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M44" s="13">
-        <f>IF(L44="","",IF(L44&gt;=0.85,"Meets/Exceeds",IF(L44&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N44" s="8" t="n"/>
-      <c r="O44" s="13" t="n"/>
-      <c r="P44" s="13" t="n"/>
-      <c r="Q44" s="96" t="n"/>
-    </row>
-    <row r="45" ht="18" customHeight="1" s="187">
-      <c r="A45" s="24" t="n"/>
-      <c r="B45" s="24" t="n"/>
-      <c r="C45" s="24" t="n"/>
-      <c r="D45" s="24" t="n"/>
-      <c r="E45" s="24" t="n"/>
-      <c r="F45" s="24" t="n"/>
-      <c r="G45" s="24" t="n"/>
-      <c r="H45" s="24" t="n"/>
-      <c r="I45" s="24" t="n"/>
-      <c r="J45" s="24" t="n"/>
-      <c r="K45" s="24" t="n"/>
-      <c r="L45" s="325">
-        <f>IF((COUNT(E45)+COUNT(F45)+COUNT(G45)+COUNT(H45)+COUNT(I45)+COUNT(J45)+COUNT(K45))=0,"",IFERROR(E45/5*0.3,0)+IFERROR(F45/5*0.2,0)+IFERROR(G45/5*0.15,0)+IFERROR(H45/5*0.15,0)+IFERROR(I45/5*0.1,0)+IFERROR(J45/5*0.05,0)+IFERROR(K45/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M45" s="11">
-        <f>IF(L45="","",IF(L45&gt;=0.85,"Meets/Exceeds",IF(L45&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N45" s="6" t="n"/>
-      <c r="O45" s="11" t="n"/>
-      <c r="P45" s="11" t="n"/>
-      <c r="Q45" s="96" t="n"/>
-    </row>
-    <row r="46" ht="18" customHeight="1" s="187">
-      <c r="A46" s="24" t="n"/>
-      <c r="B46" s="24" t="n"/>
-      <c r="C46" s="24" t="n"/>
-      <c r="D46" s="24" t="n"/>
-      <c r="E46" s="24" t="n"/>
-      <c r="F46" s="24" t="n"/>
-      <c r="G46" s="24" t="n"/>
-      <c r="H46" s="24" t="n"/>
-      <c r="I46" s="24" t="n"/>
-      <c r="J46" s="24" t="n"/>
-      <c r="K46" s="24" t="n"/>
-      <c r="L46" s="326">
-        <f>IF((COUNT(E46)+COUNT(F46)+COUNT(G46)+COUNT(H46)+COUNT(I46)+COUNT(J46)+COUNT(K46))=0,"",IFERROR(E46/5*0.3,0)+IFERROR(F46/5*0.2,0)+IFERROR(G46/5*0.15,0)+IFERROR(H46/5*0.15,0)+IFERROR(I46/5*0.1,0)+IFERROR(J46/5*0.05,0)+IFERROR(K46/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M46" s="13">
-        <f>IF(L46="","",IF(L46&gt;=0.85,"Meets/Exceeds",IF(L46&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N46" s="8" t="n"/>
-      <c r="O46" s="13" t="n"/>
-      <c r="P46" s="13" t="n"/>
-      <c r="Q46" s="96" t="n"/>
-    </row>
-    <row r="47" ht="18" customHeight="1" s="187">
-      <c r="A47" s="24" t="n"/>
-      <c r="B47" s="24" t="n"/>
-      <c r="C47" s="24" t="n"/>
-      <c r="D47" s="24" t="n"/>
-      <c r="E47" s="24" t="n"/>
-      <c r="F47" s="24" t="n"/>
-      <c r="G47" s="24" t="n"/>
-      <c r="H47" s="24" t="n"/>
-      <c r="I47" s="24" t="n"/>
-      <c r="J47" s="24" t="n"/>
-      <c r="K47" s="24" t="n"/>
-      <c r="L47" s="325">
-        <f>IF((COUNT(E47)+COUNT(F47)+COUNT(G47)+COUNT(H47)+COUNT(I47)+COUNT(J47)+COUNT(K47))=0,"",IFERROR(E47/5*0.3,0)+IFERROR(F47/5*0.2,0)+IFERROR(G47/5*0.15,0)+IFERROR(H47/5*0.15,0)+IFERROR(I47/5*0.1,0)+IFERROR(J47/5*0.05,0)+IFERROR(K47/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M47" s="11">
-        <f>IF(L47="","",IF(L47&gt;=0.85,"Meets/Exceeds",IF(L47&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N47" s="6" t="n"/>
-      <c r="O47" s="11" t="n"/>
-      <c r="P47" s="11" t="n"/>
-      <c r="Q47" s="96" t="n"/>
-    </row>
-    <row r="48" ht="18" customHeight="1" s="187">
-      <c r="A48" s="24" t="n"/>
-      <c r="B48" s="24" t="n"/>
-      <c r="C48" s="24" t="n"/>
-      <c r="D48" s="24" t="n"/>
-      <c r="E48" s="24" t="n"/>
-      <c r="F48" s="24" t="n"/>
-      <c r="G48" s="24" t="n"/>
-      <c r="H48" s="24" t="n"/>
-      <c r="I48" s="24" t="n"/>
-      <c r="J48" s="24" t="n"/>
-      <c r="K48" s="24" t="n"/>
-      <c r="L48" s="326">
-        <f>IF((COUNT(E48)+COUNT(F48)+COUNT(G48)+COUNT(H48)+COUNT(I48)+COUNT(J48)+COUNT(K48))=0,"",IFERROR(E48/5*0.3,0)+IFERROR(F48/5*0.2,0)+IFERROR(G48/5*0.15,0)+IFERROR(H48/5*0.15,0)+IFERROR(I48/5*0.1,0)+IFERROR(J48/5*0.05,0)+IFERROR(K48/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M48" s="13">
-        <f>IF(L48="","",IF(L48&gt;=0.85,"Meets/Exceeds",IF(L48&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N48" s="8" t="n"/>
-      <c r="O48" s="13" t="n"/>
-      <c r="P48" s="13" t="n"/>
-      <c r="Q48" s="96" t="n"/>
-    </row>
-    <row r="49" ht="18" customHeight="1" s="187">
-      <c r="A49" s="24" t="n"/>
-      <c r="B49" s="24" t="n"/>
-      <c r="C49" s="24" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="24" t="n"/>
-      <c r="F49" s="24" t="n"/>
-      <c r="G49" s="24" t="n"/>
-      <c r="H49" s="24" t="n"/>
-      <c r="I49" s="24" t="n"/>
-      <c r="J49" s="24" t="n"/>
-      <c r="K49" s="24" t="n"/>
-      <c r="L49" s="325">
-        <f>IF((COUNT(E49)+COUNT(F49)+COUNT(G49)+COUNT(H49)+COUNT(I49)+COUNT(J49)+COUNT(K49))=0,"",IFERROR(E49/5*0.3,0)+IFERROR(F49/5*0.2,0)+IFERROR(G49/5*0.15,0)+IFERROR(H49/5*0.15,0)+IFERROR(I49/5*0.1,0)+IFERROR(J49/5*0.05,0)+IFERROR(K49/5*0.05,0))</f>
-        <v/>
-      </c>
-      <c r="M49" s="11">
-        <f>IF(L49="","",IF(L49&gt;=0.85,"Meets/Exceeds",IF(L49&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="N49" s="6" t="n"/>
-      <c r="O49" s="11" t="n"/>
-      <c r="P49" s="11" t="n"/>
-      <c r="Q49" s="96" t="n"/>
-    </row>
-    <row r="51" ht="15.6" customHeight="1" s="187">
-      <c r="A51" s="276" t="inlineStr">
-        <is>
-          <t>TEAM AVERAGE</t>
-        </is>
-      </c>
-      <c r="B51" s="212" t="n"/>
-      <c r="C51" s="212" t="n"/>
-      <c r="D51" s="192" t="n"/>
-      <c r="E51" s="327">
-        <f>IFERROR(AVERAGE(E5:E49),"")</f>
-        <v/>
-      </c>
-      <c r="F51" s="327">
-        <f>IFERROR(AVERAGE(F5:F49),"")</f>
-        <v/>
-      </c>
-      <c r="G51" s="327">
-        <f>IFERROR(AVERAGE(G5:G49),"")</f>
-        <v/>
-      </c>
-      <c r="H51" s="327">
-        <f>IFERROR(AVERAGE(H5:H49),"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="327">
-        <f>IFERROR(AVERAGE(I5:I49),"")</f>
-        <v/>
-      </c>
-      <c r="J51" s="327">
-        <f>IFERROR(AVERAGE(J5:J49),"")</f>
-        <v/>
-      </c>
-      <c r="K51" s="327">
-        <f>IFERROR(AVERAGE(K5:K49),"")</f>
-        <v/>
-      </c>
-      <c r="L51" s="328">
-        <f>IFERROR(AVERAGE(L5:L49),"")</f>
-        <v/>
-      </c>
-      <c r="M51" s="14" t="n"/>
-      <c r="N51" s="29" t="inlineStr">
-        <is>
-          <t>Average of logged touches</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="21.95" customHeight="1" s="187">
-      <c r="A53" s="281" t="inlineStr">
-        <is>
-          <t>TEAM / JOURNEY SCORES — MULTI-TOUCH CASES</t>
-        </is>
-      </c>
-      <c r="B53" s="212" t="n"/>
-      <c r="C53" s="212" t="n"/>
-      <c r="D53" s="212" t="n"/>
-      <c r="E53" s="212" t="n"/>
-      <c r="F53" s="212" t="n"/>
-      <c r="G53" s="212" t="n"/>
-      <c r="H53" s="212" t="n"/>
-      <c r="I53" s="212" t="n"/>
-      <c r="J53" s="212" t="n"/>
-      <c r="K53" s="212" t="n"/>
-      <c r="L53" s="212" t="n"/>
-      <c r="M53" s="212" t="n"/>
-      <c r="N53" s="212" t="n"/>
-      <c r="O53" s="212" t="n"/>
-      <c r="P53" s="192" t="n"/>
-    </row>
-    <row r="54" ht="32.1" customHeight="1" s="187">
-      <c r="A54" s="279" t="inlineStr">
-        <is>
-          <t>Team Score  =  20% × Level 1 avg touch  +  30% × Level 2 avg touch  +  30% × (Journey Outcome ÷ 5)  +  20% × (Continuity of Support ÷ 5)   │   Level 2 touches carry a higher weight in the team aggregate.</t>
-        </is>
-      </c>
-      <c r="B54" s="212" t="n"/>
-      <c r="C54" s="212" t="n"/>
-      <c r="D54" s="212" t="n"/>
-      <c r="E54" s="212" t="n"/>
-      <c r="F54" s="212" t="n"/>
-      <c r="G54" s="212" t="n"/>
-      <c r="H54" s="212" t="n"/>
-      <c r="I54" s="212" t="n"/>
-      <c r="J54" s="212" t="n"/>
-      <c r="K54" s="212" t="n"/>
-      <c r="L54" s="212" t="n"/>
-      <c r="M54" s="212" t="n"/>
-      <c r="N54" s="212" t="n"/>
-      <c r="O54" s="212" t="n"/>
-      <c r="P54" s="192" t="n"/>
-    </row>
-    <row r="55" ht="26.1" customHeight="1" s="187">
-      <c r="A55" s="278" t="inlineStr">
-        <is>
-          <t>Journey / Case ID(s)</t>
-        </is>
-      </c>
-      <c r="B55" s="192" t="n"/>
-      <c r="C55" s="278" t="inlineStr">
-        <is>
-          <t>Touches</t>
-        </is>
-      </c>
-      <c r="D55" s="23" t="inlineStr">
-        <is>
-          <t>Avg Touch % (ref)</t>
-        </is>
-      </c>
-      <c r="E55" s="23" t="inlineStr">
-        <is>
-          <t>Journey Outcome</t>
-        </is>
-      </c>
-      <c r="F55" s="23" t="inlineStr">
-        <is>
-          <t>Continuity of Support</t>
-        </is>
-      </c>
-      <c r="G55" s="23" t="inlineStr">
-        <is>
-          <t>TEAM SCORE</t>
-        </is>
-      </c>
-      <c r="H55" s="278" t="inlineStr">
-        <is>
-          <t>Band</t>
-        </is>
-      </c>
-      <c r="I55" s="214" t="inlineStr">
-        <is>
-          <t>Journey notes (where the chain broke / recovered)</t>
-        </is>
-      </c>
-      <c r="J55" s="212" t="n"/>
-      <c r="K55" s="212" t="n"/>
-      <c r="L55" s="212" t="n"/>
-      <c r="M55" s="212" t="n"/>
-      <c r="N55" s="192" t="n"/>
-    </row>
-    <row r="56" ht="48" customHeight="1" s="187">
-      <c r="A56" s="329" t="n"/>
-      <c r="B56" s="244" t="n"/>
-      <c r="C56" s="13">
-        <f>IF(A56="","",COUNTIF(B5:B49,A56))</f>
-        <v/>
-      </c>
-      <c r="D56" s="330">
-        <f>IF(A56="","",IFERROR(AVERAGEIF(B5:B49,A56,L5:L49),""))</f>
-        <v/>
-      </c>
-      <c r="E56" s="7" t="n"/>
-      <c r="F56" s="7" t="n"/>
-      <c r="G56" s="98">
-        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(IFERROR(VALUE(LEFT(E56,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F56,1)),0)/5),""))</f>
-        <v/>
-      </c>
-      <c r="H56" s="13">
-        <f>IF(G56="","",IF(G56&gt;=0.85,"Meets/Exceeds",IF(G56&gt;=0.7,"Developing","Needs Improvement")))</f>
-        <v/>
-      </c>
-      <c r="I56" s="322" t="n"/>
-      <c r="J56" s="243" t="n"/>
-      <c r="K56" s="243" t="n"/>
-      <c r="L56" s="243" t="n"/>
-      <c r="M56" s="243" t="n"/>
-      <c r="N56" s="244" t="n"/>
-    </row>
-    <row r="57" ht="27.95" customHeight="1" s="187">
-      <c r="A57" s="289" t="n"/>
-      <c r="B57" s="244" t="n"/>
-      <c r="C57" s="13">
-        <f>IF(A57="","",COUNTIF(B5:B49,A57))</f>
-        <v/>
-      </c>
-      <c r="D57" s="330">
-        <f>IF(A57="","",IFERROR(AVERAGEIF(B5:B49,A57,L5:L49),""))</f>
-        <v/>
-      </c>
-      <c r="E57" s="7" t="n"/>
-      <c r="F57" s="7" t="n"/>
-      <c r="G57" s="98">
-        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(IFERROR(VALUE(LEFT(E57,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F57,1)),0)/5),""))</f>
-        <v/>
-      </c>
-      <c r="H57" s="13">
-        <f>IF(G57="","",IF(G57&gt;=0.85,"Meets/Exceeds",IF(G57&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="I57" s="331" t="n"/>
-      <c r="J57" s="243" t="n"/>
-      <c r="K57" s="243" t="n"/>
-      <c r="L57" s="243" t="n"/>
-      <c r="M57" s="243" t="n"/>
-      <c r="N57" s="244" t="n"/>
-    </row>
-    <row r="58" ht="27.95" customHeight="1" s="187">
-      <c r="A58" s="289" t="n"/>
-      <c r="B58" s="244" t="n"/>
-      <c r="C58" s="11">
-        <f>IF(A58="","",COUNTIF(B5:B49,A58))</f>
-        <v/>
-      </c>
-      <c r="D58" s="332">
-        <f>IF(A58="","",IFERROR(AVERAGEIF(B5:B49,A58,L5:L49),""))</f>
-        <v/>
-      </c>
-      <c r="E58" s="7" t="n"/>
-      <c r="F58" s="7" t="n"/>
-      <c r="G58" s="99">
-        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(IFERROR(VALUE(LEFT(E58,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F58,1)),0)/5),""))</f>
-        <v/>
-      </c>
-      <c r="H58" s="11">
-        <f>IF(G58="","",IF(G58&gt;=0.85,"Meets/Exceeds",IF(G58&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="I58" s="331" t="n"/>
-      <c r="J58" s="243" t="n"/>
-      <c r="K58" s="243" t="n"/>
-      <c r="L58" s="243" t="n"/>
-      <c r="M58" s="243" t="n"/>
-      <c r="N58" s="244" t="n"/>
-    </row>
-    <row r="59" ht="27.95" customHeight="1" s="187">
-      <c r="A59" s="289" t="n"/>
-      <c r="B59" s="244" t="n"/>
-      <c r="C59" s="13">
-        <f>IF(A59="","",COUNTIF(B5:B49,A59))</f>
-        <v/>
-      </c>
-      <c r="D59" s="330">
-        <f>IF(A59="","",IFERROR(AVERAGEIF(B5:B49,A59,L5:L49),""))</f>
-        <v/>
-      </c>
-      <c r="E59" s="7" t="n"/>
-      <c r="F59" s="7" t="n"/>
-      <c r="G59" s="98">
-        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(IFERROR(VALUE(LEFT(E59,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F59,1)),0)/5),""))</f>
-        <v/>
-      </c>
-      <c r="H59" s="13">
-        <f>IF(G59="","",IF(G59&gt;=0.85,"Meets/Exceeds",IF(G59&gt;=0.7,"Developing","Needs Improv.")))</f>
-        <v/>
-      </c>
-      <c r="I59" s="331" t="n"/>
-      <c r="J59" s="243" t="n"/>
-      <c r="K59" s="243" t="n"/>
-      <c r="L59" s="243" t="n"/>
-      <c r="M59" s="243" t="n"/>
-      <c r="N59" s="244" t="n"/>
-    </row>
-    <row r="60" ht="27.95" customHeight="1" s="187">
-      <c r="A60" s="298" t="inlineStr">
-        <is>
-          <t>Template rows: type a Case ID in the first column — Touches and Avg Touch % auto-fill from the log above, then judge Outcome and Continuity (0-5). For journeys spanning multiple Case IDs (like the pre-loaded one), enter the Avg Touch % formula over the journey's row range manually.</t>
-        </is>
-      </c>
-      <c r="B60" s="243" t="n"/>
-      <c r="C60" s="243" t="n"/>
-      <c r="D60" s="243" t="n"/>
-      <c r="E60" s="243" t="n"/>
-      <c r="F60" s="243" t="n"/>
-      <c r="G60" s="243" t="n"/>
-      <c r="H60" s="243" t="n"/>
-      <c r="I60" s="243" t="n"/>
-      <c r="J60" s="243" t="n"/>
-      <c r="K60" s="243" t="n"/>
-      <c r="L60" s="243" t="n"/>
-      <c r="M60" s="243" t="n"/>
-      <c r="N60" s="244" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="I55:N55"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="I59:N59"/>
-    <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A53:P53"/>
-    <mergeCell ref="A60:N60"/>
-    <mergeCell ref="I56:N56"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="I57:N57"/>
-    <mergeCell ref="I58:N58"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="A2:P2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="A3">
-    <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="22">
-      <formula>$G$56&gt;=0.85</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="21">
-      <formula>$G$56&gt;=0.85</formula>
-    </cfRule>
-    <cfRule type="expression" priority="15" dxfId="20">
-      <formula>AND($G$56&gt;=0.7,$G$56&lt;0.85)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="19">
-      <formula>$G$56&lt;0.7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G56:G59">
-    <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="2">
-      <formula>0.85</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="8" operator="between" dxfId="1">
-      <formula>0.7</formula>
-      <formula>0.8499</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="0">
-      <formula>0.7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H56:H59">
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
-      <formula>"Meets/Exceeds"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
-      <formula>"Developing"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
-      <formula>"Needs Improv."</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L49">
-    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="2">
-      <formula>0.85</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
-      <formula>0.7</formula>
-      <formula>0.8499</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
-      <formula>0.7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M49">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="9">
-      <formula>"Meets/Exceeds"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="8">
-      <formula>"Developing"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="7">
-      <formula>"Needs Improv."</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O49">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="2">
-      <formula>"Resolver"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
-      <formula>"Progress Builder"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="4">
-      <formula>"Maintainer"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
-      <formula>"Regression Contributor"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P49">
-    <cfRule type="cellIs" priority="21" operator="greaterThanOrEqual" dxfId="2">
-      <formula>4</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="22" operator="between" dxfId="1">
-      <formula>2</formula>
-      <formula>3</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThanOrEqual" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation sqref="E5:K49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5." type="whole">
-      <formula1>0</formula1>
-      <formula2>5</formula2>
-    </dataValidation>
-    <dataValidation sqref="O5:O49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Resolver, Progress Builder, Maintainer, Breaker, or N/A." type="list">
-      <formula1>"Resolver,Progress Builder,Maintainer,Regression Contributor,N/A"</formula1>
-    </dataValidation>
-    <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole">
-      <formula1>0</formula1>
-      <formula2>5</formula2>
-    </dataValidation>
-    <dataValidation sqref="Q5:Q49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Please select Level 1 or Level 2." promptTitle="Agent Level" prompt="Level 1 = front-line support.  Level 2 = senior / escalation support." type="list">
-      <formula1>"Level 1,Level 2"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Make Case Tracker Handoff Quality (col P) a 0-5 dropdown with anchor text
- P5:P49 is now a 0-5 list dropdown (replaces the plain whole-number rule)
- Each cell shows a click-prompt explaining what each score means
  (5 Seamless -> 0 Broken; blank = no handoff)
- Added a visible legend block below the journey table (rows 62-69)
- Values stay NUMERIC so Suggested Continuity (AVERAGEIFS over P) and the
  Team Scoring per-touch breakdown keep working — the descriptive text lives
  in the prompt and legend, not in the cell value

Verified via Excel COM: validation type=list, P-averaging intact
(P5=4,P6=2 -> suggested continuity 3), file opens with no repair prompt.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -1115,7 +1115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="348">
+  <cellXfs count="352">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -2103,6 +2103,18 @@
     </xf>
     <xf numFmtId="0" fontId="80" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="76" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4212,7 +4224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q60"/>
+  <dimension ref="A1:Q69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="187" min="1" max="1"/>
@@ -5817,24 +5829,123 @@
       <c r="M60" s="243" t="n"/>
       <c r="N60" s="244" t="n"/>
     </row>
+    <row r="62" ht="18" customHeight="1" s="187">
+      <c r="A62" s="348" t="inlineStr">
+        <is>
+          <t>HANDOFF QUALITY (Column P) — what each score means</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="16" customHeight="1" s="187">
+      <c r="A63" s="349" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B63" s="350" t="inlineStr">
+        <is>
+          <t>Seamless — the next agent had full context; the customer never had to repeat themselves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16" customHeight="1" s="187">
+      <c r="A64" s="349" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B64" s="351" t="inlineStr">
+        <is>
+          <t>Strong — a minor gap, quickly recovered; the next agent was essentially ready to continue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="16" customHeight="1" s="187">
+      <c r="A65" s="349" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B65" s="350" t="inlineStr">
+        <is>
+          <t>Adequate — the thread held, but some information had to be re-gathered by the next agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="16" customHeight="1" s="187">
+      <c r="A66" s="349" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B66" s="351" t="inlineStr">
+        <is>
+          <t>Weak — thin notes or a wrong status forced significant rework by the receiving agent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="16" customHeight="1" s="187">
+      <c r="A67" s="349" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B67" s="350" t="inlineStr">
+        <is>
+          <t>Poor — the next agent basically restarted; the customer repeated most of the case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="16" customHeight="1" s="187">
+      <c r="A68" s="349" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B68" s="351" t="inlineStr">
+        <is>
+          <t>Broken — no usable handoff; the gap itself created a new problem or complaint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="16" customHeight="1" s="187">
+      <c r="A69" s="349" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="B69" s="350" t="inlineStr">
+        <is>
+          <t>No handoff on this touch — e.g. the final touch, or a single-touch case. Leave the cell empty.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="25">
     <mergeCell ref="A59:B59"/>
+    <mergeCell ref="B65:N65"/>
+    <mergeCell ref="A53:P53"/>
+    <mergeCell ref="A60:N60"/>
+    <mergeCell ref="I56:N56"/>
+    <mergeCell ref="B68:N68"/>
+    <mergeCell ref="B64:N64"/>
+    <mergeCell ref="I58:N58"/>
+    <mergeCell ref="B63:N63"/>
     <mergeCell ref="I55:N55"/>
+    <mergeCell ref="B69:N69"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="B66:N66"/>
     <mergeCell ref="A57:B57"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="I59:N59"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A54:P54"/>
-    <mergeCell ref="A53:P53"/>
-    <mergeCell ref="A60:N60"/>
-    <mergeCell ref="I56:N56"/>
+    <mergeCell ref="B67:N67"/>
+    <mergeCell ref="A62:N62"/>
     <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A51:D51"/>
     <mergeCell ref="I57:N57"/>
-    <mergeCell ref="I58:N58"/>
     <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A55:B55"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <conditionalFormatting sqref="A3">
@@ -5931,12 +6042,11 @@
     <dataValidation sqref="O5:O49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid type" error="Pick Resolver, Progress Builder, Maintainer, Breaker, or N/A." type="list">
       <formula1>"Resolver,Progress Builder,Maintainer,Regression Contributor,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="P5:P16 P18:P49" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid score" error="Enter 0 to 5, or leave blank / type N/A for a final touch with no further handoff." type="whole">
-      <formula1>0</formula1>
-      <formula2>5</formula2>
-    </dataValidation>
     <dataValidation sqref="Q5:Q49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Please select Level 1 or Level 2." promptTitle="Agent Level" prompt="Level 1 = front-line support.  Level 2 = senior / escalation support." type="list">
       <formula1>"Level 1,Level 2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P5:P49" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pick 0-5" error="Select a whole number 0-5 from the dropdown, or leave blank if there was no handoff." promptTitle="Handoff Quality (0-5)" prompt="5 Seamless | 4 Strong (minor gap, recovered) | 3 Adequate (some re-gathering) | 2 Weak (rework from thin notes/wrong status) | 1 Poor (next agent restarts) | 0 Broken (no usable handoff). Leave blank if this touch had no handoff (e.g. final touch)." type="list">
+      <formula1>"0,1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove Journey ID column — revert to Case ID keying
Multi-ticket journeys weren't needed, so the Journey ID column (col R) added
extra entry for no benefit. Reverted the journey rollup to key on Case ID:
one Case ID groups all the touches of one journey.

Kept the journey selector (Team Scoring E6) and the Multi-Touch Guide doc
reconciliation — the selector now picks a journey by its Case ID.

Verified via Excel COM: column R empty; a 3-touch single-Case-ID journey rolls
up to 0.78; selector switches journeys (0.78 split <-> 0.90 collapsed); file
opens with no repair prompt.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -4251,7 +4251,7 @@
     <col width="60" customWidth="1" style="187" min="14" max="14"/>
     <col width="22" customWidth="1" style="187" min="15" max="15"/>
     <col width="14" customWidth="1" style="187" min="16" max="17"/>
-    <col width="16" customWidth="1" style="187" min="18" max="18"/>
+    <col width="8.43" customWidth="1" style="187" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.1" customHeight="1" s="187">
@@ -4279,7 +4279,7 @@
     <row r="2" ht="15.95" customHeight="1" s="187">
       <c r="A2" s="282" t="inlineStr">
         <is>
-          <t>One row per touch — the Case Tracker is for MULTI-TOUCH cases only. Give every touch of a journey the same Journey ID (column R) to group it — a journey may span multiple Case IDs. Weighted % and Result calculate automatically. For single-call evaluations, use the Scoring Form sheet only — no Case Tracker entry needed.</t>
+          <t>One row per touch — the Case Tracker is for MULTI-TOUCH cases only. Give every touch of a case the same Case ID to group it into one journey; Weighted % and Result calculate automatically. For single-call evaluations, use the Scoring Form sheet only — no Case Tracker entry needed.</t>
         </is>
       </c>
       <c r="B2" s="212" t="n"/>
@@ -4300,7 +4300,7 @@
     </row>
     <row r="3" ht="24" customHeight="1" s="187">
       <c r="A3" s="275">
-        <f>IF(A56="","  JOURNEY TEAM SCORE  ▸  log touches below, then enter a Journey ID + Outcome/Continuity in row 56","  LOADED JOURNEY TEAM SCORE  ▸  "&amp;A56&amp;":  "&amp;TEXT(G56,"0.0%")&amp;"   "&amp;UPPER(H56))</f>
+        <f>IF(A56="","  JOURNEY TEAM SCORE  ▸  log touches below, then enter a Case ID + Outcome/Continuity in row 56","  LOADED JOURNEY TEAM SCORE  ▸  "&amp;A56&amp;":  "&amp;TEXT(G56,"0.0%")&amp;"   "&amp;UPPER(H56))</f>
         <v/>
       </c>
       <c r="B3" s="212" t="n"/>
@@ -4405,11 +4405,6 @@
           <t>Level</t>
         </is>
       </c>
-      <c r="R4" s="23" t="inlineStr">
-        <is>
-          <t>Journey ID</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="39.95" customHeight="1" s="187">
       <c r="A5" s="24" t="n"/>
@@ -4435,7 +4430,6 @@
       <c r="O5" s="11" t="n"/>
       <c r="P5" s="11" t="n"/>
       <c r="Q5" s="96" t="n"/>
-      <c r="R5" s="24" t="n"/>
     </row>
     <row r="6" ht="39.95" customHeight="1" s="187">
       <c r="A6" s="24" t="n"/>
@@ -4461,7 +4455,6 @@
       <c r="O6" s="13" t="n"/>
       <c r="P6" s="13" t="n"/>
       <c r="Q6" s="96" t="n"/>
-      <c r="R6" s="24" t="n"/>
     </row>
     <row r="7" ht="39.95" customHeight="1" s="187">
       <c r="A7" s="24" t="n"/>
@@ -4487,7 +4480,6 @@
       <c r="O7" s="11" t="n"/>
       <c r="P7" s="11" t="n"/>
       <c r="Q7" s="96" t="n"/>
-      <c r="R7" s="24" t="n"/>
     </row>
     <row r="8" ht="39.95" customHeight="1" s="187">
       <c r="A8" s="24" t="n"/>
@@ -4513,7 +4505,6 @@
       <c r="O8" s="13" t="n"/>
       <c r="P8" s="13" t="n"/>
       <c r="Q8" s="96" t="n"/>
-      <c r="R8" s="24" t="n"/>
     </row>
     <row r="9" ht="39.95" customHeight="1" s="187">
       <c r="A9" s="24" t="n"/>
@@ -4539,7 +4530,6 @@
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
       <c r="Q9" s="96" t="n"/>
-      <c r="R9" s="24" t="n"/>
     </row>
     <row r="10" ht="39.95" customHeight="1" s="187">
       <c r="A10" s="24" t="n"/>
@@ -4565,7 +4555,6 @@
       <c r="O10" s="13" t="n"/>
       <c r="P10" s="13" t="n"/>
       <c r="Q10" s="96" t="n"/>
-      <c r="R10" s="24" t="n"/>
     </row>
     <row r="11" ht="39.95" customHeight="1" s="187">
       <c r="A11" s="24" t="n"/>
@@ -4591,7 +4580,6 @@
       <c r="O11" s="11" t="n"/>
       <c r="P11" s="11" t="n"/>
       <c r="Q11" s="96" t="n"/>
-      <c r="R11" s="24" t="n"/>
     </row>
     <row r="12" ht="39.95" customHeight="1" s="187">
       <c r="A12" s="24" t="n"/>
@@ -4617,7 +4605,6 @@
       <c r="O12" s="13" t="n"/>
       <c r="P12" s="13" t="n"/>
       <c r="Q12" s="96" t="n"/>
-      <c r="R12" s="24" t="n"/>
     </row>
     <row r="13" ht="39.95" customHeight="1" s="187">
       <c r="A13" s="24" t="n"/>
@@ -4643,7 +4630,6 @@
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
       <c r="Q13" s="96" t="n"/>
-      <c r="R13" s="24" t="n"/>
     </row>
     <row r="14" ht="39.95" customHeight="1" s="187">
       <c r="A14" s="24" t="n"/>
@@ -4669,7 +4655,6 @@
       <c r="O14" s="13" t="n"/>
       <c r="P14" s="13" t="n"/>
       <c r="Q14" s="96" t="n"/>
-      <c r="R14" s="24" t="n"/>
     </row>
     <row r="15" ht="39.95" customHeight="1" s="187">
       <c r="A15" s="24" t="n"/>
@@ -4695,7 +4680,6 @@
       <c r="O15" s="11" t="n"/>
       <c r="P15" s="11" t="n"/>
       <c r="Q15" s="96" t="n"/>
-      <c r="R15" s="24" t="n"/>
     </row>
     <row r="16" ht="39.95" customHeight="1" s="187">
       <c r="A16" s="24" t="n"/>
@@ -4721,7 +4705,6 @@
       <c r="O16" s="13" t="n"/>
       <c r="P16" s="13" t="n"/>
       <c r="Q16" s="96" t="n"/>
-      <c r="R16" s="24" t="n"/>
     </row>
     <row r="17" ht="39.95" customHeight="1" s="187">
       <c r="A17" s="24" t="n"/>
@@ -4747,7 +4730,6 @@
       <c r="O17" s="11" t="n"/>
       <c r="P17" s="11" t="n"/>
       <c r="Q17" s="96" t="n"/>
-      <c r="R17" s="24" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1" s="187">
       <c r="A18" s="24" t="n"/>
@@ -4773,7 +4755,6 @@
       <c r="O18" s="13" t="n"/>
       <c r="P18" s="13" t="n"/>
       <c r="Q18" s="96" t="n"/>
-      <c r="R18" s="24" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1" s="187">
       <c r="A19" s="24" t="n"/>
@@ -4799,7 +4780,6 @@
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
       <c r="Q19" s="96" t="n"/>
-      <c r="R19" s="24" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="187">
       <c r="A20" s="24" t="n"/>
@@ -4825,7 +4805,6 @@
       <c r="O20" s="13" t="n"/>
       <c r="P20" s="13" t="n"/>
       <c r="Q20" s="96" t="n"/>
-      <c r="R20" s="24" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1" s="187">
       <c r="A21" s="24" t="n"/>
@@ -4851,7 +4830,6 @@
       <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
       <c r="Q21" s="96" t="n"/>
-      <c r="R21" s="24" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1" s="187">
       <c r="A22" s="24" t="n"/>
@@ -4877,7 +4855,6 @@
       <c r="O22" s="13" t="n"/>
       <c r="P22" s="13" t="n"/>
       <c r="Q22" s="96" t="n"/>
-      <c r="R22" s="24" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="187">
       <c r="A23" s="24" t="n"/>
@@ -4903,7 +4880,6 @@
       <c r="O23" s="11" t="n"/>
       <c r="P23" s="11" t="n"/>
       <c r="Q23" s="96" t="n"/>
-      <c r="R23" s="24" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1" s="187">
       <c r="A24" s="24" t="n"/>
@@ -4929,7 +4905,6 @@
       <c r="O24" s="13" t="n"/>
       <c r="P24" s="13" t="n"/>
       <c r="Q24" s="96" t="n"/>
-      <c r="R24" s="24" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1" s="187">
       <c r="A25" s="24" t="n"/>
@@ -4955,7 +4930,6 @@
       <c r="O25" s="11" t="n"/>
       <c r="P25" s="11" t="n"/>
       <c r="Q25" s="96" t="n"/>
-      <c r="R25" s="24" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="187">
       <c r="A26" s="24" t="n"/>
@@ -4981,7 +4955,6 @@
       <c r="O26" s="13" t="n"/>
       <c r="P26" s="13" t="n"/>
       <c r="Q26" s="96" t="n"/>
-      <c r="R26" s="24" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="187">
       <c r="A27" s="24" t="n"/>
@@ -5007,7 +4980,6 @@
       <c r="O27" s="11" t="n"/>
       <c r="P27" s="11" t="n"/>
       <c r="Q27" s="96" t="n"/>
-      <c r="R27" s="24" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1" s="187">
       <c r="A28" s="24" t="n"/>
@@ -5033,7 +5005,6 @@
       <c r="O28" s="13" t="n"/>
       <c r="P28" s="13" t="n"/>
       <c r="Q28" s="96" t="n"/>
-      <c r="R28" s="24" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1" s="187">
       <c r="A29" s="24" t="n"/>
@@ -5059,7 +5030,6 @@
       <c r="O29" s="11" t="n"/>
       <c r="P29" s="11" t="n"/>
       <c r="Q29" s="96" t="n"/>
-      <c r="R29" s="24" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="187">
       <c r="A30" s="24" t="n"/>
@@ -5085,7 +5055,6 @@
       <c r="O30" s="13" t="n"/>
       <c r="P30" s="13" t="n"/>
       <c r="Q30" s="96" t="n"/>
-      <c r="R30" s="24" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1" s="187">
       <c r="A31" s="24" t="n"/>
@@ -5111,7 +5080,6 @@
       <c r="O31" s="11" t="n"/>
       <c r="P31" s="11" t="n"/>
       <c r="Q31" s="96" t="n"/>
-      <c r="R31" s="24" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1" s="187">
       <c r="A32" s="24" t="n"/>
@@ -5137,7 +5105,6 @@
       <c r="O32" s="13" t="n"/>
       <c r="P32" s="13" t="n"/>
       <c r="Q32" s="96" t="n"/>
-      <c r="R32" s="24" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1" s="187">
       <c r="A33" s="24" t="n"/>
@@ -5163,7 +5130,6 @@
       <c r="O33" s="11" t="n"/>
       <c r="P33" s="11" t="n"/>
       <c r="Q33" s="96" t="n"/>
-      <c r="R33" s="24" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="187">
       <c r="A34" s="24" t="n"/>
@@ -5189,7 +5155,6 @@
       <c r="O34" s="13" t="n"/>
       <c r="P34" s="13" t="n"/>
       <c r="Q34" s="96" t="n"/>
-      <c r="R34" s="24" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1" s="187">
       <c r="A35" s="24" t="n"/>
@@ -5215,7 +5180,6 @@
       <c r="O35" s="11" t="n"/>
       <c r="P35" s="11" t="n"/>
       <c r="Q35" s="96" t="n"/>
-      <c r="R35" s="24" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1" s="187">
       <c r="A36" s="24" t="n"/>
@@ -5241,7 +5205,6 @@
       <c r="O36" s="13" t="n"/>
       <c r="P36" s="13" t="n"/>
       <c r="Q36" s="96" t="n"/>
-      <c r="R36" s="24" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="187">
       <c r="A37" s="24" t="n"/>
@@ -5267,7 +5230,6 @@
       <c r="O37" s="11" t="n"/>
       <c r="P37" s="11" t="n"/>
       <c r="Q37" s="96" t="n"/>
-      <c r="R37" s="24" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1" s="187">
       <c r="A38" s="24" t="n"/>
@@ -5293,7 +5255,6 @@
       <c r="O38" s="13" t="n"/>
       <c r="P38" s="13" t="n"/>
       <c r="Q38" s="96" t="n"/>
-      <c r="R38" s="24" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1" s="187">
       <c r="A39" s="24" t="n"/>
@@ -5319,7 +5280,6 @@
       <c r="O39" s="11" t="n"/>
       <c r="P39" s="11" t="n"/>
       <c r="Q39" s="96" t="n"/>
-      <c r="R39" s="24" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="187">
       <c r="A40" s="24" t="n"/>
@@ -5345,7 +5305,6 @@
       <c r="O40" s="13" t="n"/>
       <c r="P40" s="13" t="n"/>
       <c r="Q40" s="96" t="n"/>
-      <c r="R40" s="24" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="187">
       <c r="A41" s="24" t="n"/>
@@ -5371,7 +5330,6 @@
       <c r="O41" s="11" t="n"/>
       <c r="P41" s="11" t="n"/>
       <c r="Q41" s="96" t="n"/>
-      <c r="R41" s="24" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1" s="187">
       <c r="A42" s="24" t="n"/>
@@ -5397,7 +5355,6 @@
       <c r="O42" s="13" t="n"/>
       <c r="P42" s="13" t="n"/>
       <c r="Q42" s="96" t="n"/>
-      <c r="R42" s="24" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="187">
       <c r="A43" s="24" t="n"/>
@@ -5423,7 +5380,6 @@
       <c r="O43" s="11" t="n"/>
       <c r="P43" s="11" t="n"/>
       <c r="Q43" s="96" t="n"/>
-      <c r="R43" s="24" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1" s="187">
       <c r="A44" s="24" t="n"/>
@@ -5449,7 +5405,6 @@
       <c r="O44" s="13" t="n"/>
       <c r="P44" s="13" t="n"/>
       <c r="Q44" s="96" t="n"/>
-      <c r="R44" s="24" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1" s="187">
       <c r="A45" s="24" t="n"/>
@@ -5475,7 +5430,6 @@
       <c r="O45" s="11" t="n"/>
       <c r="P45" s="11" t="n"/>
       <c r="Q45" s="96" t="n"/>
-      <c r="R45" s="24" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1" s="187">
       <c r="A46" s="24" t="n"/>
@@ -5501,7 +5455,6 @@
       <c r="O46" s="13" t="n"/>
       <c r="P46" s="13" t="n"/>
       <c r="Q46" s="96" t="n"/>
-      <c r="R46" s="24" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="187">
       <c r="A47" s="24" t="n"/>
@@ -5527,7 +5480,6 @@
       <c r="O47" s="11" t="n"/>
       <c r="P47" s="11" t="n"/>
       <c r="Q47" s="96" t="n"/>
-      <c r="R47" s="24" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1" s="187">
       <c r="A48" s="24" t="n"/>
@@ -5553,7 +5505,6 @@
       <c r="O48" s="13" t="n"/>
       <c r="P48" s="13" t="n"/>
       <c r="Q48" s="96" t="n"/>
-      <c r="R48" s="24" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1" s="187">
       <c r="A49" s="24" t="n"/>
@@ -5579,7 +5530,6 @@
       <c r="O49" s="11" t="n"/>
       <c r="P49" s="11" t="n"/>
       <c r="Q49" s="96" t="n"/>
-      <c r="R49" s="24" t="n"/>
     </row>
     <row r="51" ht="15.6" customHeight="1" s="187">
       <c r="A51" s="276" t="inlineStr">
@@ -5676,7 +5626,7 @@
     <row r="55" ht="26.1" customHeight="1" s="187">
       <c r="A55" s="278" t="inlineStr">
         <is>
-          <t>Journey ID</t>
+          <t>Journey / Case ID</t>
         </is>
       </c>
       <c r="B55" s="192" t="n"/>
@@ -5735,17 +5685,17 @@
       <c r="A56" s="329" t="n"/>
       <c r="B56" s="244" t="n"/>
       <c r="C56" s="13">
-        <f>IF(A56="","",COUNTIF($R$5:$R$49,A56))</f>
+        <f>IF(A56="","",COUNTIF($B$5:$B$49,A56))</f>
         <v/>
       </c>
       <c r="D56" s="330">
-        <f>IF(A56="","",IFERROR(AVERAGEIF($R$5:$R$49,A56,$L$5:$L$49),""))</f>
+        <f>IF(A56="","",IFERROR(AVERAGEIF($B$5:$B$49,A56,$L$5:$L$49),""))</f>
         <v/>
       </c>
       <c r="E56" s="7" t="n"/>
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="98">
-        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($R$5:$R$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($R$5:$R$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(IFERROR(VALUE(LEFT(E56,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F56,1)),0)/5),""))</f>
+        <f>IF(OR(A56="",D56="",E56="",F56=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A56,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A56,$Q$5:$Q$49,"Level 2"),0),0.5*D56)+0.3*(IFERROR(VALUE(LEFT(E56,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F56,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H56" s="13">
@@ -5759,11 +5709,11 @@
       <c r="M56" s="243" t="n"/>
       <c r="N56" s="244" t="n"/>
       <c r="O56" s="347">
-        <f>IF(A56="","",IFERROR(ROUND(LOOKUP(2,1/($R$5:$R$49=A56),$L$5:$L$49)*5,0),""))</f>
+        <f>IF(A56="","",IFERROR(ROUND(LOOKUP(2,1/($B$5:$B$49=A56),$L$5:$L$49)*5,0),""))</f>
         <v/>
       </c>
       <c r="P56" s="347">
-        <f>IF(A56="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$R$5:$R$49,A56),0),""))</f>
+        <f>IF(A56="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$B$5:$B$49,A56),0),""))</f>
         <v/>
       </c>
     </row>
@@ -5771,17 +5721,17 @@
       <c r="A57" s="289" t="n"/>
       <c r="B57" s="244" t="n"/>
       <c r="C57" s="13">
-        <f>IF(A57="","",COUNTIF($R$5:$R$49,A57))</f>
+        <f>IF(A57="","",COUNTIF($B$5:$B$49,A57))</f>
         <v/>
       </c>
       <c r="D57" s="330">
-        <f>IF(A57="","",IFERROR(AVERAGEIF($R$5:$R$49,A57,$L$5:$L$49),""))</f>
+        <f>IF(A57="","",IFERROR(AVERAGEIF($B$5:$B$49,A57,$L$5:$L$49),""))</f>
         <v/>
       </c>
       <c r="E57" s="7" t="n"/>
       <c r="F57" s="7" t="n"/>
       <c r="G57" s="98">
-        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($R$5:$R$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($R$5:$R$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(IFERROR(VALUE(LEFT(E57,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F57,1)),0)/5),""))</f>
+        <f>IF(OR(A57="",D57="",E57="",F57=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A57,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A57,$Q$5:$Q$49,"Level 2"),0),0.5*D57)+0.3*(IFERROR(VALUE(LEFT(E57,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F57,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H57" s="13">
@@ -5795,11 +5745,11 @@
       <c r="M57" s="243" t="n"/>
       <c r="N57" s="244" t="n"/>
       <c r="O57" s="347">
-        <f>IF(A57="","",IFERROR(ROUND(LOOKUP(2,1/($R$5:$R$49=A57),$L$5:$L$49)*5,0),""))</f>
+        <f>IF(A57="","",IFERROR(ROUND(LOOKUP(2,1/($B$5:$B$49=A57),$L$5:$L$49)*5,0),""))</f>
         <v/>
       </c>
       <c r="P57" s="347">
-        <f>IF(A57="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$R$5:$R$49,A57),0),""))</f>
+        <f>IF(A57="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$B$5:$B$49,A57),0),""))</f>
         <v/>
       </c>
     </row>
@@ -5807,17 +5757,17 @@
       <c r="A58" s="289" t="n"/>
       <c r="B58" s="244" t="n"/>
       <c r="C58" s="11">
-        <f>IF(A58="","",COUNTIF($R$5:$R$49,A58))</f>
+        <f>IF(A58="","",COUNTIF($B$5:$B$49,A58))</f>
         <v/>
       </c>
       <c r="D58" s="332">
-        <f>IF(A58="","",IFERROR(AVERAGEIF($R$5:$R$49,A58,$L$5:$L$49),""))</f>
+        <f>IF(A58="","",IFERROR(AVERAGEIF($B$5:$B$49,A58,$L$5:$L$49),""))</f>
         <v/>
       </c>
       <c r="E58" s="7" t="n"/>
       <c r="F58" s="7" t="n"/>
       <c r="G58" s="99">
-        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($R$5:$R$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($R$5:$R$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(IFERROR(VALUE(LEFT(E58,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F58,1)),0)/5),""))</f>
+        <f>IF(OR(A58="",D58="",E58="",F58=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A58,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A58,$Q$5:$Q$49,"Level 2"),0),0.5*D58)+0.3*(IFERROR(VALUE(LEFT(E58,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F58,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H58" s="11">
@@ -5831,11 +5781,11 @@
       <c r="M58" s="243" t="n"/>
       <c r="N58" s="244" t="n"/>
       <c r="O58" s="347">
-        <f>IF(A58="","",IFERROR(ROUND(LOOKUP(2,1/($R$5:$R$49=A58),$L$5:$L$49)*5,0),""))</f>
+        <f>IF(A58="","",IFERROR(ROUND(LOOKUP(2,1/($B$5:$B$49=A58),$L$5:$L$49)*5,0),""))</f>
         <v/>
       </c>
       <c r="P58" s="347">
-        <f>IF(A58="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$R$5:$R$49,A58),0),""))</f>
+        <f>IF(A58="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$B$5:$B$49,A58),0),""))</f>
         <v/>
       </c>
     </row>
@@ -5843,17 +5793,17 @@
       <c r="A59" s="289" t="n"/>
       <c r="B59" s="244" t="n"/>
       <c r="C59" s="13">
-        <f>IF(A59="","",COUNTIF($R$5:$R$49,A59))</f>
+        <f>IF(A59="","",COUNTIF($B$5:$B$49,A59))</f>
         <v/>
       </c>
       <c r="D59" s="330">
-        <f>IF(A59="","",IFERROR(AVERAGEIF($R$5:$R$49,A59,$L$5:$L$49),""))</f>
+        <f>IF(A59="","",IFERROR(AVERAGEIF($B$5:$B$49,A59,$L$5:$L$49),""))</f>
         <v/>
       </c>
       <c r="E59" s="7" t="n"/>
       <c r="F59" s="7" t="n"/>
       <c r="G59" s="98">
-        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($R$5:$R$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($R$5:$R$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$R$5:$R$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(IFERROR(VALUE(LEFT(E59,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F59,1)),0)/5),""))</f>
+        <f>IF(OR(A59="",D59="",E59="",F59=""),"",IFERROR(IF(AND(COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS($B$5:$B$49,A59,$Q$5:$Q$49,"Level 2")&gt;0),0.2*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 1"),0)+0.3*IFERROR(AVERAGEIFS($L$5:$L$49,$B$5:$B$49,A59,$Q$5:$Q$49,"Level 2"),0),0.5*D59)+0.3*(IFERROR(VALUE(LEFT(E59,1)),0)/5)+0.2*(IFERROR(VALUE(LEFT(F59,1)),0)/5),""))</f>
         <v/>
       </c>
       <c r="H59" s="13">
@@ -5867,18 +5817,18 @@
       <c r="M59" s="243" t="n"/>
       <c r="N59" s="244" t="n"/>
       <c r="O59" s="347">
-        <f>IF(A59="","",IFERROR(ROUND(LOOKUP(2,1/($R$5:$R$49=A59),$L$5:$L$49)*5,0),""))</f>
+        <f>IF(A59="","",IFERROR(ROUND(LOOKUP(2,1/($B$5:$B$49=A59),$L$5:$L$49)*5,0),""))</f>
         <v/>
       </c>
       <c r="P59" s="347">
-        <f>IF(A59="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$R$5:$R$49,A59),0),""))</f>
+        <f>IF(A59="","",IFERROR(ROUND(AVERAGEIFS($P$5:$P$49,$B$5:$B$49,A59),0),""))</f>
         <v/>
       </c>
     </row>
     <row r="60" ht="27.95" customHeight="1" s="187">
       <c r="A60" s="298" t="inlineStr">
         <is>
-          <t>Type a Journey ID in the first column, then judge Outcome &amp; Continuity (0-5). Touches, Avg %, Team Score and the suggested values auto-fill. Group a multi-ticket journey by typing the SAME Journey ID (column R) on every touch row — it may span more than one Case ID. No manual formula editing required.</t>
+          <t>Type a Case ID in the first column, then judge Outcome &amp; Continuity (0-5). Touches, Avg %, Team Score and the suggested values auto-fill from the touch log. Log every touch of the case under the same Case ID with an incrementing Touch #.</t>
         </is>
       </c>
       <c r="B60" s="243" t="n"/>
@@ -14465,7 +14415,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Log every touch under the same JOURNEY ID (Case Tracker column R) with an incrementing Touch # — a journey may span multiple ticket numbers, so the Journey ID, not the Case ID, is the grouping key. Per-touch weighted scores roll up automatically; enter Outcome and Continuity (0-5) once per journey and the Team Score computes.</t>
+          <t>Log every touch under the same Case ID with an incrementing Touch #. Per-touch weighted scores roll up automatically; enter Outcome and Continuity (0-5) once per journey and the Team Score computes.</t>
         </is>
       </c>
     </row>
@@ -15217,7 +15167,7 @@
     </row>
     <row r="7" ht="15.95" customHeight="1" s="187">
       <c r="B7" s="40">
-        <f>"EXECUTION  "&amp;IF($E$6="","(weight)",IF(AND(COUNTIFS('Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS('Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2")&gt;0),"(20% L1 / 30% L2)","(50% weight)"))</f>
+        <f>"EXECUTION  "&amp;IF($E$6="","(weight)",IF(AND(COUNTIFS('Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS('Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2")&gt;0),"(20% L1 / 30% L2)","(50% weight)"))</f>
         <v/>
       </c>
       <c r="C7" s="40" t="inlineStr">
@@ -15247,7 +15197,7 @@
     </row>
     <row r="9" ht="21.95" customHeight="1" s="187">
       <c r="B9" s="259">
-        <f>IF(INDEX('Case Tracker'!$D$56:$D$59,$J$4)="","Team Score computes once the selected journey row is filled.",IF(AND(COUNTIFS('Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS('Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2")&gt;0)," = 20% × L1 ("&amp;TEXT(AVERAGEIFS('Case Tracker'!$L$5:$L$49,'Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1"),"0.0%")&amp;")  +  30% × L2 ("&amp;TEXT(AVERAGEIFS('Case Tracker'!$L$5:$L$49,'Case Tracker'!$R$5:$R$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2"),"0.0%")&amp;")  +  30% × ("&amp;INDEX('Case Tracker'!$E$56:$E$59,$J$4)&amp;"÷5)  +  20% × ("&amp;INDEX('Case Tracker'!$F$56:$F$59,$J$4)&amp;"÷5)"," = 50% × Execution ("&amp;TEXT(INDEX('Case Tracker'!$D$56:$D$59,$J$4),"0.0%")&amp;")  +  30% × ("&amp;INDEX('Case Tracker'!$E$56:$E$59,$J$4)&amp;"÷5)  +  20% × ("&amp;INDEX('Case Tracker'!$F$56:$F$59,$J$4)&amp;"÷5)"))</f>
+        <f>IF(INDEX('Case Tracker'!$D$56:$D$59,$J$4)="","Team Score computes once the selected journey row is filled.",IF(AND(COUNTIFS('Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1")&gt;0,COUNTIFS('Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2")&gt;0)," = 20% × L1 ("&amp;TEXT(AVERAGEIFS('Case Tracker'!$L$5:$L$49,'Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 1"),"0.0%")&amp;")  +  30% × L2 ("&amp;TEXT(AVERAGEIFS('Case Tracker'!$L$5:$L$49,'Case Tracker'!$B$5:$B$49,$E$6,'Case Tracker'!$Q$5:$Q$49,"Level 2"),"0.0%")&amp;")  +  30% × ("&amp;INDEX('Case Tracker'!$E$56:$E$59,$J$4)&amp;"÷5)  +  20% × ("&amp;INDEX('Case Tracker'!$F$56:$F$59,$J$4)&amp;"÷5)"," = 50% × Execution ("&amp;TEXT(INDEX('Case Tracker'!$D$56:$D$59,$J$4),"0.0%")&amp;")  +  30% × ("&amp;INDEX('Case Tracker'!$E$56:$E$59,$J$4)&amp;"÷5)  +  20% × ("&amp;INDEX('Case Tracker'!$F$56:$F$59,$J$4)&amp;"÷5)"))</f>
         <v/>
       </c>
       <c r="C9" s="256" t="n"/>

</xml_diff>

<commit_message>
Add June 25 changelog entries for today's changes
Prepended a JUNE 25, 2026 section to the Changelog sheet covering:
- Three indicator weight raises (567e355)
- Indicator Guide sheet (1320f11)
- Team Scoring honest scorecard math, suggested Outcome/Continuity,
  multi-touch labelling, and journey selector (4dc604d, 4d7e85a)
- Handoff Quality 0-5 dropdown with anchors (b317f3c)
- Web form sync (85f1bdf)

Sheet rebuilt to insert the new section cleanly (preserves styles, merges,
row heights, and the existing June 10-24 history + legend). Verified via
Excel COM: structure intact, opens with no repair prompt.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA Scoring Form Template.xlsx
+++ b/QA Scoring Form Template.xlsx
@@ -25,9 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="83">
     <font>
@@ -3304,7 +3305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" style="187" min="1" max="1"/>
@@ -3358,874 +3359,1042 @@
     <row r="4" ht="20.1" customHeight="1" s="187">
       <c r="A4" s="286" t="inlineStr">
         <is>
-          <t>JUNE 24, 2026</t>
+          <t>JUNE 25, 2026</t>
         </is>
       </c>
     </row>
     <row r="5" ht="56.1" customHeight="1" s="187">
       <c r="A5" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Scoring Form</t>
+        </is>
+      </c>
+      <c r="C5" s="177" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="D5" s="285" t="inlineStr">
+        <is>
+          <t>Raised weights on three behavioral indicators to align with the Support Organization Reset: troubleshooting-before-KB (2 to 3, now Primary), logical troubleshooting process (1 to 2), and minimizing customer effort (1 to 2).</t>
+        </is>
+      </c>
+      <c r="E5" s="179" t="inlineStr">
+        <is>
+          <t>567e355</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56.1" customHeight="1" s="187">
+      <c r="A6" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Indicator Guide</t>
+        </is>
+      </c>
+      <c r="C6" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D6" s="285" t="inlineStr">
+        <is>
+          <t>Added Indicator Guide sheet — the purpose, importance, and failure mode of all 37 behavioral indicators across the 7 categories, with weight tiers (Primary / Core / Supporting).</t>
+        </is>
+      </c>
+      <c r="E6" s="179" t="inlineStr">
+        <is>
+          <t>1320f11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="56.1" customHeight="1" s="187">
+      <c r="A7" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Team Scoring</t>
+        </is>
+      </c>
+      <c r="C7" s="177" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D7" s="285" t="inlineStr">
+        <is>
+          <t>Rewrote the live scorecard so the displayed math matches the actual computation: shows the 20% L1 / 30% L2 execution split for mixed-level journeys and collapses to 50% x Execution for single-level journeys.</t>
+        </is>
+      </c>
+      <c r="E7" s="179" t="inlineStr">
+        <is>
+          <t>4dc604d</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="56.1" customHeight="1" s="187">
+      <c r="A8" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Team Scoring</t>
+        </is>
+      </c>
+      <c r="C8" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D8" s="285" t="inlineStr">
+        <is>
+          <t>Added advisory Suggested Outcome (final-touch weighted x 5) and Suggested Continuity (average Handoff Quality) reference values beside the manual journey Outcome/Continuity entries.</t>
+        </is>
+      </c>
+      <c r="E8" s="179" t="inlineStr">
+        <is>
+          <t>4dc604d</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56.1" customHeight="1" s="187">
+      <c r="A9" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Team Scoring</t>
+        </is>
+      </c>
+      <c r="C9" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D9" s="285" t="inlineStr">
+        <is>
+          <t>Added a journey-selector dropdown so the scorecard can display any logged journey instead of being fixed to one row.</t>
+        </is>
+      </c>
+      <c r="E9" s="179" t="inlineStr">
+        <is>
+          <t>4d7e85a</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56.1" customHeight="1" s="187">
+      <c r="A10" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Case Tracker</t>
+        </is>
+      </c>
+      <c r="C10" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D10" s="285" t="inlineStr">
+        <is>
+          <t>Made Handoff Quality (column P) a 0-5 dropdown with anchor descriptions (5 Seamless to 0 Broken), an on-cell prompt, and a legend block below the journey table.</t>
+        </is>
+      </c>
+      <c r="E10" s="179" t="inlineStr">
+        <is>
+          <t>b317f3c</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56.1" customHeight="1" s="187">
+      <c r="A11" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Case Tracker / Team Scoring</t>
+        </is>
+      </c>
+      <c r="C11" s="177" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="D11" s="285" t="inlineStr">
+        <is>
+          <t>Labelled both sheets as multi-touch only; single-call evaluations use the Scoring Form sheet only, with no Case Tracker entry needed.</t>
+        </is>
+      </c>
+      <c r="E11" s="179" t="inlineStr">
+        <is>
+          <t>4dc604d</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56.1" customHeight="1" s="187">
+      <c r="A12" s="176" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Web Platform</t>
+        </is>
+      </c>
+      <c r="C12" s="177" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="D12" s="285" t="inlineStr">
+        <is>
+          <t>Synced the web form (qa-scoring-form.html) to the Excel form: the three indicator weight changes, N.A. weight redistribution in the Score Summary, Handoff Quality dropdown, suggested Outcome/Continuity, and multi-touch labelling.</t>
+        </is>
+      </c>
+      <c r="E12" s="179" t="inlineStr">
+        <is>
+          <t>85f1bdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20.1" customHeight="1" s="187">
+      <c r="A13" s="286" t="inlineStr">
+        <is>
+          <t>JUNE 24, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="56.1" customHeight="1" s="187">
+      <c r="A14" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Web Platform</t>
         </is>
       </c>
-      <c r="C5" s="177" t="inlineStr">
+      <c r="C14" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D5" s="285" t="inlineStr">
+      <c r="D14" s="285" t="inlineStr">
         <is>
           <t>Expanded web QA platform to full three-tab app: Scoring Form, Case Tracker (17 columns, live weighted %, contribution type, team score), and Team Scoring (live scorecard, category heatmap, gap diagnosis, per-touch breakdown, team opportunities action plan). Single standalone HTML — no install or internet required.</t>
         </is>
       </c>
-      <c r="E5" s="179" t="inlineStr">
+      <c r="E14" s="179" t="inlineStr">
         <is>
           <t>135774f</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1" s="187">
-      <c r="A6" s="180" t="n">
+    <row r="15" ht="56.1" customHeight="1" s="187">
+      <c r="A15" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B6" s="181" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Web Platform</t>
         </is>
       </c>
-      <c r="C6" s="177" t="inlineStr">
+      <c r="C15" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D6" s="182" t="inlineStr">
+      <c r="D15" s="285" t="inlineStr">
         <is>
           <t>Built initial web-based QA Scoring Form as a single standalone HTML file. All 7 categories with 38 behavioral indicators, color-coded assessment dropdowns, auto-score calculation, coaching flags, auto-zero, save/load via localStorage, export/import JSON, print-ready.</t>
         </is>
       </c>
-      <c r="E6" s="179" t="inlineStr">
+      <c r="E15" s="179" t="inlineStr">
         <is>
           <t>7db846a</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1" s="187">
-      <c r="A7" s="176" t="n">
+    <row r="16" ht="56.1" customHeight="1" s="187">
+      <c r="A16" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Scoring Form / Example (Filled)</t>
         </is>
       </c>
-      <c r="C7" s="183" t="inlineStr">
+      <c r="C16" s="177" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="D7" s="285" t="inlineStr">
+      <c r="D16" s="285" t="inlineStr">
         <is>
           <t>Fixed auto-score formula ranges and H-column weights for 5 new gap indicators. Cat 1 formula expanded to C36:C41 with weights {3,2,1,2,2,2}; Cat 4 expanded to C75:C80 with weights {3,2,2,1,2,2}. Example (Filled) hardcoded array formulas updated to match.</t>
         </is>
       </c>
-      <c r="E7" s="179" t="inlineStr">
+      <c r="E16" s="179" t="inlineStr">
         <is>
           <t>b93c12c</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="69.95" customHeight="1" s="187">
-      <c r="A8" s="180" t="n">
+    <row r="17" ht="56.1" customHeight="1" s="187">
+      <c r="A17" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B8" s="181" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Scoring Form / Example (Filled)</t>
         </is>
       </c>
-      <c r="C8" s="177" t="inlineStr">
+      <c r="C17" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D8" s="182" t="inlineStr">
+      <c r="D17" s="285" t="inlineStr">
         <is>
           <t>Added 5 new behavioral indicators identified from Support Organization Reset Playbook alignment audit: (1) KB/self-help misuse now scoreable in Cat 1, (2) Escalation criteria updated with specific recognized triggers in Cat 5, (3) Repeat contact recognition added to Cat 4, (4) Out-of-warranty handling added to Cat 1 (N.A. for in-warranty), (5) Handoff quality added to Cat 4. Applied to both Scoring Form and Example (Filled).</t>
         </is>
       </c>
-      <c r="E8" s="179" t="inlineStr">
+      <c r="E17" s="179" t="inlineStr">
         <is>
           <t>fb76161</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="27.95" customHeight="1" s="187">
-      <c r="A9" s="176" t="n">
+    <row r="18" ht="56.1" customHeight="1" s="187">
+      <c r="A18" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="C9" s="177" t="inlineStr">
+      <c r="C18" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D9" s="285" t="inlineStr">
+      <c r="D18" s="285" t="inlineStr">
         <is>
           <t>Created QA Weight Justification.txt — written rationale for all 7 category weights, formatted for email distribution to stakeholders.</t>
         </is>
       </c>
-      <c r="E9" s="179" t="inlineStr">
+      <c r="E18" s="179" t="inlineStr">
         <is>
           <t>819d065</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="27.95" customHeight="1" s="187">
-      <c r="A10" s="180" t="n">
+    <row r="19" ht="56.1" customHeight="1" s="187">
+      <c r="A19" s="176" t="n">
         <v>46197</v>
       </c>
-      <c r="B10" s="181" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="C10" s="177" t="inlineStr">
+      <c r="C19" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D10" s="182" t="inlineStr">
+      <c r="D19" s="285" t="inlineStr">
         <is>
           <t>Committed Support Organization Reset Playbook (docx) — used as source document to audit and align behavioral indicators with organizational goals.</t>
         </is>
       </c>
-      <c r="E10" s="179" t="inlineStr">
+      <c r="E19" s="179" t="inlineStr">
         <is>
           <t>819d065</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20.1" customHeight="1" s="187">
-      <c r="A11" s="286" t="inlineStr">
+    <row r="20" ht="20.1" customHeight="1" s="187">
+      <c r="A20" s="286" t="inlineStr">
         <is>
           <t>JUNE 23, 2026</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="56.1" customHeight="1" s="187">
-      <c r="A12" s="180" t="n">
+    <row r="21" ht="56.1" customHeight="1" s="187">
+      <c r="A21" s="176" t="n">
         <v>46196</v>
       </c>
-      <c r="B12" s="181" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Example (Filled)</t>
         </is>
       </c>
-      <c r="C12" s="184" t="inlineStr">
+      <c r="C21" s="177" t="inlineStr">
         <is>
           <t>UPDATE</t>
         </is>
       </c>
-      <c r="D12" s="182" t="inlineStr">
+      <c r="D21" s="285" t="inlineStr">
         <is>
           <t>Rebuilt Example (Filled) sheet to fully align all behavioral indicators with the Scoring Form. Deleted 11 extra rows where EF had more indicators than SF, merged split indicators, repurposed rows where order differed. All 7 categories now match exactly: same wording, same count, same order.</t>
         </is>
       </c>
-      <c r="E12" s="179" t="inlineStr">
+      <c r="E21" s="179" t="inlineStr">
         <is>
           <t>820d69d</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="27.95" customHeight="1" s="187">
-      <c r="A13" s="176" t="n">
+    <row r="22" ht="56.1" customHeight="1" s="187">
+      <c r="A22" s="176" t="n">
         <v>46196</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Example (Filled)</t>
         </is>
       </c>
-      <c r="C13" s="183" t="inlineStr">
+      <c r="C22" s="177" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="D13" s="285" t="inlineStr">
+      <c r="D22" s="285" t="inlineStr">
         <is>
           <t>Fixed weight redistribution and section numbering after indicator alignment. Auto-score formulas and H-column references corrected post-row deletions.</t>
         </is>
       </c>
-      <c r="E13" s="179" t="inlineStr">
+      <c r="E22" s="179" t="inlineStr">
         <is>
           <t>96ca232</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20.1" customHeight="1" s="187">
-      <c r="A14" s="286" t="inlineStr">
+    <row r="23" ht="20.1" customHeight="1" s="187">
+      <c r="A23" s="286" t="inlineStr">
         <is>
           <t>JUNE 19, 2026</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="27.95" customHeight="1" s="187">
-      <c r="A15" s="176" t="n">
+    <row r="24" ht="56.1" customHeight="1" s="187">
+      <c r="A24" s="176" t="n">
         <v>46192</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Auto-Zero Guide</t>
         </is>
       </c>
-      <c r="C15" s="177" t="inlineStr">
+      <c r="C24" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D15" s="285" t="inlineStr">
+      <c r="D24" s="285" t="inlineStr">
         <is>
           <t>Added Auto-Zero Guide sheet explaining when and how the auto-zero mechanism triggers, with tooltips on each A–K item explaining the condition and its impact on the quality score.</t>
         </is>
       </c>
-      <c r="E15" s="179" t="inlineStr">
+      <c r="E24" s="179" t="inlineStr">
         <is>
           <t>78e2dc8</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" s="187">
-      <c r="A16" s="180" t="n">
+    <row r="25" ht="56.1" customHeight="1" s="187">
+      <c r="A25" s="176" t="n">
         <v>46192</v>
       </c>
-      <c r="B16" s="181" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C16" s="183" t="inlineStr">
+      <c r="C25" s="177" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="D16" s="182" t="inlineStr">
+      <c r="D25" s="285" t="inlineStr">
         <is>
           <t>Implemented N.A. weight redistribution: when an indicator is marked N.A., its weight is excluded from the denominator so remaining indicators carry full scoring weight. Prevents artificial score depression on inapplicable items.</t>
         </is>
       </c>
-      <c r="E16" s="179" t="inlineStr">
+      <c r="E25" s="179" t="inlineStr">
         <is>
           <t>78e2dc8</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="27.95" customHeight="1" s="187">
-      <c r="A17" s="176" t="n">
+    <row r="26" ht="56.1" customHeight="1" s="187">
+      <c r="A26" s="176" t="n">
         <v>46192</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Scoring Guide</t>
         </is>
       </c>
-      <c r="C17" s="184" t="inlineStr">
+      <c r="C26" s="177" t="inlineStr">
         <is>
           <t>UPDATE</t>
         </is>
       </c>
-      <c r="D17" s="285" t="inlineStr">
+      <c r="D26" s="285" t="inlineStr">
         <is>
           <t>Synced Scoring Guide indicator labels to match updated Scoring Form wording. Refocused Customer Ownership commitments block language.</t>
         </is>
       </c>
-      <c r="E17" s="179" t="inlineStr">
+      <c r="E26" s="179" t="inlineStr">
         <is>
           <t>de1727b</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20.1" customHeight="1" s="187">
-      <c r="A18" s="286" t="inlineStr">
-        <is>
-          <t>JUNE 18, 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1" s="187">
-      <c r="A19" s="176" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Scoring Form</t>
-        </is>
-      </c>
-      <c r="C19" s="185" t="inlineStr">
-        <is>
-          <t>REMOVED</t>
-        </is>
-      </c>
-      <c r="D19" s="285" t="inlineStr">
-        <is>
-          <t>Replaced Critical Failure Conditions section (static list) with auto-populated Coaching Flags that trigger dynamically based on Partial and Missed ratings. Each flag links directly to a required coaching action.</t>
-        </is>
-      </c>
-      <c r="E19" s="186" t="inlineStr">
-        <is>
-          <t>5e83111</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="27.95" customHeight="1" s="187">
-      <c r="A20" s="180" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B20" s="181" t="inlineStr">
-        <is>
-          <t>Scoring Form</t>
-        </is>
-      </c>
-      <c r="C20" s="177" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="D20" s="182" t="inlineStr">
-        <is>
-          <t>Added Agent Level field to Case Information section to distinguish L1 from L2 touches for team scoring purposes.</t>
-        </is>
-      </c>
-      <c r="E20" s="179" t="inlineStr">
-        <is>
-          <t>f765862</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="42" customHeight="1" s="187">
-      <c r="A21" s="176" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Case Tracker</t>
-        </is>
-      </c>
-      <c r="C21" s="177" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="D21" s="285" t="inlineStr">
-        <is>
-          <t>Added Level column (L1/L2) to Case Tracker and implemented level-weighted Team Score formula: 20% × L1 avg + 30% × L2 avg + 30% × (Outcome ÷ 5) + 20% × (Continuity ÷ 5). L2 touches carry higher weight.</t>
-        </is>
-      </c>
-      <c r="E21" s="179" t="inlineStr">
-        <is>
-          <t>3242bea</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="27.95" customHeight="1" s="187">
-      <c r="A22" s="180" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B22" s="181" t="inlineStr">
-        <is>
-          <t>Case Tracker</t>
-        </is>
-      </c>
-      <c r="C22" s="183" t="inlineStr">
-        <is>
-          <t>FIX</t>
-        </is>
-      </c>
-      <c r="D22" s="182" t="inlineStr">
-        <is>
-          <t>Added fallback formula for single-level journeys (all L1 or all L2) so Team Score computes correctly when only one agent level is present.</t>
-        </is>
-      </c>
-      <c r="E22" s="179" t="inlineStr">
-        <is>
-          <t>44b1d42</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="27.95" customHeight="1" s="187">
-      <c r="A23" s="176" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Case Tracker</t>
-        </is>
-      </c>
-      <c r="C23" s="184" t="inlineStr">
-        <is>
-          <t>UPDATE</t>
-        </is>
-      </c>
-      <c r="D23" s="285" t="inlineStr">
-        <is>
-          <t>Formatted Team Score display to 2 decimal places (0.00%). Cleared pre-loaded example entries to produce a clean template.</t>
-        </is>
-      </c>
-      <c r="E23" s="179" t="inlineStr">
-        <is>
-          <t>1e7db88</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="27.95" customHeight="1" s="187">
-      <c r="A24" s="180" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B24" s="181" t="inlineStr">
-        <is>
-          <t>Team Scoring</t>
-        </is>
-      </c>
-      <c r="C24" s="177" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="D24" s="182" t="inlineStr">
-        <is>
-          <t>Added Journey Outcome (0–5) and Continuity of Support (0–5) scoring anchors with detailed descriptors for each level. Implemented as dropdown selectors (Option B).</t>
-        </is>
-      </c>
-      <c r="E24" s="179" t="inlineStr">
-        <is>
-          <t>9022f2f</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="27.95" customHeight="1" s="187">
-      <c r="A25" s="176" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Scoring Form</t>
-        </is>
-      </c>
-      <c r="C25" s="183" t="inlineStr">
-        <is>
-          <t>FIX</t>
-        </is>
-      </c>
-      <c r="D25" s="285" t="inlineStr">
-        <is>
-          <t>Added override justification fields for each category score. Realigned conditional formatting. Fixed Score Summary off-by-one calculation.</t>
-        </is>
-      </c>
-      <c r="E25" s="179" t="inlineStr">
-        <is>
-          <t>de1727b</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="27.95" customHeight="1" s="187">
-      <c r="A26" s="180" t="n">
-        <v>46191</v>
-      </c>
-      <c r="B26" s="181" t="inlineStr">
-        <is>
-          <t>Scoring Form</t>
-        </is>
-      </c>
-      <c r="C26" s="183" t="inlineStr">
-        <is>
-          <t>FIX</t>
-        </is>
-      </c>
-      <c r="D26" s="182" t="inlineStr">
-        <is>
-          <t>Removed blank row 75 from Customer Ownership section. Sharpened row 74 wording to eliminate overlap with row 75. Cleaned template of all case-specific notes.</t>
-        </is>
-      </c>
-      <c r="E26" s="179" t="inlineStr">
-        <is>
-          <t>12ab905</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20.1" customHeight="1" s="187">
       <c r="A27" s="286" t="inlineStr">
         <is>
+          <t>JUNE 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="56.1" customHeight="1" s="187">
+      <c r="A28" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Scoring Form</t>
+        </is>
+      </c>
+      <c r="C28" s="177" t="inlineStr">
+        <is>
+          <t>REMOVED</t>
+        </is>
+      </c>
+      <c r="D28" s="285" t="inlineStr">
+        <is>
+          <t>Replaced Critical Failure Conditions section (static list) with auto-populated Coaching Flags that trigger dynamically based on Partial and Missed ratings. Each flag links directly to a required coaching action.</t>
+        </is>
+      </c>
+      <c r="E28" s="179" t="inlineStr">
+        <is>
+          <t>5e83111</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="56.1" customHeight="1" s="187">
+      <c r="A29" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Scoring Form</t>
+        </is>
+      </c>
+      <c r="C29" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D29" s="285" t="inlineStr">
+        <is>
+          <t>Added Agent Level field to Case Information section to distinguish L1 from L2 touches for team scoring purposes.</t>
+        </is>
+      </c>
+      <c r="E29" s="179" t="inlineStr">
+        <is>
+          <t>f765862</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="56.1" customHeight="1" s="187">
+      <c r="A30" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Case Tracker</t>
+        </is>
+      </c>
+      <c r="C30" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D30" s="285" t="inlineStr">
+        <is>
+          <t>Added Level column (L1/L2) to Case Tracker and implemented level-weighted Team Score formula: 20% × L1 avg + 30% × L2 avg + 30% × (Outcome ÷ 5) + 20% × (Continuity ÷ 5). L2 touches carry higher weight.</t>
+        </is>
+      </c>
+      <c r="E30" s="179" t="inlineStr">
+        <is>
+          <t>3242bea</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="56.1" customHeight="1" s="187">
+      <c r="A31" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Case Tracker</t>
+        </is>
+      </c>
+      <c r="C31" s="177" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D31" s="285" t="inlineStr">
+        <is>
+          <t>Added fallback formula for single-level journeys (all L1 or all L2) so Team Score computes correctly when only one agent level is present.</t>
+        </is>
+      </c>
+      <c r="E31" s="179" t="inlineStr">
+        <is>
+          <t>44b1d42</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="56.1" customHeight="1" s="187">
+      <c r="A32" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Case Tracker</t>
+        </is>
+      </c>
+      <c r="C32" s="177" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="D32" s="285" t="inlineStr">
+        <is>
+          <t>Formatted Team Score display to 2 decimal places (0.00%). Cleared pre-loaded example entries to produce a clean template.</t>
+        </is>
+      </c>
+      <c r="E32" s="179" t="inlineStr">
+        <is>
+          <t>1e7db88</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="56.1" customHeight="1" s="187">
+      <c r="A33" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Team Scoring</t>
+        </is>
+      </c>
+      <c r="C33" s="177" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="D33" s="285" t="inlineStr">
+        <is>
+          <t>Added Journey Outcome (0–5) and Continuity of Support (0–5) scoring anchors with detailed descriptors for each level. Implemented as dropdown selectors (Option B).</t>
+        </is>
+      </c>
+      <c r="E33" s="179" t="inlineStr">
+        <is>
+          <t>9022f2f</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="56.1" customHeight="1" s="187">
+      <c r="A34" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Scoring Form</t>
+        </is>
+      </c>
+      <c r="C34" s="177" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D34" s="285" t="inlineStr">
+        <is>
+          <t>Added override justification fields for each category score. Realigned conditional formatting. Fixed Score Summary off-by-one calculation.</t>
+        </is>
+      </c>
+      <c r="E34" s="179" t="inlineStr">
+        <is>
+          <t>de1727b</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56.1" customHeight="1" s="187">
+      <c r="A35" s="176" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Scoring Form</t>
+        </is>
+      </c>
+      <c r="C35" s="177" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D35" s="285" t="inlineStr">
+        <is>
+          <t>Removed blank row 75 from Customer Ownership section. Sharpened row 74 wording to eliminate overlap with row 75. Cleaned template of all case-specific notes.</t>
+        </is>
+      </c>
+      <c r="E35" s="179" t="inlineStr">
+        <is>
+          <t>12ab905</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20.1" customHeight="1" s="187">
+      <c r="A36" s="286" t="inlineStr">
+        <is>
           <t>JUNE 17, 2026</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="27.95" customHeight="1" s="187">
-      <c r="A28" s="180" t="n">
+    <row r="37" ht="56.1" customHeight="1" s="187">
+      <c r="A37" s="176" t="n">
         <v>46190</v>
       </c>
-      <c r="B28" s="181" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Scoring Guide</t>
         </is>
       </c>
-      <c r="C28" s="177" t="inlineStr">
+      <c r="C37" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D28" s="182" t="inlineStr">
+      <c r="D37" s="285" t="inlineStr">
         <is>
           <t>Added comprehensive Scoring Guide sheet with full Met / Partial / Missed / N.A. definitions, score anchors (0–5), and behavioral examples for each of the 7 categories.</t>
         </is>
       </c>
-      <c r="E28" s="179" t="inlineStr">
+      <c r="E37" s="179" t="inlineStr">
         <is>
           <t>c4a9656</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="42" customHeight="1" s="187">
-      <c r="A29" s="176" t="n">
+    <row r="38" ht="56.1" customHeight="1" s="187">
+      <c r="A38" s="176" t="n">
         <v>46190</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C29" s="184" t="inlineStr">
+      <c r="C38" s="177" t="inlineStr">
         <is>
           <t>UPDATE</t>
         </is>
       </c>
-      <c r="D29" s="285" t="inlineStr">
+      <c r="D38" s="285" t="inlineStr">
         <is>
           <t>Implemented team behavioral indicator proposals from Behavior Indicators Comparison file. Merged Communication rows 69+71. Updated Ownership §4 rows 73–74. Split Resolution and Technical Accuracy merged indicators back into two distinct indicators each.</t>
         </is>
       </c>
-      <c r="E29" s="179" t="inlineStr">
+      <c r="E38" s="179" t="inlineStr">
         <is>
           <t>44e7dfc</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="27.95" customHeight="1" s="187">
-      <c r="A30" s="180" t="n">
+    <row r="39" ht="56.1" customHeight="1" s="187">
+      <c r="A39" s="176" t="n">
         <v>46190</v>
       </c>
-      <c r="B30" s="181" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C30" s="185" t="inlineStr">
+      <c r="C39" s="177" t="inlineStr">
         <is>
           <t>REMOVED</t>
         </is>
       </c>
-      <c r="D30" s="182" t="inlineStr">
+      <c r="D39" s="285" t="inlineStr">
         <is>
           <t>Removed 5 duplicate Critical Failure Conditions already covered by the Auto-Zero section. Eliminated redundancy between the two mechanisms.</t>
         </is>
       </c>
-      <c r="E30" s="179" t="inlineStr">
+      <c r="E39" s="179" t="inlineStr">
         <is>
           <t>97128c7</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="27.95" customHeight="1" s="187">
-      <c r="A31" s="176" t="n">
+    <row r="40" ht="56.1" customHeight="1" s="187">
+      <c r="A40" s="176" t="n">
         <v>46190</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C31" s="183" t="inlineStr">
+      <c r="C40" s="177" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="D31" s="285" t="inlineStr">
+      <c r="D40" s="285" t="inlineStr">
         <is>
           <t>Clarified overlapping Communication indicators to eliminate scoring confusion. Removed all blank rows from the form; compacted from ~220 to 187 rows.</t>
         </is>
       </c>
-      <c r="E31" s="179" t="inlineStr">
+      <c r="E40" s="179" t="inlineStr">
         <is>
           <t>87e03d9</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20.1" customHeight="1" s="187">
-      <c r="A32" s="286" t="inlineStr">
+    <row r="41" ht="20.1" customHeight="1" s="187">
+      <c r="A41" s="286" t="inlineStr">
         <is>
           <t>JUNE 16, 2026</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="27.95" customHeight="1" s="187">
-      <c r="A33" s="176" t="n">
+    <row r="42" ht="56.1" customHeight="1" s="187">
+      <c r="A42" s="176" t="n">
         <v>46189</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C33" s="177" t="inlineStr">
+      <c r="C42" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D33" s="285" t="inlineStr">
+      <c r="D42" s="285" t="inlineStr">
         <is>
           <t>Added Escalation Follow-Up section (what L2 did to resolve the case, L1 learning points) and Next Session Focus section (specific behaviors to practice before next review).</t>
         </is>
       </c>
-      <c r="E33" s="179" t="inlineStr">
+      <c r="E42" s="179" t="inlineStr">
         <is>
           <t>87e03d9</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="27.95" customHeight="1" s="187">
-      <c r="A34" s="180" t="n">
+    <row r="43" ht="56.1" customHeight="1" s="187">
+      <c r="A43" s="176" t="n">
         <v>46189</v>
       </c>
-      <c r="B34" s="181" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Scoring Form</t>
         </is>
       </c>
-      <c r="C34" s="177" t="inlineStr">
+      <c r="C43" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D34" s="182" t="inlineStr">
+      <c r="D43" s="285" t="inlineStr">
         <is>
           <t>Added QA scoring template with completed evaluations (Good Call, Bad Call examples). Restructured overall scoring form layout with cleaner section flow.</t>
         </is>
       </c>
-      <c r="E34" s="179" t="inlineStr">
+      <c r="E43" s="179" t="inlineStr">
         <is>
           <t>201673c</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20.1" customHeight="1" s="187">
-      <c r="A35" s="286" t="inlineStr">
+    <row r="44" ht="20.1" customHeight="1" s="187">
+      <c r="A44" s="286" t="inlineStr">
         <is>
           <t>JUNE 15, 2026</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="27.95" customHeight="1" s="187">
-      <c r="A36" s="180" t="n">
+    <row r="45" ht="56.1" customHeight="1" s="187">
+      <c r="A45" s="176" t="n">
         <v>46188</v>
       </c>
-      <c r="B36" s="181" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Case Tracker</t>
         </is>
       </c>
-      <c r="C36" s="177" t="inlineStr">
+      <c r="C45" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D36" s="182" t="inlineStr">
+      <c r="D45" s="285" t="inlineStr">
         <is>
           <t>Added per-touch Contribution Type scoring (Resolver / Progress Builder / Maintainer / Regression Contributor) and Handoff Quality (0–5) column to Case Tracker.</t>
         </is>
       </c>
-      <c r="E36" s="179" t="inlineStr">
+      <c r="E45" s="179" t="inlineStr">
         <is>
           <t>11f1ee6</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="27.95" customHeight="1" s="187">
-      <c r="A37" s="176" t="n">
+    <row r="46" ht="56.1" customHeight="1" s="187">
+      <c r="A46" s="176" t="n">
         <v>46188</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>Case Tracker</t>
         </is>
       </c>
-      <c r="C37" s="184" t="inlineStr">
+      <c r="C46" s="177" t="inlineStr">
         <is>
           <t>UPDATE</t>
         </is>
       </c>
-      <c r="D37" s="285" t="inlineStr">
+      <c r="D46" s="285" t="inlineStr">
         <is>
           <t>Renamed Contribution Type value 'Breaker' to 'Regression Contributor' for more coaching-oriented, less punitive language.</t>
         </is>
       </c>
-      <c r="E37" s="179" t="inlineStr">
+      <c r="E46" s="179" t="inlineStr">
         <is>
           <t>5be05c9</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20.1" customHeight="1" s="187">
-      <c r="A38" s="286" t="inlineStr">
+    <row r="47" ht="20.1" customHeight="1" s="187">
+      <c r="A47" s="286" t="inlineStr">
         <is>
           <t>JUNE 10, 2026</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="42" customHeight="1" s="187">
-      <c r="A39" s="176" t="n">
+    <row r="48" ht="56.1" customHeight="1" s="187">
+      <c r="A48" s="176" t="n">
         <v>46183</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>All Sheets</t>
         </is>
       </c>
-      <c r="C39" s="177" t="inlineStr">
+      <c r="C48" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D39" s="285" t="inlineStr">
+      <c r="D48" s="285" t="inlineStr">
         <is>
           <t>Initial commit: QA scoring rubric established. Excel scoring form created with 7-category weighted framework (Resolution 30%, Technical Accuracy 20%, Communication 15%, Customer Ownership 15%, Escalation Judgment 10%, Customer Experience 5%, Documentation 5%).</t>
         </is>
       </c>
-      <c r="E39" s="179" t="inlineStr">
+      <c r="E48" s="179" t="inlineStr">
         <is>
           <t>6d52d9a</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="D40" s="285" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="284" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="284" t="inlineStr">
         <is>
           <t>CHANGE TYPE LEGEND</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="27.95" customHeight="1" s="187">
-      <c r="C42" s="177" t="inlineStr">
+    <row r="51" ht="27.95" customHeight="1" s="187">
+      <c r="C51" s="177" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
-      <c r="D42" s="285" t="inlineStr">
+      <c r="D51" s="285" t="inlineStr">
         <is>
           <t>Brand-new feature, section, sheet, or indicator added</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="27.95" customHeight="1" s="187">
-      <c r="C43" s="184" t="inlineStr">
+    <row r="52" ht="27.95" customHeight="1" s="187">
+      <c r="C52" s="177" t="inlineStr">
         <is>
           <t>UPDATE</t>
         </is>
       </c>
-      <c r="D43" s="285" t="inlineStr">
+      <c r="D52" s="285" t="inlineStr">
         <is>
           <t>Existing content revised, reworded, or restructured</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="27.95" customHeight="1" s="187">
-      <c r="C44" s="183" t="inlineStr">
+    <row r="53" ht="27.95" customHeight="1" s="187">
+      <c r="C53" s="177" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="D44" s="285" t="inlineStr">
+      <c r="D53" s="285" t="inlineStr">
         <is>
           <t>Formula error, calculation bug, or structural issue corrected</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="27.95" customHeight="1" s="187">
-      <c r="C45" s="185" t="inlineStr">
+    <row r="54" ht="27.95" customHeight="1" s="187">
+      <c r="C54" s="177" t="inlineStr">
         <is>
           <t>REMOVED</t>
         </is>
       </c>
-      <c r="D45" s="285" t="inlineStr">
+      <c r="D54" s="285" t="inlineStr">
         <is>
           <t>Item, row, or section deleted (usually replaced by something better)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="D46" s="285" t="n"/>
-    </row>
-    <row r="47">
-      <c r="D47" s="285" t="n"/>
-    </row>
-    <row r="48">
-      <c r="D48" s="285" t="n"/>
-    </row>
-    <row r="49">
-      <c r="D49" s="285" t="n"/>
-    </row>
-    <row r="50">
-      <c r="D50" s="285" t="n"/>
-    </row>
-    <row r="51">
-      <c r="D51" s="285" t="n"/>
-    </row>
-    <row r="52">
-      <c r="D52" s="285" t="n"/>
-    </row>
-    <row r="53">
-      <c r="D53" s="285" t="n"/>
-    </row>
-    <row r="54">
-      <c r="D54" s="285" t="n"/>
-    </row>
-    <row r="55">
-      <c r="D55" s="285" t="n"/>
-    </row>
-    <row r="56">
-      <c r="D56" s="285" t="n"/>
-    </row>
-    <row r="57">
-      <c r="D57" s="285" t="n"/>
-    </row>
-    <row r="58">
-      <c r="D58" s="285" t="n"/>
-    </row>
-    <row r="59">
-      <c r="D59" s="285" t="n"/>
-    </row>
-    <row r="60">
-      <c r="D60" s="285" t="n"/>
-    </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A35:E35"/>
+  <mergeCells count="12">
+    <mergeCell ref="A50:E50"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A44:E44"/>
     <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4239,7 +4408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R69"/>
+  <dimension ref="A1:Q69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="187" min="1" max="1"/>

</xml_diff>